<commit_message>
Deducir las luces de las vigas de fundacion de la posicion de los pilotes
Los pilotes estan dibujados como circulos de 30 cm: se extraen 33 de
la geometria vectorial, mucho mas precisos que los rotulos P##, que
estan desplazados. Cruzandolos con el eje de cada VF se obtiene la
luz real entre apoyos. VF14 pasa de 8,75 a 3,09 m, VF10c de 8,03 a
5,10 y VF18a de 7,48 a 5,50. Las cuatro que fallaban por esbeltez
pasan a verificar.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -11802,7 +11802,7 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>3.28</v>
+        <v>2.94</v>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
@@ -11882,7 +11882,11 @@
         <f>IF(OR(M7="REVISAR",P7="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M7&lt;&gt;"REVISAR",P7&lt;&gt;"REVISAR",IF(ISNUMBER(M7),N7*PI()*(O7/10)^2/4&gt;=M7,TRUE),IF(ISNUMBER(P7),Q7*PI()*(R7/10)^2/4&gt;=P7,TRUE),IF(ISNUMBER(M7),M7&lt;=0.0163*J7*K7,TRUE),IF(ISNUMBER(P7),P7&lt;=0.0163*J7*K7,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F7&lt;=Datos_vigas!$B$9*(0.53*SQRT(Datos_vigas!$B$5)*J7*K7+2*PI()*(U7/10)^2/4*Datos_vigas!$B$6*K7/V7)),"NO VERIF. CORTE","VERIFICA")))</f>
         <v/>
       </c>
-      <c r="X7" s="11" t="n"/>
+      <c r="X7" s="13" t="inlineStr">
+        <is>
+          <t>Longitud total 3.28 m. La luz de calculo es la mayor entre pilotes, deducida de la posicion de los pilotes dibujados en el plano.</t>
+        </is>
+      </c>
       <c r="Y7" s="12" t="n">
         <v>3.15</v>
       </c>
@@ -11897,7 +11901,7 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>9.279999999999999</v>
+        <v>9.01</v>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
@@ -11940,20 +11944,20 @@
         <v/>
       </c>
       <c r="N8" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O8" s="10" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="P8" s="25">
         <f>IF(NOT(ISNUMBER(I8)),"---",IF(I8&lt;=0,"---",IF(I8*100/(Datos_vigas!$B$8*J8*K8^2*Datos_vigas!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I8*100/(Datos_vigas!$B$8*J8*K8^2*Datos_vigas!$B$5)))*J8*K8*Datos_vigas!$B$5/Datos_vigas!$B$6,0.0033*J8*K8))))</f>
         <v/>
       </c>
       <c r="Q8" s="10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R8" s="10" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="S8" s="25">
         <f>F8/(J8*0.85*K8)</f>
@@ -11964,10 +11968,10 @@
         <v/>
       </c>
       <c r="U8" s="10" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="V8" s="10" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="W8" s="11">
         <f>IF(OR(M8="REVISAR",P8="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M8&lt;&gt;"REVISAR",P8&lt;&gt;"REVISAR",IF(ISNUMBER(M8),N8*PI()*(O8/10)^2/4&gt;=M8,TRUE),IF(ISNUMBER(P8),Q8*PI()*(R8/10)^2/4&gt;=P8,TRUE),IF(ISNUMBER(M8),M8&lt;=0.0163*J8*K8,TRUE),IF(ISNUMBER(P8),P8&lt;=0.0163*J8*K8,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F8&lt;=Datos_vigas!$B$9*(0.53*SQRT(Datos_vigas!$B$5)*J8*K8+2*PI()*(U8/10)^2/4*Datos_vigas!$B$6*K8/V8)),"NO VERIF. CORTE","VERIFICA")))</f>
@@ -11975,14 +11979,14 @@
       </c>
       <c r="X8" s="13" t="inlineStr">
         <is>
-          <t>Luz tomada como la longitud total rotulada. Si hay pilotes intermedios la luz de calculo es menor y los esfuerzos bajan mucho: corregir la columna LUZ. Relacion luz/altura alta. En una viga de fundacion enterrada la flecha no suele gobernar, por eso no se la incluye en la verificacion.</t>
+          <t>Longitud total 9.28 m. La luz de calculo es la mayor entre pilotes, deducida de la posicion de los pilotes dibujados en el plano. No se detectaron pilotes intermedios en este tramo. Verificar: puede estar apoyada directamente sobre el terreno, en cuyo caso no flexiona como viga de luz libre. Relacion luz/altura alta. En una viga de fundacion enterrada la flecha no suele gobernar, por eso no se la incluye en la verificacion.</t>
         </is>
       </c>
       <c r="Y8" s="12" t="n">
         <v>3.15</v>
       </c>
       <c r="Z8" s="12" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
@@ -11992,7 +11996,7 @@
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>5.33</v>
+        <v>3.8</v>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
@@ -12045,10 +12049,10 @@
         <v/>
       </c>
       <c r="Q9" s="10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R9" s="10" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="S9" s="25">
         <f>F9/(J9*0.85*K9)</f>
@@ -12070,7 +12074,7 @@
       </c>
       <c r="X9" s="13" t="inlineStr">
         <is>
-          <t>El ancho quedo cortado en el PDF: se adopta 20 cm. Confirmar si es 20 o 22.</t>
+          <t>El ancho quedo cortado en el PDF: se adopta 20 cm. Confirmar si es 20 o 22. Longitud total 5.33 m. La luz de calculo es la mayor entre pilotes, deducida de la posicion de los pilotes dibujados en el plano.</t>
         </is>
       </c>
       <c r="Y9" s="12" t="n">
@@ -12737,7 +12741,7 @@
         </is>
       </c>
       <c r="B18" s="8" t="n">
-        <v>3.5</v>
+        <v>2.04</v>
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
@@ -12817,7 +12821,11 @@
         <f>IF(OR(M18="REVISAR",P18="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M18&lt;&gt;"REVISAR",P18&lt;&gt;"REVISAR",IF(ISNUMBER(M18),N18*PI()*(O18/10)^2/4&gt;=M18,TRUE),IF(ISNUMBER(P18),Q18*PI()*(R18/10)^2/4&gt;=P18,TRUE),IF(ISNUMBER(M18),M18&lt;=0.0163*J18*K18,TRUE),IF(ISNUMBER(P18),P18&lt;=0.0163*J18*K18,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F18&lt;=Datos_vigas!$B$9*(0.53*SQRT(Datos_vigas!$B$5)*J18*K18+2*PI()*(U18/10)^2/4*Datos_vigas!$B$6*K18/V18)),"NO VERIF. CORTE","VERIFICA")))</f>
         <v/>
       </c>
-      <c r="X18" s="11" t="n"/>
+      <c r="X18" s="13" t="inlineStr">
+        <is>
+          <t>Longitud total 3.50 m. La luz de calculo es la mayor entre pilotes, deducida de la posicion de los pilotes dibujados en el plano.</t>
+        </is>
+      </c>
       <c r="Y18" s="12" t="n">
         <v>3.15</v>
       </c>
@@ -13014,7 +13022,7 @@
         </is>
       </c>
       <c r="B21" s="8" t="n">
-        <v>3.36</v>
+        <v>2.74</v>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
@@ -13090,7 +13098,11 @@
         <f>IF(OR(M21="REVISAR",P21="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M21&lt;&gt;"REVISAR",P21&lt;&gt;"REVISAR",IF(ISNUMBER(M21),N21*PI()*(O21/10)^2/4&gt;=M21,TRUE),IF(ISNUMBER(P21),Q21*PI()*(R21/10)^2/4&gt;=P21,TRUE),IF(ISNUMBER(M21),M21&lt;=0.0163*J21*K21,TRUE),IF(ISNUMBER(P21),P21&lt;=0.0163*J21*K21,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F21&lt;=Datos_vigas!$B$9*(0.53*SQRT(Datos_vigas!$B$5)*J21*K21+2*PI()*(U21/10)^2/4*Datos_vigas!$B$6*K21/V21)),"NO VERIF. CORTE","VERIFICA")))</f>
         <v/>
       </c>
-      <c r="X21" s="11" t="n"/>
+      <c r="X21" s="13" t="inlineStr">
+        <is>
+          <t>Longitud total 3.36 m. La luz de calculo es la mayor entre pilotes, deducida de la posicion de los pilotes dibujados en el plano.</t>
+        </is>
+      </c>
       <c r="Y21" s="12" t="n">
         <v>3.15</v>
       </c>
@@ -13196,7 +13208,7 @@
         </is>
       </c>
       <c r="B23" s="8" t="n">
-        <v>8.029999999999999</v>
+        <v>5.1</v>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
@@ -13239,20 +13251,20 @@
         <v/>
       </c>
       <c r="N23" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O23" s="10" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="P23" s="25">
         <f>IF(NOT(ISNUMBER(I23)),"---",IF(I23&lt;=0,"---",IF(I23*100/(Datos_vigas!$B$8*J23*K23^2*Datos_vigas!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I23*100/(Datos_vigas!$B$8*J23*K23^2*Datos_vigas!$B$5)))*J23*K23*Datos_vigas!$B$5/Datos_vigas!$B$6,0.0033*J23*K23))))</f>
         <v/>
       </c>
       <c r="Q23" s="10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R23" s="10" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="S23" s="25">
         <f>F23/(J23*0.85*K23)</f>
@@ -13274,7 +13286,7 @@
       </c>
       <c r="X23" s="13" t="inlineStr">
         <is>
-          <t>Luz tomada como la longitud total rotulada. Si hay pilotes intermedios la luz de calculo es menor y los esfuerzos bajan mucho: corregir la columna LUZ. Relacion luz/altura alta. En una viga de fundacion enterrada la flecha no suele gobernar, por eso no se la incluye en la verificacion.</t>
+          <t>Longitud total 8.03 m. La luz de calculo es la mayor entre pilotes, deducida de la posicion de los pilotes dibujados en el plano.</t>
         </is>
       </c>
       <c r="Y23" s="12" t="n">
@@ -13533,11 +13545,11 @@
         </is>
       </c>
       <c r="B27" s="8" t="n">
-        <v>8.75</v>
+        <v>3.09</v>
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>Continua</t>
+          <t>Simplemente apoyada</t>
         </is>
       </c>
       <c r="D27" s="24">
@@ -13576,20 +13588,24 @@
         <v/>
       </c>
       <c r="N27" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O27" s="10" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="P27" s="25">
         <f>IF(NOT(ISNUMBER(I27)),"---",IF(I27&lt;=0,"---",IF(I27*100/(Datos_vigas!$B$8*J27*K27^2*Datos_vigas!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I27*100/(Datos_vigas!$B$8*J27*K27^2*Datos_vigas!$B$5)))*J27*K27*Datos_vigas!$B$5/Datos_vigas!$B$6,0.0033*J27*K27))))</f>
         <v/>
       </c>
-      <c r="Q27" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="R27" s="10" t="n">
-        <v>16</v>
+      <c r="Q27" s="10" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="R27" s="10" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
       </c>
       <c r="S27" s="25">
         <f>F27/(J27*0.85*K27)</f>
@@ -13611,7 +13627,7 @@
       </c>
       <c r="X27" s="13" t="inlineStr">
         <is>
-          <t>Luz tomada como la longitud total rotulada. Si hay pilotes intermedios la luz de calculo es menor y los esfuerzos bajan mucho: corregir la columna LUZ. Relacion luz/altura alta. En una viga de fundacion enterrada la flecha no suele gobernar, por eso no se la incluye en la verificacion.</t>
+          <t>Longitud total 8.75 m. La luz de calculo es la mayor entre pilotes, deducida de la posicion de los pilotes dibujados en el plano.</t>
         </is>
       </c>
       <c r="Y27" s="12" t="n">
@@ -13723,7 +13739,7 @@
         </is>
       </c>
       <c r="B29" s="8" t="n">
-        <v>6.96</v>
+        <v>4.47</v>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
@@ -13769,17 +13785,17 @@
         <v>2</v>
       </c>
       <c r="O29" s="10" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="P29" s="25">
         <f>IF(NOT(ISNUMBER(I29)),"---",IF(I29&lt;=0,"---",IF(I29*100/(Datos_vigas!$B$8*J29*K29^2*Datos_vigas!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I29*100/(Datos_vigas!$B$8*J29*K29^2*Datos_vigas!$B$5)))*J29*K29*Datos_vigas!$B$5/Datos_vigas!$B$6,0.0033*J29*K29))))</f>
         <v/>
       </c>
       <c r="Q29" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R29" s="10" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="S29" s="25">
         <f>F29/(J29*0.85*K29)</f>
@@ -13801,7 +13817,7 @@
       </c>
       <c r="X29" s="13" t="inlineStr">
         <is>
-          <t>Luz tomada como la longitud total rotulada. Si hay pilotes intermedios la luz de calculo es menor y los esfuerzos bajan mucho: corregir la columna LUZ.</t>
+          <t>Longitud total 6.96 m. La luz de calculo es la mayor entre pilotes, deducida de la posicion de los pilotes dibujados en el plano.</t>
         </is>
       </c>
       <c r="Y29" s="12" t="n">
@@ -14004,7 +14020,7 @@
         </is>
       </c>
       <c r="B32" s="8" t="n">
-        <v>7.48</v>
+        <v>5.5</v>
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
@@ -14047,20 +14063,20 @@
         <v/>
       </c>
       <c r="N32" s="10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O32" s="10" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="P32" s="25">
         <f>IF(NOT(ISNUMBER(I32)),"---",IF(I32&lt;=0,"---",IF(I32*100/(Datos_vigas!$B$8*J32*K32^2*Datos_vigas!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I32*100/(Datos_vigas!$B$8*J32*K32^2*Datos_vigas!$B$5)))*J32*K32*Datos_vigas!$B$5/Datos_vigas!$B$6,0.0033*J32*K32))))</f>
         <v/>
       </c>
       <c r="Q32" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R32" s="10" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="S32" s="25">
         <f>F32/(J32*0.85*K32)</f>
@@ -14082,7 +14098,7 @@
       </c>
       <c r="X32" s="13" t="inlineStr">
         <is>
-          <t>Luz tomada como la longitud total rotulada. Si hay pilotes intermedios la luz de calculo es menor y los esfuerzos bajan mucho: corregir la columna LUZ. Relacion luz/altura alta. En una viga de fundacion enterrada la flecha no suele gobernar, por eso no se la incluye en la verificacion.</t>
+          <t>Longitud total 7.48 m. La luz de calculo es la mayor entre pilotes, deducida de la posicion de los pilotes dibujados en el plano.</t>
         </is>
       </c>
       <c r="Y32" s="12" t="n">
@@ -14190,7 +14206,7 @@
         </is>
       </c>
       <c r="B34" s="15" t="n">
-        <v>4.82</v>
+        <v>4.26</v>
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
@@ -14243,10 +14259,10 @@
         <v/>
       </c>
       <c r="Q34" s="17" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R34" s="17" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="S34" s="30">
         <f>F34/(J34*0.85*K34)</f>
@@ -14266,7 +14282,11 @@
         <f>IF(OR(M34="REVISAR",P34="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M34&lt;&gt;"REVISAR",P34&lt;&gt;"REVISAR",IF(ISNUMBER(M34),N34*PI()*(O34/10)^2/4&gt;=M34,TRUE),IF(ISNUMBER(P34),Q34*PI()*(R34/10)^2/4&gt;=P34,TRUE),IF(ISNUMBER(M34),M34&lt;=0.0163*J34*K34,TRUE),IF(ISNUMBER(P34),P34&lt;=0.0163*J34*K34,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F34&lt;=Datos_vigas!$B$9*(0.53*SQRT(Datos_vigas!$B$5)*J34*K34+2*PI()*(U34/10)^2/4*Datos_vigas!$B$6*K34/V34)),"NO VERIF. CORTE","VERIFICA")))</f>
         <v/>
       </c>
-      <c r="X34" s="18" t="n"/>
+      <c r="X34" s="20" t="inlineStr">
+        <is>
+          <t>Longitud total 4.82 m. La luz de calculo es la mayor entre pilotes, deducida de la posicion de los pilotes dibujados en el plano.</t>
+        </is>
+      </c>
       <c r="Y34" s="19" t="n">
         <v>3.15</v>
       </c>

</xml_diff>

<commit_message>
Agregar la planilla de pilotes y cabezales
Nueve cabezales relevados, cada uno asociado por geometria a la
columna que soporta. La cantidad de pilotes se deduce de la medida
del cabezal: 70x70 lleva uno, 129x70 y 144x70 llevan dos. La carga
admisible del pilote queda como dato editable con una estimacion de
12 t, a falta del estudio de suelos. El libro llega a quince hojas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -12,14 +12,16 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planilla losas" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planilla columnas" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vigas de fundacion" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos_vigas" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos_losas" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos_columnas" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memoria ilum. y vent." sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memoria vigas" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memoria losas" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memoria columnas" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fundacion (inventario)" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilotes y cabezales" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos_vigas" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos_losas" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos_columnas" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos_pilotes" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memoria ilum. y vent." sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memoria vigas" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memoria losas" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memoria columnas" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fundacion (inventario)" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Iluminacion y ventilacion'!$1:$3</definedName>
@@ -31,6 +33,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Planilla columnas'!$A$1:$N$16</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Vigas de fundacion'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'Vigas de fundacion'!$A$1:$X$34</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Pilotes y cabezales'!$1:$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -248,7 +251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -365,6 +368,7 @@
     <xf numFmtId="2" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -389,7 +393,6 @@
     <xf numFmtId="165" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -397,6 +400,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -3374,6 +3378,506 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="43" t="inlineStr">
+        <is>
+          <t>DATOS DE PARTIDA - PILOTES</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="45" t="inlineStr">
+        <is>
+          <t>PARAMETRO</t>
+        </is>
+      </c>
+      <c r="B3" s="46" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="C3" s="46" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="D3" s="45" t="inlineStr">
+        <is>
+          <t>origen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="47" t="inlineStr">
+        <is>
+          <t>Carga admisible por pilote</t>
+        </is>
+      </c>
+      <c r="B4" s="48" t="n">
+        <v>12</v>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>t</t>
+        </is>
+      </c>
+      <c r="D4" s="52" t="inlineStr">
+        <is>
+          <t>ESTIMADA. Falta el estudio de suelos: cambiar aca y recalcula todo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="47" t="inlineStr">
+        <is>
+          <t>Tension admisible del terreno</t>
+        </is>
+      </c>
+      <c r="B5" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>kg/cm2</t>
+        </is>
+      </c>
+      <c r="D5" s="52" t="inlineStr">
+        <is>
+          <t>Dato real, tomado del encabezado del calculo de bases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="47" t="inlineStr">
+        <is>
+          <t>Diametro del pilote</t>
+        </is>
+      </c>
+      <c r="B6" s="48" t="n">
+        <v>30</v>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>cm</t>
+        </is>
+      </c>
+      <c r="D6" s="52" t="inlineStr">
+        <is>
+          <t>Nota del plano: todos los pilotes son O30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="47" t="inlineStr">
+        <is>
+          <t>Profundidad</t>
+        </is>
+      </c>
+      <c r="B7" s="48" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D7" s="52" t="inlineStr">
+        <is>
+          <t>Nota del plano: h = -4,50 m desde la cota +-0,00 de vereda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="47" t="inlineStr">
+        <is>
+          <t>Coef. de mayoracion adoptado</t>
+        </is>
+      </c>
+      <c r="B8" s="48" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D8" s="52" t="inlineStr">
+        <is>
+          <t>Para pasar de carga mayorada a carga de servicio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n"/>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n"/>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="58" t="inlineStr">
+        <is>
+          <t>COMO SE ESTIMO LA CARGA ADMISIBLE</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="44" t="inlineStr">
+        <is>
+          <t>Pilote O30 de 4,50 m: area de punta 0,0707 m2, area lateral 4,24 m2.</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="44" t="inlineStr">
+        <is>
+          <t>Punta  0,0707 x 20 t/m2 = 1,4 t.</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="44" t="inlineStr">
+        <is>
+          <t>Friccion lateral  4,24 x adherencia:  1,5 t/m2 -&gt; 6,4 t   |   3,0 t/m2 -&gt; 12,7 t.</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="44" t="inlineStr">
+        <is>
+          <t>Total segun adherencia: entre 7,8 y 14,1 t. Se adopta 12 t como valor de trabajo.</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="44" t="inlineStr"/>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="42" t="inlineStr">
+        <is>
+          <t>LECTURA INVERSA, que es la util mientras no haya estudio de suelos:</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="44" t="inlineStr">
+        <is>
+          <t>con las cargas de esta planilla, para que el esquema funcione cada pilote</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="44" t="inlineStr">
+        <is>
+          <t>tiene que admitir del orden de 20 t. Si el estudio de suelos da menos,</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="44" t="inlineStr">
+        <is>
+          <t>faltan pilotes; si da mas, el diseno esta holgado.</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="44" t="inlineStr"/>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="44" t="inlineStr">
+        <is>
+          <t>La tension de 2 kg/cm2 que trae el calculo de bases es la del estrato</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="44" t="inlineStr">
+        <is>
+          <t>superficial, donde apoyaban las bases. Los pilotes llegan a -4,50 m y</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="44" t="inlineStr">
+        <is>
+          <t>trabajan sobre todo por friccion: son dos cosas distintas.</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n"/>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="96" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="59" t="inlineStr">
+        <is>
+          <t>MEMORIA - ILUMINACION Y VENTILACION</t>
+        </is>
+      </c>
+      <c r="B1" s="60" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="60" t="inlineStr"/>
+      <c r="B2" s="61" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="60" t="inlineStr">
+        <is>
+          <t>CRITERIO</t>
+        </is>
+      </c>
+      <c r="B3" s="60" t="inlineStr">
+        <is>
+          <t>Area de iluminacion requerida = superficie del local / 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="60" t="inlineStr"/>
+      <c r="B4" s="61" t="inlineStr">
+        <is>
+          <t>Area de ventilacion requerida = un tercio de la de iluminacion = superficie / 27</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="60" t="inlineStr"/>
+      <c r="B5" s="61" t="inlineStr">
+        <is>
+          <t>Area proyectada: la vidriada de la carpinteria para iluminacion, y la parte que</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="60" t="inlineStr"/>
+      <c r="B6" s="61" t="inlineStr">
+        <is>
+          <t>realmente abre para ventilacion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="60" t="inlineStr"/>
+      <c r="B7" s="61" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="60" t="inlineStr">
+        <is>
+          <t>RESULTADO</t>
+        </is>
+      </c>
+      <c r="B8" s="60" t="inlineStr">
+        <is>
+          <t>Los trece locales cumplen holgadamente iluminacion y ventilacion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="60" t="inlineStr"/>
+      <c r="B9" s="61" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="60" t="inlineStr">
+        <is>
+          <t>CORRECCION</t>
+        </is>
+      </c>
+      <c r="B10" s="60" t="inlineStr">
+        <is>
+          <t>Local 07, Hall / ingreso: la planilla original traia 0,66 y 0,22, que son los</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="60" t="inlineStr"/>
+      <c r="B11" s="61" t="inlineStr">
+        <is>
+          <t>valores del local 03 (Lavadero, 6,0 m2). Con sus 3,50 x 2,15 = 7,53 m2 corresponden</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="60" t="inlineStr"/>
+      <c r="B12" s="61" t="inlineStr">
+        <is>
+          <t>0,84 y 0,28. No cambia el resultado, pero el numero no cerraba con la superficie</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="60" t="inlineStr"/>
+      <c r="B13" s="61" t="inlineStr">
+        <is>
+          <t>declarada y un verificador lo puede observar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="60" t="inlineStr"/>
+      <c r="B14" s="61" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="60" t="inlineStr">
+        <is>
+          <t>A REVISAR</t>
+        </is>
+      </c>
+      <c r="B15" s="60" t="inlineStr">
+        <is>
+          <t>Local 14, Estar / Playroom: declara 5,00 m2 de ventilacion sobre 5,00 m2 de</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="60" t="inlineStr"/>
+      <c r="B16" s="61" t="inlineStr">
+        <is>
+          <t>iluminacion, es decir una carpinteria enteramente abrible. En los demas locales</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="60" t="inlineStr"/>
+      <c r="B17" s="61" t="inlineStr">
+        <is>
+          <t>la relacion es del 50 por ciento. Conviene verificar la carpinteria real.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="60" t="inlineStr"/>
+      <c r="B18" s="61" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="60" t="inlineStr"/>
+      <c r="B19" s="61" t="inlineStr">
+        <is>
+          <t>Local 02, Deposito: figura sin exigencia por no ser habitable. Son 11,8 m2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="60" t="inlineStr"/>
+      <c r="B20" s="61" t="inlineStr">
+        <is>
+          <t>cerrados: si se lo considera habitable hay que preverle conducto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="60" t="inlineStr"/>
+      <c r="B21" s="61" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="60" t="inlineStr">
+        <is>
+          <t>REDONDEOS</t>
+        </is>
+      </c>
+      <c r="B22" s="60" t="inlineStr">
+        <is>
+          <t>Diferencias menores que no afectan: local 03 da 5,95 m2 y figura 6,0;</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="60" t="inlineStr"/>
+      <c r="B23" s="61" t="inlineStr">
+        <is>
+          <t>local 09 da 12,25 y figura 12,3.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3382,552 +3886,552 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="58" t="inlineStr">
+      <c r="A1" s="59" t="inlineStr">
         <is>
           <t>MEMORIA DE CALCULO - VIGAS H°A°</t>
         </is>
       </c>
-      <c r="B1" s="59" t="inlineStr"/>
+      <c r="B1" s="60" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="59" t="inlineStr"/>
-      <c r="B2" s="60" t="inlineStr"/>
+      <c r="A2" s="60" t="inlineStr"/>
+      <c r="B2" s="61" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="59" t="inlineStr">
+      <c r="A3" s="60" t="inlineStr">
         <is>
           <t>NORMATIVA</t>
         </is>
       </c>
-      <c r="B3" s="59" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t>CIRSOC 201. Hormigon H-21 (f'c 210 kg/cm2). Acero 42/50 (fy 4200 kg/cm2).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="59" t="inlineStr">
+      <c r="A4" s="60" t="inlineStr">
         <is>
           <t>UNIDADES</t>
         </is>
       </c>
-      <c r="B4" s="59" t="inlineStr">
+      <c r="B4" s="60" t="inlineStr">
         <is>
           <t>Longitudes en m y cm. Cargas en kg/m. Momentos en kgm. Tensiones en kg/cm2.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="59" t="inlineStr">
+      <c r="A5" s="60" t="inlineStr">
         <is>
           <t>DIMENSIONES</t>
         </is>
       </c>
-      <c r="B5" s="59" t="inlineStr">
+      <c r="B5" s="60" t="inlineStr">
         <is>
           <t>b = ancho | h = altura util | d = altura total (igual criterio que la planilla de catedra).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="59" t="inlineStr"/>
-      <c r="B6" s="60" t="inlineStr"/>
+      <c r="A6" s="60" t="inlineStr"/>
+      <c r="B6" s="61" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="59" t="inlineStr">
+      <c r="A7" s="60" t="inlineStr">
         <is>
           <t>1. CARGAS</t>
         </is>
       </c>
-      <c r="B7" s="59" t="inlineStr"/>
+      <c r="B7" s="60" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="59" t="inlineStr">
+      <c r="A8" s="60" t="inlineStr">
         <is>
           <t>Entrepiso PA</t>
         </is>
       </c>
-      <c r="B8" s="60" t="inlineStr">
+      <c r="B8" s="61" t="inlineStr">
         <is>
           <t>Losa maciza 12 cm 300 + contrapiso 130 + carpeta 42 + piso 50 + cielorraso 20</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="59" t="inlineStr"/>
-      <c r="B9" s="60" t="inlineStr">
+      <c r="A9" s="60" t="inlineStr"/>
+      <c r="B9" s="61" t="inlineStr">
         <is>
           <t>g = 550 kg/m2       q = 200 kg/m2 (vivienda)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="59" t="inlineStr">
+      <c r="A10" s="60" t="inlineStr">
         <is>
           <t>Azotea</t>
         </is>
       </c>
-      <c r="B10" s="60" t="inlineStr">
+      <c r="B10" s="61" t="inlineStr">
         <is>
           <t>Losa 300 + contrapiso de pendiente 140 + carpeta 42 + aislacion y membrana 50 + cielorraso 20</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="59" t="inlineStr"/>
-      <c r="B11" s="60" t="inlineStr">
+      <c r="A11" s="60" t="inlineStr"/>
+      <c r="B11" s="61" t="inlineStr">
         <is>
           <t>g = 560 kg/m2       q = 100 kg/m2 (cubierta no accesible)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="59" t="inlineStr">
+      <c r="A12" s="60" t="inlineStr">
         <is>
           <t>Mamposteria</t>
         </is>
       </c>
-      <c r="B12" s="60" t="inlineStr">
+      <c r="B12" s="61" t="inlineStr">
         <is>
           <t>250 kg/m2. Altura 2,60 m en PA y 1,00 m de parapeto en azotea.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="59" t="inlineStr">
+      <c r="A13" s="60" t="inlineStr">
         <is>
           <t>Peso propio</t>
         </is>
       </c>
-      <c r="B13" s="60" t="inlineStr">
+      <c r="B13" s="61" t="inlineStr">
         <is>
           <t>2400 kg/m3 x b x d, viga por viga.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="59" t="inlineStr">
+      <c r="A14" s="60" t="inlineStr">
         <is>
           <t>Carga de calculo</t>
         </is>
       </c>
-      <c r="B14" s="60" t="inlineStr">
+      <c r="B14" s="61" t="inlineStr">
         <is>
           <t>p = 1,2 (g x B + peso propio + muro) + 1,6 (q x B)        B = ancho tributario</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="59" t="inlineStr"/>
-      <c r="B15" s="60" t="inlineStr"/>
+      <c r="A15" s="60" t="inlineStr"/>
+      <c r="B15" s="61" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="59" t="inlineStr">
+      <c r="A16" s="60" t="inlineStr">
         <is>
           <t>2. SOLICITACIONES</t>
         </is>
       </c>
-      <c r="B16" s="59" t="inlineStr">
+      <c r="B16" s="60" t="inlineStr">
         <is>
           <t>Coeficientes segun esquema (tabla en hoja Datos):</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="59" t="inlineStr"/>
-      <c r="B17" s="60" t="inlineStr">
+      <c r="A17" s="60" t="inlineStr"/>
+      <c r="B17" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  Simplemente apoyada   M = pL2/8                    R = 0,500 pL</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="59" t="inlineStr"/>
-      <c r="B18" s="60" t="inlineStr">
+      <c r="A18" s="60" t="inlineStr"/>
+      <c r="B18" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  Continua              M = pL2/14   Mapoyo = pL2/10  R = 0,575 pL</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="59" t="inlineStr"/>
-      <c r="B19" s="60" t="inlineStr">
+      <c r="A19" s="60" t="inlineStr"/>
+      <c r="B19" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  Empotrada-apoyada     M = 9pL2/128 Mapoyo = pL2/8   R = 0,625 pL</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="59" t="inlineStr"/>
-      <c r="B20" s="60" t="inlineStr">
+      <c r="A20" s="60" t="inlineStr"/>
+      <c r="B20" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  Biempotrada           M = pL2/24   Mapoyo = pL2/12  R = 0,500 pL</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="59" t="inlineStr"/>
-      <c r="B21" s="60" t="inlineStr">
+      <c r="A21" s="60" t="inlineStr"/>
+      <c r="B21" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  Voladizo                           Mapoyo = pL2/2   R = 1,000 pL</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="59" t="inlineStr"/>
-      <c r="B22" s="60" t="inlineStr"/>
+      <c r="A22" s="60" t="inlineStr"/>
+      <c r="B22" s="61" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="59" t="inlineStr">
+      <c r="A23" s="60" t="inlineStr">
         <is>
           <t>3. FLEXION</t>
         </is>
       </c>
-      <c r="B23" s="59" t="inlineStr">
+      <c r="B23" s="60" t="inlineStr">
         <is>
           <t>k = M / (phi b h2 f'c)      w = 1 - RAIZ(1 - 2k)      As = w b h f'c / fy</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="59" t="inlineStr"/>
-      <c r="B24" s="60" t="inlineStr">
+      <c r="A24" s="60" t="inlineStr"/>
+      <c r="B24" s="61" t="inlineStr">
         <is>
           <t>As min = 0,0033 b h       As max = 0,0163 b h (0,75 de la cuantia balanceada)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="59" t="inlineStr"/>
-      <c r="B25" s="60" t="inlineStr">
+      <c r="A25" s="60" t="inlineStr"/>
+      <c r="B25" s="61" t="inlineStr">
         <is>
           <t>Si la armadura no entra en una capa se disponen dos y el recubrimiento pasa a 6 cm.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="59" t="inlineStr"/>
-      <c r="B26" s="60" t="inlineStr"/>
+      <c r="A26" s="60" t="inlineStr"/>
+      <c r="B26" s="61" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="59" t="inlineStr">
+      <c r="A27" s="60" t="inlineStr">
         <is>
           <t>4. CORTE</t>
         </is>
       </c>
-      <c r="B27" s="59" t="inlineStr">
+      <c r="B27" s="60" t="inlineStr">
         <is>
           <t>T = R / (b x 0,85 h)       tension tangencial en el apoyo</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="59" t="inlineStr"/>
-      <c r="B28" s="60" t="inlineStr">
+      <c r="A28" s="60" t="inlineStr"/>
+      <c r="B28" s="61" t="inlineStr">
         <is>
           <t>Vc = 0,53 RAIZ(f'c) b h        phi Vn = 0,75 (Vc + Av fy h / s)  &gt;=  R</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="59" t="inlineStr"/>
-      <c r="B29" s="60" t="inlineStr">
+      <c r="A29" s="60" t="inlineStr"/>
+      <c r="B29" s="61" t="inlineStr">
         <is>
           <t>Av = 2 ramas. Se aumenta el diametro antes que cerrar la separacion por debajo de 10 cm.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="59" t="inlineStr"/>
-      <c r="B30" s="60" t="inlineStr"/>
+      <c r="A30" s="60" t="inlineStr"/>
+      <c r="B30" s="61" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="59" t="inlineStr">
+      <c r="A31" s="60" t="inlineStr">
         <is>
           <t>5. FLECHA</t>
         </is>
       </c>
-      <c r="B31" s="59" t="inlineStr">
+      <c r="B31" s="60" t="inlineStr">
         <is>
           <t>Altura minima: simplemente apoyada L/16, un extremo continuo L/18,5,</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="59" t="inlineStr"/>
-      <c r="B32" s="60" t="inlineStr">
+      <c r="A32" s="60" t="inlineStr"/>
+      <c r="B32" s="61" t="inlineStr">
         <is>
           <t>ambos extremos continuos L/21, voladizo L/8.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="59" t="inlineStr"/>
-      <c r="B33" s="60" t="inlineStr"/>
+      <c r="A33" s="60" t="inlineStr"/>
+      <c r="B33" s="61" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="59" t="inlineStr">
+      <c r="A34" s="60" t="inlineStr">
         <is>
           <t>6. VIGAS INVERTIDAS</t>
         </is>
       </c>
-      <c r="B34" s="59" t="inlineStr">
+      <c r="B34" s="60" t="inlineStr">
         <is>
           <t>Las vigas de BORDE son invertidas: sobresalen 70 cm por encima del fondo de</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="59" t="inlineStr"/>
-      <c r="B35" s="60" t="inlineStr">
+      <c r="A35" s="60" t="inlineStr"/>
+      <c r="B35" s="61" t="inlineStr">
         <is>
           <t>losa (cotas N.F.L +3,50 / N.S.V +4,20 y N.F.L +6,80 / N.S.V +7,50 del plano).</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="59" t="inlineStr"/>
-      <c r="B36" s="60" t="inlineStr">
+      <c r="A36" s="60" t="inlineStr"/>
+      <c r="B36" s="61" t="inlineStr">
         <is>
           <t>Son VI 01a, VI 01b, VI 07a, VI 07b, VI 07c, VI 11a, VI 11b, VI 11c, VI 15a y VI 15b,</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="59" t="inlineStr"/>
-      <c r="B37" s="60" t="inlineStr">
+      <c r="A37" s="60" t="inlineStr"/>
+      <c r="B37" s="61" t="inlineStr">
         <is>
           <t>identificadas por coincidir su eje con el contorno del edificio.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="59" t="inlineStr"/>
-      <c r="B38" s="60" t="inlineStr">
+      <c r="A38" s="60" t="inlineStr"/>
+      <c r="B38" s="61" t="inlineStr">
         <is>
           <t>Esto define donde la losa aporta ala comprimida:</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="59" t="inlineStr"/>
-      <c r="B39" s="60" t="inlineStr">
+      <c r="A39" s="60" t="inlineStr"/>
+      <c r="B39" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  viga COLGANTE  -&gt; la losa esta arriba  -&gt; ala util en el TRAMO (momento positivo)</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="59" t="inlineStr"/>
-      <c r="B40" s="60" t="inlineStr">
+      <c r="A40" s="60" t="inlineStr"/>
+      <c r="B40" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  viga INVERTIDA -&gt; la losa esta abajo   -&gt; ala util en el APOYO (momento negativo)</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="59" t="inlineStr"/>
-      <c r="B41" s="60" t="inlineStr">
+      <c r="A41" s="60" t="inlineStr"/>
+      <c r="B41" s="61" t="inlineStr">
         <is>
           <t>En la zona con ala se adopta b efectivo = min(L/4 ; b + 16 hf); en la otra, la</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="59" t="inlineStr"/>
-      <c r="B42" s="60" t="inlineStr">
+      <c r="A42" s="60" t="inlineStr"/>
+      <c r="B42" s="61" t="inlineStr">
         <is>
           <t>seccion es rectangular de ancho b. Las columnas b ef tramo y b ef apoyo lo muestran.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="59" t="inlineStr"/>
-      <c r="B43" s="60" t="inlineStr">
+      <c r="A43" s="60" t="inlineStr"/>
+      <c r="B43" s="61" t="inlineStr">
         <is>
           <t>PENDIENTE: una viga invertida de borde recibe la reaccion de la losa excentrica</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="59" t="inlineStr"/>
-      <c r="B44" s="60" t="inlineStr">
+      <c r="A44" s="60" t="inlineStr"/>
+      <c r="B44" s="61" t="inlineStr">
         <is>
           <t>respecto de su eje y queda sometida a TORSION. Esta planilla no la verifica.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="59" t="inlineStr"/>
-      <c r="B45" s="60" t="inlineStr"/>
+      <c r="A45" s="60" t="inlineStr"/>
+      <c r="B45" s="61" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="59" t="inlineStr">
+      <c r="A46" s="60" t="inlineStr">
         <is>
           <t>7. RESULTADO</t>
         </is>
       </c>
-      <c r="B46" s="59" t="inlineStr">
+      <c r="B46" s="60" t="inlineStr">
         <is>
           <t>30 vigas: 21 del entrepiso PA y 9 de la losa de techo. 28 verifican.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="59" t="inlineStr"/>
-      <c r="B47" s="60" t="inlineStr">
+      <c r="A47" s="60" t="inlineStr"/>
+      <c r="B47" s="61" t="inlineStr">
         <is>
           <t>VI 02 (15x60, 9,88 m): recibe L02 y L03, B = 2,88 m. La armadura de apoyo</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="59" t="inlineStr"/>
-      <c r="B48" s="60" t="inlineStr">
+      <c r="A48" s="60" t="inlineStr"/>
+      <c r="B48" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">   necesaria ronda los 25 cm2 y supera la cuantia maxima. Los apoyos estan</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="59" t="inlineStr"/>
-      <c r="B49" s="60" t="inlineStr">
+      <c r="A49" s="60" t="inlineStr"/>
+      <c r="B49" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">   confirmados en obra: tabique T07 perpendicular arriba y COL 02 abajo, sin apoyo</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="59" t="inlineStr"/>
-      <c r="B50" s="60" t="inlineStr">
+      <c r="A50" s="60" t="inlineStr"/>
+      <c r="B50" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">   intermedio. Para esta carga la seccion necesaria es 15x75.</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="59" t="inlineStr"/>
-      <c r="B51" s="60" t="inlineStr">
+      <c r="A51" s="60" t="inlineStr"/>
+      <c r="B51" s="61" t="inlineStr">
         <is>
           <t>VCH 03a (40x13, 3,83 m). Recibe L03, B = 2,08 m, y no</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="59" t="inlineStr"/>
-      <c r="B52" s="60" t="inlineStr">
+      <c r="A52" s="60" t="inlineStr"/>
+      <c r="B52" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">   verifica: haria falta mas espesor. Tampoco verifica con B = 0,60 m, asi</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="59" t="inlineStr"/>
-      <c r="B53" s="60" t="inlineStr">
+      <c r="A53" s="60" t="inlineStr"/>
+      <c r="B53" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">   que el problema no es la hipotesis de carga sino la relacion luz/espesor. Una viga</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="59" t="inlineStr"/>
-      <c r="B54" s="60" t="inlineStr">
+      <c r="A54" s="60" t="inlineStr"/>
+      <c r="B54" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">   chata del mismo espesor que la losa no puede ser apoyo lineal de un pano de 4,15 m.</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="59" t="inlineStr"/>
-      <c r="B55" s="60" t="inlineStr">
+      <c r="A55" s="60" t="inlineStr"/>
+      <c r="B55" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">   Revisar si tiene un muro debajo que acorte su luz libre.</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="59" t="inlineStr"/>
-      <c r="B56" s="60" t="inlineStr">
+      <c r="A56" s="60" t="inlineStr"/>
+      <c r="B56" s="61" t="inlineStr">
         <is>
           <t>VCH 03a (40x13, 3,71 m): excede la cuantia maxima y no llega a la altura minima por</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="59" t="inlineStr"/>
-      <c r="B57" s="60" t="inlineStr">
+      <c r="A57" s="60" t="inlineStr"/>
+      <c r="B57" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">   flecha. Revisar el ancho tributario: si solo recibe el muro y no losa, baja mucho.</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="59" t="inlineStr"/>
-      <c r="B58" s="60" t="inlineStr"/>
+      <c r="A58" s="60" t="inlineStr"/>
+      <c r="B58" s="61" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="59" t="inlineStr">
+      <c r="A59" s="60" t="inlineStr">
         <is>
           <t>8. ALCANCE</t>
         </is>
       </c>
-      <c r="B59" s="60" t="inlineStr">
+      <c r="B59" s="61" t="inlineStr">
         <is>
           <t>No se incluyen las 31 vigas de fundacion (VF01 a VF18c): su calculo depende de las</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="59" t="inlineStr"/>
-      <c r="B60" s="60" t="inlineStr">
+      <c r="A60" s="60" t="inlineStr"/>
+      <c r="B60" s="61" t="inlineStr">
         <is>
           <t>cargas que bajan por las columnas y corresponde hacerlo despues. Tampoco losas ni columnas.</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="59" t="inlineStr"/>
-      <c r="B61" s="60" t="inlineStr"/>
+      <c r="A61" s="60" t="inlineStr"/>
+      <c r="B61" s="61" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="59" t="inlineStr">
+      <c r="A62" s="60" t="inlineStr">
         <is>
           <t>LIMITACIONES</t>
         </is>
       </c>
-      <c r="B62" s="59" t="inlineStr">
+      <c r="B62" s="60" t="inlineStr">
         <is>
           <t>El ancho tributario B esta relevado solo en</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="59" t="inlineStr"/>
-      <c r="B63" s="60" t="inlineStr">
+      <c r="A63" s="60" t="inlineStr"/>
+      <c r="B63" s="61" t="inlineStr">
         <is>
           <t>VI 02 (0,80 m) y VCH 03a (2,08 m). En las demas sigue adoptado en 2,00 m, a falta</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="59" t="inlineStr"/>
-      <c r="B64" s="60" t="inlineStr">
+      <c r="A64" s="60" t="inlineStr"/>
+      <c r="B64" s="61" t="inlineStr">
         <is>
           <t>hipotesis mas influyente del calculo: ajustarla viga por viga en la columna B trib.</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="59" t="inlineStr"/>
-      <c r="B65" s="60" t="inlineStr">
+      <c r="A65" s="60" t="inlineStr"/>
+      <c r="B65" s="61" t="inlineStr">
         <is>
           <t>El esquema se asigno por criterio: continua si integra una serie a-b-c o si supera 5,5 m.</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="59" t="inlineStr"/>
-      <c r="B66" s="60" t="inlineStr">
+      <c r="A66" s="60" t="inlineStr"/>
+      <c r="B66" s="61" t="inlineStr">
         <is>
           <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
         </is>
@@ -3938,7 +4442,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3952,368 +4456,368 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="58" t="inlineStr">
+      <c r="A1" s="59" t="inlineStr">
         <is>
           <t>MEMORIA DE CALCULO - LOSAS</t>
         </is>
       </c>
-      <c r="B1" s="59" t="inlineStr"/>
+      <c r="B1" s="60" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="59" t="inlineStr"/>
-      <c r="B2" s="60" t="inlineStr"/>
+      <c r="A2" s="60" t="inlineStr"/>
+      <c r="B2" s="61" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="59" t="inlineStr">
+      <c r="A3" s="60" t="inlineStr">
         <is>
           <t>METODO</t>
         </is>
       </c>
-      <c r="B3" s="59" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t>Tensiones admisibles, igual criterio que la planilla modelo de la catedra.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="59" t="inlineStr"/>
-      <c r="B4" s="60" t="inlineStr">
+      <c r="A4" s="60" t="inlineStr"/>
+      <c r="B4" s="61" t="inlineStr">
         <is>
           <t>Se verifico contra la fila de ejemplo: momentos y reacciones coinciden exactamente.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="59" t="inlineStr">
+      <c r="A5" s="60" t="inlineStr">
         <is>
           <t>MATERIALES</t>
         </is>
       </c>
-      <c r="B5" s="59" t="inlineStr">
+      <c r="B5" s="60" t="inlineStr">
         <is>
           <t>H-21 (f'c 210 kg/cm2). Acero 42/50 (fy 4200). Tension admisible 2400 kg/cm2.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="59" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>DIMENSIONES</t>
         </is>
       </c>
-      <c r="B6" s="59" t="inlineStr">
+      <c r="B6" s="60" t="inlineStr">
         <is>
           <t>h = altura util | d = espesor total. Recubrimiento 1,5 cm.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="59" t="inlineStr"/>
-      <c r="B7" s="60" t="inlineStr"/>
+      <c r="A7" s="60" t="inlineStr"/>
+      <c r="B7" s="61" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="59" t="inlineStr">
+      <c r="A8" s="60" t="inlineStr">
         <is>
           <t>1. CARGAS</t>
         </is>
       </c>
-      <c r="B8" s="59" t="inlineStr">
+      <c r="B8" s="60" t="inlineStr">
         <is>
           <t>p = peso propio + terminaciones + q      (cargas de servicio, sin mayorar)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="59" t="inlineStr"/>
-      <c r="B9" s="60" t="inlineStr">
+      <c r="A9" s="60" t="inlineStr"/>
+      <c r="B9" s="61" t="inlineStr">
         <is>
           <t>Peso propio = 2400 x d / 100, calculado con el espesor propio de cada losa.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="59" t="inlineStr">
+      <c r="A10" s="60" t="inlineStr">
         <is>
           <t>S/PB</t>
         </is>
       </c>
-      <c r="B10" s="60" t="inlineStr">
+      <c r="B10" s="61" t="inlineStr">
         <is>
           <t>Terminaciones 242 kg/m2 (contrapiso 130 + carpeta 42 + piso 50 + cielorraso 20)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="59" t="inlineStr"/>
-      <c r="B11" s="60" t="inlineStr">
+      <c r="A11" s="60" t="inlineStr"/>
+      <c r="B11" s="61" t="inlineStr">
         <is>
           <t>q = 200 kg/m2 (vivienda)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="59" t="inlineStr">
+      <c r="A12" s="60" t="inlineStr">
         <is>
           <t>S/PA</t>
         </is>
       </c>
-      <c r="B12" s="60" t="inlineStr">
+      <c r="B12" s="61" t="inlineStr">
         <is>
           <t>Terminaciones 252 kg/m2 (contrapiso pendiente 140 + carpeta 42 + aislacion 50 +</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="59" t="inlineStr"/>
-      <c r="B13" s="60" t="inlineStr">
+      <c r="A13" s="60" t="inlineStr"/>
+      <c r="B13" s="61" t="inlineStr">
         <is>
           <t>cielorraso 20).  q = 100 kg/m2 (azotea no accesible)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="59" t="inlineStr"/>
-      <c r="B14" s="60" t="inlineStr"/>
+      <c r="A14" s="60" t="inlineStr"/>
+      <c r="B14" s="61" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="59" t="inlineStr">
+      <c r="A15" s="60" t="inlineStr">
         <is>
           <t>2. SOLICITACIONES</t>
         </is>
       </c>
-      <c r="B15" s="59" t="inlineStr">
+      <c r="B15" s="60" t="inlineStr">
         <is>
           <t>M = coeficiente x p x L2, segun el grado de empotramiento:</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="59" t="inlineStr"/>
-      <c r="B16" s="60" t="inlineStr">
+      <c r="A16" s="60" t="inlineStr"/>
+      <c r="B16" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  1/8 simplemente apoyada    1/10 y 1/14 continua    1/12 biempotrada    1/2 voladizo</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="59" t="inlineStr"/>
-      <c r="B17" s="60" t="inlineStr">
+      <c r="A17" s="60" t="inlineStr"/>
+      <c r="B17" s="61" t="inlineStr">
         <is>
           <t>R = coeficiente x p x L. En voladizo Rx = p x L y Ry no corresponde.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="59" t="inlineStr"/>
-      <c r="B18" s="60" t="inlineStr"/>
+      <c r="A18" s="60" t="inlineStr"/>
+      <c r="B18" s="61" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="59" t="inlineStr">
+      <c r="A19" s="60" t="inlineStr">
         <is>
           <t>3. ARMADURA</t>
         </is>
       </c>
-      <c r="B19" s="59" t="inlineStr">
+      <c r="B19" s="60" t="inlineStr">
         <is>
           <t>As = M x 100 / (2400 x 0,9 x h)        [cm2/m]</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="59" t="inlineStr"/>
-      <c r="B20" s="60" t="inlineStr">
+      <c r="A20" s="60" t="inlineStr"/>
+      <c r="B20" s="61" t="inlineStr">
         <is>
           <t>separacion = 100 x area de la barra / As, redondeada, con maximo 20 cm</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="59" t="inlineStr"/>
-      <c r="B21" s="60" t="inlineStr">
+      <c r="A21" s="60" t="inlineStr"/>
+      <c r="B21" s="61" t="inlineStr">
         <is>
           <t>Armadura de reparticion = As / 5, con un minimo de 0,30 cm2/m</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="59" t="inlineStr"/>
-      <c r="B22" s="60" t="inlineStr"/>
+      <c r="A22" s="60" t="inlineStr"/>
+      <c r="B22" s="61" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="59" t="inlineStr">
+      <c r="A23" s="60" t="inlineStr">
         <is>
           <t>4. ESPESORES</t>
         </is>
       </c>
-      <c r="B23" s="59" t="inlineStr">
+      <c r="B23" s="60" t="inlineStr">
         <is>
           <t>Los espesores d se leyeron del plano: estan escritos debajo del rotulo de cada losa.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="59" t="inlineStr"/>
-      <c r="B24" s="60" t="inlineStr">
+      <c r="A24" s="60" t="inlineStr"/>
+      <c r="B24" s="61" t="inlineStr">
         <is>
           <t>S/PB:  L01 11 | L02 9 | L03 13 | L04 11 | L05 11 | L06 8 | L07 12 | L08 10</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="59" t="inlineStr"/>
-      <c r="B25" s="60" t="inlineStr">
+      <c r="A25" s="60" t="inlineStr"/>
+      <c r="B25" s="61" t="inlineStr">
         <is>
           <t>S/PA:  L09 13 | L10 12</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="59" t="inlineStr"/>
-      <c r="B26" s="60" t="inlineStr"/>
+      <c r="A26" s="60" t="inlineStr"/>
+      <c r="B26" s="61" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="59" t="inlineStr">
+      <c r="A27" s="60" t="inlineStr">
         <is>
           <t>5. LUCES</t>
         </is>
       </c>
-      <c r="B27" s="59" t="inlineStr">
+      <c r="B27" s="60" t="inlineStr">
         <is>
           <t>Relevadas en obra y aportadas por el proyectista. Dos losas son voladizo</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="59" t="inlineStr"/>
-      <c r="B28" s="60" t="inlineStr">
+      <c r="A28" s="60" t="inlineStr"/>
+      <c r="B28" s="61" t="inlineStr">
         <is>
           <t>(L02 de 0,80 m y L08 de 0,75 m) y se calculan con M = p L2 / 2.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="59" t="inlineStr"/>
-      <c r="B29" s="60" t="inlineStr"/>
+      <c r="A29" s="60" t="inlineStr"/>
+      <c r="B29" s="61" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="59" t="inlineStr">
+      <c r="A30" s="60" t="inlineStr">
         <is>
           <t>6. LOSAS CRUZADAS</t>
         </is>
       </c>
-      <c r="B30" s="60" t="inlineStr">
+      <c r="B30" s="61" t="inlineStr">
         <is>
           <t>L07 (4,85 x 5,60) y L10 (4,85 x 6,00) apoyan en los cuatro bordes y su relacion</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="59" t="inlineStr"/>
-      <c r="B31" s="60" t="inlineStr">
+      <c r="A31" s="60" t="inlineStr"/>
+      <c r="B31" s="61" t="inlineStr">
         <is>
           <t>de lados es menor que 2, por lo que trabajan en las dos direcciones.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="59" t="inlineStr"/>
-      <c r="B32" s="60" t="inlineStr">
+      <c r="A32" s="60" t="inlineStr"/>
+      <c r="B32" s="61" t="inlineStr">
         <is>
           <t>Se reparte la carga por el metodo de Marcus:   kx = ly4 / (lx4 + ly4)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="59" t="inlineStr"/>
-      <c r="B33" s="60" t="inlineStr">
+      <c r="A33" s="60" t="inlineStr"/>
+      <c r="B33" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  L07: ly/lx = 1,15  -&gt;  64% en la direccion corta, 36% en la larga</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="59" t="inlineStr"/>
-      <c r="B34" s="60" t="inlineStr">
+      <c r="A34" s="60" t="inlineStr"/>
+      <c r="B34" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  L10: ly/lx = 1,24  -&gt;  70% en la direccion corta, 30% en la larga</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="59" t="inlineStr"/>
-      <c r="B35" s="60" t="inlineStr">
+      <c r="A35" s="60" t="inlineStr"/>
+      <c r="B35" s="61" t="inlineStr">
         <is>
           <t>Cada una ocupa dos renglones, uno por direccion, con la fraccion de carga que</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="59" t="inlineStr"/>
-      <c r="B36" s="60" t="inlineStr">
+      <c r="A36" s="60" t="inlineStr"/>
+      <c r="B36" s="61" t="inlineStr">
         <is>
           <t>le toca ya aplicada en la columna CARGAS. Las dos armaduras se cruzan en obra:</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="59" t="inlineStr"/>
-      <c r="B37" s="60" t="inlineStr">
+      <c r="A37" s="60" t="inlineStr"/>
+      <c r="B37" s="61" t="inlineStr">
         <is>
           <t>la de la direccion corta va abajo, la de la larga arriba de aquella.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="59" t="inlineStr"/>
-      <c r="B38" s="60" t="inlineStr">
+      <c r="A38" s="60" t="inlineStr"/>
+      <c r="B38" s="61" t="inlineStr">
         <is>
           <t>La columna auxiliar luz transv. es la que dispara el reparto: si se borra, la</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="59" t="inlineStr"/>
-      <c r="B39" s="60" t="inlineStr">
+      <c r="A39" s="60" t="inlineStr"/>
+      <c r="B39" s="61" t="inlineStr">
         <is>
           <t>fila vuelve a calcularse como losa armada en una direccion.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="59" t="inlineStr"/>
-      <c r="B40" s="60" t="inlineStr"/>
+      <c r="A40" s="60" t="inlineStr"/>
+      <c r="B40" s="61" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="59" t="inlineStr">
+      <c r="A41" s="60" t="inlineStr">
         <is>
           <t>LIMITACIONES</t>
         </is>
       </c>
-      <c r="B41" s="59" t="inlineStr">
+      <c r="B41" s="60" t="inlineStr">
         <is>
           <t>El grado de empotramiento esta cargado en 1/8 salvo los dos voladizos (1/2). Si</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="59" t="inlineStr"/>
-      <c r="B42" s="60" t="inlineStr">
+      <c r="A42" s="60" t="inlineStr"/>
+      <c r="B42" s="61" t="inlineStr">
         <is>
           <t>alguna losa es continua sobre una viga corresponde 1/10 o 1/14: corregir en la columna.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="59" t="inlineStr"/>
-      <c r="B43" s="60" t="inlineStr">
+      <c r="A43" s="60" t="inlineStr"/>
+      <c r="B43" s="61" t="inlineStr">
         <is>
           <t>El diagrama de cargas es una imagen fija: si cambias el grado, cambialo a mano.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="59" t="inlineStr"/>
-      <c r="B44" s="60" t="inlineStr">
+      <c r="A44" s="60" t="inlineStr"/>
+      <c r="B44" s="61" t="inlineStr">
         <is>
           <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
         </is>
@@ -4324,7 +4828,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4338,368 +4842,368 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="58" t="inlineStr">
+      <c r="A1" s="59" t="inlineStr">
         <is>
           <t>MEMORIA DE CALCULO - COLUMNAS</t>
         </is>
       </c>
-      <c r="B1" s="59" t="inlineStr"/>
+      <c r="B1" s="60" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="59" t="inlineStr"/>
-      <c r="B2" s="60" t="inlineStr"/>
+      <c r="A2" s="60" t="inlineStr"/>
+      <c r="B2" s="61" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="59" t="inlineStr">
+      <c r="A3" s="60" t="inlineStr">
         <is>
           <t>MATERIALES</t>
         </is>
       </c>
-      <c r="B3" s="59" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t>H-21 (f'c 210 kg/cm2). Acero 42/50 (fy 4200). phi compresion 0,65.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="59" t="inlineStr"/>
-      <c r="B4" s="60" t="inlineStr"/>
+      <c r="A4" s="60" t="inlineStr"/>
+      <c r="B4" s="61" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="59" t="inlineStr">
+      <c r="A5" s="60" t="inlineStr">
         <is>
           <t>1. RELEVAMIENTO</t>
         </is>
       </c>
-      <c r="B5" s="59" t="inlineStr">
+      <c r="B5" s="60" t="inlineStr">
         <is>
           <t>Las columnas se identificaron en el plano cruzando el rotulo COL con un rectangulo</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="59" t="inlineStr"/>
-      <c r="B6" s="60" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr"/>
+      <c r="B6" s="61" t="inlineStr">
         <is>
           <t>de la misma seccion a menos de 26 pt. Resultaron 9 en PB y 4 en PA.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="59" t="inlineStr"/>
-      <c r="B7" s="60" t="inlineStr">
+      <c r="A7" s="60" t="inlineStr"/>
+      <c r="B7" s="61" t="inlineStr">
         <is>
           <t>Las 4 de PA caen exactamente sobre C6, C7, C8 y C9 de PB, y ademas tienen la misma</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="59" t="inlineStr"/>
-      <c r="B8" s="60" t="inlineStr">
+      <c r="A8" s="60" t="inlineStr"/>
+      <c r="B8" s="61" t="inlineStr">
         <is>
           <t>seccion, lo que confirma que la correspondencia entre plantas es correcta.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="59" t="inlineStr"/>
-      <c r="B9" s="60" t="inlineStr">
+      <c r="A9" s="60" t="inlineStr"/>
+      <c r="B9" s="61" t="inlineStr">
         <is>
           <t>La planilla modelo de la catedra tiene 10 columnas en PB: puede faltar una que no</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="59" t="inlineStr"/>
-      <c r="B10" s="60" t="inlineStr">
+      <c r="A10" s="60" t="inlineStr"/>
+      <c r="B10" s="61" t="inlineStr">
         <is>
           <t>haya podido resolverse por rotulo. Conviene contarlas en el plano.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="59" t="inlineStr"/>
-      <c r="B11" s="60" t="inlineStr"/>
+      <c r="A11" s="60" t="inlineStr"/>
+      <c r="B11" s="61" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="59" t="inlineStr">
+      <c r="A12" s="60" t="inlineStr">
         <is>
           <t>2. ALTURAS</t>
         </is>
       </c>
-      <c r="B12" s="59" t="inlineStr">
+      <c r="B12" s="60" t="inlineStr">
         <is>
           <t>PB 3,15 m y PA 3,22 m, los mismos valores de la planilla de la catedra, coherentes</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="59" t="inlineStr"/>
-      <c r="B13" s="60" t="inlineStr">
+      <c r="A13" s="60" t="inlineStr"/>
+      <c r="B13" s="61" t="inlineStr">
         <is>
           <t>con los niveles del plano (N.F.L +3,50 del entrepiso y +6,80 del techo).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="59" t="inlineStr"/>
-      <c r="B14" s="60" t="inlineStr"/>
+      <c r="A14" s="60" t="inlineStr"/>
+      <c r="B14" s="61" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="59" t="inlineStr">
+      <c r="A15" s="60" t="inlineStr">
         <is>
           <t>3. ARMADURA</t>
         </is>
       </c>
-      <c r="B15" s="59" t="inlineStr">
+      <c r="B15" s="60" t="inlineStr">
         <is>
           <t>As = 0,008 x area (cuantia minima, el mismo criterio de la planilla modelo).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="59" t="inlineStr"/>
-      <c r="B16" s="60" t="inlineStr">
+      <c r="A16" s="60" t="inlineStr"/>
+      <c r="B16" s="61" t="inlineStr">
         <is>
           <t>Se adoptan 4 barras del 12 en todas: 4,52 cm2, que cubre la minima en toda seccion.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="59" t="inlineStr"/>
-      <c r="B17" s="60" t="inlineStr">
+      <c r="A17" s="60" t="inlineStr"/>
+      <c r="B17" s="61" t="inlineStr">
         <is>
           <t>Separacion de estribos = min(12 x diam. long. ; 48 x diam. estribo ; lado menor),</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="59" t="inlineStr"/>
-      <c r="B18" s="60" t="inlineStr">
+      <c r="A18" s="60" t="inlineStr"/>
+      <c r="B18" s="61" t="inlineStr">
         <is>
           <t>redondeada hacia abajo a multiplo de 5. Para 4d12 con estribo d6 da 10 cm.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="59" t="inlineStr"/>
-      <c r="B19" s="60" t="inlineStr">
+      <c r="A19" s="60" t="inlineStr"/>
+      <c r="B19" s="61" t="inlineStr">
         <is>
           <t>La planilla de la catedra adopta 20 cm: ese valor supera el limite reglamentario.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="59" t="inlineStr"/>
-      <c r="B20" s="60" t="inlineStr"/>
+      <c r="A20" s="60" t="inlineStr"/>
+      <c r="B20" s="61" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="59" t="inlineStr">
+      <c r="A21" s="60" t="inlineStr">
         <is>
           <t>4. CAPACIDAD</t>
         </is>
       </c>
-      <c r="B21" s="59" t="inlineStr">
+      <c r="B21" s="60" t="inlineStr">
         <is>
           <t>phi Pn = 0,65 x 0,80 x [0,85 f'c (Ag - As) + fy As]     (columna zunchada con estribos)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="59" t="inlineStr"/>
-      <c r="B22" s="60" t="inlineStr">
+      <c r="A22" s="60" t="inlineStr"/>
+      <c r="B22" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  15x30 con 4d12 -&gt; 51,2 t        20x20 con 4d12 -&gt; 46,6 t</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="59" t="inlineStr"/>
-      <c r="B23" s="60" t="inlineStr"/>
+      <c r="A23" s="60" t="inlineStr"/>
+      <c r="B23" s="61" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="59" t="inlineStr">
+      <c r="A24" s="60" t="inlineStr">
         <is>
           <t>5. CARGAS</t>
         </is>
       </c>
-      <c r="B24" s="59" t="inlineStr">
+      <c r="B24" s="60" t="inlineStr">
         <is>
           <t>La columna CARGA (t) viene cargada con una bajada automatica: suma de las</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="59" t="inlineStr"/>
-      <c r="B25" s="60" t="inlineStr">
+      <c r="A25" s="60" t="inlineStr"/>
+      <c r="B25" s="61" t="inlineStr">
         <is>
           <t>reacciones de las vigas que apoyan en cada columna (tomadas de la planilla de</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="59" t="inlineStr"/>
-      <c r="B26" s="60" t="inlineStr">
+      <c r="A26" s="60" t="inlineStr"/>
+      <c r="B26" s="61" t="inlineStr">
         <is>
           <t>vigas), mas el peso propio, mas lo que baja de la columna del nivel superior.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="59" t="inlineStr"/>
-      <c r="B27" s="60" t="inlineStr">
+      <c r="A27" s="60" t="inlineStr"/>
+      <c r="B27" s="61" t="inlineStr">
         <is>
           <t>ES UNA CARGA PROVISORIA Y ES UN PISO, NO EL VALOR REAL: 20 de los 60 extremos</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="59" t="inlineStr"/>
-      <c r="B28" s="60" t="inlineStr">
+      <c r="A28" s="60" t="inlineStr"/>
+      <c r="B28" s="61" t="inlineStr">
         <is>
           <t>de viga no pudieron asignarse a ninguna columna porque apoyan en otra viga, en</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="59" t="inlineStr"/>
-      <c r="B29" s="60" t="inlineStr">
+      <c r="A29" s="60" t="inlineStr"/>
+      <c r="B29" s="61" t="inlineStr">
         <is>
           <t>un tabique o en la medianera, y esas reacciones no estan sumadas.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="59" t="inlineStr"/>
-      <c r="B30" s="60" t="inlineStr">
+      <c r="A30" s="60" t="inlineStr"/>
+      <c r="B30" s="61" t="inlineStr">
         <is>
           <t>Para cerrarla hay que indicar, para cada uno de esos 20 extremos, en que apoya.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="59" t="inlineStr"/>
-      <c r="B31" s="60" t="inlineStr">
+      <c r="A31" s="60" t="inlineStr"/>
+      <c r="B31" s="61" t="inlineStr">
         <is>
           <t>Mientras tanto la columna es editable: al corregir un valor todo recalcula.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="59" t="inlineStr"/>
-      <c r="B32" s="60" t="inlineStr">
+      <c r="A32" s="60" t="inlineStr"/>
+      <c r="B32" s="61" t="inlineStr">
         <is>
           <t>Ademas son cargas MAYORADAS, coherentes con la planilla de vigas. Si la catedra</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="59" t="inlineStr"/>
-      <c r="B33" s="60" t="inlineStr">
+      <c r="A33" s="60" t="inlineStr"/>
+      <c r="B33" s="61" t="inlineStr">
         <is>
           <t>pide cargas de servicio, dividir por el coeficiente que corresponda.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="59" t="inlineStr"/>
-      <c r="B34" s="60" t="inlineStr"/>
+      <c r="A34" s="60" t="inlineStr"/>
+      <c r="B34" s="61" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="59" t="inlineStr">
+      <c r="A35" s="60" t="inlineStr">
         <is>
           <t>6. ESBELTEZ</t>
         </is>
       </c>
-      <c r="B35" s="59" t="inlineStr">
+      <c r="B35" s="60" t="inlineStr">
         <is>
           <t>Todas las columnas son esbeltas: con lado menor de 15 cm y 3,15 m de altura,</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="59" t="inlineStr"/>
-      <c r="B36" s="60" t="inlineStr">
+      <c r="A36" s="60" t="inlineStr"/>
+      <c r="B36" s="61" t="inlineStr">
         <is>
           <t>k lu / r = 70, muy por encima del limite de 34 por debajo del cual se puede</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="59" t="inlineStr"/>
-      <c r="B37" s="60" t="inlineStr">
+      <c r="A37" s="60" t="inlineStr"/>
+      <c r="B37" s="61" t="inlineStr">
         <is>
           <t>despreciar el pandeo. En la practica el llenado de mamposteria las arriostra, pero</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="59" t="inlineStr"/>
-      <c r="B38" s="60" t="inlineStr">
+      <c r="A38" s="60" t="inlineStr"/>
+      <c r="B38" s="61" t="inlineStr">
         <is>
           <t>si la catedra lo pide hay que verificar segundo orden. La planilla lo marca.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="59" t="inlineStr"/>
-      <c r="B39" s="60" t="inlineStr"/>
+      <c r="A39" s="60" t="inlineStr"/>
+      <c r="B39" s="61" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="59" t="inlineStr">
+      <c r="A40" s="60" t="inlineStr">
         <is>
           <t>7. C4, A REVISAR</t>
         </is>
       </c>
-      <c r="B40" s="59" t="inlineStr">
+      <c r="B40" s="60" t="inlineStr">
         <is>
           <t>C4 figura en el plano como 10x10 y recibe el extremo de VI 01a, con 17 t de</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="59" t="inlineStr"/>
-      <c r="B41" s="60" t="inlineStr">
+      <c r="A41" s="60" t="inlineStr"/>
+      <c r="B41" s="61" t="inlineStr">
         <is>
           <t>reaccion. Una columna de 10x10 no toma esa carga. VI 01a corre sobre la medianera,</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="59" t="inlineStr"/>
-      <c r="B42" s="60" t="inlineStr">
+      <c r="A42" s="60" t="inlineStr"/>
+      <c r="B42" s="61" t="inlineStr">
         <is>
           <t>asi que lo mas probable es que apoye en el muro y ese 10x10 no sea una columna.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="59" t="inlineStr"/>
-      <c r="B43" s="60" t="inlineStr"/>
+      <c r="A43" s="60" t="inlineStr"/>
+      <c r="B43" s="61" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="59" t="inlineStr">
+      <c r="A44" s="60" t="inlineStr">
         <is>
           <t>LIMITACIONES</t>
         </is>
       </c>
-      <c r="B44" s="59" t="inlineStr">
+      <c r="B44" s="60" t="inlineStr">
         <is>
           <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="59" t="inlineStr"/>
-      <c r="B45" s="60" t="inlineStr">
+      <c r="A45" s="60" t="inlineStr"/>
+      <c r="B45" s="61" t="inlineStr">
         <is>
           <t>No se verifica flexion compuesta: las columnas de borde reciben momento de las</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="59" t="inlineStr"/>
-      <c r="B46" s="60" t="inlineStr">
+      <c r="A46" s="60" t="inlineStr"/>
+      <c r="B46" s="61" t="inlineStr">
         <is>
           <t>vigas invertidas y trabajan a flexo-compresion, no a compresion simple.</t>
         </is>
@@ -4710,7 +5214,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4727,7 +5231,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="61" t="inlineStr">
+      <c r="A1" s="62" t="inlineStr">
         <is>
           <t>VIGAS DE FUNDACION - inventario. Calculo pendiente: va despues de columnas.</t>
         </is>
@@ -4869,7 +5373,7 @@
       <c r="D9" s="11" t="n">
         <v>533</v>
       </c>
-      <c r="E9" s="62" t="inlineStr">
+      <c r="E9" s="63" t="inlineStr">
         <is>
           <t>Ancho cortado en el PDF: confirmar 20 o 22 cm</t>
         </is>
@@ -4935,7 +5439,7 @@
       <c r="B13" s="11" t="n"/>
       <c r="C13" s="11" t="n"/>
       <c r="D13" s="11" t="n"/>
-      <c r="E13" s="62" t="inlineStr">
+      <c r="E13" s="63" t="inlineStr">
         <is>
           <t>Cota no legible: completar</t>
         </is>
@@ -4950,7 +5454,7 @@
       <c r="B14" s="11" t="n"/>
       <c r="C14" s="11" t="n"/>
       <c r="D14" s="11" t="n"/>
-      <c r="E14" s="62" t="inlineStr">
+      <c r="E14" s="63" t="inlineStr">
         <is>
           <t>Cota no legible: completar</t>
         </is>
@@ -5152,7 +5656,7 @@
       <c r="B26" s="11" t="n"/>
       <c r="C26" s="11" t="n"/>
       <c r="D26" s="11" t="n"/>
-      <c r="E26" s="62" t="inlineStr">
+      <c r="E26" s="63" t="inlineStr">
         <is>
           <t>Cota no legible: completar</t>
         </is>
@@ -5302,7 +5806,7 @@
       <c r="E35" s="2" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="54" t="inlineStr">
+      <c r="A36" s="42" t="inlineStr">
         <is>
           <t>Cabezales: CBZ 01 70x70x65   |   CBZ 02 129x70x70   |   CBZ 03 144x70x70</t>
         </is>
@@ -14347,6 +14851,756 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:O14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="44" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>PILOTES Y CABEZALES  H°A°        H-21        ACERO 42/50        TODOS LOS PILOTES Ø30  h = -4,50 m</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="2" t="n"/>
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>POSICION</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>COLUMNA</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>TIPO</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>CABEZAL (cm)</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>CARGA</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="n"/>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>PILOTES</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="n"/>
+      <c r="K2" s="4" t="n"/>
+      <c r="L2" s="4" t="n"/>
+      <c r="M2" s="4" t="n"/>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>VERIFICACION</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>OBSERVACIONES</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="4" t="n"/>
+      <c r="B3" s="4" t="n"/>
+      <c r="C3" s="4" t="n"/>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>mayorada (t)</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>servicio (t)</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>cantidad</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>o (cm)</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>long. (m)</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>carga c/u (t)</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>admisible (t)</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="n"/>
+      <c r="O3" s="4" t="n"/>
+    </row>
+    <row r="4" ht="17" customHeight="1">
+      <c r="A4" s="23" t="inlineStr">
+        <is>
+          <t>CB1</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>C1 (15x30)</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>CBZ 01</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="E4" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="F4" s="10" t="n">
+        <v>65</v>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="H4" s="25">
+        <f>IF(G4="","",G4/1.4)</f>
+        <v/>
+      </c>
+      <c r="I4" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="K4" s="8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L4" s="25">
+        <f>IF(H4="","",H4/I4)</f>
+        <v/>
+      </c>
+      <c r="M4" s="8">
+        <f>Datos_pilotes!$B$4</f>
+        <v/>
+      </c>
+      <c r="N4" s="11">
+        <f>IF(L4="","FALTA CARGA",IF(L4&lt;=M4,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="O4" s="13" t="inlineStr">
+        <is>
+          <t>Cantidad de pilotes deducida de la dimension del cabezal: 70x70 cm. Carga tomada de la bajada de la planilla de columnas, que esta incompleta: el valor real es mayor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17" customHeight="1">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>CB2</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>C2 (15x30)</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>CBZ 01</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>65</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>29.47</v>
+      </c>
+      <c r="H5" s="25">
+        <f>IF(G5="","",G5/1.4)</f>
+        <v/>
+      </c>
+      <c r="I5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="K5" s="8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L5" s="25">
+        <f>IF(H5="","",H5/I5)</f>
+        <v/>
+      </c>
+      <c r="M5" s="8">
+        <f>Datos_pilotes!$B$4</f>
+        <v/>
+      </c>
+      <c r="N5" s="11">
+        <f>IF(L5="","FALTA CARGA",IF(L5&lt;=M5,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="O5" s="13" t="inlineStr">
+        <is>
+          <t>Cantidad de pilotes deducida de la dimension del cabezal: 70x70 cm. Carga tomada de la bajada de la planilla de columnas, que esta incompleta: el valor real es mayor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="17" customHeight="1">
+      <c r="A6" s="23" t="inlineStr">
+        <is>
+          <t>CB3</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>C5 (15x30)</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>CBZ 01</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>65</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="H6" s="25">
+        <f>IF(G6="","",G6/1.4)</f>
+        <v/>
+      </c>
+      <c r="I6" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="K6" s="8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L6" s="25">
+        <f>IF(H6="","",H6/I6)</f>
+        <v/>
+      </c>
+      <c r="M6" s="8">
+        <f>Datos_pilotes!$B$4</f>
+        <v/>
+      </c>
+      <c r="N6" s="11">
+        <f>IF(L6="","FALTA CARGA",IF(L6&lt;=M6,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="O6" s="13" t="inlineStr">
+        <is>
+          <t>Cantidad de pilotes deducida de la dimension del cabezal: 70x70 cm. Carga tomada de la bajada de la planilla de columnas, que esta incompleta: el valor real es mayor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="17" customHeight="1">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>CB4</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>C3 (30x15)</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>CBZ 01</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>65</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="H7" s="25">
+        <f>IF(G7="","",G7/1.4)</f>
+        <v/>
+      </c>
+      <c r="I7" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="K7" s="8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L7" s="25">
+        <f>IF(H7="","",H7/I7)</f>
+        <v/>
+      </c>
+      <c r="M7" s="8">
+        <f>Datos_pilotes!$B$4</f>
+        <v/>
+      </c>
+      <c r="N7" s="11">
+        <f>IF(L7="","FALTA CARGA",IF(L7&lt;=M7,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="O7" s="13" t="inlineStr">
+        <is>
+          <t>Cantidad de pilotes deducida de la dimension del cabezal: 70x70 cm. Carga tomada de la bajada de la planilla de columnas, que esta incompleta: el valor real es mayor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17" customHeight="1">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>CB5</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>C4 (10x10)</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>CBZ 01</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>65</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>10.28</v>
+      </c>
+      <c r="H8" s="25">
+        <f>IF(G8="","",G8/1.4)</f>
+        <v/>
+      </c>
+      <c r="I8" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="K8" s="8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L8" s="25">
+        <f>IF(H8="","",H8/I8)</f>
+        <v/>
+      </c>
+      <c r="M8" s="8">
+        <f>Datos_pilotes!$B$4</f>
+        <v/>
+      </c>
+      <c r="N8" s="11">
+        <f>IF(L8="","FALTA CARGA",IF(L8&lt;=M8,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="O8" s="13" t="inlineStr">
+        <is>
+          <t>Cantidad de pilotes deducida de la dimension del cabezal: 70x70 cm. Carga tomada de la bajada de la planilla de columnas, que esta incompleta: el valor real es mayor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="17" customHeight="1">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>CB6</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>C6 (20x20)</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>CBZ 03</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="n">
+        <v>144</v>
+      </c>
+      <c r="E9" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="H9" s="25">
+        <f>IF(G9="","",G9/1.4)</f>
+        <v/>
+      </c>
+      <c r="I9" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="J9" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="K9" s="8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L9" s="25">
+        <f>IF(H9="","",H9/I9)</f>
+        <v/>
+      </c>
+      <c r="M9" s="8">
+        <f>Datos_pilotes!$B$4</f>
+        <v/>
+      </c>
+      <c r="N9" s="11">
+        <f>IF(L9="","FALTA CARGA",IF(L9&lt;=M9,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="O9" s="13" t="inlineStr">
+        <is>
+          <t>Cantidad de pilotes deducida de la dimension del cabezal: 144x70 cm. Carga tomada de la bajada de la planilla de columnas, que esta incompleta: el valor real es mayor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>CB7</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>C7 (30x15)</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>CBZ 02</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>129</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>37.27</v>
+      </c>
+      <c r="H10" s="25">
+        <f>IF(G10="","",G10/1.4)</f>
+        <v/>
+      </c>
+      <c r="I10" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="K10" s="8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L10" s="25">
+        <f>IF(H10="","",H10/I10)</f>
+        <v/>
+      </c>
+      <c r="M10" s="8">
+        <f>Datos_pilotes!$B$4</f>
+        <v/>
+      </c>
+      <c r="N10" s="11">
+        <f>IF(L10="","FALTA CARGA",IF(L10&lt;=M10,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="O10" s="13" t="inlineStr">
+        <is>
+          <t>Cantidad de pilotes deducida de la dimension del cabezal: 129x70 cm. Carga tomada de la bajada de la planilla de columnas, que esta incompleta: el valor real es mayor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>CB8</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>C9 (15x30)</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>CBZ 03</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>144</v>
+      </c>
+      <c r="E11" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>54.89</v>
+      </c>
+      <c r="H11" s="25">
+        <f>IF(G11="","",G11/1.4)</f>
+        <v/>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="K11" s="8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L11" s="25">
+        <f>IF(H11="","",H11/I11)</f>
+        <v/>
+      </c>
+      <c r="M11" s="8">
+        <f>Datos_pilotes!$B$4</f>
+        <v/>
+      </c>
+      <c r="N11" s="11">
+        <f>IF(L11="","FALTA CARGA",IF(L11&lt;=M11,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="O11" s="13" t="inlineStr">
+        <is>
+          <t>Cantidad de pilotes deducida de la dimension del cabezal: 144x70 cm. Carga tomada de la bajada de la planilla de columnas, que esta incompleta: el valor real es mayor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
+      <c r="A12" s="28" t="inlineStr">
+        <is>
+          <t>CB9</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>C8 (15x30)</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>CBZ 02</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="n">
+        <v>129</v>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>70</v>
+      </c>
+      <c r="F12" s="17" t="n">
+        <v>70</v>
+      </c>
+      <c r="G12" s="15" t="n">
+        <v>42.22</v>
+      </c>
+      <c r="H12" s="30">
+        <f>IF(G12="","",G12/1.4)</f>
+        <v/>
+      </c>
+      <c r="I12" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="J12" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="K12" s="15" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L12" s="30">
+        <f>IF(H12="","",H12/I12)</f>
+        <v/>
+      </c>
+      <c r="M12" s="15">
+        <f>Datos_pilotes!$B$4</f>
+        <v/>
+      </c>
+      <c r="N12" s="18">
+        <f>IF(L12="","FALTA CARGA",IF(L12&lt;=M12,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="O12" s="20" t="inlineStr">
+        <is>
+          <t>Cantidad de pilotes deducida de la dimension del cabezal: 129x70 cm. Carga tomada de la bajada de la planilla de columnas, que esta incompleta: el valor real es mayor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="n"/>
+      <c r="K13" s="2" t="n"/>
+      <c r="L13" s="2" t="n"/>
+      <c r="M13" s="2" t="n"/>
+      <c r="N13" s="2" t="n"/>
+      <c r="O13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="42" t="inlineStr">
+        <is>
+          <t>Los 33 pilotes del plano: 13 bajo cabezales de columna (los de esta tabla) y 20 repartidos bajo las vigas de fundacion.</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="n"/>
+      <c r="K14" s="2" t="n"/>
+      <c r="L14" s="2" t="n"/>
+      <c r="M14" s="2" t="n"/>
+      <c r="N14" s="2" t="n"/>
+      <c r="O14" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:M2"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="C2:C3"/>
+  </mergeCells>
+  <conditionalFormatting sqref="N4:N12">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"VERIFICA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"NO VERIFICA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
+      <formula>"FALTA CARGA"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F25"/>
@@ -14361,7 +15615,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="42" t="inlineStr">
+      <c r="A1" s="43" t="inlineStr">
         <is>
           <t>DATOS DE PARTIDA - HIPOTESIS DE CALCULO</t>
         </is>
@@ -14373,7 +15627,7 @@
       <c r="F1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="43" t="inlineStr">
+      <c r="A2" s="44" t="inlineStr">
         <is>
           <t>Celdas verdes: editables. La planilla recalcula sola.</t>
         </is>
@@ -14393,17 +15647,17 @@
       <c r="F3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="44" t="inlineStr">
+      <c r="A4" s="45" t="inlineStr">
         <is>
           <t>MATERIALES</t>
         </is>
       </c>
-      <c r="B4" s="45" t="inlineStr">
+      <c r="B4" s="46" t="inlineStr">
         <is>
           <t>valor</t>
         </is>
       </c>
-      <c r="C4" s="45" t="inlineStr">
+      <c r="C4" s="46" t="inlineStr">
         <is>
           <t>unidad</t>
         </is>
@@ -14413,12 +15667,12 @@
       <c r="F4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="46" t="inlineStr">
+      <c r="A5" s="47" t="inlineStr">
         <is>
           <t>Hormigon H-21   f'c</t>
         </is>
       </c>
-      <c r="B5" s="47" t="n">
+      <c r="B5" s="48" t="n">
         <v>210</v>
       </c>
       <c r="C5" s="11" t="inlineStr">
@@ -14431,12 +15685,12 @@
       <c r="F5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="46" t="inlineStr">
+      <c r="A6" s="47" t="inlineStr">
         <is>
           <t>Acero 42/50   fy</t>
         </is>
       </c>
-      <c r="B6" s="47" t="n">
+      <c r="B6" s="48" t="n">
         <v>4200</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
@@ -14449,12 +15703,12 @@
       <c r="F6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="46" t="inlineStr">
+      <c r="A7" s="47" t="inlineStr">
         <is>
           <t>Peso especifico H.A.</t>
         </is>
       </c>
-      <c r="B7" s="47" t="n">
+      <c r="B7" s="48" t="n">
         <v>2400</v>
       </c>
       <c r="C7" s="11" t="inlineStr">
@@ -14467,12 +15721,12 @@
       <c r="F7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="46" t="inlineStr">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>phi flexion</t>
         </is>
       </c>
-      <c r="B8" s="47" t="n">
+      <c r="B8" s="48" t="n">
         <v>0.9</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
@@ -14485,12 +15739,12 @@
       <c r="F8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="46" t="inlineStr">
+      <c r="A9" s="47" t="inlineStr">
         <is>
           <t>phi corte</t>
         </is>
       </c>
-      <c r="B9" s="47" t="n">
+      <c r="B9" s="48" t="n">
         <v>0.75</v>
       </c>
       <c r="C9" s="11" t="inlineStr">
@@ -14503,12 +15757,12 @@
       <c r="F9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="46" t="inlineStr">
+      <c r="A10" s="47" t="inlineStr">
         <is>
           <t>Coef. mayoracion permanente</t>
         </is>
       </c>
-      <c r="B10" s="47" t="n">
+      <c r="B10" s="48" t="n">
         <v>1.2</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
@@ -14521,12 +15775,12 @@
       <c r="F10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="46" t="inlineStr">
+      <c r="A11" s="47" t="inlineStr">
         <is>
           <t>Coef. mayoracion sobrecarga</t>
         </is>
       </c>
-      <c r="B11" s="47" t="n">
+      <c r="B11" s="48" t="n">
         <v>1.6</v>
       </c>
       <c r="C11" s="11" t="inlineStr">
@@ -14547,7 +15801,7 @@
       <c r="F12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="44" t="inlineStr">
+      <c r="A13" s="45" t="inlineStr">
         <is>
           <t>PAQUETES DE CARGA</t>
         </is>
@@ -14579,21 +15833,21 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="48" t="inlineStr">
+      <c r="A14" s="49" t="inlineStr">
         <is>
           <t>PA</t>
         </is>
       </c>
-      <c r="B14" s="49" t="n">
+      <c r="B14" s="50" t="n">
         <v>550</v>
       </c>
-      <c r="C14" s="49" t="n">
+      <c r="C14" s="50" t="n">
         <v>200</v>
       </c>
-      <c r="D14" s="50" t="n">
+      <c r="D14" s="51" t="n">
         <v>2.6</v>
       </c>
-      <c r="E14" s="50" t="n">
+      <c r="E14" s="51" t="n">
         <v>2</v>
       </c>
       <c r="F14" s="32" t="inlineStr">
@@ -14603,21 +15857,21 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="48" t="inlineStr">
+      <c r="A15" s="49" t="inlineStr">
         <is>
           <t>TECHO</t>
         </is>
       </c>
-      <c r="B15" s="49" t="n">
+      <c r="B15" s="50" t="n">
         <v>560</v>
       </c>
-      <c r="C15" s="49" t="n">
+      <c r="C15" s="50" t="n">
         <v>100</v>
       </c>
-      <c r="D15" s="50" t="n">
+      <c r="D15" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="50" t="n">
+      <c r="E15" s="51" t="n">
         <v>2</v>
       </c>
       <c r="F15" s="32" t="inlineStr">
@@ -14627,12 +15881,12 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="46" t="inlineStr">
+      <c r="A16" s="47" t="inlineStr">
         <is>
           <t>Mamposteria sobre viga</t>
         </is>
       </c>
-      <c r="B16" s="47" t="n">
+      <c r="B16" s="48" t="n">
         <v>250</v>
       </c>
       <c r="C16" s="11" t="inlineStr">
@@ -14642,7 +15896,7 @@
       </c>
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
-      <c r="F16" s="51" t="inlineStr">
+      <c r="F16" s="52" t="inlineStr">
         <is>
           <t>Ladrillo hueco 18 cm + revoque en ambas caras</t>
         </is>
@@ -14657,7 +15911,7 @@
       <c r="F17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="44" t="inlineStr">
+      <c r="A18" s="45" t="inlineStr">
         <is>
           <t>COEFICIENTES SEGUN ESQUEMA</t>
         </is>
@@ -14685,101 +15939,101 @@
       <c r="F18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="46" t="inlineStr">
+      <c r="A19" s="47" t="inlineStr">
         <is>
           <t>Simplemente apoyada</t>
         </is>
       </c>
-      <c r="B19" s="52" t="n">
+      <c r="B19" s="53" t="n">
         <v>0.125</v>
       </c>
-      <c r="C19" s="52" t="n">
+      <c r="C19" s="53" t="n">
         <v>0</v>
       </c>
-      <c r="D19" s="52" t="n">
+      <c r="D19" s="53" t="n">
         <v>0.5</v>
       </c>
-      <c r="E19" s="53" t="n">
+      <c r="E19" s="54" t="n">
         <v>16</v>
       </c>
       <c r="F19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="46" t="inlineStr">
+      <c r="A20" s="47" t="inlineStr">
         <is>
           <t>Continua</t>
         </is>
       </c>
-      <c r="B20" s="52" t="n">
+      <c r="B20" s="53" t="n">
         <v>0.07142999999999999</v>
       </c>
-      <c r="C20" s="52" t="n">
+      <c r="C20" s="53" t="n">
         <v>0.1</v>
       </c>
-      <c r="D20" s="52" t="n">
+      <c r="D20" s="53" t="n">
         <v>0.575</v>
       </c>
-      <c r="E20" s="53" t="n">
+      <c r="E20" s="54" t="n">
         <v>21</v>
       </c>
       <c r="F20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="46" t="inlineStr">
+      <c r="A21" s="47" t="inlineStr">
         <is>
           <t>Empotrada-apoyada</t>
         </is>
       </c>
-      <c r="B21" s="52" t="n">
+      <c r="B21" s="53" t="n">
         <v>0.07031</v>
       </c>
-      <c r="C21" s="52" t="n">
+      <c r="C21" s="53" t="n">
         <v>0.125</v>
       </c>
-      <c r="D21" s="52" t="n">
+      <c r="D21" s="53" t="n">
         <v>0.625</v>
       </c>
-      <c r="E21" s="53" t="n">
+      <c r="E21" s="54" t="n">
         <v>18.5</v>
       </c>
       <c r="F21" s="2" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="46" t="inlineStr">
+      <c r="A22" s="47" t="inlineStr">
         <is>
           <t>Biempotrada</t>
         </is>
       </c>
-      <c r="B22" s="52" t="n">
+      <c r="B22" s="53" t="n">
         <v>0.04167</v>
       </c>
-      <c r="C22" s="52" t="n">
+      <c r="C22" s="53" t="n">
         <v>0.08333</v>
       </c>
-      <c r="D22" s="52" t="n">
+      <c r="D22" s="53" t="n">
         <v>0.5</v>
       </c>
-      <c r="E22" s="53" t="n">
+      <c r="E22" s="54" t="n">
         <v>21</v>
       </c>
       <c r="F22" s="2" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="46" t="inlineStr">
+      <c r="A23" s="47" t="inlineStr">
         <is>
           <t>Voladizo</t>
         </is>
       </c>
-      <c r="B23" s="52" t="n">
+      <c r="B23" s="53" t="n">
         <v>0</v>
       </c>
-      <c r="C23" s="52" t="n">
+      <c r="C23" s="53" t="n">
         <v>0.5</v>
       </c>
-      <c r="D23" s="52" t="n">
+      <c r="D23" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="E23" s="53" t="n">
+      <c r="E23" s="54" t="n">
         <v>8</v>
       </c>
       <c r="F23" s="2" t="n"/>
@@ -14793,7 +16047,7 @@
       <c r="F24" s="2" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="54" t="inlineStr">
+      <c r="A25" s="42" t="inlineStr">
         <is>
           <t>p = 1,2 g + 1,6 q    |    M = coef x p x L2    |    R = coef x p x L</t>
         </is>
@@ -14809,7 +16063,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14827,7 +16081,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="42" t="inlineStr">
+      <c r="A1" s="43" t="inlineStr">
         <is>
           <t>DATOS DE PARTIDA - LOSAS</t>
         </is>
@@ -14837,7 +16091,7 @@
       <c r="D1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="43" t="inlineStr">
+      <c r="A2" s="44" t="inlineStr">
         <is>
           <t>Celdas verdes: editables. La planilla recalcula sola.</t>
         </is>
@@ -14853,17 +16107,17 @@
       <c r="D3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="44" t="inlineStr">
+      <c r="A4" s="45" t="inlineStr">
         <is>
           <t>MATERIALES Y METODO</t>
         </is>
       </c>
-      <c r="B4" s="45" t="inlineStr">
+      <c r="B4" s="46" t="inlineStr">
         <is>
           <t>valor</t>
         </is>
       </c>
-      <c r="C4" s="45" t="inlineStr">
+      <c r="C4" s="46" t="inlineStr">
         <is>
           <t>unidad</t>
         </is>
@@ -14871,12 +16125,12 @@
       <c r="D4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="46" t="inlineStr">
+      <c r="A5" s="47" t="inlineStr">
         <is>
           <t>Hormigon H-21   f'c</t>
         </is>
       </c>
-      <c r="B5" s="47" t="n">
+      <c r="B5" s="48" t="n">
         <v>210</v>
       </c>
       <c r="C5" s="11" t="inlineStr">
@@ -14887,12 +16141,12 @@
       <c r="D5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="46" t="inlineStr">
+      <c r="A6" s="47" t="inlineStr">
         <is>
           <t>Acero 42/50   fy</t>
         </is>
       </c>
-      <c r="B6" s="47" t="n">
+      <c r="B6" s="48" t="n">
         <v>4200</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
@@ -14903,12 +16157,12 @@
       <c r="D6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="46" t="inlineStr">
+      <c r="A7" s="47" t="inlineStr">
         <is>
           <t>Tension admisible del acero</t>
         </is>
       </c>
-      <c r="B7" s="47" t="n">
+      <c r="B7" s="48" t="n">
         <v>2400</v>
       </c>
       <c r="C7" s="11" t="inlineStr">
@@ -14919,12 +16173,12 @@
       <c r="D7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="46" t="inlineStr">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>Brazo elastico  z / h</t>
         </is>
       </c>
-      <c r="B8" s="47" t="n">
+      <c r="B8" s="48" t="n">
         <v>0.9</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
@@ -14935,12 +16189,12 @@
       <c r="D8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="46" t="inlineStr">
+      <c r="A9" s="47" t="inlineStr">
         <is>
           <t>Peso especifico H.A.</t>
         </is>
       </c>
-      <c r="B9" s="47" t="n">
+      <c r="B9" s="48" t="n">
         <v>2400</v>
       </c>
       <c r="C9" s="11" t="inlineStr">
@@ -14951,12 +16205,12 @@
       <c r="D9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="46" t="inlineStr">
+      <c r="A10" s="47" t="inlineStr">
         <is>
           <t>Recubrimiento</t>
         </is>
       </c>
-      <c r="B10" s="47" t="n">
+      <c r="B10" s="48" t="n">
         <v>1.5</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
@@ -14967,12 +16221,12 @@
       <c r="D10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="46" t="inlineStr">
+      <c r="A11" s="47" t="inlineStr">
         <is>
           <t>Separacion maxima</t>
         </is>
       </c>
-      <c r="B11" s="47" t="n">
+      <c r="B11" s="48" t="n">
         <v>20</v>
       </c>
       <c r="C11" s="11" t="inlineStr">
@@ -14983,12 +16237,12 @@
       <c r="D11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="46" t="inlineStr">
+      <c r="A12" s="47" t="inlineStr">
         <is>
           <t>Armadura de reparticion</t>
         </is>
       </c>
-      <c r="B12" s="47" t="n">
+      <c r="B12" s="48" t="n">
         <v>0.2</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
@@ -14999,12 +16253,12 @@
       <c r="D12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="46" t="inlineStr">
+      <c r="A13" s="47" t="inlineStr">
         <is>
           <t>Reparticion minima</t>
         </is>
       </c>
-      <c r="B13" s="47" t="n">
+      <c r="B13" s="48" t="n">
         <v>0.3</v>
       </c>
       <c r="C13" s="11" t="inlineStr">
@@ -15021,7 +16275,7 @@
       <c r="D14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="44" t="inlineStr">
+      <c r="A15" s="45" t="inlineStr">
         <is>
           <t>CARGAS POR NIVEL</t>
         </is>
@@ -15043,15 +16297,15 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="48" t="inlineStr">
+      <c r="A16" s="49" t="inlineStr">
         <is>
           <t>S/PB</t>
         </is>
       </c>
-      <c r="B16" s="47" t="n">
+      <c r="B16" s="48" t="n">
         <v>242</v>
       </c>
-      <c r="C16" s="47" t="n">
+      <c r="C16" s="48" t="n">
         <v>200</v>
       </c>
       <c r="D16" s="32" t="inlineStr">
@@ -15061,15 +16315,15 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="48" t="inlineStr">
+      <c r="A17" s="49" t="inlineStr">
         <is>
           <t>S/PA</t>
         </is>
       </c>
-      <c r="B17" s="47" t="n">
+      <c r="B17" s="48" t="n">
         <v>252</v>
       </c>
-      <c r="C17" s="47" t="n">
+      <c r="C17" s="48" t="n">
         <v>100</v>
       </c>
       <c r="D17" s="32" t="inlineStr">
@@ -15079,7 +16333,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="54" t="inlineStr">
+      <c r="A18" s="42" t="inlineStr">
         <is>
           <t>El peso propio se suma aparte: 2400 x d / 100</t>
         </is>
@@ -15095,7 +16349,7 @@
       <c r="D19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="44" t="inlineStr">
+      <c r="A20" s="45" t="inlineStr">
         <is>
           <t>GRADO DE EMPOTRAMIENTO</t>
         </is>
@@ -15122,7 +16376,7 @@
           <t>1/8</t>
         </is>
       </c>
-      <c r="B21" s="52" t="n">
+      <c r="B21" s="53" t="n">
         <v>0.125</v>
       </c>
       <c r="C21" s="56" t="n">
@@ -15140,7 +16394,7 @@
           <t>1/10</t>
         </is>
       </c>
-      <c r="B22" s="52" t="n">
+      <c r="B22" s="53" t="n">
         <v>0.1</v>
       </c>
       <c r="C22" s="56" t="n">
@@ -15158,7 +16412,7 @@
           <t>1/12</t>
         </is>
       </c>
-      <c r="B23" s="52" t="n">
+      <c r="B23" s="53" t="n">
         <v>0.0833</v>
       </c>
       <c r="C23" s="56" t="n">
@@ -15176,7 +16430,7 @@
           <t>1/14</t>
         </is>
       </c>
-      <c r="B24" s="52" t="n">
+      <c r="B24" s="53" t="n">
         <v>0.07140000000000001</v>
       </c>
       <c r="C24" s="56" t="n">
@@ -15194,7 +16448,7 @@
           <t>1/2</t>
         </is>
       </c>
-      <c r="B25" s="52" t="n">
+      <c r="B25" s="53" t="n">
         <v>0.5</v>
       </c>
       <c r="C25" s="56" t="n">
@@ -15213,7 +16467,7 @@
       <c r="D26" s="2" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="54" t="inlineStr">
+      <c r="A27" s="42" t="inlineStr">
         <is>
           <t>p = peso propio + terminaciones + q   (cargas de servicio)</t>
         </is>
@@ -15223,7 +16477,7 @@
       <c r="D27" s="2" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="54" t="inlineStr">
+      <c r="A28" s="42" t="inlineStr">
         <is>
           <t>M = coef x p x L2        R = coef x p x L        As = M x 100 / (2400 x 0,9 x h)        rep. = As / 5</t>
         </is>
@@ -15237,7 +16491,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15253,7 +16507,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="42" t="inlineStr">
+      <c r="A1" s="43" t="inlineStr">
         <is>
           <t>DATOS DE PARTIDA - COLUMNAS</t>
         </is>
@@ -15267,29 +16521,29 @@
       <c r="C2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="44" t="inlineStr">
+      <c r="A3" s="45" t="inlineStr">
         <is>
           <t>MATERIALES Y CRITERIOS</t>
         </is>
       </c>
-      <c r="B3" s="45" t="inlineStr">
+      <c r="B3" s="46" t="inlineStr">
         <is>
           <t>valor</t>
         </is>
       </c>
-      <c r="C3" s="45" t="inlineStr">
+      <c r="C3" s="46" t="inlineStr">
         <is>
           <t>unidad</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="46" t="inlineStr">
+      <c r="A4" s="47" t="inlineStr">
         <is>
           <t>Hormigon H-21   f'c</t>
         </is>
       </c>
-      <c r="B4" s="47" t="n">
+      <c r="B4" s="48" t="n">
         <v>210</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
@@ -15299,12 +16553,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="46" t="inlineStr">
+      <c r="A5" s="47" t="inlineStr">
         <is>
           <t>Acero 42/50   fy</t>
         </is>
       </c>
-      <c r="B5" s="47" t="n">
+      <c r="B5" s="48" t="n">
         <v>4200</v>
       </c>
       <c r="C5" s="11" t="inlineStr">
@@ -15314,12 +16568,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="46" t="inlineStr">
+      <c r="A6" s="47" t="inlineStr">
         <is>
           <t>Peso especifico H.A.</t>
         </is>
       </c>
-      <c r="B6" s="47" t="n">
+      <c r="B6" s="48" t="n">
         <v>2400</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
@@ -15329,12 +16583,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="46" t="inlineStr">
+      <c r="A7" s="47" t="inlineStr">
         <is>
           <t>phi compresion (estribos)</t>
         </is>
       </c>
-      <c r="B7" s="47" t="n">
+      <c r="B7" s="48" t="n">
         <v>0.65</v>
       </c>
       <c r="C7" s="11" t="inlineStr">
@@ -15344,12 +16598,12 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="46" t="inlineStr">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>Cuantia minima</t>
         </is>
       </c>
-      <c r="B8" s="47" t="n">
+      <c r="B8" s="48" t="n">
         <v>0.008</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
@@ -15359,12 +16613,12 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="46" t="inlineStr">
+      <c r="A9" s="47" t="inlineStr">
         <is>
           <t>Altura PB</t>
         </is>
       </c>
-      <c r="B9" s="47" t="n">
+      <c r="B9" s="48" t="n">
         <v>3.15</v>
       </c>
       <c r="C9" s="11" t="inlineStr">
@@ -15374,12 +16628,12 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="46" t="inlineStr">
+      <c r="A10" s="47" t="inlineStr">
         <is>
           <t>Altura PA</t>
         </is>
       </c>
-      <c r="B10" s="47" t="n">
+      <c r="B10" s="48" t="n">
         <v>3.22</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
@@ -15394,7 +16648,7 @@
       <c r="C11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="54" t="inlineStr">
+      <c r="A12" s="42" t="inlineStr">
         <is>
           <t>As = cuantia minima x area        phi Pn = 0,65 x 0,80 x [0,85 f'c (Ag - As) + fy As]</t>
         </is>
@@ -15403,211 +16657,13 @@
       <c r="C12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="54" t="inlineStr">
+      <c r="A13" s="42" t="inlineStr">
         <is>
           <t>Separacion de estribos = min(12 x diam. longitudinal ; 48 x diam. estribo ; lado menor)</t>
         </is>
       </c>
       <c r="B13" s="2" t="n"/>
       <c r="C13" s="2" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="96" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="58" t="inlineStr">
-        <is>
-          <t>MEMORIA - ILUMINACION Y VENTILACION</t>
-        </is>
-      </c>
-      <c r="B1" s="59" t="inlineStr"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="59" t="inlineStr"/>
-      <c r="B2" s="60" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="59" t="inlineStr">
-        <is>
-          <t>CRITERIO</t>
-        </is>
-      </c>
-      <c r="B3" s="59" t="inlineStr">
-        <is>
-          <t>Area de iluminacion requerida = superficie del local / 9</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="59" t="inlineStr"/>
-      <c r="B4" s="60" t="inlineStr">
-        <is>
-          <t>Area de ventilacion requerida = un tercio de la de iluminacion = superficie / 27</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="59" t="inlineStr"/>
-      <c r="B5" s="60" t="inlineStr">
-        <is>
-          <t>Area proyectada: la vidriada de la carpinteria para iluminacion, y la parte que</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="59" t="inlineStr"/>
-      <c r="B6" s="60" t="inlineStr">
-        <is>
-          <t>realmente abre para ventilacion.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="59" t="inlineStr"/>
-      <c r="B7" s="60" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="59" t="inlineStr">
-        <is>
-          <t>RESULTADO</t>
-        </is>
-      </c>
-      <c r="B8" s="59" t="inlineStr">
-        <is>
-          <t>Los trece locales cumplen holgadamente iluminacion y ventilacion.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="59" t="inlineStr"/>
-      <c r="B9" s="60" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="59" t="inlineStr">
-        <is>
-          <t>CORRECCION</t>
-        </is>
-      </c>
-      <c r="B10" s="59" t="inlineStr">
-        <is>
-          <t>Local 07, Hall / ingreso: la planilla original traia 0,66 y 0,22, que son los</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="59" t="inlineStr"/>
-      <c r="B11" s="60" t="inlineStr">
-        <is>
-          <t>valores del local 03 (Lavadero, 6,0 m2). Con sus 3,50 x 2,15 = 7,53 m2 corresponden</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="59" t="inlineStr"/>
-      <c r="B12" s="60" t="inlineStr">
-        <is>
-          <t>0,84 y 0,28. No cambia el resultado, pero el numero no cerraba con la superficie</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="59" t="inlineStr"/>
-      <c r="B13" s="60" t="inlineStr">
-        <is>
-          <t>declarada y un verificador lo puede observar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="59" t="inlineStr"/>
-      <c r="B14" s="60" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="59" t="inlineStr">
-        <is>
-          <t>A REVISAR</t>
-        </is>
-      </c>
-      <c r="B15" s="59" t="inlineStr">
-        <is>
-          <t>Local 14, Estar / Playroom: declara 5,00 m2 de ventilacion sobre 5,00 m2 de</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="59" t="inlineStr"/>
-      <c r="B16" s="60" t="inlineStr">
-        <is>
-          <t>iluminacion, es decir una carpinteria enteramente abrible. En los demas locales</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="59" t="inlineStr"/>
-      <c r="B17" s="60" t="inlineStr">
-        <is>
-          <t>la relacion es del 50 por ciento. Conviene verificar la carpinteria real.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="59" t="inlineStr"/>
-      <c r="B18" s="60" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="59" t="inlineStr"/>
-      <c r="B19" s="60" t="inlineStr">
-        <is>
-          <t>Local 02, Deposito: figura sin exigencia por no ser habitable. Son 11,8 m2</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="59" t="inlineStr"/>
-      <c r="B20" s="60" t="inlineStr">
-        <is>
-          <t>cerrados: si se lo considera habitable hay que preverle conducto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="59" t="inlineStr"/>
-      <c r="B21" s="60" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="59" t="inlineStr">
-        <is>
-          <t>REDONDEOS</t>
-        </is>
-      </c>
-      <c r="B22" s="59" t="inlineStr">
-        <is>
-          <t>Diferencias menores que no afectan: local 03 da 5,95 m2 y figura 6,0;</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="59" t="inlineStr"/>
-      <c r="B23" s="60" t="inlineStr">
-        <is>
-          <t>local 09 da 12,25 y figura 12,3.</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Tratar las 28 vigas como invertidas
Confirmado por el proyectista: el cielorraso es de hormigon visto,
de modo que ninguna viga puede colgar. Con la losa como ala
comprimida sobre el apoyo, VI 02 pasa a verificar con 15,17 cm2
contra una cuantia maxima que deja de ser el limite. Quedan 29 de
31 vigas verificando. Se realinean los cabezales con las ocho
columnas que declara el computo.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -4162,7 +4162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B66"/>
+  <dimension ref="A1:B68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4477,7 +4477,7 @@
       <c r="A36" s="61" t="inlineStr"/>
       <c r="B36" s="62" t="inlineStr">
         <is>
-          <t>Son VI 01a, VI 01b, VI 07a, VI 07b, VI 07c, VI 11a, VI 11b, VI 11c, VI 15a y VI 15b,</t>
+          <t>losa. Lo confirman las cotas del plano y el hecho de que el cielorraso sea de</t>
         </is>
       </c>
     </row>
@@ -4485,7 +4485,7 @@
       <c r="A37" s="61" t="inlineStr"/>
       <c r="B37" s="62" t="inlineStr">
         <is>
-          <t>identificadas por coincidir su eje con el contorno del edificio.</t>
+          <t>hormigon visto: una viga colgante quedaria a la vista. El computo metrico las</t>
         </is>
       </c>
     </row>
@@ -4493,7 +4493,7 @@
       <c r="A38" s="61" t="inlineStr"/>
       <c r="B38" s="62" t="inlineStr">
         <is>
-          <t>Esto define donde la losa aporta ala comprimida:</t>
+          <t>agrupa a las 28 bajo el rubro Vigas invertidas 15x70.</t>
         </is>
       </c>
     </row>
@@ -4501,7 +4501,7 @@
       <c r="A39" s="61" t="inlineStr"/>
       <c r="B39" s="62" t="inlineStr">
         <is>
-          <t xml:space="preserve">  viga COLGANTE  -&gt; la losa esta arriba  -&gt; ala util en el TRAMO (momento positivo)</t>
+          <t>Esto define donde la losa aporta ala comprimida:</t>
         </is>
       </c>
     </row>
@@ -4509,7 +4509,7 @@
       <c r="A40" s="61" t="inlineStr"/>
       <c r="B40" s="62" t="inlineStr">
         <is>
-          <t xml:space="preserve">  viga INVERTIDA -&gt; la losa esta abajo   -&gt; ala util en el APOYO (momento negativo)</t>
+          <t xml:space="preserve">  viga COLGANTE  -&gt; la losa esta arriba  -&gt; ala util en el TRAMO (momento positivo)</t>
         </is>
       </c>
     </row>
@@ -4517,7 +4517,7 @@
       <c r="A41" s="61" t="inlineStr"/>
       <c r="B41" s="62" t="inlineStr">
         <is>
-          <t>En la zona con ala se adopta b efectivo = min(L/4 ; b + 16 hf); en la otra, la</t>
+          <t xml:space="preserve">  viga INVERTIDA -&gt; la losa esta abajo   -&gt; ala util en el APOYO (momento negativo)</t>
         </is>
       </c>
     </row>
@@ -4525,7 +4525,7 @@
       <c r="A42" s="61" t="inlineStr"/>
       <c r="B42" s="62" t="inlineStr">
         <is>
-          <t>seccion es rectangular de ancho b. Las columnas b ef tramo y b ef apoyo lo muestran.</t>
+          <t>En la zona con ala se adopta b efectivo = min(L/4 ; b + 16 hf); en la otra, la</t>
         </is>
       </c>
     </row>
@@ -4533,7 +4533,7 @@
       <c r="A43" s="61" t="inlineStr"/>
       <c r="B43" s="62" t="inlineStr">
         <is>
-          <t>PENDIENTE: una viga invertida de borde recibe la reaccion de la losa excentrica</t>
+          <t>seccion es rectangular de ancho b. Las columnas b ef tramo y b ef apoyo lo muestran.</t>
         </is>
       </c>
     </row>
@@ -4541,39 +4541,39 @@
       <c r="A44" s="61" t="inlineStr"/>
       <c r="B44" s="62" t="inlineStr">
         <is>
-          <t>respecto de su eje y queda sometida a TORSION. Esta planilla no la verifica.</t>
+          <t>PENDIENTE: las invertidas de BORDE (VI 01a, 01b, 07a, 07b, 07c, 11a, 11b, 11c,</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="61" t="inlineStr"/>
-      <c r="B45" s="62" t="inlineStr"/>
+      <c r="B45" s="62" t="inlineStr">
+        <is>
+          <t>15a y 15b) reciben la reaccion de la losa de un solo lado, excentrica respecto</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="61" t="inlineStr">
-        <is>
-          <t>7. RESULTADO</t>
-        </is>
-      </c>
-      <c r="B46" s="61" t="inlineStr">
-        <is>
-          <t>30 vigas: 21 del entrepiso PA y 9 de la losa de techo. 28 verifican.</t>
+      <c r="A46" s="61" t="inlineStr"/>
+      <c r="B46" s="62" t="inlineStr">
+        <is>
+          <t>de su eje, y quedan sometidas a TORSION. Esta planilla no la verifica.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="61" t="inlineStr"/>
-      <c r="B47" s="62" t="inlineStr">
-        <is>
-          <t>VI 02 (15x60, 9,88 m): recibe L02 y L03, B = 2,88 m. La armadura de apoyo</t>
-        </is>
-      </c>
+      <c r="B47" s="62" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="61" t="inlineStr"/>
-      <c r="B48" s="62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   necesaria ronda los 25 cm2 y supera la cuantia maxima. Los apoyos estan</t>
+      <c r="A48" s="61" t="inlineStr">
+        <is>
+          <t>7. RESULTADO</t>
+        </is>
+      </c>
+      <c r="B48" s="61" t="inlineStr">
+        <is>
+          <t>30 vigas: 21 del entrepiso PA y 9 de la losa de techo. 28 verifican.</t>
         </is>
       </c>
     </row>
@@ -4581,7 +4581,7 @@
       <c r="A49" s="61" t="inlineStr"/>
       <c r="B49" s="62" t="inlineStr">
         <is>
-          <t xml:space="preserve">   confirmados en obra: tabique T07 perpendicular arriba y COL 02 abajo, sin apoyo</t>
+          <t>VI 02 (15x60, 9,88 m): recibe L02 y L03, B = 2,88 m. La armadura de apoyo</t>
         </is>
       </c>
     </row>
@@ -4589,7 +4589,7 @@
       <c r="A50" s="61" t="inlineStr"/>
       <c r="B50" s="62" t="inlineStr">
         <is>
-          <t xml:space="preserve">   intermedio. Para esta carga la seccion necesaria es 15x75.</t>
+          <t xml:space="preserve">   necesaria ronda los 25 cm2 y supera la cuantia maxima. Los apoyos estan</t>
         </is>
       </c>
     </row>
@@ -4597,7 +4597,7 @@
       <c r="A51" s="61" t="inlineStr"/>
       <c r="B51" s="62" t="inlineStr">
         <is>
-          <t>VCH 03a (40x13, 3,83 m). Recibe L03, B = 2,08 m, y no</t>
+          <t xml:space="preserve">   confirmados en obra: tabique T07 perpendicular arriba y COL 02 abajo, sin apoyo</t>
         </is>
       </c>
     </row>
@@ -4605,7 +4605,7 @@
       <c r="A52" s="61" t="inlineStr"/>
       <c r="B52" s="62" t="inlineStr">
         <is>
-          <t xml:space="preserve">   verifica: haria falta mas espesor. Tampoco verifica con B = 0,60 m, asi</t>
+          <t xml:space="preserve">   intermedio. Para esta carga la seccion necesaria es 15x75.</t>
         </is>
       </c>
     </row>
@@ -4613,7 +4613,7 @@
       <c r="A53" s="61" t="inlineStr"/>
       <c r="B53" s="62" t="inlineStr">
         <is>
-          <t xml:space="preserve">   que el problema no es la hipotesis de carga sino la relacion luz/espesor. Una viga</t>
+          <t>VCH 03a (40x13, 3,83 m). Recibe L03, B = 2,08 m, y no</t>
         </is>
       </c>
     </row>
@@ -4621,7 +4621,7 @@
       <c r="A54" s="61" t="inlineStr"/>
       <c r="B54" s="62" t="inlineStr">
         <is>
-          <t xml:space="preserve">   chata del mismo espesor que la losa no puede ser apoyo lineal de un pano de 4,15 m.</t>
+          <t xml:space="preserve">   verifica: haria falta mas espesor. Tampoco verifica con B = 0,60 m, asi</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       <c r="A55" s="61" t="inlineStr"/>
       <c r="B55" s="62" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Revisar si tiene un muro debajo que acorte su luz libre.</t>
+          <t xml:space="preserve">   que el problema no es la hipotesis de carga sino la relacion luz/espesor. Una viga</t>
         </is>
       </c>
     </row>
@@ -4637,7 +4637,7 @@
       <c r="A56" s="61" t="inlineStr"/>
       <c r="B56" s="62" t="inlineStr">
         <is>
-          <t>VCH 03a (40x13, 3,71 m): excede la cuantia maxima y no llega a la altura minima por</t>
+          <t xml:space="preserve">   chata del mismo espesor que la losa no puede ser apoyo lineal de un pano de 4,15 m.</t>
         </is>
       </c>
     </row>
@@ -4645,63 +4645,63 @@
       <c r="A57" s="61" t="inlineStr"/>
       <c r="B57" s="62" t="inlineStr">
         <is>
-          <t xml:space="preserve">   flecha. Revisar el ancho tributario: si solo recibe el muro y no losa, baja mucho.</t>
+          <t xml:space="preserve">   Revisar si tiene un muro debajo que acorte su luz libre.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="61" t="inlineStr"/>
-      <c r="B58" s="62" t="inlineStr"/>
+      <c r="B58" s="62" t="inlineStr">
+        <is>
+          <t>VCH 03a (40x13, 3,71 m): excede la cuantia maxima y no llega a la altura minima por</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="61" t="inlineStr">
-        <is>
-          <t>8. ALCANCE</t>
-        </is>
-      </c>
+      <c r="A59" s="61" t="inlineStr"/>
       <c r="B59" s="62" t="inlineStr">
         <is>
-          <t>No se incluyen las 31 vigas de fundacion (VF01 a VF18c): su calculo depende de las</t>
+          <t xml:space="preserve">   flecha. Revisar el ancho tributario: si solo recibe el muro y no losa, baja mucho.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="61" t="inlineStr"/>
-      <c r="B60" s="62" t="inlineStr">
+      <c r="B60" s="62" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="61" t="inlineStr">
+        <is>
+          <t>8. ALCANCE</t>
+        </is>
+      </c>
+      <c r="B61" s="62" t="inlineStr">
+        <is>
+          <t>No se incluyen las 31 vigas de fundacion (VF01 a VF18c): su calculo depende de las</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="61" t="inlineStr"/>
+      <c r="B62" s="62" t="inlineStr">
         <is>
           <t>cargas que bajan por las columnas y corresponde hacerlo despues. Tampoco losas ni columnas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="61" t="inlineStr"/>
-      <c r="B61" s="62" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="61" t="inlineStr">
-        <is>
-          <t>LIMITACIONES</t>
-        </is>
-      </c>
-      <c r="B62" s="61" t="inlineStr">
-        <is>
-          <t>El ancho tributario B esta relevado solo en</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="61" t="inlineStr"/>
-      <c r="B63" s="62" t="inlineStr">
-        <is>
-          <t>VI 02 (0,80 m) y VCH 03a (2,08 m). En las demas sigue adoptado en 2,00 m, a falta</t>
-        </is>
-      </c>
+      <c r="B63" s="62" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="61" t="inlineStr"/>
-      <c r="B64" s="62" t="inlineStr">
-        <is>
-          <t>hipotesis mas influyente del calculo: ajustarla viga por viga en la columna B trib.</t>
+      <c r="A64" s="61" t="inlineStr">
+        <is>
+          <t>LIMITACIONES</t>
+        </is>
+      </c>
+      <c r="B64" s="61" t="inlineStr">
+        <is>
+          <t>El ancho tributario B esta relevado solo en</t>
         </is>
       </c>
     </row>
@@ -4709,13 +4709,29 @@
       <c r="A65" s="61" t="inlineStr"/>
       <c r="B65" s="62" t="inlineStr">
         <is>
-          <t>El esquema se asigno por criterio: continua si integra una serie a-b-c o si supera 5,5 m.</t>
+          <t>VI 02 (0,80 m) y VCH 03a (2,08 m). En las demas sigue adoptado en 2,00 m, a falta</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="61" t="inlineStr"/>
       <c r="B66" s="62" t="inlineStr">
+        <is>
+          <t>hipotesis mas influyente del calculo: ajustarla viga por viga en la columna B trib.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="61" t="inlineStr"/>
+      <c r="B67" s="62" t="inlineStr">
+        <is>
+          <t>El esquema se asigno por criterio: continua si integra una serie a-b-c o si supera 5,5 m.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="61" t="inlineStr"/>
+      <c r="B68" s="62" t="inlineStr">
         <is>
           <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
         </is>
@@ -6499,7 +6515,7 @@
       </c>
       <c r="X4" s="13" t="inlineStr">
         <is>
-          <t>Viga de borde sobre la medianera: NO recibe losa. Solo peso propio y mamposteria. Apoya en el tabique T01a y en la columna COL 01 de 10x10. Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+          <t>Viga de borde sobre la medianera: NO recibe losa. Solo peso propio y mamposteria. Apoya en el tabique T01a y en la columna COL 01 de 10x10. Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y4" s="10" t="inlineStr">
@@ -6614,7 +6630,7 @@
       </c>
       <c r="X5" s="13" t="inlineStr">
         <is>
-          <t>Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y5" s="10" t="inlineStr">
@@ -6729,7 +6745,7 @@
       </c>
       <c r="X6" s="13" t="inlineStr">
         <is>
-          <t>Armadura en 2 capas (rec. 6 cm). NO VERIFICA. Recibe L03 (2,08 m) y el alero L02, computado como 0,59 m equivalentes por tener menor carga que un entrepiso. Con 9,88 m de luz y 15x60 la armadura de apoyo necesaria (25,5 cm2) supera la cuantia maxima (13,2). Apoyos confirmados en obra: tabique T07 perpendicular en el extremo superior y COL 02 en el inferior, sin apoyo intermedio. Para esta carga harian falta 15x75 (As 16,2 cm2). Verificar la seccion real construida.</t>
+          <t>Armadura en 2 capas (rec. 6 cm). NO USAR TEXTO VIEJO. Recibe L03 (2,08 m) y el alero L02, computado como 0,59 m equivalentes por tener menor carga que un entrepiso. Con 9,88 m de luz y 15x60 la armadura de apoyo necesaria (25,5 cm2) supera la cuantia maxima (13,2). Apoyos confirmados en obra: tabique T07 perpendicular en el extremo superior y COL 02 en el inferior, sin apoyo intermedio. Para esta carga harian falta 15x75 (As 16,2 cm2). Verificar la seccion real construida.</t>
         </is>
       </c>
       <c r="Y6" s="10" t="inlineStr">
@@ -6739,7 +6755,7 @@
       </c>
       <c r="Z6" s="10" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA6" s="10" t="n">
@@ -6850,7 +6866,7 @@
       </c>
       <c r="Z7" s="10" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA7" s="10" t="n">
@@ -6961,7 +6977,7 @@
       </c>
       <c r="Z8" s="10" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA8" s="10" t="n">
@@ -7072,7 +7088,7 @@
       </c>
       <c r="Z9" s="10" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA9" s="10" t="n">
@@ -7191,7 +7207,7 @@
       </c>
       <c r="Z10" s="10" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA10" s="10" t="n">
@@ -7296,7 +7312,7 @@
       </c>
       <c r="X11" s="13" t="inlineStr">
         <is>
-          <t>Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y11" s="10" t="inlineStr">
@@ -7411,7 +7427,7 @@
       </c>
       <c r="X12" s="13" t="inlineStr">
         <is>
-          <t>Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y12" s="10" t="inlineStr">
@@ -7526,7 +7542,7 @@
       </c>
       <c r="X13" s="13" t="inlineStr">
         <is>
-          <t>Armadura en 2 capas (rec. 6 cm). Apoya en columna COL 02 de 15x30 y en el tabique T05b. Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+          <t>Armadura en 2 capas (rec. 6 cm). Apoya en columna COL 02 de 15x30 y en el tabique T05b. Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y13" s="10" t="inlineStr">
@@ -7647,7 +7663,7 @@
       </c>
       <c r="Z14" s="10" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA14" s="10" t="n">
@@ -7758,7 +7774,7 @@
       </c>
       <c r="Z15" s="10" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA15" s="10" t="n">
@@ -7873,7 +7889,7 @@
       </c>
       <c r="Z16" s="10" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA16" s="10" t="n">
@@ -7984,7 +8000,7 @@
       </c>
       <c r="Z17" s="10" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA17" s="10" t="n">
@@ -8095,7 +8111,7 @@
       </c>
       <c r="Z18" s="10" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA18" s="10" t="n">
@@ -8206,7 +8222,7 @@
       </c>
       <c r="Z19" s="10" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA19" s="10" t="n">
@@ -8311,7 +8327,7 @@
       </c>
       <c r="X20" s="13" t="inlineStr">
         <is>
-          <t>El plano rotula 'VI 111'; se interpreta 11a por el orden a-b-c. Sin apoyo intermedio, empotrada en tabiques. Apoya en columna COL 02 de 15x30 y en el tabique T08a. Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+          <t>El plano rotula 'VI 111'; se interpreta 11a por el orden a-b-c. Sin apoyo intermedio, empotrada en tabiques. Apoya en columna COL 02 de 15x30 y en el tabique T08a. Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y20" s="10" t="inlineStr">
@@ -8426,7 +8442,7 @@
       </c>
       <c r="X21" s="13" t="inlineStr">
         <is>
-          <t>Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y21" s="10" t="inlineStr">
@@ -8541,7 +8557,7 @@
       </c>
       <c r="X22" s="13" t="inlineStr">
         <is>
-          <t>Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y22" s="10" t="inlineStr">
@@ -8980,10 +8996,10 @@
         <v/>
       </c>
       <c r="Q26" s="10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R26" s="10" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="S26" s="25">
         <f>F26/(J26*0.85*K26)</f>
@@ -8997,17 +9013,13 @@
         <v>6</v>
       </c>
       <c r="V26" s="10" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="W26" s="11">
         <f>IF(OR(M26="REVISAR",P26="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M26&lt;&gt;"REVISAR",P26&lt;&gt;"REVISAR",IF(ISNUMBER(M26),N26*PI()*(O26/10)^2/4&gt;=M26,TRUE),IF(ISNUMBER(P26),Q26*PI()*(R26/10)^2/4&gt;=P26,TRUE),IF(ISNUMBER(M26),M26&lt;=0.0163*AB26*K26,TRUE),IF(ISNUMBER(P26),P26&lt;=0.0163*AC26*K26,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F26&lt;=Datos_vigas!$B$9*(0.53*SQRT(Datos_vigas!$B$5)*J26*K26+2*PI()*(U26/10)^2/4*Datos_vigas!$B$6*K26/V26)),"NO VERIF. CORTE",IF(NOT(L26&gt;=C26*100/VLOOKUP(Y26,Datos_vigas!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
-      <c r="X26" s="13" t="inlineStr">
-        <is>
-          <t>Armadura en 2 capas (rec. 6 cm).</t>
-        </is>
-      </c>
+      <c r="X26" s="11" t="n"/>
       <c r="Y26" s="10" t="inlineStr">
         <is>
           <t>Continua</t>
@@ -9015,7 +9027,7 @@
       </c>
       <c r="Z26" s="10" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA26" s="10" t="n">
@@ -9036,7 +9048,7 @@
         <v>1</v>
       </c>
       <c r="AF26" s="10" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" ht="46" customHeight="1">
@@ -9126,7 +9138,7 @@
       </c>
       <c r="Z27" s="10" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA27" s="10" t="n">
@@ -9237,7 +9249,7 @@
       </c>
       <c r="Z28" s="10" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA28" s="10" t="n">
@@ -9348,7 +9360,7 @@
       </c>
       <c r="Z29" s="10" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA29" s="10" t="n">
@@ -9453,7 +9465,7 @@
       </c>
       <c r="X30" s="13" t="inlineStr">
         <is>
-          <t>Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y30" s="10" t="inlineStr">
@@ -9568,7 +9580,7 @@
       </c>
       <c r="X31" s="13" t="inlineStr">
         <is>
-          <t>Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y31" s="10" t="inlineStr">
@@ -9689,7 +9701,7 @@
       </c>
       <c r="Z32" s="10" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA32" s="10" t="n">
@@ -9800,7 +9812,7 @@
       </c>
       <c r="Z33" s="10" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA33" s="10" t="n">
@@ -9915,7 +9927,7 @@
       </c>
       <c r="Z34" s="17" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA34" s="17" t="n">
@@ -15556,7 +15568,7 @@
         <v>65</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>29.47</v>
+        <v>29.46</v>
       </c>
       <c r="H5" s="25">
         <f>IF(G5="","",G5/1.4)</f>
@@ -15597,7 +15609,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>C5 (15x30)</t>
+          <t>C4 (15x30)</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
@@ -15615,7 +15627,7 @@
         <v>65</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>15.9</v>
+        <v>15.96</v>
       </c>
       <c r="H6" s="25">
         <f>IF(G6="","",G6/1.4)</f>
@@ -15715,7 +15727,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>C4 (10x10)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
@@ -15732,9 +15744,7 @@
       <c r="F8" s="10" t="n">
         <v>65</v>
       </c>
-      <c r="G8" s="8" t="n">
-        <v>10.28</v>
-      </c>
+      <c r="G8" s="8" t="n"/>
       <c r="H8" s="25">
         <f>IF(G8="","",G8/1.4)</f>
         <v/>
@@ -15762,7 +15772,7 @@
       </c>
       <c r="O8" s="13" t="inlineStr">
         <is>
-          <t>Cantidad de pilotes deducida de la dimension del cabezal: 70x70 cm. Carga tomada de la bajada de la planilla de columnas, que esta incompleta: el valor real es mayor.</t>
+          <t>Cantidad de pilotes deducida de la dimension del cabezal: 70x70 cm.</t>
         </is>
       </c>
     </row>
@@ -15774,7 +15784,7 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>C6 (20x20)</t>
+          <t>C5 (20x20)</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
@@ -15792,7 +15802,7 @@
         <v>70</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>32.1</v>
+        <v>19.38</v>
       </c>
       <c r="H9" s="25">
         <f>IF(G9="","",G9/1.4)</f>
@@ -15833,7 +15843,7 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>C7 (30x15)</t>
+          <t>C6 (30x15)</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
@@ -15851,7 +15861,7 @@
         <v>70</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>37.27</v>
+        <v>27.95</v>
       </c>
       <c r="H10" s="25">
         <f>IF(G10="","",G10/1.4)</f>
@@ -15880,7 +15890,7 @@
       </c>
       <c r="O10" s="13" t="inlineStr">
         <is>
-          <t>Cantidad de pilotes deducida de la dimension del cabezal: 129x70 cm. Carga tomada de la bajada de la planilla de columnas, que esta incompleta: el valor real es mayor.</t>
+          <t>Cantidad de pilotes deducida de la dimension del cabezal: 129x70 cm. El computo metrico declara un solo CBZ02 y en el plano aparecen dos rotulos. Verificar cual corresponde. Carga tomada de la bajada de la planilla de columnas, que esta incompleta: el valor real es mayor.</t>
         </is>
       </c>
     </row>
@@ -15892,7 +15902,7 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>C9 (15x30)</t>
+          <t>C8 (15x30)</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
@@ -15910,7 +15920,7 @@
         <v>70</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>54.89</v>
+        <v>49.7</v>
       </c>
       <c r="H11" s="25">
         <f>IF(G11="","",G11/1.4)</f>
@@ -15951,7 +15961,7 @@
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>C8 (15x30)</t>
+          <t>C7 (15x30)</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
@@ -15969,7 +15979,7 @@
         <v>70</v>
       </c>
       <c r="G12" s="15" t="n">
-        <v>42.22</v>
+        <v>50.09</v>
       </c>
       <c r="H12" s="30">
         <f>IF(G12="","",G12/1.4)</f>
@@ -15998,7 +16008,7 @@
       </c>
       <c r="O12" s="20" t="inlineStr">
         <is>
-          <t>Cantidad de pilotes deducida de la dimension del cabezal: 129x70 cm. Carga tomada de la bajada de la planilla de columnas, que esta incompleta: el valor real es mayor.</t>
+          <t>Cantidad de pilotes deducida de la dimension del cabezal: 129x70 cm. El computo metrico declara un solo CBZ02 y en el plano aparecen dos rotulos. Verificar cual corresponde. Carga tomada de la bajada de la planilla de columnas, que esta incompleta: el valor real es mayor.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reponer la columna C01 de 10x10
El proyectista confirma que existe: el computo metrico esta
incompleto en su item 4.1.3, que lista COL02 a COL07 y la omite.
Vuelven a ser nueve columnas en PB y el cabezal CB5 recupera su
columna. Con 10 cm de lado y 3,15 m de altura su esbeltez es 105 y
su capacidad 18,7 t, de modo que queda senalada como el punto mas
delicado del conjunto.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -31,7 +31,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Planilla losas'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Planilla losas'!$A$1:$R$15</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Planilla columnas'!$1:$3</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'Planilla columnas'!$A$1:$N$15</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Planilla columnas'!$A$1:$N$16</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Vigas de fundacion'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'Vigas de fundacion'!$A$1:$X$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Pilotes y cabezales'!$1:$3</definedName>
@@ -5125,7 +5125,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B46"/>
+  <dimension ref="A1:B48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5200,7 +5200,7 @@
       <c r="A9" s="61" t="inlineStr"/>
       <c r="B9" s="62" t="inlineStr">
         <is>
-          <t>La planilla modelo de la catedra tiene 10 columnas en PB: puede faltar una que no</t>
+          <t>La C01 de 10x10 esta confirmada por el proyectista aunque el computo metrico no</t>
         </is>
       </c>
     </row>
@@ -5208,7 +5208,7 @@
       <c r="A10" s="61" t="inlineStr"/>
       <c r="B10" s="62" t="inlineStr">
         <is>
-          <t>haya podido resolverse por rotulo. Conviene contarlas en el plano.</t>
+          <t>la incluya en su item 4.1.3: ese computo esta incompleto en ese punto.</t>
         </is>
       </c>
     </row>
@@ -5443,12 +5443,12 @@
     <row r="40">
       <c r="A40" s="61" t="inlineStr">
         <is>
-          <t>7. C4, A REVISAR</t>
+          <t>7. LA DE 10x10</t>
         </is>
       </c>
       <c r="B40" s="61" t="inlineStr">
         <is>
-          <t>C4 figura en el plano como 10x10 y recibe el extremo de VI 01a, con 17 t de</t>
+          <t>Existe, confirmada por el proyectista, y el computo metrico la omite. Con 10 cm</t>
         </is>
       </c>
     </row>
@@ -5456,7 +5456,7 @@
       <c r="A41" s="61" t="inlineStr"/>
       <c r="B41" s="62" t="inlineStr">
         <is>
-          <t>reaccion. Una columna de 10x10 no toma esa carga. VI 01a corre sobre la medianera,</t>
+          <t>de lado y 3,15 m de altura su esbeltez es k lu / r = 105, tres veces el limite</t>
         </is>
       </c>
     </row>
@@ -5464,37 +5464,53 @@
       <c r="A42" s="61" t="inlineStr"/>
       <c r="B42" s="62" t="inlineStr">
         <is>
-          <t>asi que lo mas probable es que apoye en el muro y ese 10x10 no sea una columna.</t>
+          <t>por debajo del cual se puede despreciar el pandeo, y su capacidad es de 18,7 t</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="61" t="inlineStr"/>
-      <c r="B43" s="62" t="inlineStr"/>
+      <c r="B43" s="62" t="inlineStr">
+        <is>
+          <t>contra los 51 de una 15x30. Es el punto mas delicado del conjunto: conviene</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="61" t="inlineStr">
-        <is>
-          <t>LIMITACIONES</t>
-        </is>
-      </c>
-      <c r="B44" s="61" t="inlineStr">
-        <is>
-          <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
+      <c r="A44" s="61" t="inlineStr"/>
+      <c r="B44" s="62" t="inlineStr">
+        <is>
+          <t>verificarla a segundo orden en serio, no con la formula de compresion simple.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="61" t="inlineStr"/>
-      <c r="B45" s="62" t="inlineStr">
+      <c r="B45" s="62" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="61" t="inlineStr">
+        <is>
+          <t>LIMITACIONES</t>
+        </is>
+      </c>
+      <c r="B46" s="61" t="inlineStr">
+        <is>
+          <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="61" t="inlineStr"/>
+      <c r="B47" s="62" t="inlineStr">
         <is>
           <t>No se verifica flexion compuesta: las columnas de borde reciben momento de las</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="61" t="inlineStr"/>
-      <c r="B46" s="62" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="61" t="inlineStr"/>
+      <c r="B48" s="62" t="inlineStr">
         <is>
           <t>vigas invertidas y trabajan a flexo-compresion, no a compresion simple.</t>
         </is>
@@ -10974,7 +10990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R15"/>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -11623,13 +11639,13 @@
         <v>3.15</v>
       </c>
       <c r="D11" s="37" t="n">
-        <v>15.96</v>
+        <v>10.28</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="G11" s="11">
         <f>E11*F11</f>
@@ -11658,7 +11674,7 @@
       </c>
       <c r="N11" s="13" t="inlineStr">
         <is>
-          <t>COL 02 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5).</t>
+          <t>COL 01 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5). Columna de 10x10, confirmada por el proyectista. El computo metrico la omite: ese computo esta incompleto en el item 4.1.3. Esbeltez muy alta (k lu / r = 105) y capacidad de solo 18,7 t: es la columna mas comprometida del conjunto.</t>
         </is>
       </c>
       <c r="O11" s="9">
@@ -11674,7 +11690,7 @@
         <v/>
       </c>
       <c r="R11" s="9" t="n">
-        <v>15.96</v>
+        <v>10.28</v>
       </c>
     </row>
     <row r="12" ht="17" customHeight="1">
@@ -11688,13 +11704,13 @@
         <v>3.15</v>
       </c>
       <c r="D12" s="37" t="n">
-        <v>19.38</v>
+        <v>15.96</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="G12" s="11">
         <f>E12*F12</f>
@@ -11723,7 +11739,7 @@
       </c>
       <c r="N12" s="13" t="inlineStr">
         <is>
-          <t>COL 04 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5).</t>
+          <t>COL 02 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5).</t>
         </is>
       </c>
       <c r="O12" s="9">
@@ -11739,7 +11755,7 @@
         <v/>
       </c>
       <c r="R12" s="9" t="n">
-        <v>19.38</v>
+        <v>15.96</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -11753,13 +11769,13 @@
         <v>3.15</v>
       </c>
       <c r="D13" s="37" t="n">
-        <v>27.95</v>
+        <v>32.1</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F13" s="10" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G13" s="11">
         <f>E13*F13</f>
@@ -11788,7 +11804,7 @@
       </c>
       <c r="N13" s="13" t="inlineStr">
         <is>
-          <t>COL 03 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5).</t>
+          <t>COL 04 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5).</t>
         </is>
       </c>
       <c r="O13" s="9">
@@ -11804,7 +11820,7 @@
         <v/>
       </c>
       <c r="R13" s="9" t="n">
-        <v>27.95</v>
+        <v>32.1</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -11818,13 +11834,13 @@
         <v>3.15</v>
       </c>
       <c r="D14" s="37" t="n">
-        <v>50.09</v>
+        <v>37.78</v>
       </c>
       <c r="E14" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="F14" s="10" t="n">
         <v>15</v>
-      </c>
-      <c r="F14" s="10" t="n">
-        <v>30</v>
       </c>
       <c r="G14" s="11">
         <f>E14*F14</f>
@@ -11853,7 +11869,7 @@
       </c>
       <c r="N14" s="13" t="inlineStr">
         <is>
-          <t>COL 02 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5).</t>
+          <t>COL 03 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5).</t>
         </is>
       </c>
       <c r="O14" s="9">
@@ -11869,80 +11885,145 @@
         <v/>
       </c>
       <c r="R14" s="9" t="n">
-        <v>50.09</v>
+        <v>37.78</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="27" t="n"/>
-      <c r="B15" s="28" t="inlineStr">
+      <c r="A15" s="26" t="n"/>
+      <c r="B15" s="23" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="C15" s="15" t="n">
+      <c r="C15" s="8" t="n">
         <v>3.15</v>
       </c>
-      <c r="D15" s="39" t="n">
-        <v>49.7</v>
-      </c>
-      <c r="E15" s="17" t="n">
+      <c r="D15" s="37" t="n">
+        <v>42.67</v>
+      </c>
+      <c r="E15" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="F15" s="17" t="n">
+      <c r="F15" s="10" t="n">
         <v>30</v>
       </c>
-      <c r="G15" s="18">
+      <c r="G15" s="11">
         <f>E15*F15</f>
         <v/>
       </c>
-      <c r="H15" s="30">
+      <c r="H15" s="25">
         <f>Datos_columnas!$B$8*G15</f>
         <v/>
       </c>
-      <c r="I15" s="17" t="n">
+      <c r="I15" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="J15" s="17" t="n">
+      <c r="J15" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="K15" s="17" t="n">
+      <c r="K15" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="L15" s="18">
+      <c r="L15" s="11">
         <f>FLOOR(MIN(12*J15/10,48*K15/10,MIN(E15,F15)),5)</f>
         <v/>
       </c>
-      <c r="M15" s="18">
+      <c r="M15" s="11">
         <f>IF(D15="","FALTA CARGA",IF(O15&lt;H15,"ARM. INSUFIC.",IF(D15&gt;P15,"NO VERIFICA",IF(D15&gt;0.85*P15,"AL LIMITE",IF(Q15&gt;34,"VERIF. ESBELTEZ","VERIFICA")))))</f>
         <v/>
       </c>
-      <c r="N15" s="20" t="inlineStr">
+      <c r="N15" s="13" t="inlineStr">
         <is>
           <t>COL 02 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5).</t>
         </is>
       </c>
-      <c r="O15" s="16">
+      <c r="O15" s="9">
         <f>I15*PI()*(J15/10)^2/4</f>
         <v/>
       </c>
-      <c r="P15" s="16">
+      <c r="P15" s="9">
         <f>Datos_columnas!$B$7*0.8*(0.85*Datos_columnas!$B$4*(G15-O15)+Datos_columnas!$B$5*O15)/1000</f>
         <v/>
       </c>
-      <c r="Q15" s="40">
+      <c r="Q15" s="38">
         <f>100*C15/(0.3*MIN(E15,F15))</f>
         <v/>
       </c>
-      <c r="R15" s="16" t="n">
-        <v>49.7</v>
+      <c r="R15" s="9" t="n">
+        <v>42.67</v>
+      </c>
+    </row>
+    <row r="16" ht="17" customHeight="1">
+      <c r="A16" s="27" t="n"/>
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="D16" s="39" t="n">
+        <v>54.93</v>
+      </c>
+      <c r="E16" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="F16" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="G16" s="18">
+        <f>E16*F16</f>
+        <v/>
+      </c>
+      <c r="H16" s="30">
+        <f>Datos_columnas!$B$8*G16</f>
+        <v/>
+      </c>
+      <c r="I16" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="J16" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="K16" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="L16" s="18">
+        <f>FLOOR(MIN(12*J16/10,48*K16/10,MIN(E16,F16)),5)</f>
+        <v/>
+      </c>
+      <c r="M16" s="18">
+        <f>IF(D16="","FALTA CARGA",IF(O16&lt;H16,"ARM. INSUFIC.",IF(D16&gt;P16,"NO VERIFICA",IF(D16&gt;0.85*P16,"AL LIMITE",IF(Q16&gt;34,"VERIF. ESBELTEZ","VERIFICA")))))</f>
+        <v/>
+      </c>
+      <c r="N16" s="20" t="inlineStr">
+        <is>
+          <t>COL 02 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5).</t>
+        </is>
+      </c>
+      <c r="O16" s="16">
+        <f>I16*PI()*(J16/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="P16" s="16">
+        <f>Datos_columnas!$B$7*0.8*(0.85*Datos_columnas!$B$4*(G16-O16)+Datos_columnas!$B$5*O16)/1000</f>
+        <v/>
+      </c>
+      <c r="Q16" s="40">
+        <f>100*C16/(0.3*MIN(E16,F16))</f>
+        <v/>
+      </c>
+      <c r="R16" s="16" t="n">
+        <v>54.93</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="A4:A7"/>
     <mergeCell ref="E2:G2"/>
-    <mergeCell ref="A8:A15"/>
     <mergeCell ref="N2:N3"/>
+    <mergeCell ref="A8:A16"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="H2:J2"/>
@@ -11953,7 +12034,7 @@
     <mergeCell ref="M2:M3"/>
     <mergeCell ref="O2:R2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M4:M15">
+  <conditionalFormatting sqref="M4:M16">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"VERIFICA"</formula>
     </cfRule>
@@ -11974,7 +12055,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J15 K4:K15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J16 K4:K16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"6,8,10,12,16,20,25"</formula1>
     </dataValidation>
   </dataValidations>
@@ -15481,7 +15562,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>C4 (15x30)</t>
+          <t>C5 (15x30)</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
@@ -15599,7 +15680,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>C4 (10x10)</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
@@ -15616,7 +15697,9 @@
       <c r="F8" s="10" t="n">
         <v>65</v>
       </c>
-      <c r="G8" s="8" t="n"/>
+      <c r="G8" s="8" t="n">
+        <v>10.28</v>
+      </c>
       <c r="H8" s="25">
         <f>IF(G8="","",G8/1.4)</f>
         <v/>
@@ -15644,7 +15727,7 @@
       </c>
       <c r="O8" s="13" t="inlineStr">
         <is>
-          <t>Cantidad de pilotes deducida de la dimension del cabezal: 70x70 cm.</t>
+          <t>Cantidad de pilotes deducida de la dimension del cabezal: 70x70 cm. Carga tomada de la bajada de la planilla de columnas, que esta incompleta: el valor real es mayor.</t>
         </is>
       </c>
     </row>
@@ -15656,7 +15739,7 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>C5 (20x20)</t>
+          <t>C6 (20x20)</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
@@ -15674,7 +15757,7 @@
         <v>70</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>19.38</v>
+        <v>32.1</v>
       </c>
       <c r="H9" s="25">
         <f>IF(G9="","",G9/1.4)</f>
@@ -15715,7 +15798,7 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>C6 (30x15)</t>
+          <t>C7 (30x15)</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
@@ -15733,7 +15816,7 @@
         <v>70</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>27.95</v>
+        <v>37.78</v>
       </c>
       <c r="H10" s="25">
         <f>IF(G10="","",G10/1.4)</f>
@@ -15774,7 +15857,7 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>C8 (15x30)</t>
+          <t>C9 (15x30)</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
@@ -15792,7 +15875,7 @@
         <v>70</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>49.7</v>
+        <v>54.93</v>
       </c>
       <c r="H11" s="25">
         <f>IF(G11="","",G11/1.4)</f>
@@ -15833,7 +15916,7 @@
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>C7 (15x30)</t>
+          <t>C8 (15x30)</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
@@ -15851,7 +15934,7 @@
         <v>70</v>
       </c>
       <c r="G12" s="15" t="n">
-        <v>50.09</v>
+        <v>42.67</v>
       </c>
       <c r="H12" s="30">
         <f>IF(G12="","",G12/1.4)</f>

</xml_diff>

<commit_message>
Rehacer la hoja de tabiques con el formato y las cargas de la catedra
Mismas columnas que la planilla modelo: carga, altura, dimensiones
A y B, armadura vertical y horizontal. Se cargan las seis cargas de
PB que aporto el proyectista. El area distingue el tabique recto del
tabique en L segun si B es el espesor o la otra ala. Los seis
verifican con mucho margen; T7 a T13 quedan a la espera de su carga.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -16187,27 +16187,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:Q22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="46" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="44" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>TABIQUES DE H°A°        H-21        ACERO 42/50        espesor 12 cm</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TABIQUES  H°A°        H-21        ACERO III        espesor 12 cm</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -16221,6 +16226,11 @@
       <c r="J1" s="2" t="n"/>
       <c r="K1" s="2" t="n"/>
       <c r="L1" s="2" t="n"/>
+      <c r="M1" s="2" t="n"/>
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="2" t="n"/>
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="2" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -16235,34 +16245,43 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>DIMENSIONES</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
           <t>CARGA (t)</t>
         </is>
       </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>ALTURA (m)</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>DIMENSIONES (cm)</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="n"/>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>N por metro (t/m)</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>CAPACIDAD</t>
-        </is>
-      </c>
+          <t>ARMADURA VERTICAL</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="n"/>
       <c r="I2" s="4" t="n"/>
-      <c r="J2" s="4" t="n"/>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>ARMADURA HORIZONTAL</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="n"/>
+      <c r="L2" s="4" t="n"/>
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>VERIFICACION</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="N2" s="4" t="n"/>
+      <c r="O2" s="4" t="n"/>
+      <c r="P2" s="4" t="n"/>
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>OBSERVACIONES</t>
         </is>
@@ -16271,967 +16290,995 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="4" t="n"/>
       <c r="B3" s="4" t="n"/>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>espesor (cm)</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>largo (m)</t>
-        </is>
-      </c>
+      <c r="C3" s="4" t="n"/>
+      <c r="D3" s="4" t="n"/>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>alto (m)</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>cm2</t>
+        </is>
+      </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>esbeltez</t>
+          <t>o</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>reduccion</t>
+          <t>separacion</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>fi Pn (t/m)</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="n"/>
-      <c r="L3" s="4" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>PB   (altura de entrepiso)</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
-      <c r="H4" s="4" t="n"/>
-      <c r="I4" s="4" t="n"/>
-      <c r="J4" s="4" t="n"/>
-      <c r="K4" s="4" t="n"/>
-      <c r="L4" s="4" t="n"/>
+          <t>cm2</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>o</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>separacion</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>area (cm2)</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>sigma (kg/cm2)</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>fi Pn (t)</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>resultado</t>
+        </is>
+      </c>
+      <c r="Q3" s="4" t="n"/>
+    </row>
+    <row r="4" ht="17" customHeight="1">
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t>PB</t>
+        </is>
+      </c>
+      <c r="B4" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="E4" s="10" t="n">
+        <v>365</v>
+      </c>
+      <c r="F4" s="10" t="n">
+        <v>87</v>
+      </c>
+      <c r="G4" s="25">
+        <f>2*(100/I4)*PI()*(H4/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="H4" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="I4" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="J4" s="25">
+        <f>(100/L4)*PI()*(K4/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="K4" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="L4" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="M4" s="38">
+        <f>IF(F4&lt;=12,E4*F4,(E4+F4-12)*12)</f>
+        <v/>
+      </c>
+      <c r="N4" s="9">
+        <f>IF(C4="","",C4*1000/M4)</f>
+        <v/>
+      </c>
+      <c r="O4" s="9">
+        <f>0.55*0.65*Datos_vigas!$B$5*M4*MAX(0,1-(D4*100/(32*12))^2)/1000</f>
+        <v/>
+      </c>
+      <c r="P4" s="11">
+        <f>IF(C4="","FALTA CARGA",IF(C4&lt;=O4,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="Q4" s="11" t="inlineStr"/>
     </row>
     <row r="5" ht="17" customHeight="1">
-      <c r="A5" s="11" t="n"/>
+      <c r="A5" s="26" t="n"/>
       <c r="B5" s="23" t="inlineStr">
         <is>
-          <t>T01a</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="n">
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>420</v>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>85</v>
+      </c>
+      <c r="G5" s="25">
+        <f>2*(100/I5)*PI()*(H5/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="H5" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="I5" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="J5" s="25">
+        <f>(100/L5)*PI()*(K5/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="K5" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="L5" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="M5" s="38">
+        <f>IF(F5&lt;=12,E5*F5,(E5+F5-12)*12)</f>
+        <v/>
+      </c>
+      <c r="N5" s="9">
+        <f>IF(C5="","",C5*1000/M5)</f>
+        <v/>
+      </c>
+      <c r="O5" s="9">
+        <f>0.55*0.65*Datos_vigas!$B$5*M5*MAX(0,1-(D5*100/(32*12))^2)/1000</f>
+        <v/>
+      </c>
+      <c r="P5" s="11">
+        <f>IF(C5="","FALTA CARGA",IF(C5&lt;=O5,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="Q5" s="11" t="inlineStr"/>
+    </row>
+    <row r="6" ht="17" customHeight="1">
+      <c r="A6" s="26" t="n"/>
+      <c r="B6" s="23" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>80</v>
+      </c>
+      <c r="F6" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="D5" s="8" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="E5" s="8" t="n">
+      <c r="G6" s="25">
+        <f>2*(100/I6)*PI()*(H6/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="I6" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="J6" s="25">
+        <f>(100/L6)*PI()*(K6/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="K6" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="L6" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="M6" s="38">
+        <f>IF(F6&lt;=12,E6*F6,(E6+F6-12)*12)</f>
+        <v/>
+      </c>
+      <c r="N6" s="9">
+        <f>IF(C6="","",C6*1000/M6)</f>
+        <v/>
+      </c>
+      <c r="O6" s="9">
+        <f>0.55*0.65*Datos_vigas!$B$5*M6*MAX(0,1-(D6*100/(32*12))^2)/1000</f>
+        <v/>
+      </c>
+      <c r="P6" s="11">
+        <f>IF(C6="","FALTA CARGA",IF(C6&lt;=O6,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="Q6" s="13" t="inlineStr">
+        <is>
+          <t>Tabique recto: B = 12 cm es el espesor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="17" customHeight="1">
+      <c r="A7" s="26" t="n"/>
+      <c r="B7" s="23" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" s="8" t="n">
         <v>3.15</v>
       </c>
-      <c r="F5" s="8" t="n">
-        <v>6.16</v>
-      </c>
-      <c r="G5" s="25">
-        <f>IF(F5="","",F5/D5)</f>
-        <v/>
-      </c>
-      <c r="H5" s="38">
-        <f>E5*100/C5</f>
-        <v/>
-      </c>
-      <c r="I5" s="33">
-        <f>MAX(0,1-(E5*100/(32*C5))^2)</f>
-        <v/>
-      </c>
-      <c r="J5" s="9">
-        <f>0.55*0.65*Datos_vigas!$B$5*(100*C5)*I5/1000</f>
-        <v/>
-      </c>
-      <c r="K5" s="11">
-        <f>IF(G5="","FALTA CARGA",IF(G5&lt;=J5,"VERIFICA","NO VERIFICA"))</f>
-        <v/>
-      </c>
-      <c r="L5" s="13" t="inlineStr">
-        <is>
-          <t>Recibe el extremo de VI 01a.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="17" customHeight="1">
-      <c r="A6" s="11" t="n"/>
-      <c r="B6" s="23" t="inlineStr">
-        <is>
-          <t>T01b</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="n">
+      <c r="E7" s="10" t="n">
+        <v>355</v>
+      </c>
+      <c r="F7" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="D6" s="8" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="E6" s="8" t="n">
+      <c r="G7" s="25">
+        <f>2*(100/I7)*PI()*(H7/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="H7" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="I7" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="J7" s="25">
+        <f>(100/L7)*PI()*(K7/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="K7" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="L7" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="M7" s="38">
+        <f>IF(F7&lt;=12,E7*F7,(E7+F7-12)*12)</f>
+        <v/>
+      </c>
+      <c r="N7" s="9">
+        <f>IF(C7="","",C7*1000/M7)</f>
+        <v/>
+      </c>
+      <c r="O7" s="9">
+        <f>0.55*0.65*Datos_vigas!$B$5*M7*MAX(0,1-(D7*100/(32*12))^2)/1000</f>
+        <v/>
+      </c>
+      <c r="P7" s="11">
+        <f>IF(C7="","FALTA CARGA",IF(C7&lt;=O7,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="Q7" s="13" t="inlineStr">
+        <is>
+          <t>Tabique recto: B = 12 cm es el espesor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17" customHeight="1">
+      <c r="A8" s="26" t="n"/>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="D8" s="8" t="n">
         <v>3.15</v>
       </c>
-      <c r="F6" s="42" t="n"/>
-      <c r="G6" s="25">
-        <f>IF(F6="","",F6/D6)</f>
-        <v/>
-      </c>
-      <c r="H6" s="38">
-        <f>E6*100/C6</f>
-        <v/>
-      </c>
-      <c r="I6" s="33">
-        <f>MAX(0,1-(E6*100/(32*C6))^2)</f>
-        <v/>
-      </c>
-      <c r="J6" s="9">
-        <f>0.55*0.65*Datos_vigas!$B$5*(100*C6)*I6/1000</f>
-        <v/>
-      </c>
-      <c r="K6" s="11">
-        <f>IF(G6="","FALTA CARGA",IF(G6&lt;=J6,"VERIFICA","NO VERIFICA"))</f>
-        <v/>
-      </c>
-      <c r="L6" s="13" t="inlineStr">
-        <is>
-          <t>Falta la carga que recibe. Mientras tanto no se puede verificar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="11" t="n"/>
-      <c r="B7" s="23" t="inlineStr">
-        <is>
-          <t>T02</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="n">
+      <c r="E8" s="10" t="n">
+        <v>400</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>300</v>
+      </c>
+      <c r="G8" s="25">
+        <f>2*(100/I8)*PI()*(H8/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="I8" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="J8" s="25">
+        <f>(100/L8)*PI()*(K8/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="K8" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="L8" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="M8" s="38">
+        <f>IF(F8&lt;=12,E8*F8,(E8+F8-12)*12)</f>
+        <v/>
+      </c>
+      <c r="N8" s="9">
+        <f>IF(C8="","",C8*1000/M8)</f>
+        <v/>
+      </c>
+      <c r="O8" s="9">
+        <f>0.55*0.65*Datos_vigas!$B$5*M8*MAX(0,1-(D8*100/(32*12))^2)/1000</f>
+        <v/>
+      </c>
+      <c r="P8" s="11">
+        <f>IF(C8="","FALTA CARGA",IF(C8&lt;=O8,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="Q8" s="13" t="inlineStr">
+        <is>
+          <t>El mas cargado del conjunto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="17" customHeight="1">
+      <c r="A9" s="26" t="n"/>
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>T6</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="E9" s="10" t="n">
+        <v>270</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>90</v>
+      </c>
+      <c r="G9" s="25">
+        <f>2*(100/I9)*PI()*(H9/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="H9" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="I9" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="J9" s="25">
+        <f>(100/L9)*PI()*(K9/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="K9" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="L9" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="M9" s="38">
+        <f>IF(F9&lt;=12,E9*F9,(E9+F9-12)*12)</f>
+        <v/>
+      </c>
+      <c r="N9" s="9">
+        <f>IF(C9="","",C9*1000/M9)</f>
+        <v/>
+      </c>
+      <c r="O9" s="9">
+        <f>0.55*0.65*Datos_vigas!$B$5*M9*MAX(0,1-(D9*100/(32*12))^2)/1000</f>
+        <v/>
+      </c>
+      <c r="P9" s="11">
+        <f>IF(C9="","FALTA CARGA",IF(C9&lt;=O9,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="Q9" s="11" t="inlineStr"/>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="A10" s="26" t="n"/>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="C10" s="42" t="n"/>
+      <c r="D10" s="8" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>98</v>
+      </c>
+      <c r="F10" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="D7" s="8" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="E7" s="8" t="n">
+      <c r="G10" s="25">
+        <f>2*(100/I10)*PI()*(H10/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="H10" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="I10" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="J10" s="25">
+        <f>(100/L10)*PI()*(K10/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="K10" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="L10" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="M10" s="38">
+        <f>IF(F10&lt;=12,E10*F10,(E10+F10-12)*12)</f>
+        <v/>
+      </c>
+      <c r="N10" s="9">
+        <f>IF(C10="","",C10*1000/M10)</f>
+        <v/>
+      </c>
+      <c r="O10" s="9">
+        <f>0.55*0.65*Datos_vigas!$B$5*M10*MAX(0,1-(D10*100/(32*12))^2)/1000</f>
+        <v/>
+      </c>
+      <c r="P10" s="11">
+        <f>IF(C10="","FALTA CARGA",IF(C10&lt;=O10,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="Q10" s="13" t="inlineStr">
+        <is>
+          <t>Recibe el extremo de VI 02. Carga estimada por la bajada de vigas: 21,1 t. Falta la carga: no figura en la planilla de la catedra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="27" t="n"/>
+      <c r="B11" s="28" t="inlineStr">
+        <is>
+          <t>T8</t>
+        </is>
+      </c>
+      <c r="C11" s="43" t="n"/>
+      <c r="D11" s="15" t="n">
         <v>3.15</v>
       </c>
-      <c r="F7" s="42" t="n"/>
-      <c r="G7" s="25">
-        <f>IF(F7="","",F7/D7)</f>
-        <v/>
-      </c>
-      <c r="H7" s="38">
-        <f>E7*100/C7</f>
-        <v/>
-      </c>
-      <c r="I7" s="33">
-        <f>MAX(0,1-(E7*100/(32*C7))^2)</f>
-        <v/>
-      </c>
-      <c r="J7" s="9">
-        <f>0.55*0.65*Datos_vigas!$B$5*(100*C7)*I7/1000</f>
-        <v/>
-      </c>
-      <c r="K7" s="11">
-        <f>IF(G7="","FALTA CARGA",IF(G7&lt;=J7,"VERIFICA","NO VERIFICA"))</f>
-        <v/>
-      </c>
-      <c r="L7" s="13" t="inlineStr">
-        <is>
-          <t>Falta la carga que recibe. Mientras tanto no se puede verificar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="11" t="n"/>
-      <c r="B8" s="23" t="inlineStr">
-        <is>
-          <t>T03</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="n">
+      <c r="E11" s="17" t="n">
+        <v>290</v>
+      </c>
+      <c r="F11" s="17" t="n">
         <v>12</v>
       </c>
-      <c r="D8" s="8" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="E8" s="8" t="n">
-        <v>3.15</v>
-      </c>
-      <c r="F8" s="42" t="n"/>
-      <c r="G8" s="25">
-        <f>IF(F8="","",F8/D8)</f>
-        <v/>
-      </c>
-      <c r="H8" s="38">
-        <f>E8*100/C8</f>
-        <v/>
-      </c>
-      <c r="I8" s="33">
-        <f>MAX(0,1-(E8*100/(32*C8))^2)</f>
-        <v/>
-      </c>
-      <c r="J8" s="9">
-        <f>0.55*0.65*Datos_vigas!$B$5*(100*C8)*I8/1000</f>
-        <v/>
-      </c>
-      <c r="K8" s="11">
-        <f>IF(G8="","FALTA CARGA",IF(G8&lt;=J8,"VERIFICA","NO VERIFICA"))</f>
-        <v/>
-      </c>
-      <c r="L8" s="13" t="inlineStr">
-        <is>
-          <t>No se habia detectado en el plano: aparece en el computo. Falta la carga que recibe. Mientras tanto no se puede verificar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="17" customHeight="1">
-      <c r="A9" s="11" t="n"/>
-      <c r="B9" s="23" t="inlineStr">
-        <is>
-          <t>T04a</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="n">
+      <c r="G11" s="30">
+        <f>2*(100/I11)*PI()*(H11/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="H11" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="I11" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="J11" s="30">
+        <f>(100/L11)*PI()*(K11/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="K11" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="L11" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="M11" s="40">
+        <f>IF(F11&lt;=12,E11*F11,(E11+F11-12)*12)</f>
+        <v/>
+      </c>
+      <c r="N11" s="16">
+        <f>IF(C11="","",C11*1000/M11)</f>
+        <v/>
+      </c>
+      <c r="O11" s="16">
+        <f>0.55*0.65*Datos_vigas!$B$5*M11*MAX(0,1-(D11*100/(32*12))^2)/1000</f>
+        <v/>
+      </c>
+      <c r="P11" s="18">
+        <f>IF(C11="","FALTA CARGA",IF(C11&lt;=O11,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="Q11" s="20" t="inlineStr">
+        <is>
+          <t>Recibe el extremo de VI 11a. Carga estimada por la bajada de vigas: 14,6 t. Falta la carga: no figura en la planilla de la catedra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
+      <c r="A12" s="22" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="inlineStr">
+        <is>
+          <t>T9</t>
+        </is>
+      </c>
+      <c r="C12" s="42" t="n"/>
+      <c r="D12" s="8" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E12" s="10" t="n">
+        <v>375</v>
+      </c>
+      <c r="F12" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="D9" s="8" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="E9" s="8" t="n">
-        <v>3.15</v>
-      </c>
-      <c r="F9" s="42" t="n"/>
-      <c r="G9" s="25">
-        <f>IF(F9="","",F9/D9)</f>
-        <v/>
-      </c>
-      <c r="H9" s="38">
-        <f>E9*100/C9</f>
-        <v/>
-      </c>
-      <c r="I9" s="33">
-        <f>MAX(0,1-(E9*100/(32*C9))^2)</f>
-        <v/>
-      </c>
-      <c r="J9" s="9">
-        <f>0.55*0.65*Datos_vigas!$B$5*(100*C9)*I9/1000</f>
-        <v/>
-      </c>
-      <c r="K9" s="11">
-        <f>IF(G9="","FALTA CARGA",IF(G9&lt;=J9,"VERIFICA","NO VERIFICA"))</f>
-        <v/>
-      </c>
-      <c r="L9" s="13" t="inlineStr">
-        <is>
-          <t>Falta la carga que recibe. Mientras tanto no se puede verificar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="17" customHeight="1">
-      <c r="A10" s="11" t="n"/>
-      <c r="B10" s="23" t="inlineStr">
-        <is>
-          <t>T04b</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="n">
+      <c r="G12" s="25">
+        <f>2*(100/I12)*PI()*(H12/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="I12" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="J12" s="25">
+        <f>(100/L12)*PI()*(K12/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="K12" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="L12" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="M12" s="38">
+        <f>IF(F12&lt;=12,E12*F12,(E12+F12-12)*12)</f>
+        <v/>
+      </c>
+      <c r="N12" s="9">
+        <f>IF(C12="","",C12*1000/M12)</f>
+        <v/>
+      </c>
+      <c r="O12" s="9">
+        <f>0.55*0.65*Datos_vigas!$B$5*M12*MAX(0,1-(D12*100/(32*12))^2)/1000</f>
+        <v/>
+      </c>
+      <c r="P12" s="11">
+        <f>IF(C12="","FALTA CARGA",IF(C12&lt;=O12,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="Q12" s="13" t="inlineStr">
+        <is>
+          <t>Falta la carga: no figura en la planilla de la catedra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="17" customHeight="1">
+      <c r="A13" s="26" t="n"/>
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="C13" s="42" t="n"/>
+      <c r="D13" s="8" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E13" s="10" t="n">
+        <v>170</v>
+      </c>
+      <c r="F13" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="D10" s="8" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="E10" s="8" t="n">
-        <v>3.15</v>
-      </c>
-      <c r="F10" s="42" t="n"/>
-      <c r="G10" s="25">
-        <f>IF(F10="","",F10/D10)</f>
-        <v/>
-      </c>
-      <c r="H10" s="38">
-        <f>E10*100/C10</f>
-        <v/>
-      </c>
-      <c r="I10" s="33">
-        <f>MAX(0,1-(E10*100/(32*C10))^2)</f>
-        <v/>
-      </c>
-      <c r="J10" s="9">
-        <f>0.55*0.65*Datos_vigas!$B$5*(100*C10)*I10/1000</f>
-        <v/>
-      </c>
-      <c r="K10" s="11">
-        <f>IF(G10="","FALTA CARGA",IF(G10&lt;=J10,"VERIFICA","NO VERIFICA"))</f>
-        <v/>
-      </c>
-      <c r="L10" s="13" t="inlineStr">
-        <is>
-          <t>En el plano solo figura en la planta de fundacion. Falta la carga que recibe. Mientras tanto no se puede verificar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="17" customHeight="1">
-      <c r="A11" s="11" t="n"/>
-      <c r="B11" s="23" t="inlineStr">
-        <is>
-          <t>T05a</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="n">
+      <c r="G13" s="25">
+        <f>2*(100/I13)*PI()*(H13/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="I13" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="J13" s="25">
+        <f>(100/L13)*PI()*(K13/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="K13" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="L13" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="M13" s="38">
+        <f>IF(F13&lt;=12,E13*F13,(E13+F13-12)*12)</f>
+        <v/>
+      </c>
+      <c r="N13" s="9">
+        <f>IF(C13="","",C13*1000/M13)</f>
+        <v/>
+      </c>
+      <c r="O13" s="9">
+        <f>0.55*0.65*Datos_vigas!$B$5*M13*MAX(0,1-(D13*100/(32*12))^2)/1000</f>
+        <v/>
+      </c>
+      <c r="P13" s="11">
+        <f>IF(C13="","FALTA CARGA",IF(C13&lt;=O13,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="Q13" s="13" t="inlineStr">
+        <is>
+          <t>Falta la carga: no figura en la planilla de la catedra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" s="26" t="n"/>
+      <c r="B14" s="23" t="inlineStr">
+        <is>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="C14" s="42" t="n"/>
+      <c r="D14" s="8" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E14" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="F14" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="D11" s="8" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="E11" s="8" t="n">
-        <v>3.15</v>
-      </c>
-      <c r="F11" s="42" t="n"/>
-      <c r="G11" s="25">
-        <f>IF(F11="","",F11/D11)</f>
-        <v/>
-      </c>
-      <c r="H11" s="38">
-        <f>E11*100/C11</f>
-        <v/>
-      </c>
-      <c r="I11" s="33">
-        <f>MAX(0,1-(E11*100/(32*C11))^2)</f>
-        <v/>
-      </c>
-      <c r="J11" s="9">
-        <f>0.55*0.65*Datos_vigas!$B$5*(100*C11)*I11/1000</f>
-        <v/>
-      </c>
-      <c r="K11" s="11">
-        <f>IF(G11="","FALTA CARGA",IF(G11&lt;=J11,"VERIFICA","NO VERIFICA"))</f>
-        <v/>
-      </c>
-      <c r="L11" s="13" t="inlineStr">
-        <is>
-          <t>Falta la carga que recibe. Mientras tanto no se puede verificar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="17" customHeight="1">
-      <c r="A12" s="11" t="n"/>
-      <c r="B12" s="23" t="inlineStr">
-        <is>
-          <t>T05b</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="n">
+      <c r="G14" s="25">
+        <f>2*(100/I14)*PI()*(H14/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="I14" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="J14" s="25">
+        <f>(100/L14)*PI()*(K14/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="K14" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="L14" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="M14" s="38">
+        <f>IF(F14&lt;=12,E14*F14,(E14+F14-12)*12)</f>
+        <v/>
+      </c>
+      <c r="N14" s="9">
+        <f>IF(C14="","",C14*1000/M14)</f>
+        <v/>
+      </c>
+      <c r="O14" s="9">
+        <f>0.55*0.65*Datos_vigas!$B$5*M14*MAX(0,1-(D14*100/(32*12))^2)/1000</f>
+        <v/>
+      </c>
+      <c r="P14" s="11">
+        <f>IF(C14="","FALTA CARGA",IF(C14&lt;=O14,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="Q14" s="13" t="inlineStr">
+        <is>
+          <t>Longitud muy corta: verificar si es tabique o el machon de una abertura. Falta la carga: no figura en la planilla de la catedra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" s="26" t="n"/>
+      <c r="B15" s="23" t="inlineStr">
+        <is>
+          <t>T12</t>
+        </is>
+      </c>
+      <c r="C15" s="42" t="n"/>
+      <c r="D15" s="8" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E15" s="10" t="n">
+        <v>32</v>
+      </c>
+      <c r="F15" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="D12" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E12" s="8" t="n">
-        <v>3.15</v>
-      </c>
-      <c r="F12" s="8" t="n">
-        <v>25.47</v>
-      </c>
-      <c r="G12" s="25">
-        <f>IF(F12="","",F12/D12)</f>
-        <v/>
-      </c>
-      <c r="H12" s="38">
-        <f>E12*100/C12</f>
-        <v/>
-      </c>
-      <c r="I12" s="33">
-        <f>MAX(0,1-(E12*100/(32*C12))^2)</f>
-        <v/>
-      </c>
-      <c r="J12" s="9">
-        <f>0.55*0.65*Datos_vigas!$B$5*(100*C12)*I12/1000</f>
-        <v/>
-      </c>
-      <c r="K12" s="11">
-        <f>IF(G12="","FALTA CARGA",IF(G12&lt;=J12,"VERIFICA","NO VERIFICA"))</f>
-        <v/>
-      </c>
-      <c r="L12" s="13" t="inlineStr">
-        <is>
-          <t>Recibe el extremo de VI 07c.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="17" customHeight="1">
-      <c r="A13" s="11" t="n"/>
-      <c r="B13" s="23" t="inlineStr">
-        <is>
-          <t>T06a</t>
-        </is>
-      </c>
-      <c r="C13" s="10" t="n">
+      <c r="G15" s="25">
+        <f>2*(100/I15)*PI()*(H15/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="I15" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="J15" s="25">
+        <f>(100/L15)*PI()*(K15/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="K15" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="L15" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="M15" s="38">
+        <f>IF(F15&lt;=12,E15*F15,(E15+F15-12)*12)</f>
+        <v/>
+      </c>
+      <c r="N15" s="9">
+        <f>IF(C15="","",C15*1000/M15)</f>
+        <v/>
+      </c>
+      <c r="O15" s="9">
+        <f>0.55*0.65*Datos_vigas!$B$5*M15*MAX(0,1-(D15*100/(32*12))^2)/1000</f>
+        <v/>
+      </c>
+      <c r="P15" s="11">
+        <f>IF(C15="","FALTA CARGA",IF(C15&lt;=O15,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="Q15" s="13" t="inlineStr">
+        <is>
+          <t>Longitud muy corta: verificar si es tabique o el machon de una abertura. Falta la carga: no figura en la planilla de la catedra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="17" customHeight="1">
+      <c r="A16" s="27" t="n"/>
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>T13</t>
+        </is>
+      </c>
+      <c r="C16" s="43" t="n"/>
+      <c r="D16" s="15" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E16" s="17" t="n">
+        <v>132</v>
+      </c>
+      <c r="F16" s="17" t="n">
         <v>12</v>
       </c>
-      <c r="D13" s="8" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="E13" s="8" t="n">
-        <v>3.15</v>
-      </c>
-      <c r="F13" s="42" t="n"/>
-      <c r="G13" s="25">
-        <f>IF(F13="","",F13/D13)</f>
-        <v/>
-      </c>
-      <c r="H13" s="38">
-        <f>E13*100/C13</f>
-        <v/>
-      </c>
-      <c r="I13" s="33">
-        <f>MAX(0,1-(E13*100/(32*C13))^2)</f>
-        <v/>
-      </c>
-      <c r="J13" s="9">
-        <f>0.55*0.65*Datos_vigas!$B$5*(100*C13)*I13/1000</f>
-        <v/>
-      </c>
-      <c r="K13" s="11">
-        <f>IF(G13="","FALTA CARGA",IF(G13&lt;=J13,"VERIFICA","NO VERIFICA"))</f>
-        <v/>
-      </c>
-      <c r="L13" s="13" t="inlineStr">
-        <is>
-          <t>Falta la carga que recibe. Mientras tanto no se puede verificar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="17" customHeight="1">
-      <c r="A14" s="11" t="n"/>
-      <c r="B14" s="23" t="inlineStr">
-        <is>
-          <t>T06b</t>
-        </is>
-      </c>
-      <c r="C14" s="10" t="n">
-        <v>12</v>
-      </c>
-      <c r="D14" s="8" t="n">
-        <v>5.55</v>
-      </c>
-      <c r="E14" s="8" t="n">
-        <v>3.15</v>
-      </c>
-      <c r="F14" s="42" t="n"/>
-      <c r="G14" s="25">
-        <f>IF(F14="","",F14/D14)</f>
-        <v/>
-      </c>
-      <c r="H14" s="38">
-        <f>E14*100/C14</f>
-        <v/>
-      </c>
-      <c r="I14" s="33">
-        <f>MAX(0,1-(E14*100/(32*C14))^2)</f>
-        <v/>
-      </c>
-      <c r="J14" s="9">
-        <f>0.55*0.65*Datos_vigas!$B$5*(100*C14)*I14/1000</f>
-        <v/>
-      </c>
-      <c r="K14" s="11">
-        <f>IF(G14="","FALTA CARGA",IF(G14&lt;=J14,"VERIFICA","NO VERIFICA"))</f>
-        <v/>
-      </c>
-      <c r="L14" s="13" t="inlineStr">
-        <is>
-          <t>Perpendicular a las vigas chatas, en la union de VCH 03a con VCH 03b. Falta la carga que recibe. Mientras tanto no se puede verificar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="11" t="n"/>
-      <c r="B15" s="23" t="inlineStr">
-        <is>
-          <t>T06c</t>
-        </is>
-      </c>
-      <c r="C15" s="10" t="n">
-        <v>12</v>
-      </c>
-      <c r="D15" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="8" t="n">
-        <v>3.15</v>
-      </c>
-      <c r="F15" s="42" t="n"/>
-      <c r="G15" s="25">
-        <f>IF(F15="","",F15/D15)</f>
-        <v/>
-      </c>
-      <c r="H15" s="38">
-        <f>E15*100/C15</f>
-        <v/>
-      </c>
-      <c r="I15" s="33">
-        <f>MAX(0,1-(E15*100/(32*C15))^2)</f>
-        <v/>
-      </c>
-      <c r="J15" s="9">
-        <f>0.55*0.65*Datos_vigas!$B$5*(100*C15)*I15/1000</f>
-        <v/>
-      </c>
-      <c r="K15" s="11">
-        <f>IF(G15="","FALTA CARGA",IF(G15&lt;=J15,"VERIFICA","NO VERIFICA"))</f>
-        <v/>
-      </c>
-      <c r="L15" s="13" t="inlineStr">
-        <is>
-          <t>Falta la carga que recibe. Mientras tanto no se puede verificar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="17" customHeight="1">
-      <c r="A16" s="11" t="n"/>
-      <c r="B16" s="23" t="inlineStr">
-        <is>
-          <t>T07</t>
-        </is>
-      </c>
-      <c r="C16" s="10" t="n">
-        <v>12</v>
-      </c>
-      <c r="D16" s="8" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="E16" s="8" t="n">
-        <v>3.15</v>
-      </c>
-      <c r="F16" s="8" t="n">
-        <v>21.12</v>
-      </c>
-      <c r="G16" s="25">
-        <f>IF(F16="","",F16/D16)</f>
-        <v/>
-      </c>
-      <c r="H16" s="38">
-        <f>E16*100/C16</f>
-        <v/>
-      </c>
-      <c r="I16" s="33">
-        <f>MAX(0,1-(E16*100/(32*C16))^2)</f>
-        <v/>
-      </c>
-      <c r="J16" s="9">
-        <f>0.55*0.65*Datos_vigas!$B$5*(100*C16)*I16/1000</f>
-        <v/>
-      </c>
-      <c r="K16" s="11">
-        <f>IF(G16="","FALTA CARGA",IF(G16&lt;=J16,"VERIFICA","NO VERIFICA"))</f>
-        <v/>
-      </c>
-      <c r="L16" s="13" t="inlineStr">
-        <is>
-          <t>Recibe el extremo de VI 02, perpendicular.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="17" customHeight="1">
-      <c r="A17" s="11" t="n"/>
-      <c r="B17" s="23" t="inlineStr">
-        <is>
-          <t>T08a</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="n">
-        <v>12</v>
-      </c>
-      <c r="D17" s="8" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="E17" s="8" t="n">
-        <v>3.15</v>
-      </c>
-      <c r="F17" s="8" t="n">
-        <v>14.6</v>
-      </c>
-      <c r="G17" s="25">
-        <f>IF(F17="","",F17/D17)</f>
-        <v/>
-      </c>
-      <c r="H17" s="38">
-        <f>E17*100/C17</f>
-        <v/>
-      </c>
-      <c r="I17" s="33">
-        <f>MAX(0,1-(E17*100/(32*C17))^2)</f>
-        <v/>
-      </c>
-      <c r="J17" s="9">
-        <f>0.55*0.65*Datos_vigas!$B$5*(100*C17)*I17/1000</f>
-        <v/>
-      </c>
-      <c r="K17" s="11">
-        <f>IF(G17="","FALTA CARGA",IF(G17&lt;=J17,"VERIFICA","NO VERIFICA"))</f>
-        <v/>
-      </c>
-      <c r="L17" s="13" t="inlineStr">
-        <is>
-          <t>Recibe el extremo de VI 11a.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="17" customHeight="1">
-      <c r="A18" s="18" t="n"/>
-      <c r="B18" s="28" t="inlineStr">
-        <is>
-          <t>T08b</t>
-        </is>
-      </c>
-      <c r="C18" s="17" t="n">
-        <v>12</v>
-      </c>
-      <c r="D18" s="15" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="E18" s="15" t="n">
-        <v>3.15</v>
-      </c>
-      <c r="F18" s="43" t="n"/>
-      <c r="G18" s="30">
-        <f>IF(F18="","",F18/D18)</f>
-        <v/>
-      </c>
-      <c r="H18" s="40">
-        <f>E18*100/C18</f>
-        <v/>
-      </c>
-      <c r="I18" s="35">
-        <f>MAX(0,1-(E18*100/(32*C18))^2)</f>
-        <v/>
-      </c>
-      <c r="J18" s="16">
-        <f>0.55*0.65*Datos_vigas!$B$5*(100*C18)*I18/1000</f>
-        <v/>
-      </c>
-      <c r="K18" s="18">
-        <f>IF(G18="","FALTA CARGA",IF(G18&lt;=J18,"VERIFICA","NO VERIFICA"))</f>
-        <v/>
-      </c>
-      <c r="L18" s="20" t="inlineStr">
-        <is>
-          <t>Falta la carga que recibe. Mientras tanto no se puede verificar.</t>
-        </is>
-      </c>
+      <c r="G16" s="30">
+        <f>2*(100/I16)*PI()*(H16/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="H16" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="I16" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="J16" s="30">
+        <f>(100/L16)*PI()*(K16/10)^2/4</f>
+        <v/>
+      </c>
+      <c r="K16" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="L16" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="M16" s="40">
+        <f>IF(F16&lt;=12,E16*F16,(E16+F16-12)*12)</f>
+        <v/>
+      </c>
+      <c r="N16" s="16">
+        <f>IF(C16="","",C16*1000/M16)</f>
+        <v/>
+      </c>
+      <c r="O16" s="16">
+        <f>0.55*0.65*Datos_vigas!$B$5*M16*MAX(0,1-(D16*100/(32*12))^2)/1000</f>
+        <v/>
+      </c>
+      <c r="P16" s="18">
+        <f>IF(C16="","FALTA CARGA",IF(C16&lt;=O16,"VERIFICA","NO VERIFICA"))</f>
+        <v/>
+      </c>
+      <c r="Q16" s="20" t="inlineStr">
+        <is>
+          <t>Falta la carga: no figura en la planilla de la catedra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n"/>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
+      <c r="J17" s="2" t="n"/>
+      <c r="K17" s="2" t="n"/>
+      <c r="L17" s="2" t="n"/>
+      <c r="M17" s="2" t="n"/>
+      <c r="N17" s="2" t="n"/>
+      <c r="O17" s="2" t="n"/>
+      <c r="P17" s="2" t="n"/>
+      <c r="Q17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="44" t="inlineStr">
+        <is>
+          <t>T1 a T6: cargas y dimensiones tomadas de la planilla de la catedra.</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="n"/>
+      <c r="J18" s="2" t="n"/>
+      <c r="K18" s="2" t="n"/>
+      <c r="L18" s="2" t="n"/>
+      <c r="M18" s="2" t="n"/>
+      <c r="N18" s="2" t="n"/>
+      <c r="O18" s="2" t="n"/>
+      <c r="P18" s="2" t="n"/>
+      <c r="Q18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>PA   (altura de entrepiso)</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="n"/>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="4" t="n"/>
-      <c r="E19" s="4" t="n"/>
-      <c r="F19" s="4" t="n"/>
-      <c r="G19" s="4" t="n"/>
-      <c r="H19" s="4" t="n"/>
-      <c r="I19" s="4" t="n"/>
-      <c r="J19" s="4" t="n"/>
-      <c r="K19" s="4" t="n"/>
-      <c r="L19" s="4" t="n"/>
-    </row>
-    <row r="20" ht="17" customHeight="1">
-      <c r="A20" s="11" t="n"/>
-      <c r="B20" s="23" t="inlineStr">
-        <is>
-          <t>T09</t>
-        </is>
-      </c>
-      <c r="C20" s="10" t="n">
-        <v>12</v>
-      </c>
-      <c r="D20" s="8" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="E20" s="8" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="F20" s="42" t="n"/>
-      <c r="G20" s="25">
-        <f>IF(F20="","",F20/D20)</f>
-        <v/>
-      </c>
-      <c r="H20" s="38">
-        <f>E20*100/C20</f>
-        <v/>
-      </c>
-      <c r="I20" s="33">
-        <f>MAX(0,1-(E20*100/(32*C20))^2)</f>
-        <v/>
-      </c>
-      <c r="J20" s="9">
-        <f>0.55*0.65*Datos_vigas!$B$5*(100*C20)*I20/1000</f>
-        <v/>
-      </c>
-      <c r="K20" s="11">
-        <f>IF(G20="","FALTA CARGA",IF(G20&lt;=J20,"VERIFICA","NO VERIFICA"))</f>
-        <v/>
-      </c>
-      <c r="L20" s="13" t="inlineStr">
-        <is>
-          <t>Falta la carga que recibe. Mientras tanto no se puede verificar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="17" customHeight="1">
-      <c r="A21" s="11" t="n"/>
-      <c r="B21" s="23" t="inlineStr">
-        <is>
-          <t>T10</t>
-        </is>
-      </c>
-      <c r="C21" s="10" t="n">
-        <v>12</v>
-      </c>
-      <c r="D21" s="8" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="E21" s="8" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="F21" s="42" t="n"/>
-      <c r="G21" s="25">
-        <f>IF(F21="","",F21/D21)</f>
-        <v/>
-      </c>
-      <c r="H21" s="38">
-        <f>E21*100/C21</f>
-        <v/>
-      </c>
-      <c r="I21" s="33">
-        <f>MAX(0,1-(E21*100/(32*C21))^2)</f>
-        <v/>
-      </c>
-      <c r="J21" s="9">
-        <f>0.55*0.65*Datos_vigas!$B$5*(100*C21)*I21/1000</f>
-        <v/>
-      </c>
-      <c r="K21" s="11">
-        <f>IF(G21="","FALTA CARGA",IF(G21&lt;=J21,"VERIFICA","NO VERIFICA"))</f>
-        <v/>
-      </c>
-      <c r="L21" s="13" t="inlineStr">
-        <is>
-          <t>Falta la carga que recibe. Mientras tanto no se puede verificar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="17" customHeight="1">
-      <c r="A22" s="11" t="n"/>
-      <c r="B22" s="23" t="inlineStr">
-        <is>
-          <t>T11</t>
-        </is>
-      </c>
-      <c r="C22" s="10" t="n">
-        <v>12</v>
-      </c>
-      <c r="D22" s="8" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="E22" s="8" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="F22" s="42" t="n"/>
-      <c r="G22" s="25">
-        <f>IF(F22="","",F22/D22)</f>
-        <v/>
-      </c>
-      <c r="H22" s="38">
-        <f>E22*100/C22</f>
-        <v/>
-      </c>
-      <c r="I22" s="33">
-        <f>MAX(0,1-(E22*100/(32*C22))^2)</f>
-        <v/>
-      </c>
-      <c r="J22" s="9">
-        <f>0.55*0.65*Datos_vigas!$B$5*(100*C22)*I22/1000</f>
-        <v/>
-      </c>
-      <c r="K22" s="11">
-        <f>IF(G22="","FALTA CARGA",IF(G22&lt;=J22,"VERIFICA","NO VERIFICA"))</f>
-        <v/>
-      </c>
-      <c r="L22" s="13" t="inlineStr">
-        <is>
-          <t>Longitud muy corta: verificar si es un tabique o el machon de una abertura. Falta la carga que recibe. Mientras tanto no se puede verificar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="17" customHeight="1">
-      <c r="A23" s="11" t="n"/>
-      <c r="B23" s="23" t="inlineStr">
-        <is>
-          <t>T12</t>
-        </is>
-      </c>
-      <c r="C23" s="10" t="n">
-        <v>12</v>
-      </c>
-      <c r="D23" s="8" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="E23" s="8" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="F23" s="42" t="n"/>
-      <c r="G23" s="25">
-        <f>IF(F23="","",F23/D23)</f>
-        <v/>
-      </c>
-      <c r="H23" s="38">
-        <f>E23*100/C23</f>
-        <v/>
-      </c>
-      <c r="I23" s="33">
-        <f>MAX(0,1-(E23*100/(32*C23))^2)</f>
-        <v/>
-      </c>
-      <c r="J23" s="9">
-        <f>0.55*0.65*Datos_vigas!$B$5*(100*C23)*I23/1000</f>
-        <v/>
-      </c>
-      <c r="K23" s="11">
-        <f>IF(G23="","FALTA CARGA",IF(G23&lt;=J23,"VERIFICA","NO VERIFICA"))</f>
-        <v/>
-      </c>
-      <c r="L23" s="13" t="inlineStr">
-        <is>
-          <t>Longitud muy corta: verificar si es un tabique o el machon de una abertura. Falta la carga que recibe. Mientras tanto no se puede verificar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="17" customHeight="1">
-      <c r="A24" s="18" t="n"/>
-      <c r="B24" s="28" t="inlineStr">
-        <is>
-          <t>T13</t>
-        </is>
-      </c>
-      <c r="C24" s="17" t="n">
-        <v>12</v>
-      </c>
-      <c r="D24" s="15" t="n">
-        <v>1.32</v>
-      </c>
-      <c r="E24" s="15" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="F24" s="43" t="n"/>
-      <c r="G24" s="30">
-        <f>IF(F24="","",F24/D24)</f>
-        <v/>
-      </c>
-      <c r="H24" s="40">
-        <f>E24*100/C24</f>
-        <v/>
-      </c>
-      <c r="I24" s="35">
-        <f>MAX(0,1-(E24*100/(32*C24))^2)</f>
-        <v/>
-      </c>
-      <c r="J24" s="16">
-        <f>0.55*0.65*Datos_vigas!$B$5*(100*C24)*I24/1000</f>
-        <v/>
-      </c>
-      <c r="K24" s="18">
-        <f>IF(G24="","FALTA CARGA",IF(G24&lt;=J24,"VERIFICA","NO VERIFICA"))</f>
-        <v/>
-      </c>
-      <c r="L24" s="20" t="inlineStr">
-        <is>
-          <t>Falta la carga que recibe. Mientras tanto no se puede verificar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="n"/>
-      <c r="B25" s="2" t="n"/>
-      <c r="C25" s="2" t="n"/>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="n"/>
-      <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="n"/>
-      <c r="I25" s="2" t="n"/>
-      <c r="J25" s="2" t="n"/>
-      <c r="K25" s="2" t="n"/>
-      <c r="L25" s="2" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="41" t="inlineStr">
-        <is>
-          <t>fi Pn = 0,55 x 0,65 x f'c x Ag x [1 - (alto / 32 espesor)^2]    muro portante de hormigon armado, con reduccion por esbeltez.</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="2" t="n"/>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
-      <c r="G26" s="2" t="n"/>
-      <c r="H26" s="2" t="n"/>
-      <c r="I26" s="2" t="n"/>
-      <c r="J26" s="2" t="n"/>
-      <c r="K26" s="2" t="n"/>
-      <c r="L26" s="2" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="44" t="inlineStr">
-        <is>
-          <t>Longitudes tomadas del computo metrico (planilla N 3, item 4.1.10).</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="n"/>
-      <c r="C27" s="2" t="n"/>
-      <c r="D27" s="2" t="n"/>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
-      <c r="G27" s="2" t="n"/>
-      <c r="H27" s="2" t="n"/>
-      <c r="I27" s="2" t="n"/>
-      <c r="J27" s="2" t="n"/>
-      <c r="K27" s="2" t="n"/>
-      <c r="L27" s="2" t="n"/>
+      <c r="A19" s="44" t="inlineStr">
+        <is>
+          <t>T7 a T13: dimensiones del computo metrico; la carga todavia no esta definida.</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="n"/>
+      <c r="J19" s="2" t="n"/>
+      <c r="K19" s="2" t="n"/>
+      <c r="L19" s="2" t="n"/>
+      <c r="M19" s="2" t="n"/>
+      <c r="N19" s="2" t="n"/>
+      <c r="O19" s="2" t="n"/>
+      <c r="P19" s="2" t="n"/>
+      <c r="Q19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="44" t="inlineStr">
+        <is>
+          <t>Area: si B es menor o igual al espesor el tabique es recto y el area es A x B; si no, es un tabique en L y el area es (A + B - espesor) x espesor.</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="n"/>
+      <c r="J20" s="2" t="n"/>
+      <c r="K20" s="2" t="n"/>
+      <c r="L20" s="2" t="n"/>
+      <c r="M20" s="2" t="n"/>
+      <c r="N20" s="2" t="n"/>
+      <c r="O20" s="2" t="n"/>
+      <c r="P20" s="2" t="n"/>
+      <c r="Q20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="44" t="inlineStr">
+        <is>
+          <t>fi Pn = 0,55 x 0,65 x f'c x area x [1 - (altura / 32 espesor)^2]   muro portante de hormigon armado con reduccion por esbeltez.</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
+      <c r="I21" s="2" t="n"/>
+      <c r="J21" s="2" t="n"/>
+      <c r="K21" s="2" t="n"/>
+      <c r="L21" s="2" t="n"/>
+      <c r="M21" s="2" t="n"/>
+      <c r="N21" s="2" t="n"/>
+      <c r="O21" s="2" t="n"/>
+      <c r="P21" s="2" t="n"/>
+      <c r="Q21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="44" t="inlineStr">
+        <is>
+          <t>Armadura vertical en doble malla y horizontal en malla simple, ambas o8 c/20, iguales a las de la planilla de la catedra.</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="n"/>
+      <c r="J22" s="2" t="n"/>
+      <c r="K22" s="2" t="n"/>
+      <c r="L22" s="2" t="n"/>
+      <c r="M22" s="2" t="n"/>
+      <c r="N22" s="2" t="n"/>
+      <c r="O22" s="2" t="n"/>
+      <c r="P22" s="2" t="n"/>
+      <c r="Q22" s="2" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="A19:L19"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A4:L4"/>
+  <mergeCells count="12">
+    <mergeCell ref="G2:I2"/>
+    <mergeCell ref="A12:A16"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="A4:A11"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="D2:D3"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="A2:A3"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="M2:P2"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="Q2:Q3"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
-  <conditionalFormatting sqref="K4:K24">
+  <conditionalFormatting sqref="P4:P16">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"VERIFICA"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Cargar T7 y T8 con las reacciones de VI 02 y VI 11a
Se usan las reacciones de la planilla de vigas: 21,12 t en T7 y
13,78 t en T8. Quedan anotadas como MAYORADAS, a diferencia de las
de T1 a T6, que vienen de la planilla de la catedra y parecen de
servicio. Ocho tabiques verifican; T7 es el mas exigido, con el 73
por ciento de su capacidad.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -16187,7 +16187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q22"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -16651,7 +16651,7 @@
       </c>
       <c r="Q8" s="13" t="inlineStr">
         <is>
-          <t>El mas cargado del conjunto.</t>
+          <t>Si corresponde al T05b del plano, recibe el extremo de VI 07c, cuya reaccion da 18,1 t de servicio en mi bajada contra los 11 t de la catedra. Verificar.</t>
         </is>
       </c>
     </row>
@@ -16719,7 +16719,9 @@
           <t>T7</t>
         </is>
       </c>
-      <c r="C10" s="42" t="n"/>
+      <c r="C10" s="8" t="n">
+        <v>21.12</v>
+      </c>
       <c r="D10" s="8" t="n">
         <v>3.15</v>
       </c>
@@ -16767,7 +16769,7 @@
       </c>
       <c r="Q10" s="13" t="inlineStr">
         <is>
-          <t>Recibe el extremo de VI 02. Carga estimada por la bajada de vigas: 21,1 t. Falta la carga: no figura en la planilla de la catedra.</t>
+          <t>Carga tomada de la reaccion de VI 02 en la planilla de vigas, MAYORADA. No es comparable sin mas con las de T1 a T6.</t>
         </is>
       </c>
     </row>
@@ -16778,7 +16780,9 @@
           <t>T8</t>
         </is>
       </c>
-      <c r="C11" s="43" t="n"/>
+      <c r="C11" s="15" t="n">
+        <v>13.78</v>
+      </c>
       <c r="D11" s="15" t="n">
         <v>3.15</v>
       </c>
@@ -16826,7 +16830,7 @@
       </c>
       <c r="Q11" s="20" t="inlineStr">
         <is>
-          <t>Recibe el extremo de VI 11a. Carga estimada por la bajada de vigas: 14,6 t. Falta la carga: no figura en la planilla de la catedra.</t>
+          <t>Carga tomada de la reaccion de VI 11a en la planilla de vigas, MAYORADA.</t>
         </is>
       </c>
     </row>
@@ -17151,7 +17155,7 @@
     <row r="18">
       <c r="A18" s="44" t="inlineStr">
         <is>
-          <t>T1 a T6: cargas y dimensiones tomadas de la planilla de la catedra.</t>
+          <t>T1 a T6: cargas y dimensiones tomadas de la planilla de la catedra. Probablemente sean cargas de servicio; compararlas contra fi Pn, que es resistencia ultima, queda del lado inseguro en torno a un 40 por ciento. Con utilizaciones del 10 al 20 por ciento no cambia ningun veredicto, pero conviene saberlo.</t>
         </is>
       </c>
       <c r="B18" s="2" t="n"/>
@@ -17174,7 +17178,7 @@
     <row r="19">
       <c r="A19" s="44" t="inlineStr">
         <is>
-          <t>T7 a T13: dimensiones del computo metrico; la carga todavia no esta definida.</t>
+          <t>T7 y T8: carga tomada de la reaccion de VI 02 y VI 11a en la planilla de vigas, que son MAYORADAS. El criterio no es el mismo que en T1 a T6.</t>
         </is>
       </c>
       <c r="B19" s="2" t="n"/>
@@ -17197,7 +17201,7 @@
     <row r="20">
       <c r="A20" s="44" t="inlineStr">
         <is>
-          <t>Area: si B es menor o igual al espesor el tabique es recto y el area es A x B; si no, es un tabique en L y el area es (A + B - espesor) x espesor.</t>
+          <t>T9 a T13: dimensiones del computo metrico; la carga todavia no esta definida.</t>
         </is>
       </c>
       <c r="B20" s="2" t="n"/>
@@ -17220,7 +17224,7 @@
     <row r="21">
       <c r="A21" s="44" t="inlineStr">
         <is>
-          <t>fi Pn = 0,55 x 0,65 x f'c x area x [1 - (altura / 32 espesor)^2]   muro portante de hormigon armado con reduccion por esbeltez.</t>
+          <t>Area: si B es menor o igual al espesor el tabique es recto y el area es A x B; si no, es un tabique en L y el area es (A + B - espesor) x espesor.</t>
         </is>
       </c>
       <c r="B21" s="2" t="n"/>
@@ -17243,7 +17247,7 @@
     <row r="22">
       <c r="A22" s="44" t="inlineStr">
         <is>
-          <t>Armadura vertical en doble malla y horizontal en malla simple, ambas o8 c/20, iguales a las de la planilla de la catedra.</t>
+          <t>fi Pn = 0,55 x 0,65 x f'c x area x [1 - (altura / 32 espesor)^2]   muro portante de hormigon armado con reduccion por esbeltez.</t>
         </is>
       </c>
       <c r="B22" s="2" t="n"/>
@@ -17262,6 +17266,29 @@
       <c r="O22" s="2" t="n"/>
       <c r="P22" s="2" t="n"/>
       <c r="Q22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="44" t="inlineStr">
+        <is>
+          <t>Armadura vertical en doble malla y horizontal en malla simple, ambas o8 c/20, iguales a las de la planilla de la catedra.</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="n"/>
+      <c r="J23" s="2" t="n"/>
+      <c r="K23" s="2" t="n"/>
+      <c r="L23" s="2" t="n"/>
+      <c r="M23" s="2" t="n"/>
+      <c r="N23" s="2" t="n"/>
+      <c r="O23" s="2" t="n"/>
+      <c r="P23" s="2" t="n"/>
+      <c r="Q23" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>

<commit_message>
Incorporar los cuatro tipos de pilote de la nota del plano
La nota declara 33 pilotes repartidos en cuatro tipos: 8 del A, 5
del B, 16 del C y 4 del D. Los cuatro se funden a -4,50 m y se
diferencian en el nivel de llenado de hormigon, de modo que la
longitud del fuste va de 4,10 a 4,45 m. La diferencia de capacidad
entre tipos queda por debajo del 8 por ciento, asi que se mantiene
un unico valor estimado. Se deja asentado que el computo declara 32
pilotes y le falta uno.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -253,7 +253,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -406,6 +406,9 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -3662,7 +3665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3680,12 +3683,14 @@
       <c r="B1" s="2" t="n"/>
       <c r="C1" s="2" t="n"/>
       <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n"/>
       <c r="B2" s="2" t="n"/>
       <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="46" t="inlineStr">
@@ -3708,6 +3713,7 @@
           <t>origen</t>
         </is>
       </c>
+      <c r="E3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="48" t="inlineStr">
@@ -3728,6 +3734,7 @@
           <t>ESTIMADA. Falta el estudio de suelos: cambiar aca y recalcula todo.</t>
         </is>
       </c>
+      <c r="E4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="48" t="inlineStr">
@@ -3748,6 +3755,7 @@
           <t>Dato real, tomado del encabezado del calculo de bases.</t>
         </is>
       </c>
+      <c r="E5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="48" t="inlineStr">
@@ -3768,6 +3776,7 @@
           <t>Nota del plano: todos los pilotes son O30.</t>
         </is>
       </c>
+      <c r="E6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="48" t="inlineStr">
@@ -3788,6 +3797,7 @@
           <t>Nota del plano: h = -4,50 m desde la cota +-0,00 de vereda.</t>
         </is>
       </c>
+      <c r="E7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="48" t="inlineStr">
@@ -3808,150 +3818,350 @@
           <t>Para pasar de carga mayorada a carga de servicio.</t>
         </is>
       </c>
+      <c r="E8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n"/>
       <c r="B9" s="2" t="n"/>
       <c r="C9" s="2" t="n"/>
       <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n"/>
+      <c r="A10" s="59" t="inlineStr">
+        <is>
+          <t>TIPOS DE PILOTE  (nota general del plano: CANTIDAD 33 PILOTES)</t>
+        </is>
+      </c>
       <c r="B10" s="2" t="n"/>
       <c r="C10" s="2" t="n"/>
       <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="59" t="inlineStr">
-        <is>
-          <t>COMO SE ESTIMO LA CARGA ADMISIBLE</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n"/>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="2" t="n"/>
+      <c r="A11" s="47" t="inlineStr">
+        <is>
+          <t>tipo</t>
+        </is>
+      </c>
+      <c r="B11" s="47" t="inlineStr">
+        <is>
+          <t>cantidad</t>
+        </is>
+      </c>
+      <c r="C11" s="47" t="inlineStr">
+        <is>
+          <t>cota fundacion</t>
+        </is>
+      </c>
+      <c r="D11" s="47" t="inlineStr">
+        <is>
+          <t>nivel llenado</t>
+        </is>
+      </c>
+      <c r="E11" s="47" t="inlineStr">
+        <is>
+          <t>long. hormigon</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="44" t="inlineStr">
-        <is>
-          <t>Pilote O30 de 4,50 m: area de punta 0,0707 m2, area lateral 4,24 m2.</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
+      <c r="A12" s="48" t="inlineStr">
+        <is>
+          <t>Pilote tipo "A"</t>
+        </is>
+      </c>
+      <c r="B12" s="60" t="n">
+        <v>8</v>
+      </c>
+      <c r="C12" s="60" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="D12" s="60" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="E12" s="60" t="n">
+        <v>4.1</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="44" t="inlineStr">
-        <is>
-          <t>Punta  0,0707 x 20 t/m2 = 1,4 t.</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="n"/>
+      <c r="A13" s="48" t="inlineStr">
+        <is>
+          <t>Pilote tipo "B"</t>
+        </is>
+      </c>
+      <c r="B13" s="60" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" s="60" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="D13" s="60" t="n">
+        <v>-0.35</v>
+      </c>
+      <c r="E13" s="60" t="n">
+        <v>4.15</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="44" t="inlineStr">
-        <is>
-          <t>Friccion lateral  4,24 x adherencia:  1,5 t/m2 -&gt; 6,4 t   |   3,0 t/m2 -&gt; 12,7 t.</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
+      <c r="A14" s="48" t="inlineStr">
+        <is>
+          <t>Pilote tipo "C"</t>
+        </is>
+      </c>
+      <c r="B14" s="60" t="n">
+        <v>16</v>
+      </c>
+      <c r="C14" s="60" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="D14" s="60" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="E14" s="60" t="n">
+        <v>4.45</v>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="44" t="inlineStr">
-        <is>
-          <t>Total segun adherencia: entre 7,8 y 14,1 t. Se adopta 12 t como valor de trabajo.</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
+      <c r="A15" s="48" t="inlineStr">
+        <is>
+          <t>Pilote tipo "D"</t>
+        </is>
+      </c>
+      <c r="B15" s="60" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" s="60" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="D15" s="60" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="E15" s="60" t="n">
+        <v>4.4</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="44" t="inlineStr"/>
+      <c r="A16" s="2" t="n"/>
       <c r="B16" s="2" t="n"/>
       <c r="C16" s="2" t="n"/>
       <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="41" t="inlineStr">
-        <is>
-          <t>LECTURA INVERSA, que es la util mientras no haya estudio de suelos:</t>
+      <c r="A17" s="44" t="inlineStr">
+        <is>
+          <t>Los cuatro tipos se funden a -4,50 m; se diferencian en el nivel de llenado de hormigon, o sea en la longitud real del fuste.</t>
         </is>
       </c>
       <c r="B17" s="2" t="n"/>
       <c r="C17" s="2" t="n"/>
       <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="44" t="inlineStr">
-        <is>
-          <t>con las cargas de esta planilla, para que el esquema funcione cada pilote</t>
+      <c r="A18" s="41" t="inlineStr">
+        <is>
+          <t>El computo metrico declara 32 pilotes: le falta uno. La nota del plano dice 33, que es la cantidad que se detecta en el dibujo.</t>
         </is>
       </c>
       <c r="B18" s="2" t="n"/>
       <c r="C18" s="2" t="n"/>
       <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="44" t="inlineStr">
-        <is>
-          <t>tiene que admitir del orden de 20 t. Si el estudio de suelos da menos,</t>
-        </is>
-      </c>
+      <c r="A19" s="2" t="n"/>
       <c r="B19" s="2" t="n"/>
       <c r="C19" s="2" t="n"/>
       <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="44" t="inlineStr">
-        <is>
-          <t>faltan pilotes; si da mas, el diseno esta holgado.</t>
+      <c r="A20" s="59" t="inlineStr">
+        <is>
+          <t>COMO SE ESTIMO LA CARGA ADMISIBLE</t>
         </is>
       </c>
       <c r="B20" s="2" t="n"/>
       <c r="C20" s="2" t="n"/>
       <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="44" t="inlineStr"/>
+      <c r="A21" s="44" t="inlineStr">
+        <is>
+          <t>Pilote O30: area de punta 0,0707 m2. Punta  0,0707 x 20 t/m2 = 1,4 t.</t>
+        </is>
+      </c>
       <c r="B21" s="2" t="n"/>
       <c r="C21" s="2" t="n"/>
       <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="44" t="inlineStr">
         <is>
-          <t>La tension de 2 kg/cm2 que trae el calculo de bases es la del estrato</t>
+          <t>Area lateral segun el tipo: 3,86 m2 el A, 3,91 el B, 4,19 el C y 4,15 el D.</t>
         </is>
       </c>
       <c r="B22" s="2" t="n"/>
       <c r="C22" s="2" t="n"/>
       <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="44" t="inlineStr">
         <is>
-          <t>superficial, donde apoyaban las bases. Los pilotes llegan a -4,50 m y</t>
+          <t>Con una adherencia de 2,5 t/m2 la capacidad va de 11,1 t el tipo A a 11,9 t el C:</t>
         </is>
       </c>
       <c r="B23" s="2" t="n"/>
       <c r="C23" s="2" t="n"/>
       <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="44" t="inlineStr">
         <is>
-          <t>trabajan sobre todo por friccion: son dos cosas distintas.</t>
+          <t>la diferencia entre tipos es menor al 8 por ciento, por eso se adopta un unico</t>
         </is>
       </c>
       <c r="B24" s="2" t="n"/>
       <c r="C24" s="2" t="n"/>
       <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="44" t="inlineStr">
+        <is>
+          <t>valor de 12 t para todos, en lugar de uno por tipo.</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="44" t="inlineStr"/>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="41" t="inlineStr">
+        <is>
+          <t>LECTURA INVERSA, que es la util mientras no haya estudio de suelos:</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n"/>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="44" t="inlineStr">
+        <is>
+          <t>con las cargas de esta planilla, para que el esquema funcione cada pilote</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="44" t="inlineStr">
+        <is>
+          <t>tiene que admitir del orden de 20 t. Si el estudio de suelos da menos,</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="2" t="n"/>
+      <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="44" t="inlineStr">
+        <is>
+          <t>faltan pilotes; si da mas, el diseno esta holgado.</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="44" t="inlineStr"/>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="44" t="inlineStr">
+        <is>
+          <t>FALTA: la nota del plano remite a las planillas de cada tipo de pilote, que</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="44" t="inlineStr">
+        <is>
+          <t>traen la armadura y quiza la carga. Si aparecen, se cierra este punto.</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="44" t="inlineStr"/>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="44" t="inlineStr">
+        <is>
+          <t>La tension de 2 kg/cm2 que trae el calculo de bases es la del estrato</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="44" t="inlineStr">
+        <is>
+          <t>superficial, donde apoyaban las bases. Los pilotes llegan a -4,50 m y</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="44" t="inlineStr">
+        <is>
+          <t>trabajan sobre todo por friccion: son dos cosas distintas.</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3972,180 +4182,180 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="60" t="inlineStr">
+      <c r="A1" s="61" t="inlineStr">
         <is>
           <t>MEMORIA - ILUMINACION Y VENTILACION</t>
         </is>
       </c>
-      <c r="B1" s="61" t="inlineStr"/>
+      <c r="B1" s="62" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="61" t="inlineStr"/>
-      <c r="B2" s="62" t="inlineStr"/>
+      <c r="A2" s="62" t="inlineStr"/>
+      <c r="B2" s="63" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="61" t="inlineStr">
+      <c r="A3" s="62" t="inlineStr">
         <is>
           <t>CRITERIO</t>
         </is>
       </c>
-      <c r="B3" s="61" t="inlineStr">
+      <c r="B3" s="62" t="inlineStr">
         <is>
           <t>Area de iluminacion requerida = superficie del local / 9</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="61" t="inlineStr"/>
-      <c r="B4" s="62" t="inlineStr">
+      <c r="A4" s="62" t="inlineStr"/>
+      <c r="B4" s="63" t="inlineStr">
         <is>
           <t>Area de ventilacion requerida = un tercio de la de iluminacion = superficie / 27</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="61" t="inlineStr"/>
-      <c r="B5" s="62" t="inlineStr">
+      <c r="A5" s="62" t="inlineStr"/>
+      <c r="B5" s="63" t="inlineStr">
         <is>
           <t>Area proyectada: la vidriada de la carpinteria para iluminacion, y la parte que</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="61" t="inlineStr"/>
-      <c r="B6" s="62" t="inlineStr">
+      <c r="A6" s="62" t="inlineStr"/>
+      <c r="B6" s="63" t="inlineStr">
         <is>
           <t>realmente abre para ventilacion.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="61" t="inlineStr"/>
-      <c r="B7" s="62" t="inlineStr"/>
+      <c r="A7" s="62" t="inlineStr"/>
+      <c r="B7" s="63" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="61" t="inlineStr">
+      <c r="A8" s="62" t="inlineStr">
         <is>
           <t>RESULTADO</t>
         </is>
       </c>
-      <c r="B8" s="61" t="inlineStr">
+      <c r="B8" s="62" t="inlineStr">
         <is>
           <t>Los trece locales cumplen holgadamente iluminacion y ventilacion.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="61" t="inlineStr"/>
-      <c r="B9" s="62" t="inlineStr"/>
+      <c r="A9" s="62" t="inlineStr"/>
+      <c r="B9" s="63" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="61" t="inlineStr">
+      <c r="A10" s="62" t="inlineStr">
         <is>
           <t>CORRECCION</t>
         </is>
       </c>
-      <c r="B10" s="61" t="inlineStr">
+      <c r="B10" s="62" t="inlineStr">
         <is>
           <t>Local 07, Hall / ingreso: la planilla original traia 0,66 y 0,22, que son los</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="61" t="inlineStr"/>
-      <c r="B11" s="62" t="inlineStr">
+      <c r="A11" s="62" t="inlineStr"/>
+      <c r="B11" s="63" t="inlineStr">
         <is>
           <t>valores del local 03 (Lavadero, 6,0 m2). Con sus 3,50 x 2,15 = 7,53 m2 corresponden</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="61" t="inlineStr"/>
-      <c r="B12" s="62" t="inlineStr">
+      <c r="A12" s="62" t="inlineStr"/>
+      <c r="B12" s="63" t="inlineStr">
         <is>
           <t>0,84 y 0,28. No cambia el resultado, pero el numero no cerraba con la superficie</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="61" t="inlineStr"/>
-      <c r="B13" s="62" t="inlineStr">
+      <c r="A13" s="62" t="inlineStr"/>
+      <c r="B13" s="63" t="inlineStr">
         <is>
           <t>declarada y un verificador lo puede observar.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="61" t="inlineStr"/>
-      <c r="B14" s="62" t="inlineStr"/>
+      <c r="A14" s="62" t="inlineStr"/>
+      <c r="B14" s="63" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="61" t="inlineStr">
+      <c r="A15" s="62" t="inlineStr">
         <is>
           <t>A REVISAR</t>
         </is>
       </c>
-      <c r="B15" s="61" t="inlineStr">
+      <c r="B15" s="62" t="inlineStr">
         <is>
           <t>Local 14, Estar / Playroom: declara 5,00 m2 de ventilacion sobre 5,00 m2 de</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="61" t="inlineStr"/>
-      <c r="B16" s="62" t="inlineStr">
+      <c r="A16" s="62" t="inlineStr"/>
+      <c r="B16" s="63" t="inlineStr">
         <is>
           <t>iluminacion, es decir una carpinteria enteramente abrible. En los demas locales</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="61" t="inlineStr"/>
-      <c r="B17" s="62" t="inlineStr">
+      <c r="A17" s="62" t="inlineStr"/>
+      <c r="B17" s="63" t="inlineStr">
         <is>
           <t>la relacion es del 50 por ciento. Conviene verificar la carpinteria real.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="61" t="inlineStr"/>
-      <c r="B18" s="62" t="inlineStr"/>
+      <c r="A18" s="62" t="inlineStr"/>
+      <c r="B18" s="63" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="61" t="inlineStr"/>
-      <c r="B19" s="62" t="inlineStr">
+      <c r="A19" s="62" t="inlineStr"/>
+      <c r="B19" s="63" t="inlineStr">
         <is>
           <t>Local 02, Deposito: figura sin exigencia por no ser habitable. Son 11,8 m2</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="61" t="inlineStr"/>
-      <c r="B20" s="62" t="inlineStr">
+      <c r="A20" s="62" t="inlineStr"/>
+      <c r="B20" s="63" t="inlineStr">
         <is>
           <t>cerrados: si se lo considera habitable hay que preverle conducto.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="61" t="inlineStr"/>
-      <c r="B21" s="62" t="inlineStr"/>
+      <c r="A21" s="62" t="inlineStr"/>
+      <c r="B21" s="63" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="61" t="inlineStr">
+      <c r="A22" s="62" t="inlineStr">
         <is>
           <t>REDONDEOS</t>
         </is>
       </c>
-      <c r="B22" s="61" t="inlineStr">
+      <c r="B22" s="62" t="inlineStr">
         <is>
           <t>Diferencias menores que no afectan: local 03 da 5,95 m2 y figura 6,0;</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="61" t="inlineStr"/>
-      <c r="B23" s="62" t="inlineStr">
+      <c r="A23" s="62" t="inlineStr"/>
+      <c r="B23" s="63" t="inlineStr">
         <is>
           <t>local 09 da 12,25 y figura 12,3.</t>
         </is>
@@ -4170,592 +4380,592 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="60" t="inlineStr">
+      <c r="A1" s="61" t="inlineStr">
         <is>
           <t>MEMORIA DE CALCULO - VIGAS H°A°</t>
         </is>
       </c>
-      <c r="B1" s="61" t="inlineStr"/>
+      <c r="B1" s="62" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="61" t="inlineStr"/>
-      <c r="B2" s="62" t="inlineStr"/>
+      <c r="A2" s="62" t="inlineStr"/>
+      <c r="B2" s="63" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="61" t="inlineStr">
+      <c r="A3" s="62" t="inlineStr">
         <is>
           <t>NORMATIVA</t>
         </is>
       </c>
-      <c r="B3" s="61" t="inlineStr">
+      <c r="B3" s="62" t="inlineStr">
         <is>
           <t>CIRSOC 201. Hormigon H-21 (f'c 210 kg/cm2). Acero 42/50 (fy 4200 kg/cm2).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="61" t="inlineStr">
+      <c r="A4" s="62" t="inlineStr">
         <is>
           <t>UNIDADES</t>
         </is>
       </c>
-      <c r="B4" s="61" t="inlineStr">
+      <c r="B4" s="62" t="inlineStr">
         <is>
           <t>Longitudes en m y cm. Cargas en kg/m. Momentos en kgm. Tensiones en kg/cm2.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="61" t="inlineStr">
+      <c r="A5" s="62" t="inlineStr">
         <is>
           <t>DIMENSIONES</t>
         </is>
       </c>
-      <c r="B5" s="61" t="inlineStr">
+      <c r="B5" s="62" t="inlineStr">
         <is>
           <t>b = ancho | h = altura util | d = altura total (igual criterio que la planilla de catedra).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="61" t="inlineStr"/>
-      <c r="B6" s="62" t="inlineStr"/>
+      <c r="A6" s="62" t="inlineStr"/>
+      <c r="B6" s="63" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="61" t="inlineStr">
+      <c r="A7" s="62" t="inlineStr">
         <is>
           <t>1. CARGAS</t>
         </is>
       </c>
-      <c r="B7" s="61" t="inlineStr"/>
+      <c r="B7" s="62" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="61" t="inlineStr">
+      <c r="A8" s="62" t="inlineStr">
         <is>
           <t>Entrepiso PA</t>
         </is>
       </c>
-      <c r="B8" s="62" t="inlineStr">
+      <c r="B8" s="63" t="inlineStr">
         <is>
           <t>Losa maciza 12 cm 300 + contrapiso 130 + carpeta 42 + piso 50 + cielorraso 20</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="61" t="inlineStr"/>
-      <c r="B9" s="62" t="inlineStr">
+      <c r="A9" s="62" t="inlineStr"/>
+      <c r="B9" s="63" t="inlineStr">
         <is>
           <t>g = 550 kg/m2       q = 200 kg/m2 (vivienda)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="61" t="inlineStr">
+      <c r="A10" s="62" t="inlineStr">
         <is>
           <t>Azotea</t>
         </is>
       </c>
-      <c r="B10" s="62" t="inlineStr">
+      <c r="B10" s="63" t="inlineStr">
         <is>
           <t>Losa 300 + contrapiso de pendiente 140 + carpeta 42 + aislacion y membrana 50 + cielorraso 20</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="61" t="inlineStr"/>
-      <c r="B11" s="62" t="inlineStr">
+      <c r="A11" s="62" t="inlineStr"/>
+      <c r="B11" s="63" t="inlineStr">
         <is>
           <t>g = 560 kg/m2       q = 100 kg/m2 (cubierta no accesible)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="61" t="inlineStr">
+      <c r="A12" s="62" t="inlineStr">
         <is>
           <t>Mamposteria</t>
         </is>
       </c>
-      <c r="B12" s="62" t="inlineStr">
+      <c r="B12" s="63" t="inlineStr">
         <is>
           <t>250 kg/m2. Altura 2,60 m en PA y 1,00 m de parapeto en azotea.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="61" t="inlineStr">
+      <c r="A13" s="62" t="inlineStr">
         <is>
           <t>Peso propio</t>
         </is>
       </c>
-      <c r="B13" s="62" t="inlineStr">
+      <c r="B13" s="63" t="inlineStr">
         <is>
           <t>2400 kg/m3 x b x d, viga por viga.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="61" t="inlineStr">
+      <c r="A14" s="62" t="inlineStr">
         <is>
           <t>Carga de calculo</t>
         </is>
       </c>
-      <c r="B14" s="62" t="inlineStr">
+      <c r="B14" s="63" t="inlineStr">
         <is>
           <t>p = 1,2 (g x B + peso propio + muro) + 1,6 (q x B)        B = ancho tributario</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="61" t="inlineStr"/>
-      <c r="B15" s="62" t="inlineStr"/>
+      <c r="A15" s="62" t="inlineStr"/>
+      <c r="B15" s="63" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="61" t="inlineStr">
+      <c r="A16" s="62" t="inlineStr">
         <is>
           <t>2. SOLICITACIONES</t>
         </is>
       </c>
-      <c r="B16" s="61" t="inlineStr">
+      <c r="B16" s="62" t="inlineStr">
         <is>
           <t>Coeficientes segun esquema (tabla en hoja Datos):</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="61" t="inlineStr"/>
-      <c r="B17" s="62" t="inlineStr">
+      <c r="A17" s="62" t="inlineStr"/>
+      <c r="B17" s="63" t="inlineStr">
         <is>
           <t xml:space="preserve">  Simplemente apoyada   M = pL2/8                    R = 0,500 pL</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="61" t="inlineStr"/>
-      <c r="B18" s="62" t="inlineStr">
+      <c r="A18" s="62" t="inlineStr"/>
+      <c r="B18" s="63" t="inlineStr">
         <is>
           <t xml:space="preserve">  Continua              M = pL2/14   Mapoyo = pL2/10  R = 0,575 pL</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="61" t="inlineStr"/>
-      <c r="B19" s="62" t="inlineStr">
+      <c r="A19" s="62" t="inlineStr"/>
+      <c r="B19" s="63" t="inlineStr">
         <is>
           <t xml:space="preserve">  Empotrada-apoyada     M = 9pL2/128 Mapoyo = pL2/8   R = 0,625 pL</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="61" t="inlineStr"/>
-      <c r="B20" s="62" t="inlineStr">
+      <c r="A20" s="62" t="inlineStr"/>
+      <c r="B20" s="63" t="inlineStr">
         <is>
           <t xml:space="preserve">  Biempotrada           M = pL2/24   Mapoyo = pL2/12  R = 0,500 pL</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="61" t="inlineStr"/>
-      <c r="B21" s="62" t="inlineStr">
+      <c r="A21" s="62" t="inlineStr"/>
+      <c r="B21" s="63" t="inlineStr">
         <is>
           <t xml:space="preserve">  Voladizo                           Mapoyo = pL2/2   R = 1,000 pL</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="61" t="inlineStr"/>
-      <c r="B22" s="62" t="inlineStr"/>
+      <c r="A22" s="62" t="inlineStr"/>
+      <c r="B22" s="63" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="61" t="inlineStr">
+      <c r="A23" s="62" t="inlineStr">
         <is>
           <t>3. FLEXION</t>
         </is>
       </c>
-      <c r="B23" s="61" t="inlineStr">
+      <c r="B23" s="62" t="inlineStr">
         <is>
           <t>k = M / (phi b h2 f'c)      w = 1 - RAIZ(1 - 2k)      As = w b h f'c / fy</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="61" t="inlineStr"/>
-      <c r="B24" s="62" t="inlineStr">
+      <c r="A24" s="62" t="inlineStr"/>
+      <c r="B24" s="63" t="inlineStr">
         <is>
           <t>As min = 0,0033 b h       As max = 0,0163 b h (0,75 de la cuantia balanceada)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="61" t="inlineStr"/>
-      <c r="B25" s="62" t="inlineStr">
+      <c r="A25" s="62" t="inlineStr"/>
+      <c r="B25" s="63" t="inlineStr">
         <is>
           <t>Si la armadura no entra en una capa se disponen dos y el recubrimiento pasa a 6 cm.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="61" t="inlineStr"/>
-      <c r="B26" s="62" t="inlineStr"/>
+      <c r="A26" s="62" t="inlineStr"/>
+      <c r="B26" s="63" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="61" t="inlineStr">
+      <c r="A27" s="62" t="inlineStr">
         <is>
           <t>4. CORTE</t>
         </is>
       </c>
-      <c r="B27" s="61" t="inlineStr">
+      <c r="B27" s="62" t="inlineStr">
         <is>
           <t>T = R / (b x 0,85 h)       tension tangencial en el apoyo</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="61" t="inlineStr"/>
-      <c r="B28" s="62" t="inlineStr">
+      <c r="A28" s="62" t="inlineStr"/>
+      <c r="B28" s="63" t="inlineStr">
         <is>
           <t>Vc = 0,53 RAIZ(f'c) b h        phi Vn = 0,75 (Vc + Av fy h / s)  &gt;=  R</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="61" t="inlineStr"/>
-      <c r="B29" s="62" t="inlineStr">
+      <c r="A29" s="62" t="inlineStr"/>
+      <c r="B29" s="63" t="inlineStr">
         <is>
           <t>Av = 2 ramas. Se aumenta el diametro antes que cerrar la separacion por debajo de 10 cm.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="61" t="inlineStr"/>
-      <c r="B30" s="62" t="inlineStr"/>
+      <c r="A30" s="62" t="inlineStr"/>
+      <c r="B30" s="63" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="61" t="inlineStr">
+      <c r="A31" s="62" t="inlineStr">
         <is>
           <t>5. FLECHA</t>
         </is>
       </c>
-      <c r="B31" s="61" t="inlineStr">
+      <c r="B31" s="62" t="inlineStr">
         <is>
           <t>Altura minima: simplemente apoyada L/16, un extremo continuo L/18,5,</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="61" t="inlineStr"/>
-      <c r="B32" s="62" t="inlineStr">
+      <c r="A32" s="62" t="inlineStr"/>
+      <c r="B32" s="63" t="inlineStr">
         <is>
           <t>ambos extremos continuos L/21, voladizo L/8.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="61" t="inlineStr"/>
-      <c r="B33" s="62" t="inlineStr"/>
+      <c r="A33" s="62" t="inlineStr"/>
+      <c r="B33" s="63" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="61" t="inlineStr">
+      <c r="A34" s="62" t="inlineStr">
         <is>
           <t>6. VIGAS INVERTIDAS</t>
         </is>
       </c>
-      <c r="B34" s="61" t="inlineStr">
+      <c r="B34" s="62" t="inlineStr">
         <is>
           <t>Las vigas de BORDE son invertidas: sobresalen 70 cm por encima del fondo de</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="61" t="inlineStr"/>
-      <c r="B35" s="62" t="inlineStr">
+      <c r="A35" s="62" t="inlineStr"/>
+      <c r="B35" s="63" t="inlineStr">
         <is>
           <t>losa (cotas N.F.L +3,50 / N.S.V +4,20 y N.F.L +6,80 / N.S.V +7,50 del plano).</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="61" t="inlineStr"/>
-      <c r="B36" s="62" t="inlineStr">
+      <c r="A36" s="62" t="inlineStr"/>
+      <c r="B36" s="63" t="inlineStr">
         <is>
           <t>losa. Lo confirman las cotas del plano y el hecho de que el cielorraso sea de</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="61" t="inlineStr"/>
-      <c r="B37" s="62" t="inlineStr">
+      <c r="A37" s="62" t="inlineStr"/>
+      <c r="B37" s="63" t="inlineStr">
         <is>
           <t>VI 06 mide 14,00 m en total y es el cuarto borde de L07. Sobre su eje hay cuatro</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="61" t="inlineStr"/>
-      <c r="B38" s="62" t="inlineStr">
+      <c r="A38" s="62" t="inlineStr"/>
+      <c r="B38" s="63" t="inlineStr">
         <is>
           <t>columnas, de modo que trabaja como viga continua de tres tramos de 4,10, 4,32 y</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="61" t="inlineStr"/>
-      <c r="B39" s="62" t="inlineStr">
+      <c r="A39" s="62" t="inlineStr"/>
+      <c r="B39" s="63" t="inlineStr">
         <is>
           <t>6,53 m. Se calcula con el mayor, 6,53 m, que es el que gobierna.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="61" t="inlineStr"/>
-      <c r="B40" s="62" t="inlineStr">
+      <c r="A40" s="62" t="inlineStr"/>
+      <c r="B40" s="63" t="inlineStr">
         <is>
           <t>hormigon visto: una viga colgante quedaria a la vista. El computo metrico las</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="61" t="inlineStr"/>
-      <c r="B41" s="62" t="inlineStr">
+      <c r="A41" s="62" t="inlineStr"/>
+      <c r="B41" s="63" t="inlineStr">
         <is>
           <t>agrupa a las 28 bajo el rubro Vigas invertidas 15x70.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="61" t="inlineStr"/>
-      <c r="B42" s="62" t="inlineStr">
+      <c r="A42" s="62" t="inlineStr"/>
+      <c r="B42" s="63" t="inlineStr">
         <is>
           <t>Esto define donde la losa aporta ala comprimida:</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="61" t="inlineStr"/>
-      <c r="B43" s="62" t="inlineStr">
+      <c r="A43" s="62" t="inlineStr"/>
+      <c r="B43" s="63" t="inlineStr">
         <is>
           <t xml:space="preserve">  viga COLGANTE  -&gt; la losa esta arriba  -&gt; ala util en el TRAMO (momento positivo)</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="61" t="inlineStr"/>
-      <c r="B44" s="62" t="inlineStr">
+      <c r="A44" s="62" t="inlineStr"/>
+      <c r="B44" s="63" t="inlineStr">
         <is>
           <t xml:space="preserve">  viga INVERTIDA -&gt; la losa esta abajo   -&gt; ala util en el APOYO (momento negativo)</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="61" t="inlineStr"/>
-      <c r="B45" s="62" t="inlineStr">
+      <c r="A45" s="62" t="inlineStr"/>
+      <c r="B45" s="63" t="inlineStr">
         <is>
           <t>En la zona con ala se adopta b efectivo = min(L/4 ; b + 16 hf); en la otra, la</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="61" t="inlineStr"/>
-      <c r="B46" s="62" t="inlineStr">
+      <c r="A46" s="62" t="inlineStr"/>
+      <c r="B46" s="63" t="inlineStr">
         <is>
           <t>seccion es rectangular de ancho b. Las columnas b ef tramo y b ef apoyo lo muestran.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="61" t="inlineStr"/>
-      <c r="B47" s="62" t="inlineStr">
+      <c r="A47" s="62" t="inlineStr"/>
+      <c r="B47" s="63" t="inlineStr">
         <is>
           <t>PENDIENTE: las invertidas de BORDE (VI 01a, 01b, 07a, 07b, 07c, 11a, 11b, 11c,</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="61" t="inlineStr"/>
-      <c r="B48" s="62" t="inlineStr">
+      <c r="A48" s="62" t="inlineStr"/>
+      <c r="B48" s="63" t="inlineStr">
         <is>
           <t>15a y 15b) reciben la reaccion de la losa de un solo lado, excentrica respecto</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="61" t="inlineStr"/>
-      <c r="B49" s="62" t="inlineStr">
+      <c r="A49" s="62" t="inlineStr"/>
+      <c r="B49" s="63" t="inlineStr">
         <is>
           <t>de su eje, y quedan sometidas a TORSION. Esta planilla no la verifica.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="61" t="inlineStr"/>
-      <c r="B50" s="62" t="inlineStr"/>
+      <c r="A50" s="62" t="inlineStr"/>
+      <c r="B50" s="63" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="61" t="inlineStr">
+      <c r="A51" s="62" t="inlineStr">
         <is>
           <t>7. RESULTADO</t>
         </is>
       </c>
-      <c r="B51" s="61" t="inlineStr">
+      <c r="B51" s="62" t="inlineStr">
         <is>
           <t>30 vigas: 21 del entrepiso PA y 9 de la losa de techo. 28 verifican.</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="61" t="inlineStr"/>
-      <c r="B52" s="62" t="inlineStr">
+      <c r="A52" s="62" t="inlineStr"/>
+      <c r="B52" s="63" t="inlineStr">
         <is>
           <t>VI 02 (15x60, 9,88 m): recibe L02 y L03, B = 2,88 m. La armadura de apoyo</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="61" t="inlineStr"/>
-      <c r="B53" s="62" t="inlineStr">
+      <c r="A53" s="62" t="inlineStr"/>
+      <c r="B53" s="63" t="inlineStr">
         <is>
           <t xml:space="preserve">   necesaria ronda los 25 cm2 y supera la cuantia maxima. Los apoyos estan</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="61" t="inlineStr"/>
-      <c r="B54" s="62" t="inlineStr">
+      <c r="A54" s="62" t="inlineStr"/>
+      <c r="B54" s="63" t="inlineStr">
         <is>
           <t xml:space="preserve">   confirmados en obra: tabique T07 perpendicular arriba y COL 02 abajo, sin apoyo</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="61" t="inlineStr"/>
-      <c r="B55" s="62" t="inlineStr">
+      <c r="A55" s="62" t="inlineStr"/>
+      <c r="B55" s="63" t="inlineStr">
         <is>
           <t xml:space="preserve">   intermedio. Para esta carga la seccion necesaria es 15x75.</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="61" t="inlineStr"/>
-      <c r="B56" s="62" t="inlineStr">
+      <c r="A56" s="62" t="inlineStr"/>
+      <c r="B56" s="63" t="inlineStr">
         <is>
           <t>VCH 03a (40x13, 3,83 m). Recibe L03, B = 2,08 m, y no</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="61" t="inlineStr"/>
-      <c r="B57" s="62" t="inlineStr">
+      <c r="A57" s="62" t="inlineStr"/>
+      <c r="B57" s="63" t="inlineStr">
         <is>
           <t xml:space="preserve">   verifica: haria falta mas espesor. Tampoco verifica con B = 0,60 m, asi</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="61" t="inlineStr"/>
-      <c r="B58" s="62" t="inlineStr">
+      <c r="A58" s="62" t="inlineStr"/>
+      <c r="B58" s="63" t="inlineStr">
         <is>
           <t xml:space="preserve">   que el problema no es la hipotesis de carga sino la relacion luz/espesor. Una viga</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="61" t="inlineStr"/>
-      <c r="B59" s="62" t="inlineStr">
+      <c r="A59" s="62" t="inlineStr"/>
+      <c r="B59" s="63" t="inlineStr">
         <is>
           <t xml:space="preserve">   chata del mismo espesor que la losa no puede ser apoyo lineal de un pano de 4,15 m.</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="61" t="inlineStr"/>
-      <c r="B60" s="62" t="inlineStr">
+      <c r="A60" s="62" t="inlineStr"/>
+      <c r="B60" s="63" t="inlineStr">
         <is>
           <t xml:space="preserve">   Revisar si tiene un muro debajo que acorte su luz libre.</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="61" t="inlineStr"/>
-      <c r="B61" s="62" t="inlineStr">
+      <c r="A61" s="62" t="inlineStr"/>
+      <c r="B61" s="63" t="inlineStr">
         <is>
           <t>VCH 03a (40x13, 3,71 m): excede la cuantia maxima y no llega a la altura minima por</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="61" t="inlineStr"/>
-      <c r="B62" s="62" t="inlineStr">
+      <c r="A62" s="62" t="inlineStr"/>
+      <c r="B62" s="63" t="inlineStr">
         <is>
           <t xml:space="preserve">   flecha. Revisar el ancho tributario: si solo recibe el muro y no losa, baja mucho.</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="61" t="inlineStr"/>
-      <c r="B63" s="62" t="inlineStr"/>
+      <c r="A63" s="62" t="inlineStr"/>
+      <c r="B63" s="63" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="61" t="inlineStr">
+      <c r="A64" s="62" t="inlineStr">
         <is>
           <t>8. ALCANCE</t>
         </is>
       </c>
-      <c r="B64" s="62" t="inlineStr">
+      <c r="B64" s="63" t="inlineStr">
         <is>
           <t>No se incluyen las 31 vigas de fundacion (VF01 a VF18c): su calculo depende de las</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="61" t="inlineStr"/>
-      <c r="B65" s="62" t="inlineStr">
+      <c r="A65" s="62" t="inlineStr"/>
+      <c r="B65" s="63" t="inlineStr">
         <is>
           <t>cargas que bajan por las columnas y corresponde hacerlo despues. Tampoco losas ni columnas.</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="61" t="inlineStr"/>
-      <c r="B66" s="62" t="inlineStr"/>
+      <c r="A66" s="62" t="inlineStr"/>
+      <c r="B66" s="63" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="61" t="inlineStr">
+      <c r="A67" s="62" t="inlineStr">
         <is>
           <t>LIMITACIONES</t>
         </is>
       </c>
-      <c r="B67" s="61" t="inlineStr">
+      <c r="B67" s="62" t="inlineStr">
         <is>
           <t>El ancho tributario B esta relevado solo en</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="61" t="inlineStr"/>
-      <c r="B68" s="62" t="inlineStr">
+      <c r="A68" s="62" t="inlineStr"/>
+      <c r="B68" s="63" t="inlineStr">
         <is>
           <t>VI 02 (0,80 m) y VCH 03a (2,08 m). En las demas sigue adoptado en 2,00 m, a falta</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="61" t="inlineStr"/>
-      <c r="B69" s="62" t="inlineStr">
+      <c r="A69" s="62" t="inlineStr"/>
+      <c r="B69" s="63" t="inlineStr">
         <is>
           <t>hipotesis mas influyente del calculo: ajustarla viga por viga en la columna B trib.</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="61" t="inlineStr"/>
-      <c r="B70" s="62" t="inlineStr">
+      <c r="A70" s="62" t="inlineStr"/>
+      <c r="B70" s="63" t="inlineStr">
         <is>
           <t>El esquema se asigno por criterio: continua si integra una serie a-b-c o si supera 5,5 m.</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="61" t="inlineStr"/>
-      <c r="B71" s="62" t="inlineStr">
+      <c r="A71" s="62" t="inlineStr"/>
+      <c r="B71" s="63" t="inlineStr">
         <is>
           <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
         </is>
@@ -4780,368 +4990,368 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="60" t="inlineStr">
+      <c r="A1" s="61" t="inlineStr">
         <is>
           <t>MEMORIA DE CALCULO - LOSAS</t>
         </is>
       </c>
-      <c r="B1" s="61" t="inlineStr"/>
+      <c r="B1" s="62" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="61" t="inlineStr"/>
-      <c r="B2" s="62" t="inlineStr"/>
+      <c r="A2" s="62" t="inlineStr"/>
+      <c r="B2" s="63" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="61" t="inlineStr">
+      <c r="A3" s="62" t="inlineStr">
         <is>
           <t>METODO</t>
         </is>
       </c>
-      <c r="B3" s="61" t="inlineStr">
+      <c r="B3" s="62" t="inlineStr">
         <is>
           <t>Tensiones admisibles, igual criterio que la planilla modelo de la catedra.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="61" t="inlineStr"/>
-      <c r="B4" s="62" t="inlineStr">
+      <c r="A4" s="62" t="inlineStr"/>
+      <c r="B4" s="63" t="inlineStr">
         <is>
           <t>Se verifico contra la fila de ejemplo: momentos y reacciones coinciden exactamente.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="61" t="inlineStr">
+      <c r="A5" s="62" t="inlineStr">
         <is>
           <t>MATERIALES</t>
         </is>
       </c>
-      <c r="B5" s="61" t="inlineStr">
+      <c r="B5" s="62" t="inlineStr">
         <is>
           <t>H-21 (f'c 210 kg/cm2). Acero 42/50 (fy 4200). Tension admisible 2400 kg/cm2.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="61" t="inlineStr">
+      <c r="A6" s="62" t="inlineStr">
         <is>
           <t>DIMENSIONES</t>
         </is>
       </c>
-      <c r="B6" s="61" t="inlineStr">
+      <c r="B6" s="62" t="inlineStr">
         <is>
           <t>h = altura util | d = espesor total. Recubrimiento 1,5 cm.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="61" t="inlineStr"/>
-      <c r="B7" s="62" t="inlineStr"/>
+      <c r="A7" s="62" t="inlineStr"/>
+      <c r="B7" s="63" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="61" t="inlineStr">
+      <c r="A8" s="62" t="inlineStr">
         <is>
           <t>1. CARGAS</t>
         </is>
       </c>
-      <c r="B8" s="61" t="inlineStr">
+      <c r="B8" s="62" t="inlineStr">
         <is>
           <t>p = peso propio + terminaciones + q      (cargas de servicio, sin mayorar)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="61" t="inlineStr"/>
-      <c r="B9" s="62" t="inlineStr">
+      <c r="A9" s="62" t="inlineStr"/>
+      <c r="B9" s="63" t="inlineStr">
         <is>
           <t>Peso propio = 2400 x d / 100, calculado con el espesor propio de cada losa.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="61" t="inlineStr">
+      <c r="A10" s="62" t="inlineStr">
         <is>
           <t>S/PB</t>
         </is>
       </c>
-      <c r="B10" s="62" t="inlineStr">
+      <c r="B10" s="63" t="inlineStr">
         <is>
           <t>Terminaciones 242 kg/m2 (contrapiso 130 + carpeta 42 + piso 50 + cielorraso 20)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="61" t="inlineStr"/>
-      <c r="B11" s="62" t="inlineStr">
+      <c r="A11" s="62" t="inlineStr"/>
+      <c r="B11" s="63" t="inlineStr">
         <is>
           <t>q = 200 kg/m2 (vivienda)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="61" t="inlineStr">
+      <c r="A12" s="62" t="inlineStr">
         <is>
           <t>S/PA</t>
         </is>
       </c>
-      <c r="B12" s="62" t="inlineStr">
+      <c r="B12" s="63" t="inlineStr">
         <is>
           <t>Terminaciones 252 kg/m2 (contrapiso pendiente 140 + carpeta 42 + aislacion 50 +</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="61" t="inlineStr"/>
-      <c r="B13" s="62" t="inlineStr">
+      <c r="A13" s="62" t="inlineStr"/>
+      <c r="B13" s="63" t="inlineStr">
         <is>
           <t>cielorraso 20).  q = 100 kg/m2 (azotea no accesible)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="61" t="inlineStr"/>
-      <c r="B14" s="62" t="inlineStr"/>
+      <c r="A14" s="62" t="inlineStr"/>
+      <c r="B14" s="63" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="61" t="inlineStr">
+      <c r="A15" s="62" t="inlineStr">
         <is>
           <t>2. SOLICITACIONES</t>
         </is>
       </c>
-      <c r="B15" s="61" t="inlineStr">
+      <c r="B15" s="62" t="inlineStr">
         <is>
           <t>M = coeficiente x p x L2, segun el grado de empotramiento:</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="61" t="inlineStr"/>
-      <c r="B16" s="62" t="inlineStr">
+      <c r="A16" s="62" t="inlineStr"/>
+      <c r="B16" s="63" t="inlineStr">
         <is>
           <t xml:space="preserve">  1/8 simplemente apoyada    1/10 y 1/14 continua    1/12 biempotrada    1/2 voladizo</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="61" t="inlineStr"/>
-      <c r="B17" s="62" t="inlineStr">
+      <c r="A17" s="62" t="inlineStr"/>
+      <c r="B17" s="63" t="inlineStr">
         <is>
           <t>R = coeficiente x p x L. En voladizo Rx = p x L y Ry no corresponde.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="61" t="inlineStr"/>
-      <c r="B18" s="62" t="inlineStr"/>
+      <c r="A18" s="62" t="inlineStr"/>
+      <c r="B18" s="63" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="61" t="inlineStr">
+      <c r="A19" s="62" t="inlineStr">
         <is>
           <t>3. ARMADURA</t>
         </is>
       </c>
-      <c r="B19" s="61" t="inlineStr">
+      <c r="B19" s="62" t="inlineStr">
         <is>
           <t>As = M x 100 / (2400 x 0,9 x h)        [cm2/m]</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="61" t="inlineStr"/>
-      <c r="B20" s="62" t="inlineStr">
+      <c r="A20" s="62" t="inlineStr"/>
+      <c r="B20" s="63" t="inlineStr">
         <is>
           <t>separacion = 100 x area de la barra / As, redondeada, con maximo 20 cm</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="61" t="inlineStr"/>
-      <c r="B21" s="62" t="inlineStr">
+      <c r="A21" s="62" t="inlineStr"/>
+      <c r="B21" s="63" t="inlineStr">
         <is>
           <t>Armadura de reparticion = As / 5, con un minimo de 0,30 cm2/m</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="61" t="inlineStr"/>
-      <c r="B22" s="62" t="inlineStr"/>
+      <c r="A22" s="62" t="inlineStr"/>
+      <c r="B22" s="63" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="61" t="inlineStr">
+      <c r="A23" s="62" t="inlineStr">
         <is>
           <t>4. ESPESORES</t>
         </is>
       </c>
-      <c r="B23" s="61" t="inlineStr">
+      <c r="B23" s="62" t="inlineStr">
         <is>
           <t>Los espesores d se leyeron del plano: estan escritos debajo del rotulo de cada losa.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="61" t="inlineStr"/>
-      <c r="B24" s="62" t="inlineStr">
+      <c r="A24" s="62" t="inlineStr"/>
+      <c r="B24" s="63" t="inlineStr">
         <is>
           <t>S/PB:  L01 11 | L02 9 | L03 13 | L04 11 | L05 11 | L06 8 | L07 12 | L08 10</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="61" t="inlineStr"/>
-      <c r="B25" s="62" t="inlineStr">
+      <c r="A25" s="62" t="inlineStr"/>
+      <c r="B25" s="63" t="inlineStr">
         <is>
           <t>S/PA:  L09 13 | L10 12</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="61" t="inlineStr"/>
-      <c r="B26" s="62" t="inlineStr"/>
+      <c r="A26" s="62" t="inlineStr"/>
+      <c r="B26" s="63" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="61" t="inlineStr">
+      <c r="A27" s="62" t="inlineStr">
         <is>
           <t>5. LUCES</t>
         </is>
       </c>
-      <c r="B27" s="61" t="inlineStr">
+      <c r="B27" s="62" t="inlineStr">
         <is>
           <t>Relevadas en obra y aportadas por el proyectista. Dos losas son voladizo</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="61" t="inlineStr"/>
-      <c r="B28" s="62" t="inlineStr">
+      <c r="A28" s="62" t="inlineStr"/>
+      <c r="B28" s="63" t="inlineStr">
         <is>
           <t>(L02 de 0,80 m y L08 de 0,75 m) y se calculan con M = p L2 / 2.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="61" t="inlineStr"/>
-      <c r="B29" s="62" t="inlineStr"/>
+      <c r="A29" s="62" t="inlineStr"/>
+      <c r="B29" s="63" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="61" t="inlineStr">
+      <c r="A30" s="62" t="inlineStr">
         <is>
           <t>6. LOSAS CRUZADAS</t>
         </is>
       </c>
-      <c r="B30" s="62" t="inlineStr">
+      <c r="B30" s="63" t="inlineStr">
         <is>
           <t>L07 (4,85 x 5,60) y L10 (4,85 x 6,00) apoyan en los cuatro bordes y su relacion</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="61" t="inlineStr"/>
-      <c r="B31" s="62" t="inlineStr">
+      <c r="A31" s="62" t="inlineStr"/>
+      <c r="B31" s="63" t="inlineStr">
         <is>
           <t>de lados es menor que 2, por lo que trabajan en las dos direcciones.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="61" t="inlineStr"/>
-      <c r="B32" s="62" t="inlineStr">
+      <c r="A32" s="62" t="inlineStr"/>
+      <c r="B32" s="63" t="inlineStr">
         <is>
           <t>Se reparte la carga por el metodo de Marcus:   kx = ly4 / (lx4 + ly4)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="61" t="inlineStr"/>
-      <c r="B33" s="62" t="inlineStr">
+      <c r="A33" s="62" t="inlineStr"/>
+      <c r="B33" s="63" t="inlineStr">
         <is>
           <t xml:space="preserve">  L07: ly/lx = 1,15  -&gt;  64% en la direccion corta, 36% en la larga</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="61" t="inlineStr"/>
-      <c r="B34" s="62" t="inlineStr">
+      <c r="A34" s="62" t="inlineStr"/>
+      <c r="B34" s="63" t="inlineStr">
         <is>
           <t xml:space="preserve">  L10: ly/lx = 1,24  -&gt;  70% en la direccion corta, 30% en la larga</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="61" t="inlineStr"/>
-      <c r="B35" s="62" t="inlineStr">
+      <c r="A35" s="62" t="inlineStr"/>
+      <c r="B35" s="63" t="inlineStr">
         <is>
           <t>Cada una ocupa dos renglones, uno por direccion, con la fraccion de carga que</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="61" t="inlineStr"/>
-      <c r="B36" s="62" t="inlineStr">
+      <c r="A36" s="62" t="inlineStr"/>
+      <c r="B36" s="63" t="inlineStr">
         <is>
           <t>le toca ya aplicada en la columna CARGAS. Las dos armaduras se cruzan en obra:</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="61" t="inlineStr"/>
-      <c r="B37" s="62" t="inlineStr">
+      <c r="A37" s="62" t="inlineStr"/>
+      <c r="B37" s="63" t="inlineStr">
         <is>
           <t>la de la direccion corta va abajo, la de la larga arriba de aquella.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="61" t="inlineStr"/>
-      <c r="B38" s="62" t="inlineStr">
+      <c r="A38" s="62" t="inlineStr"/>
+      <c r="B38" s="63" t="inlineStr">
         <is>
           <t>La columna auxiliar luz transv. es la que dispara el reparto: si se borra, la</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="61" t="inlineStr"/>
-      <c r="B39" s="62" t="inlineStr">
+      <c r="A39" s="62" t="inlineStr"/>
+      <c r="B39" s="63" t="inlineStr">
         <is>
           <t>fila vuelve a calcularse como losa armada en una direccion.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="61" t="inlineStr"/>
-      <c r="B40" s="62" t="inlineStr"/>
+      <c r="A40" s="62" t="inlineStr"/>
+      <c r="B40" s="63" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="61" t="inlineStr">
+      <c r="A41" s="62" t="inlineStr">
         <is>
           <t>LIMITACIONES</t>
         </is>
       </c>
-      <c r="B41" s="61" t="inlineStr">
+      <c r="B41" s="62" t="inlineStr">
         <is>
           <t>El grado de empotramiento esta cargado en 1/8 salvo los dos voladizos (1/2). Si</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="61" t="inlineStr"/>
-      <c r="B42" s="62" t="inlineStr">
+      <c r="A42" s="62" t="inlineStr"/>
+      <c r="B42" s="63" t="inlineStr">
         <is>
           <t>alguna losa es continua sobre una viga corresponde 1/10 o 1/14: corregir en la columna.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="61" t="inlineStr"/>
-      <c r="B43" s="62" t="inlineStr">
+      <c r="A43" s="62" t="inlineStr"/>
+      <c r="B43" s="63" t="inlineStr">
         <is>
           <t>El diagrama de cargas es una imagen fija: si cambias el grado, cambialo a mano.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="61" t="inlineStr"/>
-      <c r="B44" s="62" t="inlineStr">
+      <c r="A44" s="62" t="inlineStr"/>
+      <c r="B44" s="63" t="inlineStr">
         <is>
           <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
         </is>
@@ -5166,384 +5376,384 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="60" t="inlineStr">
+      <c r="A1" s="61" t="inlineStr">
         <is>
           <t>MEMORIA DE CALCULO - COLUMNAS</t>
         </is>
       </c>
-      <c r="B1" s="61" t="inlineStr"/>
+      <c r="B1" s="62" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="61" t="inlineStr"/>
-      <c r="B2" s="62" t="inlineStr"/>
+      <c r="A2" s="62" t="inlineStr"/>
+      <c r="B2" s="63" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="61" t="inlineStr">
+      <c r="A3" s="62" t="inlineStr">
         <is>
           <t>MATERIALES</t>
         </is>
       </c>
-      <c r="B3" s="61" t="inlineStr">
+      <c r="B3" s="62" t="inlineStr">
         <is>
           <t>H-21 (f'c 210 kg/cm2). Acero 42/50 (fy 4200). phi compresion 0,65.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="61" t="inlineStr"/>
-      <c r="B4" s="62" t="inlineStr"/>
+      <c r="A4" s="62" t="inlineStr"/>
+      <c r="B4" s="63" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="61" t="inlineStr">
+      <c r="A5" s="62" t="inlineStr">
         <is>
           <t>1. RELEVAMIENTO</t>
         </is>
       </c>
-      <c r="B5" s="61" t="inlineStr">
+      <c r="B5" s="62" t="inlineStr">
         <is>
           <t>Las columnas se identificaron en el plano cruzando el rotulo COL con un rectangulo</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="61" t="inlineStr"/>
-      <c r="B6" s="62" t="inlineStr">
+      <c r="A6" s="62" t="inlineStr"/>
+      <c r="B6" s="63" t="inlineStr">
         <is>
           <t>de la misma seccion a menos de 26 pt. Resultaron 9 en PB y 4 en PA.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="61" t="inlineStr"/>
-      <c r="B7" s="62" t="inlineStr">
+      <c r="A7" s="62" t="inlineStr"/>
+      <c r="B7" s="63" t="inlineStr">
         <is>
           <t>Las 4 de PA caen exactamente sobre C6, C7, C8 y C9 de PB, y ademas tienen la misma</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="61" t="inlineStr"/>
-      <c r="B8" s="62" t="inlineStr">
+      <c r="A8" s="62" t="inlineStr"/>
+      <c r="B8" s="63" t="inlineStr">
         <is>
           <t>seccion, lo que confirma que la correspondencia entre plantas es correcta.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="61" t="inlineStr"/>
-      <c r="B9" s="62" t="inlineStr">
+      <c r="A9" s="62" t="inlineStr"/>
+      <c r="B9" s="63" t="inlineStr">
         <is>
           <t>La C01 de 10x10 esta confirmada por el proyectista aunque el computo metrico no</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="61" t="inlineStr"/>
-      <c r="B10" s="62" t="inlineStr">
+      <c r="A10" s="62" t="inlineStr"/>
+      <c r="B10" s="63" t="inlineStr">
         <is>
           <t>la incluya en su item 4.1.3: ese computo esta incompleto en ese punto.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="61" t="inlineStr"/>
-      <c r="B11" s="62" t="inlineStr"/>
+      <c r="A11" s="62" t="inlineStr"/>
+      <c r="B11" s="63" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="61" t="inlineStr">
+      <c r="A12" s="62" t="inlineStr">
         <is>
           <t>2. ALTURAS</t>
         </is>
       </c>
-      <c r="B12" s="61" t="inlineStr">
+      <c r="B12" s="62" t="inlineStr">
         <is>
           <t>PB 3,15 m y PA 3,22 m, los mismos valores de la planilla de la catedra, coherentes</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="61" t="inlineStr"/>
-      <c r="B13" s="62" t="inlineStr">
+      <c r="A13" s="62" t="inlineStr"/>
+      <c r="B13" s="63" t="inlineStr">
         <is>
           <t>con los niveles del plano (N.F.L +3,50 del entrepiso y +6,80 del techo).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="61" t="inlineStr"/>
-      <c r="B14" s="62" t="inlineStr"/>
+      <c r="A14" s="62" t="inlineStr"/>
+      <c r="B14" s="63" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="61" t="inlineStr">
+      <c r="A15" s="62" t="inlineStr">
         <is>
           <t>3. ARMADURA</t>
         </is>
       </c>
-      <c r="B15" s="61" t="inlineStr">
+      <c r="B15" s="62" t="inlineStr">
         <is>
           <t>As = 0,008 x area (cuantia minima, el mismo criterio de la planilla modelo).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="61" t="inlineStr"/>
-      <c r="B16" s="62" t="inlineStr">
+      <c r="A16" s="62" t="inlineStr"/>
+      <c r="B16" s="63" t="inlineStr">
         <is>
           <t>Se adoptan 4 barras del 12 en todas: 4,52 cm2, que cubre la minima en toda seccion.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="61" t="inlineStr"/>
-      <c r="B17" s="62" t="inlineStr">
+      <c r="A17" s="62" t="inlineStr"/>
+      <c r="B17" s="63" t="inlineStr">
         <is>
           <t>Separacion de estribos = min(12 x diam. long. ; 48 x diam. estribo ; lado menor),</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="61" t="inlineStr"/>
-      <c r="B18" s="62" t="inlineStr">
+      <c r="A18" s="62" t="inlineStr"/>
+      <c r="B18" s="63" t="inlineStr">
         <is>
           <t>redondeada hacia abajo a multiplo de 5. Para 4d12 con estribo d6 da 10 cm.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="61" t="inlineStr"/>
-      <c r="B19" s="62" t="inlineStr">
+      <c r="A19" s="62" t="inlineStr"/>
+      <c r="B19" s="63" t="inlineStr">
         <is>
           <t>La planilla de la catedra adopta 20 cm: ese valor supera el limite reglamentario.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="61" t="inlineStr"/>
-      <c r="B20" s="62" t="inlineStr"/>
+      <c r="A20" s="62" t="inlineStr"/>
+      <c r="B20" s="63" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="61" t="inlineStr">
+      <c r="A21" s="62" t="inlineStr">
         <is>
           <t>4. CAPACIDAD</t>
         </is>
       </c>
-      <c r="B21" s="61" t="inlineStr">
+      <c r="B21" s="62" t="inlineStr">
         <is>
           <t>phi Pn = 0,65 x 0,80 x [0,85 f'c (Ag - As) + fy As]     (columna zunchada con estribos)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="61" t="inlineStr"/>
-      <c r="B22" s="62" t="inlineStr">
+      <c r="A22" s="62" t="inlineStr"/>
+      <c r="B22" s="63" t="inlineStr">
         <is>
           <t xml:space="preserve">  15x30 con 4d12 -&gt; 51,2 t        20x20 con 4d12 -&gt; 46,6 t</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="61" t="inlineStr"/>
-      <c r="B23" s="62" t="inlineStr"/>
+      <c r="A23" s="62" t="inlineStr"/>
+      <c r="B23" s="63" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="61" t="inlineStr">
+      <c r="A24" s="62" t="inlineStr">
         <is>
           <t>5. CARGAS</t>
         </is>
       </c>
-      <c r="B24" s="61" t="inlineStr">
+      <c r="B24" s="62" t="inlineStr">
         <is>
           <t>La columna CARGA (t) viene cargada con una bajada automatica: suma de las</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="61" t="inlineStr"/>
-      <c r="B25" s="62" t="inlineStr">
+      <c r="A25" s="62" t="inlineStr"/>
+      <c r="B25" s="63" t="inlineStr">
         <is>
           <t>reacciones de las vigas que apoyan en cada columna (tomadas de la planilla de</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="61" t="inlineStr"/>
-      <c r="B26" s="62" t="inlineStr">
+      <c r="A26" s="62" t="inlineStr"/>
+      <c r="B26" s="63" t="inlineStr">
         <is>
           <t>vigas), mas el peso propio, mas lo que baja de la columna del nivel superior.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="61" t="inlineStr"/>
-      <c r="B27" s="62" t="inlineStr">
+      <c r="A27" s="62" t="inlineStr"/>
+      <c r="B27" s="63" t="inlineStr">
         <is>
           <t>ES UNA CARGA PROVISORIA Y ES UN PISO, NO EL VALOR REAL: 20 de los 60 extremos</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="61" t="inlineStr"/>
-      <c r="B28" s="62" t="inlineStr">
+      <c r="A28" s="62" t="inlineStr"/>
+      <c r="B28" s="63" t="inlineStr">
         <is>
           <t>de viga no pudieron asignarse a ninguna columna porque apoyan en otra viga, en</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="61" t="inlineStr"/>
-      <c r="B29" s="62" t="inlineStr">
+      <c r="A29" s="62" t="inlineStr"/>
+      <c r="B29" s="63" t="inlineStr">
         <is>
           <t>un tabique o en la medianera, y esas reacciones no estan sumadas.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="61" t="inlineStr"/>
-      <c r="B30" s="62" t="inlineStr">
+      <c r="A30" s="62" t="inlineStr"/>
+      <c r="B30" s="63" t="inlineStr">
         <is>
           <t>Para cerrarla hay que indicar, para cada uno de esos 20 extremos, en que apoya.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="61" t="inlineStr"/>
-      <c r="B31" s="62" t="inlineStr">
+      <c r="A31" s="62" t="inlineStr"/>
+      <c r="B31" s="63" t="inlineStr">
         <is>
           <t>Mientras tanto la columna es editable: al corregir un valor todo recalcula.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="61" t="inlineStr"/>
-      <c r="B32" s="62" t="inlineStr">
+      <c r="A32" s="62" t="inlineStr"/>
+      <c r="B32" s="63" t="inlineStr">
         <is>
           <t>Ademas son cargas MAYORADAS, coherentes con la planilla de vigas. Si la catedra</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="61" t="inlineStr"/>
-      <c r="B33" s="62" t="inlineStr">
+      <c r="A33" s="62" t="inlineStr"/>
+      <c r="B33" s="63" t="inlineStr">
         <is>
           <t>pide cargas de servicio, dividir por el coeficiente que corresponda.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="61" t="inlineStr"/>
-      <c r="B34" s="62" t="inlineStr"/>
+      <c r="A34" s="62" t="inlineStr"/>
+      <c r="B34" s="63" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="61" t="inlineStr">
+      <c r="A35" s="62" t="inlineStr">
         <is>
           <t>6. ESBELTEZ</t>
         </is>
       </c>
-      <c r="B35" s="61" t="inlineStr">
+      <c r="B35" s="62" t="inlineStr">
         <is>
           <t>Todas las columnas son esbeltas: con lado menor de 15 cm y 3,15 m de altura,</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="61" t="inlineStr"/>
-      <c r="B36" s="62" t="inlineStr">
+      <c r="A36" s="62" t="inlineStr"/>
+      <c r="B36" s="63" t="inlineStr">
         <is>
           <t>k lu / r = 70, muy por encima del limite de 34 por debajo del cual se puede</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="61" t="inlineStr"/>
-      <c r="B37" s="62" t="inlineStr">
+      <c r="A37" s="62" t="inlineStr"/>
+      <c r="B37" s="63" t="inlineStr">
         <is>
           <t>despreciar el pandeo. En la practica el llenado de mamposteria las arriostra, pero</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="61" t="inlineStr"/>
-      <c r="B38" s="62" t="inlineStr">
+      <c r="A38" s="62" t="inlineStr"/>
+      <c r="B38" s="63" t="inlineStr">
         <is>
           <t>si la catedra lo pide hay que verificar segundo orden. La planilla lo marca.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="61" t="inlineStr"/>
-      <c r="B39" s="62" t="inlineStr"/>
+      <c r="A39" s="62" t="inlineStr"/>
+      <c r="B39" s="63" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="61" t="inlineStr">
+      <c r="A40" s="62" t="inlineStr">
         <is>
           <t>7. LA DE 10x10</t>
         </is>
       </c>
-      <c r="B40" s="61" t="inlineStr">
+      <c r="B40" s="62" t="inlineStr">
         <is>
           <t>Existe, confirmada por el proyectista, y el computo metrico la omite. Con 10 cm</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="61" t="inlineStr"/>
-      <c r="B41" s="62" t="inlineStr">
+      <c r="A41" s="62" t="inlineStr"/>
+      <c r="B41" s="63" t="inlineStr">
         <is>
           <t>de lado y 3,15 m de altura su esbeltez es k lu / r = 105, tres veces el limite</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="61" t="inlineStr"/>
-      <c r="B42" s="62" t="inlineStr">
+      <c r="A42" s="62" t="inlineStr"/>
+      <c r="B42" s="63" t="inlineStr">
         <is>
           <t>por debajo del cual se puede despreciar el pandeo, y su capacidad es de 18,7 t</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="61" t="inlineStr"/>
-      <c r="B43" s="62" t="inlineStr">
+      <c r="A43" s="62" t="inlineStr"/>
+      <c r="B43" s="63" t="inlineStr">
         <is>
           <t>contra los 51 de una 15x30. Es el punto mas delicado del conjunto: conviene</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="61" t="inlineStr"/>
-      <c r="B44" s="62" t="inlineStr">
+      <c r="A44" s="62" t="inlineStr"/>
+      <c r="B44" s="63" t="inlineStr">
         <is>
           <t>verificarla a segundo orden en serio, no con la formula de compresion simple.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="61" t="inlineStr"/>
-      <c r="B45" s="62" t="inlineStr"/>
+      <c r="A45" s="62" t="inlineStr"/>
+      <c r="B45" s="63" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="61" t="inlineStr">
+      <c r="A46" s="62" t="inlineStr">
         <is>
           <t>LIMITACIONES</t>
         </is>
       </c>
-      <c r="B46" s="61" t="inlineStr">
+      <c r="B46" s="62" t="inlineStr">
         <is>
           <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="61" t="inlineStr"/>
-      <c r="B47" s="62" t="inlineStr">
+      <c r="A47" s="62" t="inlineStr"/>
+      <c r="B47" s="63" t="inlineStr">
         <is>
           <t>No se verifica flexion compuesta: las columnas de borde reciben momento de las</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="61" t="inlineStr"/>
-      <c r="B48" s="62" t="inlineStr">
+      <c r="A48" s="62" t="inlineStr"/>
+      <c r="B48" s="63" t="inlineStr">
         <is>
           <t>vigas invertidas y trabajan a flexo-compresion, no a compresion simple.</t>
         </is>
@@ -5571,7 +5781,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="63" t="inlineStr">
+      <c r="A1" s="64" t="inlineStr">
         <is>
           <t>VIGAS DE FUNDACION - inventario. Calculo pendiente: va despues de columnas.</t>
         </is>
@@ -5713,7 +5923,7 @@
       <c r="D9" s="11" t="n">
         <v>533</v>
       </c>
-      <c r="E9" s="64" t="inlineStr">
+      <c r="E9" s="65" t="inlineStr">
         <is>
           <t>Ancho cortado en el PDF: confirmar 20 o 22 cm</t>
         </is>
@@ -5779,7 +5989,7 @@
       <c r="B13" s="11" t="n"/>
       <c r="C13" s="11" t="n"/>
       <c r="D13" s="11" t="n"/>
-      <c r="E13" s="64" t="inlineStr">
+      <c r="E13" s="65" t="inlineStr">
         <is>
           <t>Cota no legible: completar</t>
         </is>
@@ -5794,7 +6004,7 @@
       <c r="B14" s="11" t="n"/>
       <c r="C14" s="11" t="n"/>
       <c r="D14" s="11" t="n"/>
-      <c r="E14" s="64" t="inlineStr">
+      <c r="E14" s="65" t="inlineStr">
         <is>
           <t>Cota no legible: completar</t>
         </is>
@@ -5996,7 +6206,7 @@
       <c r="B26" s="11" t="n"/>
       <c r="C26" s="11" t="n"/>
       <c r="D26" s="11" t="n"/>
-      <c r="E26" s="64" t="inlineStr">
+      <c r="E26" s="65" t="inlineStr">
         <is>
           <t>Cota no legible: completar</t>
         </is>

</xml_diff>

<commit_message>
Cargar los cinco tabiques de planta alta
El proyectista indica que vigas apoyan en cada uno: T9 recibe VI 14,
T10 recibe VI 12, T11 recibe VI 13b y T12 recibe VI 17 mas VI 15b.
T13 no recibe vigas, continua el tabique T06c de planta baja, y se
carga con su peso propio. Los trece tabiques quedan verificando.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -253,7 +253,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -368,12 +368,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -3496,7 +3490,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="45" t="inlineStr">
+      <c r="A1" s="43" t="inlineStr">
         <is>
           <t>DATOS DE PARTIDA - COLUMNAS</t>
         </is>
@@ -3510,29 +3504,29 @@
       <c r="C2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="46" t="inlineStr">
+      <c r="A3" s="44" t="inlineStr">
         <is>
           <t>MATERIALES Y CRITERIOS</t>
         </is>
       </c>
-      <c r="B3" s="47" t="inlineStr">
+      <c r="B3" s="45" t="inlineStr">
         <is>
           <t>valor</t>
         </is>
       </c>
-      <c r="C3" s="47" t="inlineStr">
+      <c r="C3" s="45" t="inlineStr">
         <is>
           <t>unidad</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="48" t="inlineStr">
+      <c r="A4" s="46" t="inlineStr">
         <is>
           <t>Hormigon H-21   f'c</t>
         </is>
       </c>
-      <c r="B4" s="49" t="n">
+      <c r="B4" s="47" t="n">
         <v>210</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
@@ -3542,12 +3536,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="48" t="inlineStr">
+      <c r="A5" s="46" t="inlineStr">
         <is>
           <t>Acero 42/50   fy</t>
         </is>
       </c>
-      <c r="B5" s="49" t="n">
+      <c r="B5" s="47" t="n">
         <v>4200</v>
       </c>
       <c r="C5" s="11" t="inlineStr">
@@ -3557,12 +3551,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="48" t="inlineStr">
+      <c r="A6" s="46" t="inlineStr">
         <is>
           <t>Peso especifico H.A.</t>
         </is>
       </c>
-      <c r="B6" s="49" t="n">
+      <c r="B6" s="47" t="n">
         <v>2400</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
@@ -3572,12 +3566,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="48" t="inlineStr">
+      <c r="A7" s="46" t="inlineStr">
         <is>
           <t>phi compresion (estribos)</t>
         </is>
       </c>
-      <c r="B7" s="49" t="n">
+      <c r="B7" s="47" t="n">
         <v>0.65</v>
       </c>
       <c r="C7" s="11" t="inlineStr">
@@ -3587,12 +3581,12 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="48" t="inlineStr">
+      <c r="A8" s="46" t="inlineStr">
         <is>
           <t>Cuantia minima</t>
         </is>
       </c>
-      <c r="B8" s="49" t="n">
+      <c r="B8" s="47" t="n">
         <v>0.008</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
@@ -3602,12 +3596,12 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="48" t="inlineStr">
+      <c r="A9" s="46" t="inlineStr">
         <is>
           <t>Altura PB</t>
         </is>
       </c>
-      <c r="B9" s="49" t="n">
+      <c r="B9" s="47" t="n">
         <v>3.15</v>
       </c>
       <c r="C9" s="11" t="inlineStr">
@@ -3617,12 +3611,12 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="48" t="inlineStr">
+      <c r="A10" s="46" t="inlineStr">
         <is>
           <t>Altura PA</t>
         </is>
       </c>
-      <c r="B10" s="49" t="n">
+      <c r="B10" s="47" t="n">
         <v>3.22</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
@@ -3675,7 +3669,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="45" t="inlineStr">
+      <c r="A1" s="43" t="inlineStr">
         <is>
           <t>DATOS DE PARTIDA - PILOTES</t>
         </is>
@@ -3693,22 +3687,22 @@
       <c r="E2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="46" t="inlineStr">
+      <c r="A3" s="44" t="inlineStr">
         <is>
           <t>PARAMETRO</t>
         </is>
       </c>
-      <c r="B3" s="47" t="inlineStr">
+      <c r="B3" s="45" t="inlineStr">
         <is>
           <t>valor</t>
         </is>
       </c>
-      <c r="C3" s="47" t="inlineStr">
+      <c r="C3" s="45" t="inlineStr">
         <is>
           <t>unidad</t>
         </is>
       </c>
-      <c r="D3" s="46" t="inlineStr">
+      <c r="D3" s="44" t="inlineStr">
         <is>
           <t>origen</t>
         </is>
@@ -3716,12 +3710,12 @@
       <c r="E3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="48" t="inlineStr">
+      <c r="A4" s="46" t="inlineStr">
         <is>
           <t>Carga admisible por pilote</t>
         </is>
       </c>
-      <c r="B4" s="49" t="n">
+      <c r="B4" s="47" t="n">
         <v>12</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
@@ -3729,7 +3723,7 @@
           <t>t</t>
         </is>
       </c>
-      <c r="D4" s="53" t="inlineStr">
+      <c r="D4" s="51" t="inlineStr">
         <is>
           <t>ESTIMADA. Falta el estudio de suelos: cambiar aca y recalcula todo.</t>
         </is>
@@ -3737,12 +3731,12 @@
       <c r="E4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="48" t="inlineStr">
+      <c r="A5" s="46" t="inlineStr">
         <is>
           <t>Tension admisible del terreno</t>
         </is>
       </c>
-      <c r="B5" s="49" t="n">
+      <c r="B5" s="47" t="n">
         <v>2</v>
       </c>
       <c r="C5" s="11" t="inlineStr">
@@ -3750,7 +3744,7 @@
           <t>kg/cm2</t>
         </is>
       </c>
-      <c r="D5" s="53" t="inlineStr">
+      <c r="D5" s="51" t="inlineStr">
         <is>
           <t>Dato real, tomado del encabezado del calculo de bases.</t>
         </is>
@@ -3758,12 +3752,12 @@
       <c r="E5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="48" t="inlineStr">
+      <c r="A6" s="46" t="inlineStr">
         <is>
           <t>Diametro del pilote</t>
         </is>
       </c>
-      <c r="B6" s="49" t="n">
+      <c r="B6" s="47" t="n">
         <v>30</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
@@ -3771,7 +3765,7 @@
           <t>cm</t>
         </is>
       </c>
-      <c r="D6" s="53" t="inlineStr">
+      <c r="D6" s="51" t="inlineStr">
         <is>
           <t>Nota del plano: todos los pilotes son O30.</t>
         </is>
@@ -3779,12 +3773,12 @@
       <c r="E6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="48" t="inlineStr">
+      <c r="A7" s="46" t="inlineStr">
         <is>
           <t>Profundidad</t>
         </is>
       </c>
-      <c r="B7" s="49" t="n">
+      <c r="B7" s="47" t="n">
         <v>-4.5</v>
       </c>
       <c r="C7" s="11" t="inlineStr">
@@ -3792,7 +3786,7 @@
           <t>m</t>
         </is>
       </c>
-      <c r="D7" s="53" t="inlineStr">
+      <c r="D7" s="51" t="inlineStr">
         <is>
           <t>Nota del plano: h = -4,50 m desde la cota +-0,00 de vereda.</t>
         </is>
@@ -3800,12 +3794,12 @@
       <c r="E7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="48" t="inlineStr">
+      <c r="A8" s="46" t="inlineStr">
         <is>
           <t>Coef. de mayoracion adoptado</t>
         </is>
       </c>
-      <c r="B8" s="49" t="n">
+      <c r="B8" s="47" t="n">
         <v>1.4</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
@@ -3813,7 +3807,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="D8" s="53" t="inlineStr">
+      <c r="D8" s="51" t="inlineStr">
         <is>
           <t>Para pasar de carga mayorada a carga de servicio.</t>
         </is>
@@ -3828,7 +3822,7 @@
       <c r="E9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="59" t="inlineStr">
+      <c r="A10" s="57" t="inlineStr">
         <is>
           <t>TIPOS DE PILOTE  (nota general del plano: CANTIDAD 33 PILOTES)</t>
         </is>
@@ -3839,105 +3833,105 @@
       <c r="E10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="47" t="inlineStr">
+      <c r="A11" s="45" t="inlineStr">
         <is>
           <t>tipo</t>
         </is>
       </c>
-      <c r="B11" s="47" t="inlineStr">
+      <c r="B11" s="45" t="inlineStr">
         <is>
           <t>cantidad</t>
         </is>
       </c>
-      <c r="C11" s="47" t="inlineStr">
+      <c r="C11" s="45" t="inlineStr">
         <is>
           <t>cota fundacion</t>
         </is>
       </c>
-      <c r="D11" s="47" t="inlineStr">
+      <c r="D11" s="45" t="inlineStr">
         <is>
           <t>nivel llenado</t>
         </is>
       </c>
-      <c r="E11" s="47" t="inlineStr">
+      <c r="E11" s="45" t="inlineStr">
         <is>
           <t>long. hormigon</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="48" t="inlineStr">
+      <c r="A12" s="46" t="inlineStr">
         <is>
           <t>Pilote tipo "A"</t>
         </is>
       </c>
-      <c r="B12" s="60" t="n">
+      <c r="B12" s="58" t="n">
         <v>8</v>
       </c>
-      <c r="C12" s="60" t="n">
+      <c r="C12" s="58" t="n">
         <v>-4.5</v>
       </c>
-      <c r="D12" s="60" t="n">
+      <c r="D12" s="58" t="n">
         <v>-0.4</v>
       </c>
-      <c r="E12" s="60" t="n">
+      <c r="E12" s="58" t="n">
         <v>4.1</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="48" t="inlineStr">
+      <c r="A13" s="46" t="inlineStr">
         <is>
           <t>Pilote tipo "B"</t>
         </is>
       </c>
-      <c r="B13" s="60" t="n">
+      <c r="B13" s="58" t="n">
         <v>5</v>
       </c>
-      <c r="C13" s="60" t="n">
+      <c r="C13" s="58" t="n">
         <v>-4.5</v>
       </c>
-      <c r="D13" s="60" t="n">
+      <c r="D13" s="58" t="n">
         <v>-0.35</v>
       </c>
-      <c r="E13" s="60" t="n">
+      <c r="E13" s="58" t="n">
         <v>4.15</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="48" t="inlineStr">
+      <c r="A14" s="46" t="inlineStr">
         <is>
           <t>Pilote tipo "C"</t>
         </is>
       </c>
-      <c r="B14" s="60" t="n">
+      <c r="B14" s="58" t="n">
         <v>16</v>
       </c>
-      <c r="C14" s="60" t="n">
+      <c r="C14" s="58" t="n">
         <v>-4.5</v>
       </c>
-      <c r="D14" s="60" t="n">
+      <c r="D14" s="58" t="n">
         <v>-0.05</v>
       </c>
-      <c r="E14" s="60" t="n">
+      <c r="E14" s="58" t="n">
         <v>4.45</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="48" t="inlineStr">
+      <c r="A15" s="46" t="inlineStr">
         <is>
           <t>Pilote tipo "D"</t>
         </is>
       </c>
-      <c r="B15" s="60" t="n">
+      <c r="B15" s="58" t="n">
         <v>4</v>
       </c>
-      <c r="C15" s="60" t="n">
+      <c r="C15" s="58" t="n">
         <v>-4.5</v>
       </c>
-      <c r="D15" s="60" t="n">
+      <c r="D15" s="58" t="n">
         <v>-0.1</v>
       </c>
-      <c r="E15" s="60" t="n">
+      <c r="E15" s="58" t="n">
         <v>4.4</v>
       </c>
     </row>
@@ -3949,7 +3943,7 @@
       <c r="E16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="44" t="inlineStr">
+      <c r="A17" s="42" t="inlineStr">
         <is>
           <t>Los cuatro tipos se funden a -4,50 m; se diferencian en el nivel de llenado de hormigon, o sea en la longitud real del fuste.</t>
         </is>
@@ -3978,7 +3972,7 @@
       <c r="E19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="59" t="inlineStr">
+      <c r="A20" s="57" t="inlineStr">
         <is>
           <t>COMO SE ESTIMO LA CARGA ADMISIBLE</t>
         </is>
@@ -3989,7 +3983,7 @@
       <c r="E20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="44" t="inlineStr">
+      <c r="A21" s="42" t="inlineStr">
         <is>
           <t>Pilote O30: area de punta 0,0707 m2. Punta  0,0707 x 20 t/m2 = 1,4 t.</t>
         </is>
@@ -4000,7 +3994,7 @@
       <c r="E21" s="2" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="44" t="inlineStr">
+      <c r="A22" s="42" t="inlineStr">
         <is>
           <t>Area lateral segun el tipo: 3,86 m2 el A, 3,91 el B, 4,19 el C y 4,15 el D.</t>
         </is>
@@ -4011,7 +4005,7 @@
       <c r="E22" s="2" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="44" t="inlineStr">
+      <c r="A23" s="42" t="inlineStr">
         <is>
           <t>Con una adherencia de 2,5 t/m2 la capacidad va de 11,1 t el tipo A a 11,9 t el C:</t>
         </is>
@@ -4022,7 +4016,7 @@
       <c r="E23" s="2" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="44" t="inlineStr">
+      <c r="A24" s="42" t="inlineStr">
         <is>
           <t>la diferencia entre tipos es menor al 8 por ciento, por eso se adopta un unico</t>
         </is>
@@ -4033,7 +4027,7 @@
       <c r="E24" s="2" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="44" t="inlineStr">
+      <c r="A25" s="42" t="inlineStr">
         <is>
           <t>valor de 12 t para todos, en lugar de uno por tipo.</t>
         </is>
@@ -4044,7 +4038,7 @@
       <c r="E25" s="2" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="44" t="inlineStr"/>
+      <c r="A26" s="42" t="inlineStr"/>
       <c r="B26" s="2" t="n"/>
       <c r="C26" s="2" t="n"/>
       <c r="D26" s="2" t="n"/>
@@ -4062,7 +4056,7 @@
       <c r="E27" s="2" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="44" t="inlineStr">
+      <c r="A28" s="42" t="inlineStr">
         <is>
           <t>con las cargas de esta planilla, para que el esquema funcione cada pilote</t>
         </is>
@@ -4073,7 +4067,7 @@
       <c r="E28" s="2" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="44" t="inlineStr">
+      <c r="A29" s="42" t="inlineStr">
         <is>
           <t>tiene que admitir del orden de 20 t. Si el estudio de suelos da menos,</t>
         </is>
@@ -4084,7 +4078,7 @@
       <c r="E29" s="2" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="44" t="inlineStr">
+      <c r="A30" s="42" t="inlineStr">
         <is>
           <t>faltan pilotes; si da mas, el diseno esta holgado.</t>
         </is>
@@ -4095,14 +4089,14 @@
       <c r="E30" s="2" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="44" t="inlineStr"/>
+      <c r="A31" s="42" t="inlineStr"/>
       <c r="B31" s="2" t="n"/>
       <c r="C31" s="2" t="n"/>
       <c r="D31" s="2" t="n"/>
       <c r="E31" s="2" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="44" t="inlineStr">
+      <c r="A32" s="42" t="inlineStr">
         <is>
           <t>FALTA: la nota del plano remite a las planillas de cada tipo de pilote, que</t>
         </is>
@@ -4113,7 +4107,7 @@
       <c r="E32" s="2" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="44" t="inlineStr">
+      <c r="A33" s="42" t="inlineStr">
         <is>
           <t>traen la armadura y quiza la carga. Si aparecen, se cierra este punto.</t>
         </is>
@@ -4124,14 +4118,14 @@
       <c r="E33" s="2" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="44" t="inlineStr"/>
+      <c r="A34" s="42" t="inlineStr"/>
       <c r="B34" s="2" t="n"/>
       <c r="C34" s="2" t="n"/>
       <c r="D34" s="2" t="n"/>
       <c r="E34" s="2" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="44" t="inlineStr">
+      <c r="A35" s="42" t="inlineStr">
         <is>
           <t>La tension de 2 kg/cm2 que trae el calculo de bases es la del estrato</t>
         </is>
@@ -4142,7 +4136,7 @@
       <c r="E35" s="2" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="44" t="inlineStr">
+      <c r="A36" s="42" t="inlineStr">
         <is>
           <t>superficial, donde apoyaban las bases. Los pilotes llegan a -4,50 m y</t>
         </is>
@@ -4153,7 +4147,7 @@
       <c r="E36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="44" t="inlineStr">
+      <c r="A37" s="42" t="inlineStr">
         <is>
           <t>trabajan sobre todo por friccion: son dos cosas distintas.</t>
         </is>
@@ -4182,180 +4176,180 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="61" t="inlineStr">
+      <c r="A1" s="59" t="inlineStr">
         <is>
           <t>MEMORIA - ILUMINACION Y VENTILACION</t>
         </is>
       </c>
-      <c r="B1" s="62" t="inlineStr"/>
+      <c r="B1" s="60" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="62" t="inlineStr"/>
-      <c r="B2" s="63" t="inlineStr"/>
+      <c r="A2" s="60" t="inlineStr"/>
+      <c r="B2" s="61" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="62" t="inlineStr">
+      <c r="A3" s="60" t="inlineStr">
         <is>
           <t>CRITERIO</t>
         </is>
       </c>
-      <c r="B3" s="62" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t>Area de iluminacion requerida = superficie del local / 9</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="62" t="inlineStr"/>
-      <c r="B4" s="63" t="inlineStr">
+      <c r="A4" s="60" t="inlineStr"/>
+      <c r="B4" s="61" t="inlineStr">
         <is>
           <t>Area de ventilacion requerida = un tercio de la de iluminacion = superficie / 27</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="62" t="inlineStr"/>
-      <c r="B5" s="63" t="inlineStr">
+      <c r="A5" s="60" t="inlineStr"/>
+      <c r="B5" s="61" t="inlineStr">
         <is>
           <t>Area proyectada: la vidriada de la carpinteria para iluminacion, y la parte que</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="62" t="inlineStr"/>
-      <c r="B6" s="63" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr"/>
+      <c r="B6" s="61" t="inlineStr">
         <is>
           <t>realmente abre para ventilacion.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="62" t="inlineStr"/>
-      <c r="B7" s="63" t="inlineStr"/>
+      <c r="A7" s="60" t="inlineStr"/>
+      <c r="B7" s="61" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="62" t="inlineStr">
+      <c r="A8" s="60" t="inlineStr">
         <is>
           <t>RESULTADO</t>
         </is>
       </c>
-      <c r="B8" s="62" t="inlineStr">
+      <c r="B8" s="60" t="inlineStr">
         <is>
           <t>Los trece locales cumplen holgadamente iluminacion y ventilacion.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="62" t="inlineStr"/>
-      <c r="B9" s="63" t="inlineStr"/>
+      <c r="A9" s="60" t="inlineStr"/>
+      <c r="B9" s="61" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="62" t="inlineStr">
+      <c r="A10" s="60" t="inlineStr">
         <is>
           <t>CORRECCION</t>
         </is>
       </c>
-      <c r="B10" s="62" t="inlineStr">
+      <c r="B10" s="60" t="inlineStr">
         <is>
           <t>Local 07, Hall / ingreso: la planilla original traia 0,66 y 0,22, que son los</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="62" t="inlineStr"/>
-      <c r="B11" s="63" t="inlineStr">
+      <c r="A11" s="60" t="inlineStr"/>
+      <c r="B11" s="61" t="inlineStr">
         <is>
           <t>valores del local 03 (Lavadero, 6,0 m2). Con sus 3,50 x 2,15 = 7,53 m2 corresponden</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="62" t="inlineStr"/>
-      <c r="B12" s="63" t="inlineStr">
+      <c r="A12" s="60" t="inlineStr"/>
+      <c r="B12" s="61" t="inlineStr">
         <is>
           <t>0,84 y 0,28. No cambia el resultado, pero el numero no cerraba con la superficie</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="62" t="inlineStr"/>
-      <c r="B13" s="63" t="inlineStr">
+      <c r="A13" s="60" t="inlineStr"/>
+      <c r="B13" s="61" t="inlineStr">
         <is>
           <t>declarada y un verificador lo puede observar.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="62" t="inlineStr"/>
-      <c r="B14" s="63" t="inlineStr"/>
+      <c r="A14" s="60" t="inlineStr"/>
+      <c r="B14" s="61" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="62" t="inlineStr">
+      <c r="A15" s="60" t="inlineStr">
         <is>
           <t>A REVISAR</t>
         </is>
       </c>
-      <c r="B15" s="62" t="inlineStr">
+      <c r="B15" s="60" t="inlineStr">
         <is>
           <t>Local 14, Estar / Playroom: declara 5,00 m2 de ventilacion sobre 5,00 m2 de</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="62" t="inlineStr"/>
-      <c r="B16" s="63" t="inlineStr">
+      <c r="A16" s="60" t="inlineStr"/>
+      <c r="B16" s="61" t="inlineStr">
         <is>
           <t>iluminacion, es decir una carpinteria enteramente abrible. En los demas locales</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="62" t="inlineStr"/>
-      <c r="B17" s="63" t="inlineStr">
+      <c r="A17" s="60" t="inlineStr"/>
+      <c r="B17" s="61" t="inlineStr">
         <is>
           <t>la relacion es del 50 por ciento. Conviene verificar la carpinteria real.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="62" t="inlineStr"/>
-      <c r="B18" s="63" t="inlineStr"/>
+      <c r="A18" s="60" t="inlineStr"/>
+      <c r="B18" s="61" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="62" t="inlineStr"/>
-      <c r="B19" s="63" t="inlineStr">
+      <c r="A19" s="60" t="inlineStr"/>
+      <c r="B19" s="61" t="inlineStr">
         <is>
           <t>Local 02, Deposito: figura sin exigencia por no ser habitable. Son 11,8 m2</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="62" t="inlineStr"/>
-      <c r="B20" s="63" t="inlineStr">
+      <c r="A20" s="60" t="inlineStr"/>
+      <c r="B20" s="61" t="inlineStr">
         <is>
           <t>cerrados: si se lo considera habitable hay que preverle conducto.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="62" t="inlineStr"/>
-      <c r="B21" s="63" t="inlineStr"/>
+      <c r="A21" s="60" t="inlineStr"/>
+      <c r="B21" s="61" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="62" t="inlineStr">
+      <c r="A22" s="60" t="inlineStr">
         <is>
           <t>REDONDEOS</t>
         </is>
       </c>
-      <c r="B22" s="62" t="inlineStr">
+      <c r="B22" s="60" t="inlineStr">
         <is>
           <t>Diferencias menores que no afectan: local 03 da 5,95 m2 y figura 6,0;</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="62" t="inlineStr"/>
-      <c r="B23" s="63" t="inlineStr">
+      <c r="A23" s="60" t="inlineStr"/>
+      <c r="B23" s="61" t="inlineStr">
         <is>
           <t>local 09 da 12,25 y figura 12,3.</t>
         </is>
@@ -4380,592 +4374,592 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="61" t="inlineStr">
+      <c r="A1" s="59" t="inlineStr">
         <is>
           <t>MEMORIA DE CALCULO - VIGAS H°A°</t>
         </is>
       </c>
-      <c r="B1" s="62" t="inlineStr"/>
+      <c r="B1" s="60" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="62" t="inlineStr"/>
-      <c r="B2" s="63" t="inlineStr"/>
+      <c r="A2" s="60" t="inlineStr"/>
+      <c r="B2" s="61" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="62" t="inlineStr">
+      <c r="A3" s="60" t="inlineStr">
         <is>
           <t>NORMATIVA</t>
         </is>
       </c>
-      <c r="B3" s="62" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t>CIRSOC 201. Hormigon H-21 (f'c 210 kg/cm2). Acero 42/50 (fy 4200 kg/cm2).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="62" t="inlineStr">
+      <c r="A4" s="60" t="inlineStr">
         <is>
           <t>UNIDADES</t>
         </is>
       </c>
-      <c r="B4" s="62" t="inlineStr">
+      <c r="B4" s="60" t="inlineStr">
         <is>
           <t>Longitudes en m y cm. Cargas en kg/m. Momentos en kgm. Tensiones en kg/cm2.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="62" t="inlineStr">
+      <c r="A5" s="60" t="inlineStr">
         <is>
           <t>DIMENSIONES</t>
         </is>
       </c>
-      <c r="B5" s="62" t="inlineStr">
+      <c r="B5" s="60" t="inlineStr">
         <is>
           <t>b = ancho | h = altura util | d = altura total (igual criterio que la planilla de catedra).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="62" t="inlineStr"/>
-      <c r="B6" s="63" t="inlineStr"/>
+      <c r="A6" s="60" t="inlineStr"/>
+      <c r="B6" s="61" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="62" t="inlineStr">
+      <c r="A7" s="60" t="inlineStr">
         <is>
           <t>1. CARGAS</t>
         </is>
       </c>
-      <c r="B7" s="62" t="inlineStr"/>
+      <c r="B7" s="60" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="62" t="inlineStr">
+      <c r="A8" s="60" t="inlineStr">
         <is>
           <t>Entrepiso PA</t>
         </is>
       </c>
-      <c r="B8" s="63" t="inlineStr">
+      <c r="B8" s="61" t="inlineStr">
         <is>
           <t>Losa maciza 12 cm 300 + contrapiso 130 + carpeta 42 + piso 50 + cielorraso 20</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="62" t="inlineStr"/>
-      <c r="B9" s="63" t="inlineStr">
+      <c r="A9" s="60" t="inlineStr"/>
+      <c r="B9" s="61" t="inlineStr">
         <is>
           <t>g = 550 kg/m2       q = 200 kg/m2 (vivienda)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="62" t="inlineStr">
+      <c r="A10" s="60" t="inlineStr">
         <is>
           <t>Azotea</t>
         </is>
       </c>
-      <c r="B10" s="63" t="inlineStr">
+      <c r="B10" s="61" t="inlineStr">
         <is>
           <t>Losa 300 + contrapiso de pendiente 140 + carpeta 42 + aislacion y membrana 50 + cielorraso 20</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="62" t="inlineStr"/>
-      <c r="B11" s="63" t="inlineStr">
+      <c r="A11" s="60" t="inlineStr"/>
+      <c r="B11" s="61" t="inlineStr">
         <is>
           <t>g = 560 kg/m2       q = 100 kg/m2 (cubierta no accesible)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="62" t="inlineStr">
+      <c r="A12" s="60" t="inlineStr">
         <is>
           <t>Mamposteria</t>
         </is>
       </c>
-      <c r="B12" s="63" t="inlineStr">
+      <c r="B12" s="61" t="inlineStr">
         <is>
           <t>250 kg/m2. Altura 2,60 m en PA y 1,00 m de parapeto en azotea.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="62" t="inlineStr">
+      <c r="A13" s="60" t="inlineStr">
         <is>
           <t>Peso propio</t>
         </is>
       </c>
-      <c r="B13" s="63" t="inlineStr">
+      <c r="B13" s="61" t="inlineStr">
         <is>
           <t>2400 kg/m3 x b x d, viga por viga.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="62" t="inlineStr">
+      <c r="A14" s="60" t="inlineStr">
         <is>
           <t>Carga de calculo</t>
         </is>
       </c>
-      <c r="B14" s="63" t="inlineStr">
+      <c r="B14" s="61" t="inlineStr">
         <is>
           <t>p = 1,2 (g x B + peso propio + muro) + 1,6 (q x B)        B = ancho tributario</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="62" t="inlineStr"/>
-      <c r="B15" s="63" t="inlineStr"/>
+      <c r="A15" s="60" t="inlineStr"/>
+      <c r="B15" s="61" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="62" t="inlineStr">
+      <c r="A16" s="60" t="inlineStr">
         <is>
           <t>2. SOLICITACIONES</t>
         </is>
       </c>
-      <c r="B16" s="62" t="inlineStr">
+      <c r="B16" s="60" t="inlineStr">
         <is>
           <t>Coeficientes segun esquema (tabla en hoja Datos):</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="62" t="inlineStr"/>
-      <c r="B17" s="63" t="inlineStr">
+      <c r="A17" s="60" t="inlineStr"/>
+      <c r="B17" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  Simplemente apoyada   M = pL2/8                    R = 0,500 pL</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="62" t="inlineStr"/>
-      <c r="B18" s="63" t="inlineStr">
+      <c r="A18" s="60" t="inlineStr"/>
+      <c r="B18" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  Continua              M = pL2/14   Mapoyo = pL2/10  R = 0,575 pL</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="62" t="inlineStr"/>
-      <c r="B19" s="63" t="inlineStr">
+      <c r="A19" s="60" t="inlineStr"/>
+      <c r="B19" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  Empotrada-apoyada     M = 9pL2/128 Mapoyo = pL2/8   R = 0,625 pL</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="62" t="inlineStr"/>
-      <c r="B20" s="63" t="inlineStr">
+      <c r="A20" s="60" t="inlineStr"/>
+      <c r="B20" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  Biempotrada           M = pL2/24   Mapoyo = pL2/12  R = 0,500 pL</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="62" t="inlineStr"/>
-      <c r="B21" s="63" t="inlineStr">
+      <c r="A21" s="60" t="inlineStr"/>
+      <c r="B21" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  Voladizo                           Mapoyo = pL2/2   R = 1,000 pL</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="62" t="inlineStr"/>
-      <c r="B22" s="63" t="inlineStr"/>
+      <c r="A22" s="60" t="inlineStr"/>
+      <c r="B22" s="61" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="62" t="inlineStr">
+      <c r="A23" s="60" t="inlineStr">
         <is>
           <t>3. FLEXION</t>
         </is>
       </c>
-      <c r="B23" s="62" t="inlineStr">
+      <c r="B23" s="60" t="inlineStr">
         <is>
           <t>k = M / (phi b h2 f'c)      w = 1 - RAIZ(1 - 2k)      As = w b h f'c / fy</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="62" t="inlineStr"/>
-      <c r="B24" s="63" t="inlineStr">
+      <c r="A24" s="60" t="inlineStr"/>
+      <c r="B24" s="61" t="inlineStr">
         <is>
           <t>As min = 0,0033 b h       As max = 0,0163 b h (0,75 de la cuantia balanceada)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="62" t="inlineStr"/>
-      <c r="B25" s="63" t="inlineStr">
+      <c r="A25" s="60" t="inlineStr"/>
+      <c r="B25" s="61" t="inlineStr">
         <is>
           <t>Si la armadura no entra en una capa se disponen dos y el recubrimiento pasa a 6 cm.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="62" t="inlineStr"/>
-      <c r="B26" s="63" t="inlineStr"/>
+      <c r="A26" s="60" t="inlineStr"/>
+      <c r="B26" s="61" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="62" t="inlineStr">
+      <c r="A27" s="60" t="inlineStr">
         <is>
           <t>4. CORTE</t>
         </is>
       </c>
-      <c r="B27" s="62" t="inlineStr">
+      <c r="B27" s="60" t="inlineStr">
         <is>
           <t>T = R / (b x 0,85 h)       tension tangencial en el apoyo</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="62" t="inlineStr"/>
-      <c r="B28" s="63" t="inlineStr">
+      <c r="A28" s="60" t="inlineStr"/>
+      <c r="B28" s="61" t="inlineStr">
         <is>
           <t>Vc = 0,53 RAIZ(f'c) b h        phi Vn = 0,75 (Vc + Av fy h / s)  &gt;=  R</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="62" t="inlineStr"/>
-      <c r="B29" s="63" t="inlineStr">
+      <c r="A29" s="60" t="inlineStr"/>
+      <c r="B29" s="61" t="inlineStr">
         <is>
           <t>Av = 2 ramas. Se aumenta el diametro antes que cerrar la separacion por debajo de 10 cm.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="62" t="inlineStr"/>
-      <c r="B30" s="63" t="inlineStr"/>
+      <c r="A30" s="60" t="inlineStr"/>
+      <c r="B30" s="61" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="62" t="inlineStr">
+      <c r="A31" s="60" t="inlineStr">
         <is>
           <t>5. FLECHA</t>
         </is>
       </c>
-      <c r="B31" s="62" t="inlineStr">
+      <c r="B31" s="60" t="inlineStr">
         <is>
           <t>Altura minima: simplemente apoyada L/16, un extremo continuo L/18,5,</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="62" t="inlineStr"/>
-      <c r="B32" s="63" t="inlineStr">
+      <c r="A32" s="60" t="inlineStr"/>
+      <c r="B32" s="61" t="inlineStr">
         <is>
           <t>ambos extremos continuos L/21, voladizo L/8.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="62" t="inlineStr"/>
-      <c r="B33" s="63" t="inlineStr"/>
+      <c r="A33" s="60" t="inlineStr"/>
+      <c r="B33" s="61" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="62" t="inlineStr">
+      <c r="A34" s="60" t="inlineStr">
         <is>
           <t>6. VIGAS INVERTIDAS</t>
         </is>
       </c>
-      <c r="B34" s="62" t="inlineStr">
+      <c r="B34" s="60" t="inlineStr">
         <is>
           <t>Las vigas de BORDE son invertidas: sobresalen 70 cm por encima del fondo de</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="62" t="inlineStr"/>
-      <c r="B35" s="63" t="inlineStr">
+      <c r="A35" s="60" t="inlineStr"/>
+      <c r="B35" s="61" t="inlineStr">
         <is>
           <t>losa (cotas N.F.L +3,50 / N.S.V +4,20 y N.F.L +6,80 / N.S.V +7,50 del plano).</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="62" t="inlineStr"/>
-      <c r="B36" s="63" t="inlineStr">
+      <c r="A36" s="60" t="inlineStr"/>
+      <c r="B36" s="61" t="inlineStr">
         <is>
           <t>losa. Lo confirman las cotas del plano y el hecho de que el cielorraso sea de</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="62" t="inlineStr"/>
-      <c r="B37" s="63" t="inlineStr">
+      <c r="A37" s="60" t="inlineStr"/>
+      <c r="B37" s="61" t="inlineStr">
         <is>
           <t>VI 06 mide 14,00 m en total y es el cuarto borde de L07. Sobre su eje hay cuatro</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="62" t="inlineStr"/>
-      <c r="B38" s="63" t="inlineStr">
+      <c r="A38" s="60" t="inlineStr"/>
+      <c r="B38" s="61" t="inlineStr">
         <is>
           <t>columnas, de modo que trabaja como viga continua de tres tramos de 4,10, 4,32 y</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="62" t="inlineStr"/>
-      <c r="B39" s="63" t="inlineStr">
+      <c r="A39" s="60" t="inlineStr"/>
+      <c r="B39" s="61" t="inlineStr">
         <is>
           <t>6,53 m. Se calcula con el mayor, 6,53 m, que es el que gobierna.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="62" t="inlineStr"/>
-      <c r="B40" s="63" t="inlineStr">
+      <c r="A40" s="60" t="inlineStr"/>
+      <c r="B40" s="61" t="inlineStr">
         <is>
           <t>hormigon visto: una viga colgante quedaria a la vista. El computo metrico las</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="62" t="inlineStr"/>
-      <c r="B41" s="63" t="inlineStr">
+      <c r="A41" s="60" t="inlineStr"/>
+      <c r="B41" s="61" t="inlineStr">
         <is>
           <t>agrupa a las 28 bajo el rubro Vigas invertidas 15x70.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="62" t="inlineStr"/>
-      <c r="B42" s="63" t="inlineStr">
+      <c r="A42" s="60" t="inlineStr"/>
+      <c r="B42" s="61" t="inlineStr">
         <is>
           <t>Esto define donde la losa aporta ala comprimida:</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="62" t="inlineStr"/>
-      <c r="B43" s="63" t="inlineStr">
+      <c r="A43" s="60" t="inlineStr"/>
+      <c r="B43" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  viga COLGANTE  -&gt; la losa esta arriba  -&gt; ala util en el TRAMO (momento positivo)</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="62" t="inlineStr"/>
-      <c r="B44" s="63" t="inlineStr">
+      <c r="A44" s="60" t="inlineStr"/>
+      <c r="B44" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  viga INVERTIDA -&gt; la losa esta abajo   -&gt; ala util en el APOYO (momento negativo)</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="62" t="inlineStr"/>
-      <c r="B45" s="63" t="inlineStr">
+      <c r="A45" s="60" t="inlineStr"/>
+      <c r="B45" s="61" t="inlineStr">
         <is>
           <t>En la zona con ala se adopta b efectivo = min(L/4 ; b + 16 hf); en la otra, la</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="62" t="inlineStr"/>
-      <c r="B46" s="63" t="inlineStr">
+      <c r="A46" s="60" t="inlineStr"/>
+      <c r="B46" s="61" t="inlineStr">
         <is>
           <t>seccion es rectangular de ancho b. Las columnas b ef tramo y b ef apoyo lo muestran.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="62" t="inlineStr"/>
-      <c r="B47" s="63" t="inlineStr">
+      <c r="A47" s="60" t="inlineStr"/>
+      <c r="B47" s="61" t="inlineStr">
         <is>
           <t>PENDIENTE: las invertidas de BORDE (VI 01a, 01b, 07a, 07b, 07c, 11a, 11b, 11c,</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="62" t="inlineStr"/>
-      <c r="B48" s="63" t="inlineStr">
+      <c r="A48" s="60" t="inlineStr"/>
+      <c r="B48" s="61" t="inlineStr">
         <is>
           <t>15a y 15b) reciben la reaccion de la losa de un solo lado, excentrica respecto</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="62" t="inlineStr"/>
-      <c r="B49" s="63" t="inlineStr">
+      <c r="A49" s="60" t="inlineStr"/>
+      <c r="B49" s="61" t="inlineStr">
         <is>
           <t>de su eje, y quedan sometidas a TORSION. Esta planilla no la verifica.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="62" t="inlineStr"/>
-      <c r="B50" s="63" t="inlineStr"/>
+      <c r="A50" s="60" t="inlineStr"/>
+      <c r="B50" s="61" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="62" t="inlineStr">
+      <c r="A51" s="60" t="inlineStr">
         <is>
           <t>7. RESULTADO</t>
         </is>
       </c>
-      <c r="B51" s="62" t="inlineStr">
+      <c r="B51" s="60" t="inlineStr">
         <is>
           <t>30 vigas: 21 del entrepiso PA y 9 de la losa de techo. 28 verifican.</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="62" t="inlineStr"/>
-      <c r="B52" s="63" t="inlineStr">
+      <c r="A52" s="60" t="inlineStr"/>
+      <c r="B52" s="61" t="inlineStr">
         <is>
           <t>VI 02 (15x60, 9,88 m): recibe L02 y L03, B = 2,88 m. La armadura de apoyo</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="62" t="inlineStr"/>
-      <c r="B53" s="63" t="inlineStr">
+      <c r="A53" s="60" t="inlineStr"/>
+      <c r="B53" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">   necesaria ronda los 25 cm2 y supera la cuantia maxima. Los apoyos estan</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="62" t="inlineStr"/>
-      <c r="B54" s="63" t="inlineStr">
+      <c r="A54" s="60" t="inlineStr"/>
+      <c r="B54" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">   confirmados en obra: tabique T07 perpendicular arriba y COL 02 abajo, sin apoyo</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="62" t="inlineStr"/>
-      <c r="B55" s="63" t="inlineStr">
+      <c r="A55" s="60" t="inlineStr"/>
+      <c r="B55" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">   intermedio. Para esta carga la seccion necesaria es 15x75.</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="62" t="inlineStr"/>
-      <c r="B56" s="63" t="inlineStr">
+      <c r="A56" s="60" t="inlineStr"/>
+      <c r="B56" s="61" t="inlineStr">
         <is>
           <t>VCH 03a (40x13, 3,83 m). Recibe L03, B = 2,08 m, y no</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="62" t="inlineStr"/>
-      <c r="B57" s="63" t="inlineStr">
+      <c r="A57" s="60" t="inlineStr"/>
+      <c r="B57" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">   verifica: haria falta mas espesor. Tampoco verifica con B = 0,60 m, asi</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="62" t="inlineStr"/>
-      <c r="B58" s="63" t="inlineStr">
+      <c r="A58" s="60" t="inlineStr"/>
+      <c r="B58" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">   que el problema no es la hipotesis de carga sino la relacion luz/espesor. Una viga</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="62" t="inlineStr"/>
-      <c r="B59" s="63" t="inlineStr">
+      <c r="A59" s="60" t="inlineStr"/>
+      <c r="B59" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">   chata del mismo espesor que la losa no puede ser apoyo lineal de un pano de 4,15 m.</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="62" t="inlineStr"/>
-      <c r="B60" s="63" t="inlineStr">
+      <c r="A60" s="60" t="inlineStr"/>
+      <c r="B60" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">   Revisar si tiene un muro debajo que acorte su luz libre.</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="62" t="inlineStr"/>
-      <c r="B61" s="63" t="inlineStr">
+      <c r="A61" s="60" t="inlineStr"/>
+      <c r="B61" s="61" t="inlineStr">
         <is>
           <t>VCH 03a (40x13, 3,71 m): excede la cuantia maxima y no llega a la altura minima por</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="62" t="inlineStr"/>
-      <c r="B62" s="63" t="inlineStr">
+      <c r="A62" s="60" t="inlineStr"/>
+      <c r="B62" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">   flecha. Revisar el ancho tributario: si solo recibe el muro y no losa, baja mucho.</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="62" t="inlineStr"/>
-      <c r="B63" s="63" t="inlineStr"/>
+      <c r="A63" s="60" t="inlineStr"/>
+      <c r="B63" s="61" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="62" t="inlineStr">
+      <c r="A64" s="60" t="inlineStr">
         <is>
           <t>8. ALCANCE</t>
         </is>
       </c>
-      <c r="B64" s="63" t="inlineStr">
+      <c r="B64" s="61" t="inlineStr">
         <is>
           <t>No se incluyen las 31 vigas de fundacion (VF01 a VF18c): su calculo depende de las</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="62" t="inlineStr"/>
-      <c r="B65" s="63" t="inlineStr">
+      <c r="A65" s="60" t="inlineStr"/>
+      <c r="B65" s="61" t="inlineStr">
         <is>
           <t>cargas que bajan por las columnas y corresponde hacerlo despues. Tampoco losas ni columnas.</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="62" t="inlineStr"/>
-      <c r="B66" s="63" t="inlineStr"/>
+      <c r="A66" s="60" t="inlineStr"/>
+      <c r="B66" s="61" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="62" t="inlineStr">
+      <c r="A67" s="60" t="inlineStr">
         <is>
           <t>LIMITACIONES</t>
         </is>
       </c>
-      <c r="B67" s="62" t="inlineStr">
+      <c r="B67" s="60" t="inlineStr">
         <is>
           <t>El ancho tributario B esta relevado solo en</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="62" t="inlineStr"/>
-      <c r="B68" s="63" t="inlineStr">
+      <c r="A68" s="60" t="inlineStr"/>
+      <c r="B68" s="61" t="inlineStr">
         <is>
           <t>VI 02 (0,80 m) y VCH 03a (2,08 m). En las demas sigue adoptado en 2,00 m, a falta</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="62" t="inlineStr"/>
-      <c r="B69" s="63" t="inlineStr">
+      <c r="A69" s="60" t="inlineStr"/>
+      <c r="B69" s="61" t="inlineStr">
         <is>
           <t>hipotesis mas influyente del calculo: ajustarla viga por viga en la columna B trib.</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="62" t="inlineStr"/>
-      <c r="B70" s="63" t="inlineStr">
+      <c r="A70" s="60" t="inlineStr"/>
+      <c r="B70" s="61" t="inlineStr">
         <is>
           <t>El esquema se asigno por criterio: continua si integra una serie a-b-c o si supera 5,5 m.</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="62" t="inlineStr"/>
-      <c r="B71" s="63" t="inlineStr">
+      <c r="A71" s="60" t="inlineStr"/>
+      <c r="B71" s="61" t="inlineStr">
         <is>
           <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
         </is>
@@ -4990,368 +4984,368 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="61" t="inlineStr">
+      <c r="A1" s="59" t="inlineStr">
         <is>
           <t>MEMORIA DE CALCULO - LOSAS</t>
         </is>
       </c>
-      <c r="B1" s="62" t="inlineStr"/>
+      <c r="B1" s="60" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="62" t="inlineStr"/>
-      <c r="B2" s="63" t="inlineStr"/>
+      <c r="A2" s="60" t="inlineStr"/>
+      <c r="B2" s="61" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="62" t="inlineStr">
+      <c r="A3" s="60" t="inlineStr">
         <is>
           <t>METODO</t>
         </is>
       </c>
-      <c r="B3" s="62" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t>Tensiones admisibles, igual criterio que la planilla modelo de la catedra.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="62" t="inlineStr"/>
-      <c r="B4" s="63" t="inlineStr">
+      <c r="A4" s="60" t="inlineStr"/>
+      <c r="B4" s="61" t="inlineStr">
         <is>
           <t>Se verifico contra la fila de ejemplo: momentos y reacciones coinciden exactamente.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="62" t="inlineStr">
+      <c r="A5" s="60" t="inlineStr">
         <is>
           <t>MATERIALES</t>
         </is>
       </c>
-      <c r="B5" s="62" t="inlineStr">
+      <c r="B5" s="60" t="inlineStr">
         <is>
           <t>H-21 (f'c 210 kg/cm2). Acero 42/50 (fy 4200). Tension admisible 2400 kg/cm2.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="62" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>DIMENSIONES</t>
         </is>
       </c>
-      <c r="B6" s="62" t="inlineStr">
+      <c r="B6" s="60" t="inlineStr">
         <is>
           <t>h = altura util | d = espesor total. Recubrimiento 1,5 cm.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="62" t="inlineStr"/>
-      <c r="B7" s="63" t="inlineStr"/>
+      <c r="A7" s="60" t="inlineStr"/>
+      <c r="B7" s="61" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="62" t="inlineStr">
+      <c r="A8" s="60" t="inlineStr">
         <is>
           <t>1. CARGAS</t>
         </is>
       </c>
-      <c r="B8" s="62" t="inlineStr">
+      <c r="B8" s="60" t="inlineStr">
         <is>
           <t>p = peso propio + terminaciones + q      (cargas de servicio, sin mayorar)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="62" t="inlineStr"/>
-      <c r="B9" s="63" t="inlineStr">
+      <c r="A9" s="60" t="inlineStr"/>
+      <c r="B9" s="61" t="inlineStr">
         <is>
           <t>Peso propio = 2400 x d / 100, calculado con el espesor propio de cada losa.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="62" t="inlineStr">
+      <c r="A10" s="60" t="inlineStr">
         <is>
           <t>S/PB</t>
         </is>
       </c>
-      <c r="B10" s="63" t="inlineStr">
+      <c r="B10" s="61" t="inlineStr">
         <is>
           <t>Terminaciones 242 kg/m2 (contrapiso 130 + carpeta 42 + piso 50 + cielorraso 20)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="62" t="inlineStr"/>
-      <c r="B11" s="63" t="inlineStr">
+      <c r="A11" s="60" t="inlineStr"/>
+      <c r="B11" s="61" t="inlineStr">
         <is>
           <t>q = 200 kg/m2 (vivienda)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="62" t="inlineStr">
+      <c r="A12" s="60" t="inlineStr">
         <is>
           <t>S/PA</t>
         </is>
       </c>
-      <c r="B12" s="63" t="inlineStr">
+      <c r="B12" s="61" t="inlineStr">
         <is>
           <t>Terminaciones 252 kg/m2 (contrapiso pendiente 140 + carpeta 42 + aislacion 50 +</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="62" t="inlineStr"/>
-      <c r="B13" s="63" t="inlineStr">
+      <c r="A13" s="60" t="inlineStr"/>
+      <c r="B13" s="61" t="inlineStr">
         <is>
           <t>cielorraso 20).  q = 100 kg/m2 (azotea no accesible)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="62" t="inlineStr"/>
-      <c r="B14" s="63" t="inlineStr"/>
+      <c r="A14" s="60" t="inlineStr"/>
+      <c r="B14" s="61" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="62" t="inlineStr">
+      <c r="A15" s="60" t="inlineStr">
         <is>
           <t>2. SOLICITACIONES</t>
         </is>
       </c>
-      <c r="B15" s="62" t="inlineStr">
+      <c r="B15" s="60" t="inlineStr">
         <is>
           <t>M = coeficiente x p x L2, segun el grado de empotramiento:</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="62" t="inlineStr"/>
-      <c r="B16" s="63" t="inlineStr">
+      <c r="A16" s="60" t="inlineStr"/>
+      <c r="B16" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  1/8 simplemente apoyada    1/10 y 1/14 continua    1/12 biempotrada    1/2 voladizo</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="62" t="inlineStr"/>
-      <c r="B17" s="63" t="inlineStr">
+      <c r="A17" s="60" t="inlineStr"/>
+      <c r="B17" s="61" t="inlineStr">
         <is>
           <t>R = coeficiente x p x L. En voladizo Rx = p x L y Ry no corresponde.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="62" t="inlineStr"/>
-      <c r="B18" s="63" t="inlineStr"/>
+      <c r="A18" s="60" t="inlineStr"/>
+      <c r="B18" s="61" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="62" t="inlineStr">
+      <c r="A19" s="60" t="inlineStr">
         <is>
           <t>3. ARMADURA</t>
         </is>
       </c>
-      <c r="B19" s="62" t="inlineStr">
+      <c r="B19" s="60" t="inlineStr">
         <is>
           <t>As = M x 100 / (2400 x 0,9 x h)        [cm2/m]</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="62" t="inlineStr"/>
-      <c r="B20" s="63" t="inlineStr">
+      <c r="A20" s="60" t="inlineStr"/>
+      <c r="B20" s="61" t="inlineStr">
         <is>
           <t>separacion = 100 x area de la barra / As, redondeada, con maximo 20 cm</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="62" t="inlineStr"/>
-      <c r="B21" s="63" t="inlineStr">
+      <c r="A21" s="60" t="inlineStr"/>
+      <c r="B21" s="61" t="inlineStr">
         <is>
           <t>Armadura de reparticion = As / 5, con un minimo de 0,30 cm2/m</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="62" t="inlineStr"/>
-      <c r="B22" s="63" t="inlineStr"/>
+      <c r="A22" s="60" t="inlineStr"/>
+      <c r="B22" s="61" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="62" t="inlineStr">
+      <c r="A23" s="60" t="inlineStr">
         <is>
           <t>4. ESPESORES</t>
         </is>
       </c>
-      <c r="B23" s="62" t="inlineStr">
+      <c r="B23" s="60" t="inlineStr">
         <is>
           <t>Los espesores d se leyeron del plano: estan escritos debajo del rotulo de cada losa.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="62" t="inlineStr"/>
-      <c r="B24" s="63" t="inlineStr">
+      <c r="A24" s="60" t="inlineStr"/>
+      <c r="B24" s="61" t="inlineStr">
         <is>
           <t>S/PB:  L01 11 | L02 9 | L03 13 | L04 11 | L05 11 | L06 8 | L07 12 | L08 10</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="62" t="inlineStr"/>
-      <c r="B25" s="63" t="inlineStr">
+      <c r="A25" s="60" t="inlineStr"/>
+      <c r="B25" s="61" t="inlineStr">
         <is>
           <t>S/PA:  L09 13 | L10 12</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="62" t="inlineStr"/>
-      <c r="B26" s="63" t="inlineStr"/>
+      <c r="A26" s="60" t="inlineStr"/>
+      <c r="B26" s="61" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="62" t="inlineStr">
+      <c r="A27" s="60" t="inlineStr">
         <is>
           <t>5. LUCES</t>
         </is>
       </c>
-      <c r="B27" s="62" t="inlineStr">
+      <c r="B27" s="60" t="inlineStr">
         <is>
           <t>Relevadas en obra y aportadas por el proyectista. Dos losas son voladizo</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="62" t="inlineStr"/>
-      <c r="B28" s="63" t="inlineStr">
+      <c r="A28" s="60" t="inlineStr"/>
+      <c r="B28" s="61" t="inlineStr">
         <is>
           <t>(L02 de 0,80 m y L08 de 0,75 m) y se calculan con M = p L2 / 2.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="62" t="inlineStr"/>
-      <c r="B29" s="63" t="inlineStr"/>
+      <c r="A29" s="60" t="inlineStr"/>
+      <c r="B29" s="61" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="62" t="inlineStr">
+      <c r="A30" s="60" t="inlineStr">
         <is>
           <t>6. LOSAS CRUZADAS</t>
         </is>
       </c>
-      <c r="B30" s="63" t="inlineStr">
+      <c r="B30" s="61" t="inlineStr">
         <is>
           <t>L07 (4,85 x 5,60) y L10 (4,85 x 6,00) apoyan en los cuatro bordes y su relacion</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="62" t="inlineStr"/>
-      <c r="B31" s="63" t="inlineStr">
+      <c r="A31" s="60" t="inlineStr"/>
+      <c r="B31" s="61" t="inlineStr">
         <is>
           <t>de lados es menor que 2, por lo que trabajan en las dos direcciones.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="62" t="inlineStr"/>
-      <c r="B32" s="63" t="inlineStr">
+      <c r="A32" s="60" t="inlineStr"/>
+      <c r="B32" s="61" t="inlineStr">
         <is>
           <t>Se reparte la carga por el metodo de Marcus:   kx = ly4 / (lx4 + ly4)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="62" t="inlineStr"/>
-      <c r="B33" s="63" t="inlineStr">
+      <c r="A33" s="60" t="inlineStr"/>
+      <c r="B33" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  L07: ly/lx = 1,15  -&gt;  64% en la direccion corta, 36% en la larga</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="62" t="inlineStr"/>
-      <c r="B34" s="63" t="inlineStr">
+      <c r="A34" s="60" t="inlineStr"/>
+      <c r="B34" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  L10: ly/lx = 1,24  -&gt;  70% en la direccion corta, 30% en la larga</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="62" t="inlineStr"/>
-      <c r="B35" s="63" t="inlineStr">
+      <c r="A35" s="60" t="inlineStr"/>
+      <c r="B35" s="61" t="inlineStr">
         <is>
           <t>Cada una ocupa dos renglones, uno por direccion, con la fraccion de carga que</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="62" t="inlineStr"/>
-      <c r="B36" s="63" t="inlineStr">
+      <c r="A36" s="60" t="inlineStr"/>
+      <c r="B36" s="61" t="inlineStr">
         <is>
           <t>le toca ya aplicada en la columna CARGAS. Las dos armaduras se cruzan en obra:</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="62" t="inlineStr"/>
-      <c r="B37" s="63" t="inlineStr">
+      <c r="A37" s="60" t="inlineStr"/>
+      <c r="B37" s="61" t="inlineStr">
         <is>
           <t>la de la direccion corta va abajo, la de la larga arriba de aquella.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="62" t="inlineStr"/>
-      <c r="B38" s="63" t="inlineStr">
+      <c r="A38" s="60" t="inlineStr"/>
+      <c r="B38" s="61" t="inlineStr">
         <is>
           <t>La columna auxiliar luz transv. es la que dispara el reparto: si se borra, la</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="62" t="inlineStr"/>
-      <c r="B39" s="63" t="inlineStr">
+      <c r="A39" s="60" t="inlineStr"/>
+      <c r="B39" s="61" t="inlineStr">
         <is>
           <t>fila vuelve a calcularse como losa armada en una direccion.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="62" t="inlineStr"/>
-      <c r="B40" s="63" t="inlineStr"/>
+      <c r="A40" s="60" t="inlineStr"/>
+      <c r="B40" s="61" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="62" t="inlineStr">
+      <c r="A41" s="60" t="inlineStr">
         <is>
           <t>LIMITACIONES</t>
         </is>
       </c>
-      <c r="B41" s="62" t="inlineStr">
+      <c r="B41" s="60" t="inlineStr">
         <is>
           <t>El grado de empotramiento esta cargado en 1/8 salvo los dos voladizos (1/2). Si</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="62" t="inlineStr"/>
-      <c r="B42" s="63" t="inlineStr">
+      <c r="A42" s="60" t="inlineStr"/>
+      <c r="B42" s="61" t="inlineStr">
         <is>
           <t>alguna losa es continua sobre una viga corresponde 1/10 o 1/14: corregir en la columna.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="62" t="inlineStr"/>
-      <c r="B43" s="63" t="inlineStr">
+      <c r="A43" s="60" t="inlineStr"/>
+      <c r="B43" s="61" t="inlineStr">
         <is>
           <t>El diagrama de cargas es una imagen fija: si cambias el grado, cambialo a mano.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="62" t="inlineStr"/>
-      <c r="B44" s="63" t="inlineStr">
+      <c r="A44" s="60" t="inlineStr"/>
+      <c r="B44" s="61" t="inlineStr">
         <is>
           <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
         </is>
@@ -5376,384 +5370,384 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="61" t="inlineStr">
+      <c r="A1" s="59" t="inlineStr">
         <is>
           <t>MEMORIA DE CALCULO - COLUMNAS</t>
         </is>
       </c>
-      <c r="B1" s="62" t="inlineStr"/>
+      <c r="B1" s="60" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="62" t="inlineStr"/>
-      <c r="B2" s="63" t="inlineStr"/>
+      <c r="A2" s="60" t="inlineStr"/>
+      <c r="B2" s="61" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="62" t="inlineStr">
+      <c r="A3" s="60" t="inlineStr">
         <is>
           <t>MATERIALES</t>
         </is>
       </c>
-      <c r="B3" s="62" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t>H-21 (f'c 210 kg/cm2). Acero 42/50 (fy 4200). phi compresion 0,65.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="62" t="inlineStr"/>
-      <c r="B4" s="63" t="inlineStr"/>
+      <c r="A4" s="60" t="inlineStr"/>
+      <c r="B4" s="61" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="62" t="inlineStr">
+      <c r="A5" s="60" t="inlineStr">
         <is>
           <t>1. RELEVAMIENTO</t>
         </is>
       </c>
-      <c r="B5" s="62" t="inlineStr">
+      <c r="B5" s="60" t="inlineStr">
         <is>
           <t>Las columnas se identificaron en el plano cruzando el rotulo COL con un rectangulo</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="62" t="inlineStr"/>
-      <c r="B6" s="63" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr"/>
+      <c r="B6" s="61" t="inlineStr">
         <is>
           <t>de la misma seccion a menos de 26 pt. Resultaron 9 en PB y 4 en PA.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="62" t="inlineStr"/>
-      <c r="B7" s="63" t="inlineStr">
+      <c r="A7" s="60" t="inlineStr"/>
+      <c r="B7" s="61" t="inlineStr">
         <is>
           <t>Las 4 de PA caen exactamente sobre C6, C7, C8 y C9 de PB, y ademas tienen la misma</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="62" t="inlineStr"/>
-      <c r="B8" s="63" t="inlineStr">
+      <c r="A8" s="60" t="inlineStr"/>
+      <c r="B8" s="61" t="inlineStr">
         <is>
           <t>seccion, lo que confirma que la correspondencia entre plantas es correcta.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="62" t="inlineStr"/>
-      <c r="B9" s="63" t="inlineStr">
+      <c r="A9" s="60" t="inlineStr"/>
+      <c r="B9" s="61" t="inlineStr">
         <is>
           <t>La C01 de 10x10 esta confirmada por el proyectista aunque el computo metrico no</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="62" t="inlineStr"/>
-      <c r="B10" s="63" t="inlineStr">
+      <c r="A10" s="60" t="inlineStr"/>
+      <c r="B10" s="61" t="inlineStr">
         <is>
           <t>la incluya en su item 4.1.3: ese computo esta incompleto en ese punto.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="62" t="inlineStr"/>
-      <c r="B11" s="63" t="inlineStr"/>
+      <c r="A11" s="60" t="inlineStr"/>
+      <c r="B11" s="61" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="62" t="inlineStr">
+      <c r="A12" s="60" t="inlineStr">
         <is>
           <t>2. ALTURAS</t>
         </is>
       </c>
-      <c r="B12" s="62" t="inlineStr">
+      <c r="B12" s="60" t="inlineStr">
         <is>
           <t>PB 3,15 m y PA 3,22 m, los mismos valores de la planilla de la catedra, coherentes</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="62" t="inlineStr"/>
-      <c r="B13" s="63" t="inlineStr">
+      <c r="A13" s="60" t="inlineStr"/>
+      <c r="B13" s="61" t="inlineStr">
         <is>
           <t>con los niveles del plano (N.F.L +3,50 del entrepiso y +6,80 del techo).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="62" t="inlineStr"/>
-      <c r="B14" s="63" t="inlineStr"/>
+      <c r="A14" s="60" t="inlineStr"/>
+      <c r="B14" s="61" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="62" t="inlineStr">
+      <c r="A15" s="60" t="inlineStr">
         <is>
           <t>3. ARMADURA</t>
         </is>
       </c>
-      <c r="B15" s="62" t="inlineStr">
+      <c r="B15" s="60" t="inlineStr">
         <is>
           <t>As = 0,008 x area (cuantia minima, el mismo criterio de la planilla modelo).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="62" t="inlineStr"/>
-      <c r="B16" s="63" t="inlineStr">
+      <c r="A16" s="60" t="inlineStr"/>
+      <c r="B16" s="61" t="inlineStr">
         <is>
           <t>Se adoptan 4 barras del 12 en todas: 4,52 cm2, que cubre la minima en toda seccion.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="62" t="inlineStr"/>
-      <c r="B17" s="63" t="inlineStr">
+      <c r="A17" s="60" t="inlineStr"/>
+      <c r="B17" s="61" t="inlineStr">
         <is>
           <t>Separacion de estribos = min(12 x diam. long. ; 48 x diam. estribo ; lado menor),</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="62" t="inlineStr"/>
-      <c r="B18" s="63" t="inlineStr">
+      <c r="A18" s="60" t="inlineStr"/>
+      <c r="B18" s="61" t="inlineStr">
         <is>
           <t>redondeada hacia abajo a multiplo de 5. Para 4d12 con estribo d6 da 10 cm.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="62" t="inlineStr"/>
-      <c r="B19" s="63" t="inlineStr">
+      <c r="A19" s="60" t="inlineStr"/>
+      <c r="B19" s="61" t="inlineStr">
         <is>
           <t>La planilla de la catedra adopta 20 cm: ese valor supera el limite reglamentario.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="62" t="inlineStr"/>
-      <c r="B20" s="63" t="inlineStr"/>
+      <c r="A20" s="60" t="inlineStr"/>
+      <c r="B20" s="61" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="62" t="inlineStr">
+      <c r="A21" s="60" t="inlineStr">
         <is>
           <t>4. CAPACIDAD</t>
         </is>
       </c>
-      <c r="B21" s="62" t="inlineStr">
+      <c r="B21" s="60" t="inlineStr">
         <is>
           <t>phi Pn = 0,65 x 0,80 x [0,85 f'c (Ag - As) + fy As]     (columna zunchada con estribos)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="62" t="inlineStr"/>
-      <c r="B22" s="63" t="inlineStr">
+      <c r="A22" s="60" t="inlineStr"/>
+      <c r="B22" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  15x30 con 4d12 -&gt; 51,2 t        20x20 con 4d12 -&gt; 46,6 t</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="62" t="inlineStr"/>
-      <c r="B23" s="63" t="inlineStr"/>
+      <c r="A23" s="60" t="inlineStr"/>
+      <c r="B23" s="61" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="62" t="inlineStr">
+      <c r="A24" s="60" t="inlineStr">
         <is>
           <t>5. CARGAS</t>
         </is>
       </c>
-      <c r="B24" s="62" t="inlineStr">
+      <c r="B24" s="60" t="inlineStr">
         <is>
           <t>La columna CARGA (t) viene cargada con una bajada automatica: suma de las</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="62" t="inlineStr"/>
-      <c r="B25" s="63" t="inlineStr">
+      <c r="A25" s="60" t="inlineStr"/>
+      <c r="B25" s="61" t="inlineStr">
         <is>
           <t>reacciones de las vigas que apoyan en cada columna (tomadas de la planilla de</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="62" t="inlineStr"/>
-      <c r="B26" s="63" t="inlineStr">
+      <c r="A26" s="60" t="inlineStr"/>
+      <c r="B26" s="61" t="inlineStr">
         <is>
           <t>vigas), mas el peso propio, mas lo que baja de la columna del nivel superior.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="62" t="inlineStr"/>
-      <c r="B27" s="63" t="inlineStr">
+      <c r="A27" s="60" t="inlineStr"/>
+      <c r="B27" s="61" t="inlineStr">
         <is>
           <t>ES UNA CARGA PROVISORIA Y ES UN PISO, NO EL VALOR REAL: 20 de los 60 extremos</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="62" t="inlineStr"/>
-      <c r="B28" s="63" t="inlineStr">
+      <c r="A28" s="60" t="inlineStr"/>
+      <c r="B28" s="61" t="inlineStr">
         <is>
           <t>de viga no pudieron asignarse a ninguna columna porque apoyan en otra viga, en</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="62" t="inlineStr"/>
-      <c r="B29" s="63" t="inlineStr">
+      <c r="A29" s="60" t="inlineStr"/>
+      <c r="B29" s="61" t="inlineStr">
         <is>
           <t>un tabique o en la medianera, y esas reacciones no estan sumadas.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="62" t="inlineStr"/>
-      <c r="B30" s="63" t="inlineStr">
+      <c r="A30" s="60" t="inlineStr"/>
+      <c r="B30" s="61" t="inlineStr">
         <is>
           <t>Para cerrarla hay que indicar, para cada uno de esos 20 extremos, en que apoya.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="62" t="inlineStr"/>
-      <c r="B31" s="63" t="inlineStr">
+      <c r="A31" s="60" t="inlineStr"/>
+      <c r="B31" s="61" t="inlineStr">
         <is>
           <t>Mientras tanto la columna es editable: al corregir un valor todo recalcula.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="62" t="inlineStr"/>
-      <c r="B32" s="63" t="inlineStr">
+      <c r="A32" s="60" t="inlineStr"/>
+      <c r="B32" s="61" t="inlineStr">
         <is>
           <t>Ademas son cargas MAYORADAS, coherentes con la planilla de vigas. Si la catedra</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="62" t="inlineStr"/>
-      <c r="B33" s="63" t="inlineStr">
+      <c r="A33" s="60" t="inlineStr"/>
+      <c r="B33" s="61" t="inlineStr">
         <is>
           <t>pide cargas de servicio, dividir por el coeficiente que corresponda.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="62" t="inlineStr"/>
-      <c r="B34" s="63" t="inlineStr"/>
+      <c r="A34" s="60" t="inlineStr"/>
+      <c r="B34" s="61" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="62" t="inlineStr">
+      <c r="A35" s="60" t="inlineStr">
         <is>
           <t>6. ESBELTEZ</t>
         </is>
       </c>
-      <c r="B35" s="62" t="inlineStr">
+      <c r="B35" s="60" t="inlineStr">
         <is>
           <t>Todas las columnas son esbeltas: con lado menor de 15 cm y 3,15 m de altura,</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="62" t="inlineStr"/>
-      <c r="B36" s="63" t="inlineStr">
+      <c r="A36" s="60" t="inlineStr"/>
+      <c r="B36" s="61" t="inlineStr">
         <is>
           <t>k lu / r = 70, muy por encima del limite de 34 por debajo del cual se puede</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="62" t="inlineStr"/>
-      <c r="B37" s="63" t="inlineStr">
+      <c r="A37" s="60" t="inlineStr"/>
+      <c r="B37" s="61" t="inlineStr">
         <is>
           <t>despreciar el pandeo. En la practica el llenado de mamposteria las arriostra, pero</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="62" t="inlineStr"/>
-      <c r="B38" s="63" t="inlineStr">
+      <c r="A38" s="60" t="inlineStr"/>
+      <c r="B38" s="61" t="inlineStr">
         <is>
           <t>si la catedra lo pide hay que verificar segundo orden. La planilla lo marca.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="62" t="inlineStr"/>
-      <c r="B39" s="63" t="inlineStr"/>
+      <c r="A39" s="60" t="inlineStr"/>
+      <c r="B39" s="61" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="62" t="inlineStr">
+      <c r="A40" s="60" t="inlineStr">
         <is>
           <t>7. LA DE 10x10</t>
         </is>
       </c>
-      <c r="B40" s="62" t="inlineStr">
+      <c r="B40" s="60" t="inlineStr">
         <is>
           <t>Existe, confirmada por el proyectista, y el computo metrico la omite. Con 10 cm</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="62" t="inlineStr"/>
-      <c r="B41" s="63" t="inlineStr">
+      <c r="A41" s="60" t="inlineStr"/>
+      <c r="B41" s="61" t="inlineStr">
         <is>
           <t>de lado y 3,15 m de altura su esbeltez es k lu / r = 105, tres veces el limite</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="62" t="inlineStr"/>
-      <c r="B42" s="63" t="inlineStr">
+      <c r="A42" s="60" t="inlineStr"/>
+      <c r="B42" s="61" t="inlineStr">
         <is>
           <t>por debajo del cual se puede despreciar el pandeo, y su capacidad es de 18,7 t</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="62" t="inlineStr"/>
-      <c r="B43" s="63" t="inlineStr">
+      <c r="A43" s="60" t="inlineStr"/>
+      <c r="B43" s="61" t="inlineStr">
         <is>
           <t>contra los 51 de una 15x30. Es el punto mas delicado del conjunto: conviene</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="62" t="inlineStr"/>
-      <c r="B44" s="63" t="inlineStr">
+      <c r="A44" s="60" t="inlineStr"/>
+      <c r="B44" s="61" t="inlineStr">
         <is>
           <t>verificarla a segundo orden en serio, no con la formula de compresion simple.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="62" t="inlineStr"/>
-      <c r="B45" s="63" t="inlineStr"/>
+      <c r="A45" s="60" t="inlineStr"/>
+      <c r="B45" s="61" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="62" t="inlineStr">
+      <c r="A46" s="60" t="inlineStr">
         <is>
           <t>LIMITACIONES</t>
         </is>
       </c>
-      <c r="B46" s="62" t="inlineStr">
+      <c r="B46" s="60" t="inlineStr">
         <is>
           <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="62" t="inlineStr"/>
-      <c r="B47" s="63" t="inlineStr">
+      <c r="A47" s="60" t="inlineStr"/>
+      <c r="B47" s="61" t="inlineStr">
         <is>
           <t>No se verifica flexion compuesta: las columnas de borde reciben momento de las</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="62" t="inlineStr"/>
-      <c r="B48" s="63" t="inlineStr">
+      <c r="A48" s="60" t="inlineStr"/>
+      <c r="B48" s="61" t="inlineStr">
         <is>
           <t>vigas invertidas y trabajan a flexo-compresion, no a compresion simple.</t>
         </is>
@@ -5781,7 +5775,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="64" t="inlineStr">
+      <c r="A1" s="62" t="inlineStr">
         <is>
           <t>VIGAS DE FUNDACION - inventario. Calculo pendiente: va despues de columnas.</t>
         </is>
@@ -5923,7 +5917,7 @@
       <c r="D9" s="11" t="n">
         <v>533</v>
       </c>
-      <c r="E9" s="65" t="inlineStr">
+      <c r="E9" s="63" t="inlineStr">
         <is>
           <t>Ancho cortado en el PDF: confirmar 20 o 22 cm</t>
         </is>
@@ -5989,7 +5983,7 @@
       <c r="B13" s="11" t="n"/>
       <c r="C13" s="11" t="n"/>
       <c r="D13" s="11" t="n"/>
-      <c r="E13" s="65" t="inlineStr">
+      <c r="E13" s="63" t="inlineStr">
         <is>
           <t>Cota no legible: completar</t>
         </is>
@@ -6004,7 +5998,7 @@
       <c r="B14" s="11" t="n"/>
       <c r="C14" s="11" t="n"/>
       <c r="D14" s="11" t="n"/>
-      <c r="E14" s="65" t="inlineStr">
+      <c r="E14" s="63" t="inlineStr">
         <is>
           <t>Cota no legible: completar</t>
         </is>
@@ -6206,7 +6200,7 @@
       <c r="B26" s="11" t="n"/>
       <c r="C26" s="11" t="n"/>
       <c r="D26" s="11" t="n"/>
-      <c r="E26" s="65" t="inlineStr">
+      <c r="E26" s="63" t="inlineStr">
         <is>
           <t>Cota no legible: completar</t>
         </is>
@@ -17055,7 +17049,9 @@
           <t>T9</t>
         </is>
       </c>
-      <c r="C12" s="42" t="n"/>
+      <c r="C12" s="8" t="n">
+        <v>6.96</v>
+      </c>
       <c r="D12" s="8" t="n">
         <v>3.2</v>
       </c>
@@ -17103,7 +17099,7 @@
       </c>
       <c r="Q12" s="13" t="inlineStr">
         <is>
-          <t>Falta la carga: no figura en la planilla de la catedra.</t>
+          <t>Recibe el extremo de VI 14. Carga mayorada.</t>
         </is>
       </c>
     </row>
@@ -17114,7 +17110,9 @@
           <t>T10</t>
         </is>
       </c>
-      <c r="C13" s="42" t="n"/>
+      <c r="C13" s="8" t="n">
+        <v>13.38</v>
+      </c>
       <c r="D13" s="8" t="n">
         <v>2.6</v>
       </c>
@@ -17162,7 +17160,7 @@
       </c>
       <c r="Q13" s="13" t="inlineStr">
         <is>
-          <t>Falta la carga: no figura en la planilla de la catedra.</t>
+          <t>Recibe el extremo de VI 12. Carga mayorada.</t>
         </is>
       </c>
     </row>
@@ -17173,7 +17171,9 @@
           <t>T11</t>
         </is>
       </c>
-      <c r="C14" s="42" t="n"/>
+      <c r="C14" s="8" t="n">
+        <v>5.07</v>
+      </c>
       <c r="D14" s="8" t="n">
         <v>2.6</v>
       </c>
@@ -17221,7 +17221,7 @@
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
-          <t>Longitud muy corta: verificar si es tabique o el machon de una abertura. Falta la carga: no figura en la planilla de la catedra.</t>
+          <t>Recibe el extremo de VI 13b sobre solo 28 cm de largo: es el tabique con mayor tension del conjunto.</t>
         </is>
       </c>
     </row>
@@ -17232,7 +17232,9 @@
           <t>T12</t>
         </is>
       </c>
-      <c r="C15" s="42" t="n"/>
+      <c r="C15" s="8" t="n">
+        <v>6.93</v>
+      </c>
       <c r="D15" s="8" t="n">
         <v>2.6</v>
       </c>
@@ -17280,7 +17282,7 @@
       </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
-          <t>Longitud muy corta: verificar si es tabique o el machon de una abertura. Falta la carga: no figura en la planilla de la catedra.</t>
+          <t>Recibe los extremos de VI 17 (1,31 t) y VI 15b (5,62 t) sobre 32 cm de largo.</t>
         </is>
       </c>
     </row>
@@ -17291,7 +17293,9 @@
           <t>T13</t>
         </is>
       </c>
-      <c r="C16" s="43" t="n"/>
+      <c r="C16" s="15" t="n">
+        <v>1.22</v>
+      </c>
       <c r="D16" s="15" t="n">
         <v>3.2</v>
       </c>
@@ -17339,7 +17343,7 @@
       </c>
       <c r="Q16" s="20" t="inlineStr">
         <is>
-          <t>Falta la carga: no figura en la planilla de la catedra.</t>
+          <t>No recibe vigas: es la continuidad del tabique T06c de planta baja. La carga indicada es solo su peso propio; lo que baje de arriba se suma a T06c.</t>
         </is>
       </c>
     </row>
@@ -17363,7 +17367,7 @@
       <c r="Q17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="44" t="inlineStr">
+      <c r="A18" s="42" t="inlineStr">
         <is>
           <t>T1 a T6: cargas y dimensiones tomadas de la planilla de la catedra. Probablemente sean cargas de servicio; compararlas contra fi Pn, que es resistencia ultima, queda del lado inseguro en torno a un 40 por ciento. Con utilizaciones del 10 al 20 por ciento no cambia ningun veredicto, pero conviene saberlo.</t>
         </is>
@@ -17386,7 +17390,7 @@
       <c r="Q18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="44" t="inlineStr">
+      <c r="A19" s="42" t="inlineStr">
         <is>
           <t>T7 y T8: carga tomada de la reaccion de VI 02 y VI 11a en la planilla de vigas, que son MAYORADAS. El criterio no es el mismo que en T1 a T6.</t>
         </is>
@@ -17409,9 +17413,9 @@
       <c r="Q19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="44" t="inlineStr">
-        <is>
-          <t>T9 a T13: dimensiones del computo metrico; la carga todavia no esta definida.</t>
+      <c r="A20" s="42" t="inlineStr">
+        <is>
+          <t>T9 a T13: dimensiones del computo metrico. Las cargas son las reacciones de las vigas de techo que apoyan en cada uno, aportadas por el proyectista: T9 recibe VI 14, T10 recibe VI 12, T11 recibe VI 13b y T12 recibe VI 17 mas VI 15b. T13 no recibe vigas: continua el tabique T06c de planta baja.</t>
         </is>
       </c>
       <c r="B20" s="2" t="n"/>
@@ -17432,7 +17436,7 @@
       <c r="Q20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="44" t="inlineStr">
+      <c r="A21" s="42" t="inlineStr">
         <is>
           <t>Area: si B es menor o igual al espesor el tabique es recto y el area es A x B; si no, es un tabique en L y el area es (A + B - espesor) x espesor.</t>
         </is>
@@ -17455,7 +17459,7 @@
       <c r="Q21" s="2" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="44" t="inlineStr">
+      <c r="A22" s="42" t="inlineStr">
         <is>
           <t>fi Pn = 0,55 x 0,65 x f'c x area x [1 - (altura / 32 espesor)^2]   muro portante de hormigon armado con reduccion por esbeltez.</t>
         </is>
@@ -17478,7 +17482,7 @@
       <c r="Q22" s="2" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="44" t="inlineStr">
+      <c r="A23" s="42" t="inlineStr">
         <is>
           <t>Armadura vertical en doble malla y horizontal en malla simple, ambas o8 c/20, iguales a las de la planilla de la catedra.</t>
         </is>
@@ -17549,7 +17553,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="45" t="inlineStr">
+      <c r="A1" s="43" t="inlineStr">
         <is>
           <t>DATOS DE PARTIDA - HIPOTESIS DE CALCULO</t>
         </is>
@@ -17561,7 +17565,7 @@
       <c r="F1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="44" t="inlineStr">
+      <c r="A2" s="42" t="inlineStr">
         <is>
           <t>Celdas verdes: editables. La planilla recalcula sola.</t>
         </is>
@@ -17581,17 +17585,17 @@
       <c r="F3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="46" t="inlineStr">
+      <c r="A4" s="44" t="inlineStr">
         <is>
           <t>MATERIALES</t>
         </is>
       </c>
-      <c r="B4" s="47" t="inlineStr">
+      <c r="B4" s="45" t="inlineStr">
         <is>
           <t>valor</t>
         </is>
       </c>
-      <c r="C4" s="47" t="inlineStr">
+      <c r="C4" s="45" t="inlineStr">
         <is>
           <t>unidad</t>
         </is>
@@ -17601,12 +17605,12 @@
       <c r="F4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="48" t="inlineStr">
+      <c r="A5" s="46" t="inlineStr">
         <is>
           <t>Hormigon H-21   f'c</t>
         </is>
       </c>
-      <c r="B5" s="49" t="n">
+      <c r="B5" s="47" t="n">
         <v>210</v>
       </c>
       <c r="C5" s="11" t="inlineStr">
@@ -17619,12 +17623,12 @@
       <c r="F5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="48" t="inlineStr">
+      <c r="A6" s="46" t="inlineStr">
         <is>
           <t>Acero 42/50   fy</t>
         </is>
       </c>
-      <c r="B6" s="49" t="n">
+      <c r="B6" s="47" t="n">
         <v>4200</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
@@ -17637,12 +17641,12 @@
       <c r="F6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="48" t="inlineStr">
+      <c r="A7" s="46" t="inlineStr">
         <is>
           <t>Peso especifico H.A.</t>
         </is>
       </c>
-      <c r="B7" s="49" t="n">
+      <c r="B7" s="47" t="n">
         <v>2400</v>
       </c>
       <c r="C7" s="11" t="inlineStr">
@@ -17655,12 +17659,12 @@
       <c r="F7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="48" t="inlineStr">
+      <c r="A8" s="46" t="inlineStr">
         <is>
           <t>phi flexion</t>
         </is>
       </c>
-      <c r="B8" s="49" t="n">
+      <c r="B8" s="47" t="n">
         <v>0.9</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
@@ -17673,12 +17677,12 @@
       <c r="F8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="48" t="inlineStr">
+      <c r="A9" s="46" t="inlineStr">
         <is>
           <t>phi corte</t>
         </is>
       </c>
-      <c r="B9" s="49" t="n">
+      <c r="B9" s="47" t="n">
         <v>0.75</v>
       </c>
       <c r="C9" s="11" t="inlineStr">
@@ -17691,12 +17695,12 @@
       <c r="F9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="48" t="inlineStr">
+      <c r="A10" s="46" t="inlineStr">
         <is>
           <t>Coef. mayoracion permanente</t>
         </is>
       </c>
-      <c r="B10" s="49" t="n">
+      <c r="B10" s="47" t="n">
         <v>1.2</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
@@ -17709,12 +17713,12 @@
       <c r="F10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="48" t="inlineStr">
+      <c r="A11" s="46" t="inlineStr">
         <is>
           <t>Coef. mayoracion sobrecarga</t>
         </is>
       </c>
-      <c r="B11" s="49" t="n">
+      <c r="B11" s="47" t="n">
         <v>1.6</v>
       </c>
       <c r="C11" s="11" t="inlineStr">
@@ -17735,7 +17739,7 @@
       <c r="F12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="46" t="inlineStr">
+      <c r="A13" s="44" t="inlineStr">
         <is>
           <t>PAQUETES DE CARGA</t>
         </is>
@@ -17767,21 +17771,21 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="50" t="inlineStr">
+      <c r="A14" s="48" t="inlineStr">
         <is>
           <t>PA</t>
         </is>
       </c>
-      <c r="B14" s="51" t="n">
+      <c r="B14" s="49" t="n">
         <v>550</v>
       </c>
-      <c r="C14" s="51" t="n">
+      <c r="C14" s="49" t="n">
         <v>200</v>
       </c>
-      <c r="D14" s="52" t="n">
+      <c r="D14" s="50" t="n">
         <v>2.6</v>
       </c>
-      <c r="E14" s="52" t="n">
+      <c r="E14" s="50" t="n">
         <v>2</v>
       </c>
       <c r="F14" s="32" t="inlineStr">
@@ -17791,21 +17795,21 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="50" t="inlineStr">
+      <c r="A15" s="48" t="inlineStr">
         <is>
           <t>TECHO</t>
         </is>
       </c>
-      <c r="B15" s="51" t="n">
+      <c r="B15" s="49" t="n">
         <v>560</v>
       </c>
-      <c r="C15" s="51" t="n">
+      <c r="C15" s="49" t="n">
         <v>100</v>
       </c>
-      <c r="D15" s="52" t="n">
+      <c r="D15" s="50" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="52" t="n">
+      <c r="E15" s="50" t="n">
         <v>2</v>
       </c>
       <c r="F15" s="32" t="inlineStr">
@@ -17815,12 +17819,12 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="48" t="inlineStr">
+      <c r="A16" s="46" t="inlineStr">
         <is>
           <t>Mamposteria sobre viga</t>
         </is>
       </c>
-      <c r="B16" s="49" t="n">
+      <c r="B16" s="47" t="n">
         <v>250</v>
       </c>
       <c r="C16" s="11" t="inlineStr">
@@ -17830,7 +17834,7 @@
       </c>
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
-      <c r="F16" s="53" t="inlineStr">
+      <c r="F16" s="51" t="inlineStr">
         <is>
           <t>Ladrillo hueco 18 cm + revoque en ambas caras</t>
         </is>
@@ -17845,7 +17849,7 @@
       <c r="F17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="46" t="inlineStr">
+      <c r="A18" s="44" t="inlineStr">
         <is>
           <t>COEFICIENTES SEGUN ESQUEMA</t>
         </is>
@@ -17873,101 +17877,101 @@
       <c r="F18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="48" t="inlineStr">
+      <c r="A19" s="46" t="inlineStr">
         <is>
           <t>Simplemente apoyada</t>
         </is>
       </c>
-      <c r="B19" s="54" t="n">
+      <c r="B19" s="52" t="n">
         <v>0.125</v>
       </c>
-      <c r="C19" s="54" t="n">
+      <c r="C19" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="D19" s="54" t="n">
+      <c r="D19" s="52" t="n">
         <v>0.5</v>
       </c>
-      <c r="E19" s="55" t="n">
+      <c r="E19" s="53" t="n">
         <v>16</v>
       </c>
       <c r="F19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="48" t="inlineStr">
+      <c r="A20" s="46" t="inlineStr">
         <is>
           <t>Continua</t>
         </is>
       </c>
-      <c r="B20" s="54" t="n">
+      <c r="B20" s="52" t="n">
         <v>0.07142999999999999</v>
       </c>
-      <c r="C20" s="54" t="n">
+      <c r="C20" s="52" t="n">
         <v>0.1</v>
       </c>
-      <c r="D20" s="54" t="n">
+      <c r="D20" s="52" t="n">
         <v>0.575</v>
       </c>
-      <c r="E20" s="55" t="n">
+      <c r="E20" s="53" t="n">
         <v>21</v>
       </c>
       <c r="F20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="48" t="inlineStr">
+      <c r="A21" s="46" t="inlineStr">
         <is>
           <t>Empotrada-apoyada</t>
         </is>
       </c>
-      <c r="B21" s="54" t="n">
+      <c r="B21" s="52" t="n">
         <v>0.07031</v>
       </c>
-      <c r="C21" s="54" t="n">
+      <c r="C21" s="52" t="n">
         <v>0.125</v>
       </c>
-      <c r="D21" s="54" t="n">
+      <c r="D21" s="52" t="n">
         <v>0.625</v>
       </c>
-      <c r="E21" s="55" t="n">
+      <c r="E21" s="53" t="n">
         <v>18.5</v>
       </c>
       <c r="F21" s="2" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="48" t="inlineStr">
+      <c r="A22" s="46" t="inlineStr">
         <is>
           <t>Biempotrada</t>
         </is>
       </c>
-      <c r="B22" s="54" t="n">
+      <c r="B22" s="52" t="n">
         <v>0.04167</v>
       </c>
-      <c r="C22" s="54" t="n">
+      <c r="C22" s="52" t="n">
         <v>0.08333</v>
       </c>
-      <c r="D22" s="54" t="n">
+      <c r="D22" s="52" t="n">
         <v>0.5</v>
       </c>
-      <c r="E22" s="55" t="n">
+      <c r="E22" s="53" t="n">
         <v>21</v>
       </c>
       <c r="F22" s="2" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="48" t="inlineStr">
+      <c r="A23" s="46" t="inlineStr">
         <is>
           <t>Voladizo</t>
         </is>
       </c>
-      <c r="B23" s="54" t="n">
+      <c r="B23" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="C23" s="54" t="n">
+      <c r="C23" s="52" t="n">
         <v>0.5</v>
       </c>
-      <c r="D23" s="54" t="n">
+      <c r="D23" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="E23" s="55" t="n">
+      <c r="E23" s="53" t="n">
         <v>8</v>
       </c>
       <c r="F23" s="2" t="n"/>
@@ -18015,7 +18019,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="45" t="inlineStr">
+      <c r="A1" s="43" t="inlineStr">
         <is>
           <t>DATOS DE PARTIDA - LOSAS</t>
         </is>
@@ -18025,7 +18029,7 @@
       <c r="D1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="44" t="inlineStr">
+      <c r="A2" s="42" t="inlineStr">
         <is>
           <t>Celdas verdes: editables. La planilla recalcula sola.</t>
         </is>
@@ -18041,17 +18045,17 @@
       <c r="D3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="46" t="inlineStr">
+      <c r="A4" s="44" t="inlineStr">
         <is>
           <t>MATERIALES Y METODO</t>
         </is>
       </c>
-      <c r="B4" s="47" t="inlineStr">
+      <c r="B4" s="45" t="inlineStr">
         <is>
           <t>valor</t>
         </is>
       </c>
-      <c r="C4" s="47" t="inlineStr">
+      <c r="C4" s="45" t="inlineStr">
         <is>
           <t>unidad</t>
         </is>
@@ -18059,12 +18063,12 @@
       <c r="D4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="48" t="inlineStr">
+      <c r="A5" s="46" t="inlineStr">
         <is>
           <t>Hormigon H-21   f'c</t>
         </is>
       </c>
-      <c r="B5" s="49" t="n">
+      <c r="B5" s="47" t="n">
         <v>210</v>
       </c>
       <c r="C5" s="11" t="inlineStr">
@@ -18075,12 +18079,12 @@
       <c r="D5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="48" t="inlineStr">
+      <c r="A6" s="46" t="inlineStr">
         <is>
           <t>Acero 42/50   fy</t>
         </is>
       </c>
-      <c r="B6" s="49" t="n">
+      <c r="B6" s="47" t="n">
         <v>4200</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
@@ -18091,12 +18095,12 @@
       <c r="D6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="48" t="inlineStr">
+      <c r="A7" s="46" t="inlineStr">
         <is>
           <t>Tension admisible del acero</t>
         </is>
       </c>
-      <c r="B7" s="49" t="n">
+      <c r="B7" s="47" t="n">
         <v>2400</v>
       </c>
       <c r="C7" s="11" t="inlineStr">
@@ -18107,12 +18111,12 @@
       <c r="D7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="48" t="inlineStr">
+      <c r="A8" s="46" t="inlineStr">
         <is>
           <t>Brazo elastico  z / h</t>
         </is>
       </c>
-      <c r="B8" s="49" t="n">
+      <c r="B8" s="47" t="n">
         <v>0.9</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
@@ -18123,12 +18127,12 @@
       <c r="D8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="48" t="inlineStr">
+      <c r="A9" s="46" t="inlineStr">
         <is>
           <t>Peso especifico H.A.</t>
         </is>
       </c>
-      <c r="B9" s="49" t="n">
+      <c r="B9" s="47" t="n">
         <v>2400</v>
       </c>
       <c r="C9" s="11" t="inlineStr">
@@ -18139,12 +18143,12 @@
       <c r="D9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="48" t="inlineStr">
+      <c r="A10" s="46" t="inlineStr">
         <is>
           <t>Recubrimiento</t>
         </is>
       </c>
-      <c r="B10" s="49" t="n">
+      <c r="B10" s="47" t="n">
         <v>1.5</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
@@ -18155,12 +18159,12 @@
       <c r="D10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="48" t="inlineStr">
+      <c r="A11" s="46" t="inlineStr">
         <is>
           <t>Separacion maxima</t>
         </is>
       </c>
-      <c r="B11" s="49" t="n">
+      <c r="B11" s="47" t="n">
         <v>20</v>
       </c>
       <c r="C11" s="11" t="inlineStr">
@@ -18171,12 +18175,12 @@
       <c r="D11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="48" t="inlineStr">
+      <c r="A12" s="46" t="inlineStr">
         <is>
           <t>Armadura de reparticion</t>
         </is>
       </c>
-      <c r="B12" s="49" t="n">
+      <c r="B12" s="47" t="n">
         <v>0.2</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
@@ -18187,12 +18191,12 @@
       <c r="D12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="48" t="inlineStr">
+      <c r="A13" s="46" t="inlineStr">
         <is>
           <t>Reparticion minima</t>
         </is>
       </c>
-      <c r="B13" s="49" t="n">
+      <c r="B13" s="47" t="n">
         <v>0.3</v>
       </c>
       <c r="C13" s="11" t="inlineStr">
@@ -18209,7 +18213,7 @@
       <c r="D14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="46" t="inlineStr">
+      <c r="A15" s="44" t="inlineStr">
         <is>
           <t>CARGAS POR NIVEL</t>
         </is>
@@ -18231,15 +18235,15 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="50" t="inlineStr">
+      <c r="A16" s="48" t="inlineStr">
         <is>
           <t>S/PB</t>
         </is>
       </c>
-      <c r="B16" s="49" t="n">
+      <c r="B16" s="47" t="n">
         <v>242</v>
       </c>
-      <c r="C16" s="49" t="n">
+      <c r="C16" s="47" t="n">
         <v>200</v>
       </c>
       <c r="D16" s="32" t="inlineStr">
@@ -18249,15 +18253,15 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="50" t="inlineStr">
+      <c r="A17" s="48" t="inlineStr">
         <is>
           <t>S/PA</t>
         </is>
       </c>
-      <c r="B17" s="49" t="n">
+      <c r="B17" s="47" t="n">
         <v>252</v>
       </c>
-      <c r="C17" s="49" t="n">
+      <c r="C17" s="47" t="n">
         <v>100</v>
       </c>
       <c r="D17" s="32" t="inlineStr">
@@ -18283,7 +18287,7 @@
       <c r="D19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="46" t="inlineStr">
+      <c r="A20" s="44" t="inlineStr">
         <is>
           <t>GRADO DE EMPOTRAMIENTO</t>
         </is>
@@ -18305,90 +18309,90 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="56" t="inlineStr">
+      <c r="A21" s="54" t="inlineStr">
         <is>
           <t>1/8</t>
         </is>
       </c>
-      <c r="B21" s="54" t="n">
+      <c r="B21" s="52" t="n">
         <v>0.125</v>
       </c>
-      <c r="C21" s="57" t="n">
+      <c r="C21" s="55" t="n">
         <v>0.5</v>
       </c>
-      <c r="D21" s="58" t="inlineStr">
+      <c r="D21" s="56" t="inlineStr">
         <is>
           <t>Simplemente apoyada</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="56" t="inlineStr">
+      <c r="A22" s="54" t="inlineStr">
         <is>
           <t>1/10</t>
         </is>
       </c>
-      <c r="B22" s="54" t="n">
+      <c r="B22" s="52" t="n">
         <v>0.1</v>
       </c>
-      <c r="C22" s="57" t="n">
+      <c r="C22" s="55" t="n">
         <v>0.55</v>
       </c>
-      <c r="D22" s="58" t="inlineStr">
+      <c r="D22" s="56" t="inlineStr">
         <is>
           <t>Continua</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="56" t="inlineStr">
+      <c r="A23" s="54" t="inlineStr">
         <is>
           <t>1/12</t>
         </is>
       </c>
-      <c r="B23" s="54" t="n">
+      <c r="B23" s="52" t="n">
         <v>0.0833</v>
       </c>
-      <c r="C23" s="57" t="n">
+      <c r="C23" s="55" t="n">
         <v>0.5</v>
       </c>
-      <c r="D23" s="58" t="inlineStr">
+      <c r="D23" s="56" t="inlineStr">
         <is>
           <t>Biempotrada</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="56" t="inlineStr">
+      <c r="A24" s="54" t="inlineStr">
         <is>
           <t>1/14</t>
         </is>
       </c>
-      <c r="B24" s="54" t="n">
+      <c r="B24" s="52" t="n">
         <v>0.07140000000000001</v>
       </c>
-      <c r="C24" s="57" t="n">
+      <c r="C24" s="55" t="n">
         <v>0.575</v>
       </c>
-      <c r="D24" s="58" t="inlineStr">
+      <c r="D24" s="56" t="inlineStr">
         <is>
           <t>Continua</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="56" t="inlineStr">
+      <c r="A25" s="54" t="inlineStr">
         <is>
           <t>1/2</t>
         </is>
       </c>
-      <c r="B25" s="54" t="n">
+      <c r="B25" s="52" t="n">
         <v>0.5</v>
       </c>
-      <c r="C25" s="57" t="n">
+      <c r="C25" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="D25" s="58" t="inlineStr">
+      <c r="D25" s="56" t="inlineStr">
         <is>
           <t>Voladizo</t>
         </is>

</xml_diff>

<commit_message>
Corregir el apoyo de VI 17 y dejar T12 observado
El proyectista aclara que VI 17 descarga en el tabique T07 a la
izquierda y en una COL 02 de 15x30 a la derecha, y que T12 acompana
a la viga en toda su longitud, o sea que va encima y no debajo.
T07 pasa a 22,43 t, el tabique mas exigido, con el 78 por ciento de
su capacidad. T12 queda con 5,62 t y marcado a revisar hasta
confirmar si T9, T10, T11 y T13 estan en la misma situacion.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -16924,7 +16924,7 @@
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>21.12</v>
+        <v>22.43</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>3.15</v>
@@ -16973,7 +16973,7 @@
       </c>
       <c r="Q10" s="13" t="inlineStr">
         <is>
-          <t>Carga tomada de la reaccion de VI 02 en la planilla de vigas, MAYORADA. No es comparable sin mas con las de T1 a T6.</t>
+          <t>Recibe los extremos de VI 02 (21,12 t) y de VI 17 (1,31 t). Cargas MAYORADAS, no comparables sin mas con las de T1 a T6. Es el tabique mas exigido del conjunto.</t>
         </is>
       </c>
     </row>
@@ -17233,7 +17233,7 @@
         </is>
       </c>
       <c r="C15" s="8" t="n">
-        <v>6.93</v>
+        <v>5.62</v>
       </c>
       <c r="D15" s="8" t="n">
         <v>2.6</v>
@@ -17282,7 +17282,7 @@
       </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
-          <t>Recibe los extremos de VI 17 (1,31 t) y VI 15b (5,62 t) sobre 32 cm de largo.</t>
+          <t>A REVISAR. Se le deja solo VI 15b. El proyectista indica que VI 17 no descarga aqui sino en T07, y que T12 acompana a VI 17 en toda su longitud, o sea que va encima de la viga y no debajo. Falta definir si lo mismo vale para T9, T10, T11 y T13.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dejar asentado por que el tabique sostiene a la viga y no al reves
Como todas las vigas son invertidas, sobresalen 70 cm por encima del
fondo de losa, mientras que los tabiques de planta alta llegan desde
el piso hasta ese fondo: el tabique queda debajo y sostiene a la
viga. La carga que se habia asignado a T9 a T13 era correcta. Se
levanta la observacion de T12 y los trece tabiques quedan cerrados.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -16391,7 +16391,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:Q24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -17282,7 +17282,7 @@
       </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
-          <t>A REVISAR. Se le deja solo VI 15b. El proyectista indica que VI 17 no descarga aqui sino en T07, y que T12 acompana a VI 17 en toda su longitud, o sea que va encima de la viga y no debajo. Falta definir si lo mismo vale para T9, T10, T11 y T13.</t>
+          <t>Recibe el extremo de VI 15b. VI 17 no descarga aqui sino en T07. T12 acompana a VI 17 en toda su longitud por debajo, de modo que esa viga esta mas sostenida de lo que supone el calculo: queda del lado seguro.</t>
         </is>
       </c>
     </row>
@@ -17415,7 +17415,7 @@
     <row r="20">
       <c r="A20" s="42" t="inlineStr">
         <is>
-          <t>T9 a T13: dimensiones del computo metrico. Las cargas son las reacciones de las vigas de techo que apoyan en cada uno, aportadas por el proyectista: T9 recibe VI 14, T10 recibe VI 12, T11 recibe VI 13b y T12 recibe VI 17 mas VI 15b. T13 no recibe vigas: continua el tabique T06c de planta baja.</t>
+          <t>Direccion de la carga: como todas las vigas son invertidas, sobresalen 70 cm por encima del fondo de losa, mientras que los tabiques de planta alta llegan desde el piso hasta ese fondo. El tabique queda debajo y sostiene a la viga, no al reves.</t>
         </is>
       </c>
       <c r="B20" s="2" t="n"/>
@@ -17438,7 +17438,7 @@
     <row r="21">
       <c r="A21" s="42" t="inlineStr">
         <is>
-          <t>Area: si B es menor o igual al espesor el tabique es recto y el area es A x B; si no, es un tabique en L y el area es (A + B - espesor) x espesor.</t>
+          <t>T9 a T13: dimensiones del computo metrico. Las cargas son las reacciones de las vigas de techo que apoyan en cada uno, aportadas por el proyectista: T9 recibe VI 14, T10 recibe VI 12, T11 recibe VI 13b y T12 recibe VI 17 mas VI 15b. T13 no recibe vigas: continua el tabique T06c de planta baja.</t>
         </is>
       </c>
       <c r="B21" s="2" t="n"/>
@@ -17461,7 +17461,7 @@
     <row r="22">
       <c r="A22" s="42" t="inlineStr">
         <is>
-          <t>fi Pn = 0,55 x 0,65 x f'c x area x [1 - (altura / 32 espesor)^2]   muro portante de hormigon armado con reduccion por esbeltez.</t>
+          <t>Area: si B es menor o igual al espesor el tabique es recto y el area es A x B; si no, es un tabique en L y el area es (A + B - espesor) x espesor.</t>
         </is>
       </c>
       <c r="B22" s="2" t="n"/>
@@ -17484,7 +17484,7 @@
     <row r="23">
       <c r="A23" s="42" t="inlineStr">
         <is>
-          <t>Armadura vertical en doble malla y horizontal en malla simple, ambas o8 c/20, iguales a las de la planilla de la catedra.</t>
+          <t>fi Pn = 0,55 x 0,65 x f'c x area x [1 - (altura / 32 espesor)^2]   muro portante de hormigon armado con reduccion por esbeltez.</t>
         </is>
       </c>
       <c r="B23" s="2" t="n"/>
@@ -17503,6 +17503,29 @@
       <c r="O23" s="2" t="n"/>
       <c r="P23" s="2" t="n"/>
       <c r="Q23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="42" t="inlineStr">
+        <is>
+          <t>Armadura vertical en doble malla y horizontal en malla simple, ambas o8 c/20, iguales a las de la planilla de la catedra.</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n"/>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
+      <c r="I24" s="2" t="n"/>
+      <c r="J24" s="2" t="n"/>
+      <c r="K24" s="2" t="n"/>
+      <c r="L24" s="2" t="n"/>
+      <c r="M24" s="2" t="n"/>
+      <c r="N24" s="2" t="n"/>
+      <c r="O24" s="2" t="n"/>
+      <c r="P24" s="2" t="n"/>
+      <c r="Q24" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>

<commit_message>
Sumar a T6 las reacciones de las dos vigas chatas
No consta si los 6,00 t de la planilla de la catedra ya incluian lo
que le llega de VCH 03a y VCH 05, de modo que se suman por ser la
hipotesis conservadora: T6 pasa a 14,10 t. Con cualquiera de las dos
lecturas el tabique usa entre el 6 y el 14 por ciento de su
capacidad, asi que la duda no cambia ningun resultado.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -16949,7 +16949,7 @@
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>6</v>
+        <v>14.1</v>
       </c>
       <c r="D9" s="8" t="n">
         <v>3.15</v>
@@ -16996,7 +16996,11 @@
         <f>IF(C9="","FALTA CARGA",IF(C9&lt;=O9,"VERIFICA","NO VERIFICA"))</f>
         <v/>
       </c>
-      <c r="Q9" s="11" t="inlineStr"/>
+      <c r="Q9" s="13" t="inlineStr">
+        <is>
+          <t>6,00 t de la planilla de la catedra mas las reacciones de VCH 03a (6,4 t) y VCH 05 (1,7 t), que apoyan en el perpendicularmente. No consta si los 6,00 t ya las incluian; se suman por ser la hipotesis conservadora. Con cualquiera de las dos lecturas el tabique usa entre el 6 y el 14 por ciento de su capacidad.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="17" customHeight="1">
       <c r="A10" s="26" t="n"/>

</xml_diff>

<commit_message>
Cargar la planilla de armadura de pilotes y cerrar VI 01b y VI 07a
La planilla del Ing. Caggiano aporta la armadura (5d12 mas espiral
d6 c/15, sin bulbo) y, sobre todo, el destino de cada tipo: 5
pilotes bajo cabezales de 65 cm y 8 bajo cabezales de 70 cm. Cruzado
con el computo eso obliga a que CBZ03 lleve tres pilotes y no dos:
5x1 + 1x2 + 2x3 = 13, mas 20 bajo vigas de fundacion, total 33.
CB8 baja de 19,6 a 13,1 t por pilote.
VI 01b descarga en T02 y VI 07a en T01a, de modo que T1 pasa a
18,74 t y T2 a 8,50 t.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -3659,7 +3659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3678,6 +3678,7 @@
       <c r="C1" s="2" t="n"/>
       <c r="D1" s="2" t="n"/>
       <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n"/>
@@ -3685,6 +3686,7 @@
       <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="44" t="inlineStr">
@@ -3708,6 +3710,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="46" t="inlineStr">
@@ -3729,6 +3732,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="46" t="inlineStr">
@@ -3750,6 +3754,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="46" t="inlineStr">
@@ -3771,6 +3776,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="46" t="inlineStr">
@@ -3792,6 +3798,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="46" t="inlineStr">
@@ -3813,13 +3820,23 @@
         </is>
       </c>
       <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n"/>
+      <c r="A9" s="57" t="inlineStr">
+        <is>
+          <t>ARMADURA DEL PILOTE  (planilla del Ing. Caggiano, 23-03-22)</t>
+        </is>
+      </c>
       <c r="B9" s="2" t="n"/>
-      <c r="C9" s="2" t="n"/>
+      <c r="C9" s="42" t="inlineStr">
+        <is>
+          <t>5 barras del 12 longitudinales, mas espiral o6 c/15 de 20 cm de diametro, 27 vueltas, longitud teorica 16,95 m. SIN BULBO.</t>
+        </is>
+      </c>
       <c r="D9" s="2" t="n"/>
       <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="57" t="inlineStr">
@@ -3831,6 +3848,7 @@
       <c r="C10" s="2" t="n"/>
       <c r="D10" s="2" t="n"/>
       <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="45" t="inlineStr">
@@ -3858,6 +3876,7 @@
           <t>long. hormigon</t>
         </is>
       </c>
+      <c r="F11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="46" t="inlineStr">
@@ -3875,7 +3894,12 @@
         <v>-0.4</v>
       </c>
       <c r="E12" s="58" t="n">
-        <v>4.1</v>
+        <v>4.6</v>
+      </c>
+      <c r="F12" s="51" t="inlineStr">
+        <is>
+          <t>bajo cabezales de 70 cm (CBZ02 y CBZ03)</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -3894,7 +3918,12 @@
         <v>-0.35</v>
       </c>
       <c r="E13" s="58" t="n">
-        <v>4.15</v>
+        <v>4.5</v>
+      </c>
+      <c r="F13" s="51" t="inlineStr">
+        <is>
+          <t>bajo cabezales de 65 cm (CBZ01)</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -3913,7 +3942,12 @@
         <v>-0.05</v>
       </c>
       <c r="E14" s="58" t="n">
-        <v>4.45</v>
+        <v>4.35</v>
+      </c>
+      <c r="F14" s="51" t="inlineStr">
+        <is>
+          <t>bajo VF de 25x35 y 20x35</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -3933,6 +3967,11 @@
       </c>
       <c r="E15" s="58" t="n">
         <v>4.4</v>
+      </c>
+      <c r="F15" s="51" t="inlineStr">
+        <is>
+          <t>bajo VF de 25x40</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -3941,6 +3980,7 @@
       <c r="C16" s="2" t="n"/>
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="42" t="inlineStr">
@@ -3952,6 +3992,7 @@
       <c r="C17" s="2" t="n"/>
       <c r="D17" s="2" t="n"/>
       <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="41" t="inlineStr">
@@ -3963,6 +4004,7 @@
       <c r="C18" s="2" t="n"/>
       <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n"/>
@@ -3970,6 +4012,7 @@
       <c r="C19" s="2" t="n"/>
       <c r="D19" s="2" t="n"/>
       <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="57" t="inlineStr">
@@ -3981,6 +4024,7 @@
       <c r="C20" s="2" t="n"/>
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="42" t="inlineStr">
@@ -3992,6 +4036,7 @@
       <c r="C21" s="2" t="n"/>
       <c r="D21" s="2" t="n"/>
       <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="42" t="inlineStr">
@@ -4003,6 +4048,7 @@
       <c r="C22" s="2" t="n"/>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="42" t="inlineStr">
@@ -4014,6 +4060,7 @@
       <c r="C23" s="2" t="n"/>
       <c r="D23" s="2" t="n"/>
       <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="42" t="inlineStr">
@@ -4025,6 +4072,7 @@
       <c r="C24" s="2" t="n"/>
       <c r="D24" s="2" t="n"/>
       <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="42" t="inlineStr">
@@ -4036,6 +4084,7 @@
       <c r="C25" s="2" t="n"/>
       <c r="D25" s="2" t="n"/>
       <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="42" t="inlineStr"/>
@@ -4043,6 +4092,7 @@
       <c r="C26" s="2" t="n"/>
       <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="41" t="inlineStr">
@@ -4054,6 +4104,7 @@
       <c r="C27" s="2" t="n"/>
       <c r="D27" s="2" t="n"/>
       <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="42" t="inlineStr">
@@ -4065,6 +4116,7 @@
       <c r="C28" s="2" t="n"/>
       <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="42" t="inlineStr">
@@ -4076,6 +4128,7 @@
       <c r="C29" s="2" t="n"/>
       <c r="D29" s="2" t="n"/>
       <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="42" t="inlineStr">
@@ -4087,6 +4140,7 @@
       <c r="C30" s="2" t="n"/>
       <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="42" t="inlineStr"/>
@@ -4094,28 +4148,31 @@
       <c r="C31" s="2" t="n"/>
       <c r="D31" s="2" t="n"/>
       <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="42" t="inlineStr">
         <is>
-          <t>FALTA: la nota del plano remite a las planillas de cada tipo de pilote, que</t>
+          <t>Capacidad ESTRUCTURAL del pilote: con 5d12 (5,65 cm2) en 707 cm2, cuantia 0,8%,</t>
         </is>
       </c>
       <c r="B32" s="2" t="n"/>
       <c r="C32" s="2" t="n"/>
       <c r="D32" s="2" t="n"/>
       <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="42" t="inlineStr">
         <is>
-          <t>traen la armadura y quiza la carga. Si aparecen, se cierra este punto.</t>
+          <t>fi Pn = 77,4 t. La seccion de hormigon no es el limite: manda el suelo.</t>
         </is>
       </c>
       <c r="B33" s="2" t="n"/>
       <c r="C33" s="2" t="n"/>
       <c r="D33" s="2" t="n"/>
       <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="42" t="inlineStr"/>
@@ -4123,39 +4180,75 @@
       <c r="C34" s="2" t="n"/>
       <c r="D34" s="2" t="n"/>
       <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="42" t="inlineStr">
         <is>
-          <t>La tension de 2 kg/cm2 que trae el calculo de bases es la del estrato</t>
+          <t>FALTA todavia la capacidad geotecnica. Las planillas de armadura de pilotes no</t>
         </is>
       </c>
       <c r="B35" s="2" t="n"/>
       <c r="C35" s="2" t="n"/>
       <c r="D35" s="2" t="n"/>
       <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="42" t="inlineStr">
         <is>
-          <t>superficial, donde apoyaban las bases. Los pilotes llegan a -4,50 m y</t>
+          <t>la traen: son planillas de doblado de hierro. Ese dato esta en el estudio de suelos.</t>
         </is>
       </c>
       <c r="B36" s="2" t="n"/>
       <c r="C36" s="2" t="n"/>
       <c r="D36" s="2" t="n"/>
       <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="42" t="inlineStr">
-        <is>
-          <t>trabajan sobre todo por friccion: son dos cosas distintas.</t>
-        </is>
-      </c>
+      <c r="A37" s="42" t="inlineStr"/>
       <c r="B37" s="2" t="n"/>
       <c r="C37" s="2" t="n"/>
       <c r="D37" s="2" t="n"/>
       <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="42" t="inlineStr">
+        <is>
+          <t>La tension de 2 kg/cm2 que trae el calculo de bases es la del estrato</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="42" t="inlineStr">
+        <is>
+          <t>superficial, donde apoyaban las bases. Los pilotes llegan a -4,50 m y</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="42" t="inlineStr">
+        <is>
+          <t>trabajan sobre todo por friccion: son dos cosas distintas.</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -16198,7 +16291,7 @@
         <v/>
       </c>
       <c r="I9" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J9" s="10" t="n">
         <v>30</v>
@@ -16220,7 +16313,7 @@
       </c>
       <c r="O9" s="13" t="inlineStr">
         <is>
-          <t>Cantidad de pilotes deducida de la dimension del cabezal: 144x70 cm. Carga tomada de la bajada de la planilla de columnas, que esta incompleta: el valor real es mayor.</t>
+          <t>Cantidad de pilotes deducida de la dimension del cabezal: 144x70 cm. Tres pilotes, no dos: la planilla de armadura declara 8 pilotes bajo cabezales de 70 cm, que son un CBZ02 y dos CBZ03. Carga tomada de la bajada de la planilla de columnas, que esta incompleta: el valor real es mayor.</t>
         </is>
       </c>
     </row>
@@ -16316,7 +16409,7 @@
         <v/>
       </c>
       <c r="I11" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>30</v>
@@ -16338,7 +16431,7 @@
       </c>
       <c r="O11" s="13" t="inlineStr">
         <is>
-          <t>Cantidad de pilotes deducida de la dimension del cabezal: 144x70 cm. Carga tomada de la bajada de la planilla de columnas, que esta incompleta: el valor real es mayor.</t>
+          <t>Cantidad de pilotes deducida de la dimension del cabezal: 144x70 cm. Tres pilotes, no dos: la planilla de armadura declara 8 pilotes bajo cabezales de 70 cm, que son un CBZ02 y dos CBZ03. Carga tomada de la bajada de la planilla de columnas, que esta incompleta: el valor real es mayor.</t>
         </is>
       </c>
     </row>
@@ -16652,7 +16745,7 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>9</v>
+        <v>18.74</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>3.15</v>
@@ -16699,7 +16792,11 @@
         <f>IF(C4="","FALTA CARGA",IF(C4&lt;=O4,"VERIFICA","NO VERIFICA"))</f>
         <v/>
       </c>
-      <c r="Q4" s="11" t="inlineStr"/>
+      <c r="Q4" s="13" t="inlineStr">
+        <is>
+          <t>9,00 t de la planilla de la catedra mas las reacciones de VI 01a (6,16 t) y VI 07a (3,58 t), que apoyan aqui. Se suman por la misma razon que en T6.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="17" customHeight="1">
       <c r="A5" s="26" t="n"/>
@@ -16709,7 +16806,7 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>6</v>
+        <v>8.5</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>3.15</v>
@@ -16756,7 +16853,11 @@
         <f>IF(C5="","FALTA CARGA",IF(C5&lt;=O5,"VERIFICA","NO VERIFICA"))</f>
         <v/>
       </c>
-      <c r="Q5" s="11" t="inlineStr"/>
+      <c r="Q5" s="13" t="inlineStr">
+        <is>
+          <t>6,00 t de la planilla de la catedra mas la reaccion de VI 01b (2,5 t), que apoya aqui y en la COL 01 de 10x10. Se suman por la misma razon que en T6.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="17" customHeight="1">
       <c r="A6" s="26" t="n"/>

</xml_diff>

<commit_message>
Sumar VI 10a al tabique T07
VI 10a descarga en la COL 01 de 10x10 y en el tabique T07, con el
que esta alineada: el tabique es su continuacion. T07 pasa de 22,43
a 24,03 t y queda al 83 por ciento de su capacidad, el elemento mas
exigido del conjunto. Verifica.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -17127,7 +17127,7 @@
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>22.43</v>
+        <v>24.03</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>3.15</v>
@@ -17176,7 +17176,7 @@
       </c>
       <c r="Q10" s="13" t="inlineStr">
         <is>
-          <t>Recibe los extremos de VI 02 (21,12 t) y de VI 17 (1,31 t). Cargas MAYORADAS, no comparables sin mas con las de T1 a T6. Es el tabique mas exigido del conjunto.</t>
+          <t>Recibe los extremos de VI 02 (21,12 t), VI 17 (1,31 t) y VI 10a (1,60 t), esta ultima alineada con el tabique, que es su continuacion. Cargas MAYORADAS, no comparables sin mas con las de T1 a T6. Es el tabique mas exigido del conjunto: 98 cm de largo tomando 24 t.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sumar VI 10b a T07, que pasa a no verificar
VI 10b descarga en el mismo tabique T07 y en una COL 02 de 15x30.
Con eso T07 acumula VI 02, VI 10b, VI 10a y VI 17: 30,62 t sobre 98
cm de tabique, el 106 por ciento de su capacidad. Es el unico
tabique que no verifica y lo hace por poco. Se deja asentado que la
formula simplificada de muro portante castiga mucho por esbeltez y
que con 104 cm de largo verificaria.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -17127,7 +17127,7 @@
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>24.03</v>
+        <v>30.62</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>3.15</v>
@@ -17176,7 +17176,7 @@
       </c>
       <c r="Q10" s="13" t="inlineStr">
         <is>
-          <t>Recibe los extremos de VI 02 (21,12 t), VI 17 (1,31 t) y VI 10a (1,60 t), esta ultima alineada con el tabique, que es su continuacion. Cargas MAYORADAS, no comparables sin mas con las de T1 a T6. Es el tabique mas exigido del conjunto: 98 cm de largo tomando 24 t.</t>
+          <t>NO VERIFICA por poco, al 106 por ciento. Recibe VI 02 (21,12 t), VI 10b (6,60 t), VI 10a (1,59 t) y VI 17 (1,31 t): 98 cm de tabique tomando 30,6 t. La capacidad sale de la formula simplificada de muro portante, cuya reduccion por esbeltez se come dos tercios: con 12 cm y 3,15 m el coeficiente vale 0,327. Un analisis mas fino del arriostramiento real daria mas capacidad. Con 104 cm de largo verificaria.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sumar VI 11c al tabique T4 y cerrar la bajada de cargas
VI 11c descarga en el T04b del plano y en una COL 02 de 15x30. Se
suma a la fila T4, que pasa a 12,52 t y usa el 12 por ciento de su
capacidad. Queda asentado que el plano distingue T04a y T04b
mientras que la planilla de la catedra tiene un solo T4, de modo
que las dos numeraciones no se corresponden una a una.
Con esto no queda ningun extremo de viga sin ubicar.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -16944,7 +16944,7 @@
         </is>
       </c>
       <c r="C7" s="8" t="n">
-        <v>5</v>
+        <v>12.52</v>
       </c>
       <c r="D7" s="8" t="n">
         <v>3.15</v>
@@ -16993,7 +16993,7 @@
       </c>
       <c r="Q7" s="13" t="inlineStr">
         <is>
-          <t>Tabique recto: B = 12 cm es el espesor.</t>
+          <t>Tabique recto: B = 12 cm es el espesor. 5,00 t de la planilla de la catedra mas la reaccion de VI 11c (7,52 t), que apoya en el T04b del plano y en una COL 02 de 15x30. OJO: el plano distingue T04a y T04b, de 0,73 m cada uno segun el computo, mientras que la catedra tiene un solo T4 de 3,55 m: las dos numeraciones no se corresponden una a una.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adoptar 22 t de capacidad por pilote, leida del propio diseno
El calculista puso un solo pilote bajo la columna mas cargada, que
baja 21,04 t de servicio: la hipotesis implicita es que el pilote
admite al menos eso. Se adopta 22 t y los nueve cabezales verifican.
Queda escrito en la memoria que esto NO es una verificacion sino la
lectura de la hipotesis del proyectista, y que para llegar a 21 t
con un O30 de 4,50 m hace falta una adherencia de 4,5 a 4,8 t/m2,
contra los 2 a 3 habituales en los limos de la region.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -3659,7 +3659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3719,7 +3719,7 @@
         </is>
       </c>
       <c r="B4" s="47" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -3728,7 +3728,7 @@
       </c>
       <c r="D4" s="51" t="inlineStr">
         <is>
-          <t>ESTIMADA. Falta el estudio de suelos: cambiar aca y recalcula todo.</t>
+          <t>ADOPTADA del propio diseno, NO verificada. Ver nota abajo. Cambiar aca cuando aparezca el estudio de suelos.</t>
         </is>
       </c>
       <c r="E4" s="2" t="n"/>
@@ -4065,7 +4065,7 @@
     <row r="24">
       <c r="A24" s="42" t="inlineStr">
         <is>
-          <t>la diferencia entre tipos es menor al 8 por ciento, por eso se adopta un unico</t>
+          <t>la diferencia entre tipos es menor al 8 por ciento, por eso se usa un unico valor</t>
         </is>
       </c>
       <c r="B24" s="2" t="n"/>
@@ -4077,7 +4077,7 @@
     <row r="25">
       <c r="A25" s="42" t="inlineStr">
         <is>
-          <t>valor de 12 t para todos, en lugar de uno por tipo.</t>
+          <t>para todos en lugar de uno por tipo.</t>
         </is>
       </c>
       <c r="B25" s="2" t="n"/>
@@ -4095,9 +4095,9 @@
       <c r="F26" s="2" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="41" t="inlineStr">
-        <is>
-          <t>LECTURA INVERSA, que es la util mientras no haya estudio de suelos:</t>
+      <c r="A27" s="42" t="inlineStr">
+        <is>
+          <t>DE DONDE SALEN LOS 22 t QUE SE ADOPTAN, Y QUE VALOR TIENEN:</t>
         </is>
       </c>
       <c r="B27" s="2" t="n"/>
@@ -4109,7 +4109,7 @@
     <row r="28">
       <c r="A28" s="42" t="inlineStr">
         <is>
-          <t>con las cargas de esta planilla, para que el esquema funcione cada pilote</t>
+          <t>El calculista puso UN solo pilote bajo la columna mas cargada, que baja 21,04 t</t>
         </is>
       </c>
       <c r="B28" s="2" t="n"/>
@@ -4121,7 +4121,7 @@
     <row r="29">
       <c r="A29" s="42" t="inlineStr">
         <is>
-          <t>tiene que admitir del orden de 20 t. Si el estudio de suelos da menos,</t>
+          <t>de servicio. Si dimensiono asi, es porque para el ese pilote admite al menos eso.</t>
         </is>
       </c>
       <c r="B29" s="2" t="n"/>
@@ -4133,7 +4133,7 @@
     <row r="30">
       <c r="A30" s="42" t="inlineStr">
         <is>
-          <t>faltan pilotes; si da mas, el diseno esta holgado.</t>
+          <t>Se adopta 22 t, el redondeo por encima de esa solicitacion.</t>
         </is>
       </c>
       <c r="B30" s="2" t="n"/>
@@ -4153,7 +4153,7 @@
     <row r="32">
       <c r="A32" s="42" t="inlineStr">
         <is>
-          <t>Capacidad ESTRUCTURAL del pilote: con 5d12 (5,65 cm2) en 707 cm2, cuantia 0,8%,</t>
+          <t>ESTO NO ES UNA VERIFICACION. Es leer la hipotesis implicita del proyectista y</t>
         </is>
       </c>
       <c r="B32" s="2" t="n"/>
@@ -4165,7 +4165,7 @@
     <row r="33">
       <c r="A33" s="42" t="inlineStr">
         <is>
-          <t>fi Pn = 77,4 t. La seccion de hormigon no es el limite: manda el suelo.</t>
+          <t>adoptarla: por construccion, todos los cabezales dan verde. Sirve para completar</t>
         </is>
       </c>
       <c r="B33" s="2" t="n"/>
@@ -4175,7 +4175,11 @@
       <c r="F33" s="2" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="42" t="inlineStr"/>
+      <c r="A34" s="42" t="inlineStr">
+        <is>
+          <t>la planilla y para dejar escrito cuanto tiene que resistir el pilote, no para</t>
+        </is>
+      </c>
       <c r="B34" s="2" t="n"/>
       <c r="C34" s="2" t="n"/>
       <c r="D34" s="2" t="n"/>
@@ -4185,7 +4189,7 @@
     <row r="35">
       <c r="A35" s="42" t="inlineStr">
         <is>
-          <t>FALTA todavia la capacidad geotecnica. Las planillas de armadura de pilotes no</t>
+          <t>afirmar que resiste. La verificacion real necesita el estudio de suelos.</t>
         </is>
       </c>
       <c r="B35" s="2" t="n"/>
@@ -4195,11 +4199,7 @@
       <c r="F35" s="2" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="42" t="inlineStr">
-        <is>
-          <t>la traen: son planillas de doblado de hierro. Ese dato esta en el estudio de suelos.</t>
-        </is>
-      </c>
+      <c r="A36" s="42" t="inlineStr"/>
       <c r="B36" s="2" t="n"/>
       <c r="C36" s="2" t="n"/>
       <c r="D36" s="2" t="n"/>
@@ -4207,7 +4207,11 @@
       <c r="F36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="42" t="inlineStr"/>
+      <c r="A37" s="42" t="inlineStr">
+        <is>
+          <t>CONTRASTE: para llegar a 21 t con un O30 de 4,50 m hace falta una adherencia</t>
+        </is>
+      </c>
       <c r="B37" s="2" t="n"/>
       <c r="C37" s="2" t="n"/>
       <c r="D37" s="2" t="n"/>
@@ -4217,7 +4221,7 @@
     <row r="38">
       <c r="A38" s="42" t="inlineStr">
         <is>
-          <t>La tension de 2 kg/cm2 que trae el calculo de bases es la del estrato</t>
+          <t>lateral de 4,5 a 4,8 t/m2. En los limos loessicos de la region de Rosario y Funes</t>
         </is>
       </c>
       <c r="B38" s="2" t="n"/>
@@ -4229,7 +4233,7 @@
     <row r="39">
       <c r="A39" s="42" t="inlineStr">
         <is>
-          <t>superficial, donde apoyaban las bases. Los pilotes llegan a -4,50 m y</t>
+          <t>los valores habituales van de 2 a 3 t/m2, que darian entre 10 y 14 t. O el estudio</t>
         </is>
       </c>
       <c r="B39" s="2" t="n"/>
@@ -4241,7 +4245,7 @@
     <row r="40">
       <c r="A40" s="42" t="inlineStr">
         <is>
-          <t>trabajan sobre todo por friccion: son dos cosas distintas.</t>
+          <t>dio un suelo mejor del tipico, o las cargas adoptadas en esta planilla estan altas,</t>
         </is>
       </c>
       <c r="B40" s="2" t="n"/>
@@ -4249,6 +4253,126 @@
       <c r="D40" s="2" t="n"/>
       <c r="E40" s="2" t="n"/>
       <c r="F40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="42" t="inlineStr">
+        <is>
+          <t>o el pilote esta ajustado. Es un punto a plantear en el trabajo.</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="n"/>
+      <c r="C41" s="2" t="n"/>
+      <c r="D41" s="2" t="n"/>
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="42" t="inlineStr"/>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="2" t="n"/>
+      <c r="D42" s="2" t="n"/>
+      <c r="E42" s="2" t="n"/>
+      <c r="F42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="42" t="inlineStr">
+        <is>
+          <t>Capacidad ESTRUCTURAL del pilote: con 5d12 (5,65 cm2) en 707 cm2, cuantia 0,8%,</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="42" t="inlineStr">
+        <is>
+          <t>fi Pn = 77,4 t. La seccion de hormigon no es el limite: manda el suelo.</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="2" t="n"/>
+      <c r="D44" s="2" t="n"/>
+      <c r="E44" s="2" t="n"/>
+      <c r="F44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="42" t="inlineStr"/>
+      <c r="B45" s="2" t="n"/>
+      <c r="C45" s="2" t="n"/>
+      <c r="D45" s="2" t="n"/>
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="42" t="inlineStr">
+        <is>
+          <t>FALTA todavia la capacidad geotecnica. Las planillas de armadura de pilotes no</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="n"/>
+      <c r="C46" s="2" t="n"/>
+      <c r="D46" s="2" t="n"/>
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="42" t="inlineStr">
+        <is>
+          <t>la traen: son planillas de doblado de hierro. Ese dato esta en el estudio de suelos.</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="n"/>
+      <c r="C47" s="2" t="n"/>
+      <c r="D47" s="2" t="n"/>
+      <c r="E47" s="2" t="n"/>
+      <c r="F47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="42" t="inlineStr"/>
+      <c r="B48" s="2" t="n"/>
+      <c r="C48" s="2" t="n"/>
+      <c r="D48" s="2" t="n"/>
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="42" t="inlineStr">
+        <is>
+          <t>La tension de 2 kg/cm2 que trae el calculo de bases es la del estrato</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="n"/>
+      <c r="C49" s="2" t="n"/>
+      <c r="D49" s="2" t="n"/>
+      <c r="E49" s="2" t="n"/>
+      <c r="F49" s="2" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="42" t="inlineStr">
+        <is>
+          <t>superficial, donde apoyaban las bases. Los pilotes llegan a -4,50 m y</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="n"/>
+      <c r="C50" s="2" t="n"/>
+      <c r="D50" s="2" t="n"/>
+      <c r="E50" s="2" t="n"/>
+      <c r="F50" s="2" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="42" t="inlineStr">
+        <is>
+          <t>trabajan sobre todo por friccion: son dos cosas distintas.</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="n"/>
+      <c r="C51" s="2" t="n"/>
+      <c r="D51" s="2" t="n"/>
+      <c r="E51" s="2" t="n"/>
+      <c r="F51" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Planilla 3: orientar las fachadas segun el norte del plano
El simbolo de norte del plano de plantas (flecha con arco) apunta hacia la
derecha de la hoja: derecha = Norte, izquierda = Sur, abajo = Este,
arriba = Oeste. Coincide con los rotulos Dormitorio Norte / Dormitorio Sur.

Los bloques pasan a ser las cuatro fachadas cardinales y cada abertura se
asigna por su posicion en planta, con la columna Orientacion cargada.
PF01, PF02 y PV01, que dan al patio interno, quedan en un bloque aparte
hasta confirmar a que lado del patio dan.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -29,7 +29,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Iluminacion y ventilacion'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Planilla 3 higrotermica'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla 3 higrotermica'!$A$1:$M$34</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla 3 higrotermica'!$A$1:$M$37</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Planilla vigas'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Planilla vigas'!$A$1:$X$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Planilla losas'!$1:$3</definedName>
@@ -7619,7 +7619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M59"/>
+  <dimension ref="A1:M64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7783,7 +7783,7 @@
     <row r="6">
       <c r="A6" s="24" t="inlineStr">
         <is>
-          <t>Plano: Vista Frente</t>
+          <t>Plano: Fachada Norte</t>
         </is>
       </c>
       <c r="B6" s="4" t="n"/>
@@ -7802,19 +7802,19 @@
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="25" t="inlineStr">
         <is>
-          <t>PA01</t>
+          <t>PV02</t>
         </is>
       </c>
       <c r="B7" s="26" t="n"/>
       <c r="C7" s="27" t="n">
-        <v>1</v>
+        <v>2.48</v>
       </c>
       <c r="D7" s="28">
         <f>IF(COUNT(B7,C7)&lt;2,"",B7*C7)</f>
         <v/>
       </c>
       <c r="E7" s="29">
-        <f>SUM(D7:D13)</f>
+        <f>SUM(D7:D11)</f>
         <v/>
       </c>
       <c r="F7" s="30">
@@ -7834,7 +7834,11 @@
       <c r="J7" s="27" t="n">
         <v>2.8</v>
       </c>
-      <c r="K7" s="25" t="n"/>
+      <c r="K7" s="25" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
       <c r="L7" s="27" t="n"/>
       <c r="M7" s="31">
         <f>IF(OR(D7="",J7=""),"",IF(J7&lt;=G7,"CUMPLE","NO CUMPLE"))</f>
@@ -7844,12 +7848,12 @@
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="25" t="inlineStr">
         <is>
-          <t>PA02</t>
+          <t>PF03</t>
         </is>
       </c>
       <c r="B8" s="26" t="n"/>
       <c r="C8" s="27" t="n">
-        <v>0.75</v>
+        <v>2.88</v>
       </c>
       <c r="D8" s="28">
         <f>IF(COUNT(B8,C8)&lt;2,"",B8*C8)</f>
@@ -7873,7 +7877,11 @@
       <c r="J8" s="27" t="n">
         <v>2.8</v>
       </c>
-      <c r="K8" s="25" t="n"/>
+      <c r="K8" s="25" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
       <c r="L8" s="27" t="n"/>
       <c r="M8" s="31">
         <f>IF(OR(D8="",J8=""),"",IF(J8&lt;=G8,"CUMPLE","NO CUMPLE"))</f>
@@ -7883,12 +7891,12 @@
     <row r="9" ht="17" customHeight="1">
       <c r="A9" s="25" t="inlineStr">
         <is>
-          <t>VA01</t>
+          <t>VA04</t>
         </is>
       </c>
       <c r="B9" s="26" t="n"/>
       <c r="C9" s="27" t="n">
-        <v>0.75</v>
+        <v>2</v>
       </c>
       <c r="D9" s="28">
         <f>IF(COUNT(B9,C9)&lt;2,"",B9*C9)</f>
@@ -7912,7 +7920,11 @@
       <c r="J9" s="27" t="n">
         <v>2.8</v>
       </c>
-      <c r="K9" s="25" t="n"/>
+      <c r="K9" s="25" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
       <c r="L9" s="27" t="n"/>
       <c r="M9" s="31">
         <f>IF(OR(D9="",J9=""),"",IF(J9&lt;=G9,"CUMPLE","NO CUMPLE"))</f>
@@ -7920,15 +7932,9 @@
       </c>
     </row>
     <row r="10" ht="17" customHeight="1">
-      <c r="A10" s="25" t="inlineStr">
-        <is>
-          <t>VA02</t>
-        </is>
-      </c>
-      <c r="B10" s="26" t="n"/>
-      <c r="C10" s="27" t="n">
-        <v>0.75</v>
-      </c>
+      <c r="A10" s="25" t="n"/>
+      <c r="B10" s="27" t="n"/>
+      <c r="C10" s="27" t="n"/>
       <c r="D10" s="28">
         <f>IF(COUNT(B10,C10)&lt;2,"",B10*C10)</f>
         <v/>
@@ -7942,15 +7948,9 @@
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H10" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
+      <c r="H10" s="25" t="n"/>
       <c r="I10" s="25" t="n"/>
-      <c r="J10" s="27" t="n">
-        <v>2.8</v>
-      </c>
+      <c r="J10" s="27" t="n"/>
       <c r="K10" s="25" t="n"/>
       <c r="L10" s="27" t="n"/>
       <c r="M10" s="31">
@@ -7959,215 +7959,190 @@
       </c>
     </row>
     <row r="11" ht="17" customHeight="1">
-      <c r="A11" s="25" t="inlineStr">
-        <is>
-          <t>VA03</t>
-        </is>
-      </c>
-      <c r="B11" s="26" t="n"/>
-      <c r="C11" s="27" t="n">
+      <c r="A11" s="33" t="n"/>
+      <c r="B11" s="34" t="n"/>
+      <c r="C11" s="34" t="n"/>
+      <c r="D11" s="35">
+        <f>IF(COUNT(B11,C11)&lt;2,"",B11*C11)</f>
+        <v/>
+      </c>
+      <c r="E11" s="36" t="n"/>
+      <c r="F11" s="37">
+        <f>IF(OR(D11="",$E$7=""),"",D11/$E$7)</f>
+        <v/>
+      </c>
+      <c r="G11" s="35">
+        <f>Datos_higro!$B$4</f>
+        <v/>
+      </c>
+      <c r="H11" s="33" t="n"/>
+      <c r="I11" s="33" t="n"/>
+      <c r="J11" s="34" t="n"/>
+      <c r="K11" s="33" t="n"/>
+      <c r="L11" s="34" t="n"/>
+      <c r="M11" s="38">
+        <f>IF(OR(D11="",J11=""),"",IF(J11&lt;=G11,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>Plano: Fachada Sur</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n"/>
+      <c r="C12" s="4" t="n"/>
+      <c r="D12" s="4" t="n"/>
+      <c r="E12" s="4" t="n"/>
+      <c r="F12" s="4" t="n"/>
+      <c r="G12" s="4" t="n"/>
+      <c r="H12" s="4" t="n"/>
+      <c r="I12" s="4" t="n"/>
+      <c r="J12" s="4" t="n"/>
+      <c r="K12" s="4" t="n"/>
+      <c r="L12" s="4" t="n"/>
+      <c r="M12" s="4" t="n"/>
+    </row>
+    <row r="13" ht="17" customHeight="1">
+      <c r="A13" s="25" t="inlineStr">
+        <is>
+          <t>VA01</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="n"/>
+      <c r="C13" s="27" t="n">
         <v>0.75</v>
       </c>
-      <c r="D11" s="28">
-        <f>IF(COUNT(B11,C11)&lt;2,"",B11*C11)</f>
-        <v/>
-      </c>
-      <c r="E11" s="32" t="n"/>
-      <c r="F11" s="30">
-        <f>IF(OR(D11="",$E$7=""),"",D11/$E$7)</f>
-        <v/>
-      </c>
-      <c r="G11" s="28">
+      <c r="D13" s="28">
+        <f>IF(COUNT(B13,C13)&lt;2,"",B13*C13)</f>
+        <v/>
+      </c>
+      <c r="E13" s="29">
+        <f>SUM(D13:D15)</f>
+        <v/>
+      </c>
+      <c r="F13" s="30">
+        <f>IF(OR(D13="",$E$13=""),"",D13/$E$13)</f>
+        <v/>
+      </c>
+      <c r="G13" s="28">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H11" s="25" t="inlineStr">
+      <c r="H13" s="25" t="inlineStr">
         <is>
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I11" s="25" t="n"/>
-      <c r="J11" s="27" t="n">
+      <c r="I13" s="25" t="n"/>
+      <c r="J13" s="27" t="n">
         <v>2.8</v>
       </c>
-      <c r="K11" s="25" t="n"/>
-      <c r="L11" s="27" t="n"/>
-      <c r="M11" s="31">
-        <f>IF(OR(D11="",J11=""),"",IF(J11&lt;=G11,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="17" customHeight="1">
-      <c r="A12" s="25" t="n"/>
-      <c r="B12" s="27" t="n"/>
-      <c r="C12" s="27" t="n"/>
-      <c r="D12" s="28">
-        <f>IF(COUNT(B12,C12)&lt;2,"",B12*C12)</f>
-        <v/>
-      </c>
-      <c r="E12" s="32" t="n"/>
-      <c r="F12" s="30">
-        <f>IF(OR(D12="",$E$7=""),"",D12/$E$7)</f>
-        <v/>
-      </c>
-      <c r="G12" s="28">
+      <c r="K13" s="25" t="inlineStr">
+        <is>
+          <t>Sur</t>
+        </is>
+      </c>
+      <c r="L13" s="27" t="n"/>
+      <c r="M13" s="31">
+        <f>IF(OR(D13="",J13=""),"",IF(J13&lt;=G13,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" s="25" t="n"/>
+      <c r="B14" s="27" t="n"/>
+      <c r="C14" s="27" t="n"/>
+      <c r="D14" s="28">
+        <f>IF(COUNT(B14,C14)&lt;2,"",B14*C14)</f>
+        <v/>
+      </c>
+      <c r="E14" s="32" t="n"/>
+      <c r="F14" s="30">
+        <f>IF(OR(D14="",$E$13=""),"",D14/$E$13)</f>
+        <v/>
+      </c>
+      <c r="G14" s="28">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H12" s="25" t="n"/>
-      <c r="I12" s="25" t="n"/>
-      <c r="J12" s="27" t="n"/>
-      <c r="K12" s="25" t="n"/>
-      <c r="L12" s="27" t="n"/>
-      <c r="M12" s="31">
-        <f>IF(OR(D12="",J12=""),"",IF(J12&lt;=G12,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="17" customHeight="1">
-      <c r="A13" s="33" t="n"/>
-      <c r="B13" s="34" t="n"/>
-      <c r="C13" s="34" t="n"/>
-      <c r="D13" s="35">
-        <f>IF(COUNT(B13,C13)&lt;2,"",B13*C13)</f>
-        <v/>
-      </c>
-      <c r="E13" s="36" t="n"/>
-      <c r="F13" s="37">
-        <f>IF(OR(D13="",$E$7=""),"",D13/$E$7)</f>
-        <v/>
-      </c>
-      <c r="G13" s="35">
+      <c r="H14" s="25" t="n"/>
+      <c r="I14" s="25" t="n"/>
+      <c r="J14" s="27" t="n"/>
+      <c r="K14" s="25" t="n"/>
+      <c r="L14" s="27" t="n"/>
+      <c r="M14" s="31">
+        <f>IF(OR(D14="",J14=""),"",IF(J14&lt;=G14,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" s="33" t="n"/>
+      <c r="B15" s="34" t="n"/>
+      <c r="C15" s="34" t="n"/>
+      <c r="D15" s="35">
+        <f>IF(COUNT(B15,C15)&lt;2,"",B15*C15)</f>
+        <v/>
+      </c>
+      <c r="E15" s="36" t="n"/>
+      <c r="F15" s="37">
+        <f>IF(OR(D15="",$E$13=""),"",D15/$E$13)</f>
+        <v/>
+      </c>
+      <c r="G15" s="35">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H13" s="33" t="n"/>
-      <c r="I13" s="33" t="n"/>
-      <c r="J13" s="34" t="n"/>
-      <c r="K13" s="33" t="n"/>
-      <c r="L13" s="34" t="n"/>
-      <c r="M13" s="38">
-        <f>IF(OR(D13="",J13=""),"",IF(J13&lt;=G13,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="24" t="inlineStr">
-        <is>
-          <t>Plano: Vista Contrafachada</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="4" t="n"/>
-      <c r="F14" s="4" t="n"/>
-      <c r="G14" s="4" t="n"/>
-      <c r="H14" s="4" t="n"/>
-      <c r="I14" s="4" t="n"/>
-      <c r="J14" s="4" t="n"/>
-      <c r="K14" s="4" t="n"/>
-      <c r="L14" s="4" t="n"/>
-      <c r="M14" s="4" t="n"/>
-    </row>
-    <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="25" t="inlineStr">
-        <is>
-          <t>PF01</t>
-        </is>
-      </c>
-      <c r="B15" s="26" t="n"/>
-      <c r="C15" s="27" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="D15" s="28">
-        <f>IF(COUNT(B15,C15)&lt;2,"",B15*C15)</f>
-        <v/>
-      </c>
-      <c r="E15" s="29">
-        <f>SUM(D15:D19)</f>
-        <v/>
-      </c>
-      <c r="F15" s="30">
-        <f>IF(OR(D15="",$E$15=""),"",D15/$E$15)</f>
-        <v/>
-      </c>
-      <c r="G15" s="28">
-        <f>Datos_higro!$B$4</f>
-        <v/>
-      </c>
-      <c r="H15" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I15" s="25" t="n"/>
-      <c r="J15" s="27" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K15" s="25" t="n"/>
-      <c r="L15" s="27" t="n"/>
-      <c r="M15" s="31">
+      <c r="H15" s="33" t="n"/>
+      <c r="I15" s="33" t="n"/>
+      <c r="J15" s="34" t="n"/>
+      <c r="K15" s="33" t="n"/>
+      <c r="L15" s="34" t="n"/>
+      <c r="M15" s="38">
         <f>IF(OR(D15="",J15=""),"",IF(J15&lt;=G15,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="16" ht="17" customHeight="1">
-      <c r="A16" s="25" t="inlineStr">
-        <is>
-          <t>PF02</t>
-        </is>
-      </c>
-      <c r="B16" s="26" t="n"/>
-      <c r="C16" s="27" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="D16" s="28">
-        <f>IF(COUNT(B16,C16)&lt;2,"",B16*C16)</f>
-        <v/>
-      </c>
-      <c r="E16" s="32" t="n"/>
-      <c r="F16" s="30">
-        <f>IF(OR(D16="",$E$15=""),"",D16/$E$15)</f>
-        <v/>
-      </c>
-      <c r="G16" s="28">
-        <f>Datos_higro!$B$4</f>
-        <v/>
-      </c>
-      <c r="H16" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I16" s="25" t="n"/>
-      <c r="J16" s="27" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K16" s="25" t="n"/>
-      <c r="L16" s="27" t="n"/>
-      <c r="M16" s="31">
-        <f>IF(OR(D16="",J16=""),"",IF(J16&lt;=G16,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
+    <row r="16">
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>Plano: Fachada Este</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="4" t="n"/>
+      <c r="D16" s="4" t="n"/>
+      <c r="E16" s="4" t="n"/>
+      <c r="F16" s="4" t="n"/>
+      <c r="G16" s="4" t="n"/>
+      <c r="H16" s="4" t="n"/>
+      <c r="I16" s="4" t="n"/>
+      <c r="J16" s="4" t="n"/>
+      <c r="K16" s="4" t="n"/>
+      <c r="L16" s="4" t="n"/>
+      <c r="M16" s="4" t="n"/>
     </row>
     <row r="17" ht="17" customHeight="1">
       <c r="A17" s="25" t="inlineStr">
         <is>
-          <t>PF03</t>
+          <t>PA01</t>
         </is>
       </c>
       <c r="B17" s="26" t="n"/>
       <c r="C17" s="27" t="n">
-        <v>2.88</v>
+        <v>1</v>
       </c>
       <c r="D17" s="28">
         <f>IF(COUNT(B17,C17)&lt;2,"",B17*C17)</f>
         <v/>
       </c>
-      <c r="E17" s="32" t="n"/>
+      <c r="E17" s="29">
+        <f>SUM(D17:D22)</f>
+        <v/>
+      </c>
       <c r="F17" s="30">
-        <f>IF(OR(D17="",$E$15=""),"",D17/$E$15)</f>
+        <f>IF(OR(D17="",$E$17=""),"",D17/$E$17)</f>
         <v/>
       </c>
       <c r="G17" s="28">
@@ -8183,7 +8158,11 @@
       <c r="J17" s="27" t="n">
         <v>2.8</v>
       </c>
-      <c r="K17" s="25" t="n"/>
+      <c r="K17" s="25" t="inlineStr">
+        <is>
+          <t>Este</t>
+        </is>
+      </c>
       <c r="L17" s="27" t="n"/>
       <c r="M17" s="31">
         <f>IF(OR(D17="",J17=""),"",IF(J17&lt;=G17,"CUMPLE","NO CUMPLE"))</f>
@@ -8191,26 +8170,42 @@
       </c>
     </row>
     <row r="18" ht="17" customHeight="1">
-      <c r="A18" s="25" t="n"/>
-      <c r="B18" s="27" t="n"/>
-      <c r="C18" s="27" t="n"/>
+      <c r="A18" s="25" t="inlineStr">
+        <is>
+          <t>PF04</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="n"/>
+      <c r="C18" s="27" t="n">
+        <v>2.7</v>
+      </c>
       <c r="D18" s="28">
         <f>IF(COUNT(B18,C18)&lt;2,"",B18*C18)</f>
         <v/>
       </c>
       <c r="E18" s="32" t="n"/>
       <c r="F18" s="30">
-        <f>IF(OR(D18="",$E$15=""),"",D18/$E$15)</f>
+        <f>IF(OR(D18="",$E$17=""),"",D18/$E$17)</f>
         <v/>
       </c>
       <c r="G18" s="28">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H18" s="25" t="n"/>
+      <c r="H18" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
       <c r="I18" s="25" t="n"/>
-      <c r="J18" s="27" t="n"/>
-      <c r="K18" s="25" t="n"/>
+      <c r="J18" s="27" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K18" s="25" t="inlineStr">
+        <is>
+          <t>Este</t>
+        </is>
+      </c>
       <c r="L18" s="27" t="n"/>
       <c r="M18" s="31">
         <f>IF(OR(D18="",J18=""),"",IF(J18&lt;=G18,"CUMPLE","NO CUMPLE"))</f>
@@ -8218,86 +8213,111 @@
       </c>
     </row>
     <row r="19" ht="17" customHeight="1">
-      <c r="A19" s="33" t="n"/>
-      <c r="B19" s="34" t="n"/>
-      <c r="C19" s="34" t="n"/>
-      <c r="D19" s="35">
+      <c r="A19" s="25" t="inlineStr">
+        <is>
+          <t>VA05</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="n"/>
+      <c r="C19" s="27" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D19" s="28">
         <f>IF(COUNT(B19,C19)&lt;2,"",B19*C19)</f>
         <v/>
       </c>
-      <c r="E19" s="36" t="n"/>
-      <c r="F19" s="37">
-        <f>IF(OR(D19="",$E$15=""),"",D19/$E$15)</f>
-        <v/>
-      </c>
-      <c r="G19" s="35">
+      <c r="E19" s="32" t="n"/>
+      <c r="F19" s="30">
+        <f>IF(OR(D19="",$E$17=""),"",D19/$E$17)</f>
+        <v/>
+      </c>
+      <c r="G19" s="28">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H19" s="33" t="n"/>
-      <c r="I19" s="33" t="n"/>
-      <c r="J19" s="34" t="n"/>
-      <c r="K19" s="33" t="n"/>
-      <c r="L19" s="34" t="n"/>
-      <c r="M19" s="38">
+      <c r="H19" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I19" s="25" t="n"/>
+      <c r="J19" s="27" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K19" s="25" t="inlineStr">
+        <is>
+          <t>Este</t>
+        </is>
+      </c>
+      <c r="L19" s="27" t="n"/>
+      <c r="M19" s="31">
         <f>IF(OR(D19="",J19=""),"",IF(J19&lt;=G19,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="24" t="inlineStr">
-        <is>
-          <t>Plano: Vista Lateral Izquierda</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="4" t="n"/>
-      <c r="G20" s="4" t="n"/>
-      <c r="H20" s="4" t="n"/>
-      <c r="I20" s="4" t="n"/>
-      <c r="J20" s="4" t="n"/>
-      <c r="K20" s="4" t="n"/>
-      <c r="L20" s="4" t="n"/>
-      <c r="M20" s="4" t="n"/>
+    <row r="20" ht="17" customHeight="1">
+      <c r="A20" s="25" t="inlineStr">
+        <is>
+          <t>PV04</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="n"/>
+      <c r="C20" s="27" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="D20" s="28">
+        <f>IF(COUNT(B20,C20)&lt;2,"",B20*C20)</f>
+        <v/>
+      </c>
+      <c r="E20" s="32" t="n"/>
+      <c r="F20" s="30">
+        <f>IF(OR(D20="",$E$17=""),"",D20/$E$17)</f>
+        <v/>
+      </c>
+      <c r="G20" s="28">
+        <f>Datos_higro!$B$4</f>
+        <v/>
+      </c>
+      <c r="H20" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I20" s="25" t="n"/>
+      <c r="J20" s="27" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K20" s="25" t="inlineStr">
+        <is>
+          <t>Este</t>
+        </is>
+      </c>
+      <c r="L20" s="27" t="n"/>
+      <c r="M20" s="31">
+        <f>IF(OR(D20="",J20=""),"",IF(J20&lt;=G20,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
     </row>
     <row r="21" ht="17" customHeight="1">
-      <c r="A21" s="25" t="inlineStr">
-        <is>
-          <t>PF04</t>
-        </is>
-      </c>
-      <c r="B21" s="26" t="n"/>
-      <c r="C21" s="27" t="n">
-        <v>2.7</v>
-      </c>
+      <c r="A21" s="25" t="n"/>
+      <c r="B21" s="27" t="n"/>
+      <c r="C21" s="27" t="n"/>
       <c r="D21" s="28">
         <f>IF(COUNT(B21,C21)&lt;2,"",B21*C21)</f>
         <v/>
       </c>
-      <c r="E21" s="29">
-        <f>SUM(D21:D26)</f>
-        <v/>
-      </c>
+      <c r="E21" s="32" t="n"/>
       <c r="F21" s="30">
-        <f>IF(OR(D21="",$E$21=""),"",D21/$E$21)</f>
+        <f>IF(OR(D21="",$E$17=""),"",D21/$E$17)</f>
         <v/>
       </c>
       <c r="G21" s="28">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H21" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
+      <c r="H21" s="25" t="n"/>
       <c r="I21" s="25" t="n"/>
-      <c r="J21" s="27" t="n">
-        <v>2.8</v>
-      </c>
+      <c r="J21" s="27" t="n"/>
       <c r="K21" s="25" t="n"/>
       <c r="L21" s="27" t="n"/>
       <c r="M21" s="31">
@@ -8306,82 +8326,50 @@
       </c>
     </row>
     <row r="22" ht="17" customHeight="1">
-      <c r="A22" s="25" t="inlineStr">
-        <is>
-          <t>PV01</t>
-        </is>
-      </c>
-      <c r="B22" s="26" t="n"/>
-      <c r="C22" s="27" t="n">
-        <v>7.7</v>
-      </c>
-      <c r="D22" s="28">
+      <c r="A22" s="33" t="n"/>
+      <c r="B22" s="34" t="n"/>
+      <c r="C22" s="34" t="n"/>
+      <c r="D22" s="35">
         <f>IF(COUNT(B22,C22)&lt;2,"",B22*C22)</f>
         <v/>
       </c>
-      <c r="E22" s="32" t="n"/>
-      <c r="F22" s="30">
-        <f>IF(OR(D22="",$E$21=""),"",D22/$E$21)</f>
-        <v/>
-      </c>
-      <c r="G22" s="28">
+      <c r="E22" s="36" t="n"/>
+      <c r="F22" s="37">
+        <f>IF(OR(D22="",$E$17=""),"",D22/$E$17)</f>
+        <v/>
+      </c>
+      <c r="G22" s="35">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H22" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I22" s="25" t="n"/>
-      <c r="J22" s="27" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K22" s="25" t="n"/>
-      <c r="L22" s="27" t="n"/>
-      <c r="M22" s="31">
+      <c r="H22" s="33" t="n"/>
+      <c r="I22" s="33" t="n"/>
+      <c r="J22" s="34" t="n"/>
+      <c r="K22" s="33" t="n"/>
+      <c r="L22" s="34" t="n"/>
+      <c r="M22" s="38">
         <f>IF(OR(D22="",J22=""),"",IF(J22&lt;=G22,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="23" ht="17" customHeight="1">
-      <c r="A23" s="25" t="inlineStr">
-        <is>
-          <t>PV02</t>
-        </is>
-      </c>
-      <c r="B23" s="26" t="n"/>
-      <c r="C23" s="27" t="n">
-        <v>2.48</v>
-      </c>
-      <c r="D23" s="28">
-        <f>IF(COUNT(B23,C23)&lt;2,"",B23*C23)</f>
-        <v/>
-      </c>
-      <c r="E23" s="32" t="n"/>
-      <c r="F23" s="30">
-        <f>IF(OR(D23="",$E$21=""),"",D23/$E$21)</f>
-        <v/>
-      </c>
-      <c r="G23" s="28">
-        <f>Datos_higro!$B$4</f>
-        <v/>
-      </c>
-      <c r="H23" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I23" s="25" t="n"/>
-      <c r="J23" s="27" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K23" s="25" t="n"/>
-      <c r="L23" s="27" t="n"/>
-      <c r="M23" s="31">
-        <f>IF(OR(D23="",J23=""),"",IF(J23&lt;=G23,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
+    <row r="23">
+      <c r="A23" s="24" t="inlineStr">
+        <is>
+          <t>Plano: Fachada Oeste</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n"/>
+      <c r="C23" s="4" t="n"/>
+      <c r="D23" s="4" t="n"/>
+      <c r="E23" s="4" t="n"/>
+      <c r="F23" s="4" t="n"/>
+      <c r="G23" s="4" t="n"/>
+      <c r="H23" s="4" t="n"/>
+      <c r="I23" s="4" t="n"/>
+      <c r="J23" s="4" t="n"/>
+      <c r="K23" s="4" t="n"/>
+      <c r="L23" s="4" t="n"/>
+      <c r="M23" s="4" t="n"/>
     </row>
     <row r="24" ht="17" customHeight="1">
       <c r="A24" s="25" t="inlineStr">
@@ -8397,9 +8385,12 @@
         <f>IF(COUNT(B24,C24)&lt;2,"",B24*C24)</f>
         <v/>
       </c>
-      <c r="E24" s="32" t="n"/>
+      <c r="E24" s="29">
+        <f>SUM(D24:D30)</f>
+        <v/>
+      </c>
       <c r="F24" s="30">
-        <f>IF(OR(D24="",$E$21=""),"",D24/$E$21)</f>
+        <f>IF(OR(D24="",$E$24=""),"",D24/$E$24)</f>
         <v/>
       </c>
       <c r="G24" s="28">
@@ -8415,7 +8406,11 @@
       <c r="J24" s="27" t="n">
         <v>2.8</v>
       </c>
-      <c r="K24" s="25" t="n"/>
+      <c r="K24" s="25" t="inlineStr">
+        <is>
+          <t>Oeste</t>
+        </is>
+      </c>
       <c r="L24" s="27" t="n"/>
       <c r="M24" s="31">
         <f>IF(OR(D24="",J24=""),"",IF(J24&lt;=G24,"CUMPLE","NO CUMPLE"))</f>
@@ -8423,26 +8418,42 @@
       </c>
     </row>
     <row r="25" ht="17" customHeight="1">
-      <c r="A25" s="25" t="n"/>
-      <c r="B25" s="27" t="n"/>
-      <c r="C25" s="27" t="n"/>
+      <c r="A25" s="25" t="inlineStr">
+        <is>
+          <t>VA02</t>
+        </is>
+      </c>
+      <c r="B25" s="26" t="n"/>
+      <c r="C25" s="27" t="n">
+        <v>0.75</v>
+      </c>
       <c r="D25" s="28">
         <f>IF(COUNT(B25,C25)&lt;2,"",B25*C25)</f>
         <v/>
       </c>
       <c r="E25" s="32" t="n"/>
       <c r="F25" s="30">
-        <f>IF(OR(D25="",$E$21=""),"",D25/$E$21)</f>
+        <f>IF(OR(D25="",$E$24=""),"",D25/$E$24)</f>
         <v/>
       </c>
       <c r="G25" s="28">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H25" s="25" t="n"/>
+      <c r="H25" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
       <c r="I25" s="25" t="n"/>
-      <c r="J25" s="27" t="n"/>
-      <c r="K25" s="25" t="n"/>
+      <c r="J25" s="27" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K25" s="25" t="inlineStr">
+        <is>
+          <t>Oeste</t>
+        </is>
+      </c>
       <c r="L25" s="27" t="n"/>
       <c r="M25" s="31">
         <f>IF(OR(D25="",J25=""),"",IF(J25&lt;=G25,"CUMPLE","NO CUMPLE"))</f>
@@ -8450,71 +8461,108 @@
       </c>
     </row>
     <row r="26" ht="17" customHeight="1">
-      <c r="A26" s="33" t="n"/>
-      <c r="B26" s="34" t="n"/>
-      <c r="C26" s="34" t="n"/>
-      <c r="D26" s="35">
+      <c r="A26" s="25" t="inlineStr">
+        <is>
+          <t>PA02</t>
+        </is>
+      </c>
+      <c r="B26" s="26" t="n"/>
+      <c r="C26" s="27" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D26" s="28">
         <f>IF(COUNT(B26,C26)&lt;2,"",B26*C26)</f>
         <v/>
       </c>
-      <c r="E26" s="36" t="n"/>
-      <c r="F26" s="37">
-        <f>IF(OR(D26="",$E$21=""),"",D26/$E$21)</f>
-        <v/>
-      </c>
-      <c r="G26" s="35">
+      <c r="E26" s="32" t="n"/>
+      <c r="F26" s="30">
+        <f>IF(OR(D26="",$E$24=""),"",D26/$E$24)</f>
+        <v/>
+      </c>
+      <c r="G26" s="28">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H26" s="33" t="n"/>
-      <c r="I26" s="33" t="n"/>
-      <c r="J26" s="34" t="n"/>
-      <c r="K26" s="33" t="n"/>
-      <c r="L26" s="34" t="n"/>
-      <c r="M26" s="38">
+      <c r="H26" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I26" s="25" t="n"/>
+      <c r="J26" s="27" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K26" s="25" t="inlineStr">
+        <is>
+          <t>Oeste</t>
+        </is>
+      </c>
+      <c r="L26" s="27" t="n"/>
+      <c r="M26" s="31">
         <f>IF(OR(D26="",J26=""),"",IF(J26&lt;=G26,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="24" t="inlineStr">
-        <is>
-          <t>Plano: Vista Lateral Derecha</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="n"/>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="4" t="n"/>
-      <c r="G27" s="4" t="n"/>
-      <c r="H27" s="4" t="n"/>
-      <c r="I27" s="4" t="n"/>
-      <c r="J27" s="4" t="n"/>
-      <c r="K27" s="4" t="n"/>
-      <c r="L27" s="4" t="n"/>
-      <c r="M27" s="4" t="n"/>
+    <row r="27" ht="17" customHeight="1">
+      <c r="A27" s="25" t="inlineStr">
+        <is>
+          <t>VA03</t>
+        </is>
+      </c>
+      <c r="B27" s="26" t="n"/>
+      <c r="C27" s="27" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D27" s="28">
+        <f>IF(COUNT(B27,C27)&lt;2,"",B27*C27)</f>
+        <v/>
+      </c>
+      <c r="E27" s="32" t="n"/>
+      <c r="F27" s="30">
+        <f>IF(OR(D27="",$E$24=""),"",D27/$E$24)</f>
+        <v/>
+      </c>
+      <c r="G27" s="28">
+        <f>Datos_higro!$B$4</f>
+        <v/>
+      </c>
+      <c r="H27" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I27" s="25" t="n"/>
+      <c r="J27" s="27" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K27" s="25" t="inlineStr">
+        <is>
+          <t>Oeste</t>
+        </is>
+      </c>
+      <c r="L27" s="27" t="n"/>
+      <c r="M27" s="31">
+        <f>IF(OR(D27="",J27=""),"",IF(J27&lt;=G27,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
     </row>
     <row r="28" ht="17" customHeight="1">
       <c r="A28" s="25" t="inlineStr">
         <is>
-          <t>VA04</t>
+          <t>PF05</t>
         </is>
       </c>
       <c r="B28" s="26" t="n"/>
       <c r="C28" s="27" t="n">
-        <v>2</v>
+        <v>0.75</v>
       </c>
       <c r="D28" s="28">
         <f>IF(COUNT(B28,C28)&lt;2,"",B28*C28)</f>
         <v/>
       </c>
-      <c r="E28" s="29">
-        <f>SUM(D28:D34)</f>
-        <v/>
-      </c>
+      <c r="E28" s="32" t="n"/>
       <c r="F28" s="30">
-        <f>IF(OR(D28="",$E$28=""),"",D28/$E$28)</f>
+        <f>IF(OR(D28="",$E$24=""),"",D28/$E$24)</f>
         <v/>
       </c>
       <c r="G28" s="28">
@@ -8530,7 +8578,11 @@
       <c r="J28" s="27" t="n">
         <v>2.8</v>
       </c>
-      <c r="K28" s="25" t="n"/>
+      <c r="K28" s="25" t="inlineStr">
+        <is>
+          <t>Oeste</t>
+        </is>
+      </c>
       <c r="L28" s="27" t="n"/>
       <c r="M28" s="31">
         <f>IF(OR(D28="",J28=""),"",IF(J28&lt;=G28,"CUMPLE","NO CUMPLE"))</f>
@@ -8538,37 +8590,25 @@
       </c>
     </row>
     <row r="29" ht="17" customHeight="1">
-      <c r="A29" s="25" t="inlineStr">
-        <is>
-          <t>VA05</t>
-        </is>
-      </c>
-      <c r="B29" s="26" t="n"/>
-      <c r="C29" s="27" t="n">
-        <v>1.4</v>
-      </c>
+      <c r="A29" s="25" t="n"/>
+      <c r="B29" s="27" t="n"/>
+      <c r="C29" s="27" t="n"/>
       <c r="D29" s="28">
         <f>IF(COUNT(B29,C29)&lt;2,"",B29*C29)</f>
         <v/>
       </c>
       <c r="E29" s="32" t="n"/>
       <c r="F29" s="30">
-        <f>IF(OR(D29="",$E$28=""),"",D29/$E$28)</f>
+        <f>IF(OR(D29="",$E$24=""),"",D29/$E$24)</f>
         <v/>
       </c>
       <c r="G29" s="28">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H29" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
+      <c r="H29" s="25" t="n"/>
       <c r="I29" s="25" t="n"/>
-      <c r="J29" s="27" t="n">
-        <v>2.8</v>
-      </c>
+      <c r="J29" s="27" t="n"/>
       <c r="K29" s="25" t="n"/>
       <c r="L29" s="27" t="n"/>
       <c r="M29" s="31">
@@ -8577,100 +8617,71 @@
       </c>
     </row>
     <row r="30" ht="17" customHeight="1">
-      <c r="A30" s="25" t="inlineStr">
-        <is>
-          <t>PF05</t>
-        </is>
-      </c>
-      <c r="B30" s="26" t="n"/>
-      <c r="C30" s="27" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D30" s="28">
+      <c r="A30" s="33" t="n"/>
+      <c r="B30" s="34" t="n"/>
+      <c r="C30" s="34" t="n"/>
+      <c r="D30" s="35">
         <f>IF(COUNT(B30,C30)&lt;2,"",B30*C30)</f>
         <v/>
       </c>
-      <c r="E30" s="32" t="n"/>
-      <c r="F30" s="30">
-        <f>IF(OR(D30="",$E$28=""),"",D30/$E$28)</f>
-        <v/>
-      </c>
-      <c r="G30" s="28">
+      <c r="E30" s="36" t="n"/>
+      <c r="F30" s="37">
+        <f>IF(OR(D30="",$E$24=""),"",D30/$E$24)</f>
+        <v/>
+      </c>
+      <c r="G30" s="35">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H30" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I30" s="25" t="n"/>
-      <c r="J30" s="27" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K30" s="25" t="n"/>
-      <c r="L30" s="27" t="n"/>
-      <c r="M30" s="31">
+      <c r="H30" s="33" t="n"/>
+      <c r="I30" s="33" t="n"/>
+      <c r="J30" s="34" t="n"/>
+      <c r="K30" s="33" t="n"/>
+      <c r="L30" s="34" t="n"/>
+      <c r="M30" s="38">
         <f>IF(OR(D30="",J30=""),"",IF(J30&lt;=G30,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="31" ht="17" customHeight="1">
-      <c r="A31" s="25" t="inlineStr">
-        <is>
-          <t>PV04</t>
-        </is>
-      </c>
-      <c r="B31" s="26" t="n"/>
-      <c r="C31" s="27" t="n">
-        <v>2.06</v>
-      </c>
-      <c r="D31" s="28">
-        <f>IF(COUNT(B31,C31)&lt;2,"",B31*C31)</f>
-        <v/>
-      </c>
-      <c r="E31" s="32" t="n"/>
-      <c r="F31" s="30">
-        <f>IF(OR(D31="",$E$28=""),"",D31/$E$28)</f>
-        <v/>
-      </c>
-      <c r="G31" s="28">
-        <f>Datos_higro!$B$4</f>
-        <v/>
-      </c>
-      <c r="H31" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I31" s="25" t="n"/>
-      <c r="J31" s="27" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K31" s="25" t="n"/>
-      <c r="L31" s="27" t="n"/>
-      <c r="M31" s="31">
-        <f>IF(OR(D31="",J31=""),"",IF(J31&lt;=G31,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
+    <row r="31">
+      <c r="A31" s="24" t="inlineStr">
+        <is>
+          <t>Plano: Patio interno (orientacion a confirmar)</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="n"/>
+      <c r="C31" s="4" t="n"/>
+      <c r="D31" s="4" t="n"/>
+      <c r="E31" s="4" t="n"/>
+      <c r="F31" s="4" t="n"/>
+      <c r="G31" s="4" t="n"/>
+      <c r="H31" s="4" t="n"/>
+      <c r="I31" s="4" t="n"/>
+      <c r="J31" s="4" t="n"/>
+      <c r="K31" s="4" t="n"/>
+      <c r="L31" s="4" t="n"/>
+      <c r="M31" s="4" t="n"/>
     </row>
     <row r="32" ht="17" customHeight="1">
       <c r="A32" s="25" t="inlineStr">
         <is>
-          <t>PV04 (2)</t>
+          <t>PF01</t>
         </is>
       </c>
       <c r="B32" s="26" t="n"/>
       <c r="C32" s="27" t="n">
-        <v>1.5</v>
+        <v>3.55</v>
       </c>
       <c r="D32" s="28">
         <f>IF(COUNT(B32,C32)&lt;2,"",B32*C32)</f>
         <v/>
       </c>
-      <c r="E32" s="32" t="n"/>
+      <c r="E32" s="29">
+        <f>SUM(D32:D37)</f>
+        <v/>
+      </c>
       <c r="F32" s="30">
-        <f>IF(OR(D32="",$E$28=""),"",D32/$E$28)</f>
+        <f>IF(OR(D32="",$E$32=""),"",D32/$E$32)</f>
         <v/>
       </c>
       <c r="G32" s="28">
@@ -8694,25 +8705,37 @@
       </c>
     </row>
     <row r="33" ht="17" customHeight="1">
-      <c r="A33" s="25" t="n"/>
-      <c r="B33" s="27" t="n"/>
-      <c r="C33" s="27" t="n"/>
+      <c r="A33" s="25" t="inlineStr">
+        <is>
+          <t>PF02</t>
+        </is>
+      </c>
+      <c r="B33" s="26" t="n"/>
+      <c r="C33" s="27" t="n">
+        <v>3.75</v>
+      </c>
       <c r="D33" s="28">
         <f>IF(COUNT(B33,C33)&lt;2,"",B33*C33)</f>
         <v/>
       </c>
       <c r="E33" s="32" t="n"/>
       <c r="F33" s="30">
-        <f>IF(OR(D33="",$E$28=""),"",D33/$E$28)</f>
+        <f>IF(OR(D33="",$E$32=""),"",D33/$E$32)</f>
         <v/>
       </c>
       <c r="G33" s="28">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H33" s="25" t="n"/>
+      <c r="H33" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
       <c r="I33" s="25" t="n"/>
-      <c r="J33" s="27" t="n"/>
+      <c r="J33" s="27" t="n">
+        <v>2.8</v>
+      </c>
       <c r="K33" s="25" t="n"/>
       <c r="L33" s="27" t="n"/>
       <c r="M33" s="31">
@@ -8721,91 +8744,139 @@
       </c>
     </row>
     <row r="34" ht="17" customHeight="1">
-      <c r="A34" s="33" t="n"/>
-      <c r="B34" s="34" t="n"/>
-      <c r="C34" s="34" t="n"/>
-      <c r="D34" s="35">
+      <c r="A34" s="25" t="inlineStr">
+        <is>
+          <t>PV01</t>
+        </is>
+      </c>
+      <c r="B34" s="26" t="n"/>
+      <c r="C34" s="27" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="D34" s="28">
         <f>IF(COUNT(B34,C34)&lt;2,"",B34*C34)</f>
         <v/>
       </c>
-      <c r="E34" s="36" t="n"/>
-      <c r="F34" s="37">
-        <f>IF(OR(D34="",$E$28=""),"",D34/$E$28)</f>
-        <v/>
-      </c>
-      <c r="G34" s="35">
+      <c r="E34" s="32" t="n"/>
+      <c r="F34" s="30">
+        <f>IF(OR(D34="",$E$32=""),"",D34/$E$32)</f>
+        <v/>
+      </c>
+      <c r="G34" s="28">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H34" s="33" t="n"/>
-      <c r="I34" s="33" t="n"/>
-      <c r="J34" s="34" t="n"/>
-      <c r="K34" s="33" t="n"/>
-      <c r="L34" s="34" t="n"/>
-      <c r="M34" s="38">
+      <c r="H34" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I34" s="25" t="n"/>
+      <c r="J34" s="27" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K34" s="25" t="n"/>
+      <c r="L34" s="27" t="n"/>
+      <c r="M34" s="31">
         <f>IF(OR(D34="",J34=""),"",IF(J34&lt;=G34,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="n"/>
-      <c r="B35" s="2" t="n"/>
-      <c r="C35" s="2" t="n"/>
-      <c r="D35" s="2" t="n"/>
-      <c r="E35" s="2" t="n"/>
-      <c r="F35" s="2" t="n"/>
-      <c r="G35" s="2" t="n"/>
-      <c r="H35" s="2" t="n"/>
-      <c r="I35" s="2" t="n"/>
-      <c r="J35" s="2" t="n"/>
-      <c r="K35" s="2" t="n"/>
-      <c r="L35" s="2" t="n"/>
-      <c r="M35" s="2" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="39" t="inlineStr">
-        <is>
-          <t>COMO SE COMPLETA</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="2" t="n"/>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="n"/>
-      <c r="G36" s="2" t="n"/>
-      <c r="H36" s="2" t="n"/>
-      <c r="I36" s="2" t="n"/>
-      <c r="J36" s="2" t="n"/>
-      <c r="K36" s="2" t="n"/>
-      <c r="L36" s="2" t="n"/>
-      <c r="M36" s="2" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="40" t="inlineStr">
-        <is>
-          <t>Descripcion, altura y ancho del vano: de la planilla de carpinterias.</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="n"/>
-      <c r="C37" s="2" t="n"/>
-      <c r="D37" s="2" t="n"/>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="n"/>
-      <c r="G37" s="2" t="n"/>
-      <c r="H37" s="2" t="n"/>
-      <c r="I37" s="2" t="n"/>
-      <c r="J37" s="2" t="n"/>
-      <c r="K37" s="2" t="n"/>
-      <c r="L37" s="2" t="n"/>
-      <c r="M37" s="2" t="n"/>
+    <row r="35" ht="17" customHeight="1">
+      <c r="A35" s="25" t="inlineStr">
+        <is>
+          <t>PV04 (2)</t>
+        </is>
+      </c>
+      <c r="B35" s="26" t="n"/>
+      <c r="C35" s="27" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D35" s="28">
+        <f>IF(COUNT(B35,C35)&lt;2,"",B35*C35)</f>
+        <v/>
+      </c>
+      <c r="E35" s="32" t="n"/>
+      <c r="F35" s="30">
+        <f>IF(OR(D35="",$E$32=""),"",D35/$E$32)</f>
+        <v/>
+      </c>
+      <c r="G35" s="28">
+        <f>Datos_higro!$B$4</f>
+        <v/>
+      </c>
+      <c r="H35" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I35" s="25" t="n"/>
+      <c r="J35" s="27" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K35" s="25" t="n"/>
+      <c r="L35" s="27" t="n"/>
+      <c r="M35" s="31">
+        <f>IF(OR(D35="",J35=""),"",IF(J35&lt;=G35,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="17" customHeight="1">
+      <c r="A36" s="25" t="n"/>
+      <c r="B36" s="27" t="n"/>
+      <c r="C36" s="27" t="n"/>
+      <c r="D36" s="28">
+        <f>IF(COUNT(B36,C36)&lt;2,"",B36*C36)</f>
+        <v/>
+      </c>
+      <c r="E36" s="32" t="n"/>
+      <c r="F36" s="30">
+        <f>IF(OR(D36="",$E$32=""),"",D36/$E$32)</f>
+        <v/>
+      </c>
+      <c r="G36" s="28">
+        <f>Datos_higro!$B$4</f>
+        <v/>
+      </c>
+      <c r="H36" s="25" t="n"/>
+      <c r="I36" s="25" t="n"/>
+      <c r="J36" s="27" t="n"/>
+      <c r="K36" s="25" t="n"/>
+      <c r="L36" s="27" t="n"/>
+      <c r="M36" s="31">
+        <f>IF(OR(D36="",J36=""),"",IF(J36&lt;=G36,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="17" customHeight="1">
+      <c r="A37" s="33" t="n"/>
+      <c r="B37" s="34" t="n"/>
+      <c r="C37" s="34" t="n"/>
+      <c r="D37" s="35">
+        <f>IF(COUNT(B37,C37)&lt;2,"",B37*C37)</f>
+        <v/>
+      </c>
+      <c r="E37" s="36" t="n"/>
+      <c r="F37" s="37">
+        <f>IF(OR(D37="",$E$32=""),"",D37/$E$32)</f>
+        <v/>
+      </c>
+      <c r="G37" s="35">
+        <f>Datos_higro!$B$4</f>
+        <v/>
+      </c>
+      <c r="H37" s="33" t="n"/>
+      <c r="I37" s="33" t="n"/>
+      <c r="J37" s="34" t="n"/>
+      <c r="K37" s="33" t="n"/>
+      <c r="L37" s="34" t="n"/>
+      <c r="M37" s="38">
+        <f>IF(OR(D37="",J37=""),"",IF(J37&lt;=G37,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="40" t="inlineStr">
-        <is>
-          <t>Area del vano, area total por plano y porcentaje: se calculan solos.</t>
-        </is>
-      </c>
+      <c r="A38" s="2" t="n"/>
       <c r="B38" s="2" t="n"/>
       <c r="C38" s="2" t="n"/>
       <c r="D38" s="2" t="n"/>
@@ -8820,9 +8891,9 @@
       <c r="M38" s="2" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="40" t="inlineStr">
-        <is>
-          <t>Tipo de vidrio y tipo de proteccion: desplegables; sus valores estan en la hoja Datos_higro.</t>
+      <c r="A39" s="39" t="inlineStr">
+        <is>
+          <t>COMO SE COMPLETA</t>
         </is>
       </c>
       <c r="B39" s="2" t="n"/>
@@ -8841,7 +8912,7 @@
     <row r="40">
       <c r="A40" s="40" t="inlineStr">
         <is>
-          <t>Transmitancia del cerramiento: cargarla segun el vidrio y el marco adoptados.</t>
+          <t>Descripcion, altura y ancho del vano: de la planilla de carpinterias.</t>
         </is>
       </c>
       <c r="B40" s="2" t="n"/>
@@ -8860,7 +8931,7 @@
     <row r="41">
       <c r="A41" s="40" t="inlineStr">
         <is>
-          <t>Orientacion y factor de exposicion solar: el factor depende de la orientacion y de la proteccion.</t>
+          <t>Area del vano, area total por plano y porcentaje: se calculan solos.</t>
         </is>
       </c>
       <c r="B41" s="2" t="n"/>
@@ -8877,7 +8948,11 @@
       <c r="M41" s="2" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="40" t="inlineStr"/>
+      <c r="A42" s="40" t="inlineStr">
+        <is>
+          <t>Tipo de vidrio y tipo de proteccion: desplegables; sus valores estan en la hoja Datos_higro.</t>
+        </is>
+      </c>
       <c r="B42" s="2" t="n"/>
       <c r="C42" s="2" t="n"/>
       <c r="D42" s="2" t="n"/>
@@ -8894,7 +8969,7 @@
     <row r="43">
       <c r="A43" s="40" t="inlineStr">
         <is>
-          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
+          <t>Transmitancia del cerramiento: cargarla segun el vidrio y el marco adoptados.</t>
         </is>
       </c>
       <c r="B43" s="2" t="n"/>
@@ -8913,7 +8988,7 @@
     <row r="44">
       <c r="A44" s="40" t="inlineStr">
         <is>
-          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
+          <t>Orientacion y factor de exposicion solar: el factor depende de la orientacion y de la proteccion.</t>
         </is>
       </c>
       <c r="B44" s="2" t="n"/>
@@ -8947,7 +9022,7 @@
     <row r="46">
       <c r="A46" s="40" t="inlineStr">
         <is>
-          <t>FALTA, y esta marcado en naranja: la ALTURA de cada vano. La planilla de carpinterias acota</t>
+          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
         </is>
       </c>
       <c r="B46" s="2" t="n"/>
@@ -8966,7 +9041,7 @@
     <row r="47">
       <c r="A47" s="40" t="inlineStr">
         <is>
-          <t>el nivel de dintel (2,52 / 2,15 / 2,10) y el cielorraso (3,00), pero no la altura libre del vano,</t>
+          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
         </is>
       </c>
       <c r="B47" s="2" t="n"/>
@@ -8983,11 +9058,7 @@
       <c r="M47" s="2" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="40" t="inlineStr">
-        <is>
-          <t>asi que no se puede deducir sin el nivel de antepecho de cada abertura.</t>
-        </is>
-      </c>
+      <c r="A48" s="40" t="inlineStr"/>
       <c r="B48" s="2" t="n"/>
       <c r="C48" s="2" t="n"/>
       <c r="D48" s="2" t="n"/>
@@ -9002,7 +9073,11 @@
       <c r="M48" s="2" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="40" t="inlineStr"/>
+      <c r="A49" s="40" t="inlineStr">
+        <is>
+          <t>FALTA, y esta marcado en naranja: la ALTURA de cada vano. La planilla de carpinterias acota</t>
+        </is>
+      </c>
       <c r="B49" s="2" t="n"/>
       <c r="C49" s="2" t="n"/>
       <c r="D49" s="2" t="n"/>
@@ -9019,7 +9094,7 @@
     <row r="50">
       <c r="A50" s="40" t="inlineStr">
         <is>
-          <t>FALTA tambien la ORIENTACION de cada plano: no hay flecha de norte en la documentacion.</t>
+          <t>el nivel de dintel (2,52 / 2,15 / 2,10) y el cielorraso (3,00), pero no la altura libre del vano,</t>
         </is>
       </c>
       <c r="B50" s="2" t="n"/>
@@ -9038,7 +9113,7 @@
     <row r="51">
       <c r="A51" s="40" t="inlineStr">
         <is>
-          <t>El plano rotula Dormitorio Norte y Dormitorio Sur, pero eso no alcanza para fijar las cuatro vistas.</t>
+          <t>asi que no se puede deducir sin el nivel de antepecho de cada abertura.</t>
         </is>
       </c>
       <c r="B51" s="2" t="n"/>
@@ -9055,11 +9130,7 @@
       <c r="M51" s="2" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="40" t="inlineStr">
-        <is>
-          <t>El agrupamiento por vista que se uso aca es PROVISORIO: se armo por el espacio exterior al que</t>
-        </is>
-      </c>
+      <c r="A52" s="40" t="inlineStr"/>
       <c r="B52" s="2" t="n"/>
       <c r="C52" s="2" t="n"/>
       <c r="D52" s="2" t="n"/>
@@ -9076,7 +9147,7 @@
     <row r="53">
       <c r="A53" s="40" t="inlineStr">
         <is>
-          <t>da cada abertura (Patio / Patio interno). Mover las filas de bloque si corresponde.</t>
+          <t>ORIENTACION: el simbolo de norte del plano de plantas (flecha con arco, arriba a la derecha)</t>
         </is>
       </c>
       <c r="B53" s="2" t="n"/>
@@ -9093,7 +9164,11 @@
       <c r="M53" s="2" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="40" t="inlineStr"/>
+      <c r="A54" s="40" t="inlineStr">
+        <is>
+          <t>apunta hacia la derecha de la hoja. Entonces: derecha = Norte, izquierda = Sur, abajo = Este,</t>
+        </is>
+      </c>
       <c r="B54" s="2" t="n"/>
       <c r="C54" s="2" t="n"/>
       <c r="D54" s="2" t="n"/>
@@ -9110,7 +9185,7 @@
     <row r="55">
       <c r="A55" s="40" t="inlineStr">
         <is>
-          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
+          <t>arriba = Oeste. Coincide con los rotulos Dormitorio Norte y Dormitorio Sur del plano.</t>
         </is>
       </c>
       <c r="B55" s="2" t="n"/>
@@ -9127,7 +9202,11 @@
       <c r="M55" s="2" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="40" t="inlineStr"/>
+      <c r="A56" s="40" t="inlineStr">
+        <is>
+          <t>Cada abertura se asigno a la fachada por su posicion en planta.</t>
+        </is>
+      </c>
       <c r="B56" s="2" t="n"/>
       <c r="C56" s="2" t="n"/>
       <c r="D56" s="2" t="n"/>
@@ -9144,7 +9223,7 @@
     <row r="57">
       <c r="A57" s="40" t="inlineStr">
         <is>
-          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
+          <t>Las tres aberturas que dan al patio interno quedan en un bloque aparte: hay que confirmar</t>
         </is>
       </c>
       <c r="B57" s="2" t="n"/>
@@ -9163,7 +9242,7 @@
     <row r="58">
       <c r="A58" s="40" t="inlineStr">
         <is>
-          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
+          <t>a que lado del patio dan antes de asignarles orientacion y factor de exposicion solar.</t>
         </is>
       </c>
       <c r="B58" s="2" t="n"/>
@@ -9180,11 +9259,7 @@
       <c r="M58" s="2" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="40" t="inlineStr">
-        <is>
-          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
-        </is>
-      </c>
+      <c r="A59" s="40" t="inlineStr"/>
       <c r="B59" s="2" t="n"/>
       <c r="C59" s="2" t="n"/>
       <c r="D59" s="2" t="n"/>
@@ -9198,22 +9273,115 @@
       <c r="L59" s="2" t="n"/>
       <c r="M59" s="2" t="n"/>
     </row>
+    <row r="60">
+      <c r="A60" s="40" t="inlineStr">
+        <is>
+          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="n"/>
+      <c r="C60" s="2" t="n"/>
+      <c r="D60" s="2" t="n"/>
+      <c r="E60" s="2" t="n"/>
+      <c r="F60" s="2" t="n"/>
+      <c r="G60" s="2" t="n"/>
+      <c r="H60" s="2" t="n"/>
+      <c r="I60" s="2" t="n"/>
+      <c r="J60" s="2" t="n"/>
+      <c r="K60" s="2" t="n"/>
+      <c r="L60" s="2" t="n"/>
+      <c r="M60" s="2" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="40" t="inlineStr"/>
+      <c r="B61" s="2" t="n"/>
+      <c r="C61" s="2" t="n"/>
+      <c r="D61" s="2" t="n"/>
+      <c r="E61" s="2" t="n"/>
+      <c r="F61" s="2" t="n"/>
+      <c r="G61" s="2" t="n"/>
+      <c r="H61" s="2" t="n"/>
+      <c r="I61" s="2" t="n"/>
+      <c r="J61" s="2" t="n"/>
+      <c r="K61" s="2" t="n"/>
+      <c r="L61" s="2" t="n"/>
+      <c r="M61" s="2" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="40" t="inlineStr">
+        <is>
+          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="n"/>
+      <c r="C62" s="2" t="n"/>
+      <c r="D62" s="2" t="n"/>
+      <c r="E62" s="2" t="n"/>
+      <c r="F62" s="2" t="n"/>
+      <c r="G62" s="2" t="n"/>
+      <c r="H62" s="2" t="n"/>
+      <c r="I62" s="2" t="n"/>
+      <c r="J62" s="2" t="n"/>
+      <c r="K62" s="2" t="n"/>
+      <c r="L62" s="2" t="n"/>
+      <c r="M62" s="2" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="40" t="inlineStr">
+        <is>
+          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="n"/>
+      <c r="C63" s="2" t="n"/>
+      <c r="D63" s="2" t="n"/>
+      <c r="E63" s="2" t="n"/>
+      <c r="F63" s="2" t="n"/>
+      <c r="G63" s="2" t="n"/>
+      <c r="H63" s="2" t="n"/>
+      <c r="I63" s="2" t="n"/>
+      <c r="J63" s="2" t="n"/>
+      <c r="K63" s="2" t="n"/>
+      <c r="L63" s="2" t="n"/>
+      <c r="M63" s="2" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="40" t="inlineStr">
+        <is>
+          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="n"/>
+      <c r="C64" s="2" t="n"/>
+      <c r="D64" s="2" t="n"/>
+      <c r="E64" s="2" t="n"/>
+      <c r="F64" s="2" t="n"/>
+      <c r="G64" s="2" t="n"/>
+      <c r="H64" s="2" t="n"/>
+      <c r="I64" s="2" t="n"/>
+      <c r="J64" s="2" t="n"/>
+      <c r="K64" s="2" t="n"/>
+      <c r="L64" s="2" t="n"/>
+      <c r="M64" s="2" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="A14:M14"/>
+  <mergeCells count="14">
+    <mergeCell ref="E13:E15"/>
+    <mergeCell ref="E32:E37"/>
     <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A27:M27"/>
-    <mergeCell ref="E15:E19"/>
+    <mergeCell ref="E17:E22"/>
+    <mergeCell ref="E7:E11"/>
+    <mergeCell ref="A23:M23"/>
+    <mergeCell ref="A31:M31"/>
     <mergeCell ref="A6:M6"/>
-    <mergeCell ref="E21:E26"/>
-    <mergeCell ref="E28:E34"/>
+    <mergeCell ref="A12:M12"/>
     <mergeCell ref="A4:M4"/>
     <mergeCell ref="A3:M3"/>
-    <mergeCell ref="E7:E13"/>
-    <mergeCell ref="A20:M20"/>
+    <mergeCell ref="E24:E30"/>
+    <mergeCell ref="A16:M16"/>
     <mergeCell ref="A2:M2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M6:M34">
+  <conditionalFormatting sqref="M6:M37">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
       <formula>"CUMPLE"</formula>
     </cfRule>
@@ -9222,13 +9390,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="H6:H34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Datos_higro!$A$8:$A$15</formula1>
     </dataValidation>
-    <dataValidation sqref="I6:I34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I6:I37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Datos_higro!$A$19:$A$25</formula1>
     </dataValidation>
-    <dataValidation sqref="K6:K34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K6:K37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Norte,Sur,Este,Oeste,Noreste,Noroeste,Sudeste,Sudoeste,Horizontal"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Planilla 3: cargar las alturas de vano medidas del dibujo
Las alturas se miden sobre las vistas de la planilla de carpinterias.
La escala se calibra con los anchos acotados de cada ficha y cierra con
error menor a 2 cm, asi que la medicion del alto es confiable.

La mayoria de las aberturas son de piso a cielorraso (3,00 m); VA02 2,15
y VA03 / VA04 / VA05 / PF05 2,52. Quedan sin medir PF04, PV01 y PV04 (2).

Control: el area vidriada cargada da 70,9 m2 sin esas tres. Sumando PV01
(7,70 x 3,00 = 23,1 m2) da del orden de 94 m2, contra los 97,4 m2 de
superficie vidriada que suma la planilla de iluminacion y ventilacion.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -331,9 +331,6 @@
     <xf numFmtId="0" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="2" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -364,6 +361,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -7619,7 +7619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M64"/>
+  <dimension ref="A1:M65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7805,23 +7805,25 @@
           <t>PV02</t>
         </is>
       </c>
-      <c r="B7" s="26" t="n"/>
-      <c r="C7" s="27" t="n">
+      <c r="B7" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="26" t="n">
         <v>2.48</v>
       </c>
-      <c r="D7" s="28">
+      <c r="D7" s="27">
         <f>IF(COUNT(B7,C7)&lt;2,"",B7*C7)</f>
         <v/>
       </c>
-      <c r="E7" s="29">
+      <c r="E7" s="28">
         <f>SUM(D7:D11)</f>
         <v/>
       </c>
-      <c r="F7" s="30">
+      <c r="F7" s="29">
         <f>IF(OR(D7="",$E$7=""),"",D7/$E$7)</f>
         <v/>
       </c>
-      <c r="G7" s="28">
+      <c r="G7" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
@@ -7831,7 +7833,7 @@
         </is>
       </c>
       <c r="I7" s="25" t="n"/>
-      <c r="J7" s="27" t="n">
+      <c r="J7" s="26" t="n">
         <v>2.8</v>
       </c>
       <c r="K7" s="25" t="inlineStr">
@@ -7839,8 +7841,8 @@
           <t>Norte</t>
         </is>
       </c>
-      <c r="L7" s="27" t="n"/>
-      <c r="M7" s="31">
+      <c r="L7" s="26" t="n"/>
+      <c r="M7" s="30">
         <f>IF(OR(D7="",J7=""),"",IF(J7&lt;=G7,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
@@ -7851,20 +7853,22 @@
           <t>PF03</t>
         </is>
       </c>
-      <c r="B8" s="26" t="n"/>
-      <c r="C8" s="27" t="n">
+      <c r="B8" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="26" t="n">
         <v>2.88</v>
       </c>
-      <c r="D8" s="28">
+      <c r="D8" s="27">
         <f>IF(COUNT(B8,C8)&lt;2,"",B8*C8)</f>
         <v/>
       </c>
-      <c r="E8" s="32" t="n"/>
-      <c r="F8" s="30">
+      <c r="E8" s="31" t="n"/>
+      <c r="F8" s="29">
         <f>IF(OR(D8="",$E$7=""),"",D8/$E$7)</f>
         <v/>
       </c>
-      <c r="G8" s="28">
+      <c r="G8" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
@@ -7874,7 +7878,7 @@
         </is>
       </c>
       <c r="I8" s="25" t="n"/>
-      <c r="J8" s="27" t="n">
+      <c r="J8" s="26" t="n">
         <v>2.8</v>
       </c>
       <c r="K8" s="25" t="inlineStr">
@@ -7882,8 +7886,8 @@
           <t>Norte</t>
         </is>
       </c>
-      <c r="L8" s="27" t="n"/>
-      <c r="M8" s="31">
+      <c r="L8" s="26" t="n"/>
+      <c r="M8" s="30">
         <f>IF(OR(D8="",J8=""),"",IF(J8&lt;=G8,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
@@ -7894,20 +7898,22 @@
           <t>VA04</t>
         </is>
       </c>
-      <c r="B9" s="26" t="n"/>
-      <c r="C9" s="27" t="n">
+      <c r="B9" s="26" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="C9" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="D9" s="28">
+      <c r="D9" s="27">
         <f>IF(COUNT(B9,C9)&lt;2,"",B9*C9)</f>
         <v/>
       </c>
-      <c r="E9" s="32" t="n"/>
-      <c r="F9" s="30">
+      <c r="E9" s="31" t="n"/>
+      <c r="F9" s="29">
         <f>IF(OR(D9="",$E$7=""),"",D9/$E$7)</f>
         <v/>
       </c>
-      <c r="G9" s="28">
+      <c r="G9" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
@@ -7917,7 +7923,7 @@
         </is>
       </c>
       <c r="I9" s="25" t="n"/>
-      <c r="J9" s="27" t="n">
+      <c r="J9" s="26" t="n">
         <v>2.8</v>
       </c>
       <c r="K9" s="25" t="inlineStr">
@@ -7925,62 +7931,62 @@
           <t>Norte</t>
         </is>
       </c>
-      <c r="L9" s="27" t="n"/>
-      <c r="M9" s="31">
+      <c r="L9" s="26" t="n"/>
+      <c r="M9" s="30">
         <f>IF(OR(D9="",J9=""),"",IF(J9&lt;=G9,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="17" customHeight="1">
       <c r="A10" s="25" t="n"/>
-      <c r="B10" s="27" t="n"/>
-      <c r="C10" s="27" t="n"/>
-      <c r="D10" s="28">
+      <c r="B10" s="26" t="n"/>
+      <c r="C10" s="26" t="n"/>
+      <c r="D10" s="27">
         <f>IF(COUNT(B10,C10)&lt;2,"",B10*C10)</f>
         <v/>
       </c>
-      <c r="E10" s="32" t="n"/>
-      <c r="F10" s="30">
+      <c r="E10" s="31" t="n"/>
+      <c r="F10" s="29">
         <f>IF(OR(D10="",$E$7=""),"",D10/$E$7)</f>
         <v/>
       </c>
-      <c r="G10" s="28">
+      <c r="G10" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
       <c r="H10" s="25" t="n"/>
       <c r="I10" s="25" t="n"/>
-      <c r="J10" s="27" t="n"/>
+      <c r="J10" s="26" t="n"/>
       <c r="K10" s="25" t="n"/>
-      <c r="L10" s="27" t="n"/>
-      <c r="M10" s="31">
+      <c r="L10" s="26" t="n"/>
+      <c r="M10" s="30">
         <f>IF(OR(D10="",J10=""),"",IF(J10&lt;=G10,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="17" customHeight="1">
-      <c r="A11" s="33" t="n"/>
-      <c r="B11" s="34" t="n"/>
-      <c r="C11" s="34" t="n"/>
-      <c r="D11" s="35">
+      <c r="A11" s="32" t="n"/>
+      <c r="B11" s="33" t="n"/>
+      <c r="C11" s="33" t="n"/>
+      <c r="D11" s="34">
         <f>IF(COUNT(B11,C11)&lt;2,"",B11*C11)</f>
         <v/>
       </c>
-      <c r="E11" s="36" t="n"/>
-      <c r="F11" s="37">
+      <c r="E11" s="35" t="n"/>
+      <c r="F11" s="36">
         <f>IF(OR(D11="",$E$7=""),"",D11/$E$7)</f>
         <v/>
       </c>
-      <c r="G11" s="35">
+      <c r="G11" s="34">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H11" s="33" t="n"/>
-      <c r="I11" s="33" t="n"/>
-      <c r="J11" s="34" t="n"/>
-      <c r="K11" s="33" t="n"/>
-      <c r="L11" s="34" t="n"/>
-      <c r="M11" s="38">
+      <c r="H11" s="32" t="n"/>
+      <c r="I11" s="32" t="n"/>
+      <c r="J11" s="33" t="n"/>
+      <c r="K11" s="32" t="n"/>
+      <c r="L11" s="33" t="n"/>
+      <c r="M11" s="37">
         <f>IF(OR(D11="",J11=""),"",IF(J11&lt;=G11,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
@@ -8010,23 +8016,25 @@
           <t>VA01</t>
         </is>
       </c>
-      <c r="B13" s="26" t="n"/>
-      <c r="C13" s="27" t="n">
+      <c r="B13" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" s="26" t="n">
         <v>0.75</v>
       </c>
-      <c r="D13" s="28">
+      <c r="D13" s="27">
         <f>IF(COUNT(B13,C13)&lt;2,"",B13*C13)</f>
         <v/>
       </c>
-      <c r="E13" s="29">
+      <c r="E13" s="28">
         <f>SUM(D13:D15)</f>
         <v/>
       </c>
-      <c r="F13" s="30">
+      <c r="F13" s="29">
         <f>IF(OR(D13="",$E$13=""),"",D13/$E$13)</f>
         <v/>
       </c>
-      <c r="G13" s="28">
+      <c r="G13" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
@@ -8036,7 +8044,7 @@
         </is>
       </c>
       <c r="I13" s="25" t="n"/>
-      <c r="J13" s="27" t="n">
+      <c r="J13" s="26" t="n">
         <v>2.8</v>
       </c>
       <c r="K13" s="25" t="inlineStr">
@@ -8044,62 +8052,62 @@
           <t>Sur</t>
         </is>
       </c>
-      <c r="L13" s="27" t="n"/>
-      <c r="M13" s="31">
+      <c r="L13" s="26" t="n"/>
+      <c r="M13" s="30">
         <f>IF(OR(D13="",J13=""),"",IF(J13&lt;=G13,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
       <c r="A14" s="25" t="n"/>
-      <c r="B14" s="27" t="n"/>
-      <c r="C14" s="27" t="n"/>
-      <c r="D14" s="28">
+      <c r="B14" s="26" t="n"/>
+      <c r="C14" s="26" t="n"/>
+      <c r="D14" s="27">
         <f>IF(COUNT(B14,C14)&lt;2,"",B14*C14)</f>
         <v/>
       </c>
-      <c r="E14" s="32" t="n"/>
-      <c r="F14" s="30">
+      <c r="E14" s="31" t="n"/>
+      <c r="F14" s="29">
         <f>IF(OR(D14="",$E$13=""),"",D14/$E$13)</f>
         <v/>
       </c>
-      <c r="G14" s="28">
+      <c r="G14" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
       <c r="H14" s="25" t="n"/>
       <c r="I14" s="25" t="n"/>
-      <c r="J14" s="27" t="n"/>
+      <c r="J14" s="26" t="n"/>
       <c r="K14" s="25" t="n"/>
-      <c r="L14" s="27" t="n"/>
-      <c r="M14" s="31">
+      <c r="L14" s="26" t="n"/>
+      <c r="M14" s="30">
         <f>IF(OR(D14="",J14=""),"",IF(J14&lt;=G14,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="33" t="n"/>
-      <c r="B15" s="34" t="n"/>
-      <c r="C15" s="34" t="n"/>
-      <c r="D15" s="35">
+      <c r="A15" s="32" t="n"/>
+      <c r="B15" s="33" t="n"/>
+      <c r="C15" s="33" t="n"/>
+      <c r="D15" s="34">
         <f>IF(COUNT(B15,C15)&lt;2,"",B15*C15)</f>
         <v/>
       </c>
-      <c r="E15" s="36" t="n"/>
-      <c r="F15" s="37">
+      <c r="E15" s="35" t="n"/>
+      <c r="F15" s="36">
         <f>IF(OR(D15="",$E$13=""),"",D15/$E$13)</f>
         <v/>
       </c>
-      <c r="G15" s="35">
+      <c r="G15" s="34">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H15" s="33" t="n"/>
-      <c r="I15" s="33" t="n"/>
-      <c r="J15" s="34" t="n"/>
-      <c r="K15" s="33" t="n"/>
-      <c r="L15" s="34" t="n"/>
-      <c r="M15" s="38">
+      <c r="H15" s="32" t="n"/>
+      <c r="I15" s="32" t="n"/>
+      <c r="J15" s="33" t="n"/>
+      <c r="K15" s="32" t="n"/>
+      <c r="L15" s="33" t="n"/>
+      <c r="M15" s="37">
         <f>IF(OR(D15="",J15=""),"",IF(J15&lt;=G15,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
@@ -8129,23 +8137,25 @@
           <t>PA01</t>
         </is>
       </c>
-      <c r="B17" s="26" t="n"/>
-      <c r="C17" s="27" t="n">
+      <c r="B17" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="28">
+      <c r="D17" s="27">
         <f>IF(COUNT(B17,C17)&lt;2,"",B17*C17)</f>
         <v/>
       </c>
-      <c r="E17" s="29">
+      <c r="E17" s="28">
         <f>SUM(D17:D22)</f>
         <v/>
       </c>
-      <c r="F17" s="30">
+      <c r="F17" s="29">
         <f>IF(OR(D17="",$E$17=""),"",D17/$E$17)</f>
         <v/>
       </c>
-      <c r="G17" s="28">
+      <c r="G17" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
@@ -8155,7 +8165,7 @@
         </is>
       </c>
       <c r="I17" s="25" t="n"/>
-      <c r="J17" s="27" t="n">
+      <c r="J17" s="26" t="n">
         <v>2.8</v>
       </c>
       <c r="K17" s="25" t="inlineStr">
@@ -8163,8 +8173,8 @@
           <t>Este</t>
         </is>
       </c>
-      <c r="L17" s="27" t="n"/>
-      <c r="M17" s="31">
+      <c r="L17" s="26" t="n"/>
+      <c r="M17" s="30">
         <f>IF(OR(D17="",J17=""),"",IF(J17&lt;=G17,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
@@ -8175,20 +8185,20 @@
           <t>PF04</t>
         </is>
       </c>
-      <c r="B18" s="26" t="n"/>
-      <c r="C18" s="27" t="n">
+      <c r="B18" s="38" t="n"/>
+      <c r="C18" s="26" t="n">
         <v>2.7</v>
       </c>
-      <c r="D18" s="28">
+      <c r="D18" s="27">
         <f>IF(COUNT(B18,C18)&lt;2,"",B18*C18)</f>
         <v/>
       </c>
-      <c r="E18" s="32" t="n"/>
-      <c r="F18" s="30">
+      <c r="E18" s="31" t="n"/>
+      <c r="F18" s="29">
         <f>IF(OR(D18="",$E$17=""),"",D18/$E$17)</f>
         <v/>
       </c>
-      <c r="G18" s="28">
+      <c r="G18" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
@@ -8198,7 +8208,7 @@
         </is>
       </c>
       <c r="I18" s="25" t="n"/>
-      <c r="J18" s="27" t="n">
+      <c r="J18" s="26" t="n">
         <v>2.8</v>
       </c>
       <c r="K18" s="25" t="inlineStr">
@@ -8206,8 +8216,8 @@
           <t>Este</t>
         </is>
       </c>
-      <c r="L18" s="27" t="n"/>
-      <c r="M18" s="31">
+      <c r="L18" s="26" t="n"/>
+      <c r="M18" s="30">
         <f>IF(OR(D18="",J18=""),"",IF(J18&lt;=G18,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
@@ -8218,20 +8228,22 @@
           <t>VA05</t>
         </is>
       </c>
-      <c r="B19" s="26" t="n"/>
-      <c r="C19" s="27" t="n">
+      <c r="B19" s="26" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="C19" s="26" t="n">
         <v>1.4</v>
       </c>
-      <c r="D19" s="28">
+      <c r="D19" s="27">
         <f>IF(COUNT(B19,C19)&lt;2,"",B19*C19)</f>
         <v/>
       </c>
-      <c r="E19" s="32" t="n"/>
-      <c r="F19" s="30">
+      <c r="E19" s="31" t="n"/>
+      <c r="F19" s="29">
         <f>IF(OR(D19="",$E$17=""),"",D19/$E$17)</f>
         <v/>
       </c>
-      <c r="G19" s="28">
+      <c r="G19" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
@@ -8241,7 +8253,7 @@
         </is>
       </c>
       <c r="I19" s="25" t="n"/>
-      <c r="J19" s="27" t="n">
+      <c r="J19" s="26" t="n">
         <v>2.8</v>
       </c>
       <c r="K19" s="25" t="inlineStr">
@@ -8249,8 +8261,8 @@
           <t>Este</t>
         </is>
       </c>
-      <c r="L19" s="27" t="n"/>
-      <c r="M19" s="31">
+      <c r="L19" s="26" t="n"/>
+      <c r="M19" s="30">
         <f>IF(OR(D19="",J19=""),"",IF(J19&lt;=G19,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
@@ -8261,20 +8273,22 @@
           <t>PV04</t>
         </is>
       </c>
-      <c r="B20" s="26" t="n"/>
-      <c r="C20" s="27" t="n">
+      <c r="B20" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" s="26" t="n">
         <v>2.06</v>
       </c>
-      <c r="D20" s="28">
+      <c r="D20" s="27">
         <f>IF(COUNT(B20,C20)&lt;2,"",B20*C20)</f>
         <v/>
       </c>
-      <c r="E20" s="32" t="n"/>
-      <c r="F20" s="30">
+      <c r="E20" s="31" t="n"/>
+      <c r="F20" s="29">
         <f>IF(OR(D20="",$E$17=""),"",D20/$E$17)</f>
         <v/>
       </c>
-      <c r="G20" s="28">
+      <c r="G20" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
@@ -8284,7 +8298,7 @@
         </is>
       </c>
       <c r="I20" s="25" t="n"/>
-      <c r="J20" s="27" t="n">
+      <c r="J20" s="26" t="n">
         <v>2.8</v>
       </c>
       <c r="K20" s="25" t="inlineStr">
@@ -8292,62 +8306,62 @@
           <t>Este</t>
         </is>
       </c>
-      <c r="L20" s="27" t="n"/>
-      <c r="M20" s="31">
+      <c r="L20" s="26" t="n"/>
+      <c r="M20" s="30">
         <f>IF(OR(D20="",J20=""),"",IF(J20&lt;=G20,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="17" customHeight="1">
       <c r="A21" s="25" t="n"/>
-      <c r="B21" s="27" t="n"/>
-      <c r="C21" s="27" t="n"/>
-      <c r="D21" s="28">
+      <c r="B21" s="26" t="n"/>
+      <c r="C21" s="26" t="n"/>
+      <c r="D21" s="27">
         <f>IF(COUNT(B21,C21)&lt;2,"",B21*C21)</f>
         <v/>
       </c>
-      <c r="E21" s="32" t="n"/>
-      <c r="F21" s="30">
+      <c r="E21" s="31" t="n"/>
+      <c r="F21" s="29">
         <f>IF(OR(D21="",$E$17=""),"",D21/$E$17)</f>
         <v/>
       </c>
-      <c r="G21" s="28">
+      <c r="G21" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
       <c r="H21" s="25" t="n"/>
       <c r="I21" s="25" t="n"/>
-      <c r="J21" s="27" t="n"/>
+      <c r="J21" s="26" t="n"/>
       <c r="K21" s="25" t="n"/>
-      <c r="L21" s="27" t="n"/>
-      <c r="M21" s="31">
+      <c r="L21" s="26" t="n"/>
+      <c r="M21" s="30">
         <f>IF(OR(D21="",J21=""),"",IF(J21&lt;=G21,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="17" customHeight="1">
-      <c r="A22" s="33" t="n"/>
-      <c r="B22" s="34" t="n"/>
-      <c r="C22" s="34" t="n"/>
-      <c r="D22" s="35">
+      <c r="A22" s="32" t="n"/>
+      <c r="B22" s="33" t="n"/>
+      <c r="C22" s="33" t="n"/>
+      <c r="D22" s="34">
         <f>IF(COUNT(B22,C22)&lt;2,"",B22*C22)</f>
         <v/>
       </c>
-      <c r="E22" s="36" t="n"/>
-      <c r="F22" s="37">
+      <c r="E22" s="35" t="n"/>
+      <c r="F22" s="36">
         <f>IF(OR(D22="",$E$17=""),"",D22/$E$17)</f>
         <v/>
       </c>
-      <c r="G22" s="35">
+      <c r="G22" s="34">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H22" s="33" t="n"/>
-      <c r="I22" s="33" t="n"/>
-      <c r="J22" s="34" t="n"/>
-      <c r="K22" s="33" t="n"/>
-      <c r="L22" s="34" t="n"/>
-      <c r="M22" s="38">
+      <c r="H22" s="32" t="n"/>
+      <c r="I22" s="32" t="n"/>
+      <c r="J22" s="33" t="n"/>
+      <c r="K22" s="32" t="n"/>
+      <c r="L22" s="33" t="n"/>
+      <c r="M22" s="37">
         <f>IF(OR(D22="",J22=""),"",IF(J22&lt;=G22,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
@@ -8377,23 +8391,25 @@
           <t>PV03</t>
         </is>
       </c>
-      <c r="B24" s="26" t="n"/>
-      <c r="C24" s="27" t="n">
+      <c r="B24" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" s="26" t="n">
         <v>1.76</v>
       </c>
-      <c r="D24" s="28">
+      <c r="D24" s="27">
         <f>IF(COUNT(B24,C24)&lt;2,"",B24*C24)</f>
         <v/>
       </c>
-      <c r="E24" s="29">
+      <c r="E24" s="28">
         <f>SUM(D24:D30)</f>
         <v/>
       </c>
-      <c r="F24" s="30">
+      <c r="F24" s="29">
         <f>IF(OR(D24="",$E$24=""),"",D24/$E$24)</f>
         <v/>
       </c>
-      <c r="G24" s="28">
+      <c r="G24" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
@@ -8403,7 +8419,7 @@
         </is>
       </c>
       <c r="I24" s="25" t="n"/>
-      <c r="J24" s="27" t="n">
+      <c r="J24" s="26" t="n">
         <v>2.8</v>
       </c>
       <c r="K24" s="25" t="inlineStr">
@@ -8411,8 +8427,8 @@
           <t>Oeste</t>
         </is>
       </c>
-      <c r="L24" s="27" t="n"/>
-      <c r="M24" s="31">
+      <c r="L24" s="26" t="n"/>
+      <c r="M24" s="30">
         <f>IF(OR(D24="",J24=""),"",IF(J24&lt;=G24,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
@@ -8423,20 +8439,22 @@
           <t>VA02</t>
         </is>
       </c>
-      <c r="B25" s="26" t="n"/>
-      <c r="C25" s="27" t="n">
+      <c r="B25" s="26" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="C25" s="26" t="n">
         <v>0.75</v>
       </c>
-      <c r="D25" s="28">
+      <c r="D25" s="27">
         <f>IF(COUNT(B25,C25)&lt;2,"",B25*C25)</f>
         <v/>
       </c>
-      <c r="E25" s="32" t="n"/>
-      <c r="F25" s="30">
+      <c r="E25" s="31" t="n"/>
+      <c r="F25" s="29">
         <f>IF(OR(D25="",$E$24=""),"",D25/$E$24)</f>
         <v/>
       </c>
-      <c r="G25" s="28">
+      <c r="G25" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
@@ -8446,7 +8464,7 @@
         </is>
       </c>
       <c r="I25" s="25" t="n"/>
-      <c r="J25" s="27" t="n">
+      <c r="J25" s="26" t="n">
         <v>2.8</v>
       </c>
       <c r="K25" s="25" t="inlineStr">
@@ -8454,8 +8472,8 @@
           <t>Oeste</t>
         </is>
       </c>
-      <c r="L25" s="27" t="n"/>
-      <c r="M25" s="31">
+      <c r="L25" s="26" t="n"/>
+      <c r="M25" s="30">
         <f>IF(OR(D25="",J25=""),"",IF(J25&lt;=G25,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
@@ -8466,20 +8484,22 @@
           <t>PA02</t>
         </is>
       </c>
-      <c r="B26" s="26" t="n"/>
-      <c r="C26" s="27" t="n">
+      <c r="B26" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C26" s="26" t="n">
         <v>0.75</v>
       </c>
-      <c r="D26" s="28">
+      <c r="D26" s="27">
         <f>IF(COUNT(B26,C26)&lt;2,"",B26*C26)</f>
         <v/>
       </c>
-      <c r="E26" s="32" t="n"/>
-      <c r="F26" s="30">
+      <c r="E26" s="31" t="n"/>
+      <c r="F26" s="29">
         <f>IF(OR(D26="",$E$24=""),"",D26/$E$24)</f>
         <v/>
       </c>
-      <c r="G26" s="28">
+      <c r="G26" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
@@ -8489,7 +8509,7 @@
         </is>
       </c>
       <c r="I26" s="25" t="n"/>
-      <c r="J26" s="27" t="n">
+      <c r="J26" s="26" t="n">
         <v>2.8</v>
       </c>
       <c r="K26" s="25" t="inlineStr">
@@ -8497,8 +8517,8 @@
           <t>Oeste</t>
         </is>
       </c>
-      <c r="L26" s="27" t="n"/>
-      <c r="M26" s="31">
+      <c r="L26" s="26" t="n"/>
+      <c r="M26" s="30">
         <f>IF(OR(D26="",J26=""),"",IF(J26&lt;=G26,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
@@ -8509,20 +8529,22 @@
           <t>VA03</t>
         </is>
       </c>
-      <c r="B27" s="26" t="n"/>
-      <c r="C27" s="27" t="n">
+      <c r="B27" s="26" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="C27" s="26" t="n">
         <v>0.75</v>
       </c>
-      <c r="D27" s="28">
+      <c r="D27" s="27">
         <f>IF(COUNT(B27,C27)&lt;2,"",B27*C27)</f>
         <v/>
       </c>
-      <c r="E27" s="32" t="n"/>
-      <c r="F27" s="30">
+      <c r="E27" s="31" t="n"/>
+      <c r="F27" s="29">
         <f>IF(OR(D27="",$E$24=""),"",D27/$E$24)</f>
         <v/>
       </c>
-      <c r="G27" s="28">
+      <c r="G27" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
@@ -8532,7 +8554,7 @@
         </is>
       </c>
       <c r="I27" s="25" t="n"/>
-      <c r="J27" s="27" t="n">
+      <c r="J27" s="26" t="n">
         <v>2.8</v>
       </c>
       <c r="K27" s="25" t="inlineStr">
@@ -8540,8 +8562,8 @@
           <t>Oeste</t>
         </is>
       </c>
-      <c r="L27" s="27" t="n"/>
-      <c r="M27" s="31">
+      <c r="L27" s="26" t="n"/>
+      <c r="M27" s="30">
         <f>IF(OR(D27="",J27=""),"",IF(J27&lt;=G27,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
@@ -8552,20 +8574,22 @@
           <t>PF05</t>
         </is>
       </c>
-      <c r="B28" s="26" t="n"/>
-      <c r="C28" s="27" t="n">
+      <c r="B28" s="26" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="C28" s="26" t="n">
         <v>0.75</v>
       </c>
-      <c r="D28" s="28">
+      <c r="D28" s="27">
         <f>IF(COUNT(B28,C28)&lt;2,"",B28*C28)</f>
         <v/>
       </c>
-      <c r="E28" s="32" t="n"/>
-      <c r="F28" s="30">
+      <c r="E28" s="31" t="n"/>
+      <c r="F28" s="29">
         <f>IF(OR(D28="",$E$24=""),"",D28/$E$24)</f>
         <v/>
       </c>
-      <c r="G28" s="28">
+      <c r="G28" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
@@ -8575,7 +8599,7 @@
         </is>
       </c>
       <c r="I28" s="25" t="n"/>
-      <c r="J28" s="27" t="n">
+      <c r="J28" s="26" t="n">
         <v>2.8</v>
       </c>
       <c r="K28" s="25" t="inlineStr">
@@ -8583,62 +8607,62 @@
           <t>Oeste</t>
         </is>
       </c>
-      <c r="L28" s="27" t="n"/>
-      <c r="M28" s="31">
+      <c r="L28" s="26" t="n"/>
+      <c r="M28" s="30">
         <f>IF(OR(D28="",J28=""),"",IF(J28&lt;=G28,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
     <row r="29" ht="17" customHeight="1">
       <c r="A29" s="25" t="n"/>
-      <c r="B29" s="27" t="n"/>
-      <c r="C29" s="27" t="n"/>
-      <c r="D29" s="28">
+      <c r="B29" s="26" t="n"/>
+      <c r="C29" s="26" t="n"/>
+      <c r="D29" s="27">
         <f>IF(COUNT(B29,C29)&lt;2,"",B29*C29)</f>
         <v/>
       </c>
-      <c r="E29" s="32" t="n"/>
-      <c r="F29" s="30">
+      <c r="E29" s="31" t="n"/>
+      <c r="F29" s="29">
         <f>IF(OR(D29="",$E$24=""),"",D29/$E$24)</f>
         <v/>
       </c>
-      <c r="G29" s="28">
+      <c r="G29" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
       <c r="H29" s="25" t="n"/>
       <c r="I29" s="25" t="n"/>
-      <c r="J29" s="27" t="n"/>
+      <c r="J29" s="26" t="n"/>
       <c r="K29" s="25" t="n"/>
-      <c r="L29" s="27" t="n"/>
-      <c r="M29" s="31">
+      <c r="L29" s="26" t="n"/>
+      <c r="M29" s="30">
         <f>IF(OR(D29="",J29=""),"",IF(J29&lt;=G29,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="17" customHeight="1">
-      <c r="A30" s="33" t="n"/>
-      <c r="B30" s="34" t="n"/>
-      <c r="C30" s="34" t="n"/>
-      <c r="D30" s="35">
+      <c r="A30" s="32" t="n"/>
+      <c r="B30" s="33" t="n"/>
+      <c r="C30" s="33" t="n"/>
+      <c r="D30" s="34">
         <f>IF(COUNT(B30,C30)&lt;2,"",B30*C30)</f>
         <v/>
       </c>
-      <c r="E30" s="36" t="n"/>
-      <c r="F30" s="37">
+      <c r="E30" s="35" t="n"/>
+      <c r="F30" s="36">
         <f>IF(OR(D30="",$E$24=""),"",D30/$E$24)</f>
         <v/>
       </c>
-      <c r="G30" s="35">
+      <c r="G30" s="34">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H30" s="33" t="n"/>
-      <c r="I30" s="33" t="n"/>
-      <c r="J30" s="34" t="n"/>
-      <c r="K30" s="33" t="n"/>
-      <c r="L30" s="34" t="n"/>
-      <c r="M30" s="38">
+      <c r="H30" s="32" t="n"/>
+      <c r="I30" s="32" t="n"/>
+      <c r="J30" s="33" t="n"/>
+      <c r="K30" s="32" t="n"/>
+      <c r="L30" s="33" t="n"/>
+      <c r="M30" s="37">
         <f>IF(OR(D30="",J30=""),"",IF(J30&lt;=G30,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
@@ -8668,23 +8692,25 @@
           <t>PF01</t>
         </is>
       </c>
-      <c r="B32" s="26" t="n"/>
-      <c r="C32" s="27" t="n">
+      <c r="B32" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C32" s="26" t="n">
         <v>3.55</v>
       </c>
-      <c r="D32" s="28">
+      <c r="D32" s="27">
         <f>IF(COUNT(B32,C32)&lt;2,"",B32*C32)</f>
         <v/>
       </c>
-      <c r="E32" s="29">
+      <c r="E32" s="28">
         <f>SUM(D32:D37)</f>
         <v/>
       </c>
-      <c r="F32" s="30">
+      <c r="F32" s="29">
         <f>IF(OR(D32="",$E$32=""),"",D32/$E$32)</f>
         <v/>
       </c>
-      <c r="G32" s="28">
+      <c r="G32" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
@@ -8694,12 +8720,12 @@
         </is>
       </c>
       <c r="I32" s="25" t="n"/>
-      <c r="J32" s="27" t="n">
+      <c r="J32" s="26" t="n">
         <v>2.8</v>
       </c>
       <c r="K32" s="25" t="n"/>
-      <c r="L32" s="27" t="n"/>
-      <c r="M32" s="31">
+      <c r="L32" s="26" t="n"/>
+      <c r="M32" s="30">
         <f>IF(OR(D32="",J32=""),"",IF(J32&lt;=G32,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
@@ -8710,20 +8736,22 @@
           <t>PF02</t>
         </is>
       </c>
-      <c r="B33" s="26" t="n"/>
-      <c r="C33" s="27" t="n">
+      <c r="B33" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C33" s="26" t="n">
         <v>3.75</v>
       </c>
-      <c r="D33" s="28">
+      <c r="D33" s="27">
         <f>IF(COUNT(B33,C33)&lt;2,"",B33*C33)</f>
         <v/>
       </c>
-      <c r="E33" s="32" t="n"/>
-      <c r="F33" s="30">
+      <c r="E33" s="31" t="n"/>
+      <c r="F33" s="29">
         <f>IF(OR(D33="",$E$32=""),"",D33/$E$32)</f>
         <v/>
       </c>
-      <c r="G33" s="28">
+      <c r="G33" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
@@ -8733,12 +8761,12 @@
         </is>
       </c>
       <c r="I33" s="25" t="n"/>
-      <c r="J33" s="27" t="n">
+      <c r="J33" s="26" t="n">
         <v>2.8</v>
       </c>
       <c r="K33" s="25" t="n"/>
-      <c r="L33" s="27" t="n"/>
-      <c r="M33" s="31">
+      <c r="L33" s="26" t="n"/>
+      <c r="M33" s="30">
         <f>IF(OR(D33="",J33=""),"",IF(J33&lt;=G33,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
@@ -8749,20 +8777,20 @@
           <t>PV01</t>
         </is>
       </c>
-      <c r="B34" s="26" t="n"/>
-      <c r="C34" s="27" t="n">
+      <c r="B34" s="38" t="n"/>
+      <c r="C34" s="26" t="n">
         <v>7.7</v>
       </c>
-      <c r="D34" s="28">
+      <c r="D34" s="27">
         <f>IF(COUNT(B34,C34)&lt;2,"",B34*C34)</f>
         <v/>
       </c>
-      <c r="E34" s="32" t="n"/>
-      <c r="F34" s="30">
+      <c r="E34" s="31" t="n"/>
+      <c r="F34" s="29">
         <f>IF(OR(D34="",$E$32=""),"",D34/$E$32)</f>
         <v/>
       </c>
-      <c r="G34" s="28">
+      <c r="G34" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
@@ -8772,12 +8800,12 @@
         </is>
       </c>
       <c r="I34" s="25" t="n"/>
-      <c r="J34" s="27" t="n">
+      <c r="J34" s="26" t="n">
         <v>2.8</v>
       </c>
       <c r="K34" s="25" t="n"/>
-      <c r="L34" s="27" t="n"/>
-      <c r="M34" s="31">
+      <c r="L34" s="26" t="n"/>
+      <c r="M34" s="30">
         <f>IF(OR(D34="",J34=""),"",IF(J34&lt;=G34,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
@@ -8788,20 +8816,20 @@
           <t>PV04 (2)</t>
         </is>
       </c>
-      <c r="B35" s="26" t="n"/>
-      <c r="C35" s="27" t="n">
+      <c r="B35" s="38" t="n"/>
+      <c r="C35" s="26" t="n">
         <v>1.5</v>
       </c>
-      <c r="D35" s="28">
+      <c r="D35" s="27">
         <f>IF(COUNT(B35,C35)&lt;2,"",B35*C35)</f>
         <v/>
       </c>
-      <c r="E35" s="32" t="n"/>
-      <c r="F35" s="30">
+      <c r="E35" s="31" t="n"/>
+      <c r="F35" s="29">
         <f>IF(OR(D35="",$E$32=""),"",D35/$E$32)</f>
         <v/>
       </c>
-      <c r="G35" s="28">
+      <c r="G35" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
@@ -8811,66 +8839,66 @@
         </is>
       </c>
       <c r="I35" s="25" t="n"/>
-      <c r="J35" s="27" t="n">
+      <c r="J35" s="26" t="n">
         <v>2.8</v>
       </c>
       <c r="K35" s="25" t="n"/>
-      <c r="L35" s="27" t="n"/>
-      <c r="M35" s="31">
+      <c r="L35" s="26" t="n"/>
+      <c r="M35" s="30">
         <f>IF(OR(D35="",J35=""),"",IF(J35&lt;=G35,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
     <row r="36" ht="17" customHeight="1">
       <c r="A36" s="25" t="n"/>
-      <c r="B36" s="27" t="n"/>
-      <c r="C36" s="27" t="n"/>
-      <c r="D36" s="28">
+      <c r="B36" s="26" t="n"/>
+      <c r="C36" s="26" t="n"/>
+      <c r="D36" s="27">
         <f>IF(COUNT(B36,C36)&lt;2,"",B36*C36)</f>
         <v/>
       </c>
-      <c r="E36" s="32" t="n"/>
-      <c r="F36" s="30">
+      <c r="E36" s="31" t="n"/>
+      <c r="F36" s="29">
         <f>IF(OR(D36="",$E$32=""),"",D36/$E$32)</f>
         <v/>
       </c>
-      <c r="G36" s="28">
+      <c r="G36" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
       <c r="H36" s="25" t="n"/>
       <c r="I36" s="25" t="n"/>
-      <c r="J36" s="27" t="n"/>
+      <c r="J36" s="26" t="n"/>
       <c r="K36" s="25" t="n"/>
-      <c r="L36" s="27" t="n"/>
-      <c r="M36" s="31">
+      <c r="L36" s="26" t="n"/>
+      <c r="M36" s="30">
         <f>IF(OR(D36="",J36=""),"",IF(J36&lt;=G36,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
     <row r="37" ht="17" customHeight="1">
-      <c r="A37" s="33" t="n"/>
-      <c r="B37" s="34" t="n"/>
-      <c r="C37" s="34" t="n"/>
-      <c r="D37" s="35">
+      <c r="A37" s="32" t="n"/>
+      <c r="B37" s="33" t="n"/>
+      <c r="C37" s="33" t="n"/>
+      <c r="D37" s="34">
         <f>IF(COUNT(B37,C37)&lt;2,"",B37*C37)</f>
         <v/>
       </c>
-      <c r="E37" s="36" t="n"/>
-      <c r="F37" s="37">
+      <c r="E37" s="35" t="n"/>
+      <c r="F37" s="36">
         <f>IF(OR(D37="",$E$32=""),"",D37/$E$32)</f>
         <v/>
       </c>
-      <c r="G37" s="35">
+      <c r="G37" s="34">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H37" s="33" t="n"/>
-      <c r="I37" s="33" t="n"/>
-      <c r="J37" s="34" t="n"/>
-      <c r="K37" s="33" t="n"/>
-      <c r="L37" s="34" t="n"/>
-      <c r="M37" s="38">
+      <c r="H37" s="32" t="n"/>
+      <c r="I37" s="32" t="n"/>
+      <c r="J37" s="33" t="n"/>
+      <c r="K37" s="32" t="n"/>
+      <c r="L37" s="33" t="n"/>
+      <c r="M37" s="37">
         <f>IF(OR(D37="",J37=""),"",IF(J37&lt;=G37,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
@@ -9075,7 +9103,7 @@
     <row r="49">
       <c r="A49" s="40" t="inlineStr">
         <is>
-          <t>FALTA, y esta marcado en naranja: la ALTURA de cada vano. La planilla de carpinterias acota</t>
+          <t>ALTURAS: medidas sobre el dibujo de las vistas de la planilla de carpinterias, con la escala</t>
         </is>
       </c>
       <c r="B49" s="2" t="n"/>
@@ -9094,7 +9122,7 @@
     <row r="50">
       <c r="A50" s="40" t="inlineStr">
         <is>
-          <t>el nivel de dintel (2,52 / 2,15 / 2,10) y el cielorraso (3,00), pero no la altura libre del vano,</t>
+          <t>verificada contra los anchos acotados (error menor a 2 cm). La mayoria de las aberturas son de</t>
         </is>
       </c>
       <c r="B50" s="2" t="n"/>
@@ -9113,7 +9141,7 @@
     <row r="51">
       <c r="A51" s="40" t="inlineStr">
         <is>
-          <t>asi que no se puede deducir sin el nivel de antepecho de cada abertura.</t>
+          <t>piso a cielorraso, 3,00 m. VERIFICARLAS contra el plano antes de presentar.</t>
         </is>
       </c>
       <c r="B51" s="2" t="n"/>
@@ -9130,7 +9158,11 @@
       <c r="M51" s="2" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="40" t="inlineStr"/>
+      <c r="A52" s="40" t="inlineStr">
+        <is>
+          <t>Quedan en naranja las tres que no se pudieron medir: PV01, PV04 (2) y PF04.</t>
+        </is>
+      </c>
       <c r="B52" s="2" t="n"/>
       <c r="C52" s="2" t="n"/>
       <c r="D52" s="2" t="n"/>
@@ -9145,11 +9177,7 @@
       <c r="M52" s="2" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="40" t="inlineStr">
-        <is>
-          <t>ORIENTACION: el simbolo de norte del plano de plantas (flecha con arco, arriba a la derecha)</t>
-        </is>
-      </c>
+      <c r="A53" s="40" t="inlineStr"/>
       <c r="B53" s="2" t="n"/>
       <c r="C53" s="2" t="n"/>
       <c r="D53" s="2" t="n"/>
@@ -9166,7 +9194,7 @@
     <row r="54">
       <c r="A54" s="40" t="inlineStr">
         <is>
-          <t>apunta hacia la derecha de la hoja. Entonces: derecha = Norte, izquierda = Sur, abajo = Este,</t>
+          <t>ORIENTACION: el simbolo de norte del plano de plantas (flecha con arco, arriba a la derecha)</t>
         </is>
       </c>
       <c r="B54" s="2" t="n"/>
@@ -9185,7 +9213,7 @@
     <row r="55">
       <c r="A55" s="40" t="inlineStr">
         <is>
-          <t>arriba = Oeste. Coincide con los rotulos Dormitorio Norte y Dormitorio Sur del plano.</t>
+          <t>apunta hacia la derecha de la hoja. Entonces: derecha = Norte, izquierda = Sur, abajo = Este,</t>
         </is>
       </c>
       <c r="B55" s="2" t="n"/>
@@ -9204,7 +9232,7 @@
     <row r="56">
       <c r="A56" s="40" t="inlineStr">
         <is>
-          <t>Cada abertura se asigno a la fachada por su posicion en planta.</t>
+          <t>arriba = Oeste. Coincide con los rotulos Dormitorio Norte y Dormitorio Sur del plano.</t>
         </is>
       </c>
       <c r="B56" s="2" t="n"/>
@@ -9223,7 +9251,7 @@
     <row r="57">
       <c r="A57" s="40" t="inlineStr">
         <is>
-          <t>Las tres aberturas que dan al patio interno quedan en un bloque aparte: hay que confirmar</t>
+          <t>Cada abertura se asigno a la fachada por su posicion en planta.</t>
         </is>
       </c>
       <c r="B57" s="2" t="n"/>
@@ -9242,7 +9270,7 @@
     <row r="58">
       <c r="A58" s="40" t="inlineStr">
         <is>
-          <t>a que lado del patio dan antes de asignarles orientacion y factor de exposicion solar.</t>
+          <t>Las tres aberturas que dan al patio interno quedan en un bloque aparte: hay que confirmar</t>
         </is>
       </c>
       <c r="B58" s="2" t="n"/>
@@ -9259,7 +9287,11 @@
       <c r="M58" s="2" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="40" t="inlineStr"/>
+      <c r="A59" s="40" t="inlineStr">
+        <is>
+          <t>a que lado del patio dan antes de asignarles orientacion y factor de exposicion solar.</t>
+        </is>
+      </c>
       <c r="B59" s="2" t="n"/>
       <c r="C59" s="2" t="n"/>
       <c r="D59" s="2" t="n"/>
@@ -9274,11 +9306,7 @@
       <c r="M59" s="2" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="40" t="inlineStr">
-        <is>
-          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
-        </is>
-      </c>
+      <c r="A60" s="40" t="inlineStr"/>
       <c r="B60" s="2" t="n"/>
       <c r="C60" s="2" t="n"/>
       <c r="D60" s="2" t="n"/>
@@ -9293,7 +9321,11 @@
       <c r="M60" s="2" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="40" t="inlineStr"/>
+      <c r="A61" s="40" t="inlineStr">
+        <is>
+          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
+        </is>
+      </c>
       <c r="B61" s="2" t="n"/>
       <c r="C61" s="2" t="n"/>
       <c r="D61" s="2" t="n"/>
@@ -9308,11 +9340,7 @@
       <c r="M61" s="2" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="40" t="inlineStr">
-        <is>
-          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
-        </is>
-      </c>
+      <c r="A62" s="40" t="inlineStr"/>
       <c r="B62" s="2" t="n"/>
       <c r="C62" s="2" t="n"/>
       <c r="D62" s="2" t="n"/>
@@ -9329,7 +9357,7 @@
     <row r="63">
       <c r="A63" s="40" t="inlineStr">
         <is>
-          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
+          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
         </is>
       </c>
       <c r="B63" s="2" t="n"/>
@@ -9348,7 +9376,7 @@
     <row r="64">
       <c r="A64" s="40" t="inlineStr">
         <is>
-          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
+          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
         </is>
       </c>
       <c r="B64" s="2" t="n"/>
@@ -9363,6 +9391,25 @@
       <c r="K64" s="2" t="n"/>
       <c r="L64" s="2" t="n"/>
       <c r="M64" s="2" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="40" t="inlineStr">
+        <is>
+          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="n"/>
+      <c r="C65" s="2" t="n"/>
+      <c r="D65" s="2" t="n"/>
+      <c r="E65" s="2" t="n"/>
+      <c r="F65" s="2" t="n"/>
+      <c r="G65" s="2" t="n"/>
+      <c r="H65" s="2" t="n"/>
+      <c r="I65" s="2" t="n"/>
+      <c r="J65" s="2" t="n"/>
+      <c r="K65" s="2" t="n"/>
+      <c r="L65" s="2" t="n"/>
+      <c r="M65" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -9852,7 +9899,7 @@
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
-      <c r="A5" s="32" t="n"/>
+      <c r="A5" s="31" t="n"/>
       <c r="B5" s="43" t="inlineStr">
         <is>
           <t>VI 01b</t>
@@ -9969,7 +10016,7 @@
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
-      <c r="A6" s="32" t="n"/>
+      <c r="A6" s="31" t="n"/>
       <c r="B6" s="43" t="inlineStr">
         <is>
           <t>VI 02</t>
@@ -10086,7 +10133,7 @@
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
-      <c r="A7" s="32" t="n"/>
+      <c r="A7" s="31" t="n"/>
       <c r="B7" s="43" t="inlineStr">
         <is>
           <t>VI 03c</t>
@@ -10199,7 +10246,7 @@
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
-      <c r="A8" s="32" t="n"/>
+      <c r="A8" s="31" t="n"/>
       <c r="B8" s="43" t="inlineStr">
         <is>
           <t>VI 04a</t>
@@ -10320,7 +10367,7 @@
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
-      <c r="A9" s="32" t="n"/>
+      <c r="A9" s="31" t="n"/>
       <c r="B9" s="43" t="inlineStr">
         <is>
           <t>VI 04b</t>
@@ -10433,7 +10480,7 @@
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
-      <c r="A10" s="32" t="n"/>
+      <c r="A10" s="31" t="n"/>
       <c r="B10" s="43" t="inlineStr">
         <is>
           <t>VI 06</t>
@@ -10554,7 +10601,7 @@
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
-      <c r="A11" s="32" t="n"/>
+      <c r="A11" s="31" t="n"/>
       <c r="B11" s="43" t="inlineStr">
         <is>
           <t>VI 07a</t>
@@ -10671,7 +10718,7 @@
       </c>
     </row>
     <row r="12" ht="46" customHeight="1">
-      <c r="A12" s="32" t="n"/>
+      <c r="A12" s="31" t="n"/>
       <c r="B12" s="43" t="inlineStr">
         <is>
           <t>VI 07b</t>
@@ -10788,7 +10835,7 @@
       </c>
     </row>
     <row r="13" ht="46" customHeight="1">
-      <c r="A13" s="32" t="n"/>
+      <c r="A13" s="31" t="n"/>
       <c r="B13" s="43" t="inlineStr">
         <is>
           <t>VI 07c</t>
@@ -10909,7 +10956,7 @@
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
-      <c r="A14" s="32" t="n"/>
+      <c r="A14" s="31" t="n"/>
       <c r="B14" s="43" t="inlineStr">
         <is>
           <t>VI 08a</t>
@@ -11022,7 +11069,7 @@
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
-      <c r="A15" s="32" t="n"/>
+      <c r="A15" s="31" t="n"/>
       <c r="B15" s="43" t="inlineStr">
         <is>
           <t>VI 08b</t>
@@ -11139,7 +11186,7 @@
       </c>
     </row>
     <row r="16" ht="46" customHeight="1">
-      <c r="A16" s="32" t="n"/>
+      <c r="A16" s="31" t="n"/>
       <c r="B16" s="43" t="inlineStr">
         <is>
           <t>VI 09</t>
@@ -11260,7 +11307,7 @@
       </c>
     </row>
     <row r="17" ht="46" customHeight="1">
-      <c r="A17" s="32" t="n"/>
+      <c r="A17" s="31" t="n"/>
       <c r="B17" s="43" t="inlineStr">
         <is>
           <t>VI 10a</t>
@@ -11373,7 +11420,7 @@
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
-      <c r="A18" s="32" t="n"/>
+      <c r="A18" s="31" t="n"/>
       <c r="B18" s="43" t="inlineStr">
         <is>
           <t>VI 10b</t>
@@ -11486,7 +11533,7 @@
       </c>
     </row>
     <row r="19" ht="46" customHeight="1">
-      <c r="A19" s="32" t="n"/>
+      <c r="A19" s="31" t="n"/>
       <c r="B19" s="43" t="inlineStr">
         <is>
           <t>VI 10c</t>
@@ -11599,7 +11646,7 @@
       </c>
     </row>
     <row r="20" ht="46" customHeight="1">
-      <c r="A20" s="32" t="n"/>
+      <c r="A20" s="31" t="n"/>
       <c r="B20" s="43" t="inlineStr">
         <is>
           <t>VI 11a</t>
@@ -11716,7 +11763,7 @@
       </c>
     </row>
     <row r="21" ht="46" customHeight="1">
-      <c r="A21" s="32" t="n"/>
+      <c r="A21" s="31" t="n"/>
       <c r="B21" s="43" t="inlineStr">
         <is>
           <t>VI 11b</t>
@@ -11833,7 +11880,7 @@
       </c>
     </row>
     <row r="22" ht="46" customHeight="1">
-      <c r="A22" s="32" t="n"/>
+      <c r="A22" s="31" t="n"/>
       <c r="B22" s="43" t="inlineStr">
         <is>
           <t>VI 11c</t>
@@ -11950,7 +11997,7 @@
       </c>
     </row>
     <row r="23" ht="46" customHeight="1">
-      <c r="A23" s="32" t="n"/>
+      <c r="A23" s="31" t="n"/>
       <c r="B23" s="43" t="inlineStr">
         <is>
           <t>VCH 03a</t>
@@ -12067,7 +12114,7 @@
       </c>
     </row>
     <row r="24" ht="46" customHeight="1">
-      <c r="A24" s="32" t="n"/>
+      <c r="A24" s="31" t="n"/>
       <c r="B24" s="43" t="inlineStr">
         <is>
           <t>VCH 03b</t>
@@ -12184,7 +12231,7 @@
       </c>
     </row>
     <row r="25" ht="46" customHeight="1">
-      <c r="A25" s="36" t="n"/>
+      <c r="A25" s="35" t="n"/>
       <c r="B25" s="46" t="inlineStr">
         <is>
           <t>VCH 05</t>
@@ -12418,7 +12465,7 @@
       </c>
     </row>
     <row r="27" ht="46" customHeight="1">
-      <c r="A27" s="32" t="n"/>
+      <c r="A27" s="31" t="n"/>
       <c r="B27" s="43" t="inlineStr">
         <is>
           <t>VI 13a</t>
@@ -12531,7 +12578,7 @@
       </c>
     </row>
     <row r="28" ht="46" customHeight="1">
-      <c r="A28" s="32" t="n"/>
+      <c r="A28" s="31" t="n"/>
       <c r="B28" s="43" t="inlineStr">
         <is>
           <t>VI 13b</t>
@@ -12644,7 +12691,7 @@
       </c>
     </row>
     <row r="29" ht="46" customHeight="1">
-      <c r="A29" s="32" t="n"/>
+      <c r="A29" s="31" t="n"/>
       <c r="B29" s="43" t="inlineStr">
         <is>
           <t>VI 14</t>
@@ -12757,7 +12804,7 @@
       </c>
     </row>
     <row r="30" ht="46" customHeight="1">
-      <c r="A30" s="32" t="n"/>
+      <c r="A30" s="31" t="n"/>
       <c r="B30" s="43" t="inlineStr">
         <is>
           <t>VI 15a</t>
@@ -12874,7 +12921,7 @@
       </c>
     </row>
     <row r="31" ht="46" customHeight="1">
-      <c r="A31" s="32" t="n"/>
+      <c r="A31" s="31" t="n"/>
       <c r="B31" s="43" t="inlineStr">
         <is>
           <t>VI 15b</t>
@@ -12991,7 +13038,7 @@
       </c>
     </row>
     <row r="32" ht="46" customHeight="1">
-      <c r="A32" s="32" t="n"/>
+      <c r="A32" s="31" t="n"/>
       <c r="B32" s="43" t="inlineStr">
         <is>
           <t>VI 16a</t>
@@ -13104,7 +13151,7 @@
       </c>
     </row>
     <row r="33" ht="46" customHeight="1">
-      <c r="A33" s="32" t="n"/>
+      <c r="A33" s="31" t="n"/>
       <c r="B33" s="43" t="inlineStr">
         <is>
           <t>VI 16b</t>
@@ -13217,7 +13264,7 @@
       </c>
     </row>
     <row r="34" ht="46" customHeight="1">
-      <c r="A34" s="36" t="n"/>
+      <c r="A34" s="35" t="n"/>
       <c r="B34" s="46" t="inlineStr">
         <is>
           <t>VI 17</t>
@@ -13663,7 +13710,7 @@
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
-      <c r="A5" s="32" t="n"/>
+      <c r="A5" s="31" t="n"/>
       <c r="B5" s="43" t="inlineStr">
         <is>
           <t>L02</t>
@@ -13735,7 +13782,7 @@
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
-      <c r="A6" s="32" t="n"/>
+      <c r="A6" s="31" t="n"/>
       <c r="B6" s="43" t="inlineStr">
         <is>
           <t>L03</t>
@@ -13803,7 +13850,7 @@
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
-      <c r="A7" s="32" t="n"/>
+      <c r="A7" s="31" t="n"/>
       <c r="B7" s="43" t="inlineStr">
         <is>
           <t>L04</t>
@@ -13871,7 +13918,7 @@
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
-      <c r="A8" s="32" t="n"/>
+      <c r="A8" s="31" t="n"/>
       <c r="B8" s="43" t="inlineStr">
         <is>
           <t>L05</t>
@@ -13939,7 +13986,7 @@
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
-      <c r="A9" s="32" t="n"/>
+      <c r="A9" s="31" t="n"/>
       <c r="B9" s="43" t="inlineStr">
         <is>
           <t>L06</t>
@@ -14007,7 +14054,7 @@
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
-      <c r="A10" s="32" t="n"/>
+      <c r="A10" s="31" t="n"/>
       <c r="B10" s="43" t="inlineStr">
         <is>
           <t>L07 (x)</t>
@@ -14081,7 +14128,7 @@
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
-      <c r="A11" s="32" t="n"/>
+      <c r="A11" s="31" t="n"/>
       <c r="B11" s="43" t="inlineStr">
         <is>
           <t>L07 (y)</t>
@@ -14155,7 +14202,7 @@
       </c>
     </row>
     <row r="12" ht="46" customHeight="1">
-      <c r="A12" s="36" t="n"/>
+      <c r="A12" s="35" t="n"/>
       <c r="B12" s="46" t="inlineStr">
         <is>
           <t>L08</t>
@@ -14299,7 +14346,7 @@
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
-      <c r="A14" s="32" t="n"/>
+      <c r="A14" s="31" t="n"/>
       <c r="B14" s="43" t="inlineStr">
         <is>
           <t>L10 (x)</t>
@@ -14373,7 +14420,7 @@
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
-      <c r="A15" s="36" t="n"/>
+      <c r="A15" s="35" t="n"/>
       <c r="B15" s="46" t="inlineStr">
         <is>
           <t>L10 (y)</t>
@@ -14729,7 +14776,7 @@
       </c>
     </row>
     <row r="5" ht="17" customHeight="1">
-      <c r="A5" s="32" t="n"/>
+      <c r="A5" s="31" t="n"/>
       <c r="B5" s="43" t="inlineStr">
         <is>
           <t>C7</t>
@@ -14794,7 +14841,7 @@
       </c>
     </row>
     <row r="6" ht="17" customHeight="1">
-      <c r="A6" s="32" t="n"/>
+      <c r="A6" s="31" t="n"/>
       <c r="B6" s="43" t="inlineStr">
         <is>
           <t>C8</t>
@@ -14859,7 +14906,7 @@
       </c>
     </row>
     <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="36" t="n"/>
+      <c r="A7" s="35" t="n"/>
       <c r="B7" s="46" t="inlineStr">
         <is>
           <t>C9</t>
@@ -14993,7 +15040,7 @@
       </c>
     </row>
     <row r="9" ht="17" customHeight="1">
-      <c r="A9" s="32" t="n"/>
+      <c r="A9" s="31" t="n"/>
       <c r="B9" s="43" t="inlineStr">
         <is>
           <t>C2</t>
@@ -15058,7 +15105,7 @@
       </c>
     </row>
     <row r="10" ht="17" customHeight="1">
-      <c r="A10" s="32" t="n"/>
+      <c r="A10" s="31" t="n"/>
       <c r="B10" s="43" t="inlineStr">
         <is>
           <t>C3</t>
@@ -15123,7 +15170,7 @@
       </c>
     </row>
     <row r="11" ht="17" customHeight="1">
-      <c r="A11" s="32" t="n"/>
+      <c r="A11" s="31" t="n"/>
       <c r="B11" s="43" t="inlineStr">
         <is>
           <t>C4</t>
@@ -15188,7 +15235,7 @@
       </c>
     </row>
     <row r="12" ht="17" customHeight="1">
-      <c r="A12" s="32" t="n"/>
+      <c r="A12" s="31" t="n"/>
       <c r="B12" s="43" t="inlineStr">
         <is>
           <t>C5</t>
@@ -15253,7 +15300,7 @@
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
-      <c r="A13" s="32" t="n"/>
+      <c r="A13" s="31" t="n"/>
       <c r="B13" s="43" t="inlineStr">
         <is>
           <t>C6</t>
@@ -15318,7 +15365,7 @@
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
-      <c r="A14" s="32" t="n"/>
+      <c r="A14" s="31" t="n"/>
       <c r="B14" s="43" t="inlineStr">
         <is>
           <t>C7</t>
@@ -15383,7 +15430,7 @@
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="32" t="n"/>
+      <c r="A15" s="31" t="n"/>
       <c r="B15" s="43" t="inlineStr">
         <is>
           <t>C8</t>
@@ -15448,7 +15495,7 @@
       </c>
     </row>
     <row r="16" ht="17" customHeight="1">
-      <c r="A16" s="36" t="n"/>
+      <c r="A16" s="35" t="n"/>
       <c r="B16" s="46" t="inlineStr">
         <is>
           <t>C9</t>
@@ -19766,7 +19813,7 @@
       </c>
     </row>
     <row r="5" ht="17" customHeight="1">
-      <c r="A5" s="32" t="n"/>
+      <c r="A5" s="31" t="n"/>
       <c r="B5" s="43" t="inlineStr">
         <is>
           <t>T2</t>
@@ -19827,7 +19874,7 @@
       </c>
     </row>
     <row r="6" ht="17" customHeight="1">
-      <c r="A6" s="32" t="n"/>
+      <c r="A6" s="31" t="n"/>
       <c r="B6" s="43" t="inlineStr">
         <is>
           <t>T3</t>
@@ -19888,7 +19935,7 @@
       </c>
     </row>
     <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="32" t="n"/>
+      <c r="A7" s="31" t="n"/>
       <c r="B7" s="43" t="inlineStr">
         <is>
           <t>T4</t>
@@ -19949,7 +19996,7 @@
       </c>
     </row>
     <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="32" t="n"/>
+      <c r="A8" s="31" t="n"/>
       <c r="B8" s="43" t="inlineStr">
         <is>
           <t>T5</t>
@@ -20010,7 +20057,7 @@
       </c>
     </row>
     <row r="9" ht="17" customHeight="1">
-      <c r="A9" s="32" t="n"/>
+      <c r="A9" s="31" t="n"/>
       <c r="B9" s="43" t="inlineStr">
         <is>
           <t>T6</t>
@@ -20071,7 +20118,7 @@
       </c>
     </row>
     <row r="10" ht="17" customHeight="1">
-      <c r="A10" s="32" t="n"/>
+      <c r="A10" s="31" t="n"/>
       <c r="B10" s="43" t="inlineStr">
         <is>
           <t>T7</t>
@@ -20132,7 +20179,7 @@
       </c>
     </row>
     <row r="11" ht="17" customHeight="1">
-      <c r="A11" s="36" t="n"/>
+      <c r="A11" s="35" t="n"/>
       <c r="B11" s="46" t="inlineStr">
         <is>
           <t>T8</t>
@@ -20258,7 +20305,7 @@
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
-      <c r="A13" s="32" t="n"/>
+      <c r="A13" s="31" t="n"/>
       <c r="B13" s="43" t="inlineStr">
         <is>
           <t>T10</t>
@@ -20319,7 +20366,7 @@
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
-      <c r="A14" s="32" t="n"/>
+      <c r="A14" s="31" t="n"/>
       <c r="B14" s="43" t="inlineStr">
         <is>
           <t>T11</t>
@@ -20380,7 +20427,7 @@
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="32" t="n"/>
+      <c r="A15" s="31" t="n"/>
       <c r="B15" s="43" t="inlineStr">
         <is>
           <t>T12</t>
@@ -20441,7 +20488,7 @@
       </c>
     </row>
     <row r="16" ht="17" customHeight="1">
-      <c r="A16" s="36" t="n"/>
+      <c r="A16" s="35" t="n"/>
       <c r="B16" s="46" t="inlineStr">
         <is>
           <t>T13</t>

</xml_diff>

<commit_message>
Planilla 3: corregir el norte y orientar las aberturas del patio interno
El simbolo de norte (circulo con aguja, en el patio interno) apunta a 45
grados hacia arriba y a la derecha. La lectura anterior, hecha sobre el
PDF de plantas donde el simbolo sale muy chico, decia que apuntaba hacia
la derecha y era incorrecta.

Las fachadas pasan a ser Noroeste (arriba), Noreste (derecha), Sudeste
(abajo) y Sudoeste (izquierda), no N-S-E-O.

Las del patio interno se orientan por la pared en la que estan: PF02 al
norte del patio mira al Sudeste, PF01 al oeste mira al Noreste y el
segundo PF01 al este mira al Sudoeste. PV01 va a la fachada Noreste: esta
entre el living comedor y la galeria.

Los rotulos Dormitorio Norte / Dormitorio Sur del plano no coinciden con
el norte real; quedan anotados como nombres de uso.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -29,7 +29,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Iluminacion y ventilacion'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Planilla 3 higrotermica'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla 3 higrotermica'!$A$1:$M$37</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla 3 higrotermica'!$A$1:$M$38</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Planilla vigas'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Planilla vigas'!$A$1:$X$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Planilla losas'!$1:$3</definedName>
@@ -7616,7 +7616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M66"/>
+  <dimension ref="A1:M71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7780,7 +7780,7 @@
     <row r="6">
       <c r="A6" s="24" t="inlineStr">
         <is>
-          <t>Plano: Fachada Norte</t>
+          <t>Plano: Fachada Noreste (borde derecho del plano)</t>
         </is>
       </c>
       <c r="B6" s="4" t="n"/>
@@ -7813,7 +7813,7 @@
         <v/>
       </c>
       <c r="E7" s="28">
-        <f>SUM(D7:D11)</f>
+        <f>SUM(D7:D13)</f>
         <v/>
       </c>
       <c r="F7" s="29">
@@ -7835,7 +7835,7 @@
       </c>
       <c r="K7" s="25" t="inlineStr">
         <is>
-          <t>Norte</t>
+          <t>Noreste</t>
         </is>
       </c>
       <c r="L7" s="26" t="n"/>
@@ -7880,7 +7880,7 @@
       </c>
       <c r="K8" s="25" t="inlineStr">
         <is>
-          <t>Norte</t>
+          <t>Noreste</t>
         </is>
       </c>
       <c r="L8" s="26" t="n"/>
@@ -7925,7 +7925,7 @@
       </c>
       <c r="K9" s="25" t="inlineStr">
         <is>
-          <t>Norte</t>
+          <t>Noreste</t>
         </is>
       </c>
       <c r="L9" s="26" t="n"/>
@@ -7935,9 +7935,17 @@
       </c>
     </row>
     <row r="10" ht="17" customHeight="1">
-      <c r="A10" s="25" t="n"/>
-      <c r="B10" s="26" t="n"/>
-      <c r="C10" s="26" t="n"/>
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>PV01</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="26" t="n">
+        <v>7.7</v>
+      </c>
       <c r="D10" s="27">
         <f>IF(COUNT(B10,C10)&lt;2,"",B10*C10)</f>
         <v/>
@@ -7951,10 +7959,20 @@
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H10" s="25" t="n"/>
+      <c r="H10" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
       <c r="I10" s="25" t="n"/>
-      <c r="J10" s="26" t="n"/>
-      <c r="K10" s="25" t="n"/>
+      <c r="J10" s="26" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K10" s="25" t="inlineStr">
+        <is>
+          <t>Noreste</t>
+        </is>
+      </c>
       <c r="L10" s="26" t="n"/>
       <c r="M10" s="30">
         <f>IF(OR(D10="",J10=""),"",IF(J10&lt;=G10,"CUMPLE","NO CUMPLE"))</f>
@@ -7962,214 +7980,237 @@
       </c>
     </row>
     <row r="11" ht="17" customHeight="1">
-      <c r="A11" s="32" t="n"/>
-      <c r="B11" s="33" t="n"/>
-      <c r="C11" s="33" t="n"/>
-      <c r="D11" s="34">
+      <c r="A11" s="25" t="inlineStr">
+        <is>
+          <t>PF01</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" s="26" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="D11" s="27">
         <f>IF(COUNT(B11,C11)&lt;2,"",B11*C11)</f>
         <v/>
       </c>
-      <c r="E11" s="35" t="n"/>
-      <c r="F11" s="36">
+      <c r="E11" s="31" t="n"/>
+      <c r="F11" s="29">
         <f>IF(OR(D11="",$E$7=""),"",D11/$E$7)</f>
         <v/>
       </c>
-      <c r="G11" s="34">
+      <c r="G11" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H11" s="32" t="n"/>
-      <c r="I11" s="32" t="n"/>
-      <c r="J11" s="33" t="n"/>
-      <c r="K11" s="32" t="n"/>
-      <c r="L11" s="33" t="n"/>
-      <c r="M11" s="37">
+      <c r="H11" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I11" s="25" t="n"/>
+      <c r="J11" s="26" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K11" s="25" t="inlineStr">
+        <is>
+          <t>Noreste</t>
+        </is>
+      </c>
+      <c r="L11" s="26" t="n"/>
+      <c r="M11" s="30">
         <f>IF(OR(D11="",J11=""),"",IF(J11&lt;=G11,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="24" t="inlineStr">
-        <is>
-          <t>Plano: Fachada Sur</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="4" t="n"/>
-      <c r="F12" s="4" t="n"/>
-      <c r="G12" s="4" t="n"/>
-      <c r="H12" s="4" t="n"/>
-      <c r="I12" s="4" t="n"/>
-      <c r="J12" s="4" t="n"/>
-      <c r="K12" s="4" t="n"/>
-      <c r="L12" s="4" t="n"/>
-      <c r="M12" s="4" t="n"/>
+    <row r="12" ht="17" customHeight="1">
+      <c r="A12" s="25" t="n"/>
+      <c r="B12" s="26" t="n"/>
+      <c r="C12" s="26" t="n"/>
+      <c r="D12" s="27">
+        <f>IF(COUNT(B12,C12)&lt;2,"",B12*C12)</f>
+        <v/>
+      </c>
+      <c r="E12" s="31" t="n"/>
+      <c r="F12" s="29">
+        <f>IF(OR(D12="",$E$7=""),"",D12/$E$7)</f>
+        <v/>
+      </c>
+      <c r="G12" s="27">
+        <f>Datos_higro!$B$4</f>
+        <v/>
+      </c>
+      <c r="H12" s="25" t="n"/>
+      <c r="I12" s="25" t="n"/>
+      <c r="J12" s="26" t="n"/>
+      <c r="K12" s="25" t="n"/>
+      <c r="L12" s="26" t="n"/>
+      <c r="M12" s="30">
+        <f>IF(OR(D12="",J12=""),"",IF(J12&lt;=G12,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
     </row>
     <row r="13" ht="17" customHeight="1">
-      <c r="A13" s="25" t="inlineStr">
+      <c r="A13" s="32" t="n"/>
+      <c r="B13" s="33" t="n"/>
+      <c r="C13" s="33" t="n"/>
+      <c r="D13" s="34">
+        <f>IF(COUNT(B13,C13)&lt;2,"",B13*C13)</f>
+        <v/>
+      </c>
+      <c r="E13" s="35" t="n"/>
+      <c r="F13" s="36">
+        <f>IF(OR(D13="",$E$7=""),"",D13/$E$7)</f>
+        <v/>
+      </c>
+      <c r="G13" s="34">
+        <f>Datos_higro!$B$4</f>
+        <v/>
+      </c>
+      <c r="H13" s="32" t="n"/>
+      <c r="I13" s="32" t="n"/>
+      <c r="J13" s="33" t="n"/>
+      <c r="K13" s="32" t="n"/>
+      <c r="L13" s="33" t="n"/>
+      <c r="M13" s="37">
+        <f>IF(OR(D13="",J13=""),"",IF(J13&lt;=G13,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t>Plano: Fachada Sudoeste (borde izquierdo)</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+      <c r="D14" s="4" t="n"/>
+      <c r="E14" s="4" t="n"/>
+      <c r="F14" s="4" t="n"/>
+      <c r="G14" s="4" t="n"/>
+      <c r="H14" s="4" t="n"/>
+      <c r="I14" s="4" t="n"/>
+      <c r="J14" s="4" t="n"/>
+      <c r="K14" s="4" t="n"/>
+      <c r="L14" s="4" t="n"/>
+      <c r="M14" s="4" t="n"/>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" s="25" t="inlineStr">
         <is>
           <t>VA01</t>
         </is>
       </c>
-      <c r="B13" s="26" t="n">
+      <c r="B15" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="26" t="n">
+      <c r="C15" s="26" t="n">
         <v>0.75</v>
       </c>
-      <c r="D13" s="27">
-        <f>IF(COUNT(B13,C13)&lt;2,"",B13*C13)</f>
-        <v/>
-      </c>
-      <c r="E13" s="28">
-        <f>SUM(D13:D15)</f>
-        <v/>
-      </c>
-      <c r="F13" s="29">
-        <f>IF(OR(D13="",$E$13=""),"",D13/$E$13)</f>
-        <v/>
-      </c>
-      <c r="G13" s="27">
+      <c r="D15" s="27">
+        <f>IF(COUNT(B15,C15)&lt;2,"",B15*C15)</f>
+        <v/>
+      </c>
+      <c r="E15" s="28">
+        <f>SUM(D15:D18)</f>
+        <v/>
+      </c>
+      <c r="F15" s="29">
+        <f>IF(OR(D15="",$E$15=""),"",D15/$E$15)</f>
+        <v/>
+      </c>
+      <c r="G15" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H13" s="25" t="inlineStr">
+      <c r="H15" s="25" t="inlineStr">
         <is>
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I13" s="25" t="n"/>
-      <c r="J13" s="26" t="n">
+      <c r="I15" s="25" t="n"/>
+      <c r="J15" s="26" t="n">
         <v>2.8</v>
       </c>
-      <c r="K13" s="25" t="inlineStr">
-        <is>
-          <t>Sur</t>
-        </is>
-      </c>
-      <c r="L13" s="26" t="n"/>
-      <c r="M13" s="30">
-        <f>IF(OR(D13="",J13=""),"",IF(J13&lt;=G13,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="17" customHeight="1">
-      <c r="A14" s="25" t="n"/>
-      <c r="B14" s="26" t="n"/>
-      <c r="C14" s="26" t="n"/>
-      <c r="D14" s="27">
-        <f>IF(COUNT(B14,C14)&lt;2,"",B14*C14)</f>
-        <v/>
-      </c>
-      <c r="E14" s="31" t="n"/>
-      <c r="F14" s="29">
-        <f>IF(OR(D14="",$E$13=""),"",D14/$E$13)</f>
-        <v/>
-      </c>
-      <c r="G14" s="27">
+      <c r="K15" s="25" t="inlineStr">
+        <is>
+          <t>Sudoeste</t>
+        </is>
+      </c>
+      <c r="L15" s="26" t="n"/>
+      <c r="M15" s="30">
+        <f>IF(OR(D15="",J15=""),"",IF(J15&lt;=G15,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="17" customHeight="1">
+      <c r="A16" s="25" t="inlineStr">
+        <is>
+          <t>PF01 (2)</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" s="26" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="D16" s="27">
+        <f>IF(COUNT(B16,C16)&lt;2,"",B16*C16)</f>
+        <v/>
+      </c>
+      <c r="E16" s="31" t="n"/>
+      <c r="F16" s="29">
+        <f>IF(OR(D16="",$E$15=""),"",D16/$E$15)</f>
+        <v/>
+      </c>
+      <c r="G16" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H14" s="25" t="n"/>
-      <c r="I14" s="25" t="n"/>
-      <c r="J14" s="26" t="n"/>
-      <c r="K14" s="25" t="n"/>
-      <c r="L14" s="26" t="n"/>
-      <c r="M14" s="30">
-        <f>IF(OR(D14="",J14=""),"",IF(J14&lt;=G14,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="32" t="n"/>
-      <c r="B15" s="33" t="n"/>
-      <c r="C15" s="33" t="n"/>
-      <c r="D15" s="34">
-        <f>IF(COUNT(B15,C15)&lt;2,"",B15*C15)</f>
-        <v/>
-      </c>
-      <c r="E15" s="35" t="n"/>
-      <c r="F15" s="36">
-        <f>IF(OR(D15="",$E$13=""),"",D15/$E$13)</f>
-        <v/>
-      </c>
-      <c r="G15" s="34">
-        <f>Datos_higro!$B$4</f>
-        <v/>
-      </c>
-      <c r="H15" s="32" t="n"/>
-      <c r="I15" s="32" t="n"/>
-      <c r="J15" s="33" t="n"/>
-      <c r="K15" s="32" t="n"/>
-      <c r="L15" s="33" t="n"/>
-      <c r="M15" s="37">
-        <f>IF(OR(D15="",J15=""),"",IF(J15&lt;=G15,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="24" t="inlineStr">
-        <is>
-          <t>Plano: Fachada Este</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="4" t="n"/>
-      <c r="E16" s="4" t="n"/>
-      <c r="F16" s="4" t="n"/>
-      <c r="G16" s="4" t="n"/>
-      <c r="H16" s="4" t="n"/>
-      <c r="I16" s="4" t="n"/>
-      <c r="J16" s="4" t="n"/>
-      <c r="K16" s="4" t="n"/>
-      <c r="L16" s="4" t="n"/>
-      <c r="M16" s="4" t="n"/>
+      <c r="H16" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I16" s="25" t="n"/>
+      <c r="J16" s="26" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K16" s="25" t="inlineStr">
+        <is>
+          <t>Sudoeste</t>
+        </is>
+      </c>
+      <c r="L16" s="26" t="n"/>
+      <c r="M16" s="30">
+        <f>IF(OR(D16="",J16=""),"",IF(J16&lt;=G16,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
     </row>
     <row r="17" ht="17" customHeight="1">
-      <c r="A17" s="25" t="inlineStr">
-        <is>
-          <t>PA01</t>
-        </is>
-      </c>
-      <c r="B17" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="C17" s="26" t="n">
-        <v>1</v>
-      </c>
+      <c r="A17" s="25" t="n"/>
+      <c r="B17" s="26" t="n"/>
+      <c r="C17" s="26" t="n"/>
       <c r="D17" s="27">
         <f>IF(COUNT(B17,C17)&lt;2,"",B17*C17)</f>
         <v/>
       </c>
-      <c r="E17" s="28">
-        <f>SUM(D17:D22)</f>
-        <v/>
-      </c>
+      <c r="E17" s="31" t="n"/>
       <c r="F17" s="29">
-        <f>IF(OR(D17="",$E$17=""),"",D17/$E$17)</f>
+        <f>IF(OR(D17="",$E$15=""),"",D17/$E$15)</f>
         <v/>
       </c>
       <c r="G17" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H17" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
+      <c r="H17" s="25" t="n"/>
       <c r="I17" s="25" t="n"/>
-      <c r="J17" s="26" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K17" s="25" t="inlineStr">
-        <is>
-          <t>Este</t>
-        </is>
-      </c>
+      <c r="J17" s="26" t="n"/>
+      <c r="K17" s="25" t="n"/>
       <c r="L17" s="26" t="n"/>
       <c r="M17" s="30">
         <f>IF(OR(D17="",J17=""),"",IF(J17&lt;=G17,"CUMPLE","NO CUMPLE"))</f>
@@ -8177,114 +8218,73 @@
       </c>
     </row>
     <row r="18" ht="17" customHeight="1">
-      <c r="A18" s="25" t="inlineStr">
-        <is>
-          <t>PF04</t>
-        </is>
-      </c>
-      <c r="B18" s="26" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="C18" s="26" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="D18" s="27">
+      <c r="A18" s="32" t="n"/>
+      <c r="B18" s="33" t="n"/>
+      <c r="C18" s="33" t="n"/>
+      <c r="D18" s="34">
         <f>IF(COUNT(B18,C18)&lt;2,"",B18*C18)</f>
         <v/>
       </c>
-      <c r="E18" s="31" t="n"/>
-      <c r="F18" s="29">
-        <f>IF(OR(D18="",$E$17=""),"",D18/$E$17)</f>
-        <v/>
-      </c>
-      <c r="G18" s="27">
+      <c r="E18" s="35" t="n"/>
+      <c r="F18" s="36">
+        <f>IF(OR(D18="",$E$15=""),"",D18/$E$15)</f>
+        <v/>
+      </c>
+      <c r="G18" s="34">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H18" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I18" s="25" t="n"/>
-      <c r="J18" s="26" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K18" s="25" t="inlineStr">
-        <is>
-          <t>Este</t>
-        </is>
-      </c>
-      <c r="L18" s="26" t="n"/>
-      <c r="M18" s="30">
+      <c r="H18" s="32" t="n"/>
+      <c r="I18" s="32" t="n"/>
+      <c r="J18" s="33" t="n"/>
+      <c r="K18" s="32" t="n"/>
+      <c r="L18" s="33" t="n"/>
+      <c r="M18" s="37">
         <f>IF(OR(D18="",J18=""),"",IF(J18&lt;=G18,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="19" ht="17" customHeight="1">
-      <c r="A19" s="25" t="inlineStr">
-        <is>
-          <t>VA05</t>
-        </is>
-      </c>
-      <c r="B19" s="26" t="n">
-        <v>2.52</v>
-      </c>
-      <c r="C19" s="26" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="D19" s="27">
-        <f>IF(COUNT(B19,C19)&lt;2,"",B19*C19)</f>
-        <v/>
-      </c>
-      <c r="E19" s="31" t="n"/>
-      <c r="F19" s="29">
-        <f>IF(OR(D19="",$E$17=""),"",D19/$E$17)</f>
-        <v/>
-      </c>
-      <c r="G19" s="27">
-        <f>Datos_higro!$B$4</f>
-        <v/>
-      </c>
-      <c r="H19" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I19" s="25" t="n"/>
-      <c r="J19" s="26" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K19" s="25" t="inlineStr">
-        <is>
-          <t>Este</t>
-        </is>
-      </c>
-      <c r="L19" s="26" t="n"/>
-      <c r="M19" s="30">
-        <f>IF(OR(D19="",J19=""),"",IF(J19&lt;=G19,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
+    <row r="19">
+      <c r="A19" s="24" t="inlineStr">
+        <is>
+          <t>Plano: Fachada Sudeste (borde inferior)</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n"/>
+      <c r="C19" s="4" t="n"/>
+      <c r="D19" s="4" t="n"/>
+      <c r="E19" s="4" t="n"/>
+      <c r="F19" s="4" t="n"/>
+      <c r="G19" s="4" t="n"/>
+      <c r="H19" s="4" t="n"/>
+      <c r="I19" s="4" t="n"/>
+      <c r="J19" s="4" t="n"/>
+      <c r="K19" s="4" t="n"/>
+      <c r="L19" s="4" t="n"/>
+      <c r="M19" s="4" t="n"/>
     </row>
     <row r="20" ht="17" customHeight="1">
       <c r="A20" s="25" t="inlineStr">
         <is>
-          <t>PV04</t>
+          <t>PA01</t>
         </is>
       </c>
       <c r="B20" s="26" t="n">
         <v>3</v>
       </c>
       <c r="C20" s="26" t="n">
-        <v>2.06</v>
+        <v>1</v>
       </c>
       <c r="D20" s="27">
         <f>IF(COUNT(B20,C20)&lt;2,"",B20*C20)</f>
         <v/>
       </c>
-      <c r="E20" s="31" t="n"/>
+      <c r="E20" s="28">
+        <f>SUM(D20:D26)</f>
+        <v/>
+      </c>
       <c r="F20" s="29">
-        <f>IF(OR(D20="",$E$17=""),"",D20/$E$17)</f>
+        <f>IF(OR(D20="",$E$20=""),"",D20/$E$20)</f>
         <v/>
       </c>
       <c r="G20" s="27">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="K20" s="25" t="inlineStr">
         <is>
-          <t>Este</t>
+          <t>Sudeste</t>
         </is>
       </c>
       <c r="L20" s="26" t="n"/>
@@ -8312,26 +8312,44 @@
       </c>
     </row>
     <row r="21" ht="17" customHeight="1">
-      <c r="A21" s="25" t="n"/>
-      <c r="B21" s="26" t="n"/>
-      <c r="C21" s="26" t="n"/>
+      <c r="A21" s="25" t="inlineStr">
+        <is>
+          <t>PF04</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C21" s="26" t="n">
+        <v>2.7</v>
+      </c>
       <c r="D21" s="27">
         <f>IF(COUNT(B21,C21)&lt;2,"",B21*C21)</f>
         <v/>
       </c>
       <c r="E21" s="31" t="n"/>
       <c r="F21" s="29">
-        <f>IF(OR(D21="",$E$17=""),"",D21/$E$17)</f>
+        <f>IF(OR(D21="",$E$20=""),"",D21/$E$20)</f>
         <v/>
       </c>
       <c r="G21" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H21" s="25" t="n"/>
+      <c r="H21" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
       <c r="I21" s="25" t="n"/>
-      <c r="J21" s="26" t="n"/>
-      <c r="K21" s="25" t="n"/>
+      <c r="J21" s="26" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K21" s="25" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
       <c r="L21" s="26" t="n"/>
       <c r="M21" s="30">
         <f>IF(OR(D21="",J21=""),"",IF(J21&lt;=G21,"CUMPLE","NO CUMPLE"))</f>
@@ -8339,73 +8357,114 @@
       </c>
     </row>
     <row r="22" ht="17" customHeight="1">
-      <c r="A22" s="32" t="n"/>
-      <c r="B22" s="33" t="n"/>
-      <c r="C22" s="33" t="n"/>
-      <c r="D22" s="34">
+      <c r="A22" s="25" t="inlineStr">
+        <is>
+          <t>VA05</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="C22" s="26" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D22" s="27">
         <f>IF(COUNT(B22,C22)&lt;2,"",B22*C22)</f>
         <v/>
       </c>
-      <c r="E22" s="35" t="n"/>
-      <c r="F22" s="36">
-        <f>IF(OR(D22="",$E$17=""),"",D22/$E$17)</f>
-        <v/>
-      </c>
-      <c r="G22" s="34">
+      <c r="E22" s="31" t="n"/>
+      <c r="F22" s="29">
+        <f>IF(OR(D22="",$E$20=""),"",D22/$E$20)</f>
+        <v/>
+      </c>
+      <c r="G22" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H22" s="32" t="n"/>
-      <c r="I22" s="32" t="n"/>
-      <c r="J22" s="33" t="n"/>
-      <c r="K22" s="32" t="n"/>
-      <c r="L22" s="33" t="n"/>
-      <c r="M22" s="37">
+      <c r="H22" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I22" s="25" t="n"/>
+      <c r="J22" s="26" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K22" s="25" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="L22" s="26" t="n"/>
+      <c r="M22" s="30">
         <f>IF(OR(D22="",J22=""),"",IF(J22&lt;=G22,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="24" t="inlineStr">
-        <is>
-          <t>Plano: Fachada Oeste</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="n"/>
-      <c r="C23" s="4" t="n"/>
-      <c r="D23" s="4" t="n"/>
-      <c r="E23" s="4" t="n"/>
-      <c r="F23" s="4" t="n"/>
-      <c r="G23" s="4" t="n"/>
-      <c r="H23" s="4" t="n"/>
-      <c r="I23" s="4" t="n"/>
-      <c r="J23" s="4" t="n"/>
-      <c r="K23" s="4" t="n"/>
-      <c r="L23" s="4" t="n"/>
-      <c r="M23" s="4" t="n"/>
+    <row r="23" ht="17" customHeight="1">
+      <c r="A23" s="25" t="inlineStr">
+        <is>
+          <t>PV04</t>
+        </is>
+      </c>
+      <c r="B23" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C23" s="26" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="D23" s="27">
+        <f>IF(COUNT(B23,C23)&lt;2,"",B23*C23)</f>
+        <v/>
+      </c>
+      <c r="E23" s="31" t="n"/>
+      <c r="F23" s="29">
+        <f>IF(OR(D23="",$E$20=""),"",D23/$E$20)</f>
+        <v/>
+      </c>
+      <c r="G23" s="27">
+        <f>Datos_higro!$B$4</f>
+        <v/>
+      </c>
+      <c r="H23" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I23" s="25" t="n"/>
+      <c r="J23" s="26" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K23" s="25" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="L23" s="26" t="n"/>
+      <c r="M23" s="30">
+        <f>IF(OR(D23="",J23=""),"",IF(J23&lt;=G23,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
     </row>
     <row r="24" ht="17" customHeight="1">
       <c r="A24" s="25" t="inlineStr">
         <is>
-          <t>PV03</t>
+          <t>PF02</t>
         </is>
       </c>
       <c r="B24" s="26" t="n">
         <v>3</v>
       </c>
       <c r="C24" s="26" t="n">
-        <v>1.76</v>
+        <v>3.75</v>
       </c>
       <c r="D24" s="27">
         <f>IF(COUNT(B24,C24)&lt;2,"",B24*C24)</f>
         <v/>
       </c>
-      <c r="E24" s="28">
-        <f>SUM(D24:D30)</f>
-        <v/>
-      </c>
+      <c r="E24" s="31" t="n"/>
       <c r="F24" s="29">
-        <f>IF(OR(D24="",$E$24=""),"",D24/$E$24)</f>
+        <f>IF(OR(D24="",$E$20=""),"",D24/$E$20)</f>
         <v/>
       </c>
       <c r="G24" s="27">
@@ -8423,7 +8482,7 @@
       </c>
       <c r="K24" s="25" t="inlineStr">
         <is>
-          <t>Oeste</t>
+          <t>Sudeste</t>
         </is>
       </c>
       <c r="L24" s="26" t="n"/>
@@ -8433,44 +8492,26 @@
       </c>
     </row>
     <row r="25" ht="17" customHeight="1">
-      <c r="A25" s="25" t="inlineStr">
-        <is>
-          <t>VA02</t>
-        </is>
-      </c>
-      <c r="B25" s="26" t="n">
-        <v>2.15</v>
-      </c>
-      <c r="C25" s="26" t="n">
-        <v>0.75</v>
-      </c>
+      <c r="A25" s="25" t="n"/>
+      <c r="B25" s="26" t="n"/>
+      <c r="C25" s="26" t="n"/>
       <c r="D25" s="27">
         <f>IF(COUNT(B25,C25)&lt;2,"",B25*C25)</f>
         <v/>
       </c>
       <c r="E25" s="31" t="n"/>
       <c r="F25" s="29">
-        <f>IF(OR(D25="",$E$24=""),"",D25/$E$24)</f>
+        <f>IF(OR(D25="",$E$20=""),"",D25/$E$20)</f>
         <v/>
       </c>
       <c r="G25" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H25" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
+      <c r="H25" s="25" t="n"/>
       <c r="I25" s="25" t="n"/>
-      <c r="J25" s="26" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K25" s="25" t="inlineStr">
-        <is>
-          <t>Oeste</t>
-        </is>
-      </c>
+      <c r="J25" s="26" t="n"/>
+      <c r="K25" s="25" t="n"/>
       <c r="L25" s="26" t="n"/>
       <c r="M25" s="30">
         <f>IF(OR(D25="",J25=""),"",IF(J25&lt;=G25,"CUMPLE","NO CUMPLE"))</f>
@@ -8478,114 +8519,73 @@
       </c>
     </row>
     <row r="26" ht="17" customHeight="1">
-      <c r="A26" s="25" t="inlineStr">
-        <is>
-          <t>PA02</t>
-        </is>
-      </c>
-      <c r="B26" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="C26" s="26" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D26" s="27">
+      <c r="A26" s="32" t="n"/>
+      <c r="B26" s="33" t="n"/>
+      <c r="C26" s="33" t="n"/>
+      <c r="D26" s="34">
         <f>IF(COUNT(B26,C26)&lt;2,"",B26*C26)</f>
         <v/>
       </c>
-      <c r="E26" s="31" t="n"/>
-      <c r="F26" s="29">
-        <f>IF(OR(D26="",$E$24=""),"",D26/$E$24)</f>
-        <v/>
-      </c>
-      <c r="G26" s="27">
+      <c r="E26" s="35" t="n"/>
+      <c r="F26" s="36">
+        <f>IF(OR(D26="",$E$20=""),"",D26/$E$20)</f>
+        <v/>
+      </c>
+      <c r="G26" s="34">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H26" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I26" s="25" t="n"/>
-      <c r="J26" s="26" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K26" s="25" t="inlineStr">
-        <is>
-          <t>Oeste</t>
-        </is>
-      </c>
-      <c r="L26" s="26" t="n"/>
-      <c r="M26" s="30">
+      <c r="H26" s="32" t="n"/>
+      <c r="I26" s="32" t="n"/>
+      <c r="J26" s="33" t="n"/>
+      <c r="K26" s="32" t="n"/>
+      <c r="L26" s="33" t="n"/>
+      <c r="M26" s="37">
         <f>IF(OR(D26="",J26=""),"",IF(J26&lt;=G26,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="27" ht="17" customHeight="1">
-      <c r="A27" s="25" t="inlineStr">
-        <is>
-          <t>VA03</t>
-        </is>
-      </c>
-      <c r="B27" s="26" t="n">
-        <v>2.52</v>
-      </c>
-      <c r="C27" s="26" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D27" s="27">
-        <f>IF(COUNT(B27,C27)&lt;2,"",B27*C27)</f>
-        <v/>
-      </c>
-      <c r="E27" s="31" t="n"/>
-      <c r="F27" s="29">
-        <f>IF(OR(D27="",$E$24=""),"",D27/$E$24)</f>
-        <v/>
-      </c>
-      <c r="G27" s="27">
-        <f>Datos_higro!$B$4</f>
-        <v/>
-      </c>
-      <c r="H27" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I27" s="25" t="n"/>
-      <c r="J27" s="26" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K27" s="25" t="inlineStr">
-        <is>
-          <t>Oeste</t>
-        </is>
-      </c>
-      <c r="L27" s="26" t="n"/>
-      <c r="M27" s="30">
-        <f>IF(OR(D27="",J27=""),"",IF(J27&lt;=G27,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
+    <row r="27">
+      <c r="A27" s="24" t="inlineStr">
+        <is>
+          <t>Plano: Fachada Noroeste (borde superior)</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n"/>
+      <c r="C27" s="4" t="n"/>
+      <c r="D27" s="4" t="n"/>
+      <c r="E27" s="4" t="n"/>
+      <c r="F27" s="4" t="n"/>
+      <c r="G27" s="4" t="n"/>
+      <c r="H27" s="4" t="n"/>
+      <c r="I27" s="4" t="n"/>
+      <c r="J27" s="4" t="n"/>
+      <c r="K27" s="4" t="n"/>
+      <c r="L27" s="4" t="n"/>
+      <c r="M27" s="4" t="n"/>
     </row>
     <row r="28" ht="17" customHeight="1">
       <c r="A28" s="25" t="inlineStr">
         <is>
-          <t>PF05</t>
+          <t>PV03</t>
         </is>
       </c>
       <c r="B28" s="26" t="n">
-        <v>2.52</v>
+        <v>3</v>
       </c>
       <c r="C28" s="26" t="n">
-        <v>0.75</v>
+        <v>1.76</v>
       </c>
       <c r="D28" s="27">
         <f>IF(COUNT(B28,C28)&lt;2,"",B28*C28)</f>
         <v/>
       </c>
-      <c r="E28" s="31" t="n"/>
+      <c r="E28" s="28">
+        <f>SUM(D28:D34)</f>
+        <v/>
+      </c>
       <c r="F28" s="29">
-        <f>IF(OR(D28="",$E$24=""),"",D28/$E$24)</f>
+        <f>IF(OR(D28="",$E$28=""),"",D28/$E$28)</f>
         <v/>
       </c>
       <c r="G28" s="27">
@@ -8603,7 +8603,7 @@
       </c>
       <c r="K28" s="25" t="inlineStr">
         <is>
-          <t>Oeste</t>
+          <t>Noroeste</t>
         </is>
       </c>
       <c r="L28" s="26" t="n"/>
@@ -8613,26 +8613,44 @@
       </c>
     </row>
     <row r="29" ht="17" customHeight="1">
-      <c r="A29" s="25" t="n"/>
-      <c r="B29" s="26" t="n"/>
-      <c r="C29" s="26" t="n"/>
+      <c r="A29" s="25" t="inlineStr">
+        <is>
+          <t>VA02</t>
+        </is>
+      </c>
+      <c r="B29" s="26" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="C29" s="26" t="n">
+        <v>0.75</v>
+      </c>
       <c r="D29" s="27">
         <f>IF(COUNT(B29,C29)&lt;2,"",B29*C29)</f>
         <v/>
       </c>
       <c r="E29" s="31" t="n"/>
       <c r="F29" s="29">
-        <f>IF(OR(D29="",$E$24=""),"",D29/$E$24)</f>
+        <f>IF(OR(D29="",$E$28=""),"",D29/$E$28)</f>
         <v/>
       </c>
       <c r="G29" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H29" s="25" t="n"/>
+      <c r="H29" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
       <c r="I29" s="25" t="n"/>
-      <c r="J29" s="26" t="n"/>
-      <c r="K29" s="25" t="n"/>
+      <c r="J29" s="26" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K29" s="25" t="inlineStr">
+        <is>
+          <t>Noroeste</t>
+        </is>
+      </c>
       <c r="L29" s="26" t="n"/>
       <c r="M29" s="30">
         <f>IF(OR(D29="",J29=""),"",IF(J29&lt;=G29,"CUMPLE","NO CUMPLE"))</f>
@@ -8640,73 +8658,114 @@
       </c>
     </row>
     <row r="30" ht="17" customHeight="1">
-      <c r="A30" s="32" t="n"/>
-      <c r="B30" s="33" t="n"/>
-      <c r="C30" s="33" t="n"/>
-      <c r="D30" s="34">
+      <c r="A30" s="25" t="inlineStr">
+        <is>
+          <t>PA02</t>
+        </is>
+      </c>
+      <c r="B30" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C30" s="26" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D30" s="27">
         <f>IF(COUNT(B30,C30)&lt;2,"",B30*C30)</f>
         <v/>
       </c>
-      <c r="E30" s="35" t="n"/>
-      <c r="F30" s="36">
-        <f>IF(OR(D30="",$E$24=""),"",D30/$E$24)</f>
-        <v/>
-      </c>
-      <c r="G30" s="34">
+      <c r="E30" s="31" t="n"/>
+      <c r="F30" s="29">
+        <f>IF(OR(D30="",$E$28=""),"",D30/$E$28)</f>
+        <v/>
+      </c>
+      <c r="G30" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H30" s="32" t="n"/>
-      <c r="I30" s="32" t="n"/>
-      <c r="J30" s="33" t="n"/>
-      <c r="K30" s="32" t="n"/>
-      <c r="L30" s="33" t="n"/>
-      <c r="M30" s="37">
+      <c r="H30" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I30" s="25" t="n"/>
+      <c r="J30" s="26" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K30" s="25" t="inlineStr">
+        <is>
+          <t>Noroeste</t>
+        </is>
+      </c>
+      <c r="L30" s="26" t="n"/>
+      <c r="M30" s="30">
         <f>IF(OR(D30="",J30=""),"",IF(J30&lt;=G30,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="24" t="inlineStr">
-        <is>
-          <t>Plano: Patio interno (orientacion a confirmar)</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="n"/>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="4" t="n"/>
-      <c r="E31" s="4" t="n"/>
-      <c r="F31" s="4" t="n"/>
-      <c r="G31" s="4" t="n"/>
-      <c r="H31" s="4" t="n"/>
-      <c r="I31" s="4" t="n"/>
-      <c r="J31" s="4" t="n"/>
-      <c r="K31" s="4" t="n"/>
-      <c r="L31" s="4" t="n"/>
-      <c r="M31" s="4" t="n"/>
+    <row r="31" ht="17" customHeight="1">
+      <c r="A31" s="25" t="inlineStr">
+        <is>
+          <t>VA03</t>
+        </is>
+      </c>
+      <c r="B31" s="26" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="C31" s="26" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D31" s="27">
+        <f>IF(COUNT(B31,C31)&lt;2,"",B31*C31)</f>
+        <v/>
+      </c>
+      <c r="E31" s="31" t="n"/>
+      <c r="F31" s="29">
+        <f>IF(OR(D31="",$E$28=""),"",D31/$E$28)</f>
+        <v/>
+      </c>
+      <c r="G31" s="27">
+        <f>Datos_higro!$B$4</f>
+        <v/>
+      </c>
+      <c r="H31" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I31" s="25" t="n"/>
+      <c r="J31" s="26" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K31" s="25" t="inlineStr">
+        <is>
+          <t>Noroeste</t>
+        </is>
+      </c>
+      <c r="L31" s="26" t="n"/>
+      <c r="M31" s="30">
+        <f>IF(OR(D31="",J31=""),"",IF(J31&lt;=G31,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
     </row>
     <row r="32" ht="17" customHeight="1">
       <c r="A32" s="25" t="inlineStr">
         <is>
-          <t>PF01</t>
+          <t>PF05</t>
         </is>
       </c>
       <c r="B32" s="26" t="n">
-        <v>3</v>
+        <v>2.52</v>
       </c>
       <c r="C32" s="26" t="n">
-        <v>3.55</v>
+        <v>0.75</v>
       </c>
       <c r="D32" s="27">
         <f>IF(COUNT(B32,C32)&lt;2,"",B32*C32)</f>
         <v/>
       </c>
-      <c r="E32" s="28">
-        <f>SUM(D32:D37)</f>
-        <v/>
-      </c>
+      <c r="E32" s="31" t="n"/>
       <c r="F32" s="29">
-        <f>IF(OR(D32="",$E$32=""),"",D32/$E$32)</f>
+        <f>IF(OR(D32="",$E$28=""),"",D32/$E$28)</f>
         <v/>
       </c>
       <c r="G32" s="27">
@@ -8722,7 +8781,11 @@
       <c r="J32" s="26" t="n">
         <v>2.8</v>
       </c>
-      <c r="K32" s="25" t="n"/>
+      <c r="K32" s="25" t="inlineStr">
+        <is>
+          <t>Noroeste</t>
+        </is>
+      </c>
       <c r="L32" s="26" t="n"/>
       <c r="M32" s="30">
         <f>IF(OR(D32="",J32=""),"",IF(J32&lt;=G32,"CUMPLE","NO CUMPLE"))</f>
@@ -8730,39 +8793,25 @@
       </c>
     </row>
     <row r="33" ht="17" customHeight="1">
-      <c r="A33" s="25" t="inlineStr">
-        <is>
-          <t>PF02</t>
-        </is>
-      </c>
-      <c r="B33" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="C33" s="26" t="n">
-        <v>3.75</v>
-      </c>
+      <c r="A33" s="25" t="n"/>
+      <c r="B33" s="26" t="n"/>
+      <c r="C33" s="26" t="n"/>
       <c r="D33" s="27">
         <f>IF(COUNT(B33,C33)&lt;2,"",B33*C33)</f>
         <v/>
       </c>
       <c r="E33" s="31" t="n"/>
       <c r="F33" s="29">
-        <f>IF(OR(D33="",$E$32=""),"",D33/$E$32)</f>
+        <f>IF(OR(D33="",$E$28=""),"",D33/$E$28)</f>
         <v/>
       </c>
       <c r="G33" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H33" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
+      <c r="H33" s="25" t="n"/>
       <c r="I33" s="25" t="n"/>
-      <c r="J33" s="26" t="n">
-        <v>2.8</v>
-      </c>
+      <c r="J33" s="26" t="n"/>
       <c r="K33" s="25" t="n"/>
       <c r="L33" s="26" t="n"/>
       <c r="M33" s="30">
@@ -8771,107 +8820,88 @@
       </c>
     </row>
     <row r="34" ht="17" customHeight="1">
-      <c r="A34" s="25" t="inlineStr">
-        <is>
-          <t>PV01</t>
-        </is>
-      </c>
-      <c r="B34" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="C34" s="26" t="n">
-        <v>7.7</v>
-      </c>
-      <c r="D34" s="27">
+      <c r="A34" s="32" t="n"/>
+      <c r="B34" s="33" t="n"/>
+      <c r="C34" s="33" t="n"/>
+      <c r="D34" s="34">
         <f>IF(COUNT(B34,C34)&lt;2,"",B34*C34)</f>
         <v/>
       </c>
-      <c r="E34" s="31" t="n"/>
-      <c r="F34" s="29">
-        <f>IF(OR(D34="",$E$32=""),"",D34/$E$32)</f>
-        <v/>
-      </c>
-      <c r="G34" s="27">
+      <c r="E34" s="35" t="n"/>
+      <c r="F34" s="36">
+        <f>IF(OR(D34="",$E$28=""),"",D34/$E$28)</f>
+        <v/>
+      </c>
+      <c r="G34" s="34">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H34" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I34" s="25" t="n"/>
-      <c r="J34" s="26" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K34" s="25" t="n"/>
-      <c r="L34" s="26" t="n"/>
-      <c r="M34" s="30">
+      <c r="H34" s="32" t="n"/>
+      <c r="I34" s="32" t="n"/>
+      <c r="J34" s="33" t="n"/>
+      <c r="K34" s="32" t="n"/>
+      <c r="L34" s="33" t="n"/>
+      <c r="M34" s="37">
         <f>IF(OR(D34="",J34=""),"",IF(J34&lt;=G34,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="35" ht="17" customHeight="1">
-      <c r="A35" s="25" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="24" t="inlineStr">
+        <is>
+          <t>Plano: Ubicacion a confirmar</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="n"/>
+      <c r="C35" s="4" t="n"/>
+      <c r="D35" s="4" t="n"/>
+      <c r="E35" s="4" t="n"/>
+      <c r="F35" s="4" t="n"/>
+      <c r="G35" s="4" t="n"/>
+      <c r="H35" s="4" t="n"/>
+      <c r="I35" s="4" t="n"/>
+      <c r="J35" s="4" t="n"/>
+      <c r="K35" s="4" t="n"/>
+      <c r="L35" s="4" t="n"/>
+      <c r="M35" s="4" t="n"/>
+    </row>
+    <row r="36" ht="17" customHeight="1">
+      <c r="A36" s="25" t="inlineStr">
         <is>
           <t>PV04 (2)</t>
         </is>
       </c>
-      <c r="B35" s="26" t="n">
+      <c r="B36" s="26" t="n">
         <v>2.95</v>
       </c>
-      <c r="C35" s="26" t="n">
+      <c r="C36" s="26" t="n">
         <v>1.5</v>
       </c>
-      <c r="D35" s="27">
-        <f>IF(COUNT(B35,C35)&lt;2,"",B35*C35)</f>
-        <v/>
-      </c>
-      <c r="E35" s="31" t="n"/>
-      <c r="F35" s="29">
-        <f>IF(OR(D35="",$E$32=""),"",D35/$E$32)</f>
-        <v/>
-      </c>
-      <c r="G35" s="27">
-        <f>Datos_higro!$B$4</f>
-        <v/>
-      </c>
-      <c r="H35" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I35" s="25" t="n"/>
-      <c r="J35" s="26" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K35" s="25" t="n"/>
-      <c r="L35" s="26" t="n"/>
-      <c r="M35" s="30">
-        <f>IF(OR(D35="",J35=""),"",IF(J35&lt;=G35,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="17" customHeight="1">
-      <c r="A36" s="25" t="n"/>
-      <c r="B36" s="26" t="n"/>
-      <c r="C36" s="26" t="n"/>
       <c r="D36" s="27">
         <f>IF(COUNT(B36,C36)&lt;2,"",B36*C36)</f>
         <v/>
       </c>
-      <c r="E36" s="31" t="n"/>
+      <c r="E36" s="28">
+        <f>SUM(D36:D38)</f>
+        <v/>
+      </c>
       <c r="F36" s="29">
-        <f>IF(OR(D36="",$E$32=""),"",D36/$E$32)</f>
+        <f>IF(OR(D36="",$E$36=""),"",D36/$E$36)</f>
         <v/>
       </c>
       <c r="G36" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H36" s="25" t="n"/>
+      <c r="H36" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
       <c r="I36" s="25" t="n"/>
-      <c r="J36" s="26" t="n"/>
+      <c r="J36" s="26" t="n">
+        <v>2.8</v>
+      </c>
       <c r="K36" s="25" t="n"/>
       <c r="L36" s="26" t="n"/>
       <c r="M36" s="30">
@@ -8880,53 +8910,61 @@
       </c>
     </row>
     <row r="37" ht="17" customHeight="1">
-      <c r="A37" s="32" t="n"/>
-      <c r="B37" s="33" t="n"/>
-      <c r="C37" s="33" t="n"/>
-      <c r="D37" s="34">
+      <c r="A37" s="25" t="n"/>
+      <c r="B37" s="26" t="n"/>
+      <c r="C37" s="26" t="n"/>
+      <c r="D37" s="27">
         <f>IF(COUNT(B37,C37)&lt;2,"",B37*C37)</f>
         <v/>
       </c>
-      <c r="E37" s="35" t="n"/>
-      <c r="F37" s="36">
-        <f>IF(OR(D37="",$E$32=""),"",D37/$E$32)</f>
-        <v/>
-      </c>
-      <c r="G37" s="34">
+      <c r="E37" s="31" t="n"/>
+      <c r="F37" s="29">
+        <f>IF(OR(D37="",$E$36=""),"",D37/$E$36)</f>
+        <v/>
+      </c>
+      <c r="G37" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H37" s="32" t="n"/>
-      <c r="I37" s="32" t="n"/>
-      <c r="J37" s="33" t="n"/>
-      <c r="K37" s="32" t="n"/>
-      <c r="L37" s="33" t="n"/>
-      <c r="M37" s="37">
+      <c r="H37" s="25" t="n"/>
+      <c r="I37" s="25" t="n"/>
+      <c r="J37" s="26" t="n"/>
+      <c r="K37" s="25" t="n"/>
+      <c r="L37" s="26" t="n"/>
+      <c r="M37" s="30">
         <f>IF(OR(D37="",J37=""),"",IF(J37&lt;=G37,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="2" t="n"/>
-      <c r="B38" s="2" t="n"/>
-      <c r="C38" s="2" t="n"/>
-      <c r="D38" s="2" t="n"/>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="2" t="n"/>
-      <c r="G38" s="2" t="n"/>
-      <c r="H38" s="2" t="n"/>
-      <c r="I38" s="2" t="n"/>
-      <c r="J38" s="2" t="n"/>
-      <c r="K38" s="2" t="n"/>
-      <c r="L38" s="2" t="n"/>
-      <c r="M38" s="2" t="n"/>
+    <row r="38" ht="17" customHeight="1">
+      <c r="A38" s="32" t="n"/>
+      <c r="B38" s="33" t="n"/>
+      <c r="C38" s="33" t="n"/>
+      <c r="D38" s="34">
+        <f>IF(COUNT(B38,C38)&lt;2,"",B38*C38)</f>
+        <v/>
+      </c>
+      <c r="E38" s="35" t="n"/>
+      <c r="F38" s="36">
+        <f>IF(OR(D38="",$E$36=""),"",D38/$E$36)</f>
+        <v/>
+      </c>
+      <c r="G38" s="34">
+        <f>Datos_higro!$B$4</f>
+        <v/>
+      </c>
+      <c r="H38" s="32" t="n"/>
+      <c r="I38" s="32" t="n"/>
+      <c r="J38" s="33" t="n"/>
+      <c r="K38" s="32" t="n"/>
+      <c r="L38" s="33" t="n"/>
+      <c r="M38" s="37">
+        <f>IF(OR(D38="",J38=""),"",IF(J38&lt;=G38,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="38" t="inlineStr">
-        <is>
-          <t>COMO SE COMPLETA</t>
-        </is>
-      </c>
+      <c r="A39" s="2" t="n"/>
       <c r="B39" s="2" t="n"/>
       <c r="C39" s="2" t="n"/>
       <c r="D39" s="2" t="n"/>
@@ -8941,9 +8979,9 @@
       <c r="M39" s="2" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="39" t="inlineStr">
-        <is>
-          <t>Descripcion, altura y ancho del vano: de la planilla de carpinterias.</t>
+      <c r="A40" s="38" t="inlineStr">
+        <is>
+          <t>COMO SE COMPLETA</t>
         </is>
       </c>
       <c r="B40" s="2" t="n"/>
@@ -8962,7 +9000,7 @@
     <row r="41">
       <c r="A41" s="39" t="inlineStr">
         <is>
-          <t>Area del vano, area total por plano y porcentaje: se calculan solos.</t>
+          <t>Descripcion, altura y ancho del vano: de la planilla de carpinterias.</t>
         </is>
       </c>
       <c r="B41" s="2" t="n"/>
@@ -8981,7 +9019,7 @@
     <row r="42">
       <c r="A42" s="39" t="inlineStr">
         <is>
-          <t>Tipo de vidrio y tipo de proteccion: desplegables; sus valores estan en la hoja Datos_higro.</t>
+          <t>Area del vano, area total por plano y porcentaje: se calculan solos.</t>
         </is>
       </c>
       <c r="B42" s="2" t="n"/>
@@ -9000,7 +9038,7 @@
     <row r="43">
       <c r="A43" s="39" t="inlineStr">
         <is>
-          <t>Transmitancia del cerramiento: cargarla segun el vidrio y el marco adoptados.</t>
+          <t>Tipo de vidrio y tipo de proteccion: desplegables; sus valores estan en la hoja Datos_higro.</t>
         </is>
       </c>
       <c r="B43" s="2" t="n"/>
@@ -9019,7 +9057,7 @@
     <row r="44">
       <c r="A44" s="39" t="inlineStr">
         <is>
-          <t>Orientacion y factor de exposicion solar: el factor depende de la orientacion y de la proteccion.</t>
+          <t>Transmitancia del cerramiento: cargarla segun el vidrio y el marco adoptados.</t>
         </is>
       </c>
       <c r="B44" s="2" t="n"/>
@@ -9036,7 +9074,11 @@
       <c r="M44" s="2" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="39" t="inlineStr"/>
+      <c r="A45" s="39" t="inlineStr">
+        <is>
+          <t>Orientacion y factor de exposicion solar: el factor depende de la orientacion y de la proteccion.</t>
+        </is>
+      </c>
       <c r="B45" s="2" t="n"/>
       <c r="C45" s="2" t="n"/>
       <c r="D45" s="2" t="n"/>
@@ -9051,11 +9093,7 @@
       <c r="M45" s="2" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="39" t="inlineStr">
-        <is>
-          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
-        </is>
-      </c>
+      <c r="A46" s="39" t="inlineStr"/>
       <c r="B46" s="2" t="n"/>
       <c r="C46" s="2" t="n"/>
       <c r="D46" s="2" t="n"/>
@@ -9072,7 +9110,7 @@
     <row r="47">
       <c r="A47" s="39" t="inlineStr">
         <is>
-          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
+          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
         </is>
       </c>
       <c r="B47" s="2" t="n"/>
@@ -9089,7 +9127,11 @@
       <c r="M47" s="2" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="39" t="inlineStr"/>
+      <c r="A48" s="39" t="inlineStr">
+        <is>
+          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
+        </is>
+      </c>
       <c r="B48" s="2" t="n"/>
       <c r="C48" s="2" t="n"/>
       <c r="D48" s="2" t="n"/>
@@ -9104,11 +9146,7 @@
       <c r="M48" s="2" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="39" t="inlineStr">
-        <is>
-          <t>ALTURAS: medidas sobre el dibujo de las vistas de la planilla de carpinterias, con la escala</t>
-        </is>
-      </c>
+      <c r="A49" s="39" t="inlineStr"/>
       <c r="B49" s="2" t="n"/>
       <c r="C49" s="2" t="n"/>
       <c r="D49" s="2" t="n"/>
@@ -9125,7 +9163,7 @@
     <row r="50">
       <c r="A50" s="39" t="inlineStr">
         <is>
-          <t>verificada contra los anchos acotados (error menor a 2 cm). La mayoria de las aberturas son de</t>
+          <t>ALTURAS: medidas sobre el dibujo de las vistas de la planilla de carpinterias, con la escala</t>
         </is>
       </c>
       <c r="B50" s="2" t="n"/>
@@ -9144,7 +9182,7 @@
     <row r="51">
       <c r="A51" s="39" t="inlineStr">
         <is>
-          <t>piso a cielorraso, 3,00 m. VERIFICARLAS contra el plano antes de presentar.</t>
+          <t>verificada contra los anchos acotados (error menor a 2 cm). La mayoria de las aberturas son de</t>
         </is>
       </c>
       <c r="B51" s="2" t="n"/>
@@ -9163,7 +9201,7 @@
     <row r="52">
       <c r="A52" s="39" t="inlineStr">
         <is>
-          <t>PF04 es la unica con antepecho: arranca a 1,09 y mide 0,60 de alto. El resto llega al piso.</t>
+          <t>piso a cielorraso, 3,00 m. VERIFICARLAS contra el plano antes de presentar.</t>
         </is>
       </c>
       <c r="B52" s="2" t="n"/>
@@ -9182,7 +9220,7 @@
     <row r="53">
       <c r="A53" s="39" t="inlineStr">
         <is>
-          <t>Las alturas de PV01 (3,00), PF04 (0,60) y PV04 (2) (2,95) las aporto el autor del proyecto.</t>
+          <t>PF04 es la unica con antepecho: arranca a 1,09 y mide 0,60 de alto. El resto llega al piso.</t>
         </is>
       </c>
       <c r="B53" s="2" t="n"/>
@@ -9199,7 +9237,11 @@
       <c r="M53" s="2" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="39" t="inlineStr"/>
+      <c r="A54" s="39" t="inlineStr">
+        <is>
+          <t>Las alturas de PV01 (3,00), PF04 (0,60) y PV04 (2) (2,95) las aporto el autor del proyecto.</t>
+        </is>
+      </c>
       <c r="B54" s="2" t="n"/>
       <c r="C54" s="2" t="n"/>
       <c r="D54" s="2" t="n"/>
@@ -9214,11 +9256,7 @@
       <c r="M54" s="2" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="39" t="inlineStr">
-        <is>
-          <t>ORIENTACION: el simbolo de norte del plano de plantas (flecha con arco, arriba a la derecha)</t>
-        </is>
-      </c>
+      <c r="A55" s="39" t="inlineStr"/>
       <c r="B55" s="2" t="n"/>
       <c r="C55" s="2" t="n"/>
       <c r="D55" s="2" t="n"/>
@@ -9235,7 +9273,7 @@
     <row r="56">
       <c r="A56" s="39" t="inlineStr">
         <is>
-          <t>apunta hacia la derecha de la hoja. Entonces: derecha = Norte, izquierda = Sur, abajo = Este,</t>
+          <t>ORIENTACION: el simbolo de norte del plano (circulo con aguja, en el patio interno) apunta a</t>
         </is>
       </c>
       <c r="B56" s="2" t="n"/>
@@ -9254,7 +9292,7 @@
     <row r="57">
       <c r="A57" s="39" t="inlineStr">
         <is>
-          <t>arriba = Oeste. Coincide con los rotulos Dormitorio Norte y Dormitorio Sur del plano.</t>
+          <t>45 grados hacia arriba y a la derecha de la hoja. Entonces las cuatro fachadas NO son N-S-E-O</t>
         </is>
       </c>
       <c r="B57" s="2" t="n"/>
@@ -9273,7 +9311,7 @@
     <row r="58">
       <c r="A58" s="39" t="inlineStr">
         <is>
-          <t>Cada abertura se asigno a la fachada por su posicion en planta.</t>
+          <t>sino: arriba = Noroeste, derecha = Noreste, abajo = Sudeste, izquierda = Sudoeste.</t>
         </is>
       </c>
       <c r="B58" s="2" t="n"/>
@@ -9292,7 +9330,7 @@
     <row r="59">
       <c r="A59" s="39" t="inlineStr">
         <is>
-          <t>Las tres aberturas que dan al patio interno quedan en un bloque aparte: hay que confirmar</t>
+          <t>Cada abertura se asigno a la fachada por su posicion en planta. Las del patio interno se</t>
         </is>
       </c>
       <c r="B59" s="2" t="n"/>
@@ -9311,7 +9349,7 @@
     <row r="60">
       <c r="A60" s="39" t="inlineStr">
         <is>
-          <t>a que lado del patio dan antes de asignarles orientacion y factor de exposicion solar.</t>
+          <t>orientan por la pared en la que estan: miran hacia adentro del patio.</t>
         </is>
       </c>
       <c r="B60" s="2" t="n"/>
@@ -9328,7 +9366,11 @@
       <c r="M60" s="2" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="39" t="inlineStr"/>
+      <c r="A61" s="39" t="inlineStr">
+        <is>
+          <t>Los rotulos Dormitorio Norte y Dormitorio Sur del plano no coinciden con el norte real;</t>
+        </is>
+      </c>
       <c r="B61" s="2" t="n"/>
       <c r="C61" s="2" t="n"/>
       <c r="D61" s="2" t="n"/>
@@ -9345,7 +9387,7 @@
     <row r="62">
       <c r="A62" s="39" t="inlineStr">
         <is>
-          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
+          <t>parecen ser nombres de uso, no orientaciones.</t>
         </is>
       </c>
       <c r="B62" s="2" t="n"/>
@@ -9379,7 +9421,7 @@
     <row r="64">
       <c r="A64" s="39" t="inlineStr">
         <is>
-          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
+          <t>PF01 figura dos veces en el plano, en las dos paredes laterales del patio interno, y por eso</t>
         </is>
       </c>
       <c r="B64" s="2" t="n"/>
@@ -9398,7 +9440,7 @@
     <row r="65">
       <c r="A65" s="39" t="inlineStr">
         <is>
-          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
+          <t>se cargan dos filas. Si fuera una sola abertura rotulada dos veces, borrar la segunda.</t>
         </is>
       </c>
       <c r="B65" s="2" t="n"/>
@@ -9415,11 +9457,7 @@
       <c r="M65" s="2" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="39" t="inlineStr">
-        <is>
-          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
-        </is>
-      </c>
+      <c r="A66" s="39" t="inlineStr"/>
       <c r="B66" s="2" t="n"/>
       <c r="C66" s="2" t="n"/>
       <c r="D66" s="2" t="n"/>
@@ -9433,24 +9471,115 @@
       <c r="L66" s="2" t="n"/>
       <c r="M66" s="2" t="n"/>
     </row>
+    <row r="67">
+      <c r="A67" s="39" t="inlineStr">
+        <is>
+          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="n"/>
+      <c r="C67" s="2" t="n"/>
+      <c r="D67" s="2" t="n"/>
+      <c r="E67" s="2" t="n"/>
+      <c r="F67" s="2" t="n"/>
+      <c r="G67" s="2" t="n"/>
+      <c r="H67" s="2" t="n"/>
+      <c r="I67" s="2" t="n"/>
+      <c r="J67" s="2" t="n"/>
+      <c r="K67" s="2" t="n"/>
+      <c r="L67" s="2" t="n"/>
+      <c r="M67" s="2" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="39" t="inlineStr"/>
+      <c r="B68" s="2" t="n"/>
+      <c r="C68" s="2" t="n"/>
+      <c r="D68" s="2" t="n"/>
+      <c r="E68" s="2" t="n"/>
+      <c r="F68" s="2" t="n"/>
+      <c r="G68" s="2" t="n"/>
+      <c r="H68" s="2" t="n"/>
+      <c r="I68" s="2" t="n"/>
+      <c r="J68" s="2" t="n"/>
+      <c r="K68" s="2" t="n"/>
+      <c r="L68" s="2" t="n"/>
+      <c r="M68" s="2" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="39" t="inlineStr">
+        <is>
+          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="n"/>
+      <c r="C69" s="2" t="n"/>
+      <c r="D69" s="2" t="n"/>
+      <c r="E69" s="2" t="n"/>
+      <c r="F69" s="2" t="n"/>
+      <c r="G69" s="2" t="n"/>
+      <c r="H69" s="2" t="n"/>
+      <c r="I69" s="2" t="n"/>
+      <c r="J69" s="2" t="n"/>
+      <c r="K69" s="2" t="n"/>
+      <c r="L69" s="2" t="n"/>
+      <c r="M69" s="2" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="39" t="inlineStr">
+        <is>
+          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="n"/>
+      <c r="C70" s="2" t="n"/>
+      <c r="D70" s="2" t="n"/>
+      <c r="E70" s="2" t="n"/>
+      <c r="F70" s="2" t="n"/>
+      <c r="G70" s="2" t="n"/>
+      <c r="H70" s="2" t="n"/>
+      <c r="I70" s="2" t="n"/>
+      <c r="J70" s="2" t="n"/>
+      <c r="K70" s="2" t="n"/>
+      <c r="L70" s="2" t="n"/>
+      <c r="M70" s="2" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="39" t="inlineStr">
+        <is>
+          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="n"/>
+      <c r="C71" s="2" t="n"/>
+      <c r="D71" s="2" t="n"/>
+      <c r="E71" s="2" t="n"/>
+      <c r="F71" s="2" t="n"/>
+      <c r="G71" s="2" t="n"/>
+      <c r="H71" s="2" t="n"/>
+      <c r="I71" s="2" t="n"/>
+      <c r="J71" s="2" t="n"/>
+      <c r="K71" s="2" t="n"/>
+      <c r="L71" s="2" t="n"/>
+      <c r="M71" s="2" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="E13:E15"/>
-    <mergeCell ref="E32:E37"/>
+    <mergeCell ref="E36:E38"/>
+    <mergeCell ref="A19:M19"/>
+    <mergeCell ref="A14:M14"/>
+    <mergeCell ref="E20:E26"/>
     <mergeCell ref="A1:M1"/>
-    <mergeCell ref="E17:E22"/>
-    <mergeCell ref="E7:E11"/>
-    <mergeCell ref="A23:M23"/>
-    <mergeCell ref="A31:M31"/>
+    <mergeCell ref="A27:M27"/>
+    <mergeCell ref="E28:E34"/>
     <mergeCell ref="A6:M6"/>
-    <mergeCell ref="A12:M12"/>
+    <mergeCell ref="A35:M35"/>
     <mergeCell ref="A4:M4"/>
     <mergeCell ref="A3:M3"/>
-    <mergeCell ref="E24:E30"/>
-    <mergeCell ref="A16:M16"/>
+    <mergeCell ref="E7:E13"/>
+    <mergeCell ref="E15:E18"/>
     <mergeCell ref="A2:M2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M6:M37">
+  <conditionalFormatting sqref="M6:M38">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
       <formula>"CUMPLE"</formula>
     </cfRule>
@@ -9459,13 +9588,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="H6:H37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Datos_higro!$A$8:$A$15</formula1>
     </dataValidation>
-    <dataValidation sqref="I6:I37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I6:I38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Datos_higro!$A$19:$A$25</formula1>
     </dataValidation>
-    <dataValidation sqref="K6:K37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K6:K38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Norte,Sur,Este,Oeste,Noreste,Noroeste,Sudeste,Sudoeste,Horizontal"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Planilla 3: incorporar los maximos de factor de exposicion solar
Se agrega a Datos_higro la tabla de FES maximo por cuadrante de la
Ordenanza 8757/11 (Norte 0,45; Este y Oeste 0,30, modificado a 0,39 por
decreto de 2021; Sur 0,90; lucernarios 0,25) y se resuelve a que
cuadrante cae cada una de las cuatro fachadas de la casa.

Como la casa esta girada 45 grados respecto del norte, ninguna fachada
cae en el cuadrante Norte ni en el Sur: las cuatro entran en el cuadrante
Este/Oeste, que es el mas exigente.

La columna VERIFICACION ahora controla las dos cosas: la transmitancia
contra el maximo admitido y el FES contra el maximo de su cuadrante.
Probado con un FES que cumple (0,25) y uno que no (0,60).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -258,7 +258,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -451,6 +451,9 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -4887,7 +4890,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -5401,6 +5404,296 @@
       <c r="B42" s="2" t="n"/>
       <c r="C42" s="2" t="n"/>
       <c r="D42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n"/>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="72" t="inlineStr">
+        <is>
+          <t>FACTOR DE EXPOSICION SOLAR MAXIMO ADMITIDO  (Ordenanza 8757/11)</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="2" t="n"/>
+      <c r="D44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="59" t="inlineStr">
+        <is>
+          <t>orientacion</t>
+        </is>
+      </c>
+      <c r="B45" s="60" t="inlineStr">
+        <is>
+          <t>FES max</t>
+        </is>
+      </c>
+      <c r="C45" s="60" t="inlineStr">
+        <is>
+          <t>cuadrante</t>
+        </is>
+      </c>
+      <c r="D45" s="59" t="inlineStr">
+        <is>
+          <t>observacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="61" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="B46" s="73" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="C46" s="74" t="inlineStr">
+        <is>
+          <t>341 a 20 grados</t>
+        </is>
+      </c>
+      <c r="D46" s="66" t="inlineStr">
+        <is>
+          <t>Cuadrante Norte (NNE-NNO).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="61" t="inlineStr">
+        <is>
+          <t>Este</t>
+        </is>
+      </c>
+      <c r="B47" s="73" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C47" s="74" t="inlineStr">
+        <is>
+          <t>21 a 160 grados</t>
+        </is>
+      </c>
+      <c r="D47" s="66" t="inlineStr">
+        <is>
+          <t>Modificado a 0,39 por decreto de 2021. Verificar vigencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="61" t="inlineStr">
+        <is>
+          <t>Oeste</t>
+        </is>
+      </c>
+      <c r="B48" s="73" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C48" s="74" t="inlineStr">
+        <is>
+          <t>201 a 340 grados</t>
+        </is>
+      </c>
+      <c r="D48" s="66" t="inlineStr">
+        <is>
+          <t>Modificado a 0,39 por decreto de 2021. Verificar vigencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="61" t="inlineStr">
+        <is>
+          <t>Sur</t>
+        </is>
+      </c>
+      <c r="B49" s="73" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C49" s="74" t="inlineStr">
+        <is>
+          <t>161 a 200 grados</t>
+        </is>
+      </c>
+      <c r="D49" s="66" t="inlineStr">
+        <is>
+          <t>Cuadrante Sur (SSE-SSO).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="61" t="inlineStr">
+        <is>
+          <t>Noreste</t>
+        </is>
+      </c>
+      <c r="B50" s="73" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C50" s="74" t="inlineStr">
+        <is>
+          <t>cae en cuadrante Este</t>
+        </is>
+      </c>
+      <c r="D50" s="66" t="inlineStr">
+        <is>
+          <t>45 grados: entra en el cuadrante Este (21 a 160).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="61" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="B51" s="73" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C51" s="74" t="inlineStr">
+        <is>
+          <t>cae en cuadrante Este</t>
+        </is>
+      </c>
+      <c r="D51" s="66" t="inlineStr">
+        <is>
+          <t>135 grados: entra en el cuadrante Este (21 a 160).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="61" t="inlineStr">
+        <is>
+          <t>Sudoeste</t>
+        </is>
+      </c>
+      <c r="B52" s="73" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C52" s="74" t="inlineStr">
+        <is>
+          <t>cae en cuadrante Oeste</t>
+        </is>
+      </c>
+      <c r="D52" s="66" t="inlineStr">
+        <is>
+          <t>225 grados: entra en el cuadrante Oeste (201 a 340).</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="61" t="inlineStr">
+        <is>
+          <t>Noroeste</t>
+        </is>
+      </c>
+      <c r="B53" s="73" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C53" s="74" t="inlineStr">
+        <is>
+          <t>cae en cuadrante Oeste</t>
+        </is>
+      </c>
+      <c r="D53" s="66" t="inlineStr">
+        <is>
+          <t>315 grados: entra en el cuadrante Oeste (201 a 340).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="61" t="inlineStr">
+        <is>
+          <t>Horizontal</t>
+        </is>
+      </c>
+      <c r="B54" s="73" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C54" s="74" t="inlineStr">
+        <is>
+          <t>lucernarios</t>
+        </is>
+      </c>
+      <c r="D54" s="66" t="inlineStr">
+        <is>
+          <t>Planos inclinados con angulo menor a 60 grados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n"/>
+      <c r="B55" s="2" t="n"/>
+      <c r="C55" s="2" t="n"/>
+      <c r="D55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="38" t="inlineStr">
+        <is>
+          <t>La casa esta girada 45 grados respecto del norte, asi que NINGUNA de sus cuatro fachadas</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="n"/>
+      <c r="C56" s="2" t="n"/>
+      <c r="D56" s="2" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="39" t="inlineStr">
+        <is>
+          <t>cae en el cuadrante Norte ni en el Sur: las cuatro entran en el cuadrante Este/Oeste, que es</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="n"/>
+      <c r="C57" s="2" t="n"/>
+      <c r="D57" s="2" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="39" t="inlineStr">
+        <is>
+          <t>el mas exigente (0,30, o 0,39 segun la modificacion de 2021). Conviene confirmarlo en la</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="n"/>
+      <c r="C58" s="2" t="n"/>
+      <c r="D58" s="2" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="39" t="inlineStr">
+        <is>
+          <t>Secretaria de Planeamiento antes de presentar: hay versiones distintas dando vueltas.</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="n"/>
+      <c r="C59" s="2" t="n"/>
+      <c r="D59" s="2" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n"/>
+      <c r="B60" s="2" t="n"/>
+      <c r="C60" s="2" t="n"/>
+      <c r="D60" s="2" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="38" t="inlineStr">
+        <is>
+          <t>Si la abertura ocupa menos del 20% del lado expuesto del local, NO hay que verificar el FES</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="n"/>
+      <c r="C61" s="2" t="n"/>
+      <c r="D61" s="2" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="39" t="inlineStr">
+        <is>
+          <t>(si la transmitancia). Fuente: preguntas frecuentes de la Secretaria de Planeamiento.</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="n"/>
+      <c r="C62" s="2" t="n"/>
+      <c r="D62" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5421,180 +5714,180 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="74" t="inlineStr">
+      <c r="A1" s="75" t="inlineStr">
         <is>
           <t>MEMORIA - ILUMINACION Y VENTILACION</t>
         </is>
       </c>
-      <c r="B1" s="75" t="inlineStr"/>
+      <c r="B1" s="76" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="75" t="inlineStr"/>
-      <c r="B2" s="76" t="inlineStr"/>
+      <c r="A2" s="76" t="inlineStr"/>
+      <c r="B2" s="77" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="75" t="inlineStr">
+      <c r="A3" s="76" t="inlineStr">
         <is>
           <t>CRITERIO</t>
         </is>
       </c>
-      <c r="B3" s="75" t="inlineStr">
+      <c r="B3" s="76" t="inlineStr">
         <is>
           <t>Area de iluminacion requerida = superficie del local / 9</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="75" t="inlineStr"/>
-      <c r="B4" s="76" t="inlineStr">
+      <c r="A4" s="76" t="inlineStr"/>
+      <c r="B4" s="77" t="inlineStr">
         <is>
           <t>Area de ventilacion requerida = un tercio de la de iluminacion = superficie / 27</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="75" t="inlineStr"/>
-      <c r="B5" s="76" t="inlineStr">
+      <c r="A5" s="76" t="inlineStr"/>
+      <c r="B5" s="77" t="inlineStr">
         <is>
           <t>Area proyectada: la vidriada de la carpinteria para iluminacion, y la parte que</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="75" t="inlineStr"/>
-      <c r="B6" s="76" t="inlineStr">
+      <c r="A6" s="76" t="inlineStr"/>
+      <c r="B6" s="77" t="inlineStr">
         <is>
           <t>realmente abre para ventilacion.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="75" t="inlineStr"/>
-      <c r="B7" s="76" t="inlineStr"/>
+      <c r="A7" s="76" t="inlineStr"/>
+      <c r="B7" s="77" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="75" t="inlineStr">
+      <c r="A8" s="76" t="inlineStr">
         <is>
           <t>RESULTADO</t>
         </is>
       </c>
-      <c r="B8" s="75" t="inlineStr">
+      <c r="B8" s="76" t="inlineStr">
         <is>
           <t>Los trece locales cumplen holgadamente iluminacion y ventilacion.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="75" t="inlineStr"/>
-      <c r="B9" s="76" t="inlineStr"/>
+      <c r="A9" s="76" t="inlineStr"/>
+      <c r="B9" s="77" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="75" t="inlineStr">
+      <c r="A10" s="76" t="inlineStr">
         <is>
           <t>CORRECCION</t>
         </is>
       </c>
-      <c r="B10" s="75" t="inlineStr">
+      <c r="B10" s="76" t="inlineStr">
         <is>
           <t>Local 07, Hall / ingreso: la planilla original traia 0,66 y 0,22, que son los</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="75" t="inlineStr"/>
-      <c r="B11" s="76" t="inlineStr">
+      <c r="A11" s="76" t="inlineStr"/>
+      <c r="B11" s="77" t="inlineStr">
         <is>
           <t>valores del local 03 (Lavadero, 6,0 m2). Con sus 3,50 x 2,15 = 7,53 m2 corresponden</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="75" t="inlineStr"/>
-      <c r="B12" s="76" t="inlineStr">
+      <c r="A12" s="76" t="inlineStr"/>
+      <c r="B12" s="77" t="inlineStr">
         <is>
           <t>0,84 y 0,28. No cambia el resultado, pero el numero no cerraba con la superficie</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="75" t="inlineStr"/>
-      <c r="B13" s="76" t="inlineStr">
+      <c r="A13" s="76" t="inlineStr"/>
+      <c r="B13" s="77" t="inlineStr">
         <is>
           <t>declarada y un verificador lo puede observar.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="75" t="inlineStr"/>
-      <c r="B14" s="76" t="inlineStr"/>
+      <c r="A14" s="76" t="inlineStr"/>
+      <c r="B14" s="77" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="75" t="inlineStr">
+      <c r="A15" s="76" t="inlineStr">
         <is>
           <t>A REVISAR</t>
         </is>
       </c>
-      <c r="B15" s="75" t="inlineStr">
+      <c r="B15" s="76" t="inlineStr">
         <is>
           <t>Local 14, Estar / Playroom: declara 5,00 m2 de ventilacion sobre 5,00 m2 de</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="75" t="inlineStr"/>
-      <c r="B16" s="76" t="inlineStr">
+      <c r="A16" s="76" t="inlineStr"/>
+      <c r="B16" s="77" t="inlineStr">
         <is>
           <t>iluminacion, es decir una carpinteria enteramente abrible. En los demas locales</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="75" t="inlineStr"/>
-      <c r="B17" s="76" t="inlineStr">
+      <c r="A17" s="76" t="inlineStr"/>
+      <c r="B17" s="77" t="inlineStr">
         <is>
           <t>la relacion es del 50 por ciento. Conviene verificar la carpinteria real.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="75" t="inlineStr"/>
-      <c r="B18" s="76" t="inlineStr"/>
+      <c r="A18" s="76" t="inlineStr"/>
+      <c r="B18" s="77" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="75" t="inlineStr"/>
-      <c r="B19" s="76" t="inlineStr">
+      <c r="A19" s="76" t="inlineStr"/>
+      <c r="B19" s="77" t="inlineStr">
         <is>
           <t>Local 02, Deposito: figura sin exigencia por no ser habitable. Son 11,8 m2</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="75" t="inlineStr"/>
-      <c r="B20" s="76" t="inlineStr">
+      <c r="A20" s="76" t="inlineStr"/>
+      <c r="B20" s="77" t="inlineStr">
         <is>
           <t>cerrados: si se lo considera habitable hay que preverle conducto.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="75" t="inlineStr"/>
-      <c r="B21" s="76" t="inlineStr"/>
+      <c r="A21" s="76" t="inlineStr"/>
+      <c r="B21" s="77" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="75" t="inlineStr">
+      <c r="A22" s="76" t="inlineStr">
         <is>
           <t>REDONDEOS</t>
         </is>
       </c>
-      <c r="B22" s="75" t="inlineStr">
+      <c r="B22" s="76" t="inlineStr">
         <is>
           <t>Diferencias menores que no afectan: local 03 da 5,95 m2 y figura 6,0;</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="75" t="inlineStr"/>
-      <c r="B23" s="76" t="inlineStr">
+      <c r="A23" s="76" t="inlineStr"/>
+      <c r="B23" s="77" t="inlineStr">
         <is>
           <t>local 09 da 12,25 y figura 12,3.</t>
         </is>
@@ -5619,592 +5912,592 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="74" t="inlineStr">
+      <c r="A1" s="75" t="inlineStr">
         <is>
           <t>MEMORIA DE CALCULO - VIGAS H°A°</t>
         </is>
       </c>
-      <c r="B1" s="75" t="inlineStr"/>
+      <c r="B1" s="76" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="75" t="inlineStr"/>
-      <c r="B2" s="76" t="inlineStr"/>
+      <c r="A2" s="76" t="inlineStr"/>
+      <c r="B2" s="77" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="75" t="inlineStr">
+      <c r="A3" s="76" t="inlineStr">
         <is>
           <t>NORMATIVA</t>
         </is>
       </c>
-      <c r="B3" s="75" t="inlineStr">
+      <c r="B3" s="76" t="inlineStr">
         <is>
           <t>CIRSOC 201. Hormigon H-21 (f'c 210 kg/cm2). Acero 42/50 (fy 4200 kg/cm2).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="75" t="inlineStr">
+      <c r="A4" s="76" t="inlineStr">
         <is>
           <t>UNIDADES</t>
         </is>
       </c>
-      <c r="B4" s="75" t="inlineStr">
+      <c r="B4" s="76" t="inlineStr">
         <is>
           <t>Longitudes en m y cm. Cargas en kg/m. Momentos en kgm. Tensiones en kg/cm2.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="75" t="inlineStr">
+      <c r="A5" s="76" t="inlineStr">
         <is>
           <t>DIMENSIONES</t>
         </is>
       </c>
-      <c r="B5" s="75" t="inlineStr">
+      <c r="B5" s="76" t="inlineStr">
         <is>
           <t>b = ancho | h = altura util | d = altura total (igual criterio que la planilla de catedra).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="75" t="inlineStr"/>
-      <c r="B6" s="76" t="inlineStr"/>
+      <c r="A6" s="76" t="inlineStr"/>
+      <c r="B6" s="77" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="75" t="inlineStr">
+      <c r="A7" s="76" t="inlineStr">
         <is>
           <t>1. CARGAS</t>
         </is>
       </c>
-      <c r="B7" s="75" t="inlineStr"/>
+      <c r="B7" s="76" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="75" t="inlineStr">
+      <c r="A8" s="76" t="inlineStr">
         <is>
           <t>Entrepiso PA</t>
         </is>
       </c>
-      <c r="B8" s="76" t="inlineStr">
+      <c r="B8" s="77" t="inlineStr">
         <is>
           <t>Losa maciza 12 cm 300 + contrapiso 130 + carpeta 42 + piso 50 + cielorraso 20</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="75" t="inlineStr"/>
-      <c r="B9" s="76" t="inlineStr">
+      <c r="A9" s="76" t="inlineStr"/>
+      <c r="B9" s="77" t="inlineStr">
         <is>
           <t>g = 550 kg/m2       q = 200 kg/m2 (vivienda)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="75" t="inlineStr">
+      <c r="A10" s="76" t="inlineStr">
         <is>
           <t>Azotea</t>
         </is>
       </c>
-      <c r="B10" s="76" t="inlineStr">
+      <c r="B10" s="77" t="inlineStr">
         <is>
           <t>Losa 300 + contrapiso de pendiente 140 + carpeta 42 + aislacion y membrana 50 + cielorraso 20</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="75" t="inlineStr"/>
-      <c r="B11" s="76" t="inlineStr">
+      <c r="A11" s="76" t="inlineStr"/>
+      <c r="B11" s="77" t="inlineStr">
         <is>
           <t>g = 560 kg/m2       q = 100 kg/m2 (cubierta no accesible)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="75" t="inlineStr">
+      <c r="A12" s="76" t="inlineStr">
         <is>
           <t>Mamposteria</t>
         </is>
       </c>
-      <c r="B12" s="76" t="inlineStr">
+      <c r="B12" s="77" t="inlineStr">
         <is>
           <t>250 kg/m2. Altura 2,60 m en PA y 1,00 m de parapeto en azotea.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="75" t="inlineStr">
+      <c r="A13" s="76" t="inlineStr">
         <is>
           <t>Peso propio</t>
         </is>
       </c>
-      <c r="B13" s="76" t="inlineStr">
+      <c r="B13" s="77" t="inlineStr">
         <is>
           <t>2400 kg/m3 x b x d, viga por viga.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="75" t="inlineStr">
+      <c r="A14" s="76" t="inlineStr">
         <is>
           <t>Carga de calculo</t>
         </is>
       </c>
-      <c r="B14" s="76" t="inlineStr">
+      <c r="B14" s="77" t="inlineStr">
         <is>
           <t>p = 1,2 (g x B + peso propio + muro) + 1,6 (q x B)        B = ancho tributario</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="75" t="inlineStr"/>
-      <c r="B15" s="76" t="inlineStr"/>
+      <c r="A15" s="76" t="inlineStr"/>
+      <c r="B15" s="77" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="75" t="inlineStr">
+      <c r="A16" s="76" t="inlineStr">
         <is>
           <t>2. SOLICITACIONES</t>
         </is>
       </c>
-      <c r="B16" s="75" t="inlineStr">
+      <c r="B16" s="76" t="inlineStr">
         <is>
           <t>Coeficientes segun esquema (tabla en hoja Datos):</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="75" t="inlineStr"/>
-      <c r="B17" s="76" t="inlineStr">
+      <c r="A17" s="76" t="inlineStr"/>
+      <c r="B17" s="77" t="inlineStr">
         <is>
           <t xml:space="preserve">  Simplemente apoyada   M = pL2/8                    R = 0,500 pL</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="75" t="inlineStr"/>
-      <c r="B18" s="76" t="inlineStr">
+      <c r="A18" s="76" t="inlineStr"/>
+      <c r="B18" s="77" t="inlineStr">
         <is>
           <t xml:space="preserve">  Continua              M = pL2/14   Mapoyo = pL2/10  R = 0,575 pL</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="75" t="inlineStr"/>
-      <c r="B19" s="76" t="inlineStr">
+      <c r="A19" s="76" t="inlineStr"/>
+      <c r="B19" s="77" t="inlineStr">
         <is>
           <t xml:space="preserve">  Empotrada-apoyada     M = 9pL2/128 Mapoyo = pL2/8   R = 0,625 pL</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="75" t="inlineStr"/>
-      <c r="B20" s="76" t="inlineStr">
+      <c r="A20" s="76" t="inlineStr"/>
+      <c r="B20" s="77" t="inlineStr">
         <is>
           <t xml:space="preserve">  Biempotrada           M = pL2/24   Mapoyo = pL2/12  R = 0,500 pL</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="75" t="inlineStr"/>
-      <c r="B21" s="76" t="inlineStr">
+      <c r="A21" s="76" t="inlineStr"/>
+      <c r="B21" s="77" t="inlineStr">
         <is>
           <t xml:space="preserve">  Voladizo                           Mapoyo = pL2/2   R = 1,000 pL</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="75" t="inlineStr"/>
-      <c r="B22" s="76" t="inlineStr"/>
+      <c r="A22" s="76" t="inlineStr"/>
+      <c r="B22" s="77" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="75" t="inlineStr">
+      <c r="A23" s="76" t="inlineStr">
         <is>
           <t>3. FLEXION</t>
         </is>
       </c>
-      <c r="B23" s="75" t="inlineStr">
+      <c r="B23" s="76" t="inlineStr">
         <is>
           <t>k = M / (phi b h2 f'c)      w = 1 - RAIZ(1 - 2k)      As = w b h f'c / fy</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="75" t="inlineStr"/>
-      <c r="B24" s="76" t="inlineStr">
+      <c r="A24" s="76" t="inlineStr"/>
+      <c r="B24" s="77" t="inlineStr">
         <is>
           <t>As min = 0,0033 b h       As max = 0,0163 b h (0,75 de la cuantia balanceada)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="75" t="inlineStr"/>
-      <c r="B25" s="76" t="inlineStr">
+      <c r="A25" s="76" t="inlineStr"/>
+      <c r="B25" s="77" t="inlineStr">
         <is>
           <t>Si la armadura no entra en una capa se disponen dos y el recubrimiento pasa a 6 cm.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="75" t="inlineStr"/>
-      <c r="B26" s="76" t="inlineStr"/>
+      <c r="A26" s="76" t="inlineStr"/>
+      <c r="B26" s="77" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="75" t="inlineStr">
+      <c r="A27" s="76" t="inlineStr">
         <is>
           <t>4. CORTE</t>
         </is>
       </c>
-      <c r="B27" s="75" t="inlineStr">
+      <c r="B27" s="76" t="inlineStr">
         <is>
           <t>T = R / (b x 0,85 h)       tension tangencial en el apoyo</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="75" t="inlineStr"/>
-      <c r="B28" s="76" t="inlineStr">
+      <c r="A28" s="76" t="inlineStr"/>
+      <c r="B28" s="77" t="inlineStr">
         <is>
           <t>Vc = 0,53 RAIZ(f'c) b h        phi Vn = 0,75 (Vc + Av fy h / s)  &gt;=  R</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="75" t="inlineStr"/>
-      <c r="B29" s="76" t="inlineStr">
+      <c r="A29" s="76" t="inlineStr"/>
+      <c r="B29" s="77" t="inlineStr">
         <is>
           <t>Av = 2 ramas. Se aumenta el diametro antes que cerrar la separacion por debajo de 10 cm.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="75" t="inlineStr"/>
-      <c r="B30" s="76" t="inlineStr"/>
+      <c r="A30" s="76" t="inlineStr"/>
+      <c r="B30" s="77" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="75" t="inlineStr">
+      <c r="A31" s="76" t="inlineStr">
         <is>
           <t>5. FLECHA</t>
         </is>
       </c>
-      <c r="B31" s="75" t="inlineStr">
+      <c r="B31" s="76" t="inlineStr">
         <is>
           <t>Altura minima: simplemente apoyada L/16, un extremo continuo L/18,5,</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="75" t="inlineStr"/>
-      <c r="B32" s="76" t="inlineStr">
+      <c r="A32" s="76" t="inlineStr"/>
+      <c r="B32" s="77" t="inlineStr">
         <is>
           <t>ambos extremos continuos L/21, voladizo L/8.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="75" t="inlineStr"/>
-      <c r="B33" s="76" t="inlineStr"/>
+      <c r="A33" s="76" t="inlineStr"/>
+      <c r="B33" s="77" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="75" t="inlineStr">
+      <c r="A34" s="76" t="inlineStr">
         <is>
           <t>6. VIGAS INVERTIDAS</t>
         </is>
       </c>
-      <c r="B34" s="75" t="inlineStr">
+      <c r="B34" s="76" t="inlineStr">
         <is>
           <t>Las vigas de BORDE son invertidas: sobresalen 70 cm por encima del fondo de</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="75" t="inlineStr"/>
-      <c r="B35" s="76" t="inlineStr">
+      <c r="A35" s="76" t="inlineStr"/>
+      <c r="B35" s="77" t="inlineStr">
         <is>
           <t>losa (cotas N.F.L +3,50 / N.S.V +4,20 y N.F.L +6,80 / N.S.V +7,50 del plano).</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="75" t="inlineStr"/>
-      <c r="B36" s="76" t="inlineStr">
+      <c r="A36" s="76" t="inlineStr"/>
+      <c r="B36" s="77" t="inlineStr">
         <is>
           <t>losa. Lo confirman las cotas del plano y el hecho de que el cielorraso sea de</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="75" t="inlineStr"/>
-      <c r="B37" s="76" t="inlineStr">
+      <c r="A37" s="76" t="inlineStr"/>
+      <c r="B37" s="77" t="inlineStr">
         <is>
           <t>VI 06 mide 14,00 m en total y es el cuarto borde de L07. Sobre su eje hay cuatro</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="75" t="inlineStr"/>
-      <c r="B38" s="76" t="inlineStr">
+      <c r="A38" s="76" t="inlineStr"/>
+      <c r="B38" s="77" t="inlineStr">
         <is>
           <t>columnas, de modo que trabaja como viga continua de tres tramos de 4,10, 4,32 y</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="75" t="inlineStr"/>
-      <c r="B39" s="76" t="inlineStr">
+      <c r="A39" s="76" t="inlineStr"/>
+      <c r="B39" s="77" t="inlineStr">
         <is>
           <t>6,53 m. Se calcula con el mayor, 6,53 m, que es el que gobierna.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="75" t="inlineStr"/>
-      <c r="B40" s="76" t="inlineStr">
+      <c r="A40" s="76" t="inlineStr"/>
+      <c r="B40" s="77" t="inlineStr">
         <is>
           <t>hormigon visto: una viga colgante quedaria a la vista. El computo metrico las</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="75" t="inlineStr"/>
-      <c r="B41" s="76" t="inlineStr">
+      <c r="A41" s="76" t="inlineStr"/>
+      <c r="B41" s="77" t="inlineStr">
         <is>
           <t>agrupa a las 28 bajo el rubro Vigas invertidas 15x70.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="75" t="inlineStr"/>
-      <c r="B42" s="76" t="inlineStr">
+      <c r="A42" s="76" t="inlineStr"/>
+      <c r="B42" s="77" t="inlineStr">
         <is>
           <t>Esto define donde la losa aporta ala comprimida:</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="75" t="inlineStr"/>
-      <c r="B43" s="76" t="inlineStr">
+      <c r="A43" s="76" t="inlineStr"/>
+      <c r="B43" s="77" t="inlineStr">
         <is>
           <t xml:space="preserve">  viga COLGANTE  -&gt; la losa esta arriba  -&gt; ala util en el TRAMO (momento positivo)</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="75" t="inlineStr"/>
-      <c r="B44" s="76" t="inlineStr">
+      <c r="A44" s="76" t="inlineStr"/>
+      <c r="B44" s="77" t="inlineStr">
         <is>
           <t xml:space="preserve">  viga INVERTIDA -&gt; la losa esta abajo   -&gt; ala util en el APOYO (momento negativo)</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="75" t="inlineStr"/>
-      <c r="B45" s="76" t="inlineStr">
+      <c r="A45" s="76" t="inlineStr"/>
+      <c r="B45" s="77" t="inlineStr">
         <is>
           <t>En la zona con ala se adopta b efectivo = min(L/4 ; b + 16 hf); en la otra, la</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="75" t="inlineStr"/>
-      <c r="B46" s="76" t="inlineStr">
+      <c r="A46" s="76" t="inlineStr"/>
+      <c r="B46" s="77" t="inlineStr">
         <is>
           <t>seccion es rectangular de ancho b. Las columnas b ef tramo y b ef apoyo lo muestran.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="75" t="inlineStr"/>
-      <c r="B47" s="76" t="inlineStr">
+      <c r="A47" s="76" t="inlineStr"/>
+      <c r="B47" s="77" t="inlineStr">
         <is>
           <t>PENDIENTE: las invertidas de BORDE (VI 01a, 01b, 07a, 07b, 07c, 11a, 11b, 11c,</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="75" t="inlineStr"/>
-      <c r="B48" s="76" t="inlineStr">
+      <c r="A48" s="76" t="inlineStr"/>
+      <c r="B48" s="77" t="inlineStr">
         <is>
           <t>15a y 15b) reciben la reaccion de la losa de un solo lado, excentrica respecto</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="75" t="inlineStr"/>
-      <c r="B49" s="76" t="inlineStr">
+      <c r="A49" s="76" t="inlineStr"/>
+      <c r="B49" s="77" t="inlineStr">
         <is>
           <t>de su eje, y quedan sometidas a TORSION. Esta planilla no la verifica.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="75" t="inlineStr"/>
-      <c r="B50" s="76" t="inlineStr"/>
+      <c r="A50" s="76" t="inlineStr"/>
+      <c r="B50" s="77" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="75" t="inlineStr">
+      <c r="A51" s="76" t="inlineStr">
         <is>
           <t>7. RESULTADO</t>
         </is>
       </c>
-      <c r="B51" s="75" t="inlineStr">
+      <c r="B51" s="76" t="inlineStr">
         <is>
           <t>30 vigas: 21 del entrepiso PA y 9 de la losa de techo. 28 verifican.</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="75" t="inlineStr"/>
-      <c r="B52" s="76" t="inlineStr">
+      <c r="A52" s="76" t="inlineStr"/>
+      <c r="B52" s="77" t="inlineStr">
         <is>
           <t>VI 02 (15x60, 9,88 m): recibe L02 y L03, B = 2,88 m. La armadura de apoyo</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="75" t="inlineStr"/>
-      <c r="B53" s="76" t="inlineStr">
+      <c r="A53" s="76" t="inlineStr"/>
+      <c r="B53" s="77" t="inlineStr">
         <is>
           <t xml:space="preserve">   necesaria ronda los 25 cm2 y supera la cuantia maxima. Los apoyos estan</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="75" t="inlineStr"/>
-      <c r="B54" s="76" t="inlineStr">
+      <c r="A54" s="76" t="inlineStr"/>
+      <c r="B54" s="77" t="inlineStr">
         <is>
           <t xml:space="preserve">   confirmados en obra: tabique T07 perpendicular arriba y COL 02 abajo, sin apoyo</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="75" t="inlineStr"/>
-      <c r="B55" s="76" t="inlineStr">
+      <c r="A55" s="76" t="inlineStr"/>
+      <c r="B55" s="77" t="inlineStr">
         <is>
           <t xml:space="preserve">   intermedio. Para esta carga la seccion necesaria es 15x75.</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="75" t="inlineStr"/>
-      <c r="B56" s="76" t="inlineStr">
+      <c r="A56" s="76" t="inlineStr"/>
+      <c r="B56" s="77" t="inlineStr">
         <is>
           <t>VCH 03a (40x13, 3,83 m). Recibe L03, B = 2,08 m, y no</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="75" t="inlineStr"/>
-      <c r="B57" s="76" t="inlineStr">
+      <c r="A57" s="76" t="inlineStr"/>
+      <c r="B57" s="77" t="inlineStr">
         <is>
           <t xml:space="preserve">   verifica: haria falta mas espesor. Tampoco verifica con B = 0,60 m, asi</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="75" t="inlineStr"/>
-      <c r="B58" s="76" t="inlineStr">
+      <c r="A58" s="76" t="inlineStr"/>
+      <c r="B58" s="77" t="inlineStr">
         <is>
           <t xml:space="preserve">   que el problema no es la hipotesis de carga sino la relacion luz/espesor. Una viga</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="75" t="inlineStr"/>
-      <c r="B59" s="76" t="inlineStr">
+      <c r="A59" s="76" t="inlineStr"/>
+      <c r="B59" s="77" t="inlineStr">
         <is>
           <t xml:space="preserve">   chata del mismo espesor que la losa no puede ser apoyo lineal de un pano de 4,15 m.</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="75" t="inlineStr"/>
-      <c r="B60" s="76" t="inlineStr">
+      <c r="A60" s="76" t="inlineStr"/>
+      <c r="B60" s="77" t="inlineStr">
         <is>
           <t xml:space="preserve">   Revisar si tiene un muro debajo que acorte su luz libre.</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="75" t="inlineStr"/>
-      <c r="B61" s="76" t="inlineStr">
+      <c r="A61" s="76" t="inlineStr"/>
+      <c r="B61" s="77" t="inlineStr">
         <is>
           <t>VCH 03a (40x13, 3,71 m): excede la cuantia maxima y no llega a la altura minima por</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="75" t="inlineStr"/>
-      <c r="B62" s="76" t="inlineStr">
+      <c r="A62" s="76" t="inlineStr"/>
+      <c r="B62" s="77" t="inlineStr">
         <is>
           <t xml:space="preserve">   flecha. Revisar el ancho tributario: si solo recibe el muro y no losa, baja mucho.</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="75" t="inlineStr"/>
-      <c r="B63" s="76" t="inlineStr"/>
+      <c r="A63" s="76" t="inlineStr"/>
+      <c r="B63" s="77" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="75" t="inlineStr">
+      <c r="A64" s="76" t="inlineStr">
         <is>
           <t>8. ALCANCE</t>
         </is>
       </c>
-      <c r="B64" s="76" t="inlineStr">
+      <c r="B64" s="77" t="inlineStr">
         <is>
           <t>No se incluyen las 31 vigas de fundacion (VF01 a VF18c): su calculo depende de las</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="75" t="inlineStr"/>
-      <c r="B65" s="76" t="inlineStr">
+      <c r="A65" s="76" t="inlineStr"/>
+      <c r="B65" s="77" t="inlineStr">
         <is>
           <t>cargas que bajan por las columnas y corresponde hacerlo despues. Tampoco losas ni columnas.</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="75" t="inlineStr"/>
-      <c r="B66" s="76" t="inlineStr"/>
+      <c r="A66" s="76" t="inlineStr"/>
+      <c r="B66" s="77" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="75" t="inlineStr">
+      <c r="A67" s="76" t="inlineStr">
         <is>
           <t>LIMITACIONES</t>
         </is>
       </c>
-      <c r="B67" s="75" t="inlineStr">
+      <c r="B67" s="76" t="inlineStr">
         <is>
           <t>El ancho tributario B esta relevado solo en</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="75" t="inlineStr"/>
-      <c r="B68" s="76" t="inlineStr">
+      <c r="A68" s="76" t="inlineStr"/>
+      <c r="B68" s="77" t="inlineStr">
         <is>
           <t>VI 02 (0,80 m) y VCH 03a (2,08 m). En las demas sigue adoptado en 2,00 m, a falta</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="75" t="inlineStr"/>
-      <c r="B69" s="76" t="inlineStr">
+      <c r="A69" s="76" t="inlineStr"/>
+      <c r="B69" s="77" t="inlineStr">
         <is>
           <t>hipotesis mas influyente del calculo: ajustarla viga por viga en la columna B trib.</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="75" t="inlineStr"/>
-      <c r="B70" s="76" t="inlineStr">
+      <c r="A70" s="76" t="inlineStr"/>
+      <c r="B70" s="77" t="inlineStr">
         <is>
           <t>El esquema se asigno por criterio: continua si integra una serie a-b-c o si supera 5,5 m.</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="75" t="inlineStr"/>
-      <c r="B71" s="76" t="inlineStr">
+      <c r="A71" s="76" t="inlineStr"/>
+      <c r="B71" s="77" t="inlineStr">
         <is>
           <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
         </is>
@@ -6229,368 +6522,368 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="74" t="inlineStr">
+      <c r="A1" s="75" t="inlineStr">
         <is>
           <t>MEMORIA DE CALCULO - LOSAS</t>
         </is>
       </c>
-      <c r="B1" s="75" t="inlineStr"/>
+      <c r="B1" s="76" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="75" t="inlineStr"/>
-      <c r="B2" s="76" t="inlineStr"/>
+      <c r="A2" s="76" t="inlineStr"/>
+      <c r="B2" s="77" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="75" t="inlineStr">
+      <c r="A3" s="76" t="inlineStr">
         <is>
           <t>METODO</t>
         </is>
       </c>
-      <c r="B3" s="75" t="inlineStr">
+      <c r="B3" s="76" t="inlineStr">
         <is>
           <t>Tensiones admisibles, igual criterio que la planilla modelo de la catedra.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="75" t="inlineStr"/>
-      <c r="B4" s="76" t="inlineStr">
+      <c r="A4" s="76" t="inlineStr"/>
+      <c r="B4" s="77" t="inlineStr">
         <is>
           <t>Se verifico contra la fila de ejemplo: momentos y reacciones coinciden exactamente.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="75" t="inlineStr">
+      <c r="A5" s="76" t="inlineStr">
         <is>
           <t>MATERIALES</t>
         </is>
       </c>
-      <c r="B5" s="75" t="inlineStr">
+      <c r="B5" s="76" t="inlineStr">
         <is>
           <t>H-21 (f'c 210 kg/cm2). Acero 42/50 (fy 4200). Tension admisible 2400 kg/cm2.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="75" t="inlineStr">
+      <c r="A6" s="76" t="inlineStr">
         <is>
           <t>DIMENSIONES</t>
         </is>
       </c>
-      <c r="B6" s="75" t="inlineStr">
+      <c r="B6" s="76" t="inlineStr">
         <is>
           <t>h = altura util | d = espesor total. Recubrimiento 1,5 cm.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="75" t="inlineStr"/>
-      <c r="B7" s="76" t="inlineStr"/>
+      <c r="A7" s="76" t="inlineStr"/>
+      <c r="B7" s="77" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="75" t="inlineStr">
+      <c r="A8" s="76" t="inlineStr">
         <is>
           <t>1. CARGAS</t>
         </is>
       </c>
-      <c r="B8" s="75" t="inlineStr">
+      <c r="B8" s="76" t="inlineStr">
         <is>
           <t>p = peso propio + terminaciones + q      (cargas de servicio, sin mayorar)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="75" t="inlineStr"/>
-      <c r="B9" s="76" t="inlineStr">
+      <c r="A9" s="76" t="inlineStr"/>
+      <c r="B9" s="77" t="inlineStr">
         <is>
           <t>Peso propio = 2400 x d / 100, calculado con el espesor propio de cada losa.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="75" t="inlineStr">
+      <c r="A10" s="76" t="inlineStr">
         <is>
           <t>S/PB</t>
         </is>
       </c>
-      <c r="B10" s="76" t="inlineStr">
+      <c r="B10" s="77" t="inlineStr">
         <is>
           <t>Terminaciones 242 kg/m2 (contrapiso 130 + carpeta 42 + piso 50 + cielorraso 20)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="75" t="inlineStr"/>
-      <c r="B11" s="76" t="inlineStr">
+      <c r="A11" s="76" t="inlineStr"/>
+      <c r="B11" s="77" t="inlineStr">
         <is>
           <t>q = 200 kg/m2 (vivienda)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="75" t="inlineStr">
+      <c r="A12" s="76" t="inlineStr">
         <is>
           <t>S/PA</t>
         </is>
       </c>
-      <c r="B12" s="76" t="inlineStr">
+      <c r="B12" s="77" t="inlineStr">
         <is>
           <t>Terminaciones 252 kg/m2 (contrapiso pendiente 140 + carpeta 42 + aislacion 50 +</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="75" t="inlineStr"/>
-      <c r="B13" s="76" t="inlineStr">
+      <c r="A13" s="76" t="inlineStr"/>
+      <c r="B13" s="77" t="inlineStr">
         <is>
           <t>cielorraso 20).  q = 100 kg/m2 (azotea no accesible)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="75" t="inlineStr"/>
-      <c r="B14" s="76" t="inlineStr"/>
+      <c r="A14" s="76" t="inlineStr"/>
+      <c r="B14" s="77" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="75" t="inlineStr">
+      <c r="A15" s="76" t="inlineStr">
         <is>
           <t>2. SOLICITACIONES</t>
         </is>
       </c>
-      <c r="B15" s="75" t="inlineStr">
+      <c r="B15" s="76" t="inlineStr">
         <is>
           <t>M = coeficiente x p x L2, segun el grado de empotramiento:</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="75" t="inlineStr"/>
-      <c r="B16" s="76" t="inlineStr">
+      <c r="A16" s="76" t="inlineStr"/>
+      <c r="B16" s="77" t="inlineStr">
         <is>
           <t xml:space="preserve">  1/8 simplemente apoyada    1/10 y 1/14 continua    1/12 biempotrada    1/2 voladizo</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="75" t="inlineStr"/>
-      <c r="B17" s="76" t="inlineStr">
+      <c r="A17" s="76" t="inlineStr"/>
+      <c r="B17" s="77" t="inlineStr">
         <is>
           <t>R = coeficiente x p x L. En voladizo Rx = p x L y Ry no corresponde.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="75" t="inlineStr"/>
-      <c r="B18" s="76" t="inlineStr"/>
+      <c r="A18" s="76" t="inlineStr"/>
+      <c r="B18" s="77" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="75" t="inlineStr">
+      <c r="A19" s="76" t="inlineStr">
         <is>
           <t>3. ARMADURA</t>
         </is>
       </c>
-      <c r="B19" s="75" t="inlineStr">
+      <c r="B19" s="76" t="inlineStr">
         <is>
           <t>As = M x 100 / (2400 x 0,9 x h)        [cm2/m]</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="75" t="inlineStr"/>
-      <c r="B20" s="76" t="inlineStr">
+      <c r="A20" s="76" t="inlineStr"/>
+      <c r="B20" s="77" t="inlineStr">
         <is>
           <t>separacion = 100 x area de la barra / As, redondeada, con maximo 20 cm</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="75" t="inlineStr"/>
-      <c r="B21" s="76" t="inlineStr">
+      <c r="A21" s="76" t="inlineStr"/>
+      <c r="B21" s="77" t="inlineStr">
         <is>
           <t>Armadura de reparticion = As / 5, con un minimo de 0,30 cm2/m</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="75" t="inlineStr"/>
-      <c r="B22" s="76" t="inlineStr"/>
+      <c r="A22" s="76" t="inlineStr"/>
+      <c r="B22" s="77" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="75" t="inlineStr">
+      <c r="A23" s="76" t="inlineStr">
         <is>
           <t>4. ESPESORES</t>
         </is>
       </c>
-      <c r="B23" s="75" t="inlineStr">
+      <c r="B23" s="76" t="inlineStr">
         <is>
           <t>Los espesores d se leyeron del plano: estan escritos debajo del rotulo de cada losa.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="75" t="inlineStr"/>
-      <c r="B24" s="76" t="inlineStr">
+      <c r="A24" s="76" t="inlineStr"/>
+      <c r="B24" s="77" t="inlineStr">
         <is>
           <t>S/PB:  L01 11 | L02 9 | L03 13 | L04 11 | L05 11 | L06 8 | L07 12 | L08 10</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="75" t="inlineStr"/>
-      <c r="B25" s="76" t="inlineStr">
+      <c r="A25" s="76" t="inlineStr"/>
+      <c r="B25" s="77" t="inlineStr">
         <is>
           <t>S/PA:  L09 13 | L10 12</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="75" t="inlineStr"/>
-      <c r="B26" s="76" t="inlineStr"/>
+      <c r="A26" s="76" t="inlineStr"/>
+      <c r="B26" s="77" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="75" t="inlineStr">
+      <c r="A27" s="76" t="inlineStr">
         <is>
           <t>5. LUCES</t>
         </is>
       </c>
-      <c r="B27" s="75" t="inlineStr">
+      <c r="B27" s="76" t="inlineStr">
         <is>
           <t>Relevadas en obra y aportadas por el proyectista. Dos losas son voladizo</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="75" t="inlineStr"/>
-      <c r="B28" s="76" t="inlineStr">
+      <c r="A28" s="76" t="inlineStr"/>
+      <c r="B28" s="77" t="inlineStr">
         <is>
           <t>(L02 de 0,80 m y L08 de 0,75 m) y se calculan con M = p L2 / 2.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="75" t="inlineStr"/>
-      <c r="B29" s="76" t="inlineStr"/>
+      <c r="A29" s="76" t="inlineStr"/>
+      <c r="B29" s="77" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="75" t="inlineStr">
+      <c r="A30" s="76" t="inlineStr">
         <is>
           <t>6. LOSAS CRUZADAS</t>
         </is>
       </c>
-      <c r="B30" s="76" t="inlineStr">
+      <c r="B30" s="77" t="inlineStr">
         <is>
           <t>L07 (4,85 x 5,60) y L10 (4,85 x 6,00) apoyan en los cuatro bordes y su relacion</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="75" t="inlineStr"/>
-      <c r="B31" s="76" t="inlineStr">
+      <c r="A31" s="76" t="inlineStr"/>
+      <c r="B31" s="77" t="inlineStr">
         <is>
           <t>de lados es menor que 2, por lo que trabajan en las dos direcciones.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="75" t="inlineStr"/>
-      <c r="B32" s="76" t="inlineStr">
+      <c r="A32" s="76" t="inlineStr"/>
+      <c r="B32" s="77" t="inlineStr">
         <is>
           <t>Se reparte la carga por el metodo de Marcus:   kx = ly4 / (lx4 + ly4)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="75" t="inlineStr"/>
-      <c r="B33" s="76" t="inlineStr">
+      <c r="A33" s="76" t="inlineStr"/>
+      <c r="B33" s="77" t="inlineStr">
         <is>
           <t xml:space="preserve">  L07: ly/lx = 1,15  -&gt;  64% en la direccion corta, 36% en la larga</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="75" t="inlineStr"/>
-      <c r="B34" s="76" t="inlineStr">
+      <c r="A34" s="76" t="inlineStr"/>
+      <c r="B34" s="77" t="inlineStr">
         <is>
           <t xml:space="preserve">  L10: ly/lx = 1,24  -&gt;  70% en la direccion corta, 30% en la larga</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="75" t="inlineStr"/>
-      <c r="B35" s="76" t="inlineStr">
+      <c r="A35" s="76" t="inlineStr"/>
+      <c r="B35" s="77" t="inlineStr">
         <is>
           <t>Cada una ocupa dos renglones, uno por direccion, con la fraccion de carga que</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="75" t="inlineStr"/>
-      <c r="B36" s="76" t="inlineStr">
+      <c r="A36" s="76" t="inlineStr"/>
+      <c r="B36" s="77" t="inlineStr">
         <is>
           <t>le toca ya aplicada en la columna CARGAS. Las dos armaduras se cruzan en obra:</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="75" t="inlineStr"/>
-      <c r="B37" s="76" t="inlineStr">
+      <c r="A37" s="76" t="inlineStr"/>
+      <c r="B37" s="77" t="inlineStr">
         <is>
           <t>la de la direccion corta va abajo, la de la larga arriba de aquella.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="75" t="inlineStr"/>
-      <c r="B38" s="76" t="inlineStr">
+      <c r="A38" s="76" t="inlineStr"/>
+      <c r="B38" s="77" t="inlineStr">
         <is>
           <t>La columna auxiliar luz transv. es la que dispara el reparto: si se borra, la</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="75" t="inlineStr"/>
-      <c r="B39" s="76" t="inlineStr">
+      <c r="A39" s="76" t="inlineStr"/>
+      <c r="B39" s="77" t="inlineStr">
         <is>
           <t>fila vuelve a calcularse como losa armada en una direccion.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="75" t="inlineStr"/>
-      <c r="B40" s="76" t="inlineStr"/>
+      <c r="A40" s="76" t="inlineStr"/>
+      <c r="B40" s="77" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="75" t="inlineStr">
+      <c r="A41" s="76" t="inlineStr">
         <is>
           <t>LIMITACIONES</t>
         </is>
       </c>
-      <c r="B41" s="75" t="inlineStr">
+      <c r="B41" s="76" t="inlineStr">
         <is>
           <t>El grado de empotramiento esta cargado en 1/8 salvo los dos voladizos (1/2). Si</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="75" t="inlineStr"/>
-      <c r="B42" s="76" t="inlineStr">
+      <c r="A42" s="76" t="inlineStr"/>
+      <c r="B42" s="77" t="inlineStr">
         <is>
           <t>alguna losa es continua sobre una viga corresponde 1/10 o 1/14: corregir en la columna.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="75" t="inlineStr"/>
-      <c r="B43" s="76" t="inlineStr">
+      <c r="A43" s="76" t="inlineStr"/>
+      <c r="B43" s="77" t="inlineStr">
         <is>
           <t>El diagrama de cargas es una imagen fija: si cambias el grado, cambialo a mano.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="75" t="inlineStr"/>
-      <c r="B44" s="76" t="inlineStr">
+      <c r="A44" s="76" t="inlineStr"/>
+      <c r="B44" s="77" t="inlineStr">
         <is>
           <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
         </is>
@@ -6615,384 +6908,384 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="74" t="inlineStr">
+      <c r="A1" s="75" t="inlineStr">
         <is>
           <t>MEMORIA DE CALCULO - COLUMNAS</t>
         </is>
       </c>
-      <c r="B1" s="75" t="inlineStr"/>
+      <c r="B1" s="76" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="75" t="inlineStr"/>
-      <c r="B2" s="76" t="inlineStr"/>
+      <c r="A2" s="76" t="inlineStr"/>
+      <c r="B2" s="77" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="75" t="inlineStr">
+      <c r="A3" s="76" t="inlineStr">
         <is>
           <t>MATERIALES</t>
         </is>
       </c>
-      <c r="B3" s="75" t="inlineStr">
+      <c r="B3" s="76" t="inlineStr">
         <is>
           <t>H-21 (f'c 210 kg/cm2). Acero 42/50 (fy 4200). phi compresion 0,65.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="75" t="inlineStr"/>
-      <c r="B4" s="76" t="inlineStr"/>
+      <c r="A4" s="76" t="inlineStr"/>
+      <c r="B4" s="77" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="75" t="inlineStr">
+      <c r="A5" s="76" t="inlineStr">
         <is>
           <t>1. RELEVAMIENTO</t>
         </is>
       </c>
-      <c r="B5" s="75" t="inlineStr">
+      <c r="B5" s="76" t="inlineStr">
         <is>
           <t>Las columnas se identificaron en el plano cruzando el rotulo COL con un rectangulo</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="75" t="inlineStr"/>
-      <c r="B6" s="76" t="inlineStr">
+      <c r="A6" s="76" t="inlineStr"/>
+      <c r="B6" s="77" t="inlineStr">
         <is>
           <t>de la misma seccion a menos de 26 pt. Resultaron 9 en PB y 4 en PA.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="75" t="inlineStr"/>
-      <c r="B7" s="76" t="inlineStr">
+      <c r="A7" s="76" t="inlineStr"/>
+      <c r="B7" s="77" t="inlineStr">
         <is>
           <t>Las 4 de PA caen exactamente sobre C6, C7, C8 y C9 de PB, y ademas tienen la misma</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="75" t="inlineStr"/>
-      <c r="B8" s="76" t="inlineStr">
+      <c r="A8" s="76" t="inlineStr"/>
+      <c r="B8" s="77" t="inlineStr">
         <is>
           <t>seccion, lo que confirma que la correspondencia entre plantas es correcta.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="75" t="inlineStr"/>
-      <c r="B9" s="76" t="inlineStr">
+      <c r="A9" s="76" t="inlineStr"/>
+      <c r="B9" s="77" t="inlineStr">
         <is>
           <t>La C01 de 10x10 esta confirmada por el proyectista aunque el computo metrico no</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="75" t="inlineStr"/>
-      <c r="B10" s="76" t="inlineStr">
+      <c r="A10" s="76" t="inlineStr"/>
+      <c r="B10" s="77" t="inlineStr">
         <is>
           <t>la incluya en su item 4.1.3: ese computo esta incompleto en ese punto.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="75" t="inlineStr"/>
-      <c r="B11" s="76" t="inlineStr"/>
+      <c r="A11" s="76" t="inlineStr"/>
+      <c r="B11" s="77" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="75" t="inlineStr">
+      <c r="A12" s="76" t="inlineStr">
         <is>
           <t>2. ALTURAS</t>
         </is>
       </c>
-      <c r="B12" s="75" t="inlineStr">
+      <c r="B12" s="76" t="inlineStr">
         <is>
           <t>PB 3,15 m y PA 3,22 m, los mismos valores de la planilla de la catedra, coherentes</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="75" t="inlineStr"/>
-      <c r="B13" s="76" t="inlineStr">
+      <c r="A13" s="76" t="inlineStr"/>
+      <c r="B13" s="77" t="inlineStr">
         <is>
           <t>con los niveles del plano (N.F.L +3,50 del entrepiso y +6,80 del techo).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="75" t="inlineStr"/>
-      <c r="B14" s="76" t="inlineStr"/>
+      <c r="A14" s="76" t="inlineStr"/>
+      <c r="B14" s="77" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="75" t="inlineStr">
+      <c r="A15" s="76" t="inlineStr">
         <is>
           <t>3. ARMADURA</t>
         </is>
       </c>
-      <c r="B15" s="75" t="inlineStr">
+      <c r="B15" s="76" t="inlineStr">
         <is>
           <t>As = 0,008 x area (cuantia minima, el mismo criterio de la planilla modelo).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="75" t="inlineStr"/>
-      <c r="B16" s="76" t="inlineStr">
+      <c r="A16" s="76" t="inlineStr"/>
+      <c r="B16" s="77" t="inlineStr">
         <is>
           <t>Se adoptan 4 barras del 12 en todas: 4,52 cm2, que cubre la minima en toda seccion.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="75" t="inlineStr"/>
-      <c r="B17" s="76" t="inlineStr">
+      <c r="A17" s="76" t="inlineStr"/>
+      <c r="B17" s="77" t="inlineStr">
         <is>
           <t>Separacion de estribos = min(12 x diam. long. ; 48 x diam. estribo ; lado menor),</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="75" t="inlineStr"/>
-      <c r="B18" s="76" t="inlineStr">
+      <c r="A18" s="76" t="inlineStr"/>
+      <c r="B18" s="77" t="inlineStr">
         <is>
           <t>redondeada hacia abajo a multiplo de 5. Para 4d12 con estribo d6 da 10 cm.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="75" t="inlineStr"/>
-      <c r="B19" s="76" t="inlineStr">
+      <c r="A19" s="76" t="inlineStr"/>
+      <c r="B19" s="77" t="inlineStr">
         <is>
           <t>La planilla de la catedra adopta 20 cm: ese valor supera el limite reglamentario.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="75" t="inlineStr"/>
-      <c r="B20" s="76" t="inlineStr"/>
+      <c r="A20" s="76" t="inlineStr"/>
+      <c r="B20" s="77" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="75" t="inlineStr">
+      <c r="A21" s="76" t="inlineStr">
         <is>
           <t>4. CAPACIDAD</t>
         </is>
       </c>
-      <c r="B21" s="75" t="inlineStr">
+      <c r="B21" s="76" t="inlineStr">
         <is>
           <t>phi Pn = 0,65 x 0,80 x [0,85 f'c (Ag - As) + fy As]     (columna zunchada con estribos)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="75" t="inlineStr"/>
-      <c r="B22" s="76" t="inlineStr">
+      <c r="A22" s="76" t="inlineStr"/>
+      <c r="B22" s="77" t="inlineStr">
         <is>
           <t xml:space="preserve">  15x30 con 4d12 -&gt; 51,2 t        20x20 con 4d12 -&gt; 46,6 t</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="75" t="inlineStr"/>
-      <c r="B23" s="76" t="inlineStr"/>
+      <c r="A23" s="76" t="inlineStr"/>
+      <c r="B23" s="77" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="75" t="inlineStr">
+      <c r="A24" s="76" t="inlineStr">
         <is>
           <t>5. CARGAS</t>
         </is>
       </c>
-      <c r="B24" s="75" t="inlineStr">
+      <c r="B24" s="76" t="inlineStr">
         <is>
           <t>La columna CARGA (t) viene cargada con una bajada automatica: suma de las</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="75" t="inlineStr"/>
-      <c r="B25" s="76" t="inlineStr">
+      <c r="A25" s="76" t="inlineStr"/>
+      <c r="B25" s="77" t="inlineStr">
         <is>
           <t>reacciones de las vigas que apoyan en cada columna (tomadas de la planilla de</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="75" t="inlineStr"/>
-      <c r="B26" s="76" t="inlineStr">
+      <c r="A26" s="76" t="inlineStr"/>
+      <c r="B26" s="77" t="inlineStr">
         <is>
           <t>vigas), mas el peso propio, mas lo que baja de la columna del nivel superior.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="75" t="inlineStr"/>
-      <c r="B27" s="76" t="inlineStr">
+      <c r="A27" s="76" t="inlineStr"/>
+      <c r="B27" s="77" t="inlineStr">
         <is>
           <t>ES UNA CARGA PROVISORIA Y ES UN PISO, NO EL VALOR REAL: 20 de los 60 extremos</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="75" t="inlineStr"/>
-      <c r="B28" s="76" t="inlineStr">
+      <c r="A28" s="76" t="inlineStr"/>
+      <c r="B28" s="77" t="inlineStr">
         <is>
           <t>de viga no pudieron asignarse a ninguna columna porque apoyan en otra viga, en</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="75" t="inlineStr"/>
-      <c r="B29" s="76" t="inlineStr">
+      <c r="A29" s="76" t="inlineStr"/>
+      <c r="B29" s="77" t="inlineStr">
         <is>
           <t>un tabique o en la medianera, y esas reacciones no estan sumadas.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="75" t="inlineStr"/>
-      <c r="B30" s="76" t="inlineStr">
+      <c r="A30" s="76" t="inlineStr"/>
+      <c r="B30" s="77" t="inlineStr">
         <is>
           <t>Para cerrarla hay que indicar, para cada uno de esos 20 extremos, en que apoya.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="75" t="inlineStr"/>
-      <c r="B31" s="76" t="inlineStr">
+      <c r="A31" s="76" t="inlineStr"/>
+      <c r="B31" s="77" t="inlineStr">
         <is>
           <t>Mientras tanto la columna es editable: al corregir un valor todo recalcula.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="75" t="inlineStr"/>
-      <c r="B32" s="76" t="inlineStr">
+      <c r="A32" s="76" t="inlineStr"/>
+      <c r="B32" s="77" t="inlineStr">
         <is>
           <t>Ademas son cargas MAYORADAS, coherentes con la planilla de vigas. Si la catedra</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="75" t="inlineStr"/>
-      <c r="B33" s="76" t="inlineStr">
+      <c r="A33" s="76" t="inlineStr"/>
+      <c r="B33" s="77" t="inlineStr">
         <is>
           <t>pide cargas de servicio, dividir por el coeficiente que corresponda.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="75" t="inlineStr"/>
-      <c r="B34" s="76" t="inlineStr"/>
+      <c r="A34" s="76" t="inlineStr"/>
+      <c r="B34" s="77" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="75" t="inlineStr">
+      <c r="A35" s="76" t="inlineStr">
         <is>
           <t>6. ESBELTEZ</t>
         </is>
       </c>
-      <c r="B35" s="75" t="inlineStr">
+      <c r="B35" s="76" t="inlineStr">
         <is>
           <t>Todas las columnas son esbeltas: con lado menor de 15 cm y 3,15 m de altura,</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="75" t="inlineStr"/>
-      <c r="B36" s="76" t="inlineStr">
+      <c r="A36" s="76" t="inlineStr"/>
+      <c r="B36" s="77" t="inlineStr">
         <is>
           <t>k lu / r = 70, muy por encima del limite de 34 por debajo del cual se puede</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="75" t="inlineStr"/>
-      <c r="B37" s="76" t="inlineStr">
+      <c r="A37" s="76" t="inlineStr"/>
+      <c r="B37" s="77" t="inlineStr">
         <is>
           <t>despreciar el pandeo. En la practica el llenado de mamposteria las arriostra, pero</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="75" t="inlineStr"/>
-      <c r="B38" s="76" t="inlineStr">
+      <c r="A38" s="76" t="inlineStr"/>
+      <c r="B38" s="77" t="inlineStr">
         <is>
           <t>si la catedra lo pide hay que verificar segundo orden. La planilla lo marca.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="75" t="inlineStr"/>
-      <c r="B39" s="76" t="inlineStr"/>
+      <c r="A39" s="76" t="inlineStr"/>
+      <c r="B39" s="77" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="75" t="inlineStr">
+      <c r="A40" s="76" t="inlineStr">
         <is>
           <t>7. LA DE 10x10</t>
         </is>
       </c>
-      <c r="B40" s="75" t="inlineStr">
+      <c r="B40" s="76" t="inlineStr">
         <is>
           <t>Existe, confirmada por el proyectista, y el computo metrico la omite. Con 10 cm</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="75" t="inlineStr"/>
-      <c r="B41" s="76" t="inlineStr">
+      <c r="A41" s="76" t="inlineStr"/>
+      <c r="B41" s="77" t="inlineStr">
         <is>
           <t>de lado y 3,15 m de altura su esbeltez es k lu / r = 105, tres veces el limite</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="75" t="inlineStr"/>
-      <c r="B42" s="76" t="inlineStr">
+      <c r="A42" s="76" t="inlineStr"/>
+      <c r="B42" s="77" t="inlineStr">
         <is>
           <t>por debajo del cual se puede despreciar el pandeo, y su capacidad es de 18,7 t</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="75" t="inlineStr"/>
-      <c r="B43" s="76" t="inlineStr">
+      <c r="A43" s="76" t="inlineStr"/>
+      <c r="B43" s="77" t="inlineStr">
         <is>
           <t>contra los 51 de una 15x30. Es el punto mas delicado del conjunto: conviene</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="75" t="inlineStr"/>
-      <c r="B44" s="76" t="inlineStr">
+      <c r="A44" s="76" t="inlineStr"/>
+      <c r="B44" s="77" t="inlineStr">
         <is>
           <t>verificarla a segundo orden en serio, no con la formula de compresion simple.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="75" t="inlineStr"/>
-      <c r="B45" s="76" t="inlineStr"/>
+      <c r="A45" s="76" t="inlineStr"/>
+      <c r="B45" s="77" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="75" t="inlineStr">
+      <c r="A46" s="76" t="inlineStr">
         <is>
           <t>LIMITACIONES</t>
         </is>
       </c>
-      <c r="B46" s="75" t="inlineStr">
+      <c r="B46" s="76" t="inlineStr">
         <is>
           <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="75" t="inlineStr"/>
-      <c r="B47" s="76" t="inlineStr">
+      <c r="A47" s="76" t="inlineStr"/>
+      <c r="B47" s="77" t="inlineStr">
         <is>
           <t>No se verifica flexion compuesta: las columnas de borde reciben momento de las</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="75" t="inlineStr"/>
-      <c r="B48" s="76" t="inlineStr">
+      <c r="A48" s="76" t="inlineStr"/>
+      <c r="B48" s="77" t="inlineStr">
         <is>
           <t>vigas invertidas y trabajan a flexo-compresion, no a compresion simple.</t>
         </is>
@@ -7020,7 +7313,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="77" t="inlineStr">
+      <c r="A1" s="78" t="inlineStr">
         <is>
           <t>VIGAS DE FUNDACION - inventario. Calculo pendiente: va despues de columnas.</t>
         </is>
@@ -7162,7 +7455,7 @@
       <c r="D9" s="11" t="n">
         <v>533</v>
       </c>
-      <c r="E9" s="78" t="inlineStr">
+      <c r="E9" s="79" t="inlineStr">
         <is>
           <t>Ancho cortado en el PDF: confirmar 20 o 22 cm</t>
         </is>
@@ -7228,7 +7521,7 @@
       <c r="B13" s="11" t="n"/>
       <c r="C13" s="11" t="n"/>
       <c r="D13" s="11" t="n"/>
-      <c r="E13" s="78" t="inlineStr">
+      <c r="E13" s="79" t="inlineStr">
         <is>
           <t>Cota no legible: completar</t>
         </is>
@@ -7243,7 +7536,7 @@
       <c r="B14" s="11" t="n"/>
       <c r="C14" s="11" t="n"/>
       <c r="D14" s="11" t="n"/>
-      <c r="E14" s="78" t="inlineStr">
+      <c r="E14" s="79" t="inlineStr">
         <is>
           <t>Cota no legible: completar</t>
         </is>
@@ -7445,7 +7738,7 @@
       <c r="B26" s="11" t="n"/>
       <c r="C26" s="11" t="n"/>
       <c r="D26" s="11" t="n"/>
-      <c r="E26" s="78" t="inlineStr">
+      <c r="E26" s="79" t="inlineStr">
         <is>
           <t>Cota no legible: completar</t>
         </is>
@@ -7616,7 +7909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M71"/>
+  <dimension ref="A1:M73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7840,7 +8133,7 @@
       </c>
       <c r="L7" s="26" t="n"/>
       <c r="M7" s="30">
-        <f>IF(OR(D7="",J7=""),"",IF(J7&lt;=G7,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D7="",J7=""),"",IF(AND(J7&lt;=G7,OR(L7="",L7&lt;=IFERROR(VLOOKUP(K7,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -7885,7 +8178,7 @@
       </c>
       <c r="L8" s="26" t="n"/>
       <c r="M8" s="30">
-        <f>IF(OR(D8="",J8=""),"",IF(J8&lt;=G8,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D8="",J8=""),"",IF(AND(J8&lt;=G8,OR(L8="",L8&lt;=IFERROR(VLOOKUP(K8,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -7930,7 +8223,7 @@
       </c>
       <c r="L9" s="26" t="n"/>
       <c r="M9" s="30">
-        <f>IF(OR(D9="",J9=""),"",IF(J9&lt;=G9,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D9="",J9=""),"",IF(AND(J9&lt;=G9,OR(L9="",L9&lt;=IFERROR(VLOOKUP(K9,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -7975,7 +8268,7 @@
       </c>
       <c r="L10" s="26" t="n"/>
       <c r="M10" s="30">
-        <f>IF(OR(D10="",J10=""),"",IF(J10&lt;=G10,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D10="",J10=""),"",IF(AND(J10&lt;=G10,OR(L10="",L10&lt;=IFERROR(VLOOKUP(K10,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8020,7 +8313,7 @@
       </c>
       <c r="L11" s="26" t="n"/>
       <c r="M11" s="30">
-        <f>IF(OR(D11="",J11=""),"",IF(J11&lt;=G11,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D11="",J11=""),"",IF(AND(J11&lt;=G11,OR(L11="",L11&lt;=IFERROR(VLOOKUP(K11,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8047,7 +8340,7 @@
       <c r="K12" s="25" t="n"/>
       <c r="L12" s="26" t="n"/>
       <c r="M12" s="30">
-        <f>IF(OR(D12="",J12=""),"",IF(J12&lt;=G12,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D12="",J12=""),"",IF(AND(J12&lt;=G12,OR(L12="",L12&lt;=IFERROR(VLOOKUP(K12,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8074,7 +8367,7 @@
       <c r="K13" s="32" t="n"/>
       <c r="L13" s="33" t="n"/>
       <c r="M13" s="37">
-        <f>IF(OR(D13="",J13=""),"",IF(J13&lt;=G13,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D13="",J13=""),"",IF(AND(J13&lt;=G13,OR(L13="",L13&lt;=IFERROR(VLOOKUP(K13,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8141,7 +8434,7 @@
       </c>
       <c r="L15" s="26" t="n"/>
       <c r="M15" s="30">
-        <f>IF(OR(D15="",J15=""),"",IF(J15&lt;=G15,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D15="",J15=""),"",IF(AND(J15&lt;=G15,OR(L15="",L15&lt;=IFERROR(VLOOKUP(K15,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8186,7 +8479,7 @@
       </c>
       <c r="L16" s="26" t="n"/>
       <c r="M16" s="30">
-        <f>IF(OR(D16="",J16=""),"",IF(J16&lt;=G16,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D16="",J16=""),"",IF(AND(J16&lt;=G16,OR(L16="",L16&lt;=IFERROR(VLOOKUP(K16,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8213,7 +8506,7 @@
       <c r="K17" s="25" t="n"/>
       <c r="L17" s="26" t="n"/>
       <c r="M17" s="30">
-        <f>IF(OR(D17="",J17=""),"",IF(J17&lt;=G17,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D17="",J17=""),"",IF(AND(J17&lt;=G17,OR(L17="",L17&lt;=IFERROR(VLOOKUP(K17,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8240,7 +8533,7 @@
       <c r="K18" s="32" t="n"/>
       <c r="L18" s="33" t="n"/>
       <c r="M18" s="37">
-        <f>IF(OR(D18="",J18=""),"",IF(J18&lt;=G18,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D18="",J18=""),"",IF(AND(J18&lt;=G18,OR(L18="",L18&lt;=IFERROR(VLOOKUP(K18,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8307,7 +8600,7 @@
       </c>
       <c r="L20" s="26" t="n"/>
       <c r="M20" s="30">
-        <f>IF(OR(D20="",J20=""),"",IF(J20&lt;=G20,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D20="",J20=""),"",IF(AND(J20&lt;=G20,OR(L20="",L20&lt;=IFERROR(VLOOKUP(K20,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8352,7 +8645,7 @@
       </c>
       <c r="L21" s="26" t="n"/>
       <c r="M21" s="30">
-        <f>IF(OR(D21="",J21=""),"",IF(J21&lt;=G21,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D21="",J21=""),"",IF(AND(J21&lt;=G21,OR(L21="",L21&lt;=IFERROR(VLOOKUP(K21,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8397,7 +8690,7 @@
       </c>
       <c r="L22" s="26" t="n"/>
       <c r="M22" s="30">
-        <f>IF(OR(D22="",J22=""),"",IF(J22&lt;=G22,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D22="",J22=""),"",IF(AND(J22&lt;=G22,OR(L22="",L22&lt;=IFERROR(VLOOKUP(K22,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8442,7 +8735,7 @@
       </c>
       <c r="L23" s="26" t="n"/>
       <c r="M23" s="30">
-        <f>IF(OR(D23="",J23=""),"",IF(J23&lt;=G23,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D23="",J23=""),"",IF(AND(J23&lt;=G23,OR(L23="",L23&lt;=IFERROR(VLOOKUP(K23,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8487,7 +8780,7 @@
       </c>
       <c r="L24" s="26" t="n"/>
       <c r="M24" s="30">
-        <f>IF(OR(D24="",J24=""),"",IF(J24&lt;=G24,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D24="",J24=""),"",IF(AND(J24&lt;=G24,OR(L24="",L24&lt;=IFERROR(VLOOKUP(K24,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8514,7 +8807,7 @@
       <c r="K25" s="25" t="n"/>
       <c r="L25" s="26" t="n"/>
       <c r="M25" s="30">
-        <f>IF(OR(D25="",J25=""),"",IF(J25&lt;=G25,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D25="",J25=""),"",IF(AND(J25&lt;=G25,OR(L25="",L25&lt;=IFERROR(VLOOKUP(K25,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8541,7 +8834,7 @@
       <c r="K26" s="32" t="n"/>
       <c r="L26" s="33" t="n"/>
       <c r="M26" s="37">
-        <f>IF(OR(D26="",J26=""),"",IF(J26&lt;=G26,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D26="",J26=""),"",IF(AND(J26&lt;=G26,OR(L26="",L26&lt;=IFERROR(VLOOKUP(K26,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8608,7 +8901,7 @@
       </c>
       <c r="L28" s="26" t="n"/>
       <c r="M28" s="30">
-        <f>IF(OR(D28="",J28=""),"",IF(J28&lt;=G28,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D28="",J28=""),"",IF(AND(J28&lt;=G28,OR(L28="",L28&lt;=IFERROR(VLOOKUP(K28,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8653,7 +8946,7 @@
       </c>
       <c r="L29" s="26" t="n"/>
       <c r="M29" s="30">
-        <f>IF(OR(D29="",J29=""),"",IF(J29&lt;=G29,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D29="",J29=""),"",IF(AND(J29&lt;=G29,OR(L29="",L29&lt;=IFERROR(VLOOKUP(K29,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8698,7 +8991,7 @@
       </c>
       <c r="L30" s="26" t="n"/>
       <c r="M30" s="30">
-        <f>IF(OR(D30="",J30=""),"",IF(J30&lt;=G30,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D30="",J30=""),"",IF(AND(J30&lt;=G30,OR(L30="",L30&lt;=IFERROR(VLOOKUP(K30,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8743,7 +9036,7 @@
       </c>
       <c r="L31" s="26" t="n"/>
       <c r="M31" s="30">
-        <f>IF(OR(D31="",J31=""),"",IF(J31&lt;=G31,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D31="",J31=""),"",IF(AND(J31&lt;=G31,OR(L31="",L31&lt;=IFERROR(VLOOKUP(K31,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8788,7 +9081,7 @@
       </c>
       <c r="L32" s="26" t="n"/>
       <c r="M32" s="30">
-        <f>IF(OR(D32="",J32=""),"",IF(J32&lt;=G32,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D32="",J32=""),"",IF(AND(J32&lt;=G32,OR(L32="",L32&lt;=IFERROR(VLOOKUP(K32,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8815,7 +9108,7 @@
       <c r="K33" s="25" t="n"/>
       <c r="L33" s="26" t="n"/>
       <c r="M33" s="30">
-        <f>IF(OR(D33="",J33=""),"",IF(J33&lt;=G33,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D33="",J33=""),"",IF(AND(J33&lt;=G33,OR(L33="",L33&lt;=IFERROR(VLOOKUP(K33,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8842,7 +9135,7 @@
       <c r="K34" s="32" t="n"/>
       <c r="L34" s="33" t="n"/>
       <c r="M34" s="37">
-        <f>IF(OR(D34="",J34=""),"",IF(J34&lt;=G34,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D34="",J34=""),"",IF(AND(J34&lt;=G34,OR(L34="",L34&lt;=IFERROR(VLOOKUP(K34,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8905,7 +9198,7 @@
       <c r="K36" s="25" t="n"/>
       <c r="L36" s="26" t="n"/>
       <c r="M36" s="30">
-        <f>IF(OR(D36="",J36=""),"",IF(J36&lt;=G36,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D36="",J36=""),"",IF(AND(J36&lt;=G36,OR(L36="",L36&lt;=IFERROR(VLOOKUP(K36,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8932,7 +9225,7 @@
       <c r="K37" s="25" t="n"/>
       <c r="L37" s="26" t="n"/>
       <c r="M37" s="30">
-        <f>IF(OR(D37="",J37=""),"",IF(J37&lt;=G37,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D37="",J37=""),"",IF(AND(J37&lt;=G37,OR(L37="",L37&lt;=IFERROR(VLOOKUP(K37,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -8959,7 +9252,7 @@
       <c r="K38" s="32" t="n"/>
       <c r="L38" s="33" t="n"/>
       <c r="M38" s="37">
-        <f>IF(OR(D38="",J38=""),"",IF(J38&lt;=G38,"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(OR(D38="",J38=""),"",IF(AND(J38&lt;=G38,OR(L38="",L38&lt;=IFERROR(VLOOKUP(K38,Datos_higro!$A$46:$B$54,2,0),99))),"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
@@ -9076,7 +9369,7 @@
     <row r="45">
       <c r="A45" s="39" t="inlineStr">
         <is>
-          <t>Orientacion y factor de exposicion solar: el factor depende de la orientacion y de la proteccion.</t>
+          <t>Orientacion: ya cargada. Factor de exposicion solar: cargarlo en la columna L segun el vidrio</t>
         </is>
       </c>
       <c r="B45" s="2" t="n"/>
@@ -9093,7 +9386,11 @@
       <c r="M45" s="2" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="39" t="inlineStr"/>
+      <c r="A46" s="39" t="inlineStr">
+        <is>
+          <t>y la proteccion solar adoptados; la verificacion lo compara contra el maximo del cuadrante,</t>
+        </is>
+      </c>
       <c r="B46" s="2" t="n"/>
       <c r="C46" s="2" t="n"/>
       <c r="D46" s="2" t="n"/>
@@ -9110,7 +9407,7 @@
     <row r="47">
       <c r="A47" s="39" t="inlineStr">
         <is>
-          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
+          <t>que esta en la tabla de la hoja Datos_higro.</t>
         </is>
       </c>
       <c r="B47" s="2" t="n"/>
@@ -9127,11 +9424,7 @@
       <c r="M47" s="2" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="39" t="inlineStr">
-        <is>
-          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
-        </is>
-      </c>
+      <c r="A48" s="39" t="inlineStr"/>
       <c r="B48" s="2" t="n"/>
       <c r="C48" s="2" t="n"/>
       <c r="D48" s="2" t="n"/>
@@ -9146,7 +9439,11 @@
       <c r="M48" s="2" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="39" t="inlineStr"/>
+      <c r="A49" s="39" t="inlineStr">
+        <is>
+          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
+        </is>
+      </c>
       <c r="B49" s="2" t="n"/>
       <c r="C49" s="2" t="n"/>
       <c r="D49" s="2" t="n"/>
@@ -9163,7 +9460,7 @@
     <row r="50">
       <c r="A50" s="39" t="inlineStr">
         <is>
-          <t>ALTURAS: medidas sobre el dibujo de las vistas de la planilla de carpinterias, con la escala</t>
+          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
         </is>
       </c>
       <c r="B50" s="2" t="n"/>
@@ -9180,11 +9477,7 @@
       <c r="M50" s="2" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="39" t="inlineStr">
-        <is>
-          <t>verificada contra los anchos acotados (error menor a 2 cm). La mayoria de las aberturas son de</t>
-        </is>
-      </c>
+      <c r="A51" s="39" t="inlineStr"/>
       <c r="B51" s="2" t="n"/>
       <c r="C51" s="2" t="n"/>
       <c r="D51" s="2" t="n"/>
@@ -9201,7 +9494,7 @@
     <row r="52">
       <c r="A52" s="39" t="inlineStr">
         <is>
-          <t>piso a cielorraso, 3,00 m. VERIFICARLAS contra el plano antes de presentar.</t>
+          <t>ALTURAS: medidas sobre el dibujo de las vistas de la planilla de carpinterias, con la escala</t>
         </is>
       </c>
       <c r="B52" s="2" t="n"/>
@@ -9220,7 +9513,7 @@
     <row r="53">
       <c r="A53" s="39" t="inlineStr">
         <is>
-          <t>PF04 es la unica con antepecho: arranca a 1,09 y mide 0,60 de alto. El resto llega al piso.</t>
+          <t>verificada contra los anchos acotados (error menor a 2 cm). La mayoria de las aberturas son de</t>
         </is>
       </c>
       <c r="B53" s="2" t="n"/>
@@ -9239,7 +9532,7 @@
     <row r="54">
       <c r="A54" s="39" t="inlineStr">
         <is>
-          <t>Las alturas de PV01 (3,00), PF04 (0,60) y PV04 (2) (2,95) las aporto el autor del proyecto.</t>
+          <t>piso a cielorraso, 3,00 m. VERIFICARLAS contra el plano antes de presentar.</t>
         </is>
       </c>
       <c r="B54" s="2" t="n"/>
@@ -9256,7 +9549,11 @@
       <c r="M54" s="2" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="39" t="inlineStr"/>
+      <c r="A55" s="39" t="inlineStr">
+        <is>
+          <t>PF04 es la unica con antepecho: arranca a 1,09 y mide 0,60 de alto. El resto llega al piso.</t>
+        </is>
+      </c>
       <c r="B55" s="2" t="n"/>
       <c r="C55" s="2" t="n"/>
       <c r="D55" s="2" t="n"/>
@@ -9273,7 +9570,7 @@
     <row r="56">
       <c r="A56" s="39" t="inlineStr">
         <is>
-          <t>ORIENTACION: el simbolo de norte del plano (circulo con aguja, en el patio interno) apunta a</t>
+          <t>Las alturas de PV01 (3,00), PF04 (0,60) y PV04 (2) (2,95) las aporto el autor del proyecto.</t>
         </is>
       </c>
       <c r="B56" s="2" t="n"/>
@@ -9290,11 +9587,7 @@
       <c r="M56" s="2" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="39" t="inlineStr">
-        <is>
-          <t>45 grados hacia arriba y a la derecha de la hoja. Entonces las cuatro fachadas NO son N-S-E-O</t>
-        </is>
-      </c>
+      <c r="A57" s="39" t="inlineStr"/>
       <c r="B57" s="2" t="n"/>
       <c r="C57" s="2" t="n"/>
       <c r="D57" s="2" t="n"/>
@@ -9311,7 +9604,7 @@
     <row r="58">
       <c r="A58" s="39" t="inlineStr">
         <is>
-          <t>sino: arriba = Noroeste, derecha = Noreste, abajo = Sudeste, izquierda = Sudoeste.</t>
+          <t>ORIENTACION: el simbolo de norte del plano (circulo con aguja, en el patio interno) apunta a</t>
         </is>
       </c>
       <c r="B58" s="2" t="n"/>
@@ -9330,7 +9623,7 @@
     <row r="59">
       <c r="A59" s="39" t="inlineStr">
         <is>
-          <t>Cada abertura se asigno a la fachada por su posicion en planta. Las del patio interno se</t>
+          <t>45 grados hacia arriba y a la derecha de la hoja. Entonces las cuatro fachadas NO son N-S-E-O</t>
         </is>
       </c>
       <c r="B59" s="2" t="n"/>
@@ -9349,7 +9642,7 @@
     <row r="60">
       <c r="A60" s="39" t="inlineStr">
         <is>
-          <t>orientan por la pared en la que estan: miran hacia adentro del patio.</t>
+          <t>sino: arriba = Noroeste, derecha = Noreste, abajo = Sudeste, izquierda = Sudoeste.</t>
         </is>
       </c>
       <c r="B60" s="2" t="n"/>
@@ -9368,7 +9661,7 @@
     <row r="61">
       <c r="A61" s="39" t="inlineStr">
         <is>
-          <t>Los rotulos Dormitorio Norte y Dormitorio Sur del plano no coinciden con el norte real;</t>
+          <t>Cada abertura se asigno a la fachada por su posicion en planta. Las del patio interno se</t>
         </is>
       </c>
       <c r="B61" s="2" t="n"/>
@@ -9387,7 +9680,7 @@
     <row r="62">
       <c r="A62" s="39" t="inlineStr">
         <is>
-          <t>parecen ser nombres de uso, no orientaciones.</t>
+          <t>orientan por la pared en la que estan: miran hacia adentro del patio.</t>
         </is>
       </c>
       <c r="B62" s="2" t="n"/>
@@ -9404,7 +9697,11 @@
       <c r="M62" s="2" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="39" t="inlineStr"/>
+      <c r="A63" s="39" t="inlineStr">
+        <is>
+          <t>Los rotulos Dormitorio Norte y Dormitorio Sur del plano no coinciden con el norte real;</t>
+        </is>
+      </c>
       <c r="B63" s="2" t="n"/>
       <c r="C63" s="2" t="n"/>
       <c r="D63" s="2" t="n"/>
@@ -9421,7 +9718,7 @@
     <row r="64">
       <c r="A64" s="39" t="inlineStr">
         <is>
-          <t>PF01 figura dos veces en el plano, en las dos paredes laterales del patio interno, y por eso</t>
+          <t>parecen ser nombres de uso, no orientaciones.</t>
         </is>
       </c>
       <c r="B64" s="2" t="n"/>
@@ -9438,11 +9735,7 @@
       <c r="M64" s="2" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="39" t="inlineStr">
-        <is>
-          <t>se cargan dos filas. Si fuera una sola abertura rotulada dos veces, borrar la segunda.</t>
-        </is>
-      </c>
+      <c r="A65" s="39" t="inlineStr"/>
       <c r="B65" s="2" t="n"/>
       <c r="C65" s="2" t="n"/>
       <c r="D65" s="2" t="n"/>
@@ -9457,7 +9750,11 @@
       <c r="M65" s="2" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="39" t="inlineStr"/>
+      <c r="A66" s="39" t="inlineStr">
+        <is>
+          <t>PF01 figura dos veces en el plano, en las dos paredes laterales del patio interno, y por eso</t>
+        </is>
+      </c>
       <c r="B66" s="2" t="n"/>
       <c r="C66" s="2" t="n"/>
       <c r="D66" s="2" t="n"/>
@@ -9474,7 +9771,7 @@
     <row r="67">
       <c r="A67" s="39" t="inlineStr">
         <is>
-          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
+          <t>se cargan dos filas. Si fuera una sola abertura rotulada dos veces, borrar la segunda.</t>
         </is>
       </c>
       <c r="B67" s="2" t="n"/>
@@ -9508,7 +9805,7 @@
     <row r="69">
       <c r="A69" s="39" t="inlineStr">
         <is>
-          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
+          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
         </is>
       </c>
       <c r="B69" s="2" t="n"/>
@@ -9525,11 +9822,7 @@
       <c r="M69" s="2" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="39" t="inlineStr">
-        <is>
-          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
-        </is>
-      </c>
+      <c r="A70" s="39" t="inlineStr"/>
       <c r="B70" s="2" t="n"/>
       <c r="C70" s="2" t="n"/>
       <c r="D70" s="2" t="n"/>
@@ -9546,7 +9839,7 @@
     <row r="71">
       <c r="A71" s="39" t="inlineStr">
         <is>
-          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
+          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
         </is>
       </c>
       <c r="B71" s="2" t="n"/>
@@ -9561,6 +9854,44 @@
       <c r="K71" s="2" t="n"/>
       <c r="L71" s="2" t="n"/>
       <c r="M71" s="2" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="39" t="inlineStr">
+        <is>
+          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="n"/>
+      <c r="C72" s="2" t="n"/>
+      <c r="D72" s="2" t="n"/>
+      <c r="E72" s="2" t="n"/>
+      <c r="F72" s="2" t="n"/>
+      <c r="G72" s="2" t="n"/>
+      <c r="H72" s="2" t="n"/>
+      <c r="I72" s="2" t="n"/>
+      <c r="J72" s="2" t="n"/>
+      <c r="K72" s="2" t="n"/>
+      <c r="L72" s="2" t="n"/>
+      <c r="M72" s="2" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="39" t="inlineStr">
+        <is>
+          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="n"/>
+      <c r="C73" s="2" t="n"/>
+      <c r="D73" s="2" t="n"/>
+      <c r="E73" s="2" t="n"/>
+      <c r="F73" s="2" t="n"/>
+      <c r="G73" s="2" t="n"/>
+      <c r="H73" s="2" t="n"/>
+      <c r="I73" s="2" t="n"/>
+      <c r="J73" s="2" t="n"/>
+      <c r="K73" s="2" t="n"/>
+      <c r="L73" s="2" t="n"/>
+      <c r="M73" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="14">

</xml_diff>

<commit_message>
Planilla 3: cargar cortina de enrollar como proteccion solar
Se carga cortina de enrollar exterior en las 18 aberturas. El factor de
exposicion solar se completa solo y da 0,25, que queda por debajo del
maximo de 0,30 del cuadrante Este/Oeste, donde caen las cuatro fachadas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -7915,7 +7915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M75"/>
+  <dimension ref="A1:M78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8128,7 +8128,11 @@
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I7" s="25" t="n"/>
+      <c r="I7" s="25" t="inlineStr">
+        <is>
+          <t>Cortina de enrollar exterior</t>
+        </is>
+      </c>
       <c r="J7" s="26" t="n">
         <v>2.8</v>
       </c>
@@ -8176,7 +8180,11 @@
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I8" s="25" t="n"/>
+      <c r="I8" s="25" t="inlineStr">
+        <is>
+          <t>Cortina de enrollar exterior</t>
+        </is>
+      </c>
       <c r="J8" s="26" t="n">
         <v>2.8</v>
       </c>
@@ -8224,7 +8232,11 @@
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I9" s="25" t="n"/>
+      <c r="I9" s="25" t="inlineStr">
+        <is>
+          <t>Cortina de enrollar exterior</t>
+        </is>
+      </c>
       <c r="J9" s="26" t="n">
         <v>2.8</v>
       </c>
@@ -8272,7 +8284,11 @@
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I10" s="25" t="n"/>
+      <c r="I10" s="25" t="inlineStr">
+        <is>
+          <t>Cortina de enrollar exterior</t>
+        </is>
+      </c>
       <c r="J10" s="26" t="n">
         <v>2.8</v>
       </c>
@@ -8320,7 +8336,11 @@
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I11" s="25" t="n"/>
+      <c r="I11" s="25" t="inlineStr">
+        <is>
+          <t>Cortina de enrollar exterior</t>
+        </is>
+      </c>
       <c r="J11" s="26" t="n">
         <v>2.8</v>
       </c>
@@ -8450,7 +8470,11 @@
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I15" s="25" t="n"/>
+      <c r="I15" s="25" t="inlineStr">
+        <is>
+          <t>Cortina de enrollar exterior</t>
+        </is>
+      </c>
       <c r="J15" s="26" t="n">
         <v>2.8</v>
       </c>
@@ -8498,7 +8522,11 @@
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I16" s="25" t="n"/>
+      <c r="I16" s="25" t="inlineStr">
+        <is>
+          <t>Cortina de enrollar exterior</t>
+        </is>
+      </c>
       <c r="J16" s="26" t="n">
         <v>2.8</v>
       </c>
@@ -8628,7 +8656,11 @@
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I20" s="25" t="n"/>
+      <c r="I20" s="25" t="inlineStr">
+        <is>
+          <t>Cortina de enrollar exterior</t>
+        </is>
+      </c>
       <c r="J20" s="26" t="n">
         <v>2.8</v>
       </c>
@@ -8676,7 +8708,11 @@
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I21" s="25" t="n"/>
+      <c r="I21" s="25" t="inlineStr">
+        <is>
+          <t>Cortina de enrollar exterior</t>
+        </is>
+      </c>
       <c r="J21" s="26" t="n">
         <v>2.8</v>
       </c>
@@ -8724,7 +8760,11 @@
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I22" s="25" t="n"/>
+      <c r="I22" s="25" t="inlineStr">
+        <is>
+          <t>Cortina de enrollar exterior</t>
+        </is>
+      </c>
       <c r="J22" s="26" t="n">
         <v>2.8</v>
       </c>
@@ -8772,7 +8812,11 @@
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I23" s="25" t="n"/>
+      <c r="I23" s="25" t="inlineStr">
+        <is>
+          <t>Cortina de enrollar exterior</t>
+        </is>
+      </c>
       <c r="J23" s="26" t="n">
         <v>2.8</v>
       </c>
@@ -8820,7 +8864,11 @@
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I24" s="25" t="n"/>
+      <c r="I24" s="25" t="inlineStr">
+        <is>
+          <t>Cortina de enrollar exterior</t>
+        </is>
+      </c>
       <c r="J24" s="26" t="n">
         <v>2.8</v>
       </c>
@@ -8950,7 +8998,11 @@
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I28" s="25" t="n"/>
+      <c r="I28" s="25" t="inlineStr">
+        <is>
+          <t>Cortina de enrollar exterior</t>
+        </is>
+      </c>
       <c r="J28" s="26" t="n">
         <v>2.8</v>
       </c>
@@ -8998,7 +9050,11 @@
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I29" s="25" t="n"/>
+      <c r="I29" s="25" t="inlineStr">
+        <is>
+          <t>Cortina de enrollar exterior</t>
+        </is>
+      </c>
       <c r="J29" s="26" t="n">
         <v>2.8</v>
       </c>
@@ -9046,7 +9102,11 @@
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I30" s="25" t="n"/>
+      <c r="I30" s="25" t="inlineStr">
+        <is>
+          <t>Cortina de enrollar exterior</t>
+        </is>
+      </c>
       <c r="J30" s="26" t="n">
         <v>2.8</v>
       </c>
@@ -9094,7 +9154,11 @@
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I31" s="25" t="n"/>
+      <c r="I31" s="25" t="inlineStr">
+        <is>
+          <t>Cortina de enrollar exterior</t>
+        </is>
+      </c>
       <c r="J31" s="26" t="n">
         <v>2.8</v>
       </c>
@@ -9142,7 +9206,11 @@
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I32" s="25" t="n"/>
+      <c r="I32" s="25" t="inlineStr">
+        <is>
+          <t>Cortina de enrollar exterior</t>
+        </is>
+      </c>
       <c r="J32" s="26" t="n">
         <v>2.8</v>
       </c>
@@ -9272,7 +9340,11 @@
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I36" s="25" t="n"/>
+      <c r="I36" s="25" t="inlineStr">
+        <is>
+          <t>Cortina de enrollar exterior</t>
+        </is>
+      </c>
       <c r="J36" s="26" t="n">
         <v>2.8</v>
       </c>
@@ -9459,7 +9531,7 @@
     <row r="45">
       <c r="A45" s="39" t="inlineStr">
         <is>
-          <t>Orientacion: ya cargada. Factor de exposicion solar: se completa SOLO al elegir el tipo de</t>
+          <t>PROTECCION: se cargo cortina de enrollar exterior en todas las aberturas. Cambiar en la</t>
         </is>
       </c>
       <c r="B45" s="2" t="n"/>
@@ -9478,7 +9550,7 @@
     <row r="46">
       <c r="A46" s="39" t="inlineStr">
         <is>
-          <t>proteccion, con los valores de la tabla de Datos_higro (Sin Proteccion 0,88; Parasol</t>
+          <t>columna I las que no la tengan; el factor de exposicion solar se recalcula solo.</t>
         </is>
       </c>
       <c r="B46" s="2" t="n"/>
@@ -9495,11 +9567,7 @@
       <c r="M46" s="2" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="39" t="inlineStr">
-        <is>
-          <t>horizontal fijo 1:2 0,35), que son los mismos de la planilla de la catedra.</t>
-        </is>
-      </c>
+      <c r="A47" s="39" t="inlineStr"/>
       <c r="B47" s="2" t="n"/>
       <c r="C47" s="2" t="n"/>
       <c r="D47" s="2" t="n"/>
@@ -9516,7 +9584,7 @@
     <row r="48">
       <c r="A48" s="39" t="inlineStr">
         <is>
-          <t>En Datos_higro esta ademas el FES maximo admitido por cuadrante segun la ordenanza, como</t>
+          <t>Orientacion: ya cargada. Factor de exposicion solar: se completa SOLO al elegir el tipo de</t>
         </is>
       </c>
       <c r="B48" s="2" t="n"/>
@@ -9535,7 +9603,7 @@
     <row r="49">
       <c r="A49" s="39" t="inlineStr">
         <is>
-          <t>referencia: la verificacion no lo controla, igual que en la planilla de la catedra.</t>
+          <t>proteccion, con los valores de la tabla de Datos_higro (Sin Proteccion 0,88; Parasol</t>
         </is>
       </c>
       <c r="B49" s="2" t="n"/>
@@ -9552,7 +9620,11 @@
       <c r="M49" s="2" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="39" t="inlineStr"/>
+      <c r="A50" s="39" t="inlineStr">
+        <is>
+          <t>horizontal fijo 1:2 0,35), que son los mismos de la planilla de la catedra.</t>
+        </is>
+      </c>
       <c r="B50" s="2" t="n"/>
       <c r="C50" s="2" t="n"/>
       <c r="D50" s="2" t="n"/>
@@ -9569,7 +9641,7 @@
     <row r="51">
       <c r="A51" s="39" t="inlineStr">
         <is>
-          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
+          <t>En Datos_higro esta ademas el FES maximo admitido por cuadrante segun la ordenanza, como</t>
         </is>
       </c>
       <c r="B51" s="2" t="n"/>
@@ -9588,7 +9660,7 @@
     <row r="52">
       <c r="A52" s="39" t="inlineStr">
         <is>
-          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
+          <t>referencia: la verificacion no lo controla, igual que en la planilla de la catedra.</t>
         </is>
       </c>
       <c r="B52" s="2" t="n"/>
@@ -9622,7 +9694,7 @@
     <row r="54">
       <c r="A54" s="39" t="inlineStr">
         <is>
-          <t>ALTURAS: medidas sobre el dibujo de las vistas de la planilla de carpinterias, con la escala</t>
+          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
         </is>
       </c>
       <c r="B54" s="2" t="n"/>
@@ -9641,7 +9713,7 @@
     <row r="55">
       <c r="A55" s="39" t="inlineStr">
         <is>
-          <t>verificada contra los anchos acotados (error menor a 2 cm). La mayoria de las aberturas son de</t>
+          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
         </is>
       </c>
       <c r="B55" s="2" t="n"/>
@@ -9658,11 +9730,7 @@
       <c r="M55" s="2" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="39" t="inlineStr">
-        <is>
-          <t>piso a cielorraso, 3,00 m. VERIFICARLAS contra el plano antes de presentar.</t>
-        </is>
-      </c>
+      <c r="A56" s="39" t="inlineStr"/>
       <c r="B56" s="2" t="n"/>
       <c r="C56" s="2" t="n"/>
       <c r="D56" s="2" t="n"/>
@@ -9679,7 +9747,7 @@
     <row r="57">
       <c r="A57" s="39" t="inlineStr">
         <is>
-          <t>PF04 es la unica con antepecho: arranca a 1,09 y mide 0,60 de alto. El resto llega al piso.</t>
+          <t>ALTURAS: medidas sobre el dibujo de las vistas de la planilla de carpinterias, con la escala</t>
         </is>
       </c>
       <c r="B57" s="2" t="n"/>
@@ -9698,7 +9766,7 @@
     <row r="58">
       <c r="A58" s="39" t="inlineStr">
         <is>
-          <t>Las alturas de PV01 (3,00), PF04 (0,60) y PV04 (2) (2,95) las aporto el autor del proyecto.</t>
+          <t>verificada contra los anchos acotados (error menor a 2 cm). La mayoria de las aberturas son de</t>
         </is>
       </c>
       <c r="B58" s="2" t="n"/>
@@ -9715,7 +9783,11 @@
       <c r="M58" s="2" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="39" t="inlineStr"/>
+      <c r="A59" s="39" t="inlineStr">
+        <is>
+          <t>piso a cielorraso, 3,00 m. VERIFICARLAS contra el plano antes de presentar.</t>
+        </is>
+      </c>
       <c r="B59" s="2" t="n"/>
       <c r="C59" s="2" t="n"/>
       <c r="D59" s="2" t="n"/>
@@ -9732,7 +9804,7 @@
     <row r="60">
       <c r="A60" s="39" t="inlineStr">
         <is>
-          <t>ORIENTACION: el simbolo de norte del plano (circulo con aguja, en el patio interno) apunta a</t>
+          <t>PF04 es la unica con antepecho: arranca a 1,09 y mide 0,60 de alto. El resto llega al piso.</t>
         </is>
       </c>
       <c r="B60" s="2" t="n"/>
@@ -9751,7 +9823,7 @@
     <row r="61">
       <c r="A61" s="39" t="inlineStr">
         <is>
-          <t>45 grados hacia arriba y a la derecha de la hoja. Entonces las cuatro fachadas NO son N-S-E-O</t>
+          <t>Las alturas de PV01 (3,00), PF04 (0,60) y PV04 (2) (2,95) las aporto el autor del proyecto.</t>
         </is>
       </c>
       <c r="B61" s="2" t="n"/>
@@ -9768,11 +9840,7 @@
       <c r="M61" s="2" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="39" t="inlineStr">
-        <is>
-          <t>sino: arriba = Noroeste, derecha = Noreste, abajo = Sudeste, izquierda = Sudoeste.</t>
-        </is>
-      </c>
+      <c r="A62" s="39" t="inlineStr"/>
       <c r="B62" s="2" t="n"/>
       <c r="C62" s="2" t="n"/>
       <c r="D62" s="2" t="n"/>
@@ -9789,7 +9857,7 @@
     <row r="63">
       <c r="A63" s="39" t="inlineStr">
         <is>
-          <t>Cada abertura se asigno a la fachada por su posicion en planta. Las del patio interno se</t>
+          <t>ORIENTACION: el simbolo de norte del plano (circulo con aguja, en el patio interno) apunta a</t>
         </is>
       </c>
       <c r="B63" s="2" t="n"/>
@@ -9808,7 +9876,7 @@
     <row r="64">
       <c r="A64" s="39" t="inlineStr">
         <is>
-          <t>orientan por la pared en la que estan: miran hacia adentro del patio.</t>
+          <t>45 grados hacia arriba y a la derecha de la hoja. Entonces las cuatro fachadas NO son N-S-E-O</t>
         </is>
       </c>
       <c r="B64" s="2" t="n"/>
@@ -9827,7 +9895,7 @@
     <row r="65">
       <c r="A65" s="39" t="inlineStr">
         <is>
-          <t>Los rotulos Dormitorio Norte y Dormitorio Sur del plano no coinciden con el norte real;</t>
+          <t>sino: arriba = Noroeste, derecha = Noreste, abajo = Sudeste, izquierda = Sudoeste.</t>
         </is>
       </c>
       <c r="B65" s="2" t="n"/>
@@ -9846,7 +9914,7 @@
     <row r="66">
       <c r="A66" s="39" t="inlineStr">
         <is>
-          <t>parecen ser nombres de uso, no orientaciones.</t>
+          <t>Cada abertura se asigno a la fachada por su posicion en planta. Las del patio interno se</t>
         </is>
       </c>
       <c r="B66" s="2" t="n"/>
@@ -9863,7 +9931,11 @@
       <c r="M66" s="2" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="39" t="inlineStr"/>
+      <c r="A67" s="39" t="inlineStr">
+        <is>
+          <t>orientan por la pared en la que estan: miran hacia adentro del patio.</t>
+        </is>
+      </c>
       <c r="B67" s="2" t="n"/>
       <c r="C67" s="2" t="n"/>
       <c r="D67" s="2" t="n"/>
@@ -9880,7 +9952,7 @@
     <row r="68">
       <c r="A68" s="39" t="inlineStr">
         <is>
-          <t>PF01 figura dos veces en el plano, en las dos paredes laterales del patio interno, y por eso</t>
+          <t>Los rotulos Dormitorio Norte y Dormitorio Sur del plano no coinciden con el norte real;</t>
         </is>
       </c>
       <c r="B68" s="2" t="n"/>
@@ -9899,7 +9971,7 @@
     <row r="69">
       <c r="A69" s="39" t="inlineStr">
         <is>
-          <t>se cargan dos filas. Si fuera una sola abertura rotulada dos veces, borrar la segunda.</t>
+          <t>parecen ser nombres de uso, no orientaciones.</t>
         </is>
       </c>
       <c r="B69" s="2" t="n"/>
@@ -9933,7 +10005,7 @@
     <row r="71">
       <c r="A71" s="39" t="inlineStr">
         <is>
-          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
+          <t>PF01 figura dos veces en el plano, en las dos paredes laterales del patio interno, y por eso</t>
         </is>
       </c>
       <c r="B71" s="2" t="n"/>
@@ -9950,7 +10022,11 @@
       <c r="M71" s="2" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="39" t="inlineStr"/>
+      <c r="A72" s="39" t="inlineStr">
+        <is>
+          <t>se cargan dos filas. Si fuera una sola abertura rotulada dos veces, borrar la segunda.</t>
+        </is>
+      </c>
       <c r="B72" s="2" t="n"/>
       <c r="C72" s="2" t="n"/>
       <c r="D72" s="2" t="n"/>
@@ -9965,11 +10041,7 @@
       <c r="M72" s="2" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="39" t="inlineStr">
-        <is>
-          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
-        </is>
-      </c>
+      <c r="A73" s="39" t="inlineStr"/>
       <c r="B73" s="2" t="n"/>
       <c r="C73" s="2" t="n"/>
       <c r="D73" s="2" t="n"/>
@@ -9986,7 +10058,7 @@
     <row r="74">
       <c r="A74" s="39" t="inlineStr">
         <is>
-          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
+          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
         </is>
       </c>
       <c r="B74" s="2" t="n"/>
@@ -10003,11 +10075,7 @@
       <c r="M74" s="2" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="39" t="inlineStr">
-        <is>
-          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
-        </is>
-      </c>
+      <c r="A75" s="39" t="inlineStr"/>
       <c r="B75" s="2" t="n"/>
       <c r="C75" s="2" t="n"/>
       <c r="D75" s="2" t="n"/>
@@ -10020,6 +10088,63 @@
       <c r="K75" s="2" t="n"/>
       <c r="L75" s="2" t="n"/>
       <c r="M75" s="2" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="39" t="inlineStr">
+        <is>
+          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="n"/>
+      <c r="C76" s="2" t="n"/>
+      <c r="D76" s="2" t="n"/>
+      <c r="E76" s="2" t="n"/>
+      <c r="F76" s="2" t="n"/>
+      <c r="G76" s="2" t="n"/>
+      <c r="H76" s="2" t="n"/>
+      <c r="I76" s="2" t="n"/>
+      <c r="J76" s="2" t="n"/>
+      <c r="K76" s="2" t="n"/>
+      <c r="L76" s="2" t="n"/>
+      <c r="M76" s="2" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="39" t="inlineStr">
+        <is>
+          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="n"/>
+      <c r="C77" s="2" t="n"/>
+      <c r="D77" s="2" t="n"/>
+      <c r="E77" s="2" t="n"/>
+      <c r="F77" s="2" t="n"/>
+      <c r="G77" s="2" t="n"/>
+      <c r="H77" s="2" t="n"/>
+      <c r="I77" s="2" t="n"/>
+      <c r="J77" s="2" t="n"/>
+      <c r="K77" s="2" t="n"/>
+      <c r="L77" s="2" t="n"/>
+      <c r="M77" s="2" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="39" t="inlineStr">
+        <is>
+          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="n"/>
+      <c r="C78" s="2" t="n"/>
+      <c r="D78" s="2" t="n"/>
+      <c r="E78" s="2" t="n"/>
+      <c r="F78" s="2" t="n"/>
+      <c r="G78" s="2" t="n"/>
+      <c r="H78" s="2" t="n"/>
+      <c r="I78" s="2" t="n"/>
+      <c r="J78" s="2" t="n"/>
+      <c r="K78" s="2" t="n"/>
+      <c r="L78" s="2" t="n"/>
+      <c r="M78" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="14">

</xml_diff>

<commit_message>
Planilla 3: sacar la cortina de los panos fijos del patio y de PF04
PF01, su gemelo, PF02, PF03 y PF04 pasan a Sin Proteccion, con factor de
exposicion solar 0,88. El resto queda con cortina de enrollar, 0,25.

Queda anotado en la hoja que ese 0,88 esta muy por encima del maximo de
0,30 que la ordenanza admite para el cuadrante Este/Oeste, donde caen las
cuatro fachadas. La verificacion no lo controla, igual que la planilla de
la catedra, pero es un punto a mirar antes de presentarlo en el municipio.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -7915,7 +7915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M78"/>
+  <dimension ref="A1:M85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8182,7 +8182,7 @@
       </c>
       <c r="I8" s="25" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Sin Proteccion</t>
         </is>
       </c>
       <c r="J8" s="26" t="n">
@@ -8338,7 +8338,7 @@
       </c>
       <c r="I11" s="25" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Sin Proteccion</t>
         </is>
       </c>
       <c r="J11" s="26" t="n">
@@ -8524,7 +8524,7 @@
       </c>
       <c r="I16" s="25" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Sin Proteccion</t>
         </is>
       </c>
       <c r="J16" s="26" t="n">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="I21" s="25" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Sin Proteccion</t>
         </is>
       </c>
       <c r="J21" s="26" t="n">
@@ -8866,7 +8866,7 @@
       </c>
       <c r="I24" s="25" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Sin Proteccion</t>
         </is>
       </c>
       <c r="J24" s="26" t="n">
@@ -9531,7 +9531,7 @@
     <row r="45">
       <c r="A45" s="39" t="inlineStr">
         <is>
-          <t>PROTECCION: se cargo cortina de enrollar exterior en todas las aberturas. Cambiar en la</t>
+          <t>PROTECCION: cortina de enrollar exterior (FES 0,25) en todas, salvo los panos fijos del patio</t>
         </is>
       </c>
       <c r="B45" s="2" t="n"/>
@@ -9550,7 +9550,7 @@
     <row r="46">
       <c r="A46" s="39" t="inlineStr">
         <is>
-          <t>columna I las que no la tengan; el factor de exposicion solar se recalcula solo.</t>
+          <t>(PF01, su gemelo, PF02 y PF03) y PF04, que no la tienen y van Sin Proteccion (FES 0,88).</t>
         </is>
       </c>
       <c r="B46" s="2" t="n"/>
@@ -9584,7 +9584,7 @@
     <row r="48">
       <c r="A48" s="39" t="inlineStr">
         <is>
-          <t>Orientacion: ya cargada. Factor de exposicion solar: se completa SOLO al elegir el tipo de</t>
+          <t>OJO con esas cinco: 0,88 esta muy por encima del maximo de 0,30 que la ordenanza admite para</t>
         </is>
       </c>
       <c r="B48" s="2" t="n"/>
@@ -9603,7 +9603,7 @@
     <row r="49">
       <c r="A49" s="39" t="inlineStr">
         <is>
-          <t>proteccion, con los valores de la tabla de Datos_higro (Sin Proteccion 0,88; Parasol</t>
+          <t>el cuadrante Este/Oeste, donde caen las cuatro fachadas de esta casa por estar girada 45</t>
         </is>
       </c>
       <c r="B49" s="2" t="n"/>
@@ -9622,7 +9622,7 @@
     <row r="50">
       <c r="A50" s="39" t="inlineStr">
         <is>
-          <t>horizontal fijo 1:2 0,35), que son los mismos de la planilla de la catedra.</t>
+          <t>grados. La verificacion de la planilla no lo controla, igual que la de la catedra, pero si lo</t>
         </is>
       </c>
       <c r="B50" s="2" t="n"/>
@@ -9641,7 +9641,7 @@
     <row r="51">
       <c r="A51" s="39" t="inlineStr">
         <is>
-          <t>En Datos_higro esta ademas el FES maximo admitido por cuadrante segun la ordenanza, como</t>
+          <t>presentas en el municipio esas cinco aberturas no pasarian el factor de exposicion solar.</t>
         </is>
       </c>
       <c r="B51" s="2" t="n"/>
@@ -9660,7 +9660,7 @@
     <row r="52">
       <c r="A52" s="39" t="inlineStr">
         <is>
-          <t>referencia: la verificacion no lo controla, igual que en la planilla de la catedra.</t>
+          <t>Hay una salida: si la abertura ocupa menos del 20% del lado expuesto del local, no se verifica</t>
         </is>
       </c>
       <c r="B52" s="2" t="n"/>
@@ -9677,7 +9677,11 @@
       <c r="M52" s="2" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="39" t="inlineStr"/>
+      <c r="A53" s="39" t="inlineStr">
+        <is>
+          <t>el FES. Conviene chequearlo local por local.</t>
+        </is>
+      </c>
       <c r="B53" s="2" t="n"/>
       <c r="C53" s="2" t="n"/>
       <c r="D53" s="2" t="n"/>
@@ -9692,11 +9696,7 @@
       <c r="M53" s="2" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="39" t="inlineStr">
-        <is>
-          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
-        </is>
-      </c>
+      <c r="A54" s="39" t="inlineStr"/>
       <c r="B54" s="2" t="n"/>
       <c r="C54" s="2" t="n"/>
       <c r="D54" s="2" t="n"/>
@@ -9713,7 +9713,7 @@
     <row r="55">
       <c r="A55" s="39" t="inlineStr">
         <is>
-          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
+          <t>Orientacion: ya cargada. Factor de exposicion solar: se completa SOLO al elegir el tipo de</t>
         </is>
       </c>
       <c r="B55" s="2" t="n"/>
@@ -9730,7 +9730,11 @@
       <c r="M55" s="2" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="39" t="inlineStr"/>
+      <c r="A56" s="39" t="inlineStr">
+        <is>
+          <t>proteccion, con los valores de la tabla de Datos_higro (Sin Proteccion 0,88; Parasol</t>
+        </is>
+      </c>
       <c r="B56" s="2" t="n"/>
       <c r="C56" s="2" t="n"/>
       <c r="D56" s="2" t="n"/>
@@ -9747,7 +9751,7 @@
     <row r="57">
       <c r="A57" s="39" t="inlineStr">
         <is>
-          <t>ALTURAS: medidas sobre el dibujo de las vistas de la planilla de carpinterias, con la escala</t>
+          <t>horizontal fijo 1:2 0,35), que son los mismos de la planilla de la catedra.</t>
         </is>
       </c>
       <c r="B57" s="2" t="n"/>
@@ -9766,7 +9770,7 @@
     <row r="58">
       <c r="A58" s="39" t="inlineStr">
         <is>
-          <t>verificada contra los anchos acotados (error menor a 2 cm). La mayoria de las aberturas son de</t>
+          <t>En Datos_higro esta ademas el FES maximo admitido por cuadrante segun la ordenanza, como</t>
         </is>
       </c>
       <c r="B58" s="2" t="n"/>
@@ -9785,7 +9789,7 @@
     <row r="59">
       <c r="A59" s="39" t="inlineStr">
         <is>
-          <t>piso a cielorraso, 3,00 m. VERIFICARLAS contra el plano antes de presentar.</t>
+          <t>referencia: la verificacion no lo controla, igual que en la planilla de la catedra.</t>
         </is>
       </c>
       <c r="B59" s="2" t="n"/>
@@ -9802,11 +9806,7 @@
       <c r="M59" s="2" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="39" t="inlineStr">
-        <is>
-          <t>PF04 es la unica con antepecho: arranca a 1,09 y mide 0,60 de alto. El resto llega al piso.</t>
-        </is>
-      </c>
+      <c r="A60" s="39" t="inlineStr"/>
       <c r="B60" s="2" t="n"/>
       <c r="C60" s="2" t="n"/>
       <c r="D60" s="2" t="n"/>
@@ -9823,7 +9823,7 @@
     <row r="61">
       <c r="A61" s="39" t="inlineStr">
         <is>
-          <t>Las alturas de PV01 (3,00), PF04 (0,60) y PV04 (2) (2,95) las aporto el autor del proyecto.</t>
+          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
         </is>
       </c>
       <c r="B61" s="2" t="n"/>
@@ -9840,7 +9840,11 @@
       <c r="M61" s="2" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="39" t="inlineStr"/>
+      <c r="A62" s="39" t="inlineStr">
+        <is>
+          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
+        </is>
+      </c>
       <c r="B62" s="2" t="n"/>
       <c r="C62" s="2" t="n"/>
       <c r="D62" s="2" t="n"/>
@@ -9855,11 +9859,7 @@
       <c r="M62" s="2" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="39" t="inlineStr">
-        <is>
-          <t>ORIENTACION: el simbolo de norte del plano (circulo con aguja, en el patio interno) apunta a</t>
-        </is>
-      </c>
+      <c r="A63" s="39" t="inlineStr"/>
       <c r="B63" s="2" t="n"/>
       <c r="C63" s="2" t="n"/>
       <c r="D63" s="2" t="n"/>
@@ -9876,7 +9876,7 @@
     <row r="64">
       <c r="A64" s="39" t="inlineStr">
         <is>
-          <t>45 grados hacia arriba y a la derecha de la hoja. Entonces las cuatro fachadas NO son N-S-E-O</t>
+          <t>ALTURAS: medidas sobre el dibujo de las vistas de la planilla de carpinterias, con la escala</t>
         </is>
       </c>
       <c r="B64" s="2" t="n"/>
@@ -9895,7 +9895,7 @@
     <row r="65">
       <c r="A65" s="39" t="inlineStr">
         <is>
-          <t>sino: arriba = Noroeste, derecha = Noreste, abajo = Sudeste, izquierda = Sudoeste.</t>
+          <t>verificada contra los anchos acotados (error menor a 2 cm). La mayoria de las aberturas son de</t>
         </is>
       </c>
       <c r="B65" s="2" t="n"/>
@@ -9914,7 +9914,7 @@
     <row r="66">
       <c r="A66" s="39" t="inlineStr">
         <is>
-          <t>Cada abertura se asigno a la fachada por su posicion en planta. Las del patio interno se</t>
+          <t>piso a cielorraso, 3,00 m. VERIFICARLAS contra el plano antes de presentar.</t>
         </is>
       </c>
       <c r="B66" s="2" t="n"/>
@@ -9933,7 +9933,7 @@
     <row r="67">
       <c r="A67" s="39" t="inlineStr">
         <is>
-          <t>orientan por la pared en la que estan: miran hacia adentro del patio.</t>
+          <t>PF04 es la unica con antepecho: arranca a 1,09 y mide 0,60 de alto. El resto llega al piso.</t>
         </is>
       </c>
       <c r="B67" s="2" t="n"/>
@@ -9952,7 +9952,7 @@
     <row r="68">
       <c r="A68" s="39" t="inlineStr">
         <is>
-          <t>Los rotulos Dormitorio Norte y Dormitorio Sur del plano no coinciden con el norte real;</t>
+          <t>Las alturas de PV01 (3,00), PF04 (0,60) y PV04 (2) (2,95) las aporto el autor del proyecto.</t>
         </is>
       </c>
       <c r="B68" s="2" t="n"/>
@@ -9969,11 +9969,7 @@
       <c r="M68" s="2" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="39" t="inlineStr">
-        <is>
-          <t>parecen ser nombres de uso, no orientaciones.</t>
-        </is>
-      </c>
+      <c r="A69" s="39" t="inlineStr"/>
       <c r="B69" s="2" t="n"/>
       <c r="C69" s="2" t="n"/>
       <c r="D69" s="2" t="n"/>
@@ -9988,7 +9984,11 @@
       <c r="M69" s="2" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="39" t="inlineStr"/>
+      <c r="A70" s="39" t="inlineStr">
+        <is>
+          <t>ORIENTACION: el simbolo de norte del plano (circulo con aguja, en el patio interno) apunta a</t>
+        </is>
+      </c>
       <c r="B70" s="2" t="n"/>
       <c r="C70" s="2" t="n"/>
       <c r="D70" s="2" t="n"/>
@@ -10005,7 +10005,7 @@
     <row r="71">
       <c r="A71" s="39" t="inlineStr">
         <is>
-          <t>PF01 figura dos veces en el plano, en las dos paredes laterales del patio interno, y por eso</t>
+          <t>45 grados hacia arriba y a la derecha de la hoja. Entonces las cuatro fachadas NO son N-S-E-O</t>
         </is>
       </c>
       <c r="B71" s="2" t="n"/>
@@ -10024,7 +10024,7 @@
     <row r="72">
       <c r="A72" s="39" t="inlineStr">
         <is>
-          <t>se cargan dos filas. Si fuera una sola abertura rotulada dos veces, borrar la segunda.</t>
+          <t>sino: arriba = Noroeste, derecha = Noreste, abajo = Sudeste, izquierda = Sudoeste.</t>
         </is>
       </c>
       <c r="B72" s="2" t="n"/>
@@ -10041,7 +10041,11 @@
       <c r="M72" s="2" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="39" t="inlineStr"/>
+      <c r="A73" s="39" t="inlineStr">
+        <is>
+          <t>Cada abertura se asigno a la fachada por su posicion en planta. Las del patio interno se</t>
+        </is>
+      </c>
       <c r="B73" s="2" t="n"/>
       <c r="C73" s="2" t="n"/>
       <c r="D73" s="2" t="n"/>
@@ -10058,7 +10062,7 @@
     <row r="74">
       <c r="A74" s="39" t="inlineStr">
         <is>
-          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
+          <t>orientan por la pared en la que estan: miran hacia adentro del patio.</t>
         </is>
       </c>
       <c r="B74" s="2" t="n"/>
@@ -10075,7 +10079,11 @@
       <c r="M74" s="2" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="39" t="inlineStr"/>
+      <c r="A75" s="39" t="inlineStr">
+        <is>
+          <t>Los rotulos Dormitorio Norte y Dormitorio Sur del plano no coinciden con el norte real;</t>
+        </is>
+      </c>
       <c r="B75" s="2" t="n"/>
       <c r="C75" s="2" t="n"/>
       <c r="D75" s="2" t="n"/>
@@ -10092,7 +10100,7 @@
     <row r="76">
       <c r="A76" s="39" t="inlineStr">
         <is>
-          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
+          <t>parecen ser nombres de uso, no orientaciones.</t>
         </is>
       </c>
       <c r="B76" s="2" t="n"/>
@@ -10109,11 +10117,7 @@
       <c r="M76" s="2" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="39" t="inlineStr">
-        <is>
-          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
-        </is>
-      </c>
+      <c r="A77" s="39" t="inlineStr"/>
       <c r="B77" s="2" t="n"/>
       <c r="C77" s="2" t="n"/>
       <c r="D77" s="2" t="n"/>
@@ -10130,7 +10134,7 @@
     <row r="78">
       <c r="A78" s="39" t="inlineStr">
         <is>
-          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
+          <t>PF01 figura dos veces en el plano, en las dos paredes laterales del patio interno, y por eso</t>
         </is>
       </c>
       <c r="B78" s="2" t="n"/>
@@ -10145,6 +10149,131 @@
       <c r="K78" s="2" t="n"/>
       <c r="L78" s="2" t="n"/>
       <c r="M78" s="2" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="39" t="inlineStr">
+        <is>
+          <t>se cargan dos filas. Si fuera una sola abertura rotulada dos veces, borrar la segunda.</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="n"/>
+      <c r="C79" s="2" t="n"/>
+      <c r="D79" s="2" t="n"/>
+      <c r="E79" s="2" t="n"/>
+      <c r="F79" s="2" t="n"/>
+      <c r="G79" s="2" t="n"/>
+      <c r="H79" s="2" t="n"/>
+      <c r="I79" s="2" t="n"/>
+      <c r="J79" s="2" t="n"/>
+      <c r="K79" s="2" t="n"/>
+      <c r="L79" s="2" t="n"/>
+      <c r="M79" s="2" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="39" t="inlineStr"/>
+      <c r="B80" s="2" t="n"/>
+      <c r="C80" s="2" t="n"/>
+      <c r="D80" s="2" t="n"/>
+      <c r="E80" s="2" t="n"/>
+      <c r="F80" s="2" t="n"/>
+      <c r="G80" s="2" t="n"/>
+      <c r="H80" s="2" t="n"/>
+      <c r="I80" s="2" t="n"/>
+      <c r="J80" s="2" t="n"/>
+      <c r="K80" s="2" t="n"/>
+      <c r="L80" s="2" t="n"/>
+      <c r="M80" s="2" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="39" t="inlineStr">
+        <is>
+          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="n"/>
+      <c r="C81" s="2" t="n"/>
+      <c r="D81" s="2" t="n"/>
+      <c r="E81" s="2" t="n"/>
+      <c r="F81" s="2" t="n"/>
+      <c r="G81" s="2" t="n"/>
+      <c r="H81" s="2" t="n"/>
+      <c r="I81" s="2" t="n"/>
+      <c r="J81" s="2" t="n"/>
+      <c r="K81" s="2" t="n"/>
+      <c r="L81" s="2" t="n"/>
+      <c r="M81" s="2" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="39" t="inlineStr"/>
+      <c r="B82" s="2" t="n"/>
+      <c r="C82" s="2" t="n"/>
+      <c r="D82" s="2" t="n"/>
+      <c r="E82" s="2" t="n"/>
+      <c r="F82" s="2" t="n"/>
+      <c r="G82" s="2" t="n"/>
+      <c r="H82" s="2" t="n"/>
+      <c r="I82" s="2" t="n"/>
+      <c r="J82" s="2" t="n"/>
+      <c r="K82" s="2" t="n"/>
+      <c r="L82" s="2" t="n"/>
+      <c r="M82" s="2" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="39" t="inlineStr">
+        <is>
+          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="n"/>
+      <c r="C83" s="2" t="n"/>
+      <c r="D83" s="2" t="n"/>
+      <c r="E83" s="2" t="n"/>
+      <c r="F83" s="2" t="n"/>
+      <c r="G83" s="2" t="n"/>
+      <c r="H83" s="2" t="n"/>
+      <c r="I83" s="2" t="n"/>
+      <c r="J83" s="2" t="n"/>
+      <c r="K83" s="2" t="n"/>
+      <c r="L83" s="2" t="n"/>
+      <c r="M83" s="2" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="39" t="inlineStr">
+        <is>
+          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="n"/>
+      <c r="C84" s="2" t="n"/>
+      <c r="D84" s="2" t="n"/>
+      <c r="E84" s="2" t="n"/>
+      <c r="F84" s="2" t="n"/>
+      <c r="G84" s="2" t="n"/>
+      <c r="H84" s="2" t="n"/>
+      <c r="I84" s="2" t="n"/>
+      <c r="J84" s="2" t="n"/>
+      <c r="K84" s="2" t="n"/>
+      <c r="L84" s="2" t="n"/>
+      <c r="M84" s="2" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="39" t="inlineStr">
+        <is>
+          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="n"/>
+      <c r="C85" s="2" t="n"/>
+      <c r="D85" s="2" t="n"/>
+      <c r="E85" s="2" t="n"/>
+      <c r="F85" s="2" t="n"/>
+      <c r="G85" s="2" t="n"/>
+      <c r="H85" s="2" t="n"/>
+      <c r="I85" s="2" t="n"/>
+      <c r="J85" s="2" t="n"/>
+      <c r="K85" s="2" t="n"/>
+      <c r="L85" s="2" t="n"/>
+      <c r="M85" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="14">

</xml_diff>

<commit_message>
Planilla 3: PF05 tampoco lleva cortina
Ningun pano fijo PF tiene proteccion solar: los seis van Sin Proteccion,
con factor de exposicion solar 0,88. Las once aberturas restantes llevan
cortina de enrollar exterior, 0,25.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -9208,7 +9208,7 @@
       </c>
       <c r="I32" s="25" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Sin Proteccion</t>
         </is>
       </c>
       <c r="J32" s="26" t="n">
@@ -9531,7 +9531,7 @@
     <row r="45">
       <c r="A45" s="39" t="inlineStr">
         <is>
-          <t>PROTECCION: cortina de enrollar exterior (FES 0,25) en todas, salvo los panos fijos del patio</t>
+          <t>PROTECCION: ningun pano fijo PF tiene cortina: PF01, su gemelo, PF02, PF03, PF04 y PF05 van</t>
         </is>
       </c>
       <c r="B45" s="2" t="n"/>
@@ -9550,7 +9550,7 @@
     <row r="46">
       <c r="A46" s="39" t="inlineStr">
         <is>
-          <t>(PF01, su gemelo, PF02 y PF03) y PF04, que no la tienen y van Sin Proteccion (FES 0,88).</t>
+          <t>Sin Proteccion (FES 0,88). Las otras doce llevan cortina de enrollar exterior (FES 0,25).</t>
         </is>
       </c>
       <c r="B46" s="2" t="n"/>
@@ -9584,7 +9584,7 @@
     <row r="48">
       <c r="A48" s="39" t="inlineStr">
         <is>
-          <t>OJO con esas cinco: 0,88 esta muy por encima del maximo de 0,30 que la ordenanza admite para</t>
+          <t>OJO con esas seis: 0,88 esta muy por encima del maximo de 0,30 que la ordenanza admite para</t>
         </is>
       </c>
       <c r="B48" s="2" t="n"/>

</xml_diff>

<commit_message>
Planilla 3: ubicar PV04 (2) en el dormitorio sur
PV04 (2) pasa a la fachada Sudeste, junto a PV04: son dos aberturas del
mismo dormitorio que comparten rotulo. Se elimina el bloque de ubicacion
a confirmar.

La planilla queda con las 18 aberturas repartidas en las cuatro fachadas,
110,70 m2 de superficie de vanos, y todas verifican.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -29,7 +29,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Iluminacion y ventilacion'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Planilla 3 higrotermica'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla 3 higrotermica'!$A$1:$M$38</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla 3 higrotermica'!$A$1:$M$35</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Planilla vigas'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Planilla vigas'!$A$1:$X$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Planilla losas'!$1:$3</definedName>
@@ -7915,7 +7915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M85"/>
+  <dimension ref="A1:M82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8640,7 +8640,7 @@
         <v/>
       </c>
       <c r="E20" s="28">
-        <f>SUM(D20:D26)</f>
+        <f>SUM(D20:D27)</f>
         <v/>
       </c>
       <c r="F20" s="29">
@@ -8837,14 +8837,14 @@
     <row r="24" ht="17" customHeight="1">
       <c r="A24" s="25" t="inlineStr">
         <is>
-          <t>PF02</t>
+          <t>PV04 (2)</t>
         </is>
       </c>
       <c r="B24" s="26" t="n">
-        <v>3</v>
+        <v>2.95</v>
       </c>
       <c r="C24" s="26" t="n">
-        <v>3.75</v>
+        <v>1.5</v>
       </c>
       <c r="D24" s="27">
         <f>IF(COUNT(B24,C24)&lt;2,"",B24*C24)</f>
@@ -8866,7 +8866,7 @@
       </c>
       <c r="I24" s="25" t="inlineStr">
         <is>
-          <t>Sin Proteccion</t>
+          <t>Cortina de enrollar exterior</t>
         </is>
       </c>
       <c r="J24" s="26" t="n">
@@ -8887,9 +8887,17 @@
       </c>
     </row>
     <row r="25" ht="17" customHeight="1">
-      <c r="A25" s="25" t="n"/>
-      <c r="B25" s="26" t="n"/>
-      <c r="C25" s="26" t="n"/>
+      <c r="A25" s="25" t="inlineStr">
+        <is>
+          <t>PF02</t>
+        </is>
+      </c>
+      <c r="B25" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" s="26" t="n">
+        <v>3.75</v>
+      </c>
       <c r="D25" s="27">
         <f>IF(COUNT(B25,C25)&lt;2,"",B25*C25)</f>
         <v/>
@@ -8903,10 +8911,24 @@
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H25" s="25" t="n"/>
-      <c r="I25" s="25" t="n"/>
-      <c r="J25" s="26" t="n"/>
-      <c r="K25" s="25" t="n"/>
+      <c r="H25" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I25" s="25" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J25" s="26" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K25" s="25" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
       <c r="L25" s="26">
         <f>IF(I25="","",IFERROR(VLOOKUP(I25,Datos_higro!$A$21:$B$27,2,0),""))</f>
         <v/>
@@ -8917,128 +8939,106 @@
       </c>
     </row>
     <row r="26" ht="17" customHeight="1">
-      <c r="A26" s="32" t="n"/>
-      <c r="B26" s="33" t="n"/>
-      <c r="C26" s="33" t="n"/>
-      <c r="D26" s="34">
+      <c r="A26" s="25" t="n"/>
+      <c r="B26" s="26" t="n"/>
+      <c r="C26" s="26" t="n"/>
+      <c r="D26" s="27">
         <f>IF(COUNT(B26,C26)&lt;2,"",B26*C26)</f>
         <v/>
       </c>
-      <c r="E26" s="35" t="n"/>
-      <c r="F26" s="36">
+      <c r="E26" s="31" t="n"/>
+      <c r="F26" s="29">
         <f>IF(OR(D26="",$E$20=""),"",D26/$E$20)</f>
         <v/>
       </c>
-      <c r="G26" s="34">
+      <c r="G26" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H26" s="32" t="n"/>
-      <c r="I26" s="32" t="n"/>
-      <c r="J26" s="33" t="n"/>
-      <c r="K26" s="32" t="n"/>
-      <c r="L26" s="33">
+      <c r="H26" s="25" t="n"/>
+      <c r="I26" s="25" t="n"/>
+      <c r="J26" s="26" t="n"/>
+      <c r="K26" s="25" t="n"/>
+      <c r="L26" s="26">
         <f>IF(I26="","",IFERROR(VLOOKUP(I26,Datos_higro!$A$21:$B$27,2,0),""))</f>
         <v/>
       </c>
-      <c r="M26" s="37">
+      <c r="M26" s="30">
         <f>IF(OR(D26="",J26=""),"",IF(J26&lt;=G26,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="24" t="inlineStr">
+    <row r="27" ht="17" customHeight="1">
+      <c r="A27" s="32" t="n"/>
+      <c r="B27" s="33" t="n"/>
+      <c r="C27" s="33" t="n"/>
+      <c r="D27" s="34">
+        <f>IF(COUNT(B27,C27)&lt;2,"",B27*C27)</f>
+        <v/>
+      </c>
+      <c r="E27" s="35" t="n"/>
+      <c r="F27" s="36">
+        <f>IF(OR(D27="",$E$20=""),"",D27/$E$20)</f>
+        <v/>
+      </c>
+      <c r="G27" s="34">
+        <f>Datos_higro!$B$4</f>
+        <v/>
+      </c>
+      <c r="H27" s="32" t="n"/>
+      <c r="I27" s="32" t="n"/>
+      <c r="J27" s="33" t="n"/>
+      <c r="K27" s="32" t="n"/>
+      <c r="L27" s="33">
+        <f>IF(I27="","",IFERROR(VLOOKUP(I27,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M27" s="37">
+        <f>IF(OR(D27="",J27=""),"",IF(J27&lt;=G27,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="24" t="inlineStr">
         <is>
           <t>Plano: Fachada Noroeste (borde superior)</t>
         </is>
       </c>
-      <c r="B27" s="4" t="n"/>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="4" t="n"/>
-      <c r="G27" s="4" t="n"/>
-      <c r="H27" s="4" t="n"/>
-      <c r="I27" s="4" t="n"/>
-      <c r="J27" s="4" t="n"/>
-      <c r="K27" s="4" t="n"/>
-      <c r="L27" s="4" t="n"/>
-      <c r="M27" s="4" t="n"/>
-    </row>
-    <row r="28" ht="17" customHeight="1">
-      <c r="A28" s="25" t="inlineStr">
-        <is>
-          <t>PV03</t>
-        </is>
-      </c>
-      <c r="B28" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="C28" s="26" t="n">
-        <v>1.76</v>
-      </c>
-      <c r="D28" s="27">
-        <f>IF(COUNT(B28,C28)&lt;2,"",B28*C28)</f>
-        <v/>
-      </c>
-      <c r="E28" s="28">
-        <f>SUM(D28:D34)</f>
-        <v/>
-      </c>
-      <c r="F28" s="29">
-        <f>IF(OR(D28="",$E$28=""),"",D28/$E$28)</f>
-        <v/>
-      </c>
-      <c r="G28" s="27">
-        <f>Datos_higro!$B$4</f>
-        <v/>
-      </c>
-      <c r="H28" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I28" s="25" t="inlineStr">
-        <is>
-          <t>Cortina de enrollar exterior</t>
-        </is>
-      </c>
-      <c r="J28" s="26" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K28" s="25" t="inlineStr">
-        <is>
-          <t>Noroeste</t>
-        </is>
-      </c>
-      <c r="L28" s="26">
-        <f>IF(I28="","",IFERROR(VLOOKUP(I28,Datos_higro!$A$21:$B$27,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M28" s="30">
-        <f>IF(OR(D28="",J28=""),"",IF(J28&lt;=G28,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
+      <c r="B28" s="4" t="n"/>
+      <c r="C28" s="4" t="n"/>
+      <c r="D28" s="4" t="n"/>
+      <c r="E28" s="4" t="n"/>
+      <c r="F28" s="4" t="n"/>
+      <c r="G28" s="4" t="n"/>
+      <c r="H28" s="4" t="n"/>
+      <c r="I28" s="4" t="n"/>
+      <c r="J28" s="4" t="n"/>
+      <c r="K28" s="4" t="n"/>
+      <c r="L28" s="4" t="n"/>
+      <c r="M28" s="4" t="n"/>
     </row>
     <row r="29" ht="17" customHeight="1">
       <c r="A29" s="25" t="inlineStr">
         <is>
-          <t>VA02</t>
+          <t>PV03</t>
         </is>
       </c>
       <c r="B29" s="26" t="n">
-        <v>2.15</v>
+        <v>3</v>
       </c>
       <c r="C29" s="26" t="n">
-        <v>0.75</v>
+        <v>1.76</v>
       </c>
       <c r="D29" s="27">
         <f>IF(COUNT(B29,C29)&lt;2,"",B29*C29)</f>
         <v/>
       </c>
-      <c r="E29" s="31" t="n"/>
+      <c r="E29" s="28">
+        <f>SUM(D29:D35)</f>
+        <v/>
+      </c>
       <c r="F29" s="29">
-        <f>IF(OR(D29="",$E$28=""),"",D29/$E$28)</f>
+        <f>IF(OR(D29="",$E$29=""),"",D29/$E$29)</f>
         <v/>
       </c>
       <c r="G29" s="27">
@@ -9075,11 +9075,11 @@
     <row r="30" ht="17" customHeight="1">
       <c r="A30" s="25" t="inlineStr">
         <is>
-          <t>PA02</t>
+          <t>VA02</t>
         </is>
       </c>
       <c r="B30" s="26" t="n">
-        <v>3</v>
+        <v>2.15</v>
       </c>
       <c r="C30" s="26" t="n">
         <v>0.75</v>
@@ -9090,7 +9090,7 @@
       </c>
       <c r="E30" s="31" t="n"/>
       <c r="F30" s="29">
-        <f>IF(OR(D30="",$E$28=""),"",D30/$E$28)</f>
+        <f>IF(OR(D30="",$E$29=""),"",D30/$E$29)</f>
         <v/>
       </c>
       <c r="G30" s="27">
@@ -9127,11 +9127,11 @@
     <row r="31" ht="17" customHeight="1">
       <c r="A31" s="25" t="inlineStr">
         <is>
-          <t>VA03</t>
+          <t>PA02</t>
         </is>
       </c>
       <c r="B31" s="26" t="n">
-        <v>2.52</v>
+        <v>3</v>
       </c>
       <c r="C31" s="26" t="n">
         <v>0.75</v>
@@ -9142,7 +9142,7 @@
       </c>
       <c r="E31" s="31" t="n"/>
       <c r="F31" s="29">
-        <f>IF(OR(D31="",$E$28=""),"",D31/$E$28)</f>
+        <f>IF(OR(D31="",$E$29=""),"",D31/$E$29)</f>
         <v/>
       </c>
       <c r="G31" s="27">
@@ -9179,7 +9179,7 @@
     <row r="32" ht="17" customHeight="1">
       <c r="A32" s="25" t="inlineStr">
         <is>
-          <t>PF05</t>
+          <t>VA03</t>
         </is>
       </c>
       <c r="B32" s="26" t="n">
@@ -9194,7 +9194,7 @@
       </c>
       <c r="E32" s="31" t="n"/>
       <c r="F32" s="29">
-        <f>IF(OR(D32="",$E$28=""),"",D32/$E$28)</f>
+        <f>IF(OR(D32="",$E$29=""),"",D32/$E$29)</f>
         <v/>
       </c>
       <c r="G32" s="27">
@@ -9208,7 +9208,7 @@
       </c>
       <c r="I32" s="25" t="inlineStr">
         <is>
-          <t>Sin Proteccion</t>
+          <t>Cortina de enrollar exterior</t>
         </is>
       </c>
       <c r="J32" s="26" t="n">
@@ -9229,26 +9229,48 @@
       </c>
     </row>
     <row r="33" ht="17" customHeight="1">
-      <c r="A33" s="25" t="n"/>
-      <c r="B33" s="26" t="n"/>
-      <c r="C33" s="26" t="n"/>
+      <c r="A33" s="25" t="inlineStr">
+        <is>
+          <t>PF05</t>
+        </is>
+      </c>
+      <c r="B33" s="26" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="C33" s="26" t="n">
+        <v>0.75</v>
+      </c>
       <c r="D33" s="27">
         <f>IF(COUNT(B33,C33)&lt;2,"",B33*C33)</f>
         <v/>
       </c>
       <c r="E33" s="31" t="n"/>
       <c r="F33" s="29">
-        <f>IF(OR(D33="",$E$28=""),"",D33/$E$28)</f>
+        <f>IF(OR(D33="",$E$29=""),"",D33/$E$29)</f>
         <v/>
       </c>
       <c r="G33" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H33" s="25" t="n"/>
-      <c r="I33" s="25" t="n"/>
-      <c r="J33" s="26" t="n"/>
-      <c r="K33" s="25" t="n"/>
+      <c r="H33" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I33" s="25" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J33" s="26" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K33" s="25" t="inlineStr">
+        <is>
+          <t>Noroeste</t>
+        </is>
+      </c>
       <c r="L33" s="26">
         <f>IF(I33="","",IFERROR(VLOOKUP(I33,Datos_higro!$A$21:$B$27,2,0),""))</f>
         <v/>
@@ -9259,167 +9281,124 @@
       </c>
     </row>
     <row r="34" ht="17" customHeight="1">
-      <c r="A34" s="32" t="n"/>
-      <c r="B34" s="33" t="n"/>
-      <c r="C34" s="33" t="n"/>
-      <c r="D34" s="34">
+      <c r="A34" s="25" t="n"/>
+      <c r="B34" s="26" t="n"/>
+      <c r="C34" s="26" t="n"/>
+      <c r="D34" s="27">
         <f>IF(COUNT(B34,C34)&lt;2,"",B34*C34)</f>
         <v/>
       </c>
-      <c r="E34" s="35" t="n"/>
-      <c r="F34" s="36">
-        <f>IF(OR(D34="",$E$28=""),"",D34/$E$28)</f>
-        <v/>
-      </c>
-      <c r="G34" s="34">
+      <c r="E34" s="31" t="n"/>
+      <c r="F34" s="29">
+        <f>IF(OR(D34="",$E$29=""),"",D34/$E$29)</f>
+        <v/>
+      </c>
+      <c r="G34" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H34" s="32" t="n"/>
-      <c r="I34" s="32" t="n"/>
-      <c r="J34" s="33" t="n"/>
-      <c r="K34" s="32" t="n"/>
-      <c r="L34" s="33">
+      <c r="H34" s="25" t="n"/>
+      <c r="I34" s="25" t="n"/>
+      <c r="J34" s="26" t="n"/>
+      <c r="K34" s="25" t="n"/>
+      <c r="L34" s="26">
         <f>IF(I34="","",IFERROR(VLOOKUP(I34,Datos_higro!$A$21:$B$27,2,0),""))</f>
         <v/>
       </c>
-      <c r="M34" s="37">
+      <c r="M34" s="30">
         <f>IF(OR(D34="",J34=""),"",IF(J34&lt;=G34,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="24" t="inlineStr">
-        <is>
-          <t>Plano: Ubicacion a confirmar</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="n"/>
-      <c r="C35" s="4" t="n"/>
-      <c r="D35" s="4" t="n"/>
-      <c r="E35" s="4" t="n"/>
-      <c r="F35" s="4" t="n"/>
-      <c r="G35" s="4" t="n"/>
-      <c r="H35" s="4" t="n"/>
-      <c r="I35" s="4" t="n"/>
-      <c r="J35" s="4" t="n"/>
-      <c r="K35" s="4" t="n"/>
-      <c r="L35" s="4" t="n"/>
-      <c r="M35" s="4" t="n"/>
-    </row>
-    <row r="36" ht="17" customHeight="1">
-      <c r="A36" s="25" t="inlineStr">
-        <is>
-          <t>PV04 (2)</t>
-        </is>
-      </c>
-      <c r="B36" s="26" t="n">
-        <v>2.95</v>
-      </c>
-      <c r="C36" s="26" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="D36" s="27">
-        <f>IF(COUNT(B36,C36)&lt;2,"",B36*C36)</f>
-        <v/>
-      </c>
-      <c r="E36" s="28">
-        <f>SUM(D36:D38)</f>
-        <v/>
-      </c>
-      <c r="F36" s="29">
-        <f>IF(OR(D36="",$E$36=""),"",D36/$E$36)</f>
-        <v/>
-      </c>
-      <c r="G36" s="27">
+    <row r="35" ht="17" customHeight="1">
+      <c r="A35" s="32" t="n"/>
+      <c r="B35" s="33" t="n"/>
+      <c r="C35" s="33" t="n"/>
+      <c r="D35" s="34">
+        <f>IF(COUNT(B35,C35)&lt;2,"",B35*C35)</f>
+        <v/>
+      </c>
+      <c r="E35" s="35" t="n"/>
+      <c r="F35" s="36">
+        <f>IF(OR(D35="",$E$29=""),"",D35/$E$29)</f>
+        <v/>
+      </c>
+      <c r="G35" s="34">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H36" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I36" s="25" t="inlineStr">
-        <is>
-          <t>Cortina de enrollar exterior</t>
-        </is>
-      </c>
-      <c r="J36" s="26" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K36" s="25" t="n"/>
-      <c r="L36" s="26">
-        <f>IF(I36="","",IFERROR(VLOOKUP(I36,Datos_higro!$A$21:$B$27,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M36" s="30">
-        <f>IF(OR(D36="",J36=""),"",IF(J36&lt;=G36,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" ht="17" customHeight="1">
-      <c r="A37" s="25" t="n"/>
-      <c r="B37" s="26" t="n"/>
-      <c r="C37" s="26" t="n"/>
-      <c r="D37" s="27">
-        <f>IF(COUNT(B37,C37)&lt;2,"",B37*C37)</f>
-        <v/>
-      </c>
-      <c r="E37" s="31" t="n"/>
-      <c r="F37" s="29">
-        <f>IF(OR(D37="",$E$36=""),"",D37/$E$36)</f>
-        <v/>
-      </c>
-      <c r="G37" s="27">
-        <f>Datos_higro!$B$4</f>
-        <v/>
-      </c>
-      <c r="H37" s="25" t="n"/>
-      <c r="I37" s="25" t="n"/>
-      <c r="J37" s="26" t="n"/>
-      <c r="K37" s="25" t="n"/>
-      <c r="L37" s="26">
-        <f>IF(I37="","",IFERROR(VLOOKUP(I37,Datos_higro!$A$21:$B$27,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M37" s="30">
-        <f>IF(OR(D37="",J37=""),"",IF(J37&lt;=G37,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" ht="17" customHeight="1">
-      <c r="A38" s="32" t="n"/>
-      <c r="B38" s="33" t="n"/>
-      <c r="C38" s="33" t="n"/>
-      <c r="D38" s="34">
-        <f>IF(COUNT(B38,C38)&lt;2,"",B38*C38)</f>
-        <v/>
-      </c>
-      <c r="E38" s="35" t="n"/>
-      <c r="F38" s="36">
-        <f>IF(OR(D38="",$E$36=""),"",D38/$E$36)</f>
-        <v/>
-      </c>
-      <c r="G38" s="34">
-        <f>Datos_higro!$B$4</f>
-        <v/>
-      </c>
-      <c r="H38" s="32" t="n"/>
-      <c r="I38" s="32" t="n"/>
-      <c r="J38" s="33" t="n"/>
-      <c r="K38" s="32" t="n"/>
-      <c r="L38" s="33">
-        <f>IF(I38="","",IFERROR(VLOOKUP(I38,Datos_higro!$A$21:$B$27,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M38" s="37">
-        <f>IF(OR(D38="",J38=""),"",IF(J38&lt;=G38,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
+      <c r="H35" s="32" t="n"/>
+      <c r="I35" s="32" t="n"/>
+      <c r="J35" s="33" t="n"/>
+      <c r="K35" s="32" t="n"/>
+      <c r="L35" s="33">
+        <f>IF(I35="","",IFERROR(VLOOKUP(I35,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M35" s="37">
+        <f>IF(OR(D35="",J35=""),"",IF(J35&lt;=G35,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n"/>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="n"/>
+      <c r="H36" s="2" t="n"/>
+      <c r="I36" s="2" t="n"/>
+      <c r="J36" s="2" t="n"/>
+      <c r="K36" s="2" t="n"/>
+      <c r="L36" s="2" t="n"/>
+      <c r="M36" s="2" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="38" t="inlineStr">
+        <is>
+          <t>COMO SE COMPLETA</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="n"/>
+      <c r="H37" s="2" t="n"/>
+      <c r="I37" s="2" t="n"/>
+      <c r="J37" s="2" t="n"/>
+      <c r="K37" s="2" t="n"/>
+      <c r="L37" s="2" t="n"/>
+      <c r="M37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="39" t="inlineStr">
+        <is>
+          <t>Descripcion, altura y ancho del vano: de la planilla de carpinterias.</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+      <c r="G38" s="2" t="n"/>
+      <c r="H38" s="2" t="n"/>
+      <c r="I38" s="2" t="n"/>
+      <c r="J38" s="2" t="n"/>
+      <c r="K38" s="2" t="n"/>
+      <c r="L38" s="2" t="n"/>
+      <c r="M38" s="2" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n"/>
+      <c r="A39" s="39" t="inlineStr">
+        <is>
+          <t>Area del vano, area total por plano y porcentaje: se calculan solos.</t>
+        </is>
+      </c>
       <c r="B39" s="2" t="n"/>
       <c r="C39" s="2" t="n"/>
       <c r="D39" s="2" t="n"/>
@@ -9434,9 +9413,9 @@
       <c r="M39" s="2" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="38" t="inlineStr">
-        <is>
-          <t>COMO SE COMPLETA</t>
+      <c r="A40" s="39" t="inlineStr">
+        <is>
+          <t>Tipo de vidrio y tipo de proteccion: desplegables; sus valores estan en la hoja Datos_higro.</t>
         </is>
       </c>
       <c r="B40" s="2" t="n"/>
@@ -9455,7 +9434,7 @@
     <row r="41">
       <c r="A41" s="39" t="inlineStr">
         <is>
-          <t>Descripcion, altura y ancho del vano: de la planilla de carpinterias.</t>
+          <t>Transmitancia del cerramiento: cargarla segun el vidrio y el marco adoptados.</t>
         </is>
       </c>
       <c r="B41" s="2" t="n"/>
@@ -9474,7 +9453,7 @@
     <row r="42">
       <c r="A42" s="39" t="inlineStr">
         <is>
-          <t>Area del vano, area total por plano y porcentaje: se calculan solos.</t>
+          <t>PROTECCION: ningun pano fijo PF tiene cortina: PF01, su gemelo, PF02, PF03, PF04 y PF05 van</t>
         </is>
       </c>
       <c r="B42" s="2" t="n"/>
@@ -9493,7 +9472,7 @@
     <row r="43">
       <c r="A43" s="39" t="inlineStr">
         <is>
-          <t>Tipo de vidrio y tipo de proteccion: desplegables; sus valores estan en la hoja Datos_higro.</t>
+          <t>Sin Proteccion (FES 0,88). Las otras doce llevan cortina de enrollar exterior (FES 0,25).</t>
         </is>
       </c>
       <c r="B43" s="2" t="n"/>
@@ -9510,11 +9489,7 @@
       <c r="M43" s="2" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="39" t="inlineStr">
-        <is>
-          <t>Transmitancia del cerramiento: cargarla segun el vidrio y el marco adoptados.</t>
-        </is>
-      </c>
+      <c r="A44" s="39" t="inlineStr"/>
       <c r="B44" s="2" t="n"/>
       <c r="C44" s="2" t="n"/>
       <c r="D44" s="2" t="n"/>
@@ -9531,7 +9506,7 @@
     <row r="45">
       <c r="A45" s="39" t="inlineStr">
         <is>
-          <t>PROTECCION: ningun pano fijo PF tiene cortina: PF01, su gemelo, PF02, PF03, PF04 y PF05 van</t>
+          <t>OJO con esas seis: 0,88 esta muy por encima del maximo de 0,30 que la ordenanza admite para</t>
         </is>
       </c>
       <c r="B45" s="2" t="n"/>
@@ -9550,7 +9525,7 @@
     <row r="46">
       <c r="A46" s="39" t="inlineStr">
         <is>
-          <t>Sin Proteccion (FES 0,88). Las otras doce llevan cortina de enrollar exterior (FES 0,25).</t>
+          <t>el cuadrante Este/Oeste, donde caen las cuatro fachadas de esta casa por estar girada 45</t>
         </is>
       </c>
       <c r="B46" s="2" t="n"/>
@@ -9567,7 +9542,11 @@
       <c r="M46" s="2" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="39" t="inlineStr"/>
+      <c r="A47" s="39" t="inlineStr">
+        <is>
+          <t>grados. La verificacion de la planilla no lo controla, igual que la de la catedra, pero si lo</t>
+        </is>
+      </c>
       <c r="B47" s="2" t="n"/>
       <c r="C47" s="2" t="n"/>
       <c r="D47" s="2" t="n"/>
@@ -9584,7 +9563,7 @@
     <row r="48">
       <c r="A48" s="39" t="inlineStr">
         <is>
-          <t>OJO con esas seis: 0,88 esta muy por encima del maximo de 0,30 que la ordenanza admite para</t>
+          <t>presentas en el municipio esas cinco aberturas no pasarian el factor de exposicion solar.</t>
         </is>
       </c>
       <c r="B48" s="2" t="n"/>
@@ -9603,7 +9582,7 @@
     <row r="49">
       <c r="A49" s="39" t="inlineStr">
         <is>
-          <t>el cuadrante Este/Oeste, donde caen las cuatro fachadas de esta casa por estar girada 45</t>
+          <t>Hay una salida: si la abertura ocupa menos del 20% del lado expuesto del local, no se verifica</t>
         </is>
       </c>
       <c r="B49" s="2" t="n"/>
@@ -9622,7 +9601,7 @@
     <row r="50">
       <c r="A50" s="39" t="inlineStr">
         <is>
-          <t>grados. La verificacion de la planilla no lo controla, igual que la de la catedra, pero si lo</t>
+          <t>el FES. Conviene chequearlo local por local.</t>
         </is>
       </c>
       <c r="B50" s="2" t="n"/>
@@ -9639,11 +9618,7 @@
       <c r="M50" s="2" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="39" t="inlineStr">
-        <is>
-          <t>presentas en el municipio esas cinco aberturas no pasarian el factor de exposicion solar.</t>
-        </is>
-      </c>
+      <c r="A51" s="39" t="inlineStr"/>
       <c r="B51" s="2" t="n"/>
       <c r="C51" s="2" t="n"/>
       <c r="D51" s="2" t="n"/>
@@ -9660,7 +9635,7 @@
     <row r="52">
       <c r="A52" s="39" t="inlineStr">
         <is>
-          <t>Hay una salida: si la abertura ocupa menos del 20% del lado expuesto del local, no se verifica</t>
+          <t>Orientacion: ya cargada. Factor de exposicion solar: se completa SOLO al elegir el tipo de</t>
         </is>
       </c>
       <c r="B52" s="2" t="n"/>
@@ -9679,7 +9654,7 @@
     <row r="53">
       <c r="A53" s="39" t="inlineStr">
         <is>
-          <t>el FES. Conviene chequearlo local por local.</t>
+          <t>proteccion, con los valores de la tabla de Datos_higro (Sin Proteccion 0,88; Parasol</t>
         </is>
       </c>
       <c r="B53" s="2" t="n"/>
@@ -9696,7 +9671,11 @@
       <c r="M53" s="2" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="39" t="inlineStr"/>
+      <c r="A54" s="39" t="inlineStr">
+        <is>
+          <t>horizontal fijo 1:2 0,35), que son los mismos de la planilla de la catedra.</t>
+        </is>
+      </c>
       <c r="B54" s="2" t="n"/>
       <c r="C54" s="2" t="n"/>
       <c r="D54" s="2" t="n"/>
@@ -9713,7 +9692,7 @@
     <row r="55">
       <c r="A55" s="39" t="inlineStr">
         <is>
-          <t>Orientacion: ya cargada. Factor de exposicion solar: se completa SOLO al elegir el tipo de</t>
+          <t>En Datos_higro esta ademas el FES maximo admitido por cuadrante segun la ordenanza, como</t>
         </is>
       </c>
       <c r="B55" s="2" t="n"/>
@@ -9732,7 +9711,7 @@
     <row r="56">
       <c r="A56" s="39" t="inlineStr">
         <is>
-          <t>proteccion, con los valores de la tabla de Datos_higro (Sin Proteccion 0,88; Parasol</t>
+          <t>referencia: la verificacion no lo controla, igual que en la planilla de la catedra.</t>
         </is>
       </c>
       <c r="B56" s="2" t="n"/>
@@ -9749,11 +9728,7 @@
       <c r="M56" s="2" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="39" t="inlineStr">
-        <is>
-          <t>horizontal fijo 1:2 0,35), que son los mismos de la planilla de la catedra.</t>
-        </is>
-      </c>
+      <c r="A57" s="39" t="inlineStr"/>
       <c r="B57" s="2" t="n"/>
       <c r="C57" s="2" t="n"/>
       <c r="D57" s="2" t="n"/>
@@ -9770,7 +9745,7 @@
     <row r="58">
       <c r="A58" s="39" t="inlineStr">
         <is>
-          <t>En Datos_higro esta ademas el FES maximo admitido por cuadrante segun la ordenanza, como</t>
+          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
         </is>
       </c>
       <c r="B58" s="2" t="n"/>
@@ -9789,7 +9764,7 @@
     <row r="59">
       <c r="A59" s="39" t="inlineStr">
         <is>
-          <t>referencia: la verificacion no lo controla, igual que en la planilla de la catedra.</t>
+          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
         </is>
       </c>
       <c r="B59" s="2" t="n"/>
@@ -9823,7 +9798,7 @@
     <row r="61">
       <c r="A61" s="39" t="inlineStr">
         <is>
-          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
+          <t>ALTURAS: medidas sobre el dibujo de las vistas de la planilla de carpinterias, con la escala</t>
         </is>
       </c>
       <c r="B61" s="2" t="n"/>
@@ -9842,7 +9817,7 @@
     <row r="62">
       <c r="A62" s="39" t="inlineStr">
         <is>
-          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
+          <t>verificada contra los anchos acotados (error menor a 2 cm). La mayoria de las aberturas son de</t>
         </is>
       </c>
       <c r="B62" s="2" t="n"/>
@@ -9859,7 +9834,11 @@
       <c r="M62" s="2" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="39" t="inlineStr"/>
+      <c r="A63" s="39" t="inlineStr">
+        <is>
+          <t>piso a cielorraso, 3,00 m. VERIFICARLAS contra el plano antes de presentar.</t>
+        </is>
+      </c>
       <c r="B63" s="2" t="n"/>
       <c r="C63" s="2" t="n"/>
       <c r="D63" s="2" t="n"/>
@@ -9876,7 +9855,7 @@
     <row r="64">
       <c r="A64" s="39" t="inlineStr">
         <is>
-          <t>ALTURAS: medidas sobre el dibujo de las vistas de la planilla de carpinterias, con la escala</t>
+          <t>PF04 es la unica con antepecho: arranca a 1,09 y mide 0,60 de alto. El resto llega al piso.</t>
         </is>
       </c>
       <c r="B64" s="2" t="n"/>
@@ -9895,7 +9874,7 @@
     <row r="65">
       <c r="A65" s="39" t="inlineStr">
         <is>
-          <t>verificada contra los anchos acotados (error menor a 2 cm). La mayoria de las aberturas son de</t>
+          <t>Las alturas de PV01 (3,00), PF04 (0,60) y PV04 (2) (2,95) las aporto el autor del proyecto.</t>
         </is>
       </c>
       <c r="B65" s="2" t="n"/>
@@ -9912,11 +9891,7 @@
       <c r="M65" s="2" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="39" t="inlineStr">
-        <is>
-          <t>piso a cielorraso, 3,00 m. VERIFICARLAS contra el plano antes de presentar.</t>
-        </is>
-      </c>
+      <c r="A66" s="39" t="inlineStr"/>
       <c r="B66" s="2" t="n"/>
       <c r="C66" s="2" t="n"/>
       <c r="D66" s="2" t="n"/>
@@ -9933,7 +9908,7 @@
     <row r="67">
       <c r="A67" s="39" t="inlineStr">
         <is>
-          <t>PF04 es la unica con antepecho: arranca a 1,09 y mide 0,60 de alto. El resto llega al piso.</t>
+          <t>ORIENTACION: el simbolo de norte del plano (circulo con aguja, en el patio interno) apunta a</t>
         </is>
       </c>
       <c r="B67" s="2" t="n"/>
@@ -9952,7 +9927,7 @@
     <row r="68">
       <c r="A68" s="39" t="inlineStr">
         <is>
-          <t>Las alturas de PV01 (3,00), PF04 (0,60) y PV04 (2) (2,95) las aporto el autor del proyecto.</t>
+          <t>45 grados hacia arriba y a la derecha de la hoja. Entonces las cuatro fachadas NO son N-S-E-O</t>
         </is>
       </c>
       <c r="B68" s="2" t="n"/>
@@ -9969,7 +9944,11 @@
       <c r="M68" s="2" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="39" t="inlineStr"/>
+      <c r="A69" s="39" t="inlineStr">
+        <is>
+          <t>sino: arriba = Noroeste, derecha = Noreste, abajo = Sudeste, izquierda = Sudoeste.</t>
+        </is>
+      </c>
       <c r="B69" s="2" t="n"/>
       <c r="C69" s="2" t="n"/>
       <c r="D69" s="2" t="n"/>
@@ -9986,7 +9965,7 @@
     <row r="70">
       <c r="A70" s="39" t="inlineStr">
         <is>
-          <t>ORIENTACION: el simbolo de norte del plano (circulo con aguja, en el patio interno) apunta a</t>
+          <t>Cada abertura se asigno a la fachada por su posicion en planta. Las del patio interno se</t>
         </is>
       </c>
       <c r="B70" s="2" t="n"/>
@@ -10005,7 +9984,7 @@
     <row r="71">
       <c r="A71" s="39" t="inlineStr">
         <is>
-          <t>45 grados hacia arriba y a la derecha de la hoja. Entonces las cuatro fachadas NO son N-S-E-O</t>
+          <t>orientan por la pared en la que estan: miran hacia adentro del patio.</t>
         </is>
       </c>
       <c r="B71" s="2" t="n"/>
@@ -10024,7 +10003,7 @@
     <row r="72">
       <c r="A72" s="39" t="inlineStr">
         <is>
-          <t>sino: arriba = Noroeste, derecha = Noreste, abajo = Sudeste, izquierda = Sudoeste.</t>
+          <t>Los rotulos Dormitorio Norte y Dormitorio Sur del plano no coinciden con el norte real;</t>
         </is>
       </c>
       <c r="B72" s="2" t="n"/>
@@ -10043,7 +10022,7 @@
     <row r="73">
       <c r="A73" s="39" t="inlineStr">
         <is>
-          <t>Cada abertura se asigno a la fachada por su posicion en planta. Las del patio interno se</t>
+          <t>parecen ser nombres de uso, no orientaciones.</t>
         </is>
       </c>
       <c r="B73" s="2" t="n"/>
@@ -10060,11 +10039,7 @@
       <c r="M73" s="2" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="39" t="inlineStr">
-        <is>
-          <t>orientan por la pared en la que estan: miran hacia adentro del patio.</t>
-        </is>
-      </c>
+      <c r="A74" s="39" t="inlineStr"/>
       <c r="B74" s="2" t="n"/>
       <c r="C74" s="2" t="n"/>
       <c r="D74" s="2" t="n"/>
@@ -10081,7 +10056,7 @@
     <row r="75">
       <c r="A75" s="39" t="inlineStr">
         <is>
-          <t>Los rotulos Dormitorio Norte y Dormitorio Sur del plano no coinciden con el norte real;</t>
+          <t>PF01 figura dos veces en el plano, en las dos paredes laterales del patio interno, y por eso</t>
         </is>
       </c>
       <c r="B75" s="2" t="n"/>
@@ -10100,7 +10075,7 @@
     <row r="76">
       <c r="A76" s="39" t="inlineStr">
         <is>
-          <t>parecen ser nombres de uso, no orientaciones.</t>
+          <t>se cargan dos filas. Si fuera una sola abertura rotulada dos veces, borrar la segunda.</t>
         </is>
       </c>
       <c r="B76" s="2" t="n"/>
@@ -10134,7 +10109,7 @@
     <row r="78">
       <c r="A78" s="39" t="inlineStr">
         <is>
-          <t>PF01 figura dos veces en el plano, en las dos paredes laterales del patio interno, y por eso</t>
+          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
         </is>
       </c>
       <c r="B78" s="2" t="n"/>
@@ -10151,11 +10126,7 @@
       <c r="M78" s="2" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="39" t="inlineStr">
-        <is>
-          <t>se cargan dos filas. Si fuera una sola abertura rotulada dos veces, borrar la segunda.</t>
-        </is>
-      </c>
+      <c r="A79" s="39" t="inlineStr"/>
       <c r="B79" s="2" t="n"/>
       <c r="C79" s="2" t="n"/>
       <c r="D79" s="2" t="n"/>
@@ -10170,7 +10141,11 @@
       <c r="M79" s="2" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="39" t="inlineStr"/>
+      <c r="A80" s="39" t="inlineStr">
+        <is>
+          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
+        </is>
+      </c>
       <c r="B80" s="2" t="n"/>
       <c r="C80" s="2" t="n"/>
       <c r="D80" s="2" t="n"/>
@@ -10187,7 +10162,7 @@
     <row r="81">
       <c r="A81" s="39" t="inlineStr">
         <is>
-          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
+          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
         </is>
       </c>
       <c r="B81" s="2" t="n"/>
@@ -10204,7 +10179,11 @@
       <c r="M81" s="2" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="39" t="inlineStr"/>
+      <c r="A82" s="39" t="inlineStr">
+        <is>
+          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
+        </is>
+      </c>
       <c r="B82" s="2" t="n"/>
       <c r="C82" s="2" t="n"/>
       <c r="D82" s="2" t="n"/>
@@ -10218,81 +10197,22 @@
       <c r="L82" s="2" t="n"/>
       <c r="M82" s="2" t="n"/>
     </row>
-    <row r="83">
-      <c r="A83" s="39" t="inlineStr">
-        <is>
-          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
-        </is>
-      </c>
-      <c r="B83" s="2" t="n"/>
-      <c r="C83" s="2" t="n"/>
-      <c r="D83" s="2" t="n"/>
-      <c r="E83" s="2" t="n"/>
-      <c r="F83" s="2" t="n"/>
-      <c r="G83" s="2" t="n"/>
-      <c r="H83" s="2" t="n"/>
-      <c r="I83" s="2" t="n"/>
-      <c r="J83" s="2" t="n"/>
-      <c r="K83" s="2" t="n"/>
-      <c r="L83" s="2" t="n"/>
-      <c r="M83" s="2" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="39" t="inlineStr">
-        <is>
-          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
-        </is>
-      </c>
-      <c r="B84" s="2" t="n"/>
-      <c r="C84" s="2" t="n"/>
-      <c r="D84" s="2" t="n"/>
-      <c r="E84" s="2" t="n"/>
-      <c r="F84" s="2" t="n"/>
-      <c r="G84" s="2" t="n"/>
-      <c r="H84" s="2" t="n"/>
-      <c r="I84" s="2" t="n"/>
-      <c r="J84" s="2" t="n"/>
-      <c r="K84" s="2" t="n"/>
-      <c r="L84" s="2" t="n"/>
-      <c r="M84" s="2" t="n"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="39" t="inlineStr">
-        <is>
-          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
-        </is>
-      </c>
-      <c r="B85" s="2" t="n"/>
-      <c r="C85" s="2" t="n"/>
-      <c r="D85" s="2" t="n"/>
-      <c r="E85" s="2" t="n"/>
-      <c r="F85" s="2" t="n"/>
-      <c r="G85" s="2" t="n"/>
-      <c r="H85" s="2" t="n"/>
-      <c r="I85" s="2" t="n"/>
-      <c r="J85" s="2" t="n"/>
-      <c r="K85" s="2" t="n"/>
-      <c r="L85" s="2" t="n"/>
-      <c r="M85" s="2" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="E36:E38"/>
+  <mergeCells count="12">
     <mergeCell ref="A19:M19"/>
     <mergeCell ref="A14:M14"/>
-    <mergeCell ref="E20:E26"/>
     <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A27:M27"/>
-    <mergeCell ref="E28:E34"/>
     <mergeCell ref="A6:M6"/>
-    <mergeCell ref="A35:M35"/>
+    <mergeCell ref="E20:E27"/>
     <mergeCell ref="A4:M4"/>
+    <mergeCell ref="E29:E35"/>
     <mergeCell ref="A3:M3"/>
     <mergeCell ref="E7:E13"/>
     <mergeCell ref="E15:E18"/>
     <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A28:M28"/>
   </mergeCells>
-  <conditionalFormatting sqref="M6:M38">
+  <conditionalFormatting sqref="M6:M35">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
       <formula>"CUMPLE"</formula>
     </cfRule>
@@ -10301,13 +10221,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="H6:H38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Datos_higro!$A$10:$A$17</formula1>
     </dataValidation>
-    <dataValidation sqref="I6:I38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I6:I35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Datos_higro!$A$21:$A$27</formula1>
     </dataValidation>
-    <dataValidation sqref="K6:K38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K6:K35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Norte,Sur,Este,Oeste,Noreste,Noroeste,Sudeste,Sudoeste,Horizontal"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Planilla 3: cargar las cantidades y las ubicaciones reales
La planilla de carpinterias trae un campo CANTIDAD que no se habia leido.
Tres aberturas van dos veces y faltaban filas:

- VA01 x2: 01 Cocina y 09 Suite
- VA04 x2: 13 Dormitorio Norte y 14 Play Room
- PF01 x2: 03 Lavadero y 07 Hall de ingreso, a los dos lados del patio
  interno, lo que confirma los dos rotulos del plano

La planilla pasa de 17 a 20 filas y de 110,70 a 117,99 m2. Las
ubicaciones dejan de ser deducidas del plano: se toman del campo
UBICACION de cada ficha, con el numero de local.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -29,7 +29,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Iluminacion y ventilacion'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Planilla 3 higrotermica'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla 3 higrotermica'!$A$1:$M$35</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla 3 higrotermica'!$A$1:$M$37</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Planilla vigas'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Planilla vigas'!$A$1:$X$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Planilla losas'!$1:$3</definedName>
@@ -7915,7 +7915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M82"/>
+  <dimension ref="A1:M86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8112,7 +8112,7 @@
         <v/>
       </c>
       <c r="E7" s="28">
-        <f>SUM(D7:D13)</f>
+        <f>SUM(D7:D14)</f>
         <v/>
       </c>
       <c r="F7" s="29">
@@ -8257,14 +8257,14 @@
     <row r="10" ht="17" customHeight="1">
       <c r="A10" s="25" t="inlineStr">
         <is>
-          <t>PV01</t>
+          <t>VA04 (2)</t>
         </is>
       </c>
       <c r="B10" s="26" t="n">
-        <v>3</v>
+        <v>2.52</v>
       </c>
       <c r="C10" s="26" t="n">
-        <v>7.7</v>
+        <v>2</v>
       </c>
       <c r="D10" s="27">
         <f>IF(COUNT(B10,C10)&lt;2,"",B10*C10)</f>
@@ -8309,14 +8309,14 @@
     <row r="11" ht="17" customHeight="1">
       <c r="A11" s="25" t="inlineStr">
         <is>
-          <t>PF01</t>
+          <t>PV01</t>
         </is>
       </c>
       <c r="B11" s="26" t="n">
         <v>3</v>
       </c>
       <c r="C11" s="26" t="n">
-        <v>3.55</v>
+        <v>7.7</v>
       </c>
       <c r="D11" s="27">
         <f>IF(COUNT(B11,C11)&lt;2,"",B11*C11)</f>
@@ -8338,7 +8338,7 @@
       </c>
       <c r="I11" s="25" t="inlineStr">
         <is>
-          <t>Sin Proteccion</t>
+          <t>Cortina de enrollar exterior</t>
         </is>
       </c>
       <c r="J11" s="26" t="n">
@@ -8359,9 +8359,17 @@
       </c>
     </row>
     <row r="12" ht="17" customHeight="1">
-      <c r="A12" s="25" t="n"/>
-      <c r="B12" s="26" t="n"/>
-      <c r="C12" s="26" t="n"/>
+      <c r="A12" s="25" t="inlineStr">
+        <is>
+          <t>PF01</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" s="26" t="n">
+        <v>3.55</v>
+      </c>
       <c r="D12" s="27">
         <f>IF(COUNT(B12,C12)&lt;2,"",B12*C12)</f>
         <v/>
@@ -8375,10 +8383,24 @@
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H12" s="25" t="n"/>
-      <c r="I12" s="25" t="n"/>
-      <c r="J12" s="26" t="n"/>
-      <c r="K12" s="25" t="n"/>
+      <c r="H12" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I12" s="25" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J12" s="26" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K12" s="25" t="inlineStr">
+        <is>
+          <t>Noreste</t>
+        </is>
+      </c>
       <c r="L12" s="26">
         <f>IF(I12="","",IFERROR(VLOOKUP(I12,Datos_higro!$A$21:$B$27,2,0),""))</f>
         <v/>
@@ -8389,128 +8411,106 @@
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
-      <c r="A13" s="32" t="n"/>
-      <c r="B13" s="33" t="n"/>
-      <c r="C13" s="33" t="n"/>
-      <c r="D13" s="34">
+      <c r="A13" s="25" t="n"/>
+      <c r="B13" s="26" t="n"/>
+      <c r="C13" s="26" t="n"/>
+      <c r="D13" s="27">
         <f>IF(COUNT(B13,C13)&lt;2,"",B13*C13)</f>
         <v/>
       </c>
-      <c r="E13" s="35" t="n"/>
-      <c r="F13" s="36">
+      <c r="E13" s="31" t="n"/>
+      <c r="F13" s="29">
         <f>IF(OR(D13="",$E$7=""),"",D13/$E$7)</f>
         <v/>
       </c>
-      <c r="G13" s="34">
+      <c r="G13" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H13" s="32" t="n"/>
-      <c r="I13" s="32" t="n"/>
-      <c r="J13" s="33" t="n"/>
-      <c r="K13" s="32" t="n"/>
-      <c r="L13" s="33">
+      <c r="H13" s="25" t="n"/>
+      <c r="I13" s="25" t="n"/>
+      <c r="J13" s="26" t="n"/>
+      <c r="K13" s="25" t="n"/>
+      <c r="L13" s="26">
         <f>IF(I13="","",IFERROR(VLOOKUP(I13,Datos_higro!$A$21:$B$27,2,0),""))</f>
         <v/>
       </c>
-      <c r="M13" s="37">
+      <c r="M13" s="30">
         <f>IF(OR(D13="",J13=""),"",IF(J13&lt;=G13,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="24" t="inlineStr">
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" s="32" t="n"/>
+      <c r="B14" s="33" t="n"/>
+      <c r="C14" s="33" t="n"/>
+      <c r="D14" s="34">
+        <f>IF(COUNT(B14,C14)&lt;2,"",B14*C14)</f>
+        <v/>
+      </c>
+      <c r="E14" s="35" t="n"/>
+      <c r="F14" s="36">
+        <f>IF(OR(D14="",$E$7=""),"",D14/$E$7)</f>
+        <v/>
+      </c>
+      <c r="G14" s="34">
+        <f>Datos_higro!$B$4</f>
+        <v/>
+      </c>
+      <c r="H14" s="32" t="n"/>
+      <c r="I14" s="32" t="n"/>
+      <c r="J14" s="33" t="n"/>
+      <c r="K14" s="32" t="n"/>
+      <c r="L14" s="33">
+        <f>IF(I14="","",IFERROR(VLOOKUP(I14,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M14" s="37">
+        <f>IF(OR(D14="",J14=""),"",IF(J14&lt;=G14,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="24" t="inlineStr">
         <is>
           <t>Plano: Fachada Sudoeste (borde izquierdo)</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="4" t="n"/>
-      <c r="F14" s="4" t="n"/>
-      <c r="G14" s="4" t="n"/>
-      <c r="H14" s="4" t="n"/>
-      <c r="I14" s="4" t="n"/>
-      <c r="J14" s="4" t="n"/>
-      <c r="K14" s="4" t="n"/>
-      <c r="L14" s="4" t="n"/>
-      <c r="M14" s="4" t="n"/>
-    </row>
-    <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="25" t="inlineStr">
-        <is>
-          <t>VA01</t>
-        </is>
-      </c>
-      <c r="B15" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="C15" s="26" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D15" s="27">
-        <f>IF(COUNT(B15,C15)&lt;2,"",B15*C15)</f>
-        <v/>
-      </c>
-      <c r="E15" s="28">
-        <f>SUM(D15:D18)</f>
-        <v/>
-      </c>
-      <c r="F15" s="29">
-        <f>IF(OR(D15="",$E$15=""),"",D15/$E$15)</f>
-        <v/>
-      </c>
-      <c r="G15" s="27">
-        <f>Datos_higro!$B$4</f>
-        <v/>
-      </c>
-      <c r="H15" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I15" s="25" t="inlineStr">
-        <is>
-          <t>Cortina de enrollar exterior</t>
-        </is>
-      </c>
-      <c r="J15" s="26" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K15" s="25" t="inlineStr">
-        <is>
-          <t>Sudoeste</t>
-        </is>
-      </c>
-      <c r="L15" s="26">
-        <f>IF(I15="","",IFERROR(VLOOKUP(I15,Datos_higro!$A$21:$B$27,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M15" s="30">
-        <f>IF(OR(D15="",J15=""),"",IF(J15&lt;=G15,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
+      <c r="B15" s="4" t="n"/>
+      <c r="C15" s="4" t="n"/>
+      <c r="D15" s="4" t="n"/>
+      <c r="E15" s="4" t="n"/>
+      <c r="F15" s="4" t="n"/>
+      <c r="G15" s="4" t="n"/>
+      <c r="H15" s="4" t="n"/>
+      <c r="I15" s="4" t="n"/>
+      <c r="J15" s="4" t="n"/>
+      <c r="K15" s="4" t="n"/>
+      <c r="L15" s="4" t="n"/>
+      <c r="M15" s="4" t="n"/>
     </row>
     <row r="16" ht="17" customHeight="1">
       <c r="A16" s="25" t="inlineStr">
         <is>
-          <t>PF01 (2)</t>
+          <t>VA01</t>
         </is>
       </c>
       <c r="B16" s="26" t="n">
         <v>3</v>
       </c>
       <c r="C16" s="26" t="n">
-        <v>3.55</v>
+        <v>0.75</v>
       </c>
       <c r="D16" s="27">
         <f>IF(COUNT(B16,C16)&lt;2,"",B16*C16)</f>
         <v/>
       </c>
-      <c r="E16" s="31" t="n"/>
+      <c r="E16" s="28">
+        <f>SUM(D16:D19)</f>
+        <v/>
+      </c>
       <c r="F16" s="29">
-        <f>IF(OR(D16="",$E$15=""),"",D16/$E$15)</f>
+        <f>IF(OR(D16="",$E$16=""),"",D16/$E$16)</f>
         <v/>
       </c>
       <c r="G16" s="27">
@@ -8524,7 +8524,7 @@
       </c>
       <c r="I16" s="25" t="inlineStr">
         <is>
-          <t>Sin Proteccion</t>
+          <t>Cortina de enrollar exterior</t>
         </is>
       </c>
       <c r="J16" s="26" t="n">
@@ -8545,26 +8545,48 @@
       </c>
     </row>
     <row r="17" ht="17" customHeight="1">
-      <c r="A17" s="25" t="n"/>
-      <c r="B17" s="26" t="n"/>
-      <c r="C17" s="26" t="n"/>
+      <c r="A17" s="25" t="inlineStr">
+        <is>
+          <t>PF01 (2)</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" s="26" t="n">
+        <v>3.55</v>
+      </c>
       <c r="D17" s="27">
         <f>IF(COUNT(B17,C17)&lt;2,"",B17*C17)</f>
         <v/>
       </c>
       <c r="E17" s="31" t="n"/>
       <c r="F17" s="29">
-        <f>IF(OR(D17="",$E$15=""),"",D17/$E$15)</f>
+        <f>IF(OR(D17="",$E$16=""),"",D17/$E$16)</f>
         <v/>
       </c>
       <c r="G17" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H17" s="25" t="n"/>
-      <c r="I17" s="25" t="n"/>
-      <c r="J17" s="26" t="n"/>
-      <c r="K17" s="25" t="n"/>
+      <c r="H17" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I17" s="25" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J17" s="26" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K17" s="25" t="inlineStr">
+        <is>
+          <t>Sudoeste</t>
+        </is>
+      </c>
       <c r="L17" s="26">
         <f>IF(I17="","",IFERROR(VLOOKUP(I17,Datos_higro!$A$21:$B$27,2,0),""))</f>
         <v/>
@@ -8575,128 +8597,106 @@
       </c>
     </row>
     <row r="18" ht="17" customHeight="1">
-      <c r="A18" s="32" t="n"/>
-      <c r="B18" s="33" t="n"/>
-      <c r="C18" s="33" t="n"/>
-      <c r="D18" s="34">
+      <c r="A18" s="25" t="n"/>
+      <c r="B18" s="26" t="n"/>
+      <c r="C18" s="26" t="n"/>
+      <c r="D18" s="27">
         <f>IF(COUNT(B18,C18)&lt;2,"",B18*C18)</f>
         <v/>
       </c>
-      <c r="E18" s="35" t="n"/>
-      <c r="F18" s="36">
-        <f>IF(OR(D18="",$E$15=""),"",D18/$E$15)</f>
-        <v/>
-      </c>
-      <c r="G18" s="34">
+      <c r="E18" s="31" t="n"/>
+      <c r="F18" s="29">
+        <f>IF(OR(D18="",$E$16=""),"",D18/$E$16)</f>
+        <v/>
+      </c>
+      <c r="G18" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H18" s="32" t="n"/>
-      <c r="I18" s="32" t="n"/>
-      <c r="J18" s="33" t="n"/>
-      <c r="K18" s="32" t="n"/>
-      <c r="L18" s="33">
+      <c r="H18" s="25" t="n"/>
+      <c r="I18" s="25" t="n"/>
+      <c r="J18" s="26" t="n"/>
+      <c r="K18" s="25" t="n"/>
+      <c r="L18" s="26">
         <f>IF(I18="","",IFERROR(VLOOKUP(I18,Datos_higro!$A$21:$B$27,2,0),""))</f>
         <v/>
       </c>
-      <c r="M18" s="37">
+      <c r="M18" s="30">
         <f>IF(OR(D18="",J18=""),"",IF(J18&lt;=G18,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="24" t="inlineStr">
+    <row r="19" ht="17" customHeight="1">
+      <c r="A19" s="32" t="n"/>
+      <c r="B19" s="33" t="n"/>
+      <c r="C19" s="33" t="n"/>
+      <c r="D19" s="34">
+        <f>IF(COUNT(B19,C19)&lt;2,"",B19*C19)</f>
+        <v/>
+      </c>
+      <c r="E19" s="35" t="n"/>
+      <c r="F19" s="36">
+        <f>IF(OR(D19="",$E$16=""),"",D19/$E$16)</f>
+        <v/>
+      </c>
+      <c r="G19" s="34">
+        <f>Datos_higro!$B$4</f>
+        <v/>
+      </c>
+      <c r="H19" s="32" t="n"/>
+      <c r="I19" s="32" t="n"/>
+      <c r="J19" s="33" t="n"/>
+      <c r="K19" s="32" t="n"/>
+      <c r="L19" s="33">
+        <f>IF(I19="","",IFERROR(VLOOKUP(I19,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M19" s="37">
+        <f>IF(OR(D19="",J19=""),"",IF(J19&lt;=G19,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="24" t="inlineStr">
         <is>
           <t>Plano: Fachada Sudeste (borde inferior)</t>
         </is>
       </c>
-      <c r="B19" s="4" t="n"/>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="4" t="n"/>
-      <c r="E19" s="4" t="n"/>
-      <c r="F19" s="4" t="n"/>
-      <c r="G19" s="4" t="n"/>
-      <c r="H19" s="4" t="n"/>
-      <c r="I19" s="4" t="n"/>
-      <c r="J19" s="4" t="n"/>
-      <c r="K19" s="4" t="n"/>
-      <c r="L19" s="4" t="n"/>
-      <c r="M19" s="4" t="n"/>
-    </row>
-    <row r="20" ht="17" customHeight="1">
-      <c r="A20" s="25" t="inlineStr">
-        <is>
-          <t>PA01</t>
-        </is>
-      </c>
-      <c r="B20" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="C20" s="26" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="27">
-        <f>IF(COUNT(B20,C20)&lt;2,"",B20*C20)</f>
-        <v/>
-      </c>
-      <c r="E20" s="28">
-        <f>SUM(D20:D27)</f>
-        <v/>
-      </c>
-      <c r="F20" s="29">
-        <f>IF(OR(D20="",$E$20=""),"",D20/$E$20)</f>
-        <v/>
-      </c>
-      <c r="G20" s="27">
-        <f>Datos_higro!$B$4</f>
-        <v/>
-      </c>
-      <c r="H20" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I20" s="25" t="inlineStr">
-        <is>
-          <t>Cortina de enrollar exterior</t>
-        </is>
-      </c>
-      <c r="J20" s="26" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K20" s="25" t="inlineStr">
-        <is>
-          <t>Sudeste</t>
-        </is>
-      </c>
-      <c r="L20" s="26">
-        <f>IF(I20="","",IFERROR(VLOOKUP(I20,Datos_higro!$A$21:$B$27,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M20" s="30">
-        <f>IF(OR(D20="",J20=""),"",IF(J20&lt;=G20,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
+      <c r="B20" s="4" t="n"/>
+      <c r="C20" s="4" t="n"/>
+      <c r="D20" s="4" t="n"/>
+      <c r="E20" s="4" t="n"/>
+      <c r="F20" s="4" t="n"/>
+      <c r="G20" s="4" t="n"/>
+      <c r="H20" s="4" t="n"/>
+      <c r="I20" s="4" t="n"/>
+      <c r="J20" s="4" t="n"/>
+      <c r="K20" s="4" t="n"/>
+      <c r="L20" s="4" t="n"/>
+      <c r="M20" s="4" t="n"/>
     </row>
     <row r="21" ht="17" customHeight="1">
       <c r="A21" s="25" t="inlineStr">
         <is>
-          <t>PF04</t>
+          <t>PA01</t>
         </is>
       </c>
       <c r="B21" s="26" t="n">
-        <v>0.6</v>
+        <v>3</v>
       </c>
       <c r="C21" s="26" t="n">
-        <v>2.7</v>
+        <v>1</v>
       </c>
       <c r="D21" s="27">
         <f>IF(COUNT(B21,C21)&lt;2,"",B21*C21)</f>
         <v/>
       </c>
-      <c r="E21" s="31" t="n"/>
+      <c r="E21" s="28">
+        <f>SUM(D21:D29)</f>
+        <v/>
+      </c>
       <c r="F21" s="29">
-        <f>IF(OR(D21="",$E$20=""),"",D21/$E$20)</f>
+        <f>IF(OR(D21="",$E$21=""),"",D21/$E$21)</f>
         <v/>
       </c>
       <c r="G21" s="27">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="I21" s="25" t="inlineStr">
         <is>
-          <t>Sin Proteccion</t>
+          <t>Cortina de enrollar exterior</t>
         </is>
       </c>
       <c r="J21" s="26" t="n">
@@ -8733,14 +8733,14 @@
     <row r="22" ht="17" customHeight="1">
       <c r="A22" s="25" t="inlineStr">
         <is>
-          <t>VA05</t>
+          <t>PF04</t>
         </is>
       </c>
       <c r="B22" s="26" t="n">
-        <v>2.52</v>
+        <v>0.6</v>
       </c>
       <c r="C22" s="26" t="n">
-        <v>1.4</v>
+        <v>2.7</v>
       </c>
       <c r="D22" s="27">
         <f>IF(COUNT(B22,C22)&lt;2,"",B22*C22)</f>
@@ -8748,7 +8748,7 @@
       </c>
       <c r="E22" s="31" t="n"/>
       <c r="F22" s="29">
-        <f>IF(OR(D22="",$E$20=""),"",D22/$E$20)</f>
+        <f>IF(OR(D22="",$E$21=""),"",D22/$E$21)</f>
         <v/>
       </c>
       <c r="G22" s="27">
@@ -8762,7 +8762,7 @@
       </c>
       <c r="I22" s="25" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Sin Proteccion</t>
         </is>
       </c>
       <c r="J22" s="26" t="n">
@@ -8785,14 +8785,14 @@
     <row r="23" ht="17" customHeight="1">
       <c r="A23" s="25" t="inlineStr">
         <is>
-          <t>PV04</t>
+          <t>VA01 (2)</t>
         </is>
       </c>
       <c r="B23" s="26" t="n">
         <v>3</v>
       </c>
       <c r="C23" s="26" t="n">
-        <v>2.06</v>
+        <v>0.75</v>
       </c>
       <c r="D23" s="27">
         <f>IF(COUNT(B23,C23)&lt;2,"",B23*C23)</f>
@@ -8800,7 +8800,7 @@
       </c>
       <c r="E23" s="31" t="n"/>
       <c r="F23" s="29">
-        <f>IF(OR(D23="",$E$20=""),"",D23/$E$20)</f>
+        <f>IF(OR(D23="",$E$21=""),"",D23/$E$21)</f>
         <v/>
       </c>
       <c r="G23" s="27">
@@ -8837,14 +8837,14 @@
     <row r="24" ht="17" customHeight="1">
       <c r="A24" s="25" t="inlineStr">
         <is>
-          <t>PV04 (2)</t>
+          <t>VA05</t>
         </is>
       </c>
       <c r="B24" s="26" t="n">
-        <v>2.95</v>
+        <v>2.52</v>
       </c>
       <c r="C24" s="26" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="D24" s="27">
         <f>IF(COUNT(B24,C24)&lt;2,"",B24*C24)</f>
@@ -8852,7 +8852,7 @@
       </c>
       <c r="E24" s="31" t="n"/>
       <c r="F24" s="29">
-        <f>IF(OR(D24="",$E$20=""),"",D24/$E$20)</f>
+        <f>IF(OR(D24="",$E$21=""),"",D24/$E$21)</f>
         <v/>
       </c>
       <c r="G24" s="27">
@@ -8889,14 +8889,14 @@
     <row r="25" ht="17" customHeight="1">
       <c r="A25" s="25" t="inlineStr">
         <is>
-          <t>PF02</t>
+          <t>PV04</t>
         </is>
       </c>
       <c r="B25" s="26" t="n">
         <v>3</v>
       </c>
       <c r="C25" s="26" t="n">
-        <v>3.75</v>
+        <v>2.06</v>
       </c>
       <c r="D25" s="27">
         <f>IF(COUNT(B25,C25)&lt;2,"",B25*C25)</f>
@@ -8904,7 +8904,7 @@
       </c>
       <c r="E25" s="31" t="n"/>
       <c r="F25" s="29">
-        <f>IF(OR(D25="",$E$20=""),"",D25/$E$20)</f>
+        <f>IF(OR(D25="",$E$21=""),"",D25/$E$21)</f>
         <v/>
       </c>
       <c r="G25" s="27">
@@ -8918,7 +8918,7 @@
       </c>
       <c r="I25" s="25" t="inlineStr">
         <is>
-          <t>Sin Proteccion</t>
+          <t>Cortina de enrollar exterior</t>
         </is>
       </c>
       <c r="J25" s="26" t="n">
@@ -8939,26 +8939,48 @@
       </c>
     </row>
     <row r="26" ht="17" customHeight="1">
-      <c r="A26" s="25" t="n"/>
-      <c r="B26" s="26" t="n"/>
-      <c r="C26" s="26" t="n"/>
+      <c r="A26" s="25" t="inlineStr">
+        <is>
+          <t>PV04 (2)</t>
+        </is>
+      </c>
+      <c r="B26" s="26" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="C26" s="26" t="n">
+        <v>1.5</v>
+      </c>
       <c r="D26" s="27">
         <f>IF(COUNT(B26,C26)&lt;2,"",B26*C26)</f>
         <v/>
       </c>
       <c r="E26" s="31" t="n"/>
       <c r="F26" s="29">
-        <f>IF(OR(D26="",$E$20=""),"",D26/$E$20)</f>
+        <f>IF(OR(D26="",$E$21=""),"",D26/$E$21)</f>
         <v/>
       </c>
       <c r="G26" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H26" s="25" t="n"/>
-      <c r="I26" s="25" t="n"/>
-      <c r="J26" s="26" t="n"/>
-      <c r="K26" s="25" t="n"/>
+      <c r="H26" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I26" s="25" t="inlineStr">
+        <is>
+          <t>Cortina de enrollar exterior</t>
+        </is>
+      </c>
+      <c r="J26" s="26" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K26" s="25" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
       <c r="L26" s="26">
         <f>IF(I26="","",IFERROR(VLOOKUP(I26,Datos_higro!$A$21:$B$27,2,0),""))</f>
         <v/>
@@ -8969,180 +8991,158 @@
       </c>
     </row>
     <row r="27" ht="17" customHeight="1">
-      <c r="A27" s="32" t="n"/>
-      <c r="B27" s="33" t="n"/>
-      <c r="C27" s="33" t="n"/>
-      <c r="D27" s="34">
+      <c r="A27" s="25" t="inlineStr">
+        <is>
+          <t>PF02</t>
+        </is>
+      </c>
+      <c r="B27" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C27" s="26" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D27" s="27">
         <f>IF(COUNT(B27,C27)&lt;2,"",B27*C27)</f>
         <v/>
       </c>
-      <c r="E27" s="35" t="n"/>
-      <c r="F27" s="36">
-        <f>IF(OR(D27="",$E$20=""),"",D27/$E$20)</f>
-        <v/>
-      </c>
-      <c r="G27" s="34">
+      <c r="E27" s="31" t="n"/>
+      <c r="F27" s="29">
+        <f>IF(OR(D27="",$E$21=""),"",D27/$E$21)</f>
+        <v/>
+      </c>
+      <c r="G27" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H27" s="32" t="n"/>
-      <c r="I27" s="32" t="n"/>
-      <c r="J27" s="33" t="n"/>
-      <c r="K27" s="32" t="n"/>
-      <c r="L27" s="33">
+      <c r="H27" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I27" s="25" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J27" s="26" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K27" s="25" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="L27" s="26">
         <f>IF(I27="","",IFERROR(VLOOKUP(I27,Datos_higro!$A$21:$B$27,2,0),""))</f>
         <v/>
       </c>
-      <c r="M27" s="37">
+      <c r="M27" s="30">
         <f>IF(OR(D27="",J27=""),"",IF(J27&lt;=G27,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="24" t="inlineStr">
+    <row r="28" ht="17" customHeight="1">
+      <c r="A28" s="25" t="n"/>
+      <c r="B28" s="26" t="n"/>
+      <c r="C28" s="26" t="n"/>
+      <c r="D28" s="27">
+        <f>IF(COUNT(B28,C28)&lt;2,"",B28*C28)</f>
+        <v/>
+      </c>
+      <c r="E28" s="31" t="n"/>
+      <c r="F28" s="29">
+        <f>IF(OR(D28="",$E$21=""),"",D28/$E$21)</f>
+        <v/>
+      </c>
+      <c r="G28" s="27">
+        <f>Datos_higro!$B$4</f>
+        <v/>
+      </c>
+      <c r="H28" s="25" t="n"/>
+      <c r="I28" s="25" t="n"/>
+      <c r="J28" s="26" t="n"/>
+      <c r="K28" s="25" t="n"/>
+      <c r="L28" s="26">
+        <f>IF(I28="","",IFERROR(VLOOKUP(I28,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M28" s="30">
+        <f>IF(OR(D28="",J28=""),"",IF(J28&lt;=G28,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="17" customHeight="1">
+      <c r="A29" s="32" t="n"/>
+      <c r="B29" s="33" t="n"/>
+      <c r="C29" s="33" t="n"/>
+      <c r="D29" s="34">
+        <f>IF(COUNT(B29,C29)&lt;2,"",B29*C29)</f>
+        <v/>
+      </c>
+      <c r="E29" s="35" t="n"/>
+      <c r="F29" s="36">
+        <f>IF(OR(D29="",$E$21=""),"",D29/$E$21)</f>
+        <v/>
+      </c>
+      <c r="G29" s="34">
+        <f>Datos_higro!$B$4</f>
+        <v/>
+      </c>
+      <c r="H29" s="32" t="n"/>
+      <c r="I29" s="32" t="n"/>
+      <c r="J29" s="33" t="n"/>
+      <c r="K29" s="32" t="n"/>
+      <c r="L29" s="33">
+        <f>IF(I29="","",IFERROR(VLOOKUP(I29,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M29" s="37">
+        <f>IF(OR(D29="",J29=""),"",IF(J29&lt;=G29,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="24" t="inlineStr">
         <is>
           <t>Plano: Fachada Noroeste (borde superior)</t>
         </is>
       </c>
-      <c r="B28" s="4" t="n"/>
-      <c r="C28" s="4" t="n"/>
-      <c r="D28" s="4" t="n"/>
-      <c r="E28" s="4" t="n"/>
-      <c r="F28" s="4" t="n"/>
-      <c r="G28" s="4" t="n"/>
-      <c r="H28" s="4" t="n"/>
-      <c r="I28" s="4" t="n"/>
-      <c r="J28" s="4" t="n"/>
-      <c r="K28" s="4" t="n"/>
-      <c r="L28" s="4" t="n"/>
-      <c r="M28" s="4" t="n"/>
-    </row>
-    <row r="29" ht="17" customHeight="1">
-      <c r="A29" s="25" t="inlineStr">
-        <is>
-          <t>PV03</t>
-        </is>
-      </c>
-      <c r="B29" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="C29" s="26" t="n">
-        <v>1.76</v>
-      </c>
-      <c r="D29" s="27">
-        <f>IF(COUNT(B29,C29)&lt;2,"",B29*C29)</f>
-        <v/>
-      </c>
-      <c r="E29" s="28">
-        <f>SUM(D29:D35)</f>
-        <v/>
-      </c>
-      <c r="F29" s="29">
-        <f>IF(OR(D29="",$E$29=""),"",D29/$E$29)</f>
-        <v/>
-      </c>
-      <c r="G29" s="27">
-        <f>Datos_higro!$B$4</f>
-        <v/>
-      </c>
-      <c r="H29" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I29" s="25" t="inlineStr">
-        <is>
-          <t>Cortina de enrollar exterior</t>
-        </is>
-      </c>
-      <c r="J29" s="26" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K29" s="25" t="inlineStr">
-        <is>
-          <t>Noroeste</t>
-        </is>
-      </c>
-      <c r="L29" s="26">
-        <f>IF(I29="","",IFERROR(VLOOKUP(I29,Datos_higro!$A$21:$B$27,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M29" s="30">
-        <f>IF(OR(D29="",J29=""),"",IF(J29&lt;=G29,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="17" customHeight="1">
-      <c r="A30" s="25" t="inlineStr">
-        <is>
-          <t>VA02</t>
-        </is>
-      </c>
-      <c r="B30" s="26" t="n">
-        <v>2.15</v>
-      </c>
-      <c r="C30" s="26" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D30" s="27">
-        <f>IF(COUNT(B30,C30)&lt;2,"",B30*C30)</f>
-        <v/>
-      </c>
-      <c r="E30" s="31" t="n"/>
-      <c r="F30" s="29">
-        <f>IF(OR(D30="",$E$29=""),"",D30/$E$29)</f>
-        <v/>
-      </c>
-      <c r="G30" s="27">
-        <f>Datos_higro!$B$4</f>
-        <v/>
-      </c>
-      <c r="H30" s="25" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I30" s="25" t="inlineStr">
-        <is>
-          <t>Cortina de enrollar exterior</t>
-        </is>
-      </c>
-      <c r="J30" s="26" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K30" s="25" t="inlineStr">
-        <is>
-          <t>Noroeste</t>
-        </is>
-      </c>
-      <c r="L30" s="26">
-        <f>IF(I30="","",IFERROR(VLOOKUP(I30,Datos_higro!$A$21:$B$27,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M30" s="30">
-        <f>IF(OR(D30="",J30=""),"",IF(J30&lt;=G30,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
+      <c r="B30" s="4" t="n"/>
+      <c r="C30" s="4" t="n"/>
+      <c r="D30" s="4" t="n"/>
+      <c r="E30" s="4" t="n"/>
+      <c r="F30" s="4" t="n"/>
+      <c r="G30" s="4" t="n"/>
+      <c r="H30" s="4" t="n"/>
+      <c r="I30" s="4" t="n"/>
+      <c r="J30" s="4" t="n"/>
+      <c r="K30" s="4" t="n"/>
+      <c r="L30" s="4" t="n"/>
+      <c r="M30" s="4" t="n"/>
     </row>
     <row r="31" ht="17" customHeight="1">
       <c r="A31" s="25" t="inlineStr">
         <is>
-          <t>PA02</t>
+          <t>PV03</t>
         </is>
       </c>
       <c r="B31" s="26" t="n">
         <v>3</v>
       </c>
       <c r="C31" s="26" t="n">
-        <v>0.75</v>
+        <v>1.76</v>
       </c>
       <c r="D31" s="27">
         <f>IF(COUNT(B31,C31)&lt;2,"",B31*C31)</f>
         <v/>
       </c>
-      <c r="E31" s="31" t="n"/>
+      <c r="E31" s="28">
+        <f>SUM(D31:D37)</f>
+        <v/>
+      </c>
       <c r="F31" s="29">
-        <f>IF(OR(D31="",$E$29=""),"",D31/$E$29)</f>
+        <f>IF(OR(D31="",$E$31=""),"",D31/$E$31)</f>
         <v/>
       </c>
       <c r="G31" s="27">
@@ -9179,11 +9179,11 @@
     <row r="32" ht="17" customHeight="1">
       <c r="A32" s="25" t="inlineStr">
         <is>
-          <t>VA03</t>
+          <t>VA02</t>
         </is>
       </c>
       <c r="B32" s="26" t="n">
-        <v>2.52</v>
+        <v>2.15</v>
       </c>
       <c r="C32" s="26" t="n">
         <v>0.75</v>
@@ -9194,7 +9194,7 @@
       </c>
       <c r="E32" s="31" t="n"/>
       <c r="F32" s="29">
-        <f>IF(OR(D32="",$E$29=""),"",D32/$E$29)</f>
+        <f>IF(OR(D32="",$E$31=""),"",D32/$E$31)</f>
         <v/>
       </c>
       <c r="G32" s="27">
@@ -9231,11 +9231,11 @@
     <row r="33" ht="17" customHeight="1">
       <c r="A33" s="25" t="inlineStr">
         <is>
-          <t>PF05</t>
+          <t>PA02</t>
         </is>
       </c>
       <c r="B33" s="26" t="n">
-        <v>2.52</v>
+        <v>3</v>
       </c>
       <c r="C33" s="26" t="n">
         <v>0.75</v>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="E33" s="31" t="n"/>
       <c r="F33" s="29">
-        <f>IF(OR(D33="",$E$29=""),"",D33/$E$29)</f>
+        <f>IF(OR(D33="",$E$31=""),"",D33/$E$31)</f>
         <v/>
       </c>
       <c r="G33" s="27">
@@ -9260,7 +9260,7 @@
       </c>
       <c r="I33" s="25" t="inlineStr">
         <is>
-          <t>Sin Proteccion</t>
+          <t>Cortina de enrollar exterior</t>
         </is>
       </c>
       <c r="J33" s="26" t="n">
@@ -9281,26 +9281,48 @@
       </c>
     </row>
     <row r="34" ht="17" customHeight="1">
-      <c r="A34" s="25" t="n"/>
-      <c r="B34" s="26" t="n"/>
-      <c r="C34" s="26" t="n"/>
+      <c r="A34" s="25" t="inlineStr">
+        <is>
+          <t>VA03</t>
+        </is>
+      </c>
+      <c r="B34" s="26" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="C34" s="26" t="n">
+        <v>0.75</v>
+      </c>
       <c r="D34" s="27">
         <f>IF(COUNT(B34,C34)&lt;2,"",B34*C34)</f>
         <v/>
       </c>
       <c r="E34" s="31" t="n"/>
       <c r="F34" s="29">
-        <f>IF(OR(D34="",$E$29=""),"",D34/$E$29)</f>
+        <f>IF(OR(D34="",$E$31=""),"",D34/$E$31)</f>
         <v/>
       </c>
       <c r="G34" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H34" s="25" t="n"/>
-      <c r="I34" s="25" t="n"/>
-      <c r="J34" s="26" t="n"/>
-      <c r="K34" s="25" t="n"/>
+      <c r="H34" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I34" s="25" t="inlineStr">
+        <is>
+          <t>Cortina de enrollar exterior</t>
+        </is>
+      </c>
+      <c r="J34" s="26" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K34" s="25" t="inlineStr">
+        <is>
+          <t>Noroeste</t>
+        </is>
+      </c>
       <c r="L34" s="26">
         <f>IF(I34="","",IFERROR(VLOOKUP(I34,Datos_higro!$A$21:$B$27,2,0),""))</f>
         <v/>
@@ -9311,75 +9333,119 @@
       </c>
     </row>
     <row r="35" ht="17" customHeight="1">
-      <c r="A35" s="32" t="n"/>
-      <c r="B35" s="33" t="n"/>
-      <c r="C35" s="33" t="n"/>
-      <c r="D35" s="34">
+      <c r="A35" s="25" t="inlineStr">
+        <is>
+          <t>PF05</t>
+        </is>
+      </c>
+      <c r="B35" s="26" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="C35" s="26" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D35" s="27">
         <f>IF(COUNT(B35,C35)&lt;2,"",B35*C35)</f>
         <v/>
       </c>
-      <c r="E35" s="35" t="n"/>
-      <c r="F35" s="36">
-        <f>IF(OR(D35="",$E$29=""),"",D35/$E$29)</f>
-        <v/>
-      </c>
-      <c r="G35" s="34">
+      <c r="E35" s="31" t="n"/>
+      <c r="F35" s="29">
+        <f>IF(OR(D35="",$E$31=""),"",D35/$E$31)</f>
+        <v/>
+      </c>
+      <c r="G35" s="27">
         <f>Datos_higro!$B$4</f>
         <v/>
       </c>
-      <c r="H35" s="32" t="n"/>
-      <c r="I35" s="32" t="n"/>
-      <c r="J35" s="33" t="n"/>
-      <c r="K35" s="32" t="n"/>
-      <c r="L35" s="33">
+      <c r="H35" s="25" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I35" s="25" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J35" s="26" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K35" s="25" t="inlineStr">
+        <is>
+          <t>Noroeste</t>
+        </is>
+      </c>
+      <c r="L35" s="26">
         <f>IF(I35="","",IFERROR(VLOOKUP(I35,Datos_higro!$A$21:$B$27,2,0),""))</f>
         <v/>
       </c>
-      <c r="M35" s="37">
+      <c r="M35" s="30">
         <f>IF(OR(D35="",J35=""),"",IF(J35&lt;=G35,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="2" t="n"/>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="2" t="n"/>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="n"/>
-      <c r="G36" s="2" t="n"/>
-      <c r="H36" s="2" t="n"/>
-      <c r="I36" s="2" t="n"/>
-      <c r="J36" s="2" t="n"/>
-      <c r="K36" s="2" t="n"/>
-      <c r="L36" s="2" t="n"/>
-      <c r="M36" s="2" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="38" t="inlineStr">
-        <is>
-          <t>COMO SE COMPLETA</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="n"/>
-      <c r="C37" s="2" t="n"/>
-      <c r="D37" s="2" t="n"/>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="n"/>
-      <c r="G37" s="2" t="n"/>
-      <c r="H37" s="2" t="n"/>
-      <c r="I37" s="2" t="n"/>
-      <c r="J37" s="2" t="n"/>
-      <c r="K37" s="2" t="n"/>
-      <c r="L37" s="2" t="n"/>
-      <c r="M37" s="2" t="n"/>
+    <row r="36" ht="17" customHeight="1">
+      <c r="A36" s="25" t="n"/>
+      <c r="B36" s="26" t="n"/>
+      <c r="C36" s="26" t="n"/>
+      <c r="D36" s="27">
+        <f>IF(COUNT(B36,C36)&lt;2,"",B36*C36)</f>
+        <v/>
+      </c>
+      <c r="E36" s="31" t="n"/>
+      <c r="F36" s="29">
+        <f>IF(OR(D36="",$E$31=""),"",D36/$E$31)</f>
+        <v/>
+      </c>
+      <c r="G36" s="27">
+        <f>Datos_higro!$B$4</f>
+        <v/>
+      </c>
+      <c r="H36" s="25" t="n"/>
+      <c r="I36" s="25" t="n"/>
+      <c r="J36" s="26" t="n"/>
+      <c r="K36" s="25" t="n"/>
+      <c r="L36" s="26">
+        <f>IF(I36="","",IFERROR(VLOOKUP(I36,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M36" s="30">
+        <f>IF(OR(D36="",J36=""),"",IF(J36&lt;=G36,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="17" customHeight="1">
+      <c r="A37" s="32" t="n"/>
+      <c r="B37" s="33" t="n"/>
+      <c r="C37" s="33" t="n"/>
+      <c r="D37" s="34">
+        <f>IF(COUNT(B37,C37)&lt;2,"",B37*C37)</f>
+        <v/>
+      </c>
+      <c r="E37" s="35" t="n"/>
+      <c r="F37" s="36">
+        <f>IF(OR(D37="",$E$31=""),"",D37/$E$31)</f>
+        <v/>
+      </c>
+      <c r="G37" s="34">
+        <f>Datos_higro!$B$4</f>
+        <v/>
+      </c>
+      <c r="H37" s="32" t="n"/>
+      <c r="I37" s="32" t="n"/>
+      <c r="J37" s="33" t="n"/>
+      <c r="K37" s="32" t="n"/>
+      <c r="L37" s="33">
+        <f>IF(I37="","",IFERROR(VLOOKUP(I37,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M37" s="37">
+        <f>IF(OR(D37="",J37=""),"",IF(J37&lt;=G37,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="39" t="inlineStr">
-        <is>
-          <t>Descripcion, altura y ancho del vano: de la planilla de carpinterias.</t>
-        </is>
-      </c>
+      <c r="A38" s="2" t="n"/>
       <c r="B38" s="2" t="n"/>
       <c r="C38" s="2" t="n"/>
       <c r="D38" s="2" t="n"/>
@@ -9394,9 +9460,9 @@
       <c r="M38" s="2" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="39" t="inlineStr">
-        <is>
-          <t>Area del vano, area total por plano y porcentaje: se calculan solos.</t>
+      <c r="A39" s="38" t="inlineStr">
+        <is>
+          <t>COMO SE COMPLETA</t>
         </is>
       </c>
       <c r="B39" s="2" t="n"/>
@@ -9415,7 +9481,7 @@
     <row r="40">
       <c r="A40" s="39" t="inlineStr">
         <is>
-          <t>Tipo de vidrio y tipo de proteccion: desplegables; sus valores estan en la hoja Datos_higro.</t>
+          <t>Descripcion, altura y ancho del vano: de la planilla de carpinterias.</t>
         </is>
       </c>
       <c r="B40" s="2" t="n"/>
@@ -9434,7 +9500,7 @@
     <row r="41">
       <c r="A41" s="39" t="inlineStr">
         <is>
-          <t>Transmitancia del cerramiento: cargarla segun el vidrio y el marco adoptados.</t>
+          <t>Area del vano, area total por plano y porcentaje: se calculan solos.</t>
         </is>
       </c>
       <c r="B41" s="2" t="n"/>
@@ -9453,7 +9519,7 @@
     <row r="42">
       <c r="A42" s="39" t="inlineStr">
         <is>
-          <t>PROTECCION: ningun pano fijo PF tiene cortina: PF01, su gemelo, PF02, PF03, PF04 y PF05 van</t>
+          <t>Tipo de vidrio y tipo de proteccion: desplegables; sus valores estan en la hoja Datos_higro.</t>
         </is>
       </c>
       <c r="B42" s="2" t="n"/>
@@ -9472,7 +9538,7 @@
     <row r="43">
       <c r="A43" s="39" t="inlineStr">
         <is>
-          <t>Sin Proteccion (FES 0,88). Las otras doce llevan cortina de enrollar exterior (FES 0,25).</t>
+          <t>Transmitancia del cerramiento: cargarla segun el vidrio y el marco adoptados.</t>
         </is>
       </c>
       <c r="B43" s="2" t="n"/>
@@ -9489,7 +9555,11 @@
       <c r="M43" s="2" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="39" t="inlineStr"/>
+      <c r="A44" s="39" t="inlineStr">
+        <is>
+          <t>PROTECCION: ningun pano fijo PF tiene cortina: PF01, su gemelo, PF02, PF03, PF04 y PF05 van</t>
+        </is>
+      </c>
       <c r="B44" s="2" t="n"/>
       <c r="C44" s="2" t="n"/>
       <c r="D44" s="2" t="n"/>
@@ -9506,7 +9576,7 @@
     <row r="45">
       <c r="A45" s="39" t="inlineStr">
         <is>
-          <t>OJO con esas seis: 0,88 esta muy por encima del maximo de 0,30 que la ordenanza admite para</t>
+          <t>Sin Proteccion (FES 0,88). Las otras doce llevan cortina de enrollar exterior (FES 0,25).</t>
         </is>
       </c>
       <c r="B45" s="2" t="n"/>
@@ -9523,11 +9593,7 @@
       <c r="M45" s="2" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="39" t="inlineStr">
-        <is>
-          <t>el cuadrante Este/Oeste, donde caen las cuatro fachadas de esta casa por estar girada 45</t>
-        </is>
-      </c>
+      <c r="A46" s="39" t="inlineStr"/>
       <c r="B46" s="2" t="n"/>
       <c r="C46" s="2" t="n"/>
       <c r="D46" s="2" t="n"/>
@@ -9544,7 +9610,7 @@
     <row r="47">
       <c r="A47" s="39" t="inlineStr">
         <is>
-          <t>grados. La verificacion de la planilla no lo controla, igual que la de la catedra, pero si lo</t>
+          <t>OJO con esas seis: 0,88 esta muy por encima del maximo de 0,30 que la ordenanza admite para</t>
         </is>
       </c>
       <c r="B47" s="2" t="n"/>
@@ -9563,7 +9629,7 @@
     <row r="48">
       <c r="A48" s="39" t="inlineStr">
         <is>
-          <t>presentas en el municipio esas cinco aberturas no pasarian el factor de exposicion solar.</t>
+          <t>el cuadrante Este/Oeste, donde caen las cuatro fachadas de esta casa por estar girada 45</t>
         </is>
       </c>
       <c r="B48" s="2" t="n"/>
@@ -9582,7 +9648,7 @@
     <row r="49">
       <c r="A49" s="39" t="inlineStr">
         <is>
-          <t>Hay una salida: si la abertura ocupa menos del 20% del lado expuesto del local, no se verifica</t>
+          <t>grados. La verificacion de la planilla no lo controla, igual que la de la catedra, pero si lo</t>
         </is>
       </c>
       <c r="B49" s="2" t="n"/>
@@ -9601,7 +9667,7 @@
     <row r="50">
       <c r="A50" s="39" t="inlineStr">
         <is>
-          <t>el FES. Conviene chequearlo local por local.</t>
+          <t>presentas en el municipio esas cinco aberturas no pasarian el factor de exposicion solar.</t>
         </is>
       </c>
       <c r="B50" s="2" t="n"/>
@@ -9618,7 +9684,11 @@
       <c r="M50" s="2" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="39" t="inlineStr"/>
+      <c r="A51" s="39" t="inlineStr">
+        <is>
+          <t>Hay una salida: si la abertura ocupa menos del 20% del lado expuesto del local, no se verifica</t>
+        </is>
+      </c>
       <c r="B51" s="2" t="n"/>
       <c r="C51" s="2" t="n"/>
       <c r="D51" s="2" t="n"/>
@@ -9635,7 +9705,7 @@
     <row r="52">
       <c r="A52" s="39" t="inlineStr">
         <is>
-          <t>Orientacion: ya cargada. Factor de exposicion solar: se completa SOLO al elegir el tipo de</t>
+          <t>el FES. Conviene chequearlo local por local.</t>
         </is>
       </c>
       <c r="B52" s="2" t="n"/>
@@ -9652,11 +9722,7 @@
       <c r="M52" s="2" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="39" t="inlineStr">
-        <is>
-          <t>proteccion, con los valores de la tabla de Datos_higro (Sin Proteccion 0,88; Parasol</t>
-        </is>
-      </c>
+      <c r="A53" s="39" t="inlineStr"/>
       <c r="B53" s="2" t="n"/>
       <c r="C53" s="2" t="n"/>
       <c r="D53" s="2" t="n"/>
@@ -9673,7 +9739,7 @@
     <row r="54">
       <c r="A54" s="39" t="inlineStr">
         <is>
-          <t>horizontal fijo 1:2 0,35), que son los mismos de la planilla de la catedra.</t>
+          <t>Orientacion: ya cargada. Factor de exposicion solar: se completa SOLO al elegir el tipo de</t>
         </is>
       </c>
       <c r="B54" s="2" t="n"/>
@@ -9692,7 +9758,7 @@
     <row r="55">
       <c r="A55" s="39" t="inlineStr">
         <is>
-          <t>En Datos_higro esta ademas el FES maximo admitido por cuadrante segun la ordenanza, como</t>
+          <t>proteccion, con los valores de la tabla de Datos_higro (Sin Proteccion 0,88; Parasol</t>
         </is>
       </c>
       <c r="B55" s="2" t="n"/>
@@ -9711,7 +9777,7 @@
     <row r="56">
       <c r="A56" s="39" t="inlineStr">
         <is>
-          <t>referencia: la verificacion no lo controla, igual que en la planilla de la catedra.</t>
+          <t>horizontal fijo 1:2 0,35), que son los mismos de la planilla de la catedra.</t>
         </is>
       </c>
       <c r="B56" s="2" t="n"/>
@@ -9728,7 +9794,11 @@
       <c r="M56" s="2" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="39" t="inlineStr"/>
+      <c r="A57" s="39" t="inlineStr">
+        <is>
+          <t>En Datos_higro esta ademas el FES maximo admitido por cuadrante segun la ordenanza, como</t>
+        </is>
+      </c>
       <c r="B57" s="2" t="n"/>
       <c r="C57" s="2" t="n"/>
       <c r="D57" s="2" t="n"/>
@@ -9745,7 +9815,7 @@
     <row r="58">
       <c r="A58" s="39" t="inlineStr">
         <is>
-          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
+          <t>referencia: la verificacion no lo controla, igual que en la planilla de la catedra.</t>
         </is>
       </c>
       <c r="B58" s="2" t="n"/>
@@ -9762,11 +9832,7 @@
       <c r="M58" s="2" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="39" t="inlineStr">
-        <is>
-          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
-        </is>
-      </c>
+      <c r="A59" s="39" t="inlineStr"/>
       <c r="B59" s="2" t="n"/>
       <c r="C59" s="2" t="n"/>
       <c r="D59" s="2" t="n"/>
@@ -9781,7 +9847,11 @@
       <c r="M59" s="2" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="39" t="inlineStr"/>
+      <c r="A60" s="39" t="inlineStr">
+        <is>
+          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
+        </is>
+      </c>
       <c r="B60" s="2" t="n"/>
       <c r="C60" s="2" t="n"/>
       <c r="D60" s="2" t="n"/>
@@ -9798,7 +9868,7 @@
     <row r="61">
       <c r="A61" s="39" t="inlineStr">
         <is>
-          <t>ALTURAS: medidas sobre el dibujo de las vistas de la planilla de carpinterias, con la escala</t>
+          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
         </is>
       </c>
       <c r="B61" s="2" t="n"/>
@@ -9815,11 +9885,7 @@
       <c r="M61" s="2" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="39" t="inlineStr">
-        <is>
-          <t>verificada contra los anchos acotados (error menor a 2 cm). La mayoria de las aberturas son de</t>
-        </is>
-      </c>
+      <c r="A62" s="39" t="inlineStr"/>
       <c r="B62" s="2" t="n"/>
       <c r="C62" s="2" t="n"/>
       <c r="D62" s="2" t="n"/>
@@ -9836,7 +9902,7 @@
     <row r="63">
       <c r="A63" s="39" t="inlineStr">
         <is>
-          <t>piso a cielorraso, 3,00 m. VERIFICARLAS contra el plano antes de presentar.</t>
+          <t>ALTURAS: medidas sobre el dibujo de las vistas de la planilla de carpinterias, con la escala</t>
         </is>
       </c>
       <c r="B63" s="2" t="n"/>
@@ -9855,7 +9921,7 @@
     <row r="64">
       <c r="A64" s="39" t="inlineStr">
         <is>
-          <t>PF04 es la unica con antepecho: arranca a 1,09 y mide 0,60 de alto. El resto llega al piso.</t>
+          <t>verificada contra los anchos acotados (error menor a 2 cm). La mayoria de las aberturas son de</t>
         </is>
       </c>
       <c r="B64" s="2" t="n"/>
@@ -9874,7 +9940,7 @@
     <row r="65">
       <c r="A65" s="39" t="inlineStr">
         <is>
-          <t>Las alturas de PV01 (3,00), PF04 (0,60) y PV04 (2) (2,95) las aporto el autor del proyecto.</t>
+          <t>piso a cielorraso, 3,00 m. VERIFICARLAS contra el plano antes de presentar.</t>
         </is>
       </c>
       <c r="B65" s="2" t="n"/>
@@ -9891,7 +9957,11 @@
       <c r="M65" s="2" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="39" t="inlineStr"/>
+      <c r="A66" s="39" t="inlineStr">
+        <is>
+          <t>PF04 es la unica con antepecho: arranca a 1,09 y mide 0,60 de alto. El resto llega al piso.</t>
+        </is>
+      </c>
       <c r="B66" s="2" t="n"/>
       <c r="C66" s="2" t="n"/>
       <c r="D66" s="2" t="n"/>
@@ -9908,7 +9978,7 @@
     <row r="67">
       <c r="A67" s="39" t="inlineStr">
         <is>
-          <t>ORIENTACION: el simbolo de norte del plano (circulo con aguja, en el patio interno) apunta a</t>
+          <t>Las alturas de PV01 (3,00), PF04 (0,60) y PV04 (2) (2,95) las aporto el autor del proyecto.</t>
         </is>
       </c>
       <c r="B67" s="2" t="n"/>
@@ -9925,11 +9995,7 @@
       <c r="M67" s="2" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="39" t="inlineStr">
-        <is>
-          <t>45 grados hacia arriba y a la derecha de la hoja. Entonces las cuatro fachadas NO son N-S-E-O</t>
-        </is>
-      </c>
+      <c r="A68" s="39" t="inlineStr"/>
       <c r="B68" s="2" t="n"/>
       <c r="C68" s="2" t="n"/>
       <c r="D68" s="2" t="n"/>
@@ -9946,7 +10012,7 @@
     <row r="69">
       <c r="A69" s="39" t="inlineStr">
         <is>
-          <t>sino: arriba = Noroeste, derecha = Noreste, abajo = Sudeste, izquierda = Sudoeste.</t>
+          <t>ORIENTACION: el simbolo de norte del plano (circulo con aguja, en el patio interno) apunta a</t>
         </is>
       </c>
       <c r="B69" s="2" t="n"/>
@@ -9965,7 +10031,7 @@
     <row r="70">
       <c r="A70" s="39" t="inlineStr">
         <is>
-          <t>Cada abertura se asigno a la fachada por su posicion en planta. Las del patio interno se</t>
+          <t>45 grados hacia arriba y a la derecha de la hoja. Entonces las cuatro fachadas NO son N-S-E-O</t>
         </is>
       </c>
       <c r="B70" s="2" t="n"/>
@@ -9984,7 +10050,7 @@
     <row r="71">
       <c r="A71" s="39" t="inlineStr">
         <is>
-          <t>orientan por la pared en la que estan: miran hacia adentro del patio.</t>
+          <t>sino: arriba = Noroeste, derecha = Noreste, abajo = Sudeste, izquierda = Sudoeste.</t>
         </is>
       </c>
       <c r="B71" s="2" t="n"/>
@@ -10003,7 +10069,7 @@
     <row r="72">
       <c r="A72" s="39" t="inlineStr">
         <is>
-          <t>Los rotulos Dormitorio Norte y Dormitorio Sur del plano no coinciden con el norte real;</t>
+          <t>Cada abertura se asigno a la fachada por su posicion en planta. Las del patio interno se</t>
         </is>
       </c>
       <c r="B72" s="2" t="n"/>
@@ -10022,7 +10088,7 @@
     <row r="73">
       <c r="A73" s="39" t="inlineStr">
         <is>
-          <t>parecen ser nombres de uso, no orientaciones.</t>
+          <t>orientan por la pared en la que estan: miran hacia adentro del patio.</t>
         </is>
       </c>
       <c r="B73" s="2" t="n"/>
@@ -10039,7 +10105,11 @@
       <c r="M73" s="2" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="39" t="inlineStr"/>
+      <c r="A74" s="39" t="inlineStr">
+        <is>
+          <t>Los rotulos Dormitorio Norte y Dormitorio Sur del plano no coinciden con el norte real;</t>
+        </is>
+      </c>
       <c r="B74" s="2" t="n"/>
       <c r="C74" s="2" t="n"/>
       <c r="D74" s="2" t="n"/>
@@ -10056,7 +10126,7 @@
     <row r="75">
       <c r="A75" s="39" t="inlineStr">
         <is>
-          <t>PF01 figura dos veces en el plano, en las dos paredes laterales del patio interno, y por eso</t>
+          <t>parecen ser nombres de uso, no orientaciones.</t>
         </is>
       </c>
       <c r="B75" s="2" t="n"/>
@@ -10073,11 +10143,7 @@
       <c r="M75" s="2" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="39" t="inlineStr">
-        <is>
-          <t>se cargan dos filas. Si fuera una sola abertura rotulada dos veces, borrar la segunda.</t>
-        </is>
-      </c>
+      <c r="A76" s="39" t="inlineStr"/>
       <c r="B76" s="2" t="n"/>
       <c r="C76" s="2" t="n"/>
       <c r="D76" s="2" t="n"/>
@@ -10092,7 +10158,11 @@
       <c r="M76" s="2" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="39" t="inlineStr"/>
+      <c r="A77" s="39" t="inlineStr">
+        <is>
+          <t>CANTIDADES: la planilla de carpinterias trae la cantidad de cada abertura. Tres van dos veces:</t>
+        </is>
+      </c>
       <c r="B77" s="2" t="n"/>
       <c r="C77" s="2" t="n"/>
       <c r="D77" s="2" t="n"/>
@@ -10109,7 +10179,7 @@
     <row r="78">
       <c r="A78" s="39" t="inlineStr">
         <is>
-          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
+          <t>VA01 (01 Cocina y 09 Suite), VA04 (13 Dormitorio Norte y 14 Play Room) y PF01 (03 Lavadero y</t>
         </is>
       </c>
       <c r="B78" s="2" t="n"/>
@@ -10126,7 +10196,11 @@
       <c r="M78" s="2" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="39" t="inlineStr"/>
+      <c r="A79" s="39" t="inlineStr">
+        <is>
+          <t>07 Hall de ingreso, a los dos lados del patio interno). Por eso la planilla tiene 20 filas y</t>
+        </is>
+      </c>
       <c r="B79" s="2" t="n"/>
       <c r="C79" s="2" t="n"/>
       <c r="D79" s="2" t="n"/>
@@ -10143,7 +10217,7 @@
     <row r="80">
       <c r="A80" s="39" t="inlineStr">
         <is>
-          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
+          <t>no 17. Las demas aberturas son de una sola unidad.</t>
         </is>
       </c>
       <c r="B80" s="2" t="n"/>
@@ -10160,11 +10234,7 @@
       <c r="M80" s="2" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="39" t="inlineStr">
-        <is>
-          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
-        </is>
-      </c>
+      <c r="A81" s="39" t="inlineStr"/>
       <c r="B81" s="2" t="n"/>
       <c r="C81" s="2" t="n"/>
       <c r="D81" s="2" t="n"/>
@@ -10181,7 +10251,7 @@
     <row r="82">
       <c r="A82" s="39" t="inlineStr">
         <is>
-          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
+          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
         </is>
       </c>
       <c r="B82" s="2" t="n"/>
@@ -10197,22 +10267,94 @@
       <c r="L82" s="2" t="n"/>
       <c r="M82" s="2" t="n"/>
     </row>
+    <row r="83">
+      <c r="A83" s="39" t="inlineStr"/>
+      <c r="B83" s="2" t="n"/>
+      <c r="C83" s="2" t="n"/>
+      <c r="D83" s="2" t="n"/>
+      <c r="E83" s="2" t="n"/>
+      <c r="F83" s="2" t="n"/>
+      <c r="G83" s="2" t="n"/>
+      <c r="H83" s="2" t="n"/>
+      <c r="I83" s="2" t="n"/>
+      <c r="J83" s="2" t="n"/>
+      <c r="K83" s="2" t="n"/>
+      <c r="L83" s="2" t="n"/>
+      <c r="M83" s="2" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="39" t="inlineStr">
+        <is>
+          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="n"/>
+      <c r="C84" s="2" t="n"/>
+      <c r="D84" s="2" t="n"/>
+      <c r="E84" s="2" t="n"/>
+      <c r="F84" s="2" t="n"/>
+      <c r="G84" s="2" t="n"/>
+      <c r="H84" s="2" t="n"/>
+      <c r="I84" s="2" t="n"/>
+      <c r="J84" s="2" t="n"/>
+      <c r="K84" s="2" t="n"/>
+      <c r="L84" s="2" t="n"/>
+      <c r="M84" s="2" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="39" t="inlineStr">
+        <is>
+          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="n"/>
+      <c r="C85" s="2" t="n"/>
+      <c r="D85" s="2" t="n"/>
+      <c r="E85" s="2" t="n"/>
+      <c r="F85" s="2" t="n"/>
+      <c r="G85" s="2" t="n"/>
+      <c r="H85" s="2" t="n"/>
+      <c r="I85" s="2" t="n"/>
+      <c r="J85" s="2" t="n"/>
+      <c r="K85" s="2" t="n"/>
+      <c r="L85" s="2" t="n"/>
+      <c r="M85" s="2" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="39" t="inlineStr">
+        <is>
+          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="n"/>
+      <c r="C86" s="2" t="n"/>
+      <c r="D86" s="2" t="n"/>
+      <c r="E86" s="2" t="n"/>
+      <c r="F86" s="2" t="n"/>
+      <c r="G86" s="2" t="n"/>
+      <c r="H86" s="2" t="n"/>
+      <c r="I86" s="2" t="n"/>
+      <c r="J86" s="2" t="n"/>
+      <c r="K86" s="2" t="n"/>
+      <c r="L86" s="2" t="n"/>
+      <c r="M86" s="2" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A19:M19"/>
-    <mergeCell ref="A14:M14"/>
     <mergeCell ref="A1:M1"/>
+    <mergeCell ref="E7:E14"/>
     <mergeCell ref="A6:M6"/>
-    <mergeCell ref="E20:E27"/>
     <mergeCell ref="A4:M4"/>
-    <mergeCell ref="E29:E35"/>
     <mergeCell ref="A3:M3"/>
-    <mergeCell ref="E7:E13"/>
-    <mergeCell ref="E15:E18"/>
+    <mergeCell ref="E21:E29"/>
+    <mergeCell ref="A30:M30"/>
+    <mergeCell ref="E16:E19"/>
+    <mergeCell ref="A15:M15"/>
+    <mergeCell ref="E31:E37"/>
+    <mergeCell ref="A20:M20"/>
     <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A28:M28"/>
   </mergeCells>
-  <conditionalFormatting sqref="M6:M35">
+  <conditionalFormatting sqref="M6:M37">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
       <formula>"CUMPLE"</formula>
     </cfRule>
@@ -10221,13 +10363,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="H6:H35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Datos_higro!$A$10:$A$17</formula1>
     </dataValidation>
-    <dataValidation sqref="I6:I35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I6:I37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Datos_higro!$A$21:$A$27</formula1>
     </dataValidation>
-    <dataValidation sqref="K6:K35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K6:K37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Norte,Sur,Este,Oeste,Noreste,Noroeste,Sudeste,Sudoeste,Horizontal"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Planilla 3: las cortinas son blackout interiores, no computan
Una cortina interior no es proteccion solar: la radiacion ya atraveso el
vidrio cuando llega a la cortina. La ordenanza acredita protecciones
exteriores. Las veinte aberturas pasan a Sin Proteccion, con factor de
exposicion solar 0,88.

Se agrega la opcion "Cortina blackout INTERIOR (no computa)" a la lista
de protecciones, con 0,88, para que quede escrito en la planilla por que
no suma.

La verificacion sigue dando CUMPLE porque, como en la planilla de la
catedra, controla la transmitancia y no el FES.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -5018,11 +5018,11 @@
     <row r="22">
       <c r="A22" s="34" t="inlineStr">
         <is>
-          <t>Parasol horizontal fijo 1:2</t>
+          <t>Cortina blackout INTERIOR (no computa)</t>
         </is>
       </c>
       <c r="B22" s="9" t="n">
-        <v>0.35</v>
+        <v>0.88</v>
       </c>
       <c r="C22" s="2" t="n"/>
       <c r="D22" s="2" t="n"/>
@@ -5030,11 +5030,11 @@
     <row r="23">
       <c r="A23" s="34" t="inlineStr">
         <is>
-          <t>Parasol horizontal fijo 1:1</t>
+          <t>Parasol horizontal fijo 1:2</t>
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>0.5</v>
+        <v>0.35</v>
       </c>
       <c r="C23" s="2" t="n"/>
       <c r="D23" s="2" t="n"/>
@@ -5042,11 +5042,11 @@
     <row r="24">
       <c r="A24" s="34" t="inlineStr">
         <is>
-          <t>Alero</t>
+          <t>Parasol horizontal fijo 1:1</t>
         </is>
       </c>
       <c r="B24" s="9" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="C24" s="2" t="n"/>
       <c r="D24" s="2" t="n"/>
@@ -5054,11 +5054,11 @@
     <row r="25">
       <c r="A25" s="34" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Alero</t>
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>0.25</v>
+        <v>0.6</v>
       </c>
       <c r="C25" s="2" t="n"/>
       <c r="D25" s="2" t="n"/>
@@ -5066,11 +5066,11 @@
     <row r="26">
       <c r="A26" s="34" t="inlineStr">
         <is>
-          <t>Persiana de madera</t>
+          <t>Cortina de enrollar exterior</t>
         </is>
       </c>
       <c r="B26" s="9" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="C26" s="2" t="n"/>
       <c r="D26" s="2" t="n"/>
@@ -5078,18 +5078,24 @@
     <row r="27">
       <c r="A27" s="34" t="inlineStr">
         <is>
-          <t>Toldo</t>
+          <t>Persiana de madera</t>
         </is>
       </c>
       <c r="B27" s="9" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="C27" s="2" t="n"/>
       <c r="D27" s="2" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n"/>
-      <c r="B28" s="2" t="n"/>
+      <c r="A28" s="34" t="inlineStr">
+        <is>
+          <t>Toldo</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="n">
+        <v>0.2</v>
+      </c>
       <c r="C28" s="2" t="n"/>
       <c r="D28" s="2" t="n"/>
     </row>
@@ -7779,7 +7785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M86"/>
+  <dimension ref="A1:M89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.4" customWidth="1" min="1" max="1"/>
@@ -7998,7 +8004,7 @@
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Sin Proteccion</t>
         </is>
       </c>
       <c r="J7" s="8" t="n">
@@ -8010,7 +8016,7 @@
         </is>
       </c>
       <c r="L7" s="8">
-        <f>IF(I7="","",IFERROR(VLOOKUP(I7,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I7="","",IFERROR(VLOOKUP(I7,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M7" s="9">
@@ -8062,7 +8068,7 @@
         </is>
       </c>
       <c r="L8" s="8">
-        <f>IF(I8="","",IFERROR(VLOOKUP(I8,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I8="","",IFERROR(VLOOKUP(I8,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M8" s="9">
@@ -8102,7 +8108,7 @@
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Sin Proteccion</t>
         </is>
       </c>
       <c r="J9" s="8" t="n">
@@ -8114,7 +8120,7 @@
         </is>
       </c>
       <c r="L9" s="8">
-        <f>IF(I9="","",IFERROR(VLOOKUP(I9,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I9="","",IFERROR(VLOOKUP(I9,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M9" s="9">
@@ -8154,7 +8160,7 @@
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Sin Proteccion</t>
         </is>
       </c>
       <c r="J10" s="8" t="n">
@@ -8166,7 +8172,7 @@
         </is>
       </c>
       <c r="L10" s="8">
-        <f>IF(I10="","",IFERROR(VLOOKUP(I10,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I10="","",IFERROR(VLOOKUP(I10,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M10" s="9">
@@ -8206,7 +8212,7 @@
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Sin Proteccion</t>
         </is>
       </c>
       <c r="J11" s="8" t="n">
@@ -8218,7 +8224,7 @@
         </is>
       </c>
       <c r="L11" s="8">
-        <f>IF(I11="","",IFERROR(VLOOKUP(I11,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I11="","",IFERROR(VLOOKUP(I11,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M11" s="9">
@@ -8270,7 +8276,7 @@
         </is>
       </c>
       <c r="L12" s="8">
-        <f>IF(I12="","",IFERROR(VLOOKUP(I12,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I12="","",IFERROR(VLOOKUP(I12,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M12" s="9">
@@ -8300,7 +8306,7 @@
       <c r="J13" s="8" t="n"/>
       <c r="K13" s="9" t="n"/>
       <c r="L13" s="8">
-        <f>IF(I13="","",IFERROR(VLOOKUP(I13,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I13="","",IFERROR(VLOOKUP(I13,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M13" s="9">
@@ -8330,7 +8336,7 @@
       <c r="J14" s="12" t="n"/>
       <c r="K14" s="13" t="n"/>
       <c r="L14" s="12">
-        <f>IF(I14="","",IFERROR(VLOOKUP(I14,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I14="","",IFERROR(VLOOKUP(I14,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M14" s="13">
@@ -8392,7 +8398,7 @@
       </c>
       <c r="I16" s="9" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Sin Proteccion</t>
         </is>
       </c>
       <c r="J16" s="8" t="n">
@@ -8404,7 +8410,7 @@
         </is>
       </c>
       <c r="L16" s="8">
-        <f>IF(I16="","",IFERROR(VLOOKUP(I16,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I16="","",IFERROR(VLOOKUP(I16,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M16" s="9">
@@ -8456,7 +8462,7 @@
         </is>
       </c>
       <c r="L17" s="8">
-        <f>IF(I17="","",IFERROR(VLOOKUP(I17,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I17="","",IFERROR(VLOOKUP(I17,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M17" s="9">
@@ -8486,7 +8492,7 @@
       <c r="J18" s="8" t="n"/>
       <c r="K18" s="9" t="n"/>
       <c r="L18" s="8">
-        <f>IF(I18="","",IFERROR(VLOOKUP(I18,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I18="","",IFERROR(VLOOKUP(I18,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M18" s="9">
@@ -8516,7 +8522,7 @@
       <c r="J19" s="12" t="n"/>
       <c r="K19" s="13" t="n"/>
       <c r="L19" s="12">
-        <f>IF(I19="","",IFERROR(VLOOKUP(I19,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I19="","",IFERROR(VLOOKUP(I19,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M19" s="13">
@@ -8578,7 +8584,7 @@
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Sin Proteccion</t>
         </is>
       </c>
       <c r="J21" s="8" t="n">
@@ -8590,7 +8596,7 @@
         </is>
       </c>
       <c r="L21" s="8">
-        <f>IF(I21="","",IFERROR(VLOOKUP(I21,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I21="","",IFERROR(VLOOKUP(I21,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M21" s="9">
@@ -8642,7 +8648,7 @@
         </is>
       </c>
       <c r="L22" s="8">
-        <f>IF(I22="","",IFERROR(VLOOKUP(I22,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I22="","",IFERROR(VLOOKUP(I22,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M22" s="9">
@@ -8682,7 +8688,7 @@
       </c>
       <c r="I23" s="9" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Sin Proteccion</t>
         </is>
       </c>
       <c r="J23" s="8" t="n">
@@ -8694,7 +8700,7 @@
         </is>
       </c>
       <c r="L23" s="8">
-        <f>IF(I23="","",IFERROR(VLOOKUP(I23,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I23="","",IFERROR(VLOOKUP(I23,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M23" s="9">
@@ -8734,7 +8740,7 @@
       </c>
       <c r="I24" s="9" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Sin Proteccion</t>
         </is>
       </c>
       <c r="J24" s="8" t="n">
@@ -8746,7 +8752,7 @@
         </is>
       </c>
       <c r="L24" s="8">
-        <f>IF(I24="","",IFERROR(VLOOKUP(I24,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I24="","",IFERROR(VLOOKUP(I24,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M24" s="9">
@@ -8786,7 +8792,7 @@
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Sin Proteccion</t>
         </is>
       </c>
       <c r="J25" s="8" t="n">
@@ -8798,7 +8804,7 @@
         </is>
       </c>
       <c r="L25" s="8">
-        <f>IF(I25="","",IFERROR(VLOOKUP(I25,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I25="","",IFERROR(VLOOKUP(I25,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M25" s="9">
@@ -8838,7 +8844,7 @@
       </c>
       <c r="I26" s="9" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Sin Proteccion</t>
         </is>
       </c>
       <c r="J26" s="8" t="n">
@@ -8850,7 +8856,7 @@
         </is>
       </c>
       <c r="L26" s="8">
-        <f>IF(I26="","",IFERROR(VLOOKUP(I26,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I26="","",IFERROR(VLOOKUP(I26,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M26" s="9">
@@ -8902,7 +8908,7 @@
         </is>
       </c>
       <c r="L27" s="8">
-        <f>IF(I27="","",IFERROR(VLOOKUP(I27,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I27="","",IFERROR(VLOOKUP(I27,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M27" s="9">
@@ -8932,7 +8938,7 @@
       <c r="J28" s="8" t="n"/>
       <c r="K28" s="9" t="n"/>
       <c r="L28" s="8">
-        <f>IF(I28="","",IFERROR(VLOOKUP(I28,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I28="","",IFERROR(VLOOKUP(I28,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M28" s="9">
@@ -8962,7 +8968,7 @@
       <c r="J29" s="12" t="n"/>
       <c r="K29" s="13" t="n"/>
       <c r="L29" s="12">
-        <f>IF(I29="","",IFERROR(VLOOKUP(I29,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I29="","",IFERROR(VLOOKUP(I29,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M29" s="13">
@@ -9024,7 +9030,7 @@
       </c>
       <c r="I31" s="9" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Sin Proteccion</t>
         </is>
       </c>
       <c r="J31" s="8" t="n">
@@ -9036,7 +9042,7 @@
         </is>
       </c>
       <c r="L31" s="8">
-        <f>IF(I31="","",IFERROR(VLOOKUP(I31,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I31="","",IFERROR(VLOOKUP(I31,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M31" s="9">
@@ -9076,7 +9082,7 @@
       </c>
       <c r="I32" s="9" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Sin Proteccion</t>
         </is>
       </c>
       <c r="J32" s="8" t="n">
@@ -9088,7 +9094,7 @@
         </is>
       </c>
       <c r="L32" s="8">
-        <f>IF(I32="","",IFERROR(VLOOKUP(I32,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I32="","",IFERROR(VLOOKUP(I32,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M32" s="9">
@@ -9128,7 +9134,7 @@
       </c>
       <c r="I33" s="9" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Sin Proteccion</t>
         </is>
       </c>
       <c r="J33" s="8" t="n">
@@ -9140,7 +9146,7 @@
         </is>
       </c>
       <c r="L33" s="8">
-        <f>IF(I33="","",IFERROR(VLOOKUP(I33,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I33="","",IFERROR(VLOOKUP(I33,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M33" s="9">
@@ -9180,7 +9186,7 @@
       </c>
       <c r="I34" s="9" t="inlineStr">
         <is>
-          <t>Cortina de enrollar exterior</t>
+          <t>Sin Proteccion</t>
         </is>
       </c>
       <c r="J34" s="8" t="n">
@@ -9192,7 +9198,7 @@
         </is>
       </c>
       <c r="L34" s="8">
-        <f>IF(I34="","",IFERROR(VLOOKUP(I34,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I34="","",IFERROR(VLOOKUP(I34,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M34" s="9">
@@ -9244,7 +9250,7 @@
         </is>
       </c>
       <c r="L35" s="8">
-        <f>IF(I35="","",IFERROR(VLOOKUP(I35,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I35="","",IFERROR(VLOOKUP(I35,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M35" s="9">
@@ -9274,7 +9280,7 @@
       <c r="J36" s="8" t="n"/>
       <c r="K36" s="9" t="n"/>
       <c r="L36" s="8">
-        <f>IF(I36="","",IFERROR(VLOOKUP(I36,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I36="","",IFERROR(VLOOKUP(I36,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M36" s="9">
@@ -9304,7 +9310,7 @@
       <c r="J37" s="12" t="n"/>
       <c r="K37" s="13" t="n"/>
       <c r="L37" s="12">
-        <f>IF(I37="","",IFERROR(VLOOKUP(I37,Datos_higro!$A$21:$B$27,2,0),""))</f>
+        <f>IF(I37="","",IFERROR(VLOOKUP(I37,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
       <c r="M37" s="13">
@@ -9425,7 +9431,7 @@
     <row r="44">
       <c r="A44" s="23" t="inlineStr">
         <is>
-          <t>PROTECCION: ningun pano fijo PF tiene cortina: PF01, su gemelo, PF02, PF03, PF04 y PF05 van</t>
+          <t>PROTECCION: la obra tiene cortinas blackout INTERIORES, y los panos fijos PF no tienen nada.</t>
         </is>
       </c>
       <c r="B44" s="2" t="n"/>
@@ -9444,7 +9450,7 @@
     <row r="45">
       <c r="A45" s="23" t="inlineStr">
         <is>
-          <t>Sin Proteccion (FES 0,88). Las otras doce llevan cortina de enrollar exterior (FES 0,25).</t>
+          <t>Una cortina interior NO computa como proteccion solar: la radiacion ya atraveso el vidrio</t>
         </is>
       </c>
       <c r="B45" s="2" t="n"/>
@@ -9461,7 +9467,11 @@
       <c r="M45" s="2" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="23" t="inlineStr"/>
+      <c r="A46" s="23" t="inlineStr">
+        <is>
+          <t>cuando llega a la cortina. La ordenanza acredita protecciones exteriores (aleros, parasoles,</t>
+        </is>
+      </c>
       <c r="B46" s="2" t="n"/>
       <c r="C46" s="2" t="n"/>
       <c r="D46" s="2" t="n"/>
@@ -9478,7 +9488,7 @@
     <row r="47">
       <c r="A47" s="23" t="inlineStr">
         <is>
-          <t>OJO con esas seis: 0,88 esta muy por encima del maximo de 0,30 que la ordenanza admite para</t>
+          <t>cortinas de enrollar exteriores, toldos). Por eso las veinte aberturas van Sin Proteccion.</t>
         </is>
       </c>
       <c r="B47" s="2" t="n"/>
@@ -9495,11 +9505,7 @@
       <c r="M47" s="2" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="23" t="inlineStr">
-        <is>
-          <t>el cuadrante Este/Oeste, donde caen las cuatro fachadas de esta casa por estar girada 45</t>
-        </is>
-      </c>
+      <c r="A48" s="23" t="inlineStr"/>
       <c r="B48" s="2" t="n"/>
       <c r="C48" s="2" t="n"/>
       <c r="D48" s="2" t="n"/>
@@ -9516,7 +9522,7 @@
     <row r="49">
       <c r="A49" s="23" t="inlineStr">
         <is>
-          <t>grados. La verificacion de la planilla no lo controla, igual que la de la catedra, pero si lo</t>
+          <t>CONSECUENCIA: el factor de exposicion solar da 0,88 esta muy por encima del maximo de 0,30 que la ordenanza admite para</t>
         </is>
       </c>
       <c r="B49" s="2" t="n"/>
@@ -9535,7 +9541,7 @@
     <row r="50">
       <c r="A50" s="23" t="inlineStr">
         <is>
-          <t>presentas en el municipio esas cinco aberturas no pasarian el factor de exposicion solar.</t>
+          <t>el cuadrante Este/Oeste, donde caen las cuatro fachadas de esta casa por estar girada 45</t>
         </is>
       </c>
       <c r="B50" s="2" t="n"/>
@@ -9554,7 +9560,7 @@
     <row r="51">
       <c r="A51" s="23" t="inlineStr">
         <is>
-          <t>Hay una salida: si la abertura ocupa menos del 20% del lado expuesto del local, no se verifica</t>
+          <t>grados. La verificacion de la planilla no lo controla, igual que la de la catedra, pero si lo</t>
         </is>
       </c>
       <c r="B51" s="2" t="n"/>
@@ -9573,7 +9579,7 @@
     <row r="52">
       <c r="A52" s="23" t="inlineStr">
         <is>
-          <t>el FES. Conviene chequearlo local por local.</t>
+          <t>presentas en el municipio esas cinco aberturas no pasarian el factor de exposicion solar.</t>
         </is>
       </c>
       <c r="B52" s="2" t="n"/>
@@ -9590,7 +9596,11 @@
       <c r="M52" s="2" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="23" t="inlineStr"/>
+      <c r="A53" s="23" t="inlineStr">
+        <is>
+          <t>Hay dos salidas posibles: (a) si la abertura ocupa menos del 20% del lado expuesto del local,</t>
+        </is>
+      </c>
       <c r="B53" s="2" t="n"/>
       <c r="C53" s="2" t="n"/>
       <c r="D53" s="2" t="n"/>
@@ -9607,7 +9617,7 @@
     <row r="54">
       <c r="A54" s="23" t="inlineStr">
         <is>
-          <t>Orientacion: ya cargada. Factor de exposicion solar: se completa SOLO al elegir el tipo de</t>
+          <t>no se verifica el FES; (b) cambiar el vidrio por uno de control solar, que baja el FES sin</t>
         </is>
       </c>
       <c r="B54" s="2" t="n"/>
@@ -9626,7 +9636,7 @@
     <row r="55">
       <c r="A55" s="23" t="inlineStr">
         <is>
-          <t>proteccion, con los valores de la tabla de Datos_higro (Sin Proteccion 0,88; Parasol</t>
+          <t>tocar la obra. Agregar una proteccion exterior seria la tercera, pero implica obra.</t>
         </is>
       </c>
       <c r="B55" s="2" t="n"/>
@@ -9643,11 +9653,7 @@
       <c r="M55" s="2" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="23" t="inlineStr">
-        <is>
-          <t>horizontal fijo 1:2 0,35), que son los mismos de la planilla de la catedra.</t>
-        </is>
-      </c>
+      <c r="A56" s="23" t="inlineStr"/>
       <c r="B56" s="2" t="n"/>
       <c r="C56" s="2" t="n"/>
       <c r="D56" s="2" t="n"/>
@@ -9664,7 +9670,7 @@
     <row r="57">
       <c r="A57" s="23" t="inlineStr">
         <is>
-          <t>En Datos_higro esta ademas el FES maximo admitido por cuadrante segun la ordenanza, como</t>
+          <t>Orientacion: ya cargada. Factor de exposicion solar: se completa SOLO al elegir el tipo de</t>
         </is>
       </c>
       <c r="B57" s="2" t="n"/>
@@ -9683,7 +9689,7 @@
     <row r="58">
       <c r="A58" s="23" t="inlineStr">
         <is>
-          <t>referencia: la verificacion no lo controla, igual que en la planilla de la catedra.</t>
+          <t>proteccion, con los valores de la tabla de Datos_higro (Sin Proteccion 0,88; Parasol</t>
         </is>
       </c>
       <c r="B58" s="2" t="n"/>
@@ -9700,7 +9706,11 @@
       <c r="M58" s="2" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="23" t="inlineStr"/>
+      <c r="A59" s="23" t="inlineStr">
+        <is>
+          <t>horizontal fijo 1:2 0,35), que son los mismos de la planilla de la catedra.</t>
+        </is>
+      </c>
       <c r="B59" s="2" t="n"/>
       <c r="C59" s="2" t="n"/>
       <c r="D59" s="2" t="n"/>
@@ -9717,7 +9727,7 @@
     <row r="60">
       <c r="A60" s="23" t="inlineStr">
         <is>
-          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
+          <t>En Datos_higro esta ademas el FES maximo admitido por cuadrante segun la ordenanza, como</t>
         </is>
       </c>
       <c r="B60" s="2" t="n"/>
@@ -9736,7 +9746,7 @@
     <row r="61">
       <c r="A61" s="23" t="inlineStr">
         <is>
-          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
+          <t>referencia: la verificacion no lo controla, igual que en la planilla de la catedra.</t>
         </is>
       </c>
       <c r="B61" s="2" t="n"/>
@@ -9770,7 +9780,7 @@
     <row r="63">
       <c r="A63" s="23" t="inlineStr">
         <is>
-          <t>ALTURAS: medidas sobre el dibujo de las vistas de la planilla de carpinterias, con la escala</t>
+          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
         </is>
       </c>
       <c r="B63" s="2" t="n"/>
@@ -9789,7 +9799,7 @@
     <row r="64">
       <c r="A64" s="23" t="inlineStr">
         <is>
-          <t>verificada contra los anchos acotados (error menor a 2 cm). La mayoria de las aberturas son de</t>
+          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
         </is>
       </c>
       <c r="B64" s="2" t="n"/>
@@ -9806,11 +9816,7 @@
       <c r="M64" s="2" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="23" t="inlineStr">
-        <is>
-          <t>piso a cielorraso, 3,00 m. VERIFICARLAS contra el plano antes de presentar.</t>
-        </is>
-      </c>
+      <c r="A65" s="23" t="inlineStr"/>
       <c r="B65" s="2" t="n"/>
       <c r="C65" s="2" t="n"/>
       <c r="D65" s="2" t="n"/>
@@ -9827,7 +9833,7 @@
     <row r="66">
       <c r="A66" s="23" t="inlineStr">
         <is>
-          <t>PF04 es la unica con antepecho: arranca a 1,09 y mide 0,60 de alto. El resto llega al piso.</t>
+          <t>ALTURAS: medidas sobre el dibujo de las vistas de la planilla de carpinterias, con la escala</t>
         </is>
       </c>
       <c r="B66" s="2" t="n"/>
@@ -9846,7 +9852,7 @@
     <row r="67">
       <c r="A67" s="23" t="inlineStr">
         <is>
-          <t>Las alturas de PV01 (3,00), PF04 (0,60) y PV04 (2) (2,95) las aporto el autor del proyecto.</t>
+          <t>verificada contra los anchos acotados (error menor a 2 cm). La mayoria de las aberturas son de</t>
         </is>
       </c>
       <c r="B67" s="2" t="n"/>
@@ -9863,7 +9869,11 @@
       <c r="M67" s="2" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="23" t="inlineStr"/>
+      <c r="A68" s="23" t="inlineStr">
+        <is>
+          <t>piso a cielorraso, 3,00 m. VERIFICARLAS contra el plano antes de presentar.</t>
+        </is>
+      </c>
       <c r="B68" s="2" t="n"/>
       <c r="C68" s="2" t="n"/>
       <c r="D68" s="2" t="n"/>
@@ -9880,7 +9890,7 @@
     <row r="69">
       <c r="A69" s="23" t="inlineStr">
         <is>
-          <t>ORIENTACION: el simbolo de norte del plano (circulo con aguja, en el patio interno) apunta a</t>
+          <t>PF04 es la unica con antepecho: arranca a 1,09 y mide 0,60 de alto. El resto llega al piso.</t>
         </is>
       </c>
       <c r="B69" s="2" t="n"/>
@@ -9899,7 +9909,7 @@
     <row r="70">
       <c r="A70" s="23" t="inlineStr">
         <is>
-          <t>45 grados hacia arriba y a la derecha de la hoja. Entonces las cuatro fachadas NO son N-S-E-O</t>
+          <t>Las alturas de PV01 (3,00), PF04 (0,60) y PV04 (2) (2,95) las aporto el autor del proyecto.</t>
         </is>
       </c>
       <c r="B70" s="2" t="n"/>
@@ -9916,11 +9926,7 @@
       <c r="M70" s="2" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="23" t="inlineStr">
-        <is>
-          <t>sino: arriba = Noroeste, derecha = Noreste, abajo = Sudeste, izquierda = Sudoeste.</t>
-        </is>
-      </c>
+      <c r="A71" s="23" t="inlineStr"/>
       <c r="B71" s="2" t="n"/>
       <c r="C71" s="2" t="n"/>
       <c r="D71" s="2" t="n"/>
@@ -9937,7 +9943,7 @@
     <row r="72">
       <c r="A72" s="23" t="inlineStr">
         <is>
-          <t>Cada abertura se asigno a la fachada por su posicion en planta. Las del patio interno se</t>
+          <t>ORIENTACION: el simbolo de norte del plano (circulo con aguja, en el patio interno) apunta a</t>
         </is>
       </c>
       <c r="B72" s="2" t="n"/>
@@ -9956,7 +9962,7 @@
     <row r="73">
       <c r="A73" s="23" t="inlineStr">
         <is>
-          <t>orientan por la pared en la que estan: miran hacia adentro del patio.</t>
+          <t>45 grados hacia arriba y a la derecha de la hoja. Entonces las cuatro fachadas NO son N-S-E-O</t>
         </is>
       </c>
       <c r="B73" s="2" t="n"/>
@@ -9975,7 +9981,7 @@
     <row r="74">
       <c r="A74" s="23" t="inlineStr">
         <is>
-          <t>Los rotulos Dormitorio Norte y Dormitorio Sur del plano no coinciden con el norte real;</t>
+          <t>sino: arriba = Noroeste, derecha = Noreste, abajo = Sudeste, izquierda = Sudoeste.</t>
         </is>
       </c>
       <c r="B74" s="2" t="n"/>
@@ -9994,7 +10000,7 @@
     <row r="75">
       <c r="A75" s="23" t="inlineStr">
         <is>
-          <t>parecen ser nombres de uso, no orientaciones.</t>
+          <t>Cada abertura se asigno a la fachada por su posicion en planta. Las del patio interno se</t>
         </is>
       </c>
       <c r="B75" s="2" t="n"/>
@@ -10011,7 +10017,11 @@
       <c r="M75" s="2" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="23" t="inlineStr"/>
+      <c r="A76" s="23" t="inlineStr">
+        <is>
+          <t>orientan por la pared en la que estan: miran hacia adentro del patio.</t>
+        </is>
+      </c>
       <c r="B76" s="2" t="n"/>
       <c r="C76" s="2" t="n"/>
       <c r="D76" s="2" t="n"/>
@@ -10028,7 +10038,7 @@
     <row r="77">
       <c r="A77" s="23" t="inlineStr">
         <is>
-          <t>CANTIDADES: la planilla de carpinterias trae la cantidad de cada abertura. Tres van dos veces:</t>
+          <t>Los rotulos Dormitorio Norte y Dormitorio Sur del plano no coinciden con el norte real;</t>
         </is>
       </c>
       <c r="B77" s="2" t="n"/>
@@ -10047,7 +10057,7 @@
     <row r="78">
       <c r="A78" s="23" t="inlineStr">
         <is>
-          <t>VA01 (01 Cocina y 09 Suite), VA04 (13 Dormitorio Norte y 14 Play Room) y PF01 (03 Lavadero y</t>
+          <t>parecen ser nombres de uso, no orientaciones.</t>
         </is>
       </c>
       <c r="B78" s="2" t="n"/>
@@ -10064,11 +10074,7 @@
       <c r="M78" s="2" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="23" t="inlineStr">
-        <is>
-          <t>07 Hall de ingreso, a los dos lados del patio interno). Por eso la planilla tiene 20 filas y</t>
-        </is>
-      </c>
+      <c r="A79" s="23" t="inlineStr"/>
       <c r="B79" s="2" t="n"/>
       <c r="C79" s="2" t="n"/>
       <c r="D79" s="2" t="n"/>
@@ -10085,7 +10091,7 @@
     <row r="80">
       <c r="A80" s="23" t="inlineStr">
         <is>
-          <t>no 17. Las demas aberturas son de una sola unidad.</t>
+          <t>CANTIDADES: la planilla de carpinterias trae la cantidad de cada abertura. Tres van dos veces:</t>
         </is>
       </c>
       <c r="B80" s="2" t="n"/>
@@ -10102,7 +10108,11 @@
       <c r="M80" s="2" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="23" t="inlineStr"/>
+      <c r="A81" s="23" t="inlineStr">
+        <is>
+          <t>VA01 (01 Cocina y 09 Suite), VA04 (13 Dormitorio Norte y 14 Play Room) y PF01 (03 Lavadero y</t>
+        </is>
+      </c>
       <c r="B81" s="2" t="n"/>
       <c r="C81" s="2" t="n"/>
       <c r="D81" s="2" t="n"/>
@@ -10119,7 +10129,7 @@
     <row r="82">
       <c r="A82" s="23" t="inlineStr">
         <is>
-          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
+          <t>07 Hall de ingreso, a los dos lados del patio interno). Por eso la planilla tiene 20 filas y</t>
         </is>
       </c>
       <c r="B82" s="2" t="n"/>
@@ -10136,7 +10146,11 @@
       <c r="M82" s="2" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="23" t="inlineStr"/>
+      <c r="A83" s="23" t="inlineStr">
+        <is>
+          <t>no 17. Las demas aberturas son de una sola unidad.</t>
+        </is>
+      </c>
       <c r="B83" s="2" t="n"/>
       <c r="C83" s="2" t="n"/>
       <c r="D83" s="2" t="n"/>
@@ -10151,11 +10165,7 @@
       <c r="M83" s="2" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="23" t="inlineStr">
-        <is>
-          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
-        </is>
-      </c>
+      <c r="A84" s="23" t="inlineStr"/>
       <c r="B84" s="2" t="n"/>
       <c r="C84" s="2" t="n"/>
       <c r="D84" s="2" t="n"/>
@@ -10172,7 +10182,7 @@
     <row r="85">
       <c r="A85" s="23" t="inlineStr">
         <is>
-          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
+          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
         </is>
       </c>
       <c r="B85" s="2" t="n"/>
@@ -10189,11 +10199,7 @@
       <c r="M85" s="2" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="23" t="inlineStr">
-        <is>
-          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
-        </is>
-      </c>
+      <c r="A86" s="23" t="inlineStr"/>
       <c r="B86" s="2" t="n"/>
       <c r="C86" s="2" t="n"/>
       <c r="D86" s="2" t="n"/>
@@ -10206,6 +10212,63 @@
       <c r="K86" s="2" t="n"/>
       <c r="L86" s="2" t="n"/>
       <c r="M86" s="2" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="23" t="inlineStr">
+        <is>
+          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="n"/>
+      <c r="C87" s="2" t="n"/>
+      <c r="D87" s="2" t="n"/>
+      <c r="E87" s="2" t="n"/>
+      <c r="F87" s="2" t="n"/>
+      <c r="G87" s="2" t="n"/>
+      <c r="H87" s="2" t="n"/>
+      <c r="I87" s="2" t="n"/>
+      <c r="J87" s="2" t="n"/>
+      <c r="K87" s="2" t="n"/>
+      <c r="L87" s="2" t="n"/>
+      <c r="M87" s="2" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="23" t="inlineStr">
+        <is>
+          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="n"/>
+      <c r="C88" s="2" t="n"/>
+      <c r="D88" s="2" t="n"/>
+      <c r="E88" s="2" t="n"/>
+      <c r="F88" s="2" t="n"/>
+      <c r="G88" s="2" t="n"/>
+      <c r="H88" s="2" t="n"/>
+      <c r="I88" s="2" t="n"/>
+      <c r="J88" s="2" t="n"/>
+      <c r="K88" s="2" t="n"/>
+      <c r="L88" s="2" t="n"/>
+      <c r="M88" s="2" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="23" t="inlineStr">
+        <is>
+          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="n"/>
+      <c r="C89" s="2" t="n"/>
+      <c r="D89" s="2" t="n"/>
+      <c r="E89" s="2" t="n"/>
+      <c r="F89" s="2" t="n"/>
+      <c r="G89" s="2" t="n"/>
+      <c r="H89" s="2" t="n"/>
+      <c r="I89" s="2" t="n"/>
+      <c r="J89" s="2" t="n"/>
+      <c r="K89" s="2" t="n"/>
+      <c r="L89" s="2" t="n"/>
+      <c r="M89" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -10237,7 +10300,7 @@
       <formula1>=Datos_higro!$A$10:$A$17</formula1>
     </dataValidation>
     <dataValidation sqref="I6:I37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Datos_higro!$A$21:$A$27</formula1>
+      <formula1>=Datos_higro!$A$21:$A$28</formula1>
     </dataValidation>
     <dataValidation sqref="K6:K37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Norte,Sur,Este,Oeste,Noreste,Noroeste,Sudeste,Sudoeste,Horizontal"</formula1>

</xml_diff>

<commit_message>
Balance termico: cargar el radiador Peisa Tropical 80-500
245 kcal/h por elemento (valor de catalogo a salto termico 60 C), 80 mm
de ancho por elemento, 575 mm de alto. El factor 1,12 del formulario
sigue valiendo: pasa del salto de catalogo al de la instalacion, 66 C, y
coincide con (66/60)^1,3 = 1,13.

Se renombra "seccion" por "elemento", que es como lo llama el catalogo.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -6055,7 +6055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56.7" customWidth="1" min="1" max="1"/>
@@ -6252,7 +6252,7 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>Caldaia Lux 700</t>
+          <t>Peisa Tropical 80-500</t>
         </is>
       </c>
       <c r="C13" s="2" t="n"/>
@@ -6261,11 +6261,11 @@
     <row r="14" ht="39.7" customHeight="1">
       <c r="A14" s="38" t="inlineStr">
         <is>
-          <t>Kcal/h por seccion del radiador</t>
+          <t>Kcal/h por elemento del radiador</t>
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>268</v>
+        <v>245</v>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
@@ -6274,7 +6274,7 @@
       </c>
       <c r="D14" s="38" t="inlineStr">
         <is>
-          <t>Caldaia Lux 700. Cambiar segun catalogo.</t>
+          <t>Peisa Tropical 80-500, valor de catalogo a salto termico 60 C.</t>
         </is>
       </c>
     </row>
@@ -6294,14 +6294,14 @@
       </c>
       <c r="D15" s="38" t="inlineStr">
         <is>
-          <t>Del formulario modelo.</t>
+          <t>Pasa del salto de catalogo (60 C) al de la instalacion (66 C). (66/60)^1,3 = 1,13.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="39.7" customHeight="1">
       <c r="A16" s="38" t="inlineStr">
         <is>
-          <t>Ancho de cada seccion</t>
+          <t>Ancho de cada elemento</t>
         </is>
       </c>
       <c r="B16" s="9" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="D16" s="38" t="inlineStr">
         <is>
-          <t>Caldaia Lux 700.</t>
+          <t>Peisa Tropical: 80 mm por elemento.</t>
         </is>
       </c>
     </row>
@@ -6555,33 +6555,33 @@
     <row r="39" ht="39.7" customHeight="1">
       <c r="A39" s="23" t="inlineStr">
         <is>
-          <t>4. Confirmar el radiador y sus Kcal/h por seccion.</t>
+          <t>4. Nada: el radiador ya esta cargado (Peisa Tropical 80-500, aluminio inyectado en blanco,</t>
         </is>
       </c>
       <c r="B39" s="2" t="n"/>
       <c r="C39" s="2" t="n"/>
       <c r="D39" s="2" t="n"/>
     </row>
-    <row r="40">
-      <c r="A40" s="23" t="inlineStr"/>
+    <row r="40" ht="39.7" customHeight="1">
+      <c r="A40" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   245 kcal/h por elemento, 80 mm de ancho, 575 mm de alto, 0,375 l por elemento).</t>
+        </is>
+      </c>
       <c r="B40" s="2" t="n"/>
       <c r="C40" s="2" t="n"/>
       <c r="D40" s="2" t="n"/>
     </row>
-    <row r="41" ht="39.7" customHeight="1">
-      <c r="A41" s="22" t="inlineStr">
-        <is>
-          <t>LO QUE YA VIENE CARGADO</t>
-        </is>
-      </c>
+    <row r="41">
+      <c r="A41" s="23" t="inlineStr"/>
       <c r="B41" s="2" t="n"/>
       <c r="C41" s="2" t="n"/>
       <c r="D41" s="2" t="n"/>
     </row>
     <row r="42" ht="39.7" customHeight="1">
-      <c r="A42" s="23" t="inlineStr">
-        <is>
-          <t>- Superficie y volumen de cada local, de la planilla de iluminacion y ventilacion.</t>
+      <c r="A42" s="22" t="inlineStr">
+        <is>
+          <t>LO QUE YA VIENE CARGADO</t>
         </is>
       </c>
       <c r="B42" s="2" t="n"/>
@@ -6591,7 +6591,7 @@
     <row r="43" ht="39.7" customHeight="1">
       <c r="A43" s="23" t="inlineStr">
         <is>
-          <t>- Las aberturas de cada local con su medida real, del campo UBICACION de la planilla de</t>
+          <t>- Superficie y volumen de cada local, de la planilla de iluminacion y ventilacion.</t>
         </is>
       </c>
       <c r="B43" s="2" t="n"/>
@@ -6601,7 +6601,7 @@
     <row r="44" ht="39.7" customHeight="1">
       <c r="A44" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  carpinterias. Son 17 aberturas repartidas en 13 locales.</t>
+          <t>- Las aberturas de cada local con su medida real, del campo UBICACION de la planilla de</t>
         </is>
       </c>
       <c r="B44" s="2" t="n"/>
@@ -6611,7 +6611,7 @@
     <row r="45" ht="39.7" customHeight="1">
       <c r="A45" s="23" t="inlineStr">
         <is>
-          <t>- Techo y piso segun la planta: en PB entrepiso arriba y piso sobre tierra; en PA techo</t>
+          <t xml:space="preserve">  carpinterias. Son 17 aberturas repartidas en 13 locales.</t>
         </is>
       </c>
       <c r="B45" s="2" t="n"/>
@@ -6621,7 +6621,7 @@
     <row r="46" ht="39.7" customHeight="1">
       <c r="A46" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  aislado arriba y piso sobre local ocupado. Si algun local no es asi, mover el area de renglon.</t>
+          <t>- Techo y piso segun la planta: en PB entrepiso arriba y piso sobre tierra; en PA techo</t>
         </is>
       </c>
       <c r="B46" s="2" t="n"/>
@@ -6631,28 +6631,38 @@
     <row r="47" ht="39.7" customHeight="1">
       <c r="A47" s="23" t="inlineStr">
         <is>
-          <t>- Infiltracion segun la cantidad de paredes exteriores que se estimo para cada local.</t>
+          <t xml:space="preserve">  aislado arriba y piso sobre local ocupado. Si algun local no es asi, mover el area de renglon.</t>
         </is>
       </c>
       <c r="B47" s="2" t="n"/>
       <c r="C47" s="2" t="n"/>
       <c r="D47" s="2" t="n"/>
     </row>
-    <row r="48">
-      <c r="A48" s="23" t="inlineStr"/>
+    <row r="48" ht="39.7" customHeight="1">
+      <c r="A48" s="23" t="inlineStr">
+        <is>
+          <t>- Infiltracion segun la cantidad de paredes exteriores que se estimo para cada local.</t>
+        </is>
+      </c>
       <c r="B48" s="2" t="n"/>
       <c r="C48" s="2" t="n"/>
       <c r="D48" s="2" t="n"/>
     </row>
-    <row r="49" ht="39.7" customHeight="1">
-      <c r="A49" s="23" t="inlineStr">
-        <is>
-          <t>La altura de local adoptada es 3.00 m, de los cortes de la planilla de carpinterias.</t>
-        </is>
-      </c>
+    <row r="49">
+      <c r="A49" s="23" t="inlineStr"/>
       <c r="B49" s="2" t="n"/>
       <c r="C49" s="2" t="n"/>
       <c r="D49" s="2" t="n"/>
+    </row>
+    <row r="50" ht="39.7" customHeight="1">
+      <c r="A50" s="23" t="inlineStr">
+        <is>
+          <t>La altura de local adoptada es 3.00 m, de los cortes de la planilla de carpinterias.</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="n"/>
+      <c r="C50" s="2" t="n"/>
+      <c r="D50" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -23522,7 +23532,7 @@
       <c r="A34" s="9" t="n"/>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h por seccion</t>
+          <t>Kcal/h por elemento</t>
         </is>
       </c>
       <c r="C34" s="8">
@@ -23540,7 +23550,7 @@
       <c r="A35" s="9" t="n"/>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>Secciones necesarias</t>
+          <t>Elementos necesarios</t>
         </is>
       </c>
       <c r="C35" s="25">
@@ -24318,7 +24328,7 @@
       <c r="A69" s="9" t="n"/>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h por seccion</t>
+          <t>Kcal/h por elemento</t>
         </is>
       </c>
       <c r="C69" s="8">
@@ -24336,7 +24346,7 @@
       <c r="A70" s="9" t="n"/>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t>Secciones necesarias</t>
+          <t>Elementos necesarios</t>
         </is>
       </c>
       <c r="C70" s="25">
@@ -25084,7 +25094,7 @@
       <c r="A103" s="9" t="n"/>
       <c r="B103" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h por seccion</t>
+          <t>Kcal/h por elemento</t>
         </is>
       </c>
       <c r="C103" s="8">
@@ -25102,7 +25112,7 @@
       <c r="A104" s="9" t="n"/>
       <c r="B104" s="10" t="inlineStr">
         <is>
-          <t>Secciones necesarias</t>
+          <t>Elementos necesarios</t>
         </is>
       </c>
       <c r="C104" s="25">
@@ -25846,7 +25856,7 @@
       <c r="A137" s="9" t="n"/>
       <c r="B137" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h por seccion</t>
+          <t>Kcal/h por elemento</t>
         </is>
       </c>
       <c r="C137" s="8">
@@ -25864,7 +25874,7 @@
       <c r="A138" s="9" t="n"/>
       <c r="B138" s="10" t="inlineStr">
         <is>
-          <t>Secciones necesarias</t>
+          <t>Elementos necesarios</t>
         </is>
       </c>
       <c r="C138" s="25">
@@ -26642,7 +26652,7 @@
       <c r="A172" s="9" t="n"/>
       <c r="B172" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h por seccion</t>
+          <t>Kcal/h por elemento</t>
         </is>
       </c>
       <c r="C172" s="8">
@@ -26660,7 +26670,7 @@
       <c r="A173" s="9" t="n"/>
       <c r="B173" s="10" t="inlineStr">
         <is>
-          <t>Secciones necesarias</t>
+          <t>Elementos necesarios</t>
         </is>
       </c>
       <c r="C173" s="25">
@@ -27408,7 +27418,7 @@
       <c r="A206" s="9" t="n"/>
       <c r="B206" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h por seccion</t>
+          <t>Kcal/h por elemento</t>
         </is>
       </c>
       <c r="C206" s="8">
@@ -27426,7 +27436,7 @@
       <c r="A207" s="9" t="n"/>
       <c r="B207" s="10" t="inlineStr">
         <is>
-          <t>Secciones necesarias</t>
+          <t>Elementos necesarios</t>
         </is>
       </c>
       <c r="C207" s="25">
@@ -28170,7 +28180,7 @@
       <c r="A240" s="9" t="n"/>
       <c r="B240" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h por seccion</t>
+          <t>Kcal/h por elemento</t>
         </is>
       </c>
       <c r="C240" s="8">
@@ -28188,7 +28198,7 @@
       <c r="A241" s="9" t="n"/>
       <c r="B241" s="10" t="inlineStr">
         <is>
-          <t>Secciones necesarias</t>
+          <t>Elementos necesarios</t>
         </is>
       </c>
       <c r="C241" s="25">
@@ -28966,7 +28976,7 @@
       <c r="A275" s="9" t="n"/>
       <c r="B275" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h por seccion</t>
+          <t>Kcal/h por elemento</t>
         </is>
       </c>
       <c r="C275" s="8">
@@ -28984,7 +28994,7 @@
       <c r="A276" s="9" t="n"/>
       <c r="B276" s="10" t="inlineStr">
         <is>
-          <t>Secciones necesarias</t>
+          <t>Elementos necesarios</t>
         </is>
       </c>
       <c r="C276" s="25">
@@ -29732,7 +29742,7 @@
       <c r="A309" s="9" t="n"/>
       <c r="B309" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h por seccion</t>
+          <t>Kcal/h por elemento</t>
         </is>
       </c>
       <c r="C309" s="8">
@@ -29750,7 +29760,7 @@
       <c r="A310" s="9" t="n"/>
       <c r="B310" s="10" t="inlineStr">
         <is>
-          <t>Secciones necesarias</t>
+          <t>Elementos necesarios</t>
         </is>
       </c>
       <c r="C310" s="25">
@@ -30528,7 +30538,7 @@
       <c r="A344" s="9" t="n"/>
       <c r="B344" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h por seccion</t>
+          <t>Kcal/h por elemento</t>
         </is>
       </c>
       <c r="C344" s="8">
@@ -30546,7 +30556,7 @@
       <c r="A345" s="9" t="n"/>
       <c r="B345" s="10" t="inlineStr">
         <is>
-          <t>Secciones necesarias</t>
+          <t>Elementos necesarios</t>
         </is>
       </c>
       <c r="C345" s="25">
@@ -31290,7 +31300,7 @@
       <c r="A378" s="9" t="n"/>
       <c r="B378" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h por seccion</t>
+          <t>Kcal/h por elemento</t>
         </is>
       </c>
       <c r="C378" s="8">
@@ -31308,7 +31318,7 @@
       <c r="A379" s="9" t="n"/>
       <c r="B379" s="10" t="inlineStr">
         <is>
-          <t>Secciones necesarias</t>
+          <t>Elementos necesarios</t>
         </is>
       </c>
       <c r="C379" s="25">
@@ -32056,7 +32066,7 @@
       <c r="A412" s="9" t="n"/>
       <c r="B412" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h por seccion</t>
+          <t>Kcal/h por elemento</t>
         </is>
       </c>
       <c r="C412" s="8">
@@ -32074,7 +32084,7 @@
       <c r="A413" s="9" t="n"/>
       <c r="B413" s="10" t="inlineStr">
         <is>
-          <t>Secciones necesarias</t>
+          <t>Elementos necesarios</t>
         </is>
       </c>
       <c r="C413" s="25">

</xml_diff>

<commit_message>
Balance termico: toalleros en los banos
Los banos 10, 11 y 17 pasan a toallero Peisa Scala / Domino en vez de
radiador de elementos. La planilla elige el modelo sola: 80 (632 kcal/h,
500 x 800) si alcanza, y 150 (1174 kcal/h, 500 x 1500) si no.

Con las perdidas de hoy los tres piden el 150. El bano de visitas queda
al limite: 737 kcal/h contra 708 que da el 80 corregido por salto
termico, asi que por 29 kcal/h se va al grande.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -6055,7 +6055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56.7" customWidth="1" min="1" max="1"/>
@@ -6318,68 +6318,82 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="n"/>
+    <row r="17" ht="39.7" customHeight="1">
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>TOALLEROS (banos)</t>
+        </is>
+      </c>
       <c r="B17" s="2" t="n"/>
       <c r="C17" s="2" t="n"/>
       <c r="D17" s="2" t="n"/>
     </row>
     <row r="18" ht="39.7" customHeight="1">
-      <c r="A18" s="22" t="inlineStr">
-        <is>
-          <t>FACTORES DE PERDIDA (Kcal/h por m2, o por m3 en infiltracion)</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="n"/>
-      <c r="C18" s="2" t="n"/>
-      <c r="D18" s="2" t="n"/>
+      <c r="A18" s="38" t="inlineStr">
+        <is>
+          <t>Toallero Scala / Domino 80</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="n">
+        <v>632</v>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Kcal/h</t>
+        </is>
+      </c>
+      <c r="D18" s="38" t="inlineStr">
+        <is>
+          <t>500 x 800 mm. Valor de catalogo a 60 C.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="39.7" customHeight="1">
-      <c r="A19" s="37" t="inlineStr">
-        <is>
-          <t>elemento</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>factor</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="n"/>
-    </row>
-    <row r="20" ht="39.7" customHeight="1">
-      <c r="A20" s="38" t="inlineStr">
-        <is>
-          <t>Ventana</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="n">
-        <v>60</v>
-      </c>
+      <c r="A19" s="38" t="inlineStr">
+        <is>
+          <t>Toallero Scala / Domino 150</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="n">
+        <v>1174</v>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Kcal/h</t>
+        </is>
+      </c>
+      <c r="D19" s="38" t="inlineStr">
+        <is>
+          <t>500 x 1500 mm. Valor de catalogo a 60 C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="2" t="n"/>
       <c r="C20" s="2" t="n"/>
       <c r="D20" s="2" t="n"/>
     </row>
     <row r="21" ht="39.7" customHeight="1">
-      <c r="A21" s="38" t="inlineStr">
-        <is>
-          <t>Pared exterior aislada</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="n">
-        <v>20</v>
-      </c>
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t>FACTORES DE PERDIDA (Kcal/h por m2, o por m3 en infiltracion)</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n"/>
       <c r="C21" s="2" t="n"/>
       <c r="D21" s="2" t="n"/>
     </row>
     <row r="22" ht="39.7" customHeight="1">
-      <c r="A22" s="38" t="inlineStr">
-        <is>
-          <t>Pared interior</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="n">
-        <v>25</v>
+      <c r="A22" s="37" t="inlineStr">
+        <is>
+          <t>elemento</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>factor</t>
+        </is>
       </c>
       <c r="C22" s="2" t="n"/>
       <c r="D22" s="2" t="n"/>
@@ -6387,11 +6401,11 @@
     <row r="23" ht="39.7" customHeight="1">
       <c r="A23" s="38" t="inlineStr">
         <is>
-          <t>Techo no aislado</t>
+          <t>Ventana</t>
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="C23" s="2" t="n"/>
       <c r="D23" s="2" t="n"/>
@@ -6399,7 +6413,7 @@
     <row r="24" ht="39.7" customHeight="1">
       <c r="A24" s="38" t="inlineStr">
         <is>
-          <t>Techo aislado</t>
+          <t>Pared exterior aislada</t>
         </is>
       </c>
       <c r="B24" s="9" t="n">
@@ -6411,11 +6425,11 @@
     <row r="25" ht="39.7" customHeight="1">
       <c r="A25" s="38" t="inlineStr">
         <is>
-          <t>Techo entrepiso</t>
+          <t>Pared interior</t>
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="C25" s="2" t="n"/>
       <c r="D25" s="2" t="n"/>
@@ -6423,11 +6437,11 @@
     <row r="26" ht="39.7" customHeight="1">
       <c r="A26" s="38" t="inlineStr">
         <is>
-          <t>Piso sobre tierra</t>
+          <t>Techo no aislado</t>
         </is>
       </c>
       <c r="B26" s="9" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C26" s="2" t="n"/>
       <c r="D26" s="2" t="n"/>
@@ -6435,11 +6449,11 @@
     <row r="27" ht="39.7" customHeight="1">
       <c r="A27" s="38" t="inlineStr">
         <is>
-          <t>Piso sobre local ocupado</t>
+          <t>Techo aislado</t>
         </is>
       </c>
       <c r="B27" s="9" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C27" s="2" t="n"/>
       <c r="D27" s="2" t="n"/>
@@ -6447,11 +6461,11 @@
     <row r="28" ht="39.7" customHeight="1">
       <c r="A28" s="38" t="inlineStr">
         <is>
-          <t>Infiltracion, una pared exterior</t>
+          <t>Techo entrepiso</t>
         </is>
       </c>
       <c r="B28" s="9" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="C28" s="2" t="n"/>
       <c r="D28" s="2" t="n"/>
@@ -6459,11 +6473,11 @@
     <row r="29" ht="39.7" customHeight="1">
       <c r="A29" s="38" t="inlineStr">
         <is>
-          <t>Infiltracion, dos paredes exteriores</t>
+          <t>Piso sobre tierra</t>
         </is>
       </c>
       <c r="B29" s="9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C29" s="2" t="n"/>
       <c r="D29" s="2" t="n"/>
@@ -6471,71 +6485,77 @@
     <row r="30" ht="39.7" customHeight="1">
       <c r="A30" s="38" t="inlineStr">
         <is>
-          <t>Infiltracion, tres o mas paredes exteriores</t>
+          <t>Piso sobre local ocupado</t>
         </is>
       </c>
       <c r="B30" s="9" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C30" s="2" t="n"/>
       <c r="D30" s="2" t="n"/>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="n"/>
-      <c r="B31" s="2" t="n"/>
+    <row r="31" ht="39.7" customHeight="1">
+      <c r="A31" s="38" t="inlineStr">
+        <is>
+          <t>Infiltracion, una pared exterior</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="n">
+        <v>6</v>
+      </c>
       <c r="C31" s="2" t="n"/>
       <c r="D31" s="2" t="n"/>
     </row>
     <row r="32" ht="39.7" customHeight="1">
-      <c r="A32" s="22" t="inlineStr">
-        <is>
-          <t>Los factores estan escritos en cada renglon del formulario, no se leen de aca: esta tabla es solo de referencia.</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="n"/>
+      <c r="A32" s="38" t="inlineStr">
+        <is>
+          <t>Infiltracion, dos paredes exteriores</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="n">
+        <v>9</v>
+      </c>
       <c r="C32" s="2" t="n"/>
       <c r="D32" s="2" t="n"/>
     </row>
-    <row r="33">
-      <c r="A33" s="2" t="n"/>
-      <c r="B33" s="2" t="n"/>
+    <row r="33" ht="39.7" customHeight="1">
+      <c r="A33" s="38" t="inlineStr">
+        <is>
+          <t>Infiltracion, tres o mas paredes exteriores</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="n">
+        <v>12</v>
+      </c>
       <c r="C33" s="2" t="n"/>
       <c r="D33" s="2" t="n"/>
     </row>
-    <row r="34" ht="39.7" customHeight="1">
-      <c r="A34" s="22" t="inlineStr">
-        <is>
-          <t>QUE FALTA CARGAR</t>
-        </is>
-      </c>
+    <row r="34">
+      <c r="A34" s="2" t="n"/>
       <c r="B34" s="2" t="n"/>
       <c r="C34" s="2" t="n"/>
       <c r="D34" s="2" t="n"/>
     </row>
     <row r="35" ht="39.7" customHeight="1">
-      <c r="A35" s="23" t="inlineStr">
-        <is>
-          <t>1. Las longitudes de pared de cada local, en las columnas H (largo) e I (alto) del formulario.</t>
+      <c r="A35" s="22" t="inlineStr">
+        <is>
+          <t>Los factores estan escritos en cada renglon del formulario, no se leen de aca: esta tabla es solo de referencia.</t>
         </is>
       </c>
       <c r="B35" s="2" t="n"/>
       <c r="C35" s="2" t="n"/>
       <c r="D35" s="2" t="n"/>
     </row>
-    <row r="36" ht="39.7" customHeight="1">
-      <c r="A36" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Las celdas estan en naranja. Al cargarlas se completan solas la dimension, el area y la perdida.</t>
-        </is>
-      </c>
+    <row r="36">
+      <c r="A36" s="2" t="n"/>
       <c r="B36" s="2" t="n"/>
       <c r="C36" s="2" t="n"/>
       <c r="D36" s="2" t="n"/>
     </row>
     <row r="37" ht="39.7" customHeight="1">
-      <c r="A37" s="23" t="inlineStr">
-        <is>
-          <t>2. Si el muro es aislado o no: el formulario trae tres renglones de cada tipo, borrar los que sobren.</t>
+      <c r="A37" s="22" t="inlineStr">
+        <is>
+          <t>QUE FALTA CARGAR</t>
         </is>
       </c>
       <c r="B37" s="2" t="n"/>
@@ -6545,7 +6565,7 @@
     <row r="38" ht="39.7" customHeight="1">
       <c r="A38" s="23" t="inlineStr">
         <is>
-          <t>3. Las tablas de FO y FZ de la catedra. Por ahora los dos valen 1,00.</t>
+          <t>1. Las longitudes de pared de cada local, en las columnas H (largo) e I (alto) del formulario.</t>
         </is>
       </c>
       <c r="B38" s="2" t="n"/>
@@ -6555,7 +6575,7 @@
     <row r="39" ht="39.7" customHeight="1">
       <c r="A39" s="23" t="inlineStr">
         <is>
-          <t>4. Nada: el radiador ya esta cargado (Peisa Tropical 80-500, aluminio inyectado en blanco,</t>
+          <t xml:space="preserve">   Las celdas estan en naranja. Al cargarlas se completan solas la dimension, el area y la perdida.</t>
         </is>
       </c>
       <c r="B39" s="2" t="n"/>
@@ -6565,23 +6585,27 @@
     <row r="40" ht="39.7" customHeight="1">
       <c r="A40" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">   245 kcal/h por elemento, 80 mm de ancho, 575 mm de alto, 0,375 l por elemento).</t>
+          <t>2. Si el muro es aislado o no: el formulario trae tres renglones de cada tipo, borrar los que sobren.</t>
         </is>
       </c>
       <c r="B40" s="2" t="n"/>
       <c r="C40" s="2" t="n"/>
       <c r="D40" s="2" t="n"/>
     </row>
-    <row r="41">
-      <c r="A41" s="23" t="inlineStr"/>
+    <row r="41" ht="39.7" customHeight="1">
+      <c r="A41" s="23" t="inlineStr">
+        <is>
+          <t>3. Las tablas de FO y FZ de la catedra. Por ahora los dos valen 1,00.</t>
+        </is>
+      </c>
       <c r="B41" s="2" t="n"/>
       <c r="C41" s="2" t="n"/>
       <c r="D41" s="2" t="n"/>
     </row>
     <row r="42" ht="39.7" customHeight="1">
-      <c r="A42" s="22" t="inlineStr">
-        <is>
-          <t>LO QUE YA VIENE CARGADO</t>
+      <c r="A42" s="23" t="inlineStr">
+        <is>
+          <t>4. Nada: el radiador ya esta cargado (Peisa Tropical 80-500, aluminio inyectado en blanco,</t>
         </is>
       </c>
       <c r="B42" s="2" t="n"/>
@@ -6591,7 +6615,7 @@
     <row r="43" ht="39.7" customHeight="1">
       <c r="A43" s="23" t="inlineStr">
         <is>
-          <t>- Superficie y volumen de cada local, de la planilla de iluminacion y ventilacion.</t>
+          <t xml:space="preserve">   245 kcal/h por elemento, 80 mm de ancho, 575 mm de alto, 0,375 l por elemento).</t>
         </is>
       </c>
       <c r="B43" s="2" t="n"/>
@@ -6601,27 +6625,23 @@
     <row r="44" ht="39.7" customHeight="1">
       <c r="A44" s="23" t="inlineStr">
         <is>
-          <t>- Las aberturas de cada local con su medida real, del campo UBICACION de la planilla de</t>
+          <t xml:space="preserve">   En los tres banos va toallero Peisa Scala o Domino en vez de radiador de elementos.</t>
         </is>
       </c>
       <c r="B44" s="2" t="n"/>
       <c r="C44" s="2" t="n"/>
       <c r="D44" s="2" t="n"/>
     </row>
-    <row r="45" ht="39.7" customHeight="1">
-      <c r="A45" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  carpinterias. Son 17 aberturas repartidas en 13 locales.</t>
-        </is>
-      </c>
+    <row r="45">
+      <c r="A45" s="23" t="inlineStr"/>
       <c r="B45" s="2" t="n"/>
       <c r="C45" s="2" t="n"/>
       <c r="D45" s="2" t="n"/>
     </row>
     <row r="46" ht="39.7" customHeight="1">
-      <c r="A46" s="23" t="inlineStr">
-        <is>
-          <t>- Techo y piso segun la planta: en PB entrepiso arriba y piso sobre tierra; en PA techo</t>
+      <c r="A46" s="22" t="inlineStr">
+        <is>
+          <t>LO QUE YA VIENE CARGADO</t>
         </is>
       </c>
       <c r="B46" s="2" t="n"/>
@@ -6631,7 +6651,7 @@
     <row r="47" ht="39.7" customHeight="1">
       <c r="A47" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  aislado arriba y piso sobre local ocupado. Si algun local no es asi, mover el area de renglon.</t>
+          <t>- Superficie y volumen de cada local, de la planilla de iluminacion y ventilacion.</t>
         </is>
       </c>
       <c r="B47" s="2" t="n"/>
@@ -6641,15 +6661,19 @@
     <row r="48" ht="39.7" customHeight="1">
       <c r="A48" s="23" t="inlineStr">
         <is>
-          <t>- Infiltracion segun la cantidad de paredes exteriores que se estimo para cada local.</t>
+          <t>- Las aberturas de cada local con su medida real, del campo UBICACION de la planilla de</t>
         </is>
       </c>
       <c r="B48" s="2" t="n"/>
       <c r="C48" s="2" t="n"/>
       <c r="D48" s="2" t="n"/>
     </row>
-    <row r="49">
-      <c r="A49" s="23" t="inlineStr"/>
+    <row r="49" ht="39.7" customHeight="1">
+      <c r="A49" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  carpinterias. Son 17 aberturas repartidas en 13 locales.</t>
+        </is>
+      </c>
       <c r="B49" s="2" t="n"/>
       <c r="C49" s="2" t="n"/>
       <c r="D49" s="2" t="n"/>
@@ -6657,12 +6681,48 @@
     <row r="50" ht="39.7" customHeight="1">
       <c r="A50" s="23" t="inlineStr">
         <is>
-          <t>La altura de local adoptada es 3.00 m, de los cortes de la planilla de carpinterias.</t>
+          <t>- Techo y piso segun la planta: en PB entrepiso arriba y piso sobre tierra; en PA techo</t>
         </is>
       </c>
       <c r="B50" s="2" t="n"/>
       <c r="C50" s="2" t="n"/>
       <c r="D50" s="2" t="n"/>
+    </row>
+    <row r="51" ht="39.7" customHeight="1">
+      <c r="A51" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  aislado arriba y piso sobre local ocupado. Si algun local no es asi, mover el area de renglon.</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="n"/>
+      <c r="C51" s="2" t="n"/>
+      <c r="D51" s="2" t="n"/>
+    </row>
+    <row r="52" ht="39.7" customHeight="1">
+      <c r="A52" s="23" t="inlineStr">
+        <is>
+          <t>- Infiltracion segun la cantidad de paredes exteriores que se estimo para cada local.</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="n"/>
+      <c r="C52" s="2" t="n"/>
+      <c r="D52" s="2" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="23" t="inlineStr"/>
+      <c r="B53" s="2" t="n"/>
+      <c r="C53" s="2" t="n"/>
+      <c r="D53" s="2" t="n"/>
+    </row>
+    <row r="54" ht="39.7" customHeight="1">
+      <c r="A54" s="23" t="inlineStr">
+        <is>
+          <t>La altura de local adoptada es 3.00 m, de los cortes de la planilla de carpinterias.</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="n"/>
+      <c r="C54" s="2" t="n"/>
+      <c r="D54" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -27418,11 +27478,11 @@
       <c r="A206" s="9" t="n"/>
       <c r="B206" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h por elemento</t>
-        </is>
-      </c>
-      <c r="C206" s="8">
-        <f>ROUND(Datos_balance!$B$14*Datos_balance!$B$15,2)</f>
+          <t>Kcal/h del toallero Scala/Domino 80</t>
+        </is>
+      </c>
+      <c r="C206" s="25">
+        <f>ROUND(Datos_balance!$B$18*Datos_balance!$B$15,0)</f>
         <v/>
       </c>
       <c r="D206" s="2" t="n"/>
@@ -27436,11 +27496,11 @@
       <c r="A207" s="9" t="n"/>
       <c r="B207" s="10" t="inlineStr">
         <is>
-          <t>Elementos necesarios</t>
+          <t>Kcal/h del toallero Scala/Domino 150</t>
         </is>
       </c>
       <c r="C207" s="25">
-        <f>ROUNDUP(F203/(Datos_balance!$B$14*Datos_balance!$B$15),0)</f>
+        <f>ROUND(Datos_balance!$B$19*Datos_balance!$B$15,0)</f>
         <v/>
       </c>
       <c r="D207" s="2" t="n"/>
@@ -27450,15 +27510,15 @@
       <c r="H207" s="2" t="n"/>
       <c r="I207" s="2" t="n"/>
     </row>
-    <row r="208" ht="39.7" customHeight="1">
+    <row r="208" ht="47" customHeight="1">
       <c r="A208" s="9" t="n"/>
       <c r="B208" s="10" t="inlineStr">
         <is>
-          <t>Ancho del radiador (cm)</t>
+          <t>Toalleros necesarios</t>
         </is>
       </c>
       <c r="C208" s="25">
-        <f>ROUNDUP(F203/(Datos_balance!$B$14*Datos_balance!$B$15),0)*Datos_balance!$B$16</f>
+        <f>IF(F203&lt;=Datos_balance!$B$18*Datos_balance!$B$15,1,ROUNDUP(F203/(Datos_balance!$B$19*Datos_balance!$B$15),0))</f>
         <v/>
       </c>
       <c r="D208" s="2" t="n"/>
@@ -27468,15 +27528,15 @@
       <c r="H208" s="2" t="n"/>
       <c r="I208" s="2" t="n"/>
     </row>
-    <row r="209" ht="39.7" customHeight="1">
+    <row r="209" ht="47" customHeight="1">
       <c r="A209" s="13" t="n"/>
       <c r="B209" s="14" t="inlineStr">
         <is>
-          <t>Radiador adoptado</t>
+          <t>Toallero adoptado</t>
         </is>
       </c>
       <c r="C209" s="13">
-        <f>Datos_balance!$B$13</f>
+        <f>IF(F203&lt;=Datos_balance!$B$18*Datos_balance!$B$15,"Peisa Scala / Domino 80  (500 x 800 mm)","Peisa Scala / Domino 150  (500 x 1500 mm)")</f>
         <v/>
       </c>
       <c r="D209" s="20" t="n"/>
@@ -28180,11 +28240,11 @@
       <c r="A240" s="9" t="n"/>
       <c r="B240" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h por elemento</t>
-        </is>
-      </c>
-      <c r="C240" s="8">
-        <f>ROUND(Datos_balance!$B$14*Datos_balance!$B$15,2)</f>
+          <t>Kcal/h del toallero Scala/Domino 80</t>
+        </is>
+      </c>
+      <c r="C240" s="25">
+        <f>ROUND(Datos_balance!$B$18*Datos_balance!$B$15,0)</f>
         <v/>
       </c>
       <c r="D240" s="2" t="n"/>
@@ -28198,11 +28258,11 @@
       <c r="A241" s="9" t="n"/>
       <c r="B241" s="10" t="inlineStr">
         <is>
-          <t>Elementos necesarios</t>
+          <t>Kcal/h del toallero Scala/Domino 150</t>
         </is>
       </c>
       <c r="C241" s="25">
-        <f>ROUNDUP(F237/(Datos_balance!$B$14*Datos_balance!$B$15),0)</f>
+        <f>ROUND(Datos_balance!$B$19*Datos_balance!$B$15,0)</f>
         <v/>
       </c>
       <c r="D241" s="2" t="n"/>
@@ -28212,15 +28272,15 @@
       <c r="H241" s="2" t="n"/>
       <c r="I241" s="2" t="n"/>
     </row>
-    <row r="242" ht="39.7" customHeight="1">
+    <row r="242" ht="47" customHeight="1">
       <c r="A242" s="9" t="n"/>
       <c r="B242" s="10" t="inlineStr">
         <is>
-          <t>Ancho del radiador (cm)</t>
+          <t>Toalleros necesarios</t>
         </is>
       </c>
       <c r="C242" s="25">
-        <f>ROUNDUP(F237/(Datos_balance!$B$14*Datos_balance!$B$15),0)*Datos_balance!$B$16</f>
+        <f>IF(F237&lt;=Datos_balance!$B$18*Datos_balance!$B$15,1,ROUNDUP(F237/(Datos_balance!$B$19*Datos_balance!$B$15),0))</f>
         <v/>
       </c>
       <c r="D242" s="2" t="n"/>
@@ -28230,15 +28290,15 @@
       <c r="H242" s="2" t="n"/>
       <c r="I242" s="2" t="n"/>
     </row>
-    <row r="243" ht="39.7" customHeight="1">
+    <row r="243" ht="47" customHeight="1">
       <c r="A243" s="13" t="n"/>
       <c r="B243" s="14" t="inlineStr">
         <is>
-          <t>Radiador adoptado</t>
+          <t>Toallero adoptado</t>
         </is>
       </c>
       <c r="C243" s="13">
-        <f>Datos_balance!$B$13</f>
+        <f>IF(F237&lt;=Datos_balance!$B$18*Datos_balance!$B$15,"Peisa Scala / Domino 80  (500 x 800 mm)","Peisa Scala / Domino 150  (500 x 1500 mm)")</f>
         <v/>
       </c>
       <c r="D243" s="20" t="n"/>
@@ -32066,11 +32126,11 @@
       <c r="A412" s="9" t="n"/>
       <c r="B412" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h por elemento</t>
-        </is>
-      </c>
-      <c r="C412" s="8">
-        <f>ROUND(Datos_balance!$B$14*Datos_balance!$B$15,2)</f>
+          <t>Kcal/h del toallero Scala/Domino 80</t>
+        </is>
+      </c>
+      <c r="C412" s="25">
+        <f>ROUND(Datos_balance!$B$18*Datos_balance!$B$15,0)</f>
         <v/>
       </c>
       <c r="D412" s="2" t="n"/>
@@ -32084,11 +32144,11 @@
       <c r="A413" s="9" t="n"/>
       <c r="B413" s="10" t="inlineStr">
         <is>
-          <t>Elementos necesarios</t>
+          <t>Kcal/h del toallero Scala/Domino 150</t>
         </is>
       </c>
       <c r="C413" s="25">
-        <f>ROUNDUP(F409/(Datos_balance!$B$14*Datos_balance!$B$15),0)</f>
+        <f>ROUND(Datos_balance!$B$19*Datos_balance!$B$15,0)</f>
         <v/>
       </c>
       <c r="D413" s="2" t="n"/>
@@ -32098,15 +32158,15 @@
       <c r="H413" s="2" t="n"/>
       <c r="I413" s="2" t="n"/>
     </row>
-    <row r="414" ht="39.7" customHeight="1">
+    <row r="414" ht="47" customHeight="1">
       <c r="A414" s="9" t="n"/>
       <c r="B414" s="10" t="inlineStr">
         <is>
-          <t>Ancho del radiador (cm)</t>
+          <t>Toalleros necesarios</t>
         </is>
       </c>
       <c r="C414" s="25">
-        <f>ROUNDUP(F409/(Datos_balance!$B$14*Datos_balance!$B$15),0)*Datos_balance!$B$16</f>
+        <f>IF(F409&lt;=Datos_balance!$B$18*Datos_balance!$B$15,1,ROUNDUP(F409/(Datos_balance!$B$19*Datos_balance!$B$15),0))</f>
         <v/>
       </c>
       <c r="D414" s="2" t="n"/>
@@ -32116,15 +32176,15 @@
       <c r="H414" s="2" t="n"/>
       <c r="I414" s="2" t="n"/>
     </row>
-    <row r="415" ht="39.7" customHeight="1">
+    <row r="415" ht="47" customHeight="1">
       <c r="A415" s="13" t="n"/>
       <c r="B415" s="14" t="inlineStr">
         <is>
-          <t>Radiador adoptado</t>
+          <t>Toallero adoptado</t>
         </is>
       </c>
       <c r="C415" s="13">
-        <f>Datos_balance!$B$13</f>
+        <f>IF(F409&lt;=Datos_balance!$B$18*Datos_balance!$B$15,"Peisa Scala / Domino 80  (500 x 800 mm)","Peisa Scala / Domino 150  (500 x 1500 mm)")</f>
         <v/>
       </c>
       <c r="D415" s="20" t="n"/>

</xml_diff>

<commit_message>
Balance termico: medida real del vestidor
5,25 x 1,09, el ancho libre sin el placard, dato del autor del proyecto.
Reemplaza la lectura que se habia hecho sobre el plano (3,38 x 1,74).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -25486,7 +25486,7 @@
       </c>
       <c r="G118" s="2" t="n"/>
       <c r="H118" s="35" t="n">
-        <v>3.38</v>
+        <v>5.25</v>
       </c>
       <c r="I118" s="35" t="n">
         <v>3</v>
@@ -25516,7 +25516,7 @@
       </c>
       <c r="G119" s="2" t="n"/>
       <c r="H119" s="35" t="n">
-        <v>1.74</v>
+        <v>1.09</v>
       </c>
       <c r="I119" s="35" t="n">
         <v>3</v>
@@ -25546,7 +25546,7 @@
       </c>
       <c r="G120" s="2" t="n"/>
       <c r="H120" s="35" t="n">
-        <v>3.38</v>
+        <v>5.25</v>
       </c>
       <c r="I120" s="35" t="n">
         <v>3</v>
@@ -25576,7 +25576,7 @@
       </c>
       <c r="G121" s="2" t="n"/>
       <c r="H121" s="35" t="n">
-        <v>1.74</v>
+        <v>1.09</v>
       </c>
       <c r="I121" s="35" t="n">
         <v>3</v>
@@ -25660,7 +25660,7 @@
         </is>
       </c>
       <c r="D125" s="8" t="n">
-        <v>5.88</v>
+        <v>5.72</v>
       </c>
       <c r="E125" s="25" t="n">
         <v>15</v>
@@ -25705,7 +25705,7 @@
         </is>
       </c>
       <c r="D127" s="8" t="n">
-        <v>5.88</v>
+        <v>5.72</v>
       </c>
       <c r="E127" s="25" t="n">
         <v>10</v>
@@ -25773,11 +25773,11 @@
       </c>
       <c r="C130" s="9" t="inlineStr">
         <is>
-          <t>5.88 m2 x 3.00</t>
+          <t>5.72 m2 x 3.00</t>
         </is>
       </c>
       <c r="D130" s="8" t="n">
-        <v>17.64</v>
+        <v>17.16</v>
       </c>
       <c r="E130" s="25" t="n">
         <v>6</v>

</xml_diff>

<commit_message>
Balance termico: el antebano es en L, dos rectangulos
3,38 x 1,66 mas 1,09 x 1,49, que dan 7,23 m2. La planilla admite ahora un
segundo rectangulo por local y suma los lados de los dos en los
renglones de pared.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -42,7 +42,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="5">'Vigas de fundacion'!$A$1:$X$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Pilotes y cabezales'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Tabiques'!$1:$3</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="8">'Balance termico'!$A$1:$F$418</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="8">'Balance termico'!$A$1:$F$420</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22778,7 +22778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I415"/>
+  <dimension ref="A1:I417"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.1" customWidth="1" min="1" max="1"/>
@@ -30930,7 +30930,7 @@
       </c>
       <c r="G359" s="2" t="n"/>
       <c r="H359" s="35" t="n">
-        <v>3.9</v>
+        <v>3.38</v>
       </c>
       <c r="I359" s="35" t="n">
         <v>3</v>
@@ -30960,7 +30960,7 @@
       </c>
       <c r="G360" s="2" t="n"/>
       <c r="H360" s="35" t="n">
-        <v>1.5</v>
+        <v>1.66</v>
       </c>
       <c r="I360" s="35" t="n">
         <v>3</v>
@@ -30990,7 +30990,7 @@
       </c>
       <c r="G361" s="2" t="n"/>
       <c r="H361" s="35" t="n">
-        <v>3.9</v>
+        <v>3.38</v>
       </c>
       <c r="I361" s="35" t="n">
         <v>3</v>
@@ -31020,85 +31020,96 @@
       </c>
       <c r="G362" s="2" t="n"/>
       <c r="H362" s="35" t="n">
-        <v>1.5</v>
+        <v>1.66</v>
       </c>
       <c r="I362" s="35" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="363" ht="39.7" customHeight="1">
-      <c r="A363" s="16" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B363" s="33" t="inlineStr">
-        <is>
-          <t>TECHOS O CIELORRASOS</t>
-        </is>
-      </c>
-      <c r="C363" s="9" t="n"/>
-      <c r="D363" s="9" t="n"/>
-      <c r="E363" s="9" t="n"/>
-      <c r="F363" s="9" t="n"/>
+    <row r="363" ht="62" customHeight="1">
+      <c r="A363" s="9" t="n"/>
+      <c r="B363" s="34" t="inlineStr">
+        <is>
+          <t>INTERIORES (    )</t>
+        </is>
+      </c>
+      <c r="C363" s="9">
+        <f>IF(COUNT(H363,I363)&lt;2,"",TEXT(H363,"0.00")&amp;" x "&amp;TEXT(I363,"0.00"))</f>
+        <v/>
+      </c>
+      <c r="D363" s="8">
+        <f>IF(COUNT(H363,I363)&lt;2,"",ROUND(H363*I363,2))</f>
+        <v/>
+      </c>
+      <c r="E363" s="25" t="n">
+        <v>25</v>
+      </c>
+      <c r="F363" s="28">
+        <f>IF(D363="","",ROUND(D363*E363,1))</f>
+        <v/>
+      </c>
       <c r="G363" s="2" t="n"/>
-      <c r="H363" s="2" t="n"/>
-      <c r="I363" s="2" t="n"/>
+      <c r="H363" s="35" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="I363" s="35" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="364" ht="62" customHeight="1">
       <c r="A364" s="9" t="n"/>
       <c r="B364" s="34" t="inlineStr">
         <is>
-          <t>TECHO NO AISLADO</t>
-        </is>
-      </c>
-      <c r="C364" s="9" t="inlineStr"/>
+          <t>INTERIORES (    )</t>
+        </is>
+      </c>
+      <c r="C364" s="9">
+        <f>IF(COUNT(H364,I364)&lt;2,"",TEXT(H364,"0.00")&amp;" x "&amp;TEXT(I364,"0.00"))</f>
+        <v/>
+      </c>
       <c r="D364" s="8">
         <f>IF(COUNT(H364,I364)&lt;2,"",ROUND(H364*I364,2))</f>
         <v/>
       </c>
       <c r="E364" s="25" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F364" s="28">
         <f>IF(D364="","",ROUND(D364*E364,1))</f>
         <v/>
       </c>
       <c r="G364" s="2" t="n"/>
-      <c r="H364" s="35" t="n"/>
-      <c r="I364" s="35" t="n"/>
+      <c r="H364" s="35" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="I364" s="35" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="365" ht="39.7" customHeight="1">
-      <c r="A365" s="9" t="n"/>
-      <c r="B365" s="34" t="inlineStr">
-        <is>
-          <t>TECHO AISLADO</t>
-        </is>
-      </c>
-      <c r="C365" s="9" t="inlineStr">
-        <is>
-          <t>por croquis</t>
-        </is>
-      </c>
-      <c r="D365" s="8" t="n">
-        <v>5.85</v>
-      </c>
-      <c r="E365" s="25" t="n">
-        <v>20</v>
-      </c>
-      <c r="F365" s="28">
-        <f>IF(D365="","",ROUND(D365*E365,1))</f>
-        <v/>
-      </c>
+      <c r="A365" s="16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B365" s="33" t="inlineStr">
+        <is>
+          <t>TECHOS O CIELORRASOS</t>
+        </is>
+      </c>
+      <c r="C365" s="9" t="n"/>
+      <c r="D365" s="9" t="n"/>
+      <c r="E365" s="9" t="n"/>
+      <c r="F365" s="9" t="n"/>
       <c r="G365" s="2" t="n"/>
-      <c r="H365" s="35" t="n"/>
-      <c r="I365" s="35" t="n"/>
+      <c r="H365" s="2" t="n"/>
+      <c r="I365" s="2" t="n"/>
     </row>
     <row r="366" ht="62" customHeight="1">
       <c r="A366" s="9" t="n"/>
       <c r="B366" s="34" t="inlineStr">
         <is>
-          <t>TECHO ENTREPISO</t>
+          <t>TECHO NO AISLADO</t>
         </is>
       </c>
       <c r="C366" s="9" t="inlineStr"/>
@@ -31107,7 +31118,7 @@
         <v/>
       </c>
       <c r="E366" s="25" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F366" s="28">
         <f>IF(D366="","",ROUND(D366*E366,1))</f>
@@ -31118,29 +31129,36 @@
       <c r="I366" s="35" t="n"/>
     </row>
     <row r="367" ht="39.7" customHeight="1">
-      <c r="A367" s="16" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B367" s="33" t="inlineStr">
-        <is>
-          <t>PISO</t>
-        </is>
-      </c>
-      <c r="C367" s="9" t="n"/>
-      <c r="D367" s="9" t="n"/>
-      <c r="E367" s="9" t="n"/>
-      <c r="F367" s="9" t="n"/>
+      <c r="A367" s="9" t="n"/>
+      <c r="B367" s="34" t="inlineStr">
+        <is>
+          <t>TECHO AISLADO</t>
+        </is>
+      </c>
+      <c r="C367" s="9" t="inlineStr">
+        <is>
+          <t>por croquis</t>
+        </is>
+      </c>
+      <c r="D367" s="8" t="n">
+        <v>7.23</v>
+      </c>
+      <c r="E367" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="F367" s="28">
+        <f>IF(D367="","",ROUND(D367*E367,1))</f>
+        <v/>
+      </c>
       <c r="G367" s="2" t="n"/>
-      <c r="H367" s="2" t="n"/>
-      <c r="I367" s="2" t="n"/>
+      <c r="H367" s="35" t="n"/>
+      <c r="I367" s="35" t="n"/>
     </row>
     <row r="368" ht="62" customHeight="1">
       <c r="A368" s="9" t="n"/>
       <c r="B368" s="34" t="inlineStr">
         <is>
-          <t>SOBRE TIERRA</t>
+          <t>TECHO ENTREPISO</t>
         </is>
       </c>
       <c r="C368" s="9" t="inlineStr"/>
@@ -31149,7 +31167,7 @@
         <v/>
       </c>
       <c r="E368" s="25" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F368" s="28">
         <f>IF(D368="","",ROUND(D368*E368,1))</f>
@@ -31160,71 +31178,64 @@
       <c r="I368" s="35" t="n"/>
     </row>
     <row r="369" ht="39.7" customHeight="1">
-      <c r="A369" s="9" t="n"/>
-      <c r="B369" s="34" t="inlineStr">
-        <is>
-          <t>SOBRE LOCAL OCUPADO</t>
-        </is>
-      </c>
-      <c r="C369" s="9" t="inlineStr">
-        <is>
-          <t>por croquis</t>
-        </is>
-      </c>
-      <c r="D369" s="8" t="n">
-        <v>5.85</v>
-      </c>
-      <c r="E369" s="25" t="n">
-        <v>15</v>
-      </c>
-      <c r="F369" s="28">
-        <f>IF(D369="","",ROUND(D369*E369,1))</f>
-        <v/>
-      </c>
+      <c r="A369" s="16" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B369" s="33" t="inlineStr">
+        <is>
+          <t>PISO</t>
+        </is>
+      </c>
+      <c r="C369" s="9" t="n"/>
+      <c r="D369" s="9" t="n"/>
+      <c r="E369" s="9" t="n"/>
+      <c r="F369" s="9" t="n"/>
       <c r="G369" s="2" t="n"/>
-      <c r="H369" s="35" t="n"/>
-      <c r="I369" s="35" t="n"/>
-    </row>
-    <row r="370" ht="39.7" customHeight="1">
-      <c r="A370" s="16" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B370" s="33" t="inlineStr">
-        <is>
-          <t>INFILTRACION</t>
-        </is>
-      </c>
-      <c r="C370" s="9" t="n"/>
-      <c r="D370" s="16" t="inlineStr">
-        <is>
-          <t>VOLUMEN (m3)</t>
-        </is>
-      </c>
-      <c r="E370" s="9" t="n"/>
-      <c r="F370" s="9" t="n"/>
+      <c r="H369" s="2" t="n"/>
+      <c r="I369" s="2" t="n"/>
+    </row>
+    <row r="370" ht="62" customHeight="1">
+      <c r="A370" s="9" t="n"/>
+      <c r="B370" s="34" t="inlineStr">
+        <is>
+          <t>SOBRE TIERRA</t>
+        </is>
+      </c>
+      <c r="C370" s="9" t="inlineStr"/>
+      <c r="D370" s="8">
+        <f>IF(COUNT(H370,I370)&lt;2,"",ROUND(H370*I370,2))</f>
+        <v/>
+      </c>
+      <c r="E370" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="F370" s="28">
+        <f>IF(D370="","",ROUND(D370*E370,1))</f>
+        <v/>
+      </c>
       <c r="G370" s="2" t="n"/>
-      <c r="H370" s="2" t="n"/>
-      <c r="I370" s="2" t="n"/>
+      <c r="H370" s="35" t="n"/>
+      <c r="I370" s="35" t="n"/>
     </row>
     <row r="371" ht="39.7" customHeight="1">
       <c r="A371" s="9" t="n"/>
       <c r="B371" s="34" t="inlineStr">
         <is>
-          <t>UNA PARED EXTERIOR</t>
+          <t>SOBRE LOCAL OCUPADO</t>
         </is>
       </c>
       <c r="C371" s="9" t="inlineStr">
         <is>
-          <t>5.85 m2 x 3.00</t>
+          <t>por croquis</t>
         </is>
       </c>
       <c r="D371" s="8" t="n">
-        <v>17.55</v>
+        <v>7.23</v>
       </c>
       <c r="E371" s="25" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="F371" s="28">
         <f>IF(D371="","",ROUND(D371*E371,1))</f>
@@ -31234,43 +31245,46 @@
       <c r="H371" s="35" t="n"/>
       <c r="I371" s="35" t="n"/>
     </row>
-    <row r="372" ht="62" customHeight="1">
-      <c r="A372" s="9" t="n"/>
-      <c r="B372" s="34" t="inlineStr">
-        <is>
-          <t>DOS PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C372" s="9" t="inlineStr"/>
-      <c r="D372" s="8">
-        <f>IF(COUNT(H372,I372)&lt;2,"",ROUND(H372*I372,2))</f>
-        <v/>
-      </c>
-      <c r="E372" s="25" t="n">
-        <v>9</v>
-      </c>
-      <c r="F372" s="28">
-        <f>IF(D372="","",ROUND(D372*E372,1))</f>
-        <v/>
-      </c>
+    <row r="372" ht="39.7" customHeight="1">
+      <c r="A372" s="16" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B372" s="33" t="inlineStr">
+        <is>
+          <t>INFILTRACION</t>
+        </is>
+      </c>
+      <c r="C372" s="9" t="n"/>
+      <c r="D372" s="16" t="inlineStr">
+        <is>
+          <t>VOLUMEN (m3)</t>
+        </is>
+      </c>
+      <c r="E372" s="9" t="n"/>
+      <c r="F372" s="9" t="n"/>
       <c r="G372" s="2" t="n"/>
-      <c r="H372" s="35" t="n"/>
-      <c r="I372" s="35" t="n"/>
-    </row>
-    <row r="373" ht="62" customHeight="1">
+      <c r="H372" s="2" t="n"/>
+      <c r="I372" s="2" t="n"/>
+    </row>
+    <row r="373" ht="39.7" customHeight="1">
       <c r="A373" s="9" t="n"/>
       <c r="B373" s="34" t="inlineStr">
         <is>
-          <t>TRES O MAS PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C373" s="9" t="inlineStr"/>
-      <c r="D373" s="8">
-        <f>IF(COUNT(H373,I373)&lt;2,"",ROUND(H373*I373,2))</f>
-        <v/>
+          <t>UNA PARED EXTERIOR</t>
+        </is>
+      </c>
+      <c r="C373" s="9" t="inlineStr">
+        <is>
+          <t>7.23 m2 x 3.00</t>
+        </is>
+      </c>
+      <c r="D373" s="8" t="n">
+        <v>21.69</v>
       </c>
       <c r="E373" s="25" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F373" s="28">
         <f>IF(D373="","",ROUND(D373*E373,1))</f>
@@ -31280,109 +31294,119 @@
       <c r="H373" s="35" t="n"/>
       <c r="I373" s="35" t="n"/>
     </row>
-    <row r="374" ht="70" customHeight="1">
-      <c r="A374" s="16" t="inlineStr">
+    <row r="374" ht="62" customHeight="1">
+      <c r="A374" s="9" t="n"/>
+      <c r="B374" s="34" t="inlineStr">
+        <is>
+          <t>DOS PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C374" s="9" t="inlineStr"/>
+      <c r="D374" s="8">
+        <f>IF(COUNT(H374,I374)&lt;2,"",ROUND(H374*I374,2))</f>
+        <v/>
+      </c>
+      <c r="E374" s="25" t="n">
+        <v>9</v>
+      </c>
+      <c r="F374" s="28">
+        <f>IF(D374="","",ROUND(D374*E374,1))</f>
+        <v/>
+      </c>
+      <c r="G374" s="2" t="n"/>
+      <c r="H374" s="35" t="n"/>
+      <c r="I374" s="35" t="n"/>
+    </row>
+    <row r="375" ht="62" customHeight="1">
+      <c r="A375" s="9" t="n"/>
+      <c r="B375" s="34" t="inlineStr">
+        <is>
+          <t>TRES O MAS PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C375" s="9" t="inlineStr"/>
+      <c r="D375" s="8">
+        <f>IF(COUNT(H375,I375)&lt;2,"",ROUND(H375*I375,2))</f>
+        <v/>
+      </c>
+      <c r="E375" s="25" t="n">
+        <v>12</v>
+      </c>
+      <c r="F375" s="28">
+        <f>IF(D375="","",ROUND(D375*E375,1))</f>
+        <v/>
+      </c>
+      <c r="G375" s="2" t="n"/>
+      <c r="H375" s="35" t="n"/>
+      <c r="I375" s="35" t="n"/>
+    </row>
+    <row r="376" ht="70" customHeight="1">
+      <c r="A376" s="16" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B374" s="33" t="inlineStr">
+      <c r="B376" s="33" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="C374" s="9" t="n"/>
-      <c r="D374" s="9" t="n"/>
-      <c r="E374" s="9" t="n"/>
-      <c r="F374" s="36">
-        <f>IF(F353="",0,F353)+IF(F355="",0,F355)+IF(F356="",0,F356)+IF(F357="",0,F357)+IF(F358="",0,F358)+IF(F359="",0,F359)+IF(F360="",0,F360)+IF(F361="",0,F361)+IF(F362="",0,F362)+IF(F364="",0,F364)+IF(F365="",0,F365)+IF(F366="",0,F366)+IF(F368="",0,F368)+IF(F369="",0,F369)+IF(F371="",0,F371)+IF(F372="",0,F372)+IF(F373="",0,F373)</f>
-        <v/>
-      </c>
-      <c r="G374" s="2" t="n"/>
-      <c r="H374" s="2" t="n"/>
-      <c r="I374" s="2" t="n"/>
-    </row>
-    <row r="375" ht="47" customHeight="1">
-      <c r="A375" s="16" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B375" s="33" t="inlineStr">
-        <is>
-          <t>PERDIDA TOTAL</t>
-        </is>
-      </c>
-      <c r="C375" s="9">
-        <f>TEXT(F374,"0.00")&amp;"  X  "&amp;Datos_balance!$B$4&amp;" (FI)  X  "&amp;Datos_balance!$B$5&amp;" (FO)  X  "&amp;Datos_balance!$B$6&amp;" (FZ)"</f>
-        <v/>
-      </c>
-      <c r="D375" s="2" t="n"/>
-      <c r="E375" s="2" t="n"/>
-      <c r="F375" s="36">
-        <f>ROUND(F374*Datos_balance!$B$4*Datos_balance!$B$5*Datos_balance!$B$6,1)</f>
-        <v/>
-      </c>
-      <c r="G375" s="2" t="n"/>
-      <c r="H375" s="2" t="n"/>
-      <c r="I375" s="2" t="n"/>
-    </row>
-    <row r="376">
-      <c r="A376" s="2" t="n"/>
-      <c r="B376" s="2" t="n"/>
-      <c r="C376" s="2" t="n"/>
-      <c r="D376" s="2" t="n"/>
-      <c r="E376" s="2" t="n"/>
-      <c r="F376" s="2" t="n"/>
+      <c r="C376" s="9" t="n"/>
+      <c r="D376" s="9" t="n"/>
+      <c r="E376" s="9" t="n"/>
+      <c r="F376" s="36">
+        <f>IF(F353="",0,F353)+IF(F355="",0,F355)+IF(F356="",0,F356)+IF(F357="",0,F357)+IF(F358="",0,F358)+IF(F359="",0,F359)+IF(F360="",0,F360)+IF(F361="",0,F361)+IF(F362="",0,F362)+IF(F363="",0,F363)+IF(F364="",0,F364)+IF(F366="",0,F366)+IF(F367="",0,F367)+IF(F368="",0,F368)+IF(F370="",0,F370)+IF(F371="",0,F371)+IF(F373="",0,F373)+IF(F374="",0,F374)+IF(F375="",0,F375)</f>
+        <v/>
+      </c>
       <c r="G376" s="2" t="n"/>
       <c r="H376" s="2" t="n"/>
       <c r="I376" s="2" t="n"/>
     </row>
-    <row r="377" ht="62" customHeight="1">
-      <c r="A377" s="9" t="n"/>
-      <c r="B377" s="10" t="inlineStr">
-        <is>
-          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
+    <row r="377" ht="47" customHeight="1">
+      <c r="A377" s="16" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B377" s="33" t="inlineStr">
+        <is>
+          <t>PERDIDA TOTAL</t>
         </is>
       </c>
       <c r="C377" s="9">
-        <f>TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2,"0")&amp;" - "&amp;TEXT(Datos_balance!$B$11,"0")&amp;" = "&amp;TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2-Datos_balance!$B$11,"0")&amp;" C"</f>
+        <f>TEXT(F376,"0.00")&amp;"  X  "&amp;Datos_balance!$B$4&amp;" (FI)  X  "&amp;Datos_balance!$B$5&amp;" (FO)  X  "&amp;Datos_balance!$B$6&amp;" (FZ)"</f>
         <v/>
       </c>
       <c r="D377" s="2" t="n"/>
       <c r="E377" s="2" t="n"/>
-      <c r="F377" s="9" t="n"/>
+      <c r="F377" s="36">
+        <f>ROUND(F376*Datos_balance!$B$4*Datos_balance!$B$5*Datos_balance!$B$6,1)</f>
+        <v/>
+      </c>
       <c r="G377" s="2" t="n"/>
       <c r="H377" s="2" t="n"/>
       <c r="I377" s="2" t="n"/>
     </row>
-    <row r="378" ht="39.7" customHeight="1">
-      <c r="A378" s="9" t="n"/>
-      <c r="B378" s="10" t="inlineStr">
-        <is>
-          <t>Kcal/h por elemento</t>
-        </is>
-      </c>
-      <c r="C378" s="8">
-        <f>ROUND(Datos_balance!$B$14*Datos_balance!$B$15,2)</f>
-        <v/>
-      </c>
+    <row r="378">
+      <c r="A378" s="2" t="n"/>
+      <c r="B378" s="2" t="n"/>
+      <c r="C378" s="2" t="n"/>
       <c r="D378" s="2" t="n"/>
       <c r="E378" s="2" t="n"/>
-      <c r="F378" s="9" t="n"/>
+      <c r="F378" s="2" t="n"/>
       <c r="G378" s="2" t="n"/>
       <c r="H378" s="2" t="n"/>
       <c r="I378" s="2" t="n"/>
     </row>
-    <row r="379" ht="39.7" customHeight="1">
+    <row r="379" ht="62" customHeight="1">
       <c r="A379" s="9" t="n"/>
       <c r="B379" s="10" t="inlineStr">
         <is>
-          <t>Elementos necesarios</t>
-        </is>
-      </c>
-      <c r="C379" s="25">
-        <f>ROUNDUP(F375/(Datos_balance!$B$14*Datos_balance!$B$15),0)</f>
+          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
+        </is>
+      </c>
+      <c r="C379" s="9">
+        <f>TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2,"0")&amp;" - "&amp;TEXT(Datos_balance!$B$11,"0")&amp;" = "&amp;TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2-Datos_balance!$B$11,"0")&amp;" C"</f>
         <v/>
       </c>
       <c r="D379" s="2" t="n"/>
@@ -31396,11 +31420,11 @@
       <c r="A380" s="9" t="n"/>
       <c r="B380" s="10" t="inlineStr">
         <is>
-          <t>Ancho del radiador (cm)</t>
-        </is>
-      </c>
-      <c r="C380" s="25">
-        <f>ROUNDUP(F375/(Datos_balance!$B$14*Datos_balance!$B$15),0)*Datos_balance!$B$16</f>
+          <t>Kcal/h por elemento</t>
+        </is>
+      </c>
+      <c r="C380" s="8">
+        <f>ROUND(Datos_balance!$B$14*Datos_balance!$B$15,2)</f>
         <v/>
       </c>
       <c r="D380" s="2" t="n"/>
@@ -31411,51 +31435,61 @@
       <c r="I380" s="2" t="n"/>
     </row>
     <row r="381" ht="39.7" customHeight="1">
-      <c r="A381" s="13" t="n"/>
-      <c r="B381" s="14" t="inlineStr">
-        <is>
-          <t>Radiador adoptado</t>
-        </is>
-      </c>
-      <c r="C381" s="13">
-        <f>Datos_balance!$B$13</f>
-        <v/>
-      </c>
-      <c r="D381" s="20" t="n"/>
-      <c r="E381" s="20" t="n"/>
-      <c r="F381" s="13" t="n"/>
+      <c r="A381" s="9" t="n"/>
+      <c r="B381" s="10" t="inlineStr">
+        <is>
+          <t>Elementos necesarios</t>
+        </is>
+      </c>
+      <c r="C381" s="25">
+        <f>ROUNDUP(F377/(Datos_balance!$B$14*Datos_balance!$B$15),0)</f>
+        <v/>
+      </c>
+      <c r="D381" s="2" t="n"/>
+      <c r="E381" s="2" t="n"/>
+      <c r="F381" s="9" t="n"/>
       <c r="G381" s="2" t="n"/>
       <c r="H381" s="2" t="n"/>
       <c r="I381" s="2" t="n"/>
     </row>
-    <row r="382">
-      <c r="A382" s="2" t="n"/>
-      <c r="B382" s="2" t="n"/>
-      <c r="C382" s="2" t="n"/>
+    <row r="382" ht="39.7" customHeight="1">
+      <c r="A382" s="9" t="n"/>
+      <c r="B382" s="10" t="inlineStr">
+        <is>
+          <t>Ancho del radiador (cm)</t>
+        </is>
+      </c>
+      <c r="C382" s="25">
+        <f>ROUNDUP(F377/(Datos_balance!$B$14*Datos_balance!$B$15),0)*Datos_balance!$B$16</f>
+        <v/>
+      </c>
       <c r="D382" s="2" t="n"/>
       <c r="E382" s="2" t="n"/>
-      <c r="F382" s="2" t="n"/>
+      <c r="F382" s="9" t="n"/>
       <c r="G382" s="2" t="n"/>
       <c r="H382" s="2" t="n"/>
       <c r="I382" s="2" t="n"/>
     </row>
-    <row r="383">
-      <c r="A383" s="2" t="n"/>
-      <c r="B383" s="2" t="n"/>
-      <c r="C383" s="2" t="n"/>
-      <c r="D383" s="2" t="n"/>
-      <c r="E383" s="2" t="n"/>
-      <c r="F383" s="2" t="n"/>
+    <row r="383" ht="39.7" customHeight="1">
+      <c r="A383" s="13" t="n"/>
+      <c r="B383" s="14" t="inlineStr">
+        <is>
+          <t>Radiador adoptado</t>
+        </is>
+      </c>
+      <c r="C383" s="13">
+        <f>Datos_balance!$B$13</f>
+        <v/>
+      </c>
+      <c r="D383" s="20" t="n"/>
+      <c r="E383" s="20" t="n"/>
+      <c r="F383" s="13" t="n"/>
       <c r="G383" s="2" t="n"/>
       <c r="H383" s="2" t="n"/>
       <c r="I383" s="2" t="n"/>
     </row>
-    <row r="384" ht="39.7" customHeight="1">
-      <c r="A384" s="5" t="inlineStr">
-        <is>
-          <t>LOCAL  17 - Bano   (PA)</t>
-        </is>
-      </c>
+    <row r="384">
+      <c r="A384" s="2" t="n"/>
       <c r="B384" s="2" t="n"/>
       <c r="C384" s="2" t="n"/>
       <c r="D384" s="2" t="n"/>
@@ -31465,99 +31499,76 @@
       <c r="H384" s="2" t="n"/>
       <c r="I384" s="2" t="n"/>
     </row>
-    <row r="385" ht="39.7" customHeight="1">
-      <c r="A385" s="3" t="inlineStr">
-        <is>
-          <t>Nro</t>
-        </is>
-      </c>
-      <c r="B385" s="3" t="inlineStr">
-        <is>
-          <t>DESCRIPCION</t>
-        </is>
-      </c>
-      <c r="C385" s="3" t="inlineStr">
-        <is>
-          <t>DIMENSIONES (m)</t>
-        </is>
-      </c>
-      <c r="D385" s="3" t="inlineStr">
-        <is>
-          <t>AREA (m2)</t>
-        </is>
-      </c>
-      <c r="E385" s="3" t="inlineStr">
-        <is>
-          <t>FACTOR</t>
-        </is>
-      </c>
-      <c r="F385" s="3" t="inlineStr">
-        <is>
-          <t>PERDIDA CALOR (Kcal/h)</t>
-        </is>
-      </c>
+    <row r="385">
+      <c r="A385" s="2" t="n"/>
+      <c r="B385" s="2" t="n"/>
+      <c r="C385" s="2" t="n"/>
+      <c r="D385" s="2" t="n"/>
+      <c r="E385" s="2" t="n"/>
+      <c r="F385" s="2" t="n"/>
       <c r="G385" s="2" t="n"/>
       <c r="H385" s="2" t="n"/>
       <c r="I385" s="2" t="n"/>
     </row>
     <row r="386" ht="39.7" customHeight="1">
-      <c r="A386" s="16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B386" s="33" t="inlineStr">
-        <is>
-          <t>VENTANA</t>
-        </is>
-      </c>
-      <c r="C386" s="9" t="n"/>
-      <c r="D386" s="9" t="n"/>
-      <c r="E386" s="9" t="n"/>
-      <c r="F386" s="9" t="n"/>
+      <c r="A386" s="5" t="inlineStr">
+        <is>
+          <t>LOCAL  17 - Bano   (PA)</t>
+        </is>
+      </c>
+      <c r="B386" s="2" t="n"/>
+      <c r="C386" s="2" t="n"/>
+      <c r="D386" s="2" t="n"/>
+      <c r="E386" s="2" t="n"/>
+      <c r="F386" s="2" t="n"/>
       <c r="G386" s="2" t="n"/>
       <c r="H386" s="2" t="n"/>
       <c r="I386" s="2" t="n"/>
     </row>
-    <row r="387" ht="62" customHeight="1">
-      <c r="A387" s="9" t="n"/>
-      <c r="B387" s="34" t="inlineStr">
-        <is>
-          <t>VA03</t>
-        </is>
-      </c>
-      <c r="C387" s="9">
-        <f>IF(COUNT(H387,I387)&lt;2,"",TEXT(H387,"0.00")&amp;" x "&amp;TEXT(I387,"0.00"))</f>
-        <v/>
-      </c>
-      <c r="D387" s="8">
-        <f>IF(COUNT(H387,I387)&lt;2,"",ROUND(H387*I387,2))</f>
-        <v/>
-      </c>
-      <c r="E387" s="25" t="n">
-        <v>60</v>
-      </c>
-      <c r="F387" s="28">
-        <f>IF(D387="","",ROUND(D387*E387,1))</f>
-        <v/>
+    <row r="387" ht="39.7" customHeight="1">
+      <c r="A387" s="3" t="inlineStr">
+        <is>
+          <t>Nro</t>
+        </is>
+      </c>
+      <c r="B387" s="3" t="inlineStr">
+        <is>
+          <t>DESCRIPCION</t>
+        </is>
+      </c>
+      <c r="C387" s="3" t="inlineStr">
+        <is>
+          <t>DIMENSIONES (m)</t>
+        </is>
+      </c>
+      <c r="D387" s="3" t="inlineStr">
+        <is>
+          <t>AREA (m2)</t>
+        </is>
+      </c>
+      <c r="E387" s="3" t="inlineStr">
+        <is>
+          <t>FACTOR</t>
+        </is>
+      </c>
+      <c r="F387" s="3" t="inlineStr">
+        <is>
+          <t>PERDIDA CALOR (Kcal/h)</t>
+        </is>
       </c>
       <c r="G387" s="2" t="n"/>
-      <c r="H387" s="35" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="I387" s="35" t="n">
-        <v>2.52</v>
-      </c>
+      <c r="H387" s="2" t="n"/>
+      <c r="I387" s="2" t="n"/>
     </row>
     <row r="388" ht="39.7" customHeight="1">
       <c r="A388" s="16" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B388" s="33" t="inlineStr">
         <is>
-          <t>PAREDES EXTERIORES</t>
+          <t>VENTANA</t>
         </is>
       </c>
       <c r="C388" s="9" t="n"/>
@@ -31572,7 +31583,7 @@
       <c r="A389" s="9" t="n"/>
       <c r="B389" s="34" t="inlineStr">
         <is>
-          <t>AISLADAS (    )</t>
+          <t>VA03</t>
         </is>
       </c>
       <c r="C389" s="9">
@@ -31584,41 +31595,38 @@
         <v/>
       </c>
       <c r="E389" s="25" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="F389" s="28">
         <f>IF(D389="","",ROUND(D389*E389,1))</f>
         <v/>
       </c>
       <c r="G389" s="2" t="n"/>
-      <c r="H389" s="35" t="n"/>
-      <c r="I389" s="35" t="n"/>
-    </row>
-    <row r="390" ht="62" customHeight="1">
-      <c r="A390" s="9" t="n"/>
-      <c r="B390" s="34" t="inlineStr">
-        <is>
-          <t>AISLADAS (    )</t>
-        </is>
-      </c>
-      <c r="C390" s="9">
-        <f>IF(COUNT(H390,I390)&lt;2,"",TEXT(H390,"0.00")&amp;" x "&amp;TEXT(I390,"0.00"))</f>
-        <v/>
-      </c>
-      <c r="D390" s="8">
-        <f>IF(COUNT(H390,I390)&lt;2,"",ROUND(H390*I390,2))</f>
-        <v/>
-      </c>
-      <c r="E390" s="25" t="n">
-        <v>20</v>
-      </c>
-      <c r="F390" s="28">
-        <f>IF(D390="","",ROUND(D390*E390,1))</f>
-        <v/>
-      </c>
+      <c r="H389" s="35" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I389" s="35" t="n">
+        <v>2.52</v>
+      </c>
+    </row>
+    <row r="390" ht="39.7" customHeight="1">
+      <c r="A390" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B390" s="33" t="inlineStr">
+        <is>
+          <t>PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C390" s="9" t="n"/>
+      <c r="D390" s="9" t="n"/>
+      <c r="E390" s="9" t="n"/>
+      <c r="F390" s="9" t="n"/>
       <c r="G390" s="2" t="n"/>
-      <c r="H390" s="35" t="n"/>
-      <c r="I390" s="35" t="n"/>
+      <c r="H390" s="2" t="n"/>
+      <c r="I390" s="2" t="n"/>
     </row>
     <row r="391" ht="62" customHeight="1">
       <c r="A391" s="9" t="n"/>
@@ -31676,7 +31684,7 @@
       <c r="A393" s="9" t="n"/>
       <c r="B393" s="34" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>AISLADAS (    )</t>
         </is>
       </c>
       <c r="C393" s="9">
@@ -31688,25 +31696,21 @@
         <v/>
       </c>
       <c r="E393" s="25" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F393" s="28">
         <f>IF(D393="","",ROUND(D393*E393,1))</f>
         <v/>
       </c>
       <c r="G393" s="2" t="n"/>
-      <c r="H393" s="35" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="I393" s="35" t="n">
-        <v>3</v>
-      </c>
+      <c r="H393" s="35" t="n"/>
+      <c r="I393" s="35" t="n"/>
     </row>
     <row r="394" ht="62" customHeight="1">
       <c r="A394" s="9" t="n"/>
       <c r="B394" s="34" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>AISLADAS (    )</t>
         </is>
       </c>
       <c r="C394" s="9">
@@ -31718,19 +31722,15 @@
         <v/>
       </c>
       <c r="E394" s="25" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F394" s="28">
         <f>IF(D394="","",ROUND(D394*E394,1))</f>
         <v/>
       </c>
       <c r="G394" s="2" t="n"/>
-      <c r="H394" s="35" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="I394" s="35" t="n">
-        <v>3</v>
-      </c>
+      <c r="H394" s="35" t="n"/>
+      <c r="I394" s="35" t="n"/>
     </row>
     <row r="395" ht="62" customHeight="1">
       <c r="A395" s="9" t="n"/>
@@ -31792,79 +31792,90 @@
         <v>3</v>
       </c>
     </row>
-    <row r="397" ht="39.7" customHeight="1">
-      <c r="A397" s="16" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B397" s="33" t="inlineStr">
-        <is>
-          <t>TECHOS O CIELORRASOS</t>
-        </is>
-      </c>
-      <c r="C397" s="9" t="n"/>
-      <c r="D397" s="9" t="n"/>
-      <c r="E397" s="9" t="n"/>
-      <c r="F397" s="9" t="n"/>
+    <row r="397" ht="62" customHeight="1">
+      <c r="A397" s="9" t="n"/>
+      <c r="B397" s="34" t="inlineStr">
+        <is>
+          <t>INTERIORES (    )</t>
+        </is>
+      </c>
+      <c r="C397" s="9">
+        <f>IF(COUNT(H397,I397)&lt;2,"",TEXT(H397,"0.00")&amp;" x "&amp;TEXT(I397,"0.00"))</f>
+        <v/>
+      </c>
+      <c r="D397" s="8">
+        <f>IF(COUNT(H397,I397)&lt;2,"",ROUND(H397*I397,2))</f>
+        <v/>
+      </c>
+      <c r="E397" s="25" t="n">
+        <v>25</v>
+      </c>
+      <c r="F397" s="28">
+        <f>IF(D397="","",ROUND(D397*E397,1))</f>
+        <v/>
+      </c>
       <c r="G397" s="2" t="n"/>
-      <c r="H397" s="2" t="n"/>
-      <c r="I397" s="2" t="n"/>
+      <c r="H397" s="35" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="I397" s="35" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="398" ht="62" customHeight="1">
       <c r="A398" s="9" t="n"/>
       <c r="B398" s="34" t="inlineStr">
         <is>
-          <t>TECHO NO AISLADO</t>
-        </is>
-      </c>
-      <c r="C398" s="9" t="inlineStr"/>
+          <t>INTERIORES (    )</t>
+        </is>
+      </c>
+      <c r="C398" s="9">
+        <f>IF(COUNT(H398,I398)&lt;2,"",TEXT(H398,"0.00")&amp;" x "&amp;TEXT(I398,"0.00"))</f>
+        <v/>
+      </c>
       <c r="D398" s="8">
         <f>IF(COUNT(H398,I398)&lt;2,"",ROUND(H398*I398,2))</f>
         <v/>
       </c>
       <c r="E398" s="25" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F398" s="28">
         <f>IF(D398="","",ROUND(D398*E398,1))</f>
         <v/>
       </c>
       <c r="G398" s="2" t="n"/>
-      <c r="H398" s="35" t="n"/>
-      <c r="I398" s="35" t="n"/>
+      <c r="H398" s="35" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="I398" s="35" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="399" ht="39.7" customHeight="1">
-      <c r="A399" s="9" t="n"/>
-      <c r="B399" s="34" t="inlineStr">
-        <is>
-          <t>TECHO AISLADO</t>
-        </is>
-      </c>
-      <c r="C399" s="9" t="inlineStr">
-        <is>
-          <t>por croquis</t>
-        </is>
-      </c>
-      <c r="D399" s="8" t="n">
-        <v>3.52</v>
-      </c>
-      <c r="E399" s="25" t="n">
-        <v>20</v>
-      </c>
-      <c r="F399" s="28">
-        <f>IF(D399="","",ROUND(D399*E399,1))</f>
-        <v/>
-      </c>
+      <c r="A399" s="16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B399" s="33" t="inlineStr">
+        <is>
+          <t>TECHOS O CIELORRASOS</t>
+        </is>
+      </c>
+      <c r="C399" s="9" t="n"/>
+      <c r="D399" s="9" t="n"/>
+      <c r="E399" s="9" t="n"/>
+      <c r="F399" s="9" t="n"/>
       <c r="G399" s="2" t="n"/>
-      <c r="H399" s="35" t="n"/>
-      <c r="I399" s="35" t="n"/>
+      <c r="H399" s="2" t="n"/>
+      <c r="I399" s="2" t="n"/>
     </row>
     <row r="400" ht="62" customHeight="1">
       <c r="A400" s="9" t="n"/>
       <c r="B400" s="34" t="inlineStr">
         <is>
-          <t>TECHO ENTREPISO</t>
+          <t>TECHO NO AISLADO</t>
         </is>
       </c>
       <c r="C400" s="9" t="inlineStr"/>
@@ -31873,7 +31884,7 @@
         <v/>
       </c>
       <c r="E400" s="25" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F400" s="28">
         <f>IF(D400="","",ROUND(D400*E400,1))</f>
@@ -31884,29 +31895,36 @@
       <c r="I400" s="35" t="n"/>
     </row>
     <row r="401" ht="39.7" customHeight="1">
-      <c r="A401" s="16" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B401" s="33" t="inlineStr">
-        <is>
-          <t>PISO</t>
-        </is>
-      </c>
-      <c r="C401" s="9" t="n"/>
-      <c r="D401" s="9" t="n"/>
-      <c r="E401" s="9" t="n"/>
-      <c r="F401" s="9" t="n"/>
+      <c r="A401" s="9" t="n"/>
+      <c r="B401" s="34" t="inlineStr">
+        <is>
+          <t>TECHO AISLADO</t>
+        </is>
+      </c>
+      <c r="C401" s="9" t="inlineStr">
+        <is>
+          <t>por croquis</t>
+        </is>
+      </c>
+      <c r="D401" s="8" t="n">
+        <v>3.52</v>
+      </c>
+      <c r="E401" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="F401" s="28">
+        <f>IF(D401="","",ROUND(D401*E401,1))</f>
+        <v/>
+      </c>
       <c r="G401" s="2" t="n"/>
-      <c r="H401" s="2" t="n"/>
-      <c r="I401" s="2" t="n"/>
+      <c r="H401" s="35" t="n"/>
+      <c r="I401" s="35" t="n"/>
     </row>
     <row r="402" ht="62" customHeight="1">
       <c r="A402" s="9" t="n"/>
       <c r="B402" s="34" t="inlineStr">
         <is>
-          <t>SOBRE TIERRA</t>
+          <t>TECHO ENTREPISO</t>
         </is>
       </c>
       <c r="C402" s="9" t="inlineStr"/>
@@ -31915,7 +31933,7 @@
         <v/>
       </c>
       <c r="E402" s="25" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F402" s="28">
         <f>IF(D402="","",ROUND(D402*E402,1))</f>
@@ -31926,71 +31944,64 @@
       <c r="I402" s="35" t="n"/>
     </row>
     <row r="403" ht="39.7" customHeight="1">
-      <c r="A403" s="9" t="n"/>
-      <c r="B403" s="34" t="inlineStr">
-        <is>
-          <t>SOBRE LOCAL OCUPADO</t>
-        </is>
-      </c>
-      <c r="C403" s="9" t="inlineStr">
-        <is>
-          <t>por croquis</t>
-        </is>
-      </c>
-      <c r="D403" s="8" t="n">
-        <v>3.52</v>
-      </c>
-      <c r="E403" s="25" t="n">
-        <v>15</v>
-      </c>
-      <c r="F403" s="28">
-        <f>IF(D403="","",ROUND(D403*E403,1))</f>
-        <v/>
-      </c>
+      <c r="A403" s="16" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B403" s="33" t="inlineStr">
+        <is>
+          <t>PISO</t>
+        </is>
+      </c>
+      <c r="C403" s="9" t="n"/>
+      <c r="D403" s="9" t="n"/>
+      <c r="E403" s="9" t="n"/>
+      <c r="F403" s="9" t="n"/>
       <c r="G403" s="2" t="n"/>
-      <c r="H403" s="35" t="n"/>
-      <c r="I403" s="35" t="n"/>
-    </row>
-    <row r="404" ht="39.7" customHeight="1">
-      <c r="A404" s="16" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B404" s="33" t="inlineStr">
-        <is>
-          <t>INFILTRACION</t>
-        </is>
-      </c>
-      <c r="C404" s="9" t="n"/>
-      <c r="D404" s="16" t="inlineStr">
-        <is>
-          <t>VOLUMEN (m3)</t>
-        </is>
-      </c>
-      <c r="E404" s="9" t="n"/>
-      <c r="F404" s="9" t="n"/>
+      <c r="H403" s="2" t="n"/>
+      <c r="I403" s="2" t="n"/>
+    </row>
+    <row r="404" ht="62" customHeight="1">
+      <c r="A404" s="9" t="n"/>
+      <c r="B404" s="34" t="inlineStr">
+        <is>
+          <t>SOBRE TIERRA</t>
+        </is>
+      </c>
+      <c r="C404" s="9" t="inlineStr"/>
+      <c r="D404" s="8">
+        <f>IF(COUNT(H404,I404)&lt;2,"",ROUND(H404*I404,2))</f>
+        <v/>
+      </c>
+      <c r="E404" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="F404" s="28">
+        <f>IF(D404="","",ROUND(D404*E404,1))</f>
+        <v/>
+      </c>
       <c r="G404" s="2" t="n"/>
-      <c r="H404" s="2" t="n"/>
-      <c r="I404" s="2" t="n"/>
+      <c r="H404" s="35" t="n"/>
+      <c r="I404" s="35" t="n"/>
     </row>
     <row r="405" ht="39.7" customHeight="1">
       <c r="A405" s="9" t="n"/>
       <c r="B405" s="34" t="inlineStr">
         <is>
-          <t>UNA PARED EXTERIOR</t>
+          <t>SOBRE LOCAL OCUPADO</t>
         </is>
       </c>
       <c r="C405" s="9" t="inlineStr">
         <is>
-          <t>3.52 m2 x 3.00</t>
+          <t>por croquis</t>
         </is>
       </c>
       <c r="D405" s="8" t="n">
-        <v>10.56</v>
+        <v>3.52</v>
       </c>
       <c r="E405" s="25" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="F405" s="28">
         <f>IF(D405="","",ROUND(D405*E405,1))</f>
@@ -32000,43 +32011,46 @@
       <c r="H405" s="35" t="n"/>
       <c r="I405" s="35" t="n"/>
     </row>
-    <row r="406" ht="62" customHeight="1">
-      <c r="A406" s="9" t="n"/>
-      <c r="B406" s="34" t="inlineStr">
-        <is>
-          <t>DOS PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C406" s="9" t="inlineStr"/>
-      <c r="D406" s="8">
-        <f>IF(COUNT(H406,I406)&lt;2,"",ROUND(H406*I406,2))</f>
-        <v/>
-      </c>
-      <c r="E406" s="25" t="n">
-        <v>9</v>
-      </c>
-      <c r="F406" s="28">
-        <f>IF(D406="","",ROUND(D406*E406,1))</f>
-        <v/>
-      </c>
+    <row r="406" ht="39.7" customHeight="1">
+      <c r="A406" s="16" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B406" s="33" t="inlineStr">
+        <is>
+          <t>INFILTRACION</t>
+        </is>
+      </c>
+      <c r="C406" s="9" t="n"/>
+      <c r="D406" s="16" t="inlineStr">
+        <is>
+          <t>VOLUMEN (m3)</t>
+        </is>
+      </c>
+      <c r="E406" s="9" t="n"/>
+      <c r="F406" s="9" t="n"/>
       <c r="G406" s="2" t="n"/>
-      <c r="H406" s="35" t="n"/>
-      <c r="I406" s="35" t="n"/>
-    </row>
-    <row r="407" ht="62" customHeight="1">
+      <c r="H406" s="2" t="n"/>
+      <c r="I406" s="2" t="n"/>
+    </row>
+    <row r="407" ht="39.7" customHeight="1">
       <c r="A407" s="9" t="n"/>
       <c r="B407" s="34" t="inlineStr">
         <is>
-          <t>TRES O MAS PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C407" s="9" t="inlineStr"/>
-      <c r="D407" s="8">
-        <f>IF(COUNT(H407,I407)&lt;2,"",ROUND(H407*I407,2))</f>
-        <v/>
+          <t>UNA PARED EXTERIOR</t>
+        </is>
+      </c>
+      <c r="C407" s="9" t="inlineStr">
+        <is>
+          <t>3.52 m2 x 3.00</t>
+        </is>
+      </c>
+      <c r="D407" s="8" t="n">
+        <v>10.56</v>
       </c>
       <c r="E407" s="25" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F407" s="28">
         <f>IF(D407="","",ROUND(D407*E407,1))</f>
@@ -32046,109 +32060,119 @@
       <c r="H407" s="35" t="n"/>
       <c r="I407" s="35" t="n"/>
     </row>
-    <row r="408" ht="70" customHeight="1">
-      <c r="A408" s="16" t="inlineStr">
+    <row r="408" ht="62" customHeight="1">
+      <c r="A408" s="9" t="n"/>
+      <c r="B408" s="34" t="inlineStr">
+        <is>
+          <t>DOS PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C408" s="9" t="inlineStr"/>
+      <c r="D408" s="8">
+        <f>IF(COUNT(H408,I408)&lt;2,"",ROUND(H408*I408,2))</f>
+        <v/>
+      </c>
+      <c r="E408" s="25" t="n">
+        <v>9</v>
+      </c>
+      <c r="F408" s="28">
+        <f>IF(D408="","",ROUND(D408*E408,1))</f>
+        <v/>
+      </c>
+      <c r="G408" s="2" t="n"/>
+      <c r="H408" s="35" t="n"/>
+      <c r="I408" s="35" t="n"/>
+    </row>
+    <row r="409" ht="62" customHeight="1">
+      <c r="A409" s="9" t="n"/>
+      <c r="B409" s="34" t="inlineStr">
+        <is>
+          <t>TRES O MAS PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C409" s="9" t="inlineStr"/>
+      <c r="D409" s="8">
+        <f>IF(COUNT(H409,I409)&lt;2,"",ROUND(H409*I409,2))</f>
+        <v/>
+      </c>
+      <c r="E409" s="25" t="n">
+        <v>12</v>
+      </c>
+      <c r="F409" s="28">
+        <f>IF(D409="","",ROUND(D409*E409,1))</f>
+        <v/>
+      </c>
+      <c r="G409" s="2" t="n"/>
+      <c r="H409" s="35" t="n"/>
+      <c r="I409" s="35" t="n"/>
+    </row>
+    <row r="410" ht="70" customHeight="1">
+      <c r="A410" s="16" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B408" s="33" t="inlineStr">
+      <c r="B410" s="33" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="C408" s="9" t="n"/>
-      <c r="D408" s="9" t="n"/>
-      <c r="E408" s="9" t="n"/>
-      <c r="F408" s="36">
-        <f>IF(F387="",0,F387)+IF(F389="",0,F389)+IF(F390="",0,F390)+IF(F391="",0,F391)+IF(F392="",0,F392)+IF(F393="",0,F393)+IF(F394="",0,F394)+IF(F395="",0,F395)+IF(F396="",0,F396)+IF(F398="",0,F398)+IF(F399="",0,F399)+IF(F400="",0,F400)+IF(F402="",0,F402)+IF(F403="",0,F403)+IF(F405="",0,F405)+IF(F406="",0,F406)+IF(F407="",0,F407)</f>
-        <v/>
-      </c>
-      <c r="G408" s="2" t="n"/>
-      <c r="H408" s="2" t="n"/>
-      <c r="I408" s="2" t="n"/>
-    </row>
-    <row r="409" ht="47" customHeight="1">
-      <c r="A409" s="16" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B409" s="33" t="inlineStr">
-        <is>
-          <t>PERDIDA TOTAL</t>
-        </is>
-      </c>
-      <c r="C409" s="9">
-        <f>TEXT(F408,"0.00")&amp;"  X  "&amp;Datos_balance!$B$4&amp;" (FI)  X  "&amp;Datos_balance!$B$5&amp;" (FO)  X  "&amp;Datos_balance!$B$6&amp;" (FZ)"</f>
-        <v/>
-      </c>
-      <c r="D409" s="2" t="n"/>
-      <c r="E409" s="2" t="n"/>
-      <c r="F409" s="36">
-        <f>ROUND(F408*Datos_balance!$B$4*Datos_balance!$B$5*Datos_balance!$B$6,1)</f>
-        <v/>
-      </c>
-      <c r="G409" s="2" t="n"/>
-      <c r="H409" s="2" t="n"/>
-      <c r="I409" s="2" t="n"/>
-    </row>
-    <row r="410">
-      <c r="A410" s="2" t="n"/>
-      <c r="B410" s="2" t="n"/>
-      <c r="C410" s="2" t="n"/>
-      <c r="D410" s="2" t="n"/>
-      <c r="E410" s="2" t="n"/>
-      <c r="F410" s="2" t="n"/>
+      <c r="C410" s="9" t="n"/>
+      <c r="D410" s="9" t="n"/>
+      <c r="E410" s="9" t="n"/>
+      <c r="F410" s="36">
+        <f>IF(F389="",0,F389)+IF(F391="",0,F391)+IF(F392="",0,F392)+IF(F393="",0,F393)+IF(F394="",0,F394)+IF(F395="",0,F395)+IF(F396="",0,F396)+IF(F397="",0,F397)+IF(F398="",0,F398)+IF(F400="",0,F400)+IF(F401="",0,F401)+IF(F402="",0,F402)+IF(F404="",0,F404)+IF(F405="",0,F405)+IF(F407="",0,F407)+IF(F408="",0,F408)+IF(F409="",0,F409)</f>
+        <v/>
+      </c>
       <c r="G410" s="2" t="n"/>
       <c r="H410" s="2" t="n"/>
       <c r="I410" s="2" t="n"/>
     </row>
-    <row r="411" ht="62" customHeight="1">
-      <c r="A411" s="9" t="n"/>
-      <c r="B411" s="10" t="inlineStr">
-        <is>
-          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
+    <row r="411" ht="47" customHeight="1">
+      <c r="A411" s="16" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B411" s="33" t="inlineStr">
+        <is>
+          <t>PERDIDA TOTAL</t>
         </is>
       </c>
       <c r="C411" s="9">
-        <f>TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2,"0")&amp;" - "&amp;TEXT(Datos_balance!$B$11,"0")&amp;" = "&amp;TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2-Datos_balance!$B$11,"0")&amp;" C"</f>
+        <f>TEXT(F410,"0.00")&amp;"  X  "&amp;Datos_balance!$B$4&amp;" (FI)  X  "&amp;Datos_balance!$B$5&amp;" (FO)  X  "&amp;Datos_balance!$B$6&amp;" (FZ)"</f>
         <v/>
       </c>
       <c r="D411" s="2" t="n"/>
       <c r="E411" s="2" t="n"/>
-      <c r="F411" s="9" t="n"/>
+      <c r="F411" s="36">
+        <f>ROUND(F410*Datos_balance!$B$4*Datos_balance!$B$5*Datos_balance!$B$6,1)</f>
+        <v/>
+      </c>
       <c r="G411" s="2" t="n"/>
       <c r="H411" s="2" t="n"/>
       <c r="I411" s="2" t="n"/>
     </row>
-    <row r="412" ht="39.7" customHeight="1">
-      <c r="A412" s="9" t="n"/>
-      <c r="B412" s="10" t="inlineStr">
-        <is>
-          <t>Kcal/h del toallero Scala/Domino 80</t>
-        </is>
-      </c>
-      <c r="C412" s="25">
-        <f>ROUND(Datos_balance!$B$18*Datos_balance!$B$15,0)</f>
-        <v/>
-      </c>
+    <row r="412">
+      <c r="A412" s="2" t="n"/>
+      <c r="B412" s="2" t="n"/>
+      <c r="C412" s="2" t="n"/>
       <c r="D412" s="2" t="n"/>
       <c r="E412" s="2" t="n"/>
-      <c r="F412" s="9" t="n"/>
+      <c r="F412" s="2" t="n"/>
       <c r="G412" s="2" t="n"/>
       <c r="H412" s="2" t="n"/>
       <c r="I412" s="2" t="n"/>
     </row>
-    <row r="413" ht="39.7" customHeight="1">
+    <row r="413" ht="62" customHeight="1">
       <c r="A413" s="9" t="n"/>
       <c r="B413" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h del toallero Scala/Domino 150</t>
-        </is>
-      </c>
-      <c r="C413" s="25">
-        <f>ROUND(Datos_balance!$B$19*Datos_balance!$B$15,0)</f>
+          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
+        </is>
+      </c>
+      <c r="C413" s="9">
+        <f>TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2,"0")&amp;" - "&amp;TEXT(Datos_balance!$B$11,"0")&amp;" = "&amp;TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2-Datos_balance!$B$11,"0")&amp;" C"</f>
         <v/>
       </c>
       <c r="D413" s="2" t="n"/>
@@ -32158,15 +32182,15 @@
       <c r="H413" s="2" t="n"/>
       <c r="I413" s="2" t="n"/>
     </row>
-    <row r="414" ht="47" customHeight="1">
+    <row r="414" ht="39.7" customHeight="1">
       <c r="A414" s="9" t="n"/>
       <c r="B414" s="10" t="inlineStr">
         <is>
-          <t>Toalleros necesarios</t>
+          <t>Kcal/h del toallero Scala/Domino 80</t>
         </is>
       </c>
       <c r="C414" s="25">
-        <f>IF(F409&lt;=Datos_balance!$B$18*Datos_balance!$B$15,1,ROUNDUP(F409/(Datos_balance!$B$19*Datos_balance!$B$15),0))</f>
+        <f>ROUND(Datos_balance!$B$18*Datos_balance!$B$15,0)</f>
         <v/>
       </c>
       <c r="D414" s="2" t="n"/>
@@ -32176,23 +32200,59 @@
       <c r="H414" s="2" t="n"/>
       <c r="I414" s="2" t="n"/>
     </row>
-    <row r="415" ht="47" customHeight="1">
-      <c r="A415" s="13" t="n"/>
-      <c r="B415" s="14" t="inlineStr">
-        <is>
-          <t>Toallero adoptado</t>
-        </is>
-      </c>
-      <c r="C415" s="13">
-        <f>IF(F409&lt;=Datos_balance!$B$18*Datos_balance!$B$15,"Peisa Scala / Domino 80  (500 x 800 mm)","Peisa Scala / Domino 150  (500 x 1500 mm)")</f>
-        <v/>
-      </c>
-      <c r="D415" s="20" t="n"/>
-      <c r="E415" s="20" t="n"/>
-      <c r="F415" s="13" t="n"/>
+    <row r="415" ht="39.7" customHeight="1">
+      <c r="A415" s="9" t="n"/>
+      <c r="B415" s="10" t="inlineStr">
+        <is>
+          <t>Kcal/h del toallero Scala/Domino 150</t>
+        </is>
+      </c>
+      <c r="C415" s="25">
+        <f>ROUND(Datos_balance!$B$19*Datos_balance!$B$15,0)</f>
+        <v/>
+      </c>
+      <c r="D415" s="2" t="n"/>
+      <c r="E415" s="2" t="n"/>
+      <c r="F415" s="9" t="n"/>
       <c r="G415" s="2" t="n"/>
       <c r="H415" s="2" t="n"/>
       <c r="I415" s="2" t="n"/>
+    </row>
+    <row r="416" ht="47" customHeight="1">
+      <c r="A416" s="9" t="n"/>
+      <c r="B416" s="10" t="inlineStr">
+        <is>
+          <t>Toalleros necesarios</t>
+        </is>
+      </c>
+      <c r="C416" s="25">
+        <f>IF(F411&lt;=Datos_balance!$B$18*Datos_balance!$B$15,1,ROUNDUP(F411/(Datos_balance!$B$19*Datos_balance!$B$15),0))</f>
+        <v/>
+      </c>
+      <c r="D416" s="2" t="n"/>
+      <c r="E416" s="2" t="n"/>
+      <c r="F416" s="9" t="n"/>
+      <c r="G416" s="2" t="n"/>
+      <c r="H416" s="2" t="n"/>
+      <c r="I416" s="2" t="n"/>
+    </row>
+    <row r="417" ht="47" customHeight="1">
+      <c r="A417" s="13" t="n"/>
+      <c r="B417" s="14" t="inlineStr">
+        <is>
+          <t>Toallero adoptado</t>
+        </is>
+      </c>
+      <c r="C417" s="13">
+        <f>IF(F411&lt;=Datos_balance!$B$18*Datos_balance!$B$15,"Peisa Scala / Domino 80  (500 x 800 mm)","Peisa Scala / Domino 150  (500 x 1500 mm)")</f>
+        <v/>
+      </c>
+      <c r="D417" s="20" t="n"/>
+      <c r="E417" s="20" t="n"/>
+      <c r="F417" s="13" t="n"/>
+      <c r="G417" s="2" t="n"/>
+      <c r="H417" s="2" t="n"/>
+      <c r="I417" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="85">
@@ -32204,29 +32264,28 @@
     <mergeCell ref="C413:E413"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="C379:E379"/>
-    <mergeCell ref="A384:F384"/>
     <mergeCell ref="C415:E415"/>
     <mergeCell ref="C71:E71"/>
     <mergeCell ref="C241:E241"/>
     <mergeCell ref="C347:E347"/>
+    <mergeCell ref="A386:F386"/>
     <mergeCell ref="C243:E243"/>
     <mergeCell ref="C140:E140"/>
     <mergeCell ref="A40:F40"/>
     <mergeCell ref="C34:E34"/>
-    <mergeCell ref="C375:E375"/>
     <mergeCell ref="C275:E275"/>
     <mergeCell ref="C344:E344"/>
     <mergeCell ref="C206:E206"/>
     <mergeCell ref="C377:E377"/>
     <mergeCell ref="A315:F315"/>
+    <mergeCell ref="C417:E417"/>
     <mergeCell ref="C309:E309"/>
     <mergeCell ref="C103:E103"/>
     <mergeCell ref="A212:F212"/>
     <mergeCell ref="C205:E205"/>
+    <mergeCell ref="C383:E383"/>
     <mergeCell ref="C311:E311"/>
-    <mergeCell ref="C412:E412"/>
     <mergeCell ref="C169:E169"/>
-    <mergeCell ref="C409:E409"/>
     <mergeCell ref="C380:E380"/>
     <mergeCell ref="C70:E70"/>
     <mergeCell ref="C272:E272"/>
@@ -32240,6 +32299,7 @@
     <mergeCell ref="C104:E104"/>
     <mergeCell ref="A178:F178"/>
     <mergeCell ref="C35:E35"/>
+    <mergeCell ref="C416:E416"/>
     <mergeCell ref="C173:E173"/>
     <mergeCell ref="C276:E276"/>
     <mergeCell ref="C36:E36"/>
@@ -32254,7 +32314,6 @@
     <mergeCell ref="C136:E136"/>
     <mergeCell ref="A143:F143"/>
     <mergeCell ref="A350:F350"/>
-    <mergeCell ref="C378:E378"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="C172:E172"/>
     <mergeCell ref="A281:F281"/>
@@ -32263,6 +32322,7 @@
     <mergeCell ref="C137:E137"/>
     <mergeCell ref="C134:E134"/>
     <mergeCell ref="A246:F246"/>
+    <mergeCell ref="C382:E382"/>
     <mergeCell ref="C277:E277"/>
     <mergeCell ref="C139:E139"/>
     <mergeCell ref="C105:E105"/>

</xml_diff>

<commit_message>
Balance termico: sacar el antebano, no se calefacciona
Quedan 11 locales. En planta alta se calefaccionan el bano y los dos
dormitorios; el play room sigue cargado, pendiente de confirmar.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -42,7 +42,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="5">'Vigas de fundacion'!$A$1:$X$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Pilotes y cabezales'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Tabiques'!$1:$3</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="8">'Balance termico'!$A$1:$F$420</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="8">'Balance termico'!$A$1:$F$386</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22778,7 +22778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I417"/>
+  <dimension ref="A1:I383"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.1" customWidth="1" min="1" max="1"/>
@@ -30751,7 +30751,7 @@
     <row r="352" ht="39.7" customHeight="1">
       <c r="A352" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  16 - Antebano   (PA)</t>
+          <t>LOCAL  17 - Bano   (PA)</t>
         </is>
       </c>
       <c r="B352" s="2" t="n"/>
@@ -30821,7 +30821,7 @@
       <c r="A355" s="9" t="n"/>
       <c r="B355" s="34" t="inlineStr">
         <is>
-          <t>(sin aberturas)</t>
+          <t>VA03</t>
         </is>
       </c>
       <c r="C355" s="9">
@@ -30840,8 +30840,12 @@
         <v/>
       </c>
       <c r="G355" s="2" t="n"/>
-      <c r="H355" s="35" t="n"/>
-      <c r="I355" s="35" t="n"/>
+      <c r="H355" s="35" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I355" s="35" t="n">
+        <v>2.52</v>
+      </c>
     </row>
     <row r="356" ht="39.7" customHeight="1">
       <c r="A356" s="16" t="inlineStr">
@@ -30990,7 +30994,7 @@
       </c>
       <c r="G361" s="2" t="n"/>
       <c r="H361" s="35" t="n">
-        <v>3.9</v>
+        <v>2.2</v>
       </c>
       <c r="I361" s="35" t="n">
         <v>3</v>
@@ -31020,7 +31024,7 @@
       </c>
       <c r="G362" s="2" t="n"/>
       <c r="H362" s="35" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="I362" s="35" t="n">
         <v>3</v>
@@ -31050,7 +31054,7 @@
       </c>
       <c r="G363" s="2" t="n"/>
       <c r="H363" s="35" t="n">
-        <v>3.9</v>
+        <v>2.2</v>
       </c>
       <c r="I363" s="35" t="n">
         <v>3</v>
@@ -31080,7 +31084,7 @@
       </c>
       <c r="G364" s="2" t="n"/>
       <c r="H364" s="35" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="I364" s="35" t="n">
         <v>3</v>
@@ -31141,7 +31145,7 @@
         </is>
       </c>
       <c r="D367" s="8" t="n">
-        <v>5.85</v>
+        <v>3.52</v>
       </c>
       <c r="E367" s="25" t="n">
         <v>20</v>
@@ -31232,7 +31236,7 @@
         </is>
       </c>
       <c r="D371" s="8" t="n">
-        <v>5.85</v>
+        <v>3.52</v>
       </c>
       <c r="E371" s="25" t="n">
         <v>15</v>
@@ -31277,11 +31281,11 @@
       </c>
       <c r="C373" s="9" t="inlineStr">
         <is>
-          <t>5.85 m2 x 3.00</t>
+          <t>3.52 m2 x 3.00</t>
         </is>
       </c>
       <c r="D373" s="8" t="n">
-        <v>17.55</v>
+        <v>10.56</v>
       </c>
       <c r="E373" s="25" t="n">
         <v>6</v>
@@ -31420,11 +31424,11 @@
       <c r="A380" s="9" t="n"/>
       <c r="B380" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h por elemento</t>
-        </is>
-      </c>
-      <c r="C380" s="8">
-        <f>ROUND(Datos_balance!$B$14*Datos_balance!$B$15,2)</f>
+          <t>Kcal/h del toallero Scala/Domino 80</t>
+        </is>
+      </c>
+      <c r="C380" s="25">
+        <f>ROUND(Datos_balance!$B$18*Datos_balance!$B$15,0)</f>
         <v/>
       </c>
       <c r="D380" s="2" t="n"/>
@@ -31438,11 +31442,11 @@
       <c r="A381" s="9" t="n"/>
       <c r="B381" s="10" t="inlineStr">
         <is>
-          <t>Elementos necesarios</t>
+          <t>Kcal/h del toallero Scala/Domino 150</t>
         </is>
       </c>
       <c r="C381" s="25">
-        <f>ROUNDUP(F377/(Datos_balance!$B$14*Datos_balance!$B$15),0)</f>
+        <f>ROUND(Datos_balance!$B$19*Datos_balance!$B$15,0)</f>
         <v/>
       </c>
       <c r="D381" s="2" t="n"/>
@@ -31452,15 +31456,15 @@
       <c r="H381" s="2" t="n"/>
       <c r="I381" s="2" t="n"/>
     </row>
-    <row r="382" ht="39.7" customHeight="1">
+    <row r="382" ht="47" customHeight="1">
       <c r="A382" s="9" t="n"/>
       <c r="B382" s="10" t="inlineStr">
         <is>
-          <t>Ancho del radiador (cm)</t>
+          <t>Toalleros necesarios</t>
         </is>
       </c>
       <c r="C382" s="25">
-        <f>ROUNDUP(F377/(Datos_balance!$B$14*Datos_balance!$B$15),0)*Datos_balance!$B$16</f>
+        <f>IF(F377&lt;=Datos_balance!$B$18*Datos_balance!$B$15,1,ROUNDUP(F377/(Datos_balance!$B$19*Datos_balance!$B$15),0))</f>
         <v/>
       </c>
       <c r="D382" s="2" t="n"/>
@@ -31470,15 +31474,15 @@
       <c r="H382" s="2" t="n"/>
       <c r="I382" s="2" t="n"/>
     </row>
-    <row r="383" ht="39.7" customHeight="1">
+    <row r="383" ht="47" customHeight="1">
       <c r="A383" s="13" t="n"/>
       <c r="B383" s="14" t="inlineStr">
         <is>
-          <t>Radiador adoptado</t>
+          <t>Toallero adoptado</t>
         </is>
       </c>
       <c r="C383" s="13">
-        <f>Datos_balance!$B$13</f>
+        <f>IF(F377&lt;=Datos_balance!$B$18*Datos_balance!$B$15,"Peisa Scala / Domino 80  (500 x 800 mm)","Peisa Scala / Domino 150  (500 x 1500 mm)")</f>
         <v/>
       </c>
       <c r="D383" s="20" t="n"/>
@@ -31488,774 +31492,8 @@
       <c r="H383" s="2" t="n"/>
       <c r="I383" s="2" t="n"/>
     </row>
-    <row r="384">
-      <c r="A384" s="2" t="n"/>
-      <c r="B384" s="2" t="n"/>
-      <c r="C384" s="2" t="n"/>
-      <c r="D384" s="2" t="n"/>
-      <c r="E384" s="2" t="n"/>
-      <c r="F384" s="2" t="n"/>
-      <c r="G384" s="2" t="n"/>
-      <c r="H384" s="2" t="n"/>
-      <c r="I384" s="2" t="n"/>
-    </row>
-    <row r="385">
-      <c r="A385" s="2" t="n"/>
-      <c r="B385" s="2" t="n"/>
-      <c r="C385" s="2" t="n"/>
-      <c r="D385" s="2" t="n"/>
-      <c r="E385" s="2" t="n"/>
-      <c r="F385" s="2" t="n"/>
-      <c r="G385" s="2" t="n"/>
-      <c r="H385" s="2" t="n"/>
-      <c r="I385" s="2" t="n"/>
-    </row>
-    <row r="386" ht="39.7" customHeight="1">
-      <c r="A386" s="5" t="inlineStr">
-        <is>
-          <t>LOCAL  17 - Bano   (PA)</t>
-        </is>
-      </c>
-      <c r="B386" s="2" t="n"/>
-      <c r="C386" s="2" t="n"/>
-      <c r="D386" s="2" t="n"/>
-      <c r="E386" s="2" t="n"/>
-      <c r="F386" s="2" t="n"/>
-      <c r="G386" s="2" t="n"/>
-      <c r="H386" s="2" t="n"/>
-      <c r="I386" s="2" t="n"/>
-    </row>
-    <row r="387" ht="39.7" customHeight="1">
-      <c r="A387" s="3" t="inlineStr">
-        <is>
-          <t>Nro</t>
-        </is>
-      </c>
-      <c r="B387" s="3" t="inlineStr">
-        <is>
-          <t>DESCRIPCION</t>
-        </is>
-      </c>
-      <c r="C387" s="3" t="inlineStr">
-        <is>
-          <t>DIMENSIONES (m)</t>
-        </is>
-      </c>
-      <c r="D387" s="3" t="inlineStr">
-        <is>
-          <t>AREA (m2)</t>
-        </is>
-      </c>
-      <c r="E387" s="3" t="inlineStr">
-        <is>
-          <t>FACTOR</t>
-        </is>
-      </c>
-      <c r="F387" s="3" t="inlineStr">
-        <is>
-          <t>PERDIDA CALOR (Kcal/h)</t>
-        </is>
-      </c>
-      <c r="G387" s="2" t="n"/>
-      <c r="H387" s="2" t="n"/>
-      <c r="I387" s="2" t="n"/>
-    </row>
-    <row r="388" ht="39.7" customHeight="1">
-      <c r="A388" s="16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B388" s="33" t="inlineStr">
-        <is>
-          <t>VENTANA</t>
-        </is>
-      </c>
-      <c r="C388" s="9" t="n"/>
-      <c r="D388" s="9" t="n"/>
-      <c r="E388" s="9" t="n"/>
-      <c r="F388" s="9" t="n"/>
-      <c r="G388" s="2" t="n"/>
-      <c r="H388" s="2" t="n"/>
-      <c r="I388" s="2" t="n"/>
-    </row>
-    <row r="389" ht="62" customHeight="1">
-      <c r="A389" s="9" t="n"/>
-      <c r="B389" s="34" t="inlineStr">
-        <is>
-          <t>VA03</t>
-        </is>
-      </c>
-      <c r="C389" s="9">
-        <f>IF(COUNT(H389,I389)&lt;2,"",TEXT(H389,"0.00")&amp;" x "&amp;TEXT(I389,"0.00"))</f>
-        <v/>
-      </c>
-      <c r="D389" s="8">
-        <f>IF(COUNT(H389,I389)&lt;2,"",ROUND(H389*I389,2))</f>
-        <v/>
-      </c>
-      <c r="E389" s="25" t="n">
-        <v>60</v>
-      </c>
-      <c r="F389" s="28">
-        <f>IF(D389="","",ROUND(D389*E389,1))</f>
-        <v/>
-      </c>
-      <c r="G389" s="2" t="n"/>
-      <c r="H389" s="35" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="I389" s="35" t="n">
-        <v>2.52</v>
-      </c>
-    </row>
-    <row r="390" ht="39.7" customHeight="1">
-      <c r="A390" s="16" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B390" s="33" t="inlineStr">
-        <is>
-          <t>PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C390" s="9" t="n"/>
-      <c r="D390" s="9" t="n"/>
-      <c r="E390" s="9" t="n"/>
-      <c r="F390" s="9" t="n"/>
-      <c r="G390" s="2" t="n"/>
-      <c r="H390" s="2" t="n"/>
-      <c r="I390" s="2" t="n"/>
-    </row>
-    <row r="391" ht="62" customHeight="1">
-      <c r="A391" s="9" t="n"/>
-      <c r="B391" s="34" t="inlineStr">
-        <is>
-          <t>AISLADAS (    )</t>
-        </is>
-      </c>
-      <c r="C391" s="9">
-        <f>IF(COUNT(H391,I391)&lt;2,"",TEXT(H391,"0.00")&amp;" x "&amp;TEXT(I391,"0.00"))</f>
-        <v/>
-      </c>
-      <c r="D391" s="8">
-        <f>IF(COUNT(H391,I391)&lt;2,"",ROUND(H391*I391,2))</f>
-        <v/>
-      </c>
-      <c r="E391" s="25" t="n">
-        <v>20</v>
-      </c>
-      <c r="F391" s="28">
-        <f>IF(D391="","",ROUND(D391*E391,1))</f>
-        <v/>
-      </c>
-      <c r="G391" s="2" t="n"/>
-      <c r="H391" s="35" t="n"/>
-      <c r="I391" s="35" t="n"/>
-    </row>
-    <row r="392" ht="62" customHeight="1">
-      <c r="A392" s="9" t="n"/>
-      <c r="B392" s="34" t="inlineStr">
-        <is>
-          <t>AISLADAS (    )</t>
-        </is>
-      </c>
-      <c r="C392" s="9">
-        <f>IF(COUNT(H392,I392)&lt;2,"",TEXT(H392,"0.00")&amp;" x "&amp;TEXT(I392,"0.00"))</f>
-        <v/>
-      </c>
-      <c r="D392" s="8">
-        <f>IF(COUNT(H392,I392)&lt;2,"",ROUND(H392*I392,2))</f>
-        <v/>
-      </c>
-      <c r="E392" s="25" t="n">
-        <v>20</v>
-      </c>
-      <c r="F392" s="28">
-        <f>IF(D392="","",ROUND(D392*E392,1))</f>
-        <v/>
-      </c>
-      <c r="G392" s="2" t="n"/>
-      <c r="H392" s="35" t="n"/>
-      <c r="I392" s="35" t="n"/>
-    </row>
-    <row r="393" ht="62" customHeight="1">
-      <c r="A393" s="9" t="n"/>
-      <c r="B393" s="34" t="inlineStr">
-        <is>
-          <t>AISLADAS (    )</t>
-        </is>
-      </c>
-      <c r="C393" s="9">
-        <f>IF(COUNT(H393,I393)&lt;2,"",TEXT(H393,"0.00")&amp;" x "&amp;TEXT(I393,"0.00"))</f>
-        <v/>
-      </c>
-      <c r="D393" s="8">
-        <f>IF(COUNT(H393,I393)&lt;2,"",ROUND(H393*I393,2))</f>
-        <v/>
-      </c>
-      <c r="E393" s="25" t="n">
-        <v>20</v>
-      </c>
-      <c r="F393" s="28">
-        <f>IF(D393="","",ROUND(D393*E393,1))</f>
-        <v/>
-      </c>
-      <c r="G393" s="2" t="n"/>
-      <c r="H393" s="35" t="n"/>
-      <c r="I393" s="35" t="n"/>
-    </row>
-    <row r="394" ht="62" customHeight="1">
-      <c r="A394" s="9" t="n"/>
-      <c r="B394" s="34" t="inlineStr">
-        <is>
-          <t>AISLADAS (    )</t>
-        </is>
-      </c>
-      <c r="C394" s="9">
-        <f>IF(COUNT(H394,I394)&lt;2,"",TEXT(H394,"0.00")&amp;" x "&amp;TEXT(I394,"0.00"))</f>
-        <v/>
-      </c>
-      <c r="D394" s="8">
-        <f>IF(COUNT(H394,I394)&lt;2,"",ROUND(H394*I394,2))</f>
-        <v/>
-      </c>
-      <c r="E394" s="25" t="n">
-        <v>20</v>
-      </c>
-      <c r="F394" s="28">
-        <f>IF(D394="","",ROUND(D394*E394,1))</f>
-        <v/>
-      </c>
-      <c r="G394" s="2" t="n"/>
-      <c r="H394" s="35" t="n"/>
-      <c r="I394" s="35" t="n"/>
-    </row>
-    <row r="395" ht="62" customHeight="1">
-      <c r="A395" s="9" t="n"/>
-      <c r="B395" s="34" t="inlineStr">
-        <is>
-          <t>INTERIORES (    )</t>
-        </is>
-      </c>
-      <c r="C395" s="9">
-        <f>IF(COUNT(H395,I395)&lt;2,"",TEXT(H395,"0.00")&amp;" x "&amp;TEXT(I395,"0.00"))</f>
-        <v/>
-      </c>
-      <c r="D395" s="8">
-        <f>IF(COUNT(H395,I395)&lt;2,"",ROUND(H395*I395,2))</f>
-        <v/>
-      </c>
-      <c r="E395" s="25" t="n">
-        <v>25</v>
-      </c>
-      <c r="F395" s="28">
-        <f>IF(D395="","",ROUND(D395*E395,1))</f>
-        <v/>
-      </c>
-      <c r="G395" s="2" t="n"/>
-      <c r="H395" s="35" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="I395" s="35" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="396" ht="62" customHeight="1">
-      <c r="A396" s="9" t="n"/>
-      <c r="B396" s="34" t="inlineStr">
-        <is>
-          <t>INTERIORES (    )</t>
-        </is>
-      </c>
-      <c r="C396" s="9">
-        <f>IF(COUNT(H396,I396)&lt;2,"",TEXT(H396,"0.00")&amp;" x "&amp;TEXT(I396,"0.00"))</f>
-        <v/>
-      </c>
-      <c r="D396" s="8">
-        <f>IF(COUNT(H396,I396)&lt;2,"",ROUND(H396*I396,2))</f>
-        <v/>
-      </c>
-      <c r="E396" s="25" t="n">
-        <v>25</v>
-      </c>
-      <c r="F396" s="28">
-        <f>IF(D396="","",ROUND(D396*E396,1))</f>
-        <v/>
-      </c>
-      <c r="G396" s="2" t="n"/>
-      <c r="H396" s="35" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="I396" s="35" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="397" ht="62" customHeight="1">
-      <c r="A397" s="9" t="n"/>
-      <c r="B397" s="34" t="inlineStr">
-        <is>
-          <t>INTERIORES (    )</t>
-        </is>
-      </c>
-      <c r="C397" s="9">
-        <f>IF(COUNT(H397,I397)&lt;2,"",TEXT(H397,"0.00")&amp;" x "&amp;TEXT(I397,"0.00"))</f>
-        <v/>
-      </c>
-      <c r="D397" s="8">
-        <f>IF(COUNT(H397,I397)&lt;2,"",ROUND(H397*I397,2))</f>
-        <v/>
-      </c>
-      <c r="E397" s="25" t="n">
-        <v>25</v>
-      </c>
-      <c r="F397" s="28">
-        <f>IF(D397="","",ROUND(D397*E397,1))</f>
-        <v/>
-      </c>
-      <c r="G397" s="2" t="n"/>
-      <c r="H397" s="35" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="I397" s="35" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="398" ht="62" customHeight="1">
-      <c r="A398" s="9" t="n"/>
-      <c r="B398" s="34" t="inlineStr">
-        <is>
-          <t>INTERIORES (    )</t>
-        </is>
-      </c>
-      <c r="C398" s="9">
-        <f>IF(COUNT(H398,I398)&lt;2,"",TEXT(H398,"0.00")&amp;" x "&amp;TEXT(I398,"0.00"))</f>
-        <v/>
-      </c>
-      <c r="D398" s="8">
-        <f>IF(COUNT(H398,I398)&lt;2,"",ROUND(H398*I398,2))</f>
-        <v/>
-      </c>
-      <c r="E398" s="25" t="n">
-        <v>25</v>
-      </c>
-      <c r="F398" s="28">
-        <f>IF(D398="","",ROUND(D398*E398,1))</f>
-        <v/>
-      </c>
-      <c r="G398" s="2" t="n"/>
-      <c r="H398" s="35" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="I398" s="35" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="399" ht="39.7" customHeight="1">
-      <c r="A399" s="16" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B399" s="33" t="inlineStr">
-        <is>
-          <t>TECHOS O CIELORRASOS</t>
-        </is>
-      </c>
-      <c r="C399" s="9" t="n"/>
-      <c r="D399" s="9" t="n"/>
-      <c r="E399" s="9" t="n"/>
-      <c r="F399" s="9" t="n"/>
-      <c r="G399" s="2" t="n"/>
-      <c r="H399" s="2" t="n"/>
-      <c r="I399" s="2" t="n"/>
-    </row>
-    <row r="400" ht="62" customHeight="1">
-      <c r="A400" s="9" t="n"/>
-      <c r="B400" s="34" t="inlineStr">
-        <is>
-          <t>TECHO NO AISLADO</t>
-        </is>
-      </c>
-      <c r="C400" s="9" t="inlineStr"/>
-      <c r="D400" s="8">
-        <f>IF(COUNT(H400,I400)&lt;2,"",ROUND(H400*I400,2))</f>
-        <v/>
-      </c>
-      <c r="E400" s="25" t="n">
-        <v>30</v>
-      </c>
-      <c r="F400" s="28">
-        <f>IF(D400="","",ROUND(D400*E400,1))</f>
-        <v/>
-      </c>
-      <c r="G400" s="2" t="n"/>
-      <c r="H400" s="35" t="n"/>
-      <c r="I400" s="35" t="n"/>
-    </row>
-    <row r="401" ht="39.7" customHeight="1">
-      <c r="A401" s="9" t="n"/>
-      <c r="B401" s="34" t="inlineStr">
-        <is>
-          <t>TECHO AISLADO</t>
-        </is>
-      </c>
-      <c r="C401" s="9" t="inlineStr">
-        <is>
-          <t>por croquis</t>
-        </is>
-      </c>
-      <c r="D401" s="8" t="n">
-        <v>3.52</v>
-      </c>
-      <c r="E401" s="25" t="n">
-        <v>20</v>
-      </c>
-      <c r="F401" s="28">
-        <f>IF(D401="","",ROUND(D401*E401,1))</f>
-        <v/>
-      </c>
-      <c r="G401" s="2" t="n"/>
-      <c r="H401" s="35" t="n"/>
-      <c r="I401" s="35" t="n"/>
-    </row>
-    <row r="402" ht="62" customHeight="1">
-      <c r="A402" s="9" t="n"/>
-      <c r="B402" s="34" t="inlineStr">
-        <is>
-          <t>TECHO ENTREPISO</t>
-        </is>
-      </c>
-      <c r="C402" s="9" t="inlineStr"/>
-      <c r="D402" s="8">
-        <f>IF(COUNT(H402,I402)&lt;2,"",ROUND(H402*I402,2))</f>
-        <v/>
-      </c>
-      <c r="E402" s="25" t="n">
-        <v>15</v>
-      </c>
-      <c r="F402" s="28">
-        <f>IF(D402="","",ROUND(D402*E402,1))</f>
-        <v/>
-      </c>
-      <c r="G402" s="2" t="n"/>
-      <c r="H402" s="35" t="n"/>
-      <c r="I402" s="35" t="n"/>
-    </row>
-    <row r="403" ht="39.7" customHeight="1">
-      <c r="A403" s="16" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B403" s="33" t="inlineStr">
-        <is>
-          <t>PISO</t>
-        </is>
-      </c>
-      <c r="C403" s="9" t="n"/>
-      <c r="D403" s="9" t="n"/>
-      <c r="E403" s="9" t="n"/>
-      <c r="F403" s="9" t="n"/>
-      <c r="G403" s="2" t="n"/>
-      <c r="H403" s="2" t="n"/>
-      <c r="I403" s="2" t="n"/>
-    </row>
-    <row r="404" ht="62" customHeight="1">
-      <c r="A404" s="9" t="n"/>
-      <c r="B404" s="34" t="inlineStr">
-        <is>
-          <t>SOBRE TIERRA</t>
-        </is>
-      </c>
-      <c r="C404" s="9" t="inlineStr"/>
-      <c r="D404" s="8">
-        <f>IF(COUNT(H404,I404)&lt;2,"",ROUND(H404*I404,2))</f>
-        <v/>
-      </c>
-      <c r="E404" s="25" t="n">
-        <v>10</v>
-      </c>
-      <c r="F404" s="28">
-        <f>IF(D404="","",ROUND(D404*E404,1))</f>
-        <v/>
-      </c>
-      <c r="G404" s="2" t="n"/>
-      <c r="H404" s="35" t="n"/>
-      <c r="I404" s="35" t="n"/>
-    </row>
-    <row r="405" ht="39.7" customHeight="1">
-      <c r="A405" s="9" t="n"/>
-      <c r="B405" s="34" t="inlineStr">
-        <is>
-          <t>SOBRE LOCAL OCUPADO</t>
-        </is>
-      </c>
-      <c r="C405" s="9" t="inlineStr">
-        <is>
-          <t>por croquis</t>
-        </is>
-      </c>
-      <c r="D405" s="8" t="n">
-        <v>3.52</v>
-      </c>
-      <c r="E405" s="25" t="n">
-        <v>15</v>
-      </c>
-      <c r="F405" s="28">
-        <f>IF(D405="","",ROUND(D405*E405,1))</f>
-        <v/>
-      </c>
-      <c r="G405" s="2" t="n"/>
-      <c r="H405" s="35" t="n"/>
-      <c r="I405" s="35" t="n"/>
-    </row>
-    <row r="406" ht="39.7" customHeight="1">
-      <c r="A406" s="16" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B406" s="33" t="inlineStr">
-        <is>
-          <t>INFILTRACION</t>
-        </is>
-      </c>
-      <c r="C406" s="9" t="n"/>
-      <c r="D406" s="16" t="inlineStr">
-        <is>
-          <t>VOLUMEN (m3)</t>
-        </is>
-      </c>
-      <c r="E406" s="9" t="n"/>
-      <c r="F406" s="9" t="n"/>
-      <c r="G406" s="2" t="n"/>
-      <c r="H406" s="2" t="n"/>
-      <c r="I406" s="2" t="n"/>
-    </row>
-    <row r="407" ht="39.7" customHeight="1">
-      <c r="A407" s="9" t="n"/>
-      <c r="B407" s="34" t="inlineStr">
-        <is>
-          <t>UNA PARED EXTERIOR</t>
-        </is>
-      </c>
-      <c r="C407" s="9" t="inlineStr">
-        <is>
-          <t>3.52 m2 x 3.00</t>
-        </is>
-      </c>
-      <c r="D407" s="8" t="n">
-        <v>10.56</v>
-      </c>
-      <c r="E407" s="25" t="n">
-        <v>6</v>
-      </c>
-      <c r="F407" s="28">
-        <f>IF(D407="","",ROUND(D407*E407,1))</f>
-        <v/>
-      </c>
-      <c r="G407" s="2" t="n"/>
-      <c r="H407" s="35" t="n"/>
-      <c r="I407" s="35" t="n"/>
-    </row>
-    <row r="408" ht="62" customHeight="1">
-      <c r="A408" s="9" t="n"/>
-      <c r="B408" s="34" t="inlineStr">
-        <is>
-          <t>DOS PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C408" s="9" t="inlineStr"/>
-      <c r="D408" s="8">
-        <f>IF(COUNT(H408,I408)&lt;2,"",ROUND(H408*I408,2))</f>
-        <v/>
-      </c>
-      <c r="E408" s="25" t="n">
-        <v>9</v>
-      </c>
-      <c r="F408" s="28">
-        <f>IF(D408="","",ROUND(D408*E408,1))</f>
-        <v/>
-      </c>
-      <c r="G408" s="2" t="n"/>
-      <c r="H408" s="35" t="n"/>
-      <c r="I408" s="35" t="n"/>
-    </row>
-    <row r="409" ht="62" customHeight="1">
-      <c r="A409" s="9" t="n"/>
-      <c r="B409" s="34" t="inlineStr">
-        <is>
-          <t>TRES O MAS PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C409" s="9" t="inlineStr"/>
-      <c r="D409" s="8">
-        <f>IF(COUNT(H409,I409)&lt;2,"",ROUND(H409*I409,2))</f>
-        <v/>
-      </c>
-      <c r="E409" s="25" t="n">
-        <v>12</v>
-      </c>
-      <c r="F409" s="28">
-        <f>IF(D409="","",ROUND(D409*E409,1))</f>
-        <v/>
-      </c>
-      <c r="G409" s="2" t="n"/>
-      <c r="H409" s="35" t="n"/>
-      <c r="I409" s="35" t="n"/>
-    </row>
-    <row r="410" ht="70" customHeight="1">
-      <c r="A410" s="16" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B410" s="33" t="inlineStr">
-        <is>
-          <t>SUBTOTAL</t>
-        </is>
-      </c>
-      <c r="C410" s="9" t="n"/>
-      <c r="D410" s="9" t="n"/>
-      <c r="E410" s="9" t="n"/>
-      <c r="F410" s="36">
-        <f>IF(F389="",0,F389)+IF(F391="",0,F391)+IF(F392="",0,F392)+IF(F393="",0,F393)+IF(F394="",0,F394)+IF(F395="",0,F395)+IF(F396="",0,F396)+IF(F397="",0,F397)+IF(F398="",0,F398)+IF(F400="",0,F400)+IF(F401="",0,F401)+IF(F402="",0,F402)+IF(F404="",0,F404)+IF(F405="",0,F405)+IF(F407="",0,F407)+IF(F408="",0,F408)+IF(F409="",0,F409)</f>
-        <v/>
-      </c>
-      <c r="G410" s="2" t="n"/>
-      <c r="H410" s="2" t="n"/>
-      <c r="I410" s="2" t="n"/>
-    </row>
-    <row r="411" ht="47" customHeight="1">
-      <c r="A411" s="16" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B411" s="33" t="inlineStr">
-        <is>
-          <t>PERDIDA TOTAL</t>
-        </is>
-      </c>
-      <c r="C411" s="9">
-        <f>TEXT(F410,"0.00")&amp;"  X  "&amp;Datos_balance!$B$4&amp;" (FI)  X  "&amp;Datos_balance!$B$5&amp;" (FO)  X  "&amp;Datos_balance!$B$6&amp;" (FZ)"</f>
-        <v/>
-      </c>
-      <c r="D411" s="2" t="n"/>
-      <c r="E411" s="2" t="n"/>
-      <c r="F411" s="36">
-        <f>ROUND(F410*Datos_balance!$B$4*Datos_balance!$B$5*Datos_balance!$B$6,1)</f>
-        <v/>
-      </c>
-      <c r="G411" s="2" t="n"/>
-      <c r="H411" s="2" t="n"/>
-      <c r="I411" s="2" t="n"/>
-    </row>
-    <row r="412">
-      <c r="A412" s="2" t="n"/>
-      <c r="B412" s="2" t="n"/>
-      <c r="C412" s="2" t="n"/>
-      <c r="D412" s="2" t="n"/>
-      <c r="E412" s="2" t="n"/>
-      <c r="F412" s="2" t="n"/>
-      <c r="G412" s="2" t="n"/>
-      <c r="H412" s="2" t="n"/>
-      <c r="I412" s="2" t="n"/>
-    </row>
-    <row r="413" ht="62" customHeight="1">
-      <c r="A413" s="9" t="n"/>
-      <c r="B413" s="10" t="inlineStr">
-        <is>
-          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
-        </is>
-      </c>
-      <c r="C413" s="9">
-        <f>TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2,"0")&amp;" - "&amp;TEXT(Datos_balance!$B$11,"0")&amp;" = "&amp;TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2-Datos_balance!$B$11,"0")&amp;" C"</f>
-        <v/>
-      </c>
-      <c r="D413" s="2" t="n"/>
-      <c r="E413" s="2" t="n"/>
-      <c r="F413" s="9" t="n"/>
-      <c r="G413" s="2" t="n"/>
-      <c r="H413" s="2" t="n"/>
-      <c r="I413" s="2" t="n"/>
-    </row>
-    <row r="414" ht="39.7" customHeight="1">
-      <c r="A414" s="9" t="n"/>
-      <c r="B414" s="10" t="inlineStr">
-        <is>
-          <t>Kcal/h del toallero Scala/Domino 80</t>
-        </is>
-      </c>
-      <c r="C414" s="25">
-        <f>ROUND(Datos_balance!$B$18*Datos_balance!$B$15,0)</f>
-        <v/>
-      </c>
-      <c r="D414" s="2" t="n"/>
-      <c r="E414" s="2" t="n"/>
-      <c r="F414" s="9" t="n"/>
-      <c r="G414" s="2" t="n"/>
-      <c r="H414" s="2" t="n"/>
-      <c r="I414" s="2" t="n"/>
-    </row>
-    <row r="415" ht="39.7" customHeight="1">
-      <c r="A415" s="9" t="n"/>
-      <c r="B415" s="10" t="inlineStr">
-        <is>
-          <t>Kcal/h del toallero Scala/Domino 150</t>
-        </is>
-      </c>
-      <c r="C415" s="25">
-        <f>ROUND(Datos_balance!$B$19*Datos_balance!$B$15,0)</f>
-        <v/>
-      </c>
-      <c r="D415" s="2" t="n"/>
-      <c r="E415" s="2" t="n"/>
-      <c r="F415" s="9" t="n"/>
-      <c r="G415" s="2" t="n"/>
-      <c r="H415" s="2" t="n"/>
-      <c r="I415" s="2" t="n"/>
-    </row>
-    <row r="416" ht="47" customHeight="1">
-      <c r="A416" s="9" t="n"/>
-      <c r="B416" s="10" t="inlineStr">
-        <is>
-          <t>Toalleros necesarios</t>
-        </is>
-      </c>
-      <c r="C416" s="25">
-        <f>IF(F411&lt;=Datos_balance!$B$18*Datos_balance!$B$15,1,ROUNDUP(F411/(Datos_balance!$B$19*Datos_balance!$B$15),0))</f>
-        <v/>
-      </c>
-      <c r="D416" s="2" t="n"/>
-      <c r="E416" s="2" t="n"/>
-      <c r="F416" s="9" t="n"/>
-      <c r="G416" s="2" t="n"/>
-      <c r="H416" s="2" t="n"/>
-      <c r="I416" s="2" t="n"/>
-    </row>
-    <row r="417" ht="47" customHeight="1">
-      <c r="A417" s="13" t="n"/>
-      <c r="B417" s="14" t="inlineStr">
-        <is>
-          <t>Toallero adoptado</t>
-        </is>
-      </c>
-      <c r="C417" s="13">
-        <f>IF(F411&lt;=Datos_balance!$B$18*Datos_balance!$B$15,"Peisa Scala / Domino 80  (500 x 800 mm)","Peisa Scala / Domino 150  (500 x 1500 mm)")</f>
-        <v/>
-      </c>
-      <c r="D417" s="20" t="n"/>
-      <c r="E417" s="20" t="n"/>
-      <c r="F417" s="13" t="n"/>
-      <c r="G417" s="2" t="n"/>
-      <c r="H417" s="2" t="n"/>
-      <c r="I417" s="2" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="85">
+  <mergeCells count="78">
     <mergeCell ref="C274:E274"/>
     <mergeCell ref="C345:E345"/>
     <mergeCell ref="C142:E142"/>
@@ -32263,22 +31501,18 @@
     <mergeCell ref="A75:F75"/>
     <mergeCell ref="C242:E242"/>
     <mergeCell ref="A317:F317"/>
-    <mergeCell ref="C413:E413"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="C379:E379"/>
     <mergeCell ref="C244:E244"/>
-    <mergeCell ref="C415:E415"/>
     <mergeCell ref="C71:E71"/>
     <mergeCell ref="C241:E241"/>
     <mergeCell ref="C347:E347"/>
-    <mergeCell ref="A386:F386"/>
     <mergeCell ref="C243:E243"/>
     <mergeCell ref="C140:E140"/>
     <mergeCell ref="A40:F40"/>
     <mergeCell ref="C34:E34"/>
     <mergeCell ref="C141:E141"/>
     <mergeCell ref="C377:E377"/>
-    <mergeCell ref="C417:E417"/>
     <mergeCell ref="C103:E103"/>
     <mergeCell ref="C205:E205"/>
     <mergeCell ref="A283:F283"/>
@@ -32291,7 +31525,6 @@
     <mergeCell ref="C312:E312"/>
     <mergeCell ref="C346:E346"/>
     <mergeCell ref="C106:E106"/>
-    <mergeCell ref="C414:E414"/>
     <mergeCell ref="C209:E209"/>
     <mergeCell ref="C348:E348"/>
     <mergeCell ref="C381:E381"/>
@@ -32300,14 +31533,12 @@
     <mergeCell ref="C33:E33"/>
     <mergeCell ref="C104:E104"/>
     <mergeCell ref="C35:E35"/>
-    <mergeCell ref="C416:E416"/>
     <mergeCell ref="C173:E173"/>
     <mergeCell ref="C276:E276"/>
     <mergeCell ref="A145:F145"/>
     <mergeCell ref="C36:E36"/>
     <mergeCell ref="C207:E207"/>
     <mergeCell ref="C278:E278"/>
-    <mergeCell ref="C411:E411"/>
     <mergeCell ref="A109:F109"/>
     <mergeCell ref="A180:F180"/>
     <mergeCell ref="C72:E72"/>

</xml_diff>

<commit_message>
Cocina: orientacion de los muros exteriores, y correccion de la Planilla 3
El muro exterior de 7,63, el de la bacha, da al Noreste; el de 3,56 que
da al patio, al Noroeste. Asi queda en el balance termico.

Con eso se corrige la Planilla 3: las cuatro aberturas de la cocina
estaban repartidas en tres orientaciones, lo que es imposible con solo
dos muros exteriores. VA01 y PF04 pasan de Sudoeste y Sudeste a
Noroeste; PF03 y PV02 ya estaban bien en Noreste.

Verificacion geometrica: PF03 2,88 + PV02 2,48 = 5,36 entran en el muro
de 7,63, y PF04 2,70 + VA01 0,75 = 3,45 entran en el de 3,56. Las dos
paredes cierran, lo que respalda el reparto.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -8912,21 +8912,21 @@
     <row r="16" ht="70" customHeight="1">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>VA01</t>
+          <t>PF01 (2)</t>
         </is>
       </c>
       <c r="B16" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C16" s="8" t="n">
-        <v>0.75</v>
+        <v>3.55</v>
       </c>
       <c r="D16" s="8">
         <f>IF(COUNT(B16,C16)&lt;2,"",B16*C16)</f>
         <v/>
       </c>
       <c r="E16" s="17">
-        <f>SUM(D16:D19)</f>
+        <f>SUM(D16:D18)</f>
         <v/>
       </c>
       <c r="F16" s="18">
@@ -8965,17 +8965,9 @@
       </c>
     </row>
     <row r="17" ht="70" customHeight="1">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>PF01 (2)</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="C17" s="8" t="n">
-        <v>3.55</v>
-      </c>
+      <c r="A17" s="9" t="n"/>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="8" t="n"/>
       <c r="D17" s="8">
         <f>IF(COUNT(B17,C17)&lt;2,"",B17*C17)</f>
         <v/>
@@ -8989,24 +8981,10 @@
         <f>IF(A17="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H17" s="9" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I17" s="9" t="inlineStr">
-        <is>
-          <t>Sin Proteccion</t>
-        </is>
-      </c>
-      <c r="J17" s="8" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K17" s="9" t="inlineStr">
-        <is>
-          <t>Sudoeste</t>
-        </is>
-      </c>
+      <c r="H17" s="9" t="n"/>
+      <c r="I17" s="9" t="n"/>
+      <c r="J17" s="8" t="n"/>
+      <c r="K17" s="9" t="n"/>
       <c r="L17" s="8">
         <f>IF(I17="","",IFERROR(VLOOKUP(I17,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
@@ -9017,106 +8995,128 @@
       </c>
     </row>
     <row r="18" ht="70" customHeight="1">
-      <c r="A18" s="9" t="n"/>
-      <c r="B18" s="8" t="n"/>
-      <c r="C18" s="8" t="n"/>
-      <c r="D18" s="8">
+      <c r="A18" s="13" t="n"/>
+      <c r="B18" s="12" t="n"/>
+      <c r="C18" s="12" t="n"/>
+      <c r="D18" s="12">
         <f>IF(COUNT(B18,C18)&lt;2,"",B18*C18)</f>
         <v/>
       </c>
-      <c r="E18" s="19" t="n"/>
-      <c r="F18" s="18">
+      <c r="E18" s="20" t="n"/>
+      <c r="F18" s="21">
         <f>IF(OR(D18="",$E$16=""),"",D18/$E$16)</f>
         <v/>
       </c>
-      <c r="G18" s="8">
+      <c r="G18" s="12">
         <f>IF(A18="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H18" s="9" t="n"/>
-      <c r="I18" s="9" t="n"/>
-      <c r="J18" s="8" t="n"/>
-      <c r="K18" s="9" t="n"/>
-      <c r="L18" s="8">
+      <c r="H18" s="13" t="n"/>
+      <c r="I18" s="13" t="n"/>
+      <c r="J18" s="12" t="n"/>
+      <c r="K18" s="13" t="n"/>
+      <c r="L18" s="12">
         <f>IF(I18="","",IFERROR(VLOOKUP(I18,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
-      <c r="M18" s="9">
+      <c r="M18" s="13">
         <f>IF(OR(D18="",J18=""),"",IF(J18&lt;=G18,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="19" ht="70" customHeight="1">
-      <c r="A19" s="13" t="n"/>
-      <c r="B19" s="12" t="n"/>
-      <c r="C19" s="12" t="n"/>
-      <c r="D19" s="12">
-        <f>IF(COUNT(B19,C19)&lt;2,"",B19*C19)</f>
-        <v/>
-      </c>
-      <c r="E19" s="20" t="n"/>
-      <c r="F19" s="21">
-        <f>IF(OR(D19="",$E$16=""),"",D19/$E$16)</f>
-        <v/>
-      </c>
-      <c r="G19" s="12">
-        <f>IF(A19="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H19" s="13" t="n"/>
-      <c r="I19" s="13" t="n"/>
-      <c r="J19" s="12" t="n"/>
-      <c r="K19" s="13" t="n"/>
-      <c r="L19" s="12">
-        <f>IF(I19="","",IFERROR(VLOOKUP(I19,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M19" s="13">
-        <f>IF(OR(D19="",J19=""),"",IF(J19&lt;=G19,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="39.7" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="19" ht="39.7" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Plano: Fachada Sudeste (borde inferior)</t>
         </is>
       </c>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="4" t="n"/>
-      <c r="G20" s="4" t="n"/>
-      <c r="H20" s="4" t="n"/>
-      <c r="I20" s="4" t="n"/>
-      <c r="J20" s="4" t="n"/>
-      <c r="K20" s="4" t="n"/>
-      <c r="L20" s="4" t="n"/>
-      <c r="M20" s="4" t="n"/>
+      <c r="B19" s="4" t="n"/>
+      <c r="C19" s="4" t="n"/>
+      <c r="D19" s="4" t="n"/>
+      <c r="E19" s="4" t="n"/>
+      <c r="F19" s="4" t="n"/>
+      <c r="G19" s="4" t="n"/>
+      <c r="H19" s="4" t="n"/>
+      <c r="I19" s="4" t="n"/>
+      <c r="J19" s="4" t="n"/>
+      <c r="K19" s="4" t="n"/>
+      <c r="L19" s="4" t="n"/>
+      <c r="M19" s="4" t="n"/>
+    </row>
+    <row r="20" ht="70" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>PA01</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="8">
+        <f>IF(COUNT(B20,C20)&lt;2,"",B20*C20)</f>
+        <v/>
+      </c>
+      <c r="E20" s="17">
+        <f>SUM(D20:D27)</f>
+        <v/>
+      </c>
+      <c r="F20" s="18">
+        <f>IF(OR(D20="",$E$20=""),"",D20/$E$20)</f>
+        <v/>
+      </c>
+      <c r="G20" s="8">
+        <f>IF(A20="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K20" s="9" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="L20" s="8">
+        <f>IF(I20="","",IFERROR(VLOOKUP(I20,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M20" s="9">
+        <f>IF(OR(D20="",J20=""),"",IF(J20&lt;=G20,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
     </row>
     <row r="21" ht="70" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>PA01</t>
+          <t>VA01 (2)</t>
         </is>
       </c>
       <c r="B21" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C21" s="8" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="D21" s="8">
         <f>IF(COUNT(B21,C21)&lt;2,"",B21*C21)</f>
         <v/>
       </c>
-      <c r="E21" s="17">
-        <f>SUM(D21:D29)</f>
-        <v/>
-      </c>
+      <c r="E21" s="19" t="n"/>
       <c r="F21" s="18">
-        <f>IF(OR(D21="",$E$21=""),"",D21/$E$21)</f>
+        <f>IF(OR(D21="",$E$20=""),"",D21/$E$20)</f>
         <v/>
       </c>
       <c r="G21" s="8">
@@ -9153,14 +9153,14 @@
     <row r="22" ht="70" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>PF04</t>
+          <t>VA05</t>
         </is>
       </c>
       <c r="B22" s="8" t="n">
-        <v>0.6</v>
+        <v>2.52</v>
       </c>
       <c r="C22" s="8" t="n">
-        <v>2.7</v>
+        <v>1.4</v>
       </c>
       <c r="D22" s="8">
         <f>IF(COUNT(B22,C22)&lt;2,"",B22*C22)</f>
@@ -9168,7 +9168,7 @@
       </c>
       <c r="E22" s="19" t="n"/>
       <c r="F22" s="18">
-        <f>IF(OR(D22="",$E$21=""),"",D22/$E$21)</f>
+        <f>IF(OR(D22="",$E$20=""),"",D22/$E$20)</f>
         <v/>
       </c>
       <c r="G22" s="8">
@@ -9205,14 +9205,14 @@
     <row r="23" ht="70" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>VA01 (2)</t>
+          <t>PV04</t>
         </is>
       </c>
       <c r="B23" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C23" s="8" t="n">
-        <v>0.75</v>
+        <v>2.06</v>
       </c>
       <c r="D23" s="8">
         <f>IF(COUNT(B23,C23)&lt;2,"",B23*C23)</f>
@@ -9220,7 +9220,7 @@
       </c>
       <c r="E23" s="19" t="n"/>
       <c r="F23" s="18">
-        <f>IF(OR(D23="",$E$21=""),"",D23/$E$21)</f>
+        <f>IF(OR(D23="",$E$20=""),"",D23/$E$20)</f>
         <v/>
       </c>
       <c r="G23" s="8">
@@ -9257,14 +9257,14 @@
     <row r="24" ht="70" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>VA05</t>
+          <t>PV04 (2)</t>
         </is>
       </c>
       <c r="B24" s="8" t="n">
-        <v>2.52</v>
+        <v>2.95</v>
       </c>
       <c r="C24" s="8" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="D24" s="8">
         <f>IF(COUNT(B24,C24)&lt;2,"",B24*C24)</f>
@@ -9272,7 +9272,7 @@
       </c>
       <c r="E24" s="19" t="n"/>
       <c r="F24" s="18">
-        <f>IF(OR(D24="",$E$21=""),"",D24/$E$21)</f>
+        <f>IF(OR(D24="",$E$20=""),"",D24/$E$20)</f>
         <v/>
       </c>
       <c r="G24" s="8">
@@ -9309,14 +9309,14 @@
     <row r="25" ht="70" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>PV04</t>
+          <t>PF02</t>
         </is>
       </c>
       <c r="B25" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C25" s="8" t="n">
-        <v>2.06</v>
+        <v>3.75</v>
       </c>
       <c r="D25" s="8">
         <f>IF(COUNT(B25,C25)&lt;2,"",B25*C25)</f>
@@ -9324,7 +9324,7 @@
       </c>
       <c r="E25" s="19" t="n"/>
       <c r="F25" s="18">
-        <f>IF(OR(D25="",$E$21=""),"",D25/$E$21)</f>
+        <f>IF(OR(D25="",$E$20=""),"",D25/$E$20)</f>
         <v/>
       </c>
       <c r="G25" s="8">
@@ -9359,48 +9359,26 @@
       </c>
     </row>
     <row r="26" ht="70" customHeight="1">
-      <c r="A26" s="9" t="inlineStr">
-        <is>
-          <t>PV04 (2)</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="n">
-        <v>2.95</v>
-      </c>
-      <c r="C26" s="8" t="n">
-        <v>1.5</v>
-      </c>
+      <c r="A26" s="9" t="n"/>
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="8" t="n"/>
       <c r="D26" s="8">
         <f>IF(COUNT(B26,C26)&lt;2,"",B26*C26)</f>
         <v/>
       </c>
       <c r="E26" s="19" t="n"/>
       <c r="F26" s="18">
-        <f>IF(OR(D26="",$E$21=""),"",D26/$E$21)</f>
+        <f>IF(OR(D26="",$E$20=""),"",D26/$E$20)</f>
         <v/>
       </c>
       <c r="G26" s="8">
         <f>IF(A26="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H26" s="9" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I26" s="9" t="inlineStr">
-        <is>
-          <t>Sin Proteccion</t>
-        </is>
-      </c>
-      <c r="J26" s="8" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K26" s="9" t="inlineStr">
-        <is>
-          <t>Sudeste</t>
-        </is>
-      </c>
+      <c r="H26" s="9" t="n"/>
+      <c r="I26" s="9" t="n"/>
+      <c r="J26" s="8" t="n"/>
+      <c r="K26" s="9" t="n"/>
       <c r="L26" s="8">
         <f>IF(I26="","",IFERROR(VLOOKUP(I26,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
@@ -9411,158 +9389,180 @@
       </c>
     </row>
     <row r="27" ht="70" customHeight="1">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>PF02</t>
-        </is>
-      </c>
-      <c r="B27" s="8" t="n">
+      <c r="A27" s="13" t="n"/>
+      <c r="B27" s="12" t="n"/>
+      <c r="C27" s="12" t="n"/>
+      <c r="D27" s="12">
+        <f>IF(COUNT(B27,C27)&lt;2,"",B27*C27)</f>
+        <v/>
+      </c>
+      <c r="E27" s="20" t="n"/>
+      <c r="F27" s="21">
+        <f>IF(OR(D27="",$E$20=""),"",D27/$E$20)</f>
+        <v/>
+      </c>
+      <c r="G27" s="12">
+        <f>IF(A27="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H27" s="13" t="n"/>
+      <c r="I27" s="13" t="n"/>
+      <c r="J27" s="12" t="n"/>
+      <c r="K27" s="13" t="n"/>
+      <c r="L27" s="12">
+        <f>IF(I27="","",IFERROR(VLOOKUP(I27,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M27" s="13">
+        <f>IF(OR(D27="",J27=""),"",IF(J27&lt;=G27,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="39.7" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Plano: Fachada Noroeste (borde superior)</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="n"/>
+      <c r="C28" s="4" t="n"/>
+      <c r="D28" s="4" t="n"/>
+      <c r="E28" s="4" t="n"/>
+      <c r="F28" s="4" t="n"/>
+      <c r="G28" s="4" t="n"/>
+      <c r="H28" s="4" t="n"/>
+      <c r="I28" s="4" t="n"/>
+      <c r="J28" s="4" t="n"/>
+      <c r="K28" s="4" t="n"/>
+      <c r="L28" s="4" t="n"/>
+      <c r="M28" s="4" t="n"/>
+    </row>
+    <row r="29" ht="70" customHeight="1">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>PV03</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="C27" s="8" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="D27" s="8">
-        <f>IF(COUNT(B27,C27)&lt;2,"",B27*C27)</f>
-        <v/>
-      </c>
-      <c r="E27" s="19" t="n"/>
-      <c r="F27" s="18">
-        <f>IF(OR(D27="",$E$21=""),"",D27/$E$21)</f>
-        <v/>
-      </c>
-      <c r="G27" s="8">
-        <f>IF(A27="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H27" s="9" t="inlineStr">
+      <c r="C29" s="8" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="D29" s="8">
+        <f>IF(COUNT(B29,C29)&lt;2,"",B29*C29)</f>
+        <v/>
+      </c>
+      <c r="E29" s="17">
+        <f>SUM(D29:D37)</f>
+        <v/>
+      </c>
+      <c r="F29" s="18">
+        <f>IF(OR(D29="",$E$29=""),"",D29/$E$29)</f>
+        <v/>
+      </c>
+      <c r="G29" s="8">
+        <f>IF(A29="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H29" s="9" t="inlineStr">
         <is>
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I27" s="9" t="inlineStr">
+      <c r="I29" s="9" t="inlineStr">
         <is>
           <t>Sin Proteccion</t>
         </is>
       </c>
-      <c r="J27" s="8" t="n">
+      <c r="J29" s="8" t="n">
         <v>2.8</v>
       </c>
-      <c r="K27" s="9" t="inlineStr">
-        <is>
-          <t>Sudeste</t>
-        </is>
-      </c>
-      <c r="L27" s="8">
-        <f>IF(I27="","",IFERROR(VLOOKUP(I27,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M27" s="9">
-        <f>IF(OR(D27="",J27=""),"",IF(J27&lt;=G27,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="70" customHeight="1">
-      <c r="A28" s="9" t="n"/>
-      <c r="B28" s="8" t="n"/>
-      <c r="C28" s="8" t="n"/>
-      <c r="D28" s="8">
-        <f>IF(COUNT(B28,C28)&lt;2,"",B28*C28)</f>
-        <v/>
-      </c>
-      <c r="E28" s="19" t="n"/>
-      <c r="F28" s="18">
-        <f>IF(OR(D28="",$E$21=""),"",D28/$E$21)</f>
-        <v/>
-      </c>
-      <c r="G28" s="8">
-        <f>IF(A28="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H28" s="9" t="n"/>
-      <c r="I28" s="9" t="n"/>
-      <c r="J28" s="8" t="n"/>
-      <c r="K28" s="9" t="n"/>
-      <c r="L28" s="8">
-        <f>IF(I28="","",IFERROR(VLOOKUP(I28,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M28" s="9">
-        <f>IF(OR(D28="",J28=""),"",IF(J28&lt;=G28,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="70" customHeight="1">
-      <c r="A29" s="13" t="n"/>
-      <c r="B29" s="12" t="n"/>
-      <c r="C29" s="12" t="n"/>
-      <c r="D29" s="12">
-        <f>IF(COUNT(B29,C29)&lt;2,"",B29*C29)</f>
-        <v/>
-      </c>
-      <c r="E29" s="20" t="n"/>
-      <c r="F29" s="21">
-        <f>IF(OR(D29="",$E$21=""),"",D29/$E$21)</f>
-        <v/>
-      </c>
-      <c r="G29" s="12">
-        <f>IF(A29="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H29" s="13" t="n"/>
-      <c r="I29" s="13" t="n"/>
-      <c r="J29" s="12" t="n"/>
-      <c r="K29" s="13" t="n"/>
-      <c r="L29" s="12">
+      <c r="K29" s="9" t="inlineStr">
+        <is>
+          <t>Noroeste</t>
+        </is>
+      </c>
+      <c r="L29" s="8">
         <f>IF(I29="","",IFERROR(VLOOKUP(I29,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
-      <c r="M29" s="13">
+      <c r="M29" s="9">
         <f>IF(OR(D29="",J29=""),"",IF(J29&lt;=G29,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="30" ht="39.7" customHeight="1">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>Plano: Fachada Noroeste (borde superior)</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="n"/>
-      <c r="C30" s="4" t="n"/>
-      <c r="D30" s="4" t="n"/>
-      <c r="E30" s="4" t="n"/>
-      <c r="F30" s="4" t="n"/>
-      <c r="G30" s="4" t="n"/>
-      <c r="H30" s="4" t="n"/>
-      <c r="I30" s="4" t="n"/>
-      <c r="J30" s="4" t="n"/>
-      <c r="K30" s="4" t="n"/>
-      <c r="L30" s="4" t="n"/>
-      <c r="M30" s="4" t="n"/>
+    <row r="30" ht="70" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>VA01</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C30" s="8" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D30" s="8">
+        <f>IF(COUNT(B30,C30)&lt;2,"",B30*C30)</f>
+        <v/>
+      </c>
+      <c r="E30" s="19" t="n"/>
+      <c r="F30" s="18">
+        <f>IF(OR(D30="",$E$29=""),"",D30/$E$29)</f>
+        <v/>
+      </c>
+      <c r="G30" s="8">
+        <f>IF(A30="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H30" s="9" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I30" s="9" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J30" s="8" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K30" s="9" t="inlineStr">
+        <is>
+          <t>Noroeste</t>
+        </is>
+      </c>
+      <c r="L30" s="8">
+        <f>IF(I30="","",IFERROR(VLOOKUP(I30,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M30" s="9">
+        <f>IF(OR(D30="",J30=""),"",IF(J30&lt;=G30,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
     </row>
     <row r="31" ht="70" customHeight="1">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>PV03</t>
+          <t>PF04</t>
         </is>
       </c>
       <c r="B31" s="8" t="n">
-        <v>3</v>
+        <v>0.6</v>
       </c>
       <c r="C31" s="8" t="n">
-        <v>1.76</v>
+        <v>2.7</v>
       </c>
       <c r="D31" s="8">
         <f>IF(COUNT(B31,C31)&lt;2,"",B31*C31)</f>
         <v/>
       </c>
-      <c r="E31" s="17">
-        <f>SUM(D31:D37)</f>
-        <v/>
-      </c>
+      <c r="E31" s="19" t="n"/>
       <c r="F31" s="18">
-        <f>IF(OR(D31="",$E$31=""),"",D31/$E$31)</f>
+        <f>IF(OR(D31="",$E$29=""),"",D31/$E$29)</f>
         <v/>
       </c>
       <c r="G31" s="8">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="E32" s="19" t="n"/>
       <c r="F32" s="18">
-        <f>IF(OR(D32="",$E$31=""),"",D32/$E$31)</f>
+        <f>IF(OR(D32="",$E$29=""),"",D32/$E$29)</f>
         <v/>
       </c>
       <c r="G32" s="8">
@@ -9666,7 +9666,7 @@
       </c>
       <c r="E33" s="19" t="n"/>
       <c r="F33" s="18">
-        <f>IF(OR(D33="",$E$31=""),"",D33/$E$31)</f>
+        <f>IF(OR(D33="",$E$29=""),"",D33/$E$29)</f>
         <v/>
       </c>
       <c r="G33" s="8">
@@ -9718,7 +9718,7 @@
       </c>
       <c r="E34" s="19" t="n"/>
       <c r="F34" s="18">
-        <f>IF(OR(D34="",$E$31=""),"",D34/$E$31)</f>
+        <f>IF(OR(D34="",$E$29=""),"",D34/$E$29)</f>
         <v/>
       </c>
       <c r="G34" s="8">
@@ -9770,7 +9770,7 @@
       </c>
       <c r="E35" s="19" t="n"/>
       <c r="F35" s="18">
-        <f>IF(OR(D35="",$E$31=""),"",D35/$E$31)</f>
+        <f>IF(OR(D35="",$E$29=""),"",D35/$E$29)</f>
         <v/>
       </c>
       <c r="G35" s="8">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="E36" s="19" t="n"/>
       <c r="F36" s="18">
-        <f>IF(OR(D36="",$E$31=""),"",D36/$E$31)</f>
+        <f>IF(OR(D36="",$E$29=""),"",D36/$E$29)</f>
         <v/>
       </c>
       <c r="G36" s="8">
@@ -9844,7 +9844,7 @@
       </c>
       <c r="E37" s="20" t="n"/>
       <c r="F37" s="21">
-        <f>IF(OR(D37="",$E$31=""),"",D37/$E$31)</f>
+        <f>IF(OR(D37="",$E$29=""),"",D37/$E$29)</f>
         <v/>
       </c>
       <c r="G37" s="12">
@@ -10819,19 +10819,19 @@
   </sheetData>
   <mergeCells count="14">
     <mergeCell ref="A1:A3"/>
+    <mergeCell ref="A19:M19"/>
     <mergeCell ref="E7:E14"/>
+    <mergeCell ref="E16:E18"/>
     <mergeCell ref="A6:M6"/>
     <mergeCell ref="B3:L3"/>
     <mergeCell ref="B2:L2"/>
     <mergeCell ref="A4:M4"/>
-    <mergeCell ref="E21:E29"/>
-    <mergeCell ref="A30:M30"/>
-    <mergeCell ref="E16:E19"/>
+    <mergeCell ref="E20:E27"/>
     <mergeCell ref="A15:M15"/>
-    <mergeCell ref="E31:E37"/>
-    <mergeCell ref="A20:M20"/>
+    <mergeCell ref="E29:E37"/>
     <mergeCell ref="M1:M3"/>
     <mergeCell ref="B1:L1"/>
+    <mergeCell ref="A28:M28"/>
   </mergeCells>
   <conditionalFormatting sqref="M6:M37">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
@@ -23038,7 +23038,7 @@
       <c r="A11" s="9" t="n"/>
       <c r="B11" s="34" t="inlineStr">
         <is>
-          <t>AISLADAS (?)</t>
+          <t>AISLADAS (NE)</t>
         </is>
       </c>
       <c r="C11" s="9">
@@ -23068,7 +23068,7 @@
       <c r="A12" s="9" t="n"/>
       <c r="B12" s="34" t="inlineStr">
         <is>
-          <t>AISLADAS (?)</t>
+          <t>AISLADAS (NO)</t>
         </is>
       </c>
       <c r="C12" s="9">

</xml_diff>

<commit_message>
Balance termico: incorporar la escalera
1,00 x 4,10, con la PF05 como abertura. Quedaba fuera del balance aunque
tiene un pano fijo al exterior de 0,75 x 2,52, asi que su perdida no se
le computaba a nadie.

Entra como bloque propio. Si conviene anexarla al hall o al living, que
es a donde se abre, se pasa su superficie y su abertura a ese local.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -42,7 +42,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="5">'Vigas de fundacion'!$A$1:$X$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Pilotes y cabezales'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Tabiques'!$1:$3</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="8">'Balance termico'!$A$1:$F$382</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="8">'Balance termico'!$A$1:$F$416</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22778,7 +22778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I379"/>
+  <dimension ref="A1:I413"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.1" customWidth="1" min="1" max="1"/>
@@ -25965,7 +25965,7 @@
     <row r="141" ht="39.7" customHeight="1">
       <c r="A141" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  09 - Dormitorio suite   (PB)</t>
+          <t>LOCAL  Escalera   (PB)</t>
         </is>
       </c>
       <c r="B141" s="2" t="n"/>
@@ -26035,7 +26035,7 @@
       <c r="A144" s="9" t="n"/>
       <c r="B144" s="34" t="inlineStr">
         <is>
-          <t>VA01 (2)</t>
+          <t>PF05</t>
         </is>
       </c>
       <c r="C144" s="9">
@@ -26058,57 +26058,53 @@
         <v>0.75</v>
       </c>
       <c r="I144" s="35" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="145" ht="62" customHeight="1">
-      <c r="A145" s="9" t="n"/>
-      <c r="B145" s="34" t="inlineStr">
-        <is>
-          <t>PV03</t>
-        </is>
-      </c>
-      <c r="C145" s="9">
-        <f>IF(COUNT(H145,I145)&lt;2,"",TEXT(H145,"0.00")&amp;" x "&amp;TEXT(I145,"0.00"))</f>
-        <v/>
-      </c>
-      <c r="D145" s="8">
-        <f>IF(COUNT(H145,I145)&lt;2,"",ROUND(H145*I145,2))</f>
-        <v/>
-      </c>
-      <c r="E145" s="25" t="n">
-        <v>60</v>
-      </c>
-      <c r="F145" s="28">
-        <f>IF(D145="","",ROUND(D145*E145,1))</f>
-        <v/>
-      </c>
+        <v>2.52</v>
+      </c>
+    </row>
+    <row r="145" ht="39.7" customHeight="1">
+      <c r="A145" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B145" s="33" t="inlineStr">
+        <is>
+          <t>PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C145" s="9" t="n"/>
+      <c r="D145" s="9" t="n"/>
+      <c r="E145" s="9" t="n"/>
+      <c r="F145" s="9" t="n"/>
       <c r="G145" s="2" t="n"/>
-      <c r="H145" s="35" t="n">
-        <v>1.76</v>
-      </c>
-      <c r="I145" s="35" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="146" ht="39.7" customHeight="1">
-      <c r="A146" s="16" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B146" s="33" t="inlineStr">
-        <is>
-          <t>PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C146" s="9" t="n"/>
-      <c r="D146" s="9" t="n"/>
-      <c r="E146" s="9" t="n"/>
-      <c r="F146" s="9" t="n"/>
+      <c r="H145" s="2" t="n"/>
+      <c r="I145" s="2" t="n"/>
+    </row>
+    <row r="146" ht="62" customHeight="1">
+      <c r="A146" s="9" t="n"/>
+      <c r="B146" s="34" t="inlineStr">
+        <is>
+          <t>AISLADAS (    )</t>
+        </is>
+      </c>
+      <c r="C146" s="9">
+        <f>IF(COUNT(H146,I146)&lt;2,"",TEXT(H146,"0.00")&amp;" x "&amp;TEXT(I146,"0.00"))</f>
+        <v/>
+      </c>
+      <c r="D146" s="8">
+        <f>IF(COUNT(H146,I146)&lt;2,"",ROUND(H146*I146,2))</f>
+        <v/>
+      </c>
+      <c r="E146" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="F146" s="28">
+        <f>IF(D146="","",ROUND(D146*E146,1))</f>
+        <v/>
+      </c>
       <c r="G146" s="2" t="n"/>
-      <c r="H146" s="2" t="n"/>
-      <c r="I146" s="2" t="n"/>
+      <c r="H146" s="35" t="n"/>
+      <c r="I146" s="35" t="n"/>
     </row>
     <row r="147" ht="62" customHeight="1">
       <c r="A147" s="9" t="n"/>
@@ -26192,7 +26188,7 @@
       <c r="A150" s="9" t="n"/>
       <c r="B150" s="34" t="inlineStr">
         <is>
-          <t>AISLADAS (    )</t>
+          <t>INTERIORES (    )</t>
         </is>
       </c>
       <c r="C150" s="9">
@@ -26204,15 +26200,19 @@
         <v/>
       </c>
       <c r="E150" s="25" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F150" s="28">
         <f>IF(D150="","",ROUND(D150*E150,1))</f>
         <v/>
       </c>
       <c r="G150" s="2" t="n"/>
-      <c r="H150" s="35" t="n"/>
-      <c r="I150" s="35" t="n"/>
+      <c r="H150" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="I150" s="35" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="151" ht="62" customHeight="1">
       <c r="A151" s="9" t="n"/>
@@ -26238,7 +26238,7 @@
       </c>
       <c r="G151" s="2" t="n"/>
       <c r="H151" s="35" t="n">
-        <v>3.5</v>
+        <v>4.1</v>
       </c>
       <c r="I151" s="35" t="n">
         <v>3</v>
@@ -26268,7 +26268,7 @@
       </c>
       <c r="G152" s="2" t="n"/>
       <c r="H152" s="35" t="n">
-        <v>3.5</v>
+        <v>1</v>
       </c>
       <c r="I152" s="35" t="n">
         <v>3</v>
@@ -26298,66 +26298,59 @@
       </c>
       <c r="G153" s="2" t="n"/>
       <c r="H153" s="35" t="n">
-        <v>3.5</v>
+        <v>4.1</v>
       </c>
       <c r="I153" s="35" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="154" ht="62" customHeight="1">
-      <c r="A154" s="9" t="n"/>
-      <c r="B154" s="34" t="inlineStr">
-        <is>
-          <t>INTERIORES (    )</t>
-        </is>
-      </c>
-      <c r="C154" s="9">
-        <f>IF(COUNT(H154,I154)&lt;2,"",TEXT(H154,"0.00")&amp;" x "&amp;TEXT(I154,"0.00"))</f>
-        <v/>
-      </c>
-      <c r="D154" s="8">
-        <f>IF(COUNT(H154,I154)&lt;2,"",ROUND(H154*I154,2))</f>
-        <v/>
-      </c>
-      <c r="E154" s="25" t="n">
-        <v>25</v>
-      </c>
-      <c r="F154" s="28">
-        <f>IF(D154="","",ROUND(D154*E154,1))</f>
-        <v/>
-      </c>
+    <row r="154" ht="39.7" customHeight="1">
+      <c r="A154" s="16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B154" s="33" t="inlineStr">
+        <is>
+          <t>TECHOS O CIELORRASOS</t>
+        </is>
+      </c>
+      <c r="C154" s="9" t="n"/>
+      <c r="D154" s="9" t="n"/>
+      <c r="E154" s="9" t="n"/>
+      <c r="F154" s="9" t="n"/>
       <c r="G154" s="2" t="n"/>
-      <c r="H154" s="35" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="I154" s="35" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="155" ht="39.7" customHeight="1">
-      <c r="A155" s="16" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B155" s="33" t="inlineStr">
-        <is>
-          <t>TECHOS O CIELORRASOS</t>
-        </is>
-      </c>
-      <c r="C155" s="9" t="n"/>
-      <c r="D155" s="9" t="n"/>
-      <c r="E155" s="9" t="n"/>
-      <c r="F155" s="9" t="n"/>
+      <c r="H154" s="2" t="n"/>
+      <c r="I154" s="2" t="n"/>
+    </row>
+    <row r="155" ht="62" customHeight="1">
+      <c r="A155" s="9" t="n"/>
+      <c r="B155" s="34" t="inlineStr">
+        <is>
+          <t>TECHO NO AISLADO</t>
+        </is>
+      </c>
+      <c r="C155" s="9" t="inlineStr"/>
+      <c r="D155" s="8">
+        <f>IF(COUNT(H155,I155)&lt;2,"",ROUND(H155*I155,2))</f>
+        <v/>
+      </c>
+      <c r="E155" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="F155" s="28">
+        <f>IF(D155="","",ROUND(D155*E155,1))</f>
+        <v/>
+      </c>
       <c r="G155" s="2" t="n"/>
-      <c r="H155" s="2" t="n"/>
-      <c r="I155" s="2" t="n"/>
+      <c r="H155" s="35" t="n"/>
+      <c r="I155" s="35" t="n"/>
     </row>
     <row r="156" ht="62" customHeight="1">
       <c r="A156" s="9" t="n"/>
       <c r="B156" s="34" t="inlineStr">
         <is>
-          <t>TECHO NO AISLADO</t>
+          <t>TECHO AISLADO</t>
         </is>
       </c>
       <c r="C156" s="9" t="inlineStr"/>
@@ -26366,7 +26359,7 @@
         <v/>
       </c>
       <c r="E156" s="25" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F156" s="28">
         <f>IF(D156="","",ROUND(D156*E156,1))</f>
@@ -26376,20 +26369,23 @@
       <c r="H156" s="35" t="n"/>
       <c r="I156" s="35" t="n"/>
     </row>
-    <row r="157" ht="62" customHeight="1">
+    <row r="157" ht="39.7" customHeight="1">
       <c r="A157" s="9" t="n"/>
       <c r="B157" s="34" t="inlineStr">
         <is>
-          <t>TECHO AISLADO</t>
-        </is>
-      </c>
-      <c r="C157" s="9" t="inlineStr"/>
-      <c r="D157" s="8">
-        <f>IF(COUNT(H157,I157)&lt;2,"",ROUND(H157*I157,2))</f>
-        <v/>
+          <t>TECHO ENTREPISO</t>
+        </is>
+      </c>
+      <c r="C157" s="9" t="inlineStr">
+        <is>
+          <t>por croquis</t>
+        </is>
+      </c>
+      <c r="D157" s="8" t="n">
+        <v>4.1</v>
       </c>
       <c r="E157" s="25" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F157" s="28">
         <f>IF(D157="","",ROUND(D157*E157,1))</f>
@@ -26400,67 +26396,64 @@
       <c r="I157" s="35" t="n"/>
     </row>
     <row r="158" ht="39.7" customHeight="1">
-      <c r="A158" s="9" t="n"/>
-      <c r="B158" s="34" t="inlineStr">
-        <is>
-          <t>TECHO ENTREPISO</t>
-        </is>
-      </c>
-      <c r="C158" s="9" t="inlineStr">
+      <c r="A158" s="16" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B158" s="33" t="inlineStr">
+        <is>
+          <t>PISO</t>
+        </is>
+      </c>
+      <c r="C158" s="9" t="n"/>
+      <c r="D158" s="9" t="n"/>
+      <c r="E158" s="9" t="n"/>
+      <c r="F158" s="9" t="n"/>
+      <c r="G158" s="2" t="n"/>
+      <c r="H158" s="2" t="n"/>
+      <c r="I158" s="2" t="n"/>
+    </row>
+    <row r="159" ht="39.7" customHeight="1">
+      <c r="A159" s="9" t="n"/>
+      <c r="B159" s="34" t="inlineStr">
+        <is>
+          <t>SOBRE TIERRA</t>
+        </is>
+      </c>
+      <c r="C159" s="9" t="inlineStr">
         <is>
           <t>por croquis</t>
         </is>
       </c>
-      <c r="D158" s="8" t="n">
-        <v>12.25</v>
-      </c>
-      <c r="E158" s="25" t="n">
-        <v>15</v>
-      </c>
-      <c r="F158" s="28">
-        <f>IF(D158="","",ROUND(D158*E158,1))</f>
-        <v/>
-      </c>
-      <c r="G158" s="2" t="n"/>
-      <c r="H158" s="35" t="n"/>
-      <c r="I158" s="35" t="n"/>
-    </row>
-    <row r="159" ht="39.7" customHeight="1">
-      <c r="A159" s="16" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B159" s="33" t="inlineStr">
-        <is>
-          <t>PISO</t>
-        </is>
-      </c>
-      <c r="C159" s="9" t="n"/>
-      <c r="D159" s="9" t="n"/>
-      <c r="E159" s="9" t="n"/>
-      <c r="F159" s="9" t="n"/>
+      <c r="D159" s="8" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="E159" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="F159" s="28">
+        <f>IF(D159="","",ROUND(D159*E159,1))</f>
+        <v/>
+      </c>
       <c r="G159" s="2" t="n"/>
-      <c r="H159" s="2" t="n"/>
-      <c r="I159" s="2" t="n"/>
-    </row>
-    <row r="160" ht="39.7" customHeight="1">
+      <c r="H159" s="35" t="n"/>
+      <c r="I159" s="35" t="n"/>
+    </row>
+    <row r="160" ht="62" customHeight="1">
       <c r="A160" s="9" t="n"/>
       <c r="B160" s="34" t="inlineStr">
         <is>
-          <t>SOBRE TIERRA</t>
-        </is>
-      </c>
-      <c r="C160" s="9" t="inlineStr">
-        <is>
-          <t>por croquis</t>
-        </is>
-      </c>
-      <c r="D160" s="8" t="n">
-        <v>12.25</v>
+          <t>SOBRE LOCAL OCUPADO</t>
+        </is>
+      </c>
+      <c r="C160" s="9" t="inlineStr"/>
+      <c r="D160" s="8">
+        <f>IF(COUNT(H160,I160)&lt;2,"",ROUND(H160*I160,2))</f>
+        <v/>
       </c>
       <c r="E160" s="25" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F160" s="28">
         <f>IF(D160="","",ROUND(D160*E160,1))</f>
@@ -26470,57 +26463,60 @@
       <c r="H160" s="35" t="n"/>
       <c r="I160" s="35" t="n"/>
     </row>
-    <row r="161" ht="62" customHeight="1">
-      <c r="A161" s="9" t="n"/>
-      <c r="B161" s="34" t="inlineStr">
-        <is>
-          <t>SOBRE LOCAL OCUPADO</t>
-        </is>
-      </c>
-      <c r="C161" s="9" t="inlineStr"/>
-      <c r="D161" s="8">
-        <f>IF(COUNT(H161,I161)&lt;2,"",ROUND(H161*I161,2))</f>
-        <v/>
-      </c>
-      <c r="E161" s="25" t="n">
-        <v>15</v>
-      </c>
-      <c r="F161" s="28">
-        <f>IF(D161="","",ROUND(D161*E161,1))</f>
-        <v/>
-      </c>
+    <row r="161" ht="39.7" customHeight="1">
+      <c r="A161" s="16" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B161" s="33" t="inlineStr">
+        <is>
+          <t>INFILTRACION</t>
+        </is>
+      </c>
+      <c r="C161" s="9" t="n"/>
+      <c r="D161" s="16" t="inlineStr">
+        <is>
+          <t>VOLUMEN (m3)</t>
+        </is>
+      </c>
+      <c r="E161" s="9" t="n"/>
+      <c r="F161" s="9" t="n"/>
       <c r="G161" s="2" t="n"/>
-      <c r="H161" s="35" t="n"/>
-      <c r="I161" s="35" t="n"/>
+      <c r="H161" s="2" t="n"/>
+      <c r="I161" s="2" t="n"/>
     </row>
     <row r="162" ht="39.7" customHeight="1">
-      <c r="A162" s="16" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B162" s="33" t="inlineStr">
-        <is>
-          <t>INFILTRACION</t>
-        </is>
-      </c>
-      <c r="C162" s="9" t="n"/>
-      <c r="D162" s="16" t="inlineStr">
-        <is>
-          <t>VOLUMEN (m3)</t>
-        </is>
-      </c>
-      <c r="E162" s="9" t="n"/>
-      <c r="F162" s="9" t="n"/>
+      <c r="A162" s="9" t="n"/>
+      <c r="B162" s="34" t="inlineStr">
+        <is>
+          <t>UNA PARED EXTERIOR</t>
+        </is>
+      </c>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>4.10 m2 x 3.00</t>
+        </is>
+      </c>
+      <c r="D162" s="8" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="E162" s="25" t="n">
+        <v>6</v>
+      </c>
+      <c r="F162" s="28">
+        <f>IF(D162="","",ROUND(D162*E162,1))</f>
+        <v/>
+      </c>
       <c r="G162" s="2" t="n"/>
-      <c r="H162" s="2" t="n"/>
-      <c r="I162" s="2" t="n"/>
+      <c r="H162" s="35" t="n"/>
+      <c r="I162" s="35" t="n"/>
     </row>
     <row r="163" ht="62" customHeight="1">
       <c r="A163" s="9" t="n"/>
       <c r="B163" s="34" t="inlineStr">
         <is>
-          <t>UNA PARED EXTERIOR</t>
+          <t>DOS PAREDES EXTERIORES</t>
         </is>
       </c>
       <c r="C163" s="9" t="inlineStr"/>
@@ -26529,7 +26525,7 @@
         <v/>
       </c>
       <c r="E163" s="25" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F163" s="28">
         <f>IF(D163="","",ROUND(D163*E163,1))</f>
@@ -26539,23 +26535,20 @@
       <c r="H163" s="35" t="n"/>
       <c r="I163" s="35" t="n"/>
     </row>
-    <row r="164" ht="39.7" customHeight="1">
+    <row r="164" ht="62" customHeight="1">
       <c r="A164" s="9" t="n"/>
       <c r="B164" s="34" t="inlineStr">
         <is>
-          <t>DOS PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C164" s="9" t="inlineStr">
-        <is>
-          <t>12.25 m2 x 3.00</t>
-        </is>
-      </c>
-      <c r="D164" s="8" t="n">
-        <v>36.75</v>
+          <t>TRES O MAS PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C164" s="9" t="inlineStr"/>
+      <c r="D164" s="8">
+        <f>IF(COUNT(H164,I164)&lt;2,"",ROUND(H164*I164,2))</f>
+        <v/>
       </c>
       <c r="E164" s="25" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F164" s="28">
         <f>IF(D164="","",ROUND(D164*E164,1))</f>
@@ -26565,96 +26558,91 @@
       <c r="H164" s="35" t="n"/>
       <c r="I164" s="35" t="n"/>
     </row>
-    <row r="165" ht="62" customHeight="1">
-      <c r="A165" s="9" t="n"/>
-      <c r="B165" s="34" t="inlineStr">
-        <is>
-          <t>TRES O MAS PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C165" s="9" t="inlineStr"/>
-      <c r="D165" s="8">
-        <f>IF(COUNT(H165,I165)&lt;2,"",ROUND(H165*I165,2))</f>
-        <v/>
-      </c>
-      <c r="E165" s="25" t="n">
-        <v>12</v>
-      </c>
-      <c r="F165" s="28">
-        <f>IF(D165="","",ROUND(D165*E165,1))</f>
+    <row r="165" ht="70" customHeight="1">
+      <c r="A165" s="16" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B165" s="33" t="inlineStr">
+        <is>
+          <t>SUBTOTAL</t>
+        </is>
+      </c>
+      <c r="C165" s="9" t="n"/>
+      <c r="D165" s="9" t="n"/>
+      <c r="E165" s="9" t="n"/>
+      <c r="F165" s="36">
+        <f>IF(F144="",0,F144)+IF(F146="",0,F146)+IF(F147="",0,F147)+IF(F148="",0,F148)+IF(F149="",0,F149)+IF(F150="",0,F150)+IF(F151="",0,F151)+IF(F152="",0,F152)+IF(F153="",0,F153)+IF(F155="",0,F155)+IF(F156="",0,F156)+IF(F157="",0,F157)+IF(F159="",0,F159)+IF(F160="",0,F160)+IF(F162="",0,F162)+IF(F163="",0,F163)+IF(F164="",0,F164)</f>
         <v/>
       </c>
       <c r="G165" s="2" t="n"/>
-      <c r="H165" s="35" t="n"/>
-      <c r="I165" s="35" t="n"/>
-    </row>
-    <row r="166" ht="70" customHeight="1">
+      <c r="H165" s="2" t="n"/>
+      <c r="I165" s="2" t="n"/>
+    </row>
+    <row r="166" ht="47" customHeight="1">
       <c r="A166" s="16" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B166" s="33" t="inlineStr">
         <is>
-          <t>SUBTOTAL</t>
-        </is>
-      </c>
-      <c r="C166" s="9" t="n"/>
-      <c r="D166" s="9" t="n"/>
-      <c r="E166" s="9" t="n"/>
+          <t>PERDIDA TOTAL</t>
+        </is>
+      </c>
+      <c r="C166" s="9">
+        <f>TEXT(F165,"0.00")&amp;"  X  "&amp;Datos_balance!$B$4&amp;" (FI)  X  "&amp;Datos_balance!$B$5&amp;" (FO)  X  "&amp;Datos_balance!$B$6&amp;" (FZ)"</f>
+        <v/>
+      </c>
+      <c r="D166" s="2" t="n"/>
+      <c r="E166" s="2" t="n"/>
       <c r="F166" s="36">
-        <f>IF(F144="",0,F144)+IF(F145="",0,F145)+IF(F147="",0,F147)+IF(F148="",0,F148)+IF(F149="",0,F149)+IF(F150="",0,F150)+IF(F151="",0,F151)+IF(F152="",0,F152)+IF(F153="",0,F153)+IF(F154="",0,F154)+IF(F156="",0,F156)+IF(F157="",0,F157)+IF(F158="",0,F158)+IF(F160="",0,F160)+IF(F161="",0,F161)+IF(F163="",0,F163)+IF(F164="",0,F164)+IF(F165="",0,F165)</f>
+        <f>ROUND(F165*Datos_balance!$B$4*Datos_balance!$B$5*Datos_balance!$B$6,1)</f>
         <v/>
       </c>
       <c r="G166" s="2" t="n"/>
       <c r="H166" s="2" t="n"/>
       <c r="I166" s="2" t="n"/>
     </row>
-    <row r="167" ht="47" customHeight="1">
-      <c r="A167" s="16" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B167" s="33" t="inlineStr">
-        <is>
-          <t>PERDIDA TOTAL</t>
-        </is>
-      </c>
-      <c r="C167" s="9">
-        <f>TEXT(F166,"0.00")&amp;"  X  "&amp;Datos_balance!$B$4&amp;" (FI)  X  "&amp;Datos_balance!$B$5&amp;" (FO)  X  "&amp;Datos_balance!$B$6&amp;" (FZ)"</f>
-        <v/>
-      </c>
+    <row r="167">
+      <c r="A167" s="2" t="n"/>
+      <c r="B167" s="2" t="n"/>
+      <c r="C167" s="2" t="n"/>
       <c r="D167" s="2" t="n"/>
       <c r="E167" s="2" t="n"/>
-      <c r="F167" s="36">
-        <f>ROUND(F166*Datos_balance!$B$4*Datos_balance!$B$5*Datos_balance!$B$6,1)</f>
-        <v/>
-      </c>
+      <c r="F167" s="2" t="n"/>
       <c r="G167" s="2" t="n"/>
       <c r="H167" s="2" t="n"/>
       <c r="I167" s="2" t="n"/>
     </row>
-    <row r="168">
-      <c r="A168" s="2" t="n"/>
-      <c r="B168" s="2" t="n"/>
-      <c r="C168" s="2" t="n"/>
+    <row r="168" ht="62" customHeight="1">
+      <c r="A168" s="9" t="n"/>
+      <c r="B168" s="10" t="inlineStr">
+        <is>
+          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
+        </is>
+      </c>
+      <c r="C168" s="9">
+        <f>TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2,"0")&amp;" - "&amp;TEXT(Datos_balance!$B$11,"0")&amp;" = "&amp;TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2-Datos_balance!$B$11,"0")&amp;" C"</f>
+        <v/>
+      </c>
       <c r="D168" s="2" t="n"/>
       <c r="E168" s="2" t="n"/>
-      <c r="F168" s="2" t="n"/>
+      <c r="F168" s="9" t="n"/>
       <c r="G168" s="2" t="n"/>
       <c r="H168" s="2" t="n"/>
       <c r="I168" s="2" t="n"/>
     </row>
-    <row r="169" ht="62" customHeight="1">
+    <row r="169" ht="39.7" customHeight="1">
       <c r="A169" s="9" t="n"/>
       <c r="B169" s="10" t="inlineStr">
         <is>
-          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
-        </is>
-      </c>
-      <c r="C169" s="9">
-        <f>TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2,"0")&amp;" - "&amp;TEXT(Datos_balance!$B$11,"0")&amp;" = "&amp;TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2-Datos_balance!$B$11,"0")&amp;" C"</f>
+          <t>Kcal/h por elemento</t>
+        </is>
+      </c>
+      <c r="C169" s="8">
+        <f>ROUND(Datos_balance!$B$14*Datos_balance!$B$15,2)</f>
         <v/>
       </c>
       <c r="D169" s="2" t="n"/>
@@ -26668,11 +26656,11 @@
       <c r="A170" s="9" t="n"/>
       <c r="B170" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h por elemento</t>
-        </is>
-      </c>
-      <c r="C170" s="8">
-        <f>ROUND(Datos_balance!$B$14*Datos_balance!$B$15,2)</f>
+          <t>Elementos necesarios</t>
+        </is>
+      </c>
+      <c r="C170" s="25">
+        <f>ROUNDUP(F166/(Datos_balance!$B$14*Datos_balance!$B$15),0)</f>
         <v/>
       </c>
       <c r="D170" s="2" t="n"/>
@@ -26686,11 +26674,11 @@
       <c r="A171" s="9" t="n"/>
       <c r="B171" s="10" t="inlineStr">
         <is>
-          <t>Elementos necesarios</t>
+          <t>Ancho del radiador (cm)</t>
         </is>
       </c>
       <c r="C171" s="25">
-        <f>ROUNDUP(F167/(Datos_balance!$B$14*Datos_balance!$B$15),0)</f>
+        <f>ROUNDUP(F166/(Datos_balance!$B$14*Datos_balance!$B$15),0)*Datos_balance!$B$16</f>
         <v/>
       </c>
       <c r="D171" s="2" t="n"/>
@@ -26701,37 +26689,30 @@
       <c r="I171" s="2" t="n"/>
     </row>
     <row r="172" ht="39.7" customHeight="1">
-      <c r="A172" s="9" t="n"/>
-      <c r="B172" s="10" t="inlineStr">
-        <is>
-          <t>Ancho del radiador (cm)</t>
-        </is>
-      </c>
-      <c r="C172" s="25">
-        <f>ROUNDUP(F167/(Datos_balance!$B$14*Datos_balance!$B$15),0)*Datos_balance!$B$16</f>
-        <v/>
-      </c>
-      <c r="D172" s="2" t="n"/>
-      <c r="E172" s="2" t="n"/>
-      <c r="F172" s="9" t="n"/>
+      <c r="A172" s="13" t="n"/>
+      <c r="B172" s="14" t="inlineStr">
+        <is>
+          <t>Radiador adoptado</t>
+        </is>
+      </c>
+      <c r="C172" s="13">
+        <f>Datos_balance!$B$13</f>
+        <v/>
+      </c>
+      <c r="D172" s="20" t="n"/>
+      <c r="E172" s="20" t="n"/>
+      <c r="F172" s="13" t="n"/>
       <c r="G172" s="2" t="n"/>
       <c r="H172" s="2" t="n"/>
       <c r="I172" s="2" t="n"/>
     </row>
-    <row r="173" ht="39.7" customHeight="1">
-      <c r="A173" s="13" t="n"/>
-      <c r="B173" s="14" t="inlineStr">
-        <is>
-          <t>Radiador adoptado</t>
-        </is>
-      </c>
-      <c r="C173" s="13">
-        <f>Datos_balance!$B$13</f>
-        <v/>
-      </c>
-      <c r="D173" s="20" t="n"/>
-      <c r="E173" s="20" t="n"/>
-      <c r="F173" s="13" t="n"/>
+    <row r="173">
+      <c r="A173" s="2" t="n"/>
+      <c r="B173" s="2" t="n"/>
+      <c r="C173" s="2" t="n"/>
+      <c r="D173" s="2" t="n"/>
+      <c r="E173" s="2" t="n"/>
+      <c r="F173" s="2" t="n"/>
       <c r="G173" s="2" t="n"/>
       <c r="H173" s="2" t="n"/>
       <c r="I173" s="2" t="n"/>
@@ -26747,8 +26728,12 @@
       <c r="H174" s="2" t="n"/>
       <c r="I174" s="2" t="n"/>
     </row>
-    <row r="175">
-      <c r="A175" s="2" t="n"/>
+    <row r="175" ht="39.7" customHeight="1">
+      <c r="A175" s="5" t="inlineStr">
+        <is>
+          <t>LOCAL  09 - Dormitorio suite   (PB)</t>
+        </is>
+      </c>
       <c r="B175" s="2" t="n"/>
       <c r="C175" s="2" t="n"/>
       <c r="D175" s="2" t="n"/>
@@ -26759,79 +26744,94 @@
       <c r="I175" s="2" t="n"/>
     </row>
     <row r="176" ht="39.7" customHeight="1">
-      <c r="A176" s="5" t="inlineStr">
-        <is>
-          <t>LOCAL  10 - Bano suite   (PB)</t>
-        </is>
-      </c>
-      <c r="B176" s="2" t="n"/>
-      <c r="C176" s="2" t="n"/>
-      <c r="D176" s="2" t="n"/>
-      <c r="E176" s="2" t="n"/>
-      <c r="F176" s="2" t="n"/>
+      <c r="A176" s="3" t="inlineStr">
+        <is>
+          <t>Nro</t>
+        </is>
+      </c>
+      <c r="B176" s="3" t="inlineStr">
+        <is>
+          <t>DESCRIPCION</t>
+        </is>
+      </c>
+      <c r="C176" s="3" t="inlineStr">
+        <is>
+          <t>DIMENSIONES (m)</t>
+        </is>
+      </c>
+      <c r="D176" s="3" t="inlineStr">
+        <is>
+          <t>AREA (m2)</t>
+        </is>
+      </c>
+      <c r="E176" s="3" t="inlineStr">
+        <is>
+          <t>FACTOR</t>
+        </is>
+      </c>
+      <c r="F176" s="3" t="inlineStr">
+        <is>
+          <t>PERDIDA CALOR (Kcal/h)</t>
+        </is>
+      </c>
       <c r="G176" s="2" t="n"/>
       <c r="H176" s="2" t="n"/>
       <c r="I176" s="2" t="n"/>
     </row>
     <row r="177" ht="39.7" customHeight="1">
-      <c r="A177" s="3" t="inlineStr">
-        <is>
-          <t>Nro</t>
-        </is>
-      </c>
-      <c r="B177" s="3" t="inlineStr">
-        <is>
-          <t>DESCRIPCION</t>
-        </is>
-      </c>
-      <c r="C177" s="3" t="inlineStr">
-        <is>
-          <t>DIMENSIONES (m)</t>
-        </is>
-      </c>
-      <c r="D177" s="3" t="inlineStr">
-        <is>
-          <t>AREA (m2)</t>
-        </is>
-      </c>
-      <c r="E177" s="3" t="inlineStr">
-        <is>
-          <t>FACTOR</t>
-        </is>
-      </c>
-      <c r="F177" s="3" t="inlineStr">
-        <is>
-          <t>PERDIDA CALOR (Kcal/h)</t>
-        </is>
-      </c>
+      <c r="A177" s="16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B177" s="33" t="inlineStr">
+        <is>
+          <t>VENTANA</t>
+        </is>
+      </c>
+      <c r="C177" s="9" t="n"/>
+      <c r="D177" s="9" t="n"/>
+      <c r="E177" s="9" t="n"/>
+      <c r="F177" s="9" t="n"/>
       <c r="G177" s="2" t="n"/>
       <c r="H177" s="2" t="n"/>
       <c r="I177" s="2" t="n"/>
     </row>
-    <row r="178" ht="39.7" customHeight="1">
-      <c r="A178" s="16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B178" s="33" t="inlineStr">
-        <is>
-          <t>VENTANA</t>
-        </is>
-      </c>
-      <c r="C178" s="9" t="n"/>
-      <c r="D178" s="9" t="n"/>
-      <c r="E178" s="9" t="n"/>
-      <c r="F178" s="9" t="n"/>
+    <row r="178" ht="62" customHeight="1">
+      <c r="A178" s="9" t="n"/>
+      <c r="B178" s="34" t="inlineStr">
+        <is>
+          <t>VA01 (2)</t>
+        </is>
+      </c>
+      <c r="C178" s="9">
+        <f>IF(COUNT(H178,I178)&lt;2,"",TEXT(H178,"0.00")&amp;" x "&amp;TEXT(I178,"0.00"))</f>
+        <v/>
+      </c>
+      <c r="D178" s="8">
+        <f>IF(COUNT(H178,I178)&lt;2,"",ROUND(H178*I178,2))</f>
+        <v/>
+      </c>
+      <c r="E178" s="25" t="n">
+        <v>60</v>
+      </c>
+      <c r="F178" s="28">
+        <f>IF(D178="","",ROUND(D178*E178,1))</f>
+        <v/>
+      </c>
       <c r="G178" s="2" t="n"/>
-      <c r="H178" s="2" t="n"/>
-      <c r="I178" s="2" t="n"/>
+      <c r="H178" s="35" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I178" s="35" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="179" ht="62" customHeight="1">
       <c r="A179" s="9" t="n"/>
       <c r="B179" s="34" t="inlineStr">
         <is>
-          <t>VA02</t>
+          <t>PV03</t>
         </is>
       </c>
       <c r="C179" s="9">
@@ -26851,10 +26851,10 @@
       </c>
       <c r="G179" s="2" t="n"/>
       <c r="H179" s="35" t="n">
-        <v>0.75</v>
+        <v>1.76</v>
       </c>
       <c r="I179" s="35" t="n">
-        <v>2.15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="180" ht="39.7" customHeight="1">
@@ -27004,7 +27004,7 @@
       </c>
       <c r="G185" s="2" t="n"/>
       <c r="H185" s="35" t="n">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="I185" s="35" t="n">
         <v>3</v>
@@ -27034,7 +27034,7 @@
       </c>
       <c r="G186" s="2" t="n"/>
       <c r="H186" s="35" t="n">
-        <v>1.7</v>
+        <v>3.5</v>
       </c>
       <c r="I186" s="35" t="n">
         <v>3</v>
@@ -27064,7 +27064,7 @@
       </c>
       <c r="G187" s="2" t="n"/>
       <c r="H187" s="35" t="n">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="I187" s="35" t="n">
         <v>3</v>
@@ -27094,7 +27094,7 @@
       </c>
       <c r="G188" s="2" t="n"/>
       <c r="H188" s="35" t="n">
-        <v>1.7</v>
+        <v>3.5</v>
       </c>
       <c r="I188" s="35" t="n">
         <v>3</v>
@@ -27178,7 +27178,7 @@
         </is>
       </c>
       <c r="D192" s="8" t="n">
-        <v>5.61</v>
+        <v>12.25</v>
       </c>
       <c r="E192" s="25" t="n">
         <v>15</v>
@@ -27223,7 +27223,7 @@
         </is>
       </c>
       <c r="D194" s="8" t="n">
-        <v>5.61</v>
+        <v>12.25</v>
       </c>
       <c r="E194" s="25" t="n">
         <v>10</v>
@@ -27282,20 +27282,17 @@
       <c r="H196" s="2" t="n"/>
       <c r="I196" s="2" t="n"/>
     </row>
-    <row r="197" ht="39.7" customHeight="1">
+    <row r="197" ht="62" customHeight="1">
       <c r="A197" s="9" t="n"/>
       <c r="B197" s="34" t="inlineStr">
         <is>
           <t>UNA PARED EXTERIOR</t>
         </is>
       </c>
-      <c r="C197" s="9" t="inlineStr">
-        <is>
-          <t>5.61 m2 x 3.00</t>
-        </is>
-      </c>
-      <c r="D197" s="8" t="n">
-        <v>16.83</v>
+      <c r="C197" s="9" t="inlineStr"/>
+      <c r="D197" s="8">
+        <f>IF(COUNT(H197,I197)&lt;2,"",ROUND(H197*I197,2))</f>
+        <v/>
       </c>
       <c r="E197" s="25" t="n">
         <v>6</v>
@@ -27308,17 +27305,20 @@
       <c r="H197" s="35" t="n"/>
       <c r="I197" s="35" t="n"/>
     </row>
-    <row r="198" ht="62" customHeight="1">
+    <row r="198" ht="39.7" customHeight="1">
       <c r="A198" s="9" t="n"/>
       <c r="B198" s="34" t="inlineStr">
         <is>
           <t>DOS PAREDES EXTERIORES</t>
         </is>
       </c>
-      <c r="C198" s="9" t="inlineStr"/>
-      <c r="D198" s="8">
-        <f>IF(COUNT(H198,I198)&lt;2,"",ROUND(H198*I198,2))</f>
-        <v/>
+      <c r="C198" s="9" t="inlineStr">
+        <is>
+          <t>12.25 m2 x 3.00</t>
+        </is>
+      </c>
+      <c r="D198" s="8" t="n">
+        <v>36.75</v>
       </c>
       <c r="E198" s="25" t="n">
         <v>9</v>
@@ -27369,7 +27369,7 @@
       <c r="D200" s="9" t="n"/>
       <c r="E200" s="9" t="n"/>
       <c r="F200" s="36">
-        <f>IF(F179="",0,F179)+IF(F181="",0,F181)+IF(F182="",0,F182)+IF(F183="",0,F183)+IF(F184="",0,F184)+IF(F185="",0,F185)+IF(F186="",0,F186)+IF(F187="",0,F187)+IF(F188="",0,F188)+IF(F190="",0,F190)+IF(F191="",0,F191)+IF(F192="",0,F192)+IF(F194="",0,F194)+IF(F195="",0,F195)+IF(F197="",0,F197)+IF(F198="",0,F198)+IF(F199="",0,F199)</f>
+        <f>IF(F178="",0,F178)+IF(F179="",0,F179)+IF(F181="",0,F181)+IF(F182="",0,F182)+IF(F183="",0,F183)+IF(F184="",0,F184)+IF(F185="",0,F185)+IF(F186="",0,F186)+IF(F187="",0,F187)+IF(F188="",0,F188)+IF(F190="",0,F190)+IF(F191="",0,F191)+IF(F192="",0,F192)+IF(F194="",0,F194)+IF(F195="",0,F195)+IF(F197="",0,F197)+IF(F198="",0,F198)+IF(F199="",0,F199)</f>
         <v/>
       </c>
       <c r="G200" s="2" t="n"/>
@@ -27434,11 +27434,11 @@
       <c r="A204" s="9" t="n"/>
       <c r="B204" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h del toallero Scala/Domino 80</t>
-        </is>
-      </c>
-      <c r="C204" s="25">
-        <f>ROUND(Datos_balance!$B$18*Datos_balance!$B$15,0)</f>
+          <t>Kcal/h por elemento</t>
+        </is>
+      </c>
+      <c r="C204" s="8">
+        <f>ROUND(Datos_balance!$B$14*Datos_balance!$B$15,2)</f>
         <v/>
       </c>
       <c r="D204" s="2" t="n"/>
@@ -27452,11 +27452,11 @@
       <c r="A205" s="9" t="n"/>
       <c r="B205" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h del toallero Scala/Domino 150</t>
+          <t>Elementos necesarios</t>
         </is>
       </c>
       <c r="C205" s="25">
-        <f>ROUND(Datos_balance!$B$19*Datos_balance!$B$15,0)</f>
+        <f>ROUNDUP(F201/(Datos_balance!$B$14*Datos_balance!$B$15),0)</f>
         <v/>
       </c>
       <c r="D205" s="2" t="n"/>
@@ -27466,15 +27466,15 @@
       <c r="H205" s="2" t="n"/>
       <c r="I205" s="2" t="n"/>
     </row>
-    <row r="206" ht="47" customHeight="1">
+    <row r="206" ht="39.7" customHeight="1">
       <c r="A206" s="9" t="n"/>
       <c r="B206" s="10" t="inlineStr">
         <is>
-          <t>Toalleros necesarios</t>
+          <t>Ancho del radiador (cm)</t>
         </is>
       </c>
       <c r="C206" s="25">
-        <f>IF(F201&lt;=Datos_balance!$B$18*Datos_balance!$B$15,1,ROUNDUP(F201/(Datos_balance!$B$19*Datos_balance!$B$15),0))</f>
+        <f>ROUNDUP(F201/(Datos_balance!$B$14*Datos_balance!$B$15),0)*Datos_balance!$B$16</f>
         <v/>
       </c>
       <c r="D206" s="2" t="n"/>
@@ -27484,15 +27484,15 @@
       <c r="H206" s="2" t="n"/>
       <c r="I206" s="2" t="n"/>
     </row>
-    <row r="207" ht="47" customHeight="1">
+    <row r="207" ht="39.7" customHeight="1">
       <c r="A207" s="13" t="n"/>
       <c r="B207" s="14" t="inlineStr">
         <is>
-          <t>Toallero adoptado</t>
+          <t>Radiador adoptado</t>
         </is>
       </c>
       <c r="C207" s="13">
-        <f>IF(F201&lt;=Datos_balance!$B$18*Datos_balance!$B$15,"Peisa Scala / Domino 80  (500 x 800 mm)","Peisa Scala / Domino 150  (500 x 1500 mm)")</f>
+        <f>Datos_balance!$B$13</f>
         <v/>
       </c>
       <c r="D207" s="20" t="n"/>
@@ -27527,7 +27527,7 @@
     <row r="210" ht="39.7" customHeight="1">
       <c r="A210" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  11 - Bano visitas   (PB)</t>
+          <t>LOCAL  10 - Bano suite   (PB)</t>
         </is>
       </c>
       <c r="B210" s="2" t="n"/>
@@ -27597,7 +27597,7 @@
       <c r="A213" s="9" t="n"/>
       <c r="B213" s="34" t="inlineStr">
         <is>
-          <t>(sin aberturas)</t>
+          <t>VA02</t>
         </is>
       </c>
       <c r="C213" s="9">
@@ -27616,8 +27616,12 @@
         <v/>
       </c>
       <c r="G213" s="2" t="n"/>
-      <c r="H213" s="35" t="n"/>
-      <c r="I213" s="35" t="n"/>
+      <c r="H213" s="35" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I213" s="35" t="n">
+        <v>2.15</v>
+      </c>
     </row>
     <row r="214" ht="39.7" customHeight="1">
       <c r="A214" s="16" t="inlineStr">
@@ -27766,7 +27770,7 @@
       </c>
       <c r="G219" s="2" t="n"/>
       <c r="H219" s="35" t="n">
-        <v>2.4</v>
+        <v>3.3</v>
       </c>
       <c r="I219" s="35" t="n">
         <v>3</v>
@@ -27796,7 +27800,7 @@
       </c>
       <c r="G220" s="2" t="n"/>
       <c r="H220" s="35" t="n">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
       <c r="I220" s="35" t="n">
         <v>3</v>
@@ -27826,7 +27830,7 @@
       </c>
       <c r="G221" s="2" t="n"/>
       <c r="H221" s="35" t="n">
-        <v>2.4</v>
+        <v>3.3</v>
       </c>
       <c r="I221" s="35" t="n">
         <v>3</v>
@@ -27856,7 +27860,7 @@
       </c>
       <c r="G222" s="2" t="n"/>
       <c r="H222" s="35" t="n">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
       <c r="I222" s="35" t="n">
         <v>3</v>
@@ -27940,7 +27944,7 @@
         </is>
       </c>
       <c r="D226" s="8" t="n">
-        <v>3.12</v>
+        <v>5.61</v>
       </c>
       <c r="E226" s="25" t="n">
         <v>15</v>
@@ -27985,7 +27989,7 @@
         </is>
       </c>
       <c r="D228" s="8" t="n">
-        <v>3.12</v>
+        <v>5.61</v>
       </c>
       <c r="E228" s="25" t="n">
         <v>10</v>
@@ -28053,11 +28057,11 @@
       </c>
       <c r="C231" s="9" t="inlineStr">
         <is>
-          <t>3.12 m2 x 3.00</t>
+          <t>5.61 m2 x 3.00</t>
         </is>
       </c>
       <c r="D231" s="8" t="n">
-        <v>9.359999999999999</v>
+        <v>16.83</v>
       </c>
       <c r="E231" s="25" t="n">
         <v>6</v>
@@ -28289,7 +28293,7 @@
     <row r="244" ht="39.7" customHeight="1">
       <c r="A244" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  13 - Dormitorio Norte   (PA)</t>
+          <t>LOCAL  11 - Bano visitas   (PB)</t>
         </is>
       </c>
       <c r="B244" s="2" t="n"/>
@@ -28359,7 +28363,7 @@
       <c r="A247" s="9" t="n"/>
       <c r="B247" s="34" t="inlineStr">
         <is>
-          <t>VA04</t>
+          <t>(sin aberturas)</t>
         </is>
       </c>
       <c r="C247" s="9">
@@ -28378,61 +28382,53 @@
         <v/>
       </c>
       <c r="G247" s="2" t="n"/>
-      <c r="H247" s="35" t="n">
-        <v>2</v>
-      </c>
-      <c r="I247" s="35" t="n">
-        <v>2.52</v>
-      </c>
-    </row>
-    <row r="248" ht="62" customHeight="1">
-      <c r="A248" s="9" t="n"/>
-      <c r="B248" s="34" t="inlineStr">
-        <is>
-          <t>VA05</t>
-        </is>
-      </c>
-      <c r="C248" s="9">
-        <f>IF(COUNT(H248,I248)&lt;2,"",TEXT(H248,"0.00")&amp;" x "&amp;TEXT(I248,"0.00"))</f>
-        <v/>
-      </c>
-      <c r="D248" s="8">
-        <f>IF(COUNT(H248,I248)&lt;2,"",ROUND(H248*I248,2))</f>
-        <v/>
-      </c>
-      <c r="E248" s="25" t="n">
-        <v>60</v>
-      </c>
-      <c r="F248" s="28">
-        <f>IF(D248="","",ROUND(D248*E248,1))</f>
-        <v/>
-      </c>
+      <c r="H247" s="35" t="n"/>
+      <c r="I247" s="35" t="n"/>
+    </row>
+    <row r="248" ht="39.7" customHeight="1">
+      <c r="A248" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B248" s="33" t="inlineStr">
+        <is>
+          <t>PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C248" s="9" t="n"/>
+      <c r="D248" s="9" t="n"/>
+      <c r="E248" s="9" t="n"/>
+      <c r="F248" s="9" t="n"/>
       <c r="G248" s="2" t="n"/>
-      <c r="H248" s="35" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="I248" s="35" t="n">
-        <v>2.52</v>
-      </c>
-    </row>
-    <row r="249" ht="39.7" customHeight="1">
-      <c r="A249" s="16" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B249" s="33" t="inlineStr">
-        <is>
-          <t>PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C249" s="9" t="n"/>
-      <c r="D249" s="9" t="n"/>
-      <c r="E249" s="9" t="n"/>
-      <c r="F249" s="9" t="n"/>
+      <c r="H248" s="2" t="n"/>
+      <c r="I248" s="2" t="n"/>
+    </row>
+    <row r="249" ht="62" customHeight="1">
+      <c r="A249" s="9" t="n"/>
+      <c r="B249" s="34" t="inlineStr">
+        <is>
+          <t>AISLADAS (    )</t>
+        </is>
+      </c>
+      <c r="C249" s="9">
+        <f>IF(COUNT(H249,I249)&lt;2,"",TEXT(H249,"0.00")&amp;" x "&amp;TEXT(I249,"0.00"))</f>
+        <v/>
+      </c>
+      <c r="D249" s="8">
+        <f>IF(COUNT(H249,I249)&lt;2,"",ROUND(H249*I249,2))</f>
+        <v/>
+      </c>
+      <c r="E249" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="F249" s="28">
+        <f>IF(D249="","",ROUND(D249*E249,1))</f>
+        <v/>
+      </c>
       <c r="G249" s="2" t="n"/>
-      <c r="H249" s="2" t="n"/>
-      <c r="I249" s="2" t="n"/>
+      <c r="H249" s="35" t="n"/>
+      <c r="I249" s="35" t="n"/>
     </row>
     <row r="250" ht="62" customHeight="1">
       <c r="A250" s="9" t="n"/>
@@ -28516,7 +28512,7 @@
       <c r="A253" s="9" t="n"/>
       <c r="B253" s="34" t="inlineStr">
         <is>
-          <t>AISLADAS (    )</t>
+          <t>INTERIORES (    )</t>
         </is>
       </c>
       <c r="C253" s="9">
@@ -28528,15 +28524,19 @@
         <v/>
       </c>
       <c r="E253" s="25" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F253" s="28">
         <f>IF(D253="","",ROUND(D253*E253,1))</f>
         <v/>
       </c>
       <c r="G253" s="2" t="n"/>
-      <c r="H253" s="35" t="n"/>
-      <c r="I253" s="35" t="n"/>
+      <c r="H253" s="35" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="I253" s="35" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="254" ht="62" customHeight="1">
       <c r="A254" s="9" t="n"/>
@@ -28562,7 +28562,7 @@
       </c>
       <c r="G254" s="2" t="n"/>
       <c r="H254" s="35" t="n">
-        <v>4.25</v>
+        <v>1.3</v>
       </c>
       <c r="I254" s="35" t="n">
         <v>3</v>
@@ -28592,7 +28592,7 @@
       </c>
       <c r="G255" s="2" t="n"/>
       <c r="H255" s="35" t="n">
-        <v>4</v>
+        <v>2.4</v>
       </c>
       <c r="I255" s="35" t="n">
         <v>3</v>
@@ -28622,66 +28622,59 @@
       </c>
       <c r="G256" s="2" t="n"/>
       <c r="H256" s="35" t="n">
-        <v>4.25</v>
+        <v>1.3</v>
       </c>
       <c r="I256" s="35" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="257" ht="62" customHeight="1">
-      <c r="A257" s="9" t="n"/>
-      <c r="B257" s="34" t="inlineStr">
-        <is>
-          <t>INTERIORES (    )</t>
-        </is>
-      </c>
-      <c r="C257" s="9">
-        <f>IF(COUNT(H257,I257)&lt;2,"",TEXT(H257,"0.00")&amp;" x "&amp;TEXT(I257,"0.00"))</f>
-        <v/>
-      </c>
-      <c r="D257" s="8">
-        <f>IF(COUNT(H257,I257)&lt;2,"",ROUND(H257*I257,2))</f>
-        <v/>
-      </c>
-      <c r="E257" s="25" t="n">
-        <v>25</v>
-      </c>
-      <c r="F257" s="28">
-        <f>IF(D257="","",ROUND(D257*E257,1))</f>
-        <v/>
-      </c>
+    <row r="257" ht="39.7" customHeight="1">
+      <c r="A257" s="16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B257" s="33" t="inlineStr">
+        <is>
+          <t>TECHOS O CIELORRASOS</t>
+        </is>
+      </c>
+      <c r="C257" s="9" t="n"/>
+      <c r="D257" s="9" t="n"/>
+      <c r="E257" s="9" t="n"/>
+      <c r="F257" s="9" t="n"/>
       <c r="G257" s="2" t="n"/>
-      <c r="H257" s="35" t="n">
-        <v>4</v>
-      </c>
-      <c r="I257" s="35" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="258" ht="39.7" customHeight="1">
-      <c r="A258" s="16" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B258" s="33" t="inlineStr">
-        <is>
-          <t>TECHOS O CIELORRASOS</t>
-        </is>
-      </c>
-      <c r="C258" s="9" t="n"/>
-      <c r="D258" s="9" t="n"/>
-      <c r="E258" s="9" t="n"/>
-      <c r="F258" s="9" t="n"/>
+      <c r="H257" s="2" t="n"/>
+      <c r="I257" s="2" t="n"/>
+    </row>
+    <row r="258" ht="62" customHeight="1">
+      <c r="A258" s="9" t="n"/>
+      <c r="B258" s="34" t="inlineStr">
+        <is>
+          <t>TECHO NO AISLADO</t>
+        </is>
+      </c>
+      <c r="C258" s="9" t="inlineStr"/>
+      <c r="D258" s="8">
+        <f>IF(COUNT(H258,I258)&lt;2,"",ROUND(H258*I258,2))</f>
+        <v/>
+      </c>
+      <c r="E258" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="F258" s="28">
+        <f>IF(D258="","",ROUND(D258*E258,1))</f>
+        <v/>
+      </c>
       <c r="G258" s="2" t="n"/>
-      <c r="H258" s="2" t="n"/>
-      <c r="I258" s="2" t="n"/>
+      <c r="H258" s="35" t="n"/>
+      <c r="I258" s="35" t="n"/>
     </row>
     <row r="259" ht="62" customHeight="1">
       <c r="A259" s="9" t="n"/>
       <c r="B259" s="34" t="inlineStr">
         <is>
-          <t>TECHO NO AISLADO</t>
+          <t>TECHO AISLADO</t>
         </is>
       </c>
       <c r="C259" s="9" t="inlineStr"/>
@@ -28690,7 +28683,7 @@
         <v/>
       </c>
       <c r="E259" s="25" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F259" s="28">
         <f>IF(D259="","",ROUND(D259*E259,1))</f>
@@ -28704,7 +28697,7 @@
       <c r="A260" s="9" t="n"/>
       <c r="B260" s="34" t="inlineStr">
         <is>
-          <t>TECHO AISLADO</t>
+          <t>TECHO ENTREPISO</t>
         </is>
       </c>
       <c r="C260" s="9" t="inlineStr">
@@ -28713,10 +28706,10 @@
         </is>
       </c>
       <c r="D260" s="8" t="n">
-        <v>17</v>
+        <v>3.12</v>
       </c>
       <c r="E260" s="25" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F260" s="28">
         <f>IF(D260="","",ROUND(D260*E260,1))</f>
@@ -28726,53 +28719,56 @@
       <c r="H260" s="35" t="n"/>
       <c r="I260" s="35" t="n"/>
     </row>
-    <row r="261" ht="62" customHeight="1">
-      <c r="A261" s="9" t="n"/>
-      <c r="B261" s="34" t="inlineStr">
-        <is>
-          <t>TECHO ENTREPISO</t>
-        </is>
-      </c>
-      <c r="C261" s="9" t="inlineStr"/>
-      <c r="D261" s="8">
-        <f>IF(COUNT(H261,I261)&lt;2,"",ROUND(H261*I261,2))</f>
-        <v/>
-      </c>
-      <c r="E261" s="25" t="n">
-        <v>15</v>
-      </c>
-      <c r="F261" s="28">
-        <f>IF(D261="","",ROUND(D261*E261,1))</f>
-        <v/>
-      </c>
+    <row r="261" ht="39.7" customHeight="1">
+      <c r="A261" s="16" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B261" s="33" t="inlineStr">
+        <is>
+          <t>PISO</t>
+        </is>
+      </c>
+      <c r="C261" s="9" t="n"/>
+      <c r="D261" s="9" t="n"/>
+      <c r="E261" s="9" t="n"/>
+      <c r="F261" s="9" t="n"/>
       <c r="G261" s="2" t="n"/>
-      <c r="H261" s="35" t="n"/>
-      <c r="I261" s="35" t="n"/>
+      <c r="H261" s="2" t="n"/>
+      <c r="I261" s="2" t="n"/>
     </row>
     <row r="262" ht="39.7" customHeight="1">
-      <c r="A262" s="16" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B262" s="33" t="inlineStr">
-        <is>
-          <t>PISO</t>
-        </is>
-      </c>
-      <c r="C262" s="9" t="n"/>
-      <c r="D262" s="9" t="n"/>
-      <c r="E262" s="9" t="n"/>
-      <c r="F262" s="9" t="n"/>
+      <c r="A262" s="9" t="n"/>
+      <c r="B262" s="34" t="inlineStr">
+        <is>
+          <t>SOBRE TIERRA</t>
+        </is>
+      </c>
+      <c r="C262" s="9" t="inlineStr">
+        <is>
+          <t>por croquis</t>
+        </is>
+      </c>
+      <c r="D262" s="8" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="E262" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="F262" s="28">
+        <f>IF(D262="","",ROUND(D262*E262,1))</f>
+        <v/>
+      </c>
       <c r="G262" s="2" t="n"/>
-      <c r="H262" s="2" t="n"/>
-      <c r="I262" s="2" t="n"/>
+      <c r="H262" s="35" t="n"/>
+      <c r="I262" s="35" t="n"/>
     </row>
     <row r="263" ht="62" customHeight="1">
       <c r="A263" s="9" t="n"/>
       <c r="B263" s="34" t="inlineStr">
         <is>
-          <t>SOBRE TIERRA</t>
+          <t>SOBRE LOCAL OCUPADO</t>
         </is>
       </c>
       <c r="C263" s="9" t="inlineStr"/>
@@ -28781,7 +28777,7 @@
         <v/>
       </c>
       <c r="E263" s="25" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F263" s="28">
         <f>IF(D263="","",ROUND(D263*E263,1))</f>
@@ -28792,59 +28788,59 @@
       <c r="I263" s="35" t="n"/>
     </row>
     <row r="264" ht="39.7" customHeight="1">
-      <c r="A264" s="9" t="n"/>
-      <c r="B264" s="34" t="inlineStr">
-        <is>
-          <t>SOBRE LOCAL OCUPADO</t>
-        </is>
-      </c>
-      <c r="C264" s="9" t="inlineStr">
-        <is>
-          <t>por croquis</t>
-        </is>
-      </c>
-      <c r="D264" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="E264" s="25" t="n">
-        <v>15</v>
-      </c>
-      <c r="F264" s="28">
-        <f>IF(D264="","",ROUND(D264*E264,1))</f>
-        <v/>
-      </c>
+      <c r="A264" s="16" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B264" s="33" t="inlineStr">
+        <is>
+          <t>INFILTRACION</t>
+        </is>
+      </c>
+      <c r="C264" s="9" t="n"/>
+      <c r="D264" s="16" t="inlineStr">
+        <is>
+          <t>VOLUMEN (m3)</t>
+        </is>
+      </c>
+      <c r="E264" s="9" t="n"/>
+      <c r="F264" s="9" t="n"/>
       <c r="G264" s="2" t="n"/>
-      <c r="H264" s="35" t="n"/>
-      <c r="I264" s="35" t="n"/>
+      <c r="H264" s="2" t="n"/>
+      <c r="I264" s="2" t="n"/>
     </row>
     <row r="265" ht="39.7" customHeight="1">
-      <c r="A265" s="16" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B265" s="33" t="inlineStr">
-        <is>
-          <t>INFILTRACION</t>
-        </is>
-      </c>
-      <c r="C265" s="9" t="n"/>
-      <c r="D265" s="16" t="inlineStr">
-        <is>
-          <t>VOLUMEN (m3)</t>
-        </is>
-      </c>
-      <c r="E265" s="9" t="n"/>
-      <c r="F265" s="9" t="n"/>
+      <c r="A265" s="9" t="n"/>
+      <c r="B265" s="34" t="inlineStr">
+        <is>
+          <t>UNA PARED EXTERIOR</t>
+        </is>
+      </c>
+      <c r="C265" s="9" t="inlineStr">
+        <is>
+          <t>3.12 m2 x 3.00</t>
+        </is>
+      </c>
+      <c r="D265" s="8" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="E265" s="25" t="n">
+        <v>6</v>
+      </c>
+      <c r="F265" s="28">
+        <f>IF(D265="","",ROUND(D265*E265,1))</f>
+        <v/>
+      </c>
       <c r="G265" s="2" t="n"/>
-      <c r="H265" s="2" t="n"/>
-      <c r="I265" s="2" t="n"/>
+      <c r="H265" s="35" t="n"/>
+      <c r="I265" s="35" t="n"/>
     </row>
     <row r="266" ht="62" customHeight="1">
       <c r="A266" s="9" t="n"/>
       <c r="B266" s="34" t="inlineStr">
         <is>
-          <t>UNA PARED EXTERIOR</t>
+          <t>DOS PAREDES EXTERIORES</t>
         </is>
       </c>
       <c r="C266" s="9" t="inlineStr"/>
@@ -28853,7 +28849,7 @@
         <v/>
       </c>
       <c r="E266" s="25" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F266" s="28">
         <f>IF(D266="","",ROUND(D266*E266,1))</f>
@@ -28863,23 +28859,20 @@
       <c r="H266" s="35" t="n"/>
       <c r="I266" s="35" t="n"/>
     </row>
-    <row r="267" ht="39.7" customHeight="1">
+    <row r="267" ht="62" customHeight="1">
       <c r="A267" s="9" t="n"/>
       <c r="B267" s="34" t="inlineStr">
         <is>
-          <t>DOS PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C267" s="9" t="inlineStr">
-        <is>
-          <t>17.00 m2 x 3.00</t>
-        </is>
-      </c>
-      <c r="D267" s="8" t="n">
-        <v>51</v>
+          <t>TRES O MAS PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C267" s="9" t="inlineStr"/>
+      <c r="D267" s="8">
+        <f>IF(COUNT(H267,I267)&lt;2,"",ROUND(H267*I267,2))</f>
+        <v/>
       </c>
       <c r="E267" s="25" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F267" s="28">
         <f>IF(D267="","",ROUND(D267*E267,1))</f>
@@ -28889,96 +28882,91 @@
       <c r="H267" s="35" t="n"/>
       <c r="I267" s="35" t="n"/>
     </row>
-    <row r="268" ht="62" customHeight="1">
-      <c r="A268" s="9" t="n"/>
-      <c r="B268" s="34" t="inlineStr">
-        <is>
-          <t>TRES O MAS PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C268" s="9" t="inlineStr"/>
-      <c r="D268" s="8">
-        <f>IF(COUNT(H268,I268)&lt;2,"",ROUND(H268*I268,2))</f>
-        <v/>
-      </c>
-      <c r="E268" s="25" t="n">
-        <v>12</v>
-      </c>
-      <c r="F268" s="28">
-        <f>IF(D268="","",ROUND(D268*E268,1))</f>
+    <row r="268" ht="70" customHeight="1">
+      <c r="A268" s="16" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B268" s="33" t="inlineStr">
+        <is>
+          <t>SUBTOTAL</t>
+        </is>
+      </c>
+      <c r="C268" s="9" t="n"/>
+      <c r="D268" s="9" t="n"/>
+      <c r="E268" s="9" t="n"/>
+      <c r="F268" s="36">
+        <f>IF(F247="",0,F247)+IF(F249="",0,F249)+IF(F250="",0,F250)+IF(F251="",0,F251)+IF(F252="",0,F252)+IF(F253="",0,F253)+IF(F254="",0,F254)+IF(F255="",0,F255)+IF(F256="",0,F256)+IF(F258="",0,F258)+IF(F259="",0,F259)+IF(F260="",0,F260)+IF(F262="",0,F262)+IF(F263="",0,F263)+IF(F265="",0,F265)+IF(F266="",0,F266)+IF(F267="",0,F267)</f>
         <v/>
       </c>
       <c r="G268" s="2" t="n"/>
-      <c r="H268" s="35" t="n"/>
-      <c r="I268" s="35" t="n"/>
-    </row>
-    <row r="269" ht="70" customHeight="1">
+      <c r="H268" s="2" t="n"/>
+      <c r="I268" s="2" t="n"/>
+    </row>
+    <row r="269" ht="47" customHeight="1">
       <c r="A269" s="16" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B269" s="33" t="inlineStr">
         <is>
-          <t>SUBTOTAL</t>
-        </is>
-      </c>
-      <c r="C269" s="9" t="n"/>
-      <c r="D269" s="9" t="n"/>
-      <c r="E269" s="9" t="n"/>
+          <t>PERDIDA TOTAL</t>
+        </is>
+      </c>
+      <c r="C269" s="9">
+        <f>TEXT(F268,"0.00")&amp;"  X  "&amp;Datos_balance!$B$4&amp;" (FI)  X  "&amp;Datos_balance!$B$5&amp;" (FO)  X  "&amp;Datos_balance!$B$6&amp;" (FZ)"</f>
+        <v/>
+      </c>
+      <c r="D269" s="2" t="n"/>
+      <c r="E269" s="2" t="n"/>
       <c r="F269" s="36">
-        <f>IF(F247="",0,F247)+IF(F248="",0,F248)+IF(F250="",0,F250)+IF(F251="",0,F251)+IF(F252="",0,F252)+IF(F253="",0,F253)+IF(F254="",0,F254)+IF(F255="",0,F255)+IF(F256="",0,F256)+IF(F257="",0,F257)+IF(F259="",0,F259)+IF(F260="",0,F260)+IF(F261="",0,F261)+IF(F263="",0,F263)+IF(F264="",0,F264)+IF(F266="",0,F266)+IF(F267="",0,F267)+IF(F268="",0,F268)</f>
+        <f>ROUND(F268*Datos_balance!$B$4*Datos_balance!$B$5*Datos_balance!$B$6,1)</f>
         <v/>
       </c>
       <c r="G269" s="2" t="n"/>
       <c r="H269" s="2" t="n"/>
       <c r="I269" s="2" t="n"/>
     </row>
-    <row r="270" ht="47" customHeight="1">
-      <c r="A270" s="16" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B270" s="33" t="inlineStr">
-        <is>
-          <t>PERDIDA TOTAL</t>
-        </is>
-      </c>
-      <c r="C270" s="9">
-        <f>TEXT(F269,"0.00")&amp;"  X  "&amp;Datos_balance!$B$4&amp;" (FI)  X  "&amp;Datos_balance!$B$5&amp;" (FO)  X  "&amp;Datos_balance!$B$6&amp;" (FZ)"</f>
-        <v/>
-      </c>
+    <row r="270">
+      <c r="A270" s="2" t="n"/>
+      <c r="B270" s="2" t="n"/>
+      <c r="C270" s="2" t="n"/>
       <c r="D270" s="2" t="n"/>
       <c r="E270" s="2" t="n"/>
-      <c r="F270" s="36">
-        <f>ROUND(F269*Datos_balance!$B$4*Datos_balance!$B$5*Datos_balance!$B$6,1)</f>
-        <v/>
-      </c>
+      <c r="F270" s="2" t="n"/>
       <c r="G270" s="2" t="n"/>
       <c r="H270" s="2" t="n"/>
       <c r="I270" s="2" t="n"/>
     </row>
-    <row r="271">
-      <c r="A271" s="2" t="n"/>
-      <c r="B271" s="2" t="n"/>
-      <c r="C271" s="2" t="n"/>
+    <row r="271" ht="62" customHeight="1">
+      <c r="A271" s="9" t="n"/>
+      <c r="B271" s="10" t="inlineStr">
+        <is>
+          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
+        </is>
+      </c>
+      <c r="C271" s="9">
+        <f>TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2,"0")&amp;" - "&amp;TEXT(Datos_balance!$B$11,"0")&amp;" = "&amp;TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2-Datos_balance!$B$11,"0")&amp;" C"</f>
+        <v/>
+      </c>
       <c r="D271" s="2" t="n"/>
       <c r="E271" s="2" t="n"/>
-      <c r="F271" s="2" t="n"/>
+      <c r="F271" s="9" t="n"/>
       <c r="G271" s="2" t="n"/>
       <c r="H271" s="2" t="n"/>
       <c r="I271" s="2" t="n"/>
     </row>
-    <row r="272" ht="62" customHeight="1">
+    <row r="272" ht="39.7" customHeight="1">
       <c r="A272" s="9" t="n"/>
       <c r="B272" s="10" t="inlineStr">
         <is>
-          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
-        </is>
-      </c>
-      <c r="C272" s="9">
-        <f>TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2,"0")&amp;" - "&amp;TEXT(Datos_balance!$B$11,"0")&amp;" = "&amp;TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2-Datos_balance!$B$11,"0")&amp;" C"</f>
+          <t>Kcal/h del toallero Scala/Domino 80</t>
+        </is>
+      </c>
+      <c r="C272" s="25">
+        <f>ROUND(Datos_balance!$B$18*Datos_balance!$B$15,0)</f>
         <v/>
       </c>
       <c r="D272" s="2" t="n"/>
@@ -28992,11 +28980,11 @@
       <c r="A273" s="9" t="n"/>
       <c r="B273" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h por elemento</t>
-        </is>
-      </c>
-      <c r="C273" s="8">
-        <f>ROUND(Datos_balance!$B$14*Datos_balance!$B$15,2)</f>
+          <t>Kcal/h del toallero Scala/Domino 150</t>
+        </is>
+      </c>
+      <c r="C273" s="25">
+        <f>ROUND(Datos_balance!$B$19*Datos_balance!$B$15,0)</f>
         <v/>
       </c>
       <c r="D273" s="2" t="n"/>
@@ -29006,15 +28994,15 @@
       <c r="H273" s="2" t="n"/>
       <c r="I273" s="2" t="n"/>
     </row>
-    <row r="274" ht="39.7" customHeight="1">
+    <row r="274" ht="47" customHeight="1">
       <c r="A274" s="9" t="n"/>
       <c r="B274" s="10" t="inlineStr">
         <is>
-          <t>Elementos necesarios</t>
+          <t>Toalleros necesarios</t>
         </is>
       </c>
       <c r="C274" s="25">
-        <f>ROUNDUP(F270/(Datos_balance!$B$14*Datos_balance!$B$15),0)</f>
+        <f>IF(F269&lt;=Datos_balance!$B$18*Datos_balance!$B$15,1,ROUNDUP(F269/(Datos_balance!$B$19*Datos_balance!$B$15),0))</f>
         <v/>
       </c>
       <c r="D274" s="2" t="n"/>
@@ -29024,38 +29012,31 @@
       <c r="H274" s="2" t="n"/>
       <c r="I274" s="2" t="n"/>
     </row>
-    <row r="275" ht="39.7" customHeight="1">
-      <c r="A275" s="9" t="n"/>
-      <c r="B275" s="10" t="inlineStr">
-        <is>
-          <t>Ancho del radiador (cm)</t>
-        </is>
-      </c>
-      <c r="C275" s="25">
-        <f>ROUNDUP(F270/(Datos_balance!$B$14*Datos_balance!$B$15),0)*Datos_balance!$B$16</f>
-        <v/>
-      </c>
-      <c r="D275" s="2" t="n"/>
-      <c r="E275" s="2" t="n"/>
-      <c r="F275" s="9" t="n"/>
+    <row r="275" ht="47" customHeight="1">
+      <c r="A275" s="13" t="n"/>
+      <c r="B275" s="14" t="inlineStr">
+        <is>
+          <t>Toallero adoptado</t>
+        </is>
+      </c>
+      <c r="C275" s="13">
+        <f>IF(F269&lt;=Datos_balance!$B$18*Datos_balance!$B$15,"Peisa Scala / Domino 80  (500 x 800 mm)","Peisa Scala / Domino 150  (500 x 1500 mm)")</f>
+        <v/>
+      </c>
+      <c r="D275" s="20" t="n"/>
+      <c r="E275" s="20" t="n"/>
+      <c r="F275" s="13" t="n"/>
       <c r="G275" s="2" t="n"/>
       <c r="H275" s="2" t="n"/>
       <c r="I275" s="2" t="n"/>
     </row>
-    <row r="276" ht="39.7" customHeight="1">
-      <c r="A276" s="13" t="n"/>
-      <c r="B276" s="14" t="inlineStr">
-        <is>
-          <t>Radiador adoptado</t>
-        </is>
-      </c>
-      <c r="C276" s="13">
-        <f>Datos_balance!$B$13</f>
-        <v/>
-      </c>
-      <c r="D276" s="20" t="n"/>
-      <c r="E276" s="20" t="n"/>
-      <c r="F276" s="13" t="n"/>
+    <row r="276">
+      <c r="A276" s="2" t="n"/>
+      <c r="B276" s="2" t="n"/>
+      <c r="C276" s="2" t="n"/>
+      <c r="D276" s="2" t="n"/>
+      <c r="E276" s="2" t="n"/>
+      <c r="F276" s="2" t="n"/>
       <c r="G276" s="2" t="n"/>
       <c r="H276" s="2" t="n"/>
       <c r="I276" s="2" t="n"/>
@@ -29071,8 +29052,12 @@
       <c r="H277" s="2" t="n"/>
       <c r="I277" s="2" t="n"/>
     </row>
-    <row r="278">
-      <c r="A278" s="2" t="n"/>
+    <row r="278" ht="39.7" customHeight="1">
+      <c r="A278" s="5" t="inlineStr">
+        <is>
+          <t>LOCAL  13 - Dormitorio Norte   (PA)</t>
+        </is>
+      </c>
       <c r="B278" s="2" t="n"/>
       <c r="C278" s="2" t="n"/>
       <c r="D278" s="2" t="n"/>
@@ -29083,79 +29068,94 @@
       <c r="I278" s="2" t="n"/>
     </row>
     <row r="279" ht="39.7" customHeight="1">
-      <c r="A279" s="5" t="inlineStr">
-        <is>
-          <t>LOCAL  14 - Play room   (PA)</t>
-        </is>
-      </c>
-      <c r="B279" s="2" t="n"/>
-      <c r="C279" s="2" t="n"/>
-      <c r="D279" s="2" t="n"/>
-      <c r="E279" s="2" t="n"/>
-      <c r="F279" s="2" t="n"/>
+      <c r="A279" s="3" t="inlineStr">
+        <is>
+          <t>Nro</t>
+        </is>
+      </c>
+      <c r="B279" s="3" t="inlineStr">
+        <is>
+          <t>DESCRIPCION</t>
+        </is>
+      </c>
+      <c r="C279" s="3" t="inlineStr">
+        <is>
+          <t>DIMENSIONES (m)</t>
+        </is>
+      </c>
+      <c r="D279" s="3" t="inlineStr">
+        <is>
+          <t>AREA (m2)</t>
+        </is>
+      </c>
+      <c r="E279" s="3" t="inlineStr">
+        <is>
+          <t>FACTOR</t>
+        </is>
+      </c>
+      <c r="F279" s="3" t="inlineStr">
+        <is>
+          <t>PERDIDA CALOR (Kcal/h)</t>
+        </is>
+      </c>
       <c r="G279" s="2" t="n"/>
       <c r="H279" s="2" t="n"/>
       <c r="I279" s="2" t="n"/>
     </row>
     <row r="280" ht="39.7" customHeight="1">
-      <c r="A280" s="3" t="inlineStr">
-        <is>
-          <t>Nro</t>
-        </is>
-      </c>
-      <c r="B280" s="3" t="inlineStr">
-        <is>
-          <t>DESCRIPCION</t>
-        </is>
-      </c>
-      <c r="C280" s="3" t="inlineStr">
-        <is>
-          <t>DIMENSIONES (m)</t>
-        </is>
-      </c>
-      <c r="D280" s="3" t="inlineStr">
-        <is>
-          <t>AREA (m2)</t>
-        </is>
-      </c>
-      <c r="E280" s="3" t="inlineStr">
-        <is>
-          <t>FACTOR</t>
-        </is>
-      </c>
-      <c r="F280" s="3" t="inlineStr">
-        <is>
-          <t>PERDIDA CALOR (Kcal/h)</t>
-        </is>
-      </c>
+      <c r="A280" s="16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B280" s="33" t="inlineStr">
+        <is>
+          <t>VENTANA</t>
+        </is>
+      </c>
+      <c r="C280" s="9" t="n"/>
+      <c r="D280" s="9" t="n"/>
+      <c r="E280" s="9" t="n"/>
+      <c r="F280" s="9" t="n"/>
       <c r="G280" s="2" t="n"/>
       <c r="H280" s="2" t="n"/>
       <c r="I280" s="2" t="n"/>
     </row>
-    <row r="281" ht="39.7" customHeight="1">
-      <c r="A281" s="16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B281" s="33" t="inlineStr">
-        <is>
-          <t>VENTANA</t>
-        </is>
-      </c>
-      <c r="C281" s="9" t="n"/>
-      <c r="D281" s="9" t="n"/>
-      <c r="E281" s="9" t="n"/>
-      <c r="F281" s="9" t="n"/>
+    <row r="281" ht="62" customHeight="1">
+      <c r="A281" s="9" t="n"/>
+      <c r="B281" s="34" t="inlineStr">
+        <is>
+          <t>VA04</t>
+        </is>
+      </c>
+      <c r="C281" s="9">
+        <f>IF(COUNT(H281,I281)&lt;2,"",TEXT(H281,"0.00")&amp;" x "&amp;TEXT(I281,"0.00"))</f>
+        <v/>
+      </c>
+      <c r="D281" s="8">
+        <f>IF(COUNT(H281,I281)&lt;2,"",ROUND(H281*I281,2))</f>
+        <v/>
+      </c>
+      <c r="E281" s="25" t="n">
+        <v>60</v>
+      </c>
+      <c r="F281" s="28">
+        <f>IF(D281="","",ROUND(D281*E281,1))</f>
+        <v/>
+      </c>
       <c r="G281" s="2" t="n"/>
-      <c r="H281" s="2" t="n"/>
-      <c r="I281" s="2" t="n"/>
+      <c r="H281" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="I281" s="35" t="n">
+        <v>2.52</v>
+      </c>
     </row>
     <row r="282" ht="62" customHeight="1">
       <c r="A282" s="9" t="n"/>
       <c r="B282" s="34" t="inlineStr">
         <is>
-          <t>VA04 (2)</t>
+          <t>VA05</t>
         </is>
       </c>
       <c r="C282" s="9">
@@ -29175,7 +29175,7 @@
       </c>
       <c r="G282" s="2" t="n"/>
       <c r="H282" s="35" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="I282" s="35" t="n">
         <v>2.52</v>
@@ -29328,7 +29328,7 @@
       </c>
       <c r="G288" s="2" t="n"/>
       <c r="H288" s="35" t="n">
-        <v>4</v>
+        <v>4.25</v>
       </c>
       <c r="I288" s="35" t="n">
         <v>3</v>
@@ -29358,7 +29358,7 @@
       </c>
       <c r="G289" s="2" t="n"/>
       <c r="H289" s="35" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="I289" s="35" t="n">
         <v>3</v>
@@ -29388,7 +29388,7 @@
       </c>
       <c r="G290" s="2" t="n"/>
       <c r="H290" s="35" t="n">
-        <v>4</v>
+        <v>4.25</v>
       </c>
       <c r="I290" s="35" t="n">
         <v>3</v>
@@ -29418,7 +29418,7 @@
       </c>
       <c r="G291" s="2" t="n"/>
       <c r="H291" s="35" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="I291" s="35" t="n">
         <v>3</v>
@@ -29479,7 +29479,7 @@
         </is>
       </c>
       <c r="D294" s="8" t="n">
-        <v>16.4</v>
+        <v>17</v>
       </c>
       <c r="E294" s="25" t="n">
         <v>20</v>
@@ -29570,7 +29570,7 @@
         </is>
       </c>
       <c r="D298" s="8" t="n">
-        <v>16.4</v>
+        <v>17</v>
       </c>
       <c r="E298" s="25" t="n">
         <v>15</v>
@@ -29638,11 +29638,11 @@
       </c>
       <c r="C301" s="9" t="inlineStr">
         <is>
-          <t>16.40 m2 x 3.00</t>
+          <t>17.00 m2 x 3.00</t>
         </is>
       </c>
       <c r="D301" s="8" t="n">
-        <v>49.2</v>
+        <v>51</v>
       </c>
       <c r="E301" s="25" t="n">
         <v>9</v>
@@ -29693,7 +29693,7 @@
       <c r="D303" s="9" t="n"/>
       <c r="E303" s="9" t="n"/>
       <c r="F303" s="36">
-        <f>IF(F282="",0,F282)+IF(F284="",0,F284)+IF(F285="",0,F285)+IF(F286="",0,F286)+IF(F287="",0,F287)+IF(F288="",0,F288)+IF(F289="",0,F289)+IF(F290="",0,F290)+IF(F291="",0,F291)+IF(F293="",0,F293)+IF(F294="",0,F294)+IF(F295="",0,F295)+IF(F297="",0,F297)+IF(F298="",0,F298)+IF(F300="",0,F300)+IF(F301="",0,F301)+IF(F302="",0,F302)</f>
+        <f>IF(F281="",0,F281)+IF(F282="",0,F282)+IF(F284="",0,F284)+IF(F285="",0,F285)+IF(F286="",0,F286)+IF(F287="",0,F287)+IF(F288="",0,F288)+IF(F289="",0,F289)+IF(F290="",0,F290)+IF(F291="",0,F291)+IF(F293="",0,F293)+IF(F294="",0,F294)+IF(F295="",0,F295)+IF(F297="",0,F297)+IF(F298="",0,F298)+IF(F300="",0,F300)+IF(F301="",0,F301)+IF(F302="",0,F302)</f>
         <v/>
       </c>
       <c r="G303" s="2" t="n"/>
@@ -29851,7 +29851,7 @@
     <row r="313" ht="39.7" customHeight="1">
       <c r="A313" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  15 - Dormitorio Sur   (PA)</t>
+          <t>LOCAL  14 - Play room   (PA)</t>
         </is>
       </c>
       <c r="B313" s="2" t="n"/>
@@ -29921,7 +29921,7 @@
       <c r="A316" s="9" t="n"/>
       <c r="B316" s="34" t="inlineStr">
         <is>
-          <t>PV04</t>
+          <t>VA04 (2)</t>
         </is>
       </c>
       <c r="C316" s="9">
@@ -29941,60 +29941,56 @@
       </c>
       <c r="G316" s="2" t="n"/>
       <c r="H316" s="35" t="n">
-        <v>2.06</v>
+        <v>2</v>
       </c>
       <c r="I316" s="35" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="317" ht="62" customHeight="1">
-      <c r="A317" s="9" t="n"/>
-      <c r="B317" s="34" t="inlineStr">
-        <is>
-          <t>PV04 (2)</t>
-        </is>
-      </c>
-      <c r="C317" s="9">
-        <f>IF(COUNT(H317,I317)&lt;2,"",TEXT(H317,"0.00")&amp;" x "&amp;TEXT(I317,"0.00"))</f>
-        <v/>
-      </c>
-      <c r="D317" s="8">
-        <f>IF(COUNT(H317,I317)&lt;2,"",ROUND(H317*I317,2))</f>
-        <v/>
-      </c>
-      <c r="E317" s="25" t="n">
-        <v>60</v>
-      </c>
-      <c r="F317" s="28">
-        <f>IF(D317="","",ROUND(D317*E317,1))</f>
-        <v/>
-      </c>
+        <v>2.52</v>
+      </c>
+    </row>
+    <row r="317" ht="39.7" customHeight="1">
+      <c r="A317" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B317" s="33" t="inlineStr">
+        <is>
+          <t>PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C317" s="9" t="n"/>
+      <c r="D317" s="9" t="n"/>
+      <c r="E317" s="9" t="n"/>
+      <c r="F317" s="9" t="n"/>
       <c r="G317" s="2" t="n"/>
-      <c r="H317" s="35" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="I317" s="35" t="n">
-        <v>2.95</v>
-      </c>
-    </row>
-    <row r="318" ht="39.7" customHeight="1">
-      <c r="A318" s="16" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B318" s="33" t="inlineStr">
-        <is>
-          <t>PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C318" s="9" t="n"/>
-      <c r="D318" s="9" t="n"/>
-      <c r="E318" s="9" t="n"/>
-      <c r="F318" s="9" t="n"/>
+      <c r="H317" s="2" t="n"/>
+      <c r="I317" s="2" t="n"/>
+    </row>
+    <row r="318" ht="62" customHeight="1">
+      <c r="A318" s="9" t="n"/>
+      <c r="B318" s="34" t="inlineStr">
+        <is>
+          <t>AISLADAS (    )</t>
+        </is>
+      </c>
+      <c r="C318" s="9">
+        <f>IF(COUNT(H318,I318)&lt;2,"",TEXT(H318,"0.00")&amp;" x "&amp;TEXT(I318,"0.00"))</f>
+        <v/>
+      </c>
+      <c r="D318" s="8">
+        <f>IF(COUNT(H318,I318)&lt;2,"",ROUND(H318*I318,2))</f>
+        <v/>
+      </c>
+      <c r="E318" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="F318" s="28">
+        <f>IF(D318="","",ROUND(D318*E318,1))</f>
+        <v/>
+      </c>
       <c r="G318" s="2" t="n"/>
-      <c r="H318" s="2" t="n"/>
-      <c r="I318" s="2" t="n"/>
+      <c r="H318" s="35" t="n"/>
+      <c r="I318" s="35" t="n"/>
     </row>
     <row r="319" ht="62" customHeight="1">
       <c r="A319" s="9" t="n"/>
@@ -30078,7 +30074,7 @@
       <c r="A322" s="9" t="n"/>
       <c r="B322" s="34" t="inlineStr">
         <is>
-          <t>AISLADAS (    )</t>
+          <t>INTERIORES (    )</t>
         </is>
       </c>
       <c r="C322" s="9">
@@ -30090,15 +30086,19 @@
         <v/>
       </c>
       <c r="E322" s="25" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F322" s="28">
         <f>IF(D322="","",ROUND(D322*E322,1))</f>
         <v/>
       </c>
       <c r="G322" s="2" t="n"/>
-      <c r="H322" s="35" t="n"/>
-      <c r="I322" s="35" t="n"/>
+      <c r="H322" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="I322" s="35" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="323" ht="62" customHeight="1">
       <c r="A323" s="9" t="n"/>
@@ -30124,7 +30124,7 @@
       </c>
       <c r="G323" s="2" t="n"/>
       <c r="H323" s="35" t="n">
-        <v>3.5</v>
+        <v>4.1</v>
       </c>
       <c r="I323" s="35" t="n">
         <v>3</v>
@@ -30154,7 +30154,7 @@
       </c>
       <c r="G324" s="2" t="n"/>
       <c r="H324" s="35" t="n">
-        <v>4.05</v>
+        <v>4</v>
       </c>
       <c r="I324" s="35" t="n">
         <v>3</v>
@@ -30184,75 +30184,71 @@
       </c>
       <c r="G325" s="2" t="n"/>
       <c r="H325" s="35" t="n">
-        <v>3.5</v>
+        <v>4.1</v>
       </c>
       <c r="I325" s="35" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="326" ht="62" customHeight="1">
-      <c r="A326" s="9" t="n"/>
-      <c r="B326" s="34" t="inlineStr">
-        <is>
-          <t>INTERIORES (    )</t>
-        </is>
-      </c>
-      <c r="C326" s="9">
-        <f>IF(COUNT(H326,I326)&lt;2,"",TEXT(H326,"0.00")&amp;" x "&amp;TEXT(I326,"0.00"))</f>
-        <v/>
-      </c>
-      <c r="D326" s="8">
-        <f>IF(COUNT(H326,I326)&lt;2,"",ROUND(H326*I326,2))</f>
-        <v/>
-      </c>
-      <c r="E326" s="25" t="n">
-        <v>25</v>
-      </c>
-      <c r="F326" s="28">
-        <f>IF(D326="","",ROUND(D326*E326,1))</f>
-        <v/>
-      </c>
+    <row r="326" ht="39.7" customHeight="1">
+      <c r="A326" s="16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B326" s="33" t="inlineStr">
+        <is>
+          <t>TECHOS O CIELORRASOS</t>
+        </is>
+      </c>
+      <c r="C326" s="9" t="n"/>
+      <c r="D326" s="9" t="n"/>
+      <c r="E326" s="9" t="n"/>
+      <c r="F326" s="9" t="n"/>
       <c r="G326" s="2" t="n"/>
-      <c r="H326" s="35" t="n">
-        <v>4.05</v>
-      </c>
-      <c r="I326" s="35" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="327" ht="39.7" customHeight="1">
-      <c r="A327" s="16" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B327" s="33" t="inlineStr">
-        <is>
-          <t>TECHOS O CIELORRASOS</t>
-        </is>
-      </c>
-      <c r="C327" s="9" t="n"/>
-      <c r="D327" s="9" t="n"/>
-      <c r="E327" s="9" t="n"/>
-      <c r="F327" s="9" t="n"/>
+      <c r="H326" s="2" t="n"/>
+      <c r="I326" s="2" t="n"/>
+    </row>
+    <row r="327" ht="62" customHeight="1">
+      <c r="A327" s="9" t="n"/>
+      <c r="B327" s="34" t="inlineStr">
+        <is>
+          <t>TECHO NO AISLADO</t>
+        </is>
+      </c>
+      <c r="C327" s="9" t="inlineStr"/>
+      <c r="D327" s="8">
+        <f>IF(COUNT(H327,I327)&lt;2,"",ROUND(H327*I327,2))</f>
+        <v/>
+      </c>
+      <c r="E327" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="F327" s="28">
+        <f>IF(D327="","",ROUND(D327*E327,1))</f>
+        <v/>
+      </c>
       <c r="G327" s="2" t="n"/>
-      <c r="H327" s="2" t="n"/>
-      <c r="I327" s="2" t="n"/>
-    </row>
-    <row r="328" ht="62" customHeight="1">
+      <c r="H327" s="35" t="n"/>
+      <c r="I327" s="35" t="n"/>
+    </row>
+    <row r="328" ht="39.7" customHeight="1">
       <c r="A328" s="9" t="n"/>
       <c r="B328" s="34" t="inlineStr">
         <is>
-          <t>TECHO NO AISLADO</t>
-        </is>
-      </c>
-      <c r="C328" s="9" t="inlineStr"/>
-      <c r="D328" s="8">
-        <f>IF(COUNT(H328,I328)&lt;2,"",ROUND(H328*I328,2))</f>
-        <v/>
+          <t>TECHO AISLADO</t>
+        </is>
+      </c>
+      <c r="C328" s="9" t="inlineStr">
+        <is>
+          <t>por croquis</t>
+        </is>
+      </c>
+      <c r="D328" s="8" t="n">
+        <v>16.4</v>
       </c>
       <c r="E328" s="25" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F328" s="28">
         <f>IF(D328="","",ROUND(D328*E328,1))</f>
@@ -30262,23 +30258,20 @@
       <c r="H328" s="35" t="n"/>
       <c r="I328" s="35" t="n"/>
     </row>
-    <row r="329" ht="39.7" customHeight="1">
+    <row r="329" ht="62" customHeight="1">
       <c r="A329" s="9" t="n"/>
       <c r="B329" s="34" t="inlineStr">
         <is>
-          <t>TECHO AISLADO</t>
-        </is>
-      </c>
-      <c r="C329" s="9" t="inlineStr">
-        <is>
-          <t>por croquis</t>
-        </is>
-      </c>
-      <c r="D329" s="8" t="n">
-        <v>14.17</v>
+          <t>TECHO ENTREPISO</t>
+        </is>
+      </c>
+      <c r="C329" s="9" t="inlineStr"/>
+      <c r="D329" s="8">
+        <f>IF(COUNT(H329,I329)&lt;2,"",ROUND(H329*I329,2))</f>
+        <v/>
       </c>
       <c r="E329" s="25" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F329" s="28">
         <f>IF(D329="","",ROUND(D329*E329,1))</f>
@@ -30288,62 +30281,65 @@
       <c r="H329" s="35" t="n"/>
       <c r="I329" s="35" t="n"/>
     </row>
-    <row r="330" ht="62" customHeight="1">
-      <c r="A330" s="9" t="n"/>
-      <c r="B330" s="34" t="inlineStr">
-        <is>
-          <t>TECHO ENTREPISO</t>
-        </is>
-      </c>
-      <c r="C330" s="9" t="inlineStr"/>
-      <c r="D330" s="8">
-        <f>IF(COUNT(H330,I330)&lt;2,"",ROUND(H330*I330,2))</f>
-        <v/>
-      </c>
-      <c r="E330" s="25" t="n">
-        <v>15</v>
-      </c>
-      <c r="F330" s="28">
-        <f>IF(D330="","",ROUND(D330*E330,1))</f>
-        <v/>
-      </c>
+    <row r="330" ht="39.7" customHeight="1">
+      <c r="A330" s="16" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B330" s="33" t="inlineStr">
+        <is>
+          <t>PISO</t>
+        </is>
+      </c>
+      <c r="C330" s="9" t="n"/>
+      <c r="D330" s="9" t="n"/>
+      <c r="E330" s="9" t="n"/>
+      <c r="F330" s="9" t="n"/>
       <c r="G330" s="2" t="n"/>
-      <c r="H330" s="35" t="n"/>
-      <c r="I330" s="35" t="n"/>
-    </row>
-    <row r="331" ht="39.7" customHeight="1">
-      <c r="A331" s="16" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B331" s="33" t="inlineStr">
-        <is>
-          <t>PISO</t>
-        </is>
-      </c>
-      <c r="C331" s="9" t="n"/>
-      <c r="D331" s="9" t="n"/>
-      <c r="E331" s="9" t="n"/>
-      <c r="F331" s="9" t="n"/>
+      <c r="H330" s="2" t="n"/>
+      <c r="I330" s="2" t="n"/>
+    </row>
+    <row r="331" ht="62" customHeight="1">
+      <c r="A331" s="9" t="n"/>
+      <c r="B331" s="34" t="inlineStr">
+        <is>
+          <t>SOBRE TIERRA</t>
+        </is>
+      </c>
+      <c r="C331" s="9" t="inlineStr"/>
+      <c r="D331" s="8">
+        <f>IF(COUNT(H331,I331)&lt;2,"",ROUND(H331*I331,2))</f>
+        <v/>
+      </c>
+      <c r="E331" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="F331" s="28">
+        <f>IF(D331="","",ROUND(D331*E331,1))</f>
+        <v/>
+      </c>
       <c r="G331" s="2" t="n"/>
-      <c r="H331" s="2" t="n"/>
-      <c r="I331" s="2" t="n"/>
-    </row>
-    <row r="332" ht="62" customHeight="1">
+      <c r="H331" s="35" t="n"/>
+      <c r="I331" s="35" t="n"/>
+    </row>
+    <row r="332" ht="39.7" customHeight="1">
       <c r="A332" s="9" t="n"/>
       <c r="B332" s="34" t="inlineStr">
         <is>
-          <t>SOBRE TIERRA</t>
-        </is>
-      </c>
-      <c r="C332" s="9" t="inlineStr"/>
-      <c r="D332" s="8">
-        <f>IF(COUNT(H332,I332)&lt;2,"",ROUND(H332*I332,2))</f>
-        <v/>
+          <t>SOBRE LOCAL OCUPADO</t>
+        </is>
+      </c>
+      <c r="C332" s="9" t="inlineStr">
+        <is>
+          <t>por croquis</t>
+        </is>
+      </c>
+      <c r="D332" s="8" t="n">
+        <v>16.4</v>
       </c>
       <c r="E332" s="25" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F332" s="28">
         <f>IF(D332="","",ROUND(D332*E332,1))</f>
@@ -30354,68 +30350,68 @@
       <c r="I332" s="35" t="n"/>
     </row>
     <row r="333" ht="39.7" customHeight="1">
-      <c r="A333" s="9" t="n"/>
-      <c r="B333" s="34" t="inlineStr">
-        <is>
-          <t>SOBRE LOCAL OCUPADO</t>
-        </is>
-      </c>
-      <c r="C333" s="9" t="inlineStr">
-        <is>
-          <t>por croquis</t>
-        </is>
-      </c>
-      <c r="D333" s="8" t="n">
-        <v>14.17</v>
-      </c>
-      <c r="E333" s="25" t="n">
-        <v>15</v>
-      </c>
-      <c r="F333" s="28">
-        <f>IF(D333="","",ROUND(D333*E333,1))</f>
-        <v/>
-      </c>
+      <c r="A333" s="16" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B333" s="33" t="inlineStr">
+        <is>
+          <t>INFILTRACION</t>
+        </is>
+      </c>
+      <c r="C333" s="9" t="n"/>
+      <c r="D333" s="16" t="inlineStr">
+        <is>
+          <t>VOLUMEN (m3)</t>
+        </is>
+      </c>
+      <c r="E333" s="9" t="n"/>
+      <c r="F333" s="9" t="n"/>
       <c r="G333" s="2" t="n"/>
-      <c r="H333" s="35" t="n"/>
-      <c r="I333" s="35" t="n"/>
-    </row>
-    <row r="334" ht="39.7" customHeight="1">
-      <c r="A334" s="16" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B334" s="33" t="inlineStr">
-        <is>
-          <t>INFILTRACION</t>
-        </is>
-      </c>
-      <c r="C334" s="9" t="n"/>
-      <c r="D334" s="16" t="inlineStr">
-        <is>
-          <t>VOLUMEN (m3)</t>
-        </is>
-      </c>
-      <c r="E334" s="9" t="n"/>
-      <c r="F334" s="9" t="n"/>
+      <c r="H333" s="2" t="n"/>
+      <c r="I333" s="2" t="n"/>
+    </row>
+    <row r="334" ht="62" customHeight="1">
+      <c r="A334" s="9" t="n"/>
+      <c r="B334" s="34" t="inlineStr">
+        <is>
+          <t>UNA PARED EXTERIOR</t>
+        </is>
+      </c>
+      <c r="C334" s="9" t="inlineStr"/>
+      <c r="D334" s="8">
+        <f>IF(COUNT(H334,I334)&lt;2,"",ROUND(H334*I334,2))</f>
+        <v/>
+      </c>
+      <c r="E334" s="25" t="n">
+        <v>6</v>
+      </c>
+      <c r="F334" s="28">
+        <f>IF(D334="","",ROUND(D334*E334,1))</f>
+        <v/>
+      </c>
       <c r="G334" s="2" t="n"/>
-      <c r="H334" s="2" t="n"/>
-      <c r="I334" s="2" t="n"/>
-    </row>
-    <row r="335" ht="62" customHeight="1">
+      <c r="H334" s="35" t="n"/>
+      <c r="I334" s="35" t="n"/>
+    </row>
+    <row r="335" ht="39.7" customHeight="1">
       <c r="A335" s="9" t="n"/>
       <c r="B335" s="34" t="inlineStr">
         <is>
-          <t>UNA PARED EXTERIOR</t>
-        </is>
-      </c>
-      <c r="C335" s="9" t="inlineStr"/>
-      <c r="D335" s="8">
-        <f>IF(COUNT(H335,I335)&lt;2,"",ROUND(H335*I335,2))</f>
-        <v/>
+          <t>DOS PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C335" s="9" t="inlineStr">
+        <is>
+          <t>16.40 m2 x 3.00</t>
+        </is>
+      </c>
+      <c r="D335" s="8" t="n">
+        <v>49.2</v>
       </c>
       <c r="E335" s="25" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F335" s="28">
         <f>IF(D335="","",ROUND(D335*E335,1))</f>
@@ -30425,23 +30421,20 @@
       <c r="H335" s="35" t="n"/>
       <c r="I335" s="35" t="n"/>
     </row>
-    <row r="336" ht="39.7" customHeight="1">
+    <row r="336" ht="62" customHeight="1">
       <c r="A336" s="9" t="n"/>
       <c r="B336" s="34" t="inlineStr">
         <is>
-          <t>DOS PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C336" s="9" t="inlineStr">
-        <is>
-          <t>14.17 m2 x 3.00</t>
-        </is>
-      </c>
-      <c r="D336" s="8" t="n">
-        <v>42.51</v>
+          <t>TRES O MAS PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C336" s="9" t="inlineStr"/>
+      <c r="D336" s="8">
+        <f>IF(COUNT(H336,I336)&lt;2,"",ROUND(H336*I336,2))</f>
+        <v/>
       </c>
       <c r="E336" s="25" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F336" s="28">
         <f>IF(D336="","",ROUND(D336*E336,1))</f>
@@ -30451,96 +30444,91 @@
       <c r="H336" s="35" t="n"/>
       <c r="I336" s="35" t="n"/>
     </row>
-    <row r="337" ht="62" customHeight="1">
-      <c r="A337" s="9" t="n"/>
-      <c r="B337" s="34" t="inlineStr">
-        <is>
-          <t>TRES O MAS PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C337" s="9" t="inlineStr"/>
-      <c r="D337" s="8">
-        <f>IF(COUNT(H337,I337)&lt;2,"",ROUND(H337*I337,2))</f>
-        <v/>
-      </c>
-      <c r="E337" s="25" t="n">
-        <v>12</v>
-      </c>
-      <c r="F337" s="28">
-        <f>IF(D337="","",ROUND(D337*E337,1))</f>
+    <row r="337" ht="70" customHeight="1">
+      <c r="A337" s="16" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B337" s="33" t="inlineStr">
+        <is>
+          <t>SUBTOTAL</t>
+        </is>
+      </c>
+      <c r="C337" s="9" t="n"/>
+      <c r="D337" s="9" t="n"/>
+      <c r="E337" s="9" t="n"/>
+      <c r="F337" s="36">
+        <f>IF(F316="",0,F316)+IF(F318="",0,F318)+IF(F319="",0,F319)+IF(F320="",0,F320)+IF(F321="",0,F321)+IF(F322="",0,F322)+IF(F323="",0,F323)+IF(F324="",0,F324)+IF(F325="",0,F325)+IF(F327="",0,F327)+IF(F328="",0,F328)+IF(F329="",0,F329)+IF(F331="",0,F331)+IF(F332="",0,F332)+IF(F334="",0,F334)+IF(F335="",0,F335)+IF(F336="",0,F336)</f>
         <v/>
       </c>
       <c r="G337" s="2" t="n"/>
-      <c r="H337" s="35" t="n"/>
-      <c r="I337" s="35" t="n"/>
-    </row>
-    <row r="338" ht="70" customHeight="1">
+      <c r="H337" s="2" t="n"/>
+      <c r="I337" s="2" t="n"/>
+    </row>
+    <row r="338" ht="47" customHeight="1">
       <c r="A338" s="16" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B338" s="33" t="inlineStr">
         <is>
-          <t>SUBTOTAL</t>
-        </is>
-      </c>
-      <c r="C338" s="9" t="n"/>
-      <c r="D338" s="9" t="n"/>
-      <c r="E338" s="9" t="n"/>
+          <t>PERDIDA TOTAL</t>
+        </is>
+      </c>
+      <c r="C338" s="9">
+        <f>TEXT(F337,"0.00")&amp;"  X  "&amp;Datos_balance!$B$4&amp;" (FI)  X  "&amp;Datos_balance!$B$5&amp;" (FO)  X  "&amp;Datos_balance!$B$6&amp;" (FZ)"</f>
+        <v/>
+      </c>
+      <c r="D338" s="2" t="n"/>
+      <c r="E338" s="2" t="n"/>
       <c r="F338" s="36">
-        <f>IF(F316="",0,F316)+IF(F317="",0,F317)+IF(F319="",0,F319)+IF(F320="",0,F320)+IF(F321="",0,F321)+IF(F322="",0,F322)+IF(F323="",0,F323)+IF(F324="",0,F324)+IF(F325="",0,F325)+IF(F326="",0,F326)+IF(F328="",0,F328)+IF(F329="",0,F329)+IF(F330="",0,F330)+IF(F332="",0,F332)+IF(F333="",0,F333)+IF(F335="",0,F335)+IF(F336="",0,F336)+IF(F337="",0,F337)</f>
+        <f>ROUND(F337*Datos_balance!$B$4*Datos_balance!$B$5*Datos_balance!$B$6,1)</f>
         <v/>
       </c>
       <c r="G338" s="2" t="n"/>
       <c r="H338" s="2" t="n"/>
       <c r="I338" s="2" t="n"/>
     </row>
-    <row r="339" ht="47" customHeight="1">
-      <c r="A339" s="16" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B339" s="33" t="inlineStr">
-        <is>
-          <t>PERDIDA TOTAL</t>
-        </is>
-      </c>
-      <c r="C339" s="9">
-        <f>TEXT(F338,"0.00")&amp;"  X  "&amp;Datos_balance!$B$4&amp;" (FI)  X  "&amp;Datos_balance!$B$5&amp;" (FO)  X  "&amp;Datos_balance!$B$6&amp;" (FZ)"</f>
-        <v/>
-      </c>
+    <row r="339">
+      <c r="A339" s="2" t="n"/>
+      <c r="B339" s="2" t="n"/>
+      <c r="C339" s="2" t="n"/>
       <c r="D339" s="2" t="n"/>
       <c r="E339" s="2" t="n"/>
-      <c r="F339" s="36">
-        <f>ROUND(F338*Datos_balance!$B$4*Datos_balance!$B$5*Datos_balance!$B$6,1)</f>
-        <v/>
-      </c>
+      <c r="F339" s="2" t="n"/>
       <c r="G339" s="2" t="n"/>
       <c r="H339" s="2" t="n"/>
       <c r="I339" s="2" t="n"/>
     </row>
-    <row r="340">
-      <c r="A340" s="2" t="n"/>
-      <c r="B340" s="2" t="n"/>
-      <c r="C340" s="2" t="n"/>
+    <row r="340" ht="62" customHeight="1">
+      <c r="A340" s="9" t="n"/>
+      <c r="B340" s="10" t="inlineStr">
+        <is>
+          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
+        </is>
+      </c>
+      <c r="C340" s="9">
+        <f>TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2,"0")&amp;" - "&amp;TEXT(Datos_balance!$B$11,"0")&amp;" = "&amp;TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2-Datos_balance!$B$11,"0")&amp;" C"</f>
+        <v/>
+      </c>
       <c r="D340" s="2" t="n"/>
       <c r="E340" s="2" t="n"/>
-      <c r="F340" s="2" t="n"/>
+      <c r="F340" s="9" t="n"/>
       <c r="G340" s="2" t="n"/>
       <c r="H340" s="2" t="n"/>
       <c r="I340" s="2" t="n"/>
     </row>
-    <row r="341" ht="62" customHeight="1">
+    <row r="341" ht="39.7" customHeight="1">
       <c r="A341" s="9" t="n"/>
       <c r="B341" s="10" t="inlineStr">
         <is>
-          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
-        </is>
-      </c>
-      <c r="C341" s="9">
-        <f>TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2,"0")&amp;" - "&amp;TEXT(Datos_balance!$B$11,"0")&amp;" = "&amp;TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2-Datos_balance!$B$11,"0")&amp;" C"</f>
+          <t>Kcal/h por elemento</t>
+        </is>
+      </c>
+      <c r="C341" s="8">
+        <f>ROUND(Datos_balance!$B$14*Datos_balance!$B$15,2)</f>
         <v/>
       </c>
       <c r="D341" s="2" t="n"/>
@@ -30554,11 +30542,11 @@
       <c r="A342" s="9" t="n"/>
       <c r="B342" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h por elemento</t>
-        </is>
-      </c>
-      <c r="C342" s="8">
-        <f>ROUND(Datos_balance!$B$14*Datos_balance!$B$15,2)</f>
+          <t>Elementos necesarios</t>
+        </is>
+      </c>
+      <c r="C342" s="25">
+        <f>ROUNDUP(F338/(Datos_balance!$B$14*Datos_balance!$B$15),0)</f>
         <v/>
       </c>
       <c r="D342" s="2" t="n"/>
@@ -30572,11 +30560,11 @@
       <c r="A343" s="9" t="n"/>
       <c r="B343" s="10" t="inlineStr">
         <is>
-          <t>Elementos necesarios</t>
+          <t>Ancho del radiador (cm)</t>
         </is>
       </c>
       <c r="C343" s="25">
-        <f>ROUNDUP(F339/(Datos_balance!$B$14*Datos_balance!$B$15),0)</f>
+        <f>ROUNDUP(F338/(Datos_balance!$B$14*Datos_balance!$B$15),0)*Datos_balance!$B$16</f>
         <v/>
       </c>
       <c r="D343" s="2" t="n"/>
@@ -30587,37 +30575,30 @@
       <c r="I343" s="2" t="n"/>
     </row>
     <row r="344" ht="39.7" customHeight="1">
-      <c r="A344" s="9" t="n"/>
-      <c r="B344" s="10" t="inlineStr">
-        <is>
-          <t>Ancho del radiador (cm)</t>
-        </is>
-      </c>
-      <c r="C344" s="25">
-        <f>ROUNDUP(F339/(Datos_balance!$B$14*Datos_balance!$B$15),0)*Datos_balance!$B$16</f>
-        <v/>
-      </c>
-      <c r="D344" s="2" t="n"/>
-      <c r="E344" s="2" t="n"/>
-      <c r="F344" s="9" t="n"/>
+      <c r="A344" s="13" t="n"/>
+      <c r="B344" s="14" t="inlineStr">
+        <is>
+          <t>Radiador adoptado</t>
+        </is>
+      </c>
+      <c r="C344" s="13">
+        <f>Datos_balance!$B$13</f>
+        <v/>
+      </c>
+      <c r="D344" s="20" t="n"/>
+      <c r="E344" s="20" t="n"/>
+      <c r="F344" s="13" t="n"/>
       <c r="G344" s="2" t="n"/>
       <c r="H344" s="2" t="n"/>
       <c r="I344" s="2" t="n"/>
     </row>
-    <row r="345" ht="39.7" customHeight="1">
-      <c r="A345" s="13" t="n"/>
-      <c r="B345" s="14" t="inlineStr">
-        <is>
-          <t>Radiador adoptado</t>
-        </is>
-      </c>
-      <c r="C345" s="13">
-        <f>Datos_balance!$B$13</f>
-        <v/>
-      </c>
-      <c r="D345" s="20" t="n"/>
-      <c r="E345" s="20" t="n"/>
-      <c r="F345" s="13" t="n"/>
+    <row r="345">
+      <c r="A345" s="2" t="n"/>
+      <c r="B345" s="2" t="n"/>
+      <c r="C345" s="2" t="n"/>
+      <c r="D345" s="2" t="n"/>
+      <c r="E345" s="2" t="n"/>
+      <c r="F345" s="2" t="n"/>
       <c r="G345" s="2" t="n"/>
       <c r="H345" s="2" t="n"/>
       <c r="I345" s="2" t="n"/>
@@ -30633,8 +30614,12 @@
       <c r="H346" s="2" t="n"/>
       <c r="I346" s="2" t="n"/>
     </row>
-    <row r="347">
-      <c r="A347" s="2" t="n"/>
+    <row r="347" ht="39.7" customHeight="1">
+      <c r="A347" s="5" t="inlineStr">
+        <is>
+          <t>LOCAL  15 - Dormitorio Sur   (PA)</t>
+        </is>
+      </c>
       <c r="B347" s="2" t="n"/>
       <c r="C347" s="2" t="n"/>
       <c r="D347" s="2" t="n"/>
@@ -30645,79 +30630,94 @@
       <c r="I347" s="2" t="n"/>
     </row>
     <row r="348" ht="39.7" customHeight="1">
-      <c r="A348" s="5" t="inlineStr">
-        <is>
-          <t>LOCAL  17 - Bano   (PA)</t>
-        </is>
-      </c>
-      <c r="B348" s="2" t="n"/>
-      <c r="C348" s="2" t="n"/>
-      <c r="D348" s="2" t="n"/>
-      <c r="E348" s="2" t="n"/>
-      <c r="F348" s="2" t="n"/>
+      <c r="A348" s="3" t="inlineStr">
+        <is>
+          <t>Nro</t>
+        </is>
+      </c>
+      <c r="B348" s="3" t="inlineStr">
+        <is>
+          <t>DESCRIPCION</t>
+        </is>
+      </c>
+      <c r="C348" s="3" t="inlineStr">
+        <is>
+          <t>DIMENSIONES (m)</t>
+        </is>
+      </c>
+      <c r="D348" s="3" t="inlineStr">
+        <is>
+          <t>AREA (m2)</t>
+        </is>
+      </c>
+      <c r="E348" s="3" t="inlineStr">
+        <is>
+          <t>FACTOR</t>
+        </is>
+      </c>
+      <c r="F348" s="3" t="inlineStr">
+        <is>
+          <t>PERDIDA CALOR (Kcal/h)</t>
+        </is>
+      </c>
       <c r="G348" s="2" t="n"/>
       <c r="H348" s="2" t="n"/>
       <c r="I348" s="2" t="n"/>
     </row>
     <row r="349" ht="39.7" customHeight="1">
-      <c r="A349" s="3" t="inlineStr">
-        <is>
-          <t>Nro</t>
-        </is>
-      </c>
-      <c r="B349" s="3" t="inlineStr">
-        <is>
-          <t>DESCRIPCION</t>
-        </is>
-      </c>
-      <c r="C349" s="3" t="inlineStr">
-        <is>
-          <t>DIMENSIONES (m)</t>
-        </is>
-      </c>
-      <c r="D349" s="3" t="inlineStr">
-        <is>
-          <t>AREA (m2)</t>
-        </is>
-      </c>
-      <c r="E349" s="3" t="inlineStr">
-        <is>
-          <t>FACTOR</t>
-        </is>
-      </c>
-      <c r="F349" s="3" t="inlineStr">
-        <is>
-          <t>PERDIDA CALOR (Kcal/h)</t>
-        </is>
-      </c>
+      <c r="A349" s="16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B349" s="33" t="inlineStr">
+        <is>
+          <t>VENTANA</t>
+        </is>
+      </c>
+      <c r="C349" s="9" t="n"/>
+      <c r="D349" s="9" t="n"/>
+      <c r="E349" s="9" t="n"/>
+      <c r="F349" s="9" t="n"/>
       <c r="G349" s="2" t="n"/>
       <c r="H349" s="2" t="n"/>
       <c r="I349" s="2" t="n"/>
     </row>
-    <row r="350" ht="39.7" customHeight="1">
-      <c r="A350" s="16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B350" s="33" t="inlineStr">
-        <is>
-          <t>VENTANA</t>
-        </is>
-      </c>
-      <c r="C350" s="9" t="n"/>
-      <c r="D350" s="9" t="n"/>
-      <c r="E350" s="9" t="n"/>
-      <c r="F350" s="9" t="n"/>
+    <row r="350" ht="62" customHeight="1">
+      <c r="A350" s="9" t="n"/>
+      <c r="B350" s="34" t="inlineStr">
+        <is>
+          <t>PV04</t>
+        </is>
+      </c>
+      <c r="C350" s="9">
+        <f>IF(COUNT(H350,I350)&lt;2,"",TEXT(H350,"0.00")&amp;" x "&amp;TEXT(I350,"0.00"))</f>
+        <v/>
+      </c>
+      <c r="D350" s="8">
+        <f>IF(COUNT(H350,I350)&lt;2,"",ROUND(H350*I350,2))</f>
+        <v/>
+      </c>
+      <c r="E350" s="25" t="n">
+        <v>60</v>
+      </c>
+      <c r="F350" s="28">
+        <f>IF(D350="","",ROUND(D350*E350,1))</f>
+        <v/>
+      </c>
       <c r="G350" s="2" t="n"/>
-      <c r="H350" s="2" t="n"/>
-      <c r="I350" s="2" t="n"/>
+      <c r="H350" s="35" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="I350" s="35" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="351" ht="62" customHeight="1">
       <c r="A351" s="9" t="n"/>
       <c r="B351" s="34" t="inlineStr">
         <is>
-          <t>VA03</t>
+          <t>PV04 (2)</t>
         </is>
       </c>
       <c r="C351" s="9">
@@ -30737,10 +30737,10 @@
       </c>
       <c r="G351" s="2" t="n"/>
       <c r="H351" s="35" t="n">
-        <v>0.75</v>
+        <v>1.5</v>
       </c>
       <c r="I351" s="35" t="n">
-        <v>2.52</v>
+        <v>2.95</v>
       </c>
     </row>
     <row r="352" ht="39.7" customHeight="1">
@@ -30890,7 +30890,7 @@
       </c>
       <c r="G357" s="2" t="n"/>
       <c r="H357" s="35" t="n">
-        <v>2.2</v>
+        <v>3.5</v>
       </c>
       <c r="I357" s="35" t="n">
         <v>3</v>
@@ -30920,7 +30920,7 @@
       </c>
       <c r="G358" s="2" t="n"/>
       <c r="H358" s="35" t="n">
-        <v>1.6</v>
+        <v>4.05</v>
       </c>
       <c r="I358" s="35" t="n">
         <v>3</v>
@@ -30950,7 +30950,7 @@
       </c>
       <c r="G359" s="2" t="n"/>
       <c r="H359" s="35" t="n">
-        <v>2.2</v>
+        <v>3.5</v>
       </c>
       <c r="I359" s="35" t="n">
         <v>3</v>
@@ -30980,7 +30980,7 @@
       </c>
       <c r="G360" s="2" t="n"/>
       <c r="H360" s="35" t="n">
-        <v>1.6</v>
+        <v>4.05</v>
       </c>
       <c r="I360" s="35" t="n">
         <v>3</v>
@@ -31041,7 +31041,7 @@
         </is>
       </c>
       <c r="D363" s="8" t="n">
-        <v>3.52</v>
+        <v>14.17</v>
       </c>
       <c r="E363" s="25" t="n">
         <v>20</v>
@@ -31132,7 +31132,7 @@
         </is>
       </c>
       <c r="D367" s="8" t="n">
-        <v>3.52</v>
+        <v>14.17</v>
       </c>
       <c r="E367" s="25" t="n">
         <v>15</v>
@@ -31168,20 +31168,17 @@
       <c r="H368" s="2" t="n"/>
       <c r="I368" s="2" t="n"/>
     </row>
-    <row r="369" ht="39.7" customHeight="1">
+    <row r="369" ht="62" customHeight="1">
       <c r="A369" s="9" t="n"/>
       <c r="B369" s="34" t="inlineStr">
         <is>
           <t>UNA PARED EXTERIOR</t>
         </is>
       </c>
-      <c r="C369" s="9" t="inlineStr">
-        <is>
-          <t>3.52 m2 x 3.00</t>
-        </is>
-      </c>
-      <c r="D369" s="8" t="n">
-        <v>10.56</v>
+      <c r="C369" s="9" t="inlineStr"/>
+      <c r="D369" s="8">
+        <f>IF(COUNT(H369,I369)&lt;2,"",ROUND(H369*I369,2))</f>
+        <v/>
       </c>
       <c r="E369" s="25" t="n">
         <v>6</v>
@@ -31194,17 +31191,20 @@
       <c r="H369" s="35" t="n"/>
       <c r="I369" s="35" t="n"/>
     </row>
-    <row r="370" ht="62" customHeight="1">
+    <row r="370" ht="39.7" customHeight="1">
       <c r="A370" s="9" t="n"/>
       <c r="B370" s="34" t="inlineStr">
         <is>
           <t>DOS PAREDES EXTERIORES</t>
         </is>
       </c>
-      <c r="C370" s="9" t="inlineStr"/>
-      <c r="D370" s="8">
-        <f>IF(COUNT(H370,I370)&lt;2,"",ROUND(H370*I370,2))</f>
-        <v/>
+      <c r="C370" s="9" t="inlineStr">
+        <is>
+          <t>14.17 m2 x 3.00</t>
+        </is>
+      </c>
+      <c r="D370" s="8" t="n">
+        <v>42.51</v>
       </c>
       <c r="E370" s="25" t="n">
         <v>9</v>
@@ -31255,7 +31255,7 @@
       <c r="D372" s="9" t="n"/>
       <c r="E372" s="9" t="n"/>
       <c r="F372" s="36">
-        <f>IF(F351="",0,F351)+IF(F353="",0,F353)+IF(F354="",0,F354)+IF(F355="",0,F355)+IF(F356="",0,F356)+IF(F357="",0,F357)+IF(F358="",0,F358)+IF(F359="",0,F359)+IF(F360="",0,F360)+IF(F362="",0,F362)+IF(F363="",0,F363)+IF(F364="",0,F364)+IF(F366="",0,F366)+IF(F367="",0,F367)+IF(F369="",0,F369)+IF(F370="",0,F370)+IF(F371="",0,F371)</f>
+        <f>IF(F350="",0,F350)+IF(F351="",0,F351)+IF(F353="",0,F353)+IF(F354="",0,F354)+IF(F355="",0,F355)+IF(F356="",0,F356)+IF(F357="",0,F357)+IF(F358="",0,F358)+IF(F359="",0,F359)+IF(F360="",0,F360)+IF(F362="",0,F362)+IF(F363="",0,F363)+IF(F364="",0,F364)+IF(F366="",0,F366)+IF(F367="",0,F367)+IF(F369="",0,F369)+IF(F370="",0,F370)+IF(F371="",0,F371)</f>
         <v/>
       </c>
       <c r="G372" s="2" t="n"/>
@@ -31320,11 +31320,11 @@
       <c r="A376" s="9" t="n"/>
       <c r="B376" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h del toallero Scala/Domino 80</t>
-        </is>
-      </c>
-      <c r="C376" s="25">
-        <f>ROUND(Datos_balance!$B$18*Datos_balance!$B$15,0)</f>
+          <t>Kcal/h por elemento</t>
+        </is>
+      </c>
+      <c r="C376" s="8">
+        <f>ROUND(Datos_balance!$B$14*Datos_balance!$B$15,2)</f>
         <v/>
       </c>
       <c r="D376" s="2" t="n"/>
@@ -31338,11 +31338,11 @@
       <c r="A377" s="9" t="n"/>
       <c r="B377" s="10" t="inlineStr">
         <is>
-          <t>Kcal/h del toallero Scala/Domino 150</t>
+          <t>Elementos necesarios</t>
         </is>
       </c>
       <c r="C377" s="25">
-        <f>ROUND(Datos_balance!$B$19*Datos_balance!$B$15,0)</f>
+        <f>ROUNDUP(F373/(Datos_balance!$B$14*Datos_balance!$B$15),0)</f>
         <v/>
       </c>
       <c r="D377" s="2" t="n"/>
@@ -31352,15 +31352,15 @@
       <c r="H377" s="2" t="n"/>
       <c r="I377" s="2" t="n"/>
     </row>
-    <row r="378" ht="47" customHeight="1">
+    <row r="378" ht="39.7" customHeight="1">
       <c r="A378" s="9" t="n"/>
       <c r="B378" s="10" t="inlineStr">
         <is>
-          <t>Toalleros necesarios</t>
+          <t>Ancho del radiador (cm)</t>
         </is>
       </c>
       <c r="C378" s="25">
-        <f>IF(F373&lt;=Datos_balance!$B$18*Datos_balance!$B$15,1,ROUNDUP(F373/(Datos_balance!$B$19*Datos_balance!$B$15),0))</f>
+        <f>ROUNDUP(F373/(Datos_balance!$B$14*Datos_balance!$B$15),0)*Datos_balance!$B$16</f>
         <v/>
       </c>
       <c r="D378" s="2" t="n"/>
@@ -31370,15 +31370,15 @@
       <c r="H378" s="2" t="n"/>
       <c r="I378" s="2" t="n"/>
     </row>
-    <row r="379" ht="47" customHeight="1">
+    <row r="379" ht="39.7" customHeight="1">
       <c r="A379" s="13" t="n"/>
       <c r="B379" s="14" t="inlineStr">
         <is>
-          <t>Toallero adoptado</t>
+          <t>Radiador adoptado</t>
         </is>
       </c>
       <c r="C379" s="13">
-        <f>IF(F373&lt;=Datos_balance!$B$18*Datos_balance!$B$15,"Peisa Scala / Domino 80  (500 x 800 mm)","Peisa Scala / Domino 150  (500 x 1500 mm)")</f>
+        <f>Datos_balance!$B$13</f>
         <v/>
       </c>
       <c r="D379" s="20" t="n"/>
@@ -31388,17 +31388,785 @@
       <c r="H379" s="2" t="n"/>
       <c r="I379" s="2" t="n"/>
     </row>
+    <row r="380">
+      <c r="A380" s="2" t="n"/>
+      <c r="B380" s="2" t="n"/>
+      <c r="C380" s="2" t="n"/>
+      <c r="D380" s="2" t="n"/>
+      <c r="E380" s="2" t="n"/>
+      <c r="F380" s="2" t="n"/>
+      <c r="G380" s="2" t="n"/>
+      <c r="H380" s="2" t="n"/>
+      <c r="I380" s="2" t="n"/>
+    </row>
+    <row r="381">
+      <c r="A381" s="2" t="n"/>
+      <c r="B381" s="2" t="n"/>
+      <c r="C381" s="2" t="n"/>
+      <c r="D381" s="2" t="n"/>
+      <c r="E381" s="2" t="n"/>
+      <c r="F381" s="2" t="n"/>
+      <c r="G381" s="2" t="n"/>
+      <c r="H381" s="2" t="n"/>
+      <c r="I381" s="2" t="n"/>
+    </row>
+    <row r="382" ht="39.7" customHeight="1">
+      <c r="A382" s="5" t="inlineStr">
+        <is>
+          <t>LOCAL  17 - Bano   (PA)</t>
+        </is>
+      </c>
+      <c r="B382" s="2" t="n"/>
+      <c r="C382" s="2" t="n"/>
+      <c r="D382" s="2" t="n"/>
+      <c r="E382" s="2" t="n"/>
+      <c r="F382" s="2" t="n"/>
+      <c r="G382" s="2" t="n"/>
+      <c r="H382" s="2" t="n"/>
+      <c r="I382" s="2" t="n"/>
+    </row>
+    <row r="383" ht="39.7" customHeight="1">
+      <c r="A383" s="3" t="inlineStr">
+        <is>
+          <t>Nro</t>
+        </is>
+      </c>
+      <c r="B383" s="3" t="inlineStr">
+        <is>
+          <t>DESCRIPCION</t>
+        </is>
+      </c>
+      <c r="C383" s="3" t="inlineStr">
+        <is>
+          <t>DIMENSIONES (m)</t>
+        </is>
+      </c>
+      <c r="D383" s="3" t="inlineStr">
+        <is>
+          <t>AREA (m2)</t>
+        </is>
+      </c>
+      <c r="E383" s="3" t="inlineStr">
+        <is>
+          <t>FACTOR</t>
+        </is>
+      </c>
+      <c r="F383" s="3" t="inlineStr">
+        <is>
+          <t>PERDIDA CALOR (Kcal/h)</t>
+        </is>
+      </c>
+      <c r="G383" s="2" t="n"/>
+      <c r="H383" s="2" t="n"/>
+      <c r="I383" s="2" t="n"/>
+    </row>
+    <row r="384" ht="39.7" customHeight="1">
+      <c r="A384" s="16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B384" s="33" t="inlineStr">
+        <is>
+          <t>VENTANA</t>
+        </is>
+      </c>
+      <c r="C384" s="9" t="n"/>
+      <c r="D384" s="9" t="n"/>
+      <c r="E384" s="9" t="n"/>
+      <c r="F384" s="9" t="n"/>
+      <c r="G384" s="2" t="n"/>
+      <c r="H384" s="2" t="n"/>
+      <c r="I384" s="2" t="n"/>
+    </row>
+    <row r="385" ht="62" customHeight="1">
+      <c r="A385" s="9" t="n"/>
+      <c r="B385" s="34" t="inlineStr">
+        <is>
+          <t>VA03</t>
+        </is>
+      </c>
+      <c r="C385" s="9">
+        <f>IF(COUNT(H385,I385)&lt;2,"",TEXT(H385,"0.00")&amp;" x "&amp;TEXT(I385,"0.00"))</f>
+        <v/>
+      </c>
+      <c r="D385" s="8">
+        <f>IF(COUNT(H385,I385)&lt;2,"",ROUND(H385*I385,2))</f>
+        <v/>
+      </c>
+      <c r="E385" s="25" t="n">
+        <v>60</v>
+      </c>
+      <c r="F385" s="28">
+        <f>IF(D385="","",ROUND(D385*E385,1))</f>
+        <v/>
+      </c>
+      <c r="G385" s="2" t="n"/>
+      <c r="H385" s="35" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I385" s="35" t="n">
+        <v>2.52</v>
+      </c>
+    </row>
+    <row r="386" ht="39.7" customHeight="1">
+      <c r="A386" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B386" s="33" t="inlineStr">
+        <is>
+          <t>PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C386" s="9" t="n"/>
+      <c r="D386" s="9" t="n"/>
+      <c r="E386" s="9" t="n"/>
+      <c r="F386" s="9" t="n"/>
+      <c r="G386" s="2" t="n"/>
+      <c r="H386" s="2" t="n"/>
+      <c r="I386" s="2" t="n"/>
+    </row>
+    <row r="387" ht="62" customHeight="1">
+      <c r="A387" s="9" t="n"/>
+      <c r="B387" s="34" t="inlineStr">
+        <is>
+          <t>AISLADAS (    )</t>
+        </is>
+      </c>
+      <c r="C387" s="9">
+        <f>IF(COUNT(H387,I387)&lt;2,"",TEXT(H387,"0.00")&amp;" x "&amp;TEXT(I387,"0.00"))</f>
+        <v/>
+      </c>
+      <c r="D387" s="8">
+        <f>IF(COUNT(H387,I387)&lt;2,"",ROUND(H387*I387,2))</f>
+        <v/>
+      </c>
+      <c r="E387" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="F387" s="28">
+        <f>IF(D387="","",ROUND(D387*E387,1))</f>
+        <v/>
+      </c>
+      <c r="G387" s="2" t="n"/>
+      <c r="H387" s="35" t="n"/>
+      <c r="I387" s="35" t="n"/>
+    </row>
+    <row r="388" ht="62" customHeight="1">
+      <c r="A388" s="9" t="n"/>
+      <c r="B388" s="34" t="inlineStr">
+        <is>
+          <t>AISLADAS (    )</t>
+        </is>
+      </c>
+      <c r="C388" s="9">
+        <f>IF(COUNT(H388,I388)&lt;2,"",TEXT(H388,"0.00")&amp;" x "&amp;TEXT(I388,"0.00"))</f>
+        <v/>
+      </c>
+      <c r="D388" s="8">
+        <f>IF(COUNT(H388,I388)&lt;2,"",ROUND(H388*I388,2))</f>
+        <v/>
+      </c>
+      <c r="E388" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="F388" s="28">
+        <f>IF(D388="","",ROUND(D388*E388,1))</f>
+        <v/>
+      </c>
+      <c r="G388" s="2" t="n"/>
+      <c r="H388" s="35" t="n"/>
+      <c r="I388" s="35" t="n"/>
+    </row>
+    <row r="389" ht="62" customHeight="1">
+      <c r="A389" s="9" t="n"/>
+      <c r="B389" s="34" t="inlineStr">
+        <is>
+          <t>AISLADAS (    )</t>
+        </is>
+      </c>
+      <c r="C389" s="9">
+        <f>IF(COUNT(H389,I389)&lt;2,"",TEXT(H389,"0.00")&amp;" x "&amp;TEXT(I389,"0.00"))</f>
+        <v/>
+      </c>
+      <c r="D389" s="8">
+        <f>IF(COUNT(H389,I389)&lt;2,"",ROUND(H389*I389,2))</f>
+        <v/>
+      </c>
+      <c r="E389" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="F389" s="28">
+        <f>IF(D389="","",ROUND(D389*E389,1))</f>
+        <v/>
+      </c>
+      <c r="G389" s="2" t="n"/>
+      <c r="H389" s="35" t="n"/>
+      <c r="I389" s="35" t="n"/>
+    </row>
+    <row r="390" ht="62" customHeight="1">
+      <c r="A390" s="9" t="n"/>
+      <c r="B390" s="34" t="inlineStr">
+        <is>
+          <t>AISLADAS (    )</t>
+        </is>
+      </c>
+      <c r="C390" s="9">
+        <f>IF(COUNT(H390,I390)&lt;2,"",TEXT(H390,"0.00")&amp;" x "&amp;TEXT(I390,"0.00"))</f>
+        <v/>
+      </c>
+      <c r="D390" s="8">
+        <f>IF(COUNT(H390,I390)&lt;2,"",ROUND(H390*I390,2))</f>
+        <v/>
+      </c>
+      <c r="E390" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="F390" s="28">
+        <f>IF(D390="","",ROUND(D390*E390,1))</f>
+        <v/>
+      </c>
+      <c r="G390" s="2" t="n"/>
+      <c r="H390" s="35" t="n"/>
+      <c r="I390" s="35" t="n"/>
+    </row>
+    <row r="391" ht="62" customHeight="1">
+      <c r="A391" s="9" t="n"/>
+      <c r="B391" s="34" t="inlineStr">
+        <is>
+          <t>INTERIORES (    )</t>
+        </is>
+      </c>
+      <c r="C391" s="9">
+        <f>IF(COUNT(H391,I391)&lt;2,"",TEXT(H391,"0.00")&amp;" x "&amp;TEXT(I391,"0.00"))</f>
+        <v/>
+      </c>
+      <c r="D391" s="8">
+        <f>IF(COUNT(H391,I391)&lt;2,"",ROUND(H391*I391,2))</f>
+        <v/>
+      </c>
+      <c r="E391" s="25" t="n">
+        <v>25</v>
+      </c>
+      <c r="F391" s="28">
+        <f>IF(D391="","",ROUND(D391*E391,1))</f>
+        <v/>
+      </c>
+      <c r="G391" s="2" t="n"/>
+      <c r="H391" s="35" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="I391" s="35" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="392" ht="62" customHeight="1">
+      <c r="A392" s="9" t="n"/>
+      <c r="B392" s="34" t="inlineStr">
+        <is>
+          <t>INTERIORES (    )</t>
+        </is>
+      </c>
+      <c r="C392" s="9">
+        <f>IF(COUNT(H392,I392)&lt;2,"",TEXT(H392,"0.00")&amp;" x "&amp;TEXT(I392,"0.00"))</f>
+        <v/>
+      </c>
+      <c r="D392" s="8">
+        <f>IF(COUNT(H392,I392)&lt;2,"",ROUND(H392*I392,2))</f>
+        <v/>
+      </c>
+      <c r="E392" s="25" t="n">
+        <v>25</v>
+      </c>
+      <c r="F392" s="28">
+        <f>IF(D392="","",ROUND(D392*E392,1))</f>
+        <v/>
+      </c>
+      <c r="G392" s="2" t="n"/>
+      <c r="H392" s="35" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="I392" s="35" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="393" ht="62" customHeight="1">
+      <c r="A393" s="9" t="n"/>
+      <c r="B393" s="34" t="inlineStr">
+        <is>
+          <t>INTERIORES (    )</t>
+        </is>
+      </c>
+      <c r="C393" s="9">
+        <f>IF(COUNT(H393,I393)&lt;2,"",TEXT(H393,"0.00")&amp;" x "&amp;TEXT(I393,"0.00"))</f>
+        <v/>
+      </c>
+      <c r="D393" s="8">
+        <f>IF(COUNT(H393,I393)&lt;2,"",ROUND(H393*I393,2))</f>
+        <v/>
+      </c>
+      <c r="E393" s="25" t="n">
+        <v>25</v>
+      </c>
+      <c r="F393" s="28">
+        <f>IF(D393="","",ROUND(D393*E393,1))</f>
+        <v/>
+      </c>
+      <c r="G393" s="2" t="n"/>
+      <c r="H393" s="35" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="I393" s="35" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="394" ht="62" customHeight="1">
+      <c r="A394" s="9" t="n"/>
+      <c r="B394" s="34" t="inlineStr">
+        <is>
+          <t>INTERIORES (    )</t>
+        </is>
+      </c>
+      <c r="C394" s="9">
+        <f>IF(COUNT(H394,I394)&lt;2,"",TEXT(H394,"0.00")&amp;" x "&amp;TEXT(I394,"0.00"))</f>
+        <v/>
+      </c>
+      <c r="D394" s="8">
+        <f>IF(COUNT(H394,I394)&lt;2,"",ROUND(H394*I394,2))</f>
+        <v/>
+      </c>
+      <c r="E394" s="25" t="n">
+        <v>25</v>
+      </c>
+      <c r="F394" s="28">
+        <f>IF(D394="","",ROUND(D394*E394,1))</f>
+        <v/>
+      </c>
+      <c r="G394" s="2" t="n"/>
+      <c r="H394" s="35" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="I394" s="35" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="395" ht="39.7" customHeight="1">
+      <c r="A395" s="16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B395" s="33" t="inlineStr">
+        <is>
+          <t>TECHOS O CIELORRASOS</t>
+        </is>
+      </c>
+      <c r="C395" s="9" t="n"/>
+      <c r="D395" s="9" t="n"/>
+      <c r="E395" s="9" t="n"/>
+      <c r="F395" s="9" t="n"/>
+      <c r="G395" s="2" t="n"/>
+      <c r="H395" s="2" t="n"/>
+      <c r="I395" s="2" t="n"/>
+    </row>
+    <row r="396" ht="62" customHeight="1">
+      <c r="A396" s="9" t="n"/>
+      <c r="B396" s="34" t="inlineStr">
+        <is>
+          <t>TECHO NO AISLADO</t>
+        </is>
+      </c>
+      <c r="C396" s="9" t="inlineStr"/>
+      <c r="D396" s="8">
+        <f>IF(COUNT(H396,I396)&lt;2,"",ROUND(H396*I396,2))</f>
+        <v/>
+      </c>
+      <c r="E396" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="F396" s="28">
+        <f>IF(D396="","",ROUND(D396*E396,1))</f>
+        <v/>
+      </c>
+      <c r="G396" s="2" t="n"/>
+      <c r="H396" s="35" t="n"/>
+      <c r="I396" s="35" t="n"/>
+    </row>
+    <row r="397" ht="39.7" customHeight="1">
+      <c r="A397" s="9" t="n"/>
+      <c r="B397" s="34" t="inlineStr">
+        <is>
+          <t>TECHO AISLADO</t>
+        </is>
+      </c>
+      <c r="C397" s="9" t="inlineStr">
+        <is>
+          <t>por croquis</t>
+        </is>
+      </c>
+      <c r="D397" s="8" t="n">
+        <v>3.52</v>
+      </c>
+      <c r="E397" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="F397" s="28">
+        <f>IF(D397="","",ROUND(D397*E397,1))</f>
+        <v/>
+      </c>
+      <c r="G397" s="2" t="n"/>
+      <c r="H397" s="35" t="n"/>
+      <c r="I397" s="35" t="n"/>
+    </row>
+    <row r="398" ht="62" customHeight="1">
+      <c r="A398" s="9" t="n"/>
+      <c r="B398" s="34" t="inlineStr">
+        <is>
+          <t>TECHO ENTREPISO</t>
+        </is>
+      </c>
+      <c r="C398" s="9" t="inlineStr"/>
+      <c r="D398" s="8">
+        <f>IF(COUNT(H398,I398)&lt;2,"",ROUND(H398*I398,2))</f>
+        <v/>
+      </c>
+      <c r="E398" s="25" t="n">
+        <v>15</v>
+      </c>
+      <c r="F398" s="28">
+        <f>IF(D398="","",ROUND(D398*E398,1))</f>
+        <v/>
+      </c>
+      <c r="G398" s="2" t="n"/>
+      <c r="H398" s="35" t="n"/>
+      <c r="I398" s="35" t="n"/>
+    </row>
+    <row r="399" ht="39.7" customHeight="1">
+      <c r="A399" s="16" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B399" s="33" t="inlineStr">
+        <is>
+          <t>PISO</t>
+        </is>
+      </c>
+      <c r="C399" s="9" t="n"/>
+      <c r="D399" s="9" t="n"/>
+      <c r="E399" s="9" t="n"/>
+      <c r="F399" s="9" t="n"/>
+      <c r="G399" s="2" t="n"/>
+      <c r="H399" s="2" t="n"/>
+      <c r="I399" s="2" t="n"/>
+    </row>
+    <row r="400" ht="62" customHeight="1">
+      <c r="A400" s="9" t="n"/>
+      <c r="B400" s="34" t="inlineStr">
+        <is>
+          <t>SOBRE TIERRA</t>
+        </is>
+      </c>
+      <c r="C400" s="9" t="inlineStr"/>
+      <c r="D400" s="8">
+        <f>IF(COUNT(H400,I400)&lt;2,"",ROUND(H400*I400,2))</f>
+        <v/>
+      </c>
+      <c r="E400" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="F400" s="28">
+        <f>IF(D400="","",ROUND(D400*E400,1))</f>
+        <v/>
+      </c>
+      <c r="G400" s="2" t="n"/>
+      <c r="H400" s="35" t="n"/>
+      <c r="I400" s="35" t="n"/>
+    </row>
+    <row r="401" ht="39.7" customHeight="1">
+      <c r="A401" s="9" t="n"/>
+      <c r="B401" s="34" t="inlineStr">
+        <is>
+          <t>SOBRE LOCAL OCUPADO</t>
+        </is>
+      </c>
+      <c r="C401" s="9" t="inlineStr">
+        <is>
+          <t>por croquis</t>
+        </is>
+      </c>
+      <c r="D401" s="8" t="n">
+        <v>3.52</v>
+      </c>
+      <c r="E401" s="25" t="n">
+        <v>15</v>
+      </c>
+      <c r="F401" s="28">
+        <f>IF(D401="","",ROUND(D401*E401,1))</f>
+        <v/>
+      </c>
+      <c r="G401" s="2" t="n"/>
+      <c r="H401" s="35" t="n"/>
+      <c r="I401" s="35" t="n"/>
+    </row>
+    <row r="402" ht="39.7" customHeight="1">
+      <c r="A402" s="16" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B402" s="33" t="inlineStr">
+        <is>
+          <t>INFILTRACION</t>
+        </is>
+      </c>
+      <c r="C402" s="9" t="n"/>
+      <c r="D402" s="16" t="inlineStr">
+        <is>
+          <t>VOLUMEN (m3)</t>
+        </is>
+      </c>
+      <c r="E402" s="9" t="n"/>
+      <c r="F402" s="9" t="n"/>
+      <c r="G402" s="2" t="n"/>
+      <c r="H402" s="2" t="n"/>
+      <c r="I402" s="2" t="n"/>
+    </row>
+    <row r="403" ht="39.7" customHeight="1">
+      <c r="A403" s="9" t="n"/>
+      <c r="B403" s="34" t="inlineStr">
+        <is>
+          <t>UNA PARED EXTERIOR</t>
+        </is>
+      </c>
+      <c r="C403" s="9" t="inlineStr">
+        <is>
+          <t>3.52 m2 x 3.00</t>
+        </is>
+      </c>
+      <c r="D403" s="8" t="n">
+        <v>10.56</v>
+      </c>
+      <c r="E403" s="25" t="n">
+        <v>6</v>
+      </c>
+      <c r="F403" s="28">
+        <f>IF(D403="","",ROUND(D403*E403,1))</f>
+        <v/>
+      </c>
+      <c r="G403" s="2" t="n"/>
+      <c r="H403" s="35" t="n"/>
+      <c r="I403" s="35" t="n"/>
+    </row>
+    <row r="404" ht="62" customHeight="1">
+      <c r="A404" s="9" t="n"/>
+      <c r="B404" s="34" t="inlineStr">
+        <is>
+          <t>DOS PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C404" s="9" t="inlineStr"/>
+      <c r="D404" s="8">
+        <f>IF(COUNT(H404,I404)&lt;2,"",ROUND(H404*I404,2))</f>
+        <v/>
+      </c>
+      <c r="E404" s="25" t="n">
+        <v>9</v>
+      </c>
+      <c r="F404" s="28">
+        <f>IF(D404="","",ROUND(D404*E404,1))</f>
+        <v/>
+      </c>
+      <c r="G404" s="2" t="n"/>
+      <c r="H404" s="35" t="n"/>
+      <c r="I404" s="35" t="n"/>
+    </row>
+    <row r="405" ht="62" customHeight="1">
+      <c r="A405" s="9" t="n"/>
+      <c r="B405" s="34" t="inlineStr">
+        <is>
+          <t>TRES O MAS PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C405" s="9" t="inlineStr"/>
+      <c r="D405" s="8">
+        <f>IF(COUNT(H405,I405)&lt;2,"",ROUND(H405*I405,2))</f>
+        <v/>
+      </c>
+      <c r="E405" s="25" t="n">
+        <v>12</v>
+      </c>
+      <c r="F405" s="28">
+        <f>IF(D405="","",ROUND(D405*E405,1))</f>
+        <v/>
+      </c>
+      <c r="G405" s="2" t="n"/>
+      <c r="H405" s="35" t="n"/>
+      <c r="I405" s="35" t="n"/>
+    </row>
+    <row r="406" ht="70" customHeight="1">
+      <c r="A406" s="16" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B406" s="33" t="inlineStr">
+        <is>
+          <t>SUBTOTAL</t>
+        </is>
+      </c>
+      <c r="C406" s="9" t="n"/>
+      <c r="D406" s="9" t="n"/>
+      <c r="E406" s="9" t="n"/>
+      <c r="F406" s="36">
+        <f>IF(F385="",0,F385)+IF(F387="",0,F387)+IF(F388="",0,F388)+IF(F389="",0,F389)+IF(F390="",0,F390)+IF(F391="",0,F391)+IF(F392="",0,F392)+IF(F393="",0,F393)+IF(F394="",0,F394)+IF(F396="",0,F396)+IF(F397="",0,F397)+IF(F398="",0,F398)+IF(F400="",0,F400)+IF(F401="",0,F401)+IF(F403="",0,F403)+IF(F404="",0,F404)+IF(F405="",0,F405)</f>
+        <v/>
+      </c>
+      <c r="G406" s="2" t="n"/>
+      <c r="H406" s="2" t="n"/>
+      <c r="I406" s="2" t="n"/>
+    </row>
+    <row r="407" ht="47" customHeight="1">
+      <c r="A407" s="16" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B407" s="33" t="inlineStr">
+        <is>
+          <t>PERDIDA TOTAL</t>
+        </is>
+      </c>
+      <c r="C407" s="9">
+        <f>TEXT(F406,"0.00")&amp;"  X  "&amp;Datos_balance!$B$4&amp;" (FI)  X  "&amp;Datos_balance!$B$5&amp;" (FO)  X  "&amp;Datos_balance!$B$6&amp;" (FZ)"</f>
+        <v/>
+      </c>
+      <c r="D407" s="2" t="n"/>
+      <c r="E407" s="2" t="n"/>
+      <c r="F407" s="36">
+        <f>ROUND(F406*Datos_balance!$B$4*Datos_balance!$B$5*Datos_balance!$B$6,1)</f>
+        <v/>
+      </c>
+      <c r="G407" s="2" t="n"/>
+      <c r="H407" s="2" t="n"/>
+      <c r="I407" s="2" t="n"/>
+    </row>
+    <row r="408">
+      <c r="A408" s="2" t="n"/>
+      <c r="B408" s="2" t="n"/>
+      <c r="C408" s="2" t="n"/>
+      <c r="D408" s="2" t="n"/>
+      <c r="E408" s="2" t="n"/>
+      <c r="F408" s="2" t="n"/>
+      <c r="G408" s="2" t="n"/>
+      <c r="H408" s="2" t="n"/>
+      <c r="I408" s="2" t="n"/>
+    </row>
+    <row r="409" ht="62" customHeight="1">
+      <c r="A409" s="9" t="n"/>
+      <c r="B409" s="10" t="inlineStr">
+        <is>
+          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
+        </is>
+      </c>
+      <c r="C409" s="9">
+        <f>TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2,"0")&amp;" - "&amp;TEXT(Datos_balance!$B$11,"0")&amp;" = "&amp;TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2-Datos_balance!$B$11,"0")&amp;" C"</f>
+        <v/>
+      </c>
+      <c r="D409" s="2" t="n"/>
+      <c r="E409" s="2" t="n"/>
+      <c r="F409" s="9" t="n"/>
+      <c r="G409" s="2" t="n"/>
+      <c r="H409" s="2" t="n"/>
+      <c r="I409" s="2" t="n"/>
+    </row>
+    <row r="410" ht="39.7" customHeight="1">
+      <c r="A410" s="9" t="n"/>
+      <c r="B410" s="10" t="inlineStr">
+        <is>
+          <t>Kcal/h del toallero Scala/Domino 80</t>
+        </is>
+      </c>
+      <c r="C410" s="25">
+        <f>ROUND(Datos_balance!$B$18*Datos_balance!$B$15,0)</f>
+        <v/>
+      </c>
+      <c r="D410" s="2" t="n"/>
+      <c r="E410" s="2" t="n"/>
+      <c r="F410" s="9" t="n"/>
+      <c r="G410" s="2" t="n"/>
+      <c r="H410" s="2" t="n"/>
+      <c r="I410" s="2" t="n"/>
+    </row>
+    <row r="411" ht="39.7" customHeight="1">
+      <c r="A411" s="9" t="n"/>
+      <c r="B411" s="10" t="inlineStr">
+        <is>
+          <t>Kcal/h del toallero Scala/Domino 150</t>
+        </is>
+      </c>
+      <c r="C411" s="25">
+        <f>ROUND(Datos_balance!$B$19*Datos_balance!$B$15,0)</f>
+        <v/>
+      </c>
+      <c r="D411" s="2" t="n"/>
+      <c r="E411" s="2" t="n"/>
+      <c r="F411" s="9" t="n"/>
+      <c r="G411" s="2" t="n"/>
+      <c r="H411" s="2" t="n"/>
+      <c r="I411" s="2" t="n"/>
+    </row>
+    <row r="412" ht="47" customHeight="1">
+      <c r="A412" s="9" t="n"/>
+      <c r="B412" s="10" t="inlineStr">
+        <is>
+          <t>Toalleros necesarios</t>
+        </is>
+      </c>
+      <c r="C412" s="25">
+        <f>IF(F407&lt;=Datos_balance!$B$18*Datos_balance!$B$15,1,ROUNDUP(F407/(Datos_balance!$B$19*Datos_balance!$B$15),0))</f>
+        <v/>
+      </c>
+      <c r="D412" s="2" t="n"/>
+      <c r="E412" s="2" t="n"/>
+      <c r="F412" s="9" t="n"/>
+      <c r="G412" s="2" t="n"/>
+      <c r="H412" s="2" t="n"/>
+      <c r="I412" s="2" t="n"/>
+    </row>
+    <row r="413" ht="47" customHeight="1">
+      <c r="A413" s="13" t="n"/>
+      <c r="B413" s="14" t="inlineStr">
+        <is>
+          <t>Toallero adoptado</t>
+        </is>
+      </c>
+      <c r="C413" s="13">
+        <f>IF(F407&lt;=Datos_balance!$B$18*Datos_balance!$B$15,"Peisa Scala / Domino 80  (500 x 800 mm)","Peisa Scala / Domino 150  (500 x 1500 mm)")</f>
+        <v/>
+      </c>
+      <c r="D413" s="20" t="n"/>
+      <c r="E413" s="20" t="n"/>
+      <c r="F413" s="13" t="n"/>
+      <c r="G413" s="2" t="n"/>
+      <c r="H413" s="2" t="n"/>
+      <c r="I413" s="2" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="78">
+  <mergeCells count="85">
     <mergeCell ref="C274:E274"/>
-    <mergeCell ref="C345:E345"/>
     <mergeCell ref="C31:E31"/>
     <mergeCell ref="C373:E373"/>
+    <mergeCell ref="C413:E413"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="C379:E379"/>
+    <mergeCell ref="A175:F175"/>
     <mergeCell ref="C241:E241"/>
     <mergeCell ref="C307:E307"/>
     <mergeCell ref="C342:E342"/>
+    <mergeCell ref="A347:F347"/>
     <mergeCell ref="C101:E101"/>
     <mergeCell ref="C204:E204"/>
     <mergeCell ref="C375:E375"/>
@@ -31409,21 +32177,21 @@
     <mergeCell ref="C309:E309"/>
     <mergeCell ref="C205:E205"/>
     <mergeCell ref="C99:E99"/>
-    <mergeCell ref="C270:E270"/>
-    <mergeCell ref="C167:E167"/>
+    <mergeCell ref="C168:E168"/>
     <mergeCell ref="C238:E238"/>
+    <mergeCell ref="C412:E412"/>
     <mergeCell ref="C273:E273"/>
     <mergeCell ref="C169:E169"/>
+    <mergeCell ref="A278:F278"/>
+    <mergeCell ref="C409:E409"/>
     <mergeCell ref="A141:F141"/>
     <mergeCell ref="C272:E272"/>
     <mergeCell ref="C32:E32"/>
-    <mergeCell ref="C339:E339"/>
     <mergeCell ref="C170:E170"/>
-    <mergeCell ref="A348:F348"/>
-    <mergeCell ref="A176:F176"/>
+    <mergeCell ref="C338:E338"/>
     <mergeCell ref="C33:E33"/>
-    <mergeCell ref="C173:E173"/>
-    <mergeCell ref="C276:E276"/>
+    <mergeCell ref="C269:E269"/>
+    <mergeCell ref="C340:E340"/>
     <mergeCell ref="A105:F105"/>
     <mergeCell ref="A210:F210"/>
     <mergeCell ref="A71:F71"/>
@@ -31431,13 +32199,13 @@
     <mergeCell ref="A313:F313"/>
     <mergeCell ref="C135:E135"/>
     <mergeCell ref="A244:F244"/>
+    <mergeCell ref="C411:E411"/>
     <mergeCell ref="C67:E67"/>
     <mergeCell ref="C96:E96"/>
     <mergeCell ref="C136:E136"/>
     <mergeCell ref="C376:E376"/>
     <mergeCell ref="C30:E30"/>
     <mergeCell ref="C235:E235"/>
-    <mergeCell ref="A279:F279"/>
     <mergeCell ref="C62:E62"/>
     <mergeCell ref="C98:E98"/>
     <mergeCell ref="A36:F36"/>
@@ -31447,6 +32215,7 @@
     <mergeCell ref="C64:E64"/>
     <mergeCell ref="C306:E306"/>
     <mergeCell ref="C171:E171"/>
+    <mergeCell ref="C407:E407"/>
     <mergeCell ref="C137:E137"/>
     <mergeCell ref="C134:E134"/>
     <mergeCell ref="C201:E201"/>
@@ -31456,17 +32225,21 @@
     <mergeCell ref="C132:E132"/>
     <mergeCell ref="C203:E203"/>
     <mergeCell ref="C240:E240"/>
+    <mergeCell ref="C410:E410"/>
     <mergeCell ref="C66:E66"/>
     <mergeCell ref="C237:E237"/>
     <mergeCell ref="C308:E308"/>
     <mergeCell ref="C102:E102"/>
+    <mergeCell ref="C100:E100"/>
+    <mergeCell ref="A382:F382"/>
     <mergeCell ref="C304:E304"/>
     <mergeCell ref="C68:E68"/>
     <mergeCell ref="C239:E239"/>
     <mergeCell ref="C310:E310"/>
+    <mergeCell ref="C166:E166"/>
     <mergeCell ref="C343:E343"/>
     <mergeCell ref="C29:E29"/>
-    <mergeCell ref="C100:E100"/>
+    <mergeCell ref="C271:E271"/>
     <mergeCell ref="C65:E65"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Balance termico: altura de local por cielorraso suspendido
Los locales con cielorraso suspendido de yeso tienen 2,80 m de altura
libre y no 3,00: vestidor, suite, bano suite y bano visitas en planta
baja, y los dos dormitorios, el bano y el antebano en planta alta. Dato
del autor del proyecto.

Afecta la superficie de muro y el volumen de infiltracion de esos siete
locales. El total pasa de 28.660 a 28.103 kcal/h.

Los detalles constructivos confirman ademas que el muro exterior lleva
25 mm de poliestireno expandido de alta densidad entre el cierre de
ladrillo Brimax y la terminacion de frente, asi que califica como pared
aislada y va a factor 20.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -6720,7 +6720,7 @@
     <row r="54" ht="39.7" customHeight="1">
       <c r="A54" s="23" t="inlineStr">
         <is>
-          <t>La altura de local adoptada es 3.00 m, de los cortes de la planilla de carpinterias.</t>
+          <t>Altura de local: 3,00 m en general. En los locales con cielorraso suspendido de yeso (vestidor, suite, bano suite, bano visitas, los dos dormitorios de PA y el bano de PA) la altura libre es 2,80 m, dato del autor del proyecto.</t>
         </is>
       </c>
       <c r="B54" s="2" t="n"/>
@@ -22832,7 +22832,7 @@
     <row r="3" ht="39.7" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  01 - Cocina / comedor   (PB)</t>
+          <t>LOCAL  01 - Cocina / comedor   (PB)   -   altura 3.00 m</t>
         </is>
       </c>
       <c r="B3" s="2" t="n"/>
@@ -23617,7 +23617,7 @@
     <row r="38" ht="39.7" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  06 - Living / comedor   (PB)</t>
+          <t>LOCAL  06 - Living / comedor   (PB)   -   altura 3.00 m</t>
         </is>
       </c>
       <c r="B38" s="2" t="n"/>
@@ -24453,7 +24453,7 @@
     <row r="75" ht="39.7" customHeight="1">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  07 - Hall / ingreso   (PB)</t>
+          <t>LOCAL  07 - Hall / ingreso   (PB)   -   altura 3.00 m</t>
         </is>
       </c>
       <c r="B75" s="2" t="n"/>
@@ -25181,7 +25181,7 @@
     <row r="107" ht="39.7" customHeight="1">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  08 - Vestidor   (PB)</t>
+          <t>LOCAL  08 - Vestidor   (PB)   -   altura 2.80 m</t>
         </is>
       </c>
       <c r="B107" s="2" t="n"/>
@@ -25423,7 +25423,7 @@
         <v>4.87</v>
       </c>
       <c r="I116" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="117" ht="62" customHeight="1">
@@ -25453,7 +25453,7 @@
         <v>1.66</v>
       </c>
       <c r="I117" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="118" ht="62" customHeight="1">
@@ -25483,7 +25483,7 @@
         <v>3.38</v>
       </c>
       <c r="I118" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="119" ht="62" customHeight="1">
@@ -25513,7 +25513,7 @@
         <v>0.57</v>
       </c>
       <c r="I119" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="120" ht="62" customHeight="1">
@@ -25543,7 +25543,7 @@
         <v>1.49</v>
       </c>
       <c r="I120" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="121" ht="62" customHeight="1">
@@ -25573,7 +25573,7 @@
         <v>1.09</v>
       </c>
       <c r="I121" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="122" ht="39.7" customHeight="1">
@@ -25767,11 +25767,11 @@
       </c>
       <c r="C130" s="9" t="inlineStr">
         <is>
-          <t>7.23 m2 x 3.00</t>
+          <t>7.23 m2 x 2.80</t>
         </is>
       </c>
       <c r="D130" s="8" t="n">
-        <v>21.69</v>
+        <v>20.24</v>
       </c>
       <c r="E130" s="25" t="n">
         <v>6</v>
@@ -26036,7 +26036,7 @@
     <row r="145" ht="39.7" customHeight="1">
       <c r="A145" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  Escalera   (PB)</t>
+          <t>LOCAL  Escalera   (PB)   -   altura 3.00 m</t>
         </is>
       </c>
       <c r="B145" s="2" t="n"/>
@@ -26764,7 +26764,7 @@
     <row r="177" ht="39.7" customHeight="1">
       <c r="A177" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  09 - Dormitorio suite   (PB)</t>
+          <t>LOCAL  09 - Dormitorio suite   (PB)   -   altura 2.80 m</t>
         </is>
       </c>
       <c r="B177" s="2" t="n"/>
@@ -27040,7 +27040,7 @@
         <v>3.5</v>
       </c>
       <c r="I187" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="188" ht="62" customHeight="1">
@@ -27070,7 +27070,7 @@
         <v>3.5</v>
       </c>
       <c r="I188" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="189" ht="62" customHeight="1">
@@ -27100,7 +27100,7 @@
         <v>3.5</v>
       </c>
       <c r="I189" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="190" ht="62" customHeight="1">
@@ -27130,7 +27130,7 @@
         <v>3.5</v>
       </c>
       <c r="I190" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="191" ht="39.7" customHeight="1">
@@ -27347,11 +27347,11 @@
       </c>
       <c r="C200" s="9" t="inlineStr">
         <is>
-          <t>12.25 m2 x 3.00</t>
+          <t>12.25 m2 x 2.80</t>
         </is>
       </c>
       <c r="D200" s="8" t="n">
-        <v>36.75</v>
+        <v>34.3</v>
       </c>
       <c r="E200" s="25" t="n">
         <v>9</v>
@@ -27593,7 +27593,7 @@
     <row r="214" ht="39.7" customHeight="1">
       <c r="A214" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  10 - Bano suite   (PB)</t>
+          <t>LOCAL  10 - Bano suite   (PB)   -   altura 2.80 m</t>
         </is>
       </c>
       <c r="B214" s="2" t="n"/>
@@ -27839,7 +27839,7 @@
         <v>3.3</v>
       </c>
       <c r="I223" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="224" ht="62" customHeight="1">
@@ -27869,7 +27869,7 @@
         <v>1.7</v>
       </c>
       <c r="I224" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="225" ht="62" customHeight="1">
@@ -27899,7 +27899,7 @@
         <v>3.3</v>
       </c>
       <c r="I225" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="226" ht="62" customHeight="1">
@@ -27929,7 +27929,7 @@
         <v>1.7</v>
       </c>
       <c r="I226" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="227" ht="39.7" customHeight="1">
@@ -28123,11 +28123,11 @@
       </c>
       <c r="C235" s="9" t="inlineStr">
         <is>
-          <t>5.61 m2 x 3.00</t>
+          <t>5.61 m2 x 2.80</t>
         </is>
       </c>
       <c r="D235" s="8" t="n">
-        <v>16.83</v>
+        <v>15.71</v>
       </c>
       <c r="E235" s="25" t="n">
         <v>6</v>
@@ -28392,7 +28392,7 @@
     <row r="250" ht="39.7" customHeight="1">
       <c r="A250" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  11 - Bano visitas   (PB)</t>
+          <t>LOCAL  11 - Bano visitas   (PB)   -   altura 2.80 m</t>
         </is>
       </c>
       <c r="B250" s="2" t="n"/>
@@ -28634,7 +28634,7 @@
         <v>2.4</v>
       </c>
       <c r="I259" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="260" ht="62" customHeight="1">
@@ -28664,7 +28664,7 @@
         <v>1.3</v>
       </c>
       <c r="I260" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="261" ht="62" customHeight="1">
@@ -28694,7 +28694,7 @@
         <v>2.4</v>
       </c>
       <c r="I261" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="262" ht="62" customHeight="1">
@@ -28724,7 +28724,7 @@
         <v>1.3</v>
       </c>
       <c r="I262" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="263" ht="39.7" customHeight="1">
@@ -28918,11 +28918,11 @@
       </c>
       <c r="C271" s="9" t="inlineStr">
         <is>
-          <t>3.12 m2 x 3.00</t>
+          <t>3.12 m2 x 2.80</t>
         </is>
       </c>
       <c r="D271" s="8" t="n">
-        <v>9.359999999999999</v>
+        <v>8.74</v>
       </c>
       <c r="E271" s="25" t="n">
         <v>6</v>
@@ -29187,7 +29187,7 @@
     <row r="286" ht="39.7" customHeight="1">
       <c r="A286" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  13 - Dormitorio Norte   (PA)</t>
+          <t>LOCAL  13 - Dormitorio Norte   (PA)   -   altura 2.80 m</t>
         </is>
       </c>
       <c r="B286" s="2" t="n"/>
@@ -29463,7 +29463,7 @@
         <v>4.25</v>
       </c>
       <c r="I296" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="297" ht="62" customHeight="1">
@@ -29493,7 +29493,7 @@
         <v>4</v>
       </c>
       <c r="I297" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="298" ht="62" customHeight="1">
@@ -29523,7 +29523,7 @@
         <v>4.25</v>
       </c>
       <c r="I298" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="299" ht="62" customHeight="1">
@@ -29553,7 +29553,7 @@
         <v>4</v>
       </c>
       <c r="I299" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="300" ht="39.7" customHeight="1">
@@ -29770,11 +29770,11 @@
       </c>
       <c r="C309" s="9" t="inlineStr">
         <is>
-          <t>17.00 m2 x 3.00</t>
+          <t>17.00 m2 x 2.80</t>
         </is>
       </c>
       <c r="D309" s="8" t="n">
-        <v>51</v>
+        <v>47.6</v>
       </c>
       <c r="E309" s="25" t="n">
         <v>9</v>
@@ -30016,7 +30016,7 @@
     <row r="323" ht="39.7" customHeight="1">
       <c r="A323" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  14 - Play room   (PA)</t>
+          <t>LOCAL  14 - Play room   (PA)   -   altura 3.00 m</t>
         </is>
       </c>
       <c r="B323" s="2" t="n"/>
@@ -30822,7 +30822,7 @@
     <row r="359" ht="39.7" customHeight="1">
       <c r="A359" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  15 - Dormitorio Sur   (PA)</t>
+          <t>LOCAL  15 - Dormitorio Sur   (PA)   -   altura 2.80 m</t>
         </is>
       </c>
       <c r="B359" s="2" t="n"/>
@@ -31098,7 +31098,7 @@
         <v>3.5</v>
       </c>
       <c r="I369" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="370" ht="62" customHeight="1">
@@ -31128,7 +31128,7 @@
         <v>4.05</v>
       </c>
       <c r="I370" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="371" ht="62" customHeight="1">
@@ -31158,7 +31158,7 @@
         <v>3.5</v>
       </c>
       <c r="I371" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="372" ht="62" customHeight="1">
@@ -31188,7 +31188,7 @@
         <v>4.05</v>
       </c>
       <c r="I372" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="373" ht="39.7" customHeight="1">
@@ -31405,11 +31405,11 @@
       </c>
       <c r="C382" s="9" t="inlineStr">
         <is>
-          <t>14.17 m2 x 3.00</t>
+          <t>14.17 m2 x 2.80</t>
         </is>
       </c>
       <c r="D382" s="8" t="n">
-        <v>42.51</v>
+        <v>39.68</v>
       </c>
       <c r="E382" s="25" t="n">
         <v>9</v>
@@ -31651,7 +31651,7 @@
     <row r="396" ht="39.7" customHeight="1">
       <c r="A396" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  17 - Bano   (PA)</t>
+          <t>LOCAL  17 - Bano   (PA)   -   altura 2.80 m</t>
         </is>
       </c>
       <c r="B396" s="2" t="n"/>
@@ -31897,7 +31897,7 @@
         <v>2.2</v>
       </c>
       <c r="I405" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="406" ht="62" customHeight="1">
@@ -31927,7 +31927,7 @@
         <v>1.6</v>
       </c>
       <c r="I406" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="407" ht="62" customHeight="1">
@@ -31957,7 +31957,7 @@
         <v>2.2</v>
       </c>
       <c r="I407" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="408" ht="62" customHeight="1">
@@ -31987,7 +31987,7 @@
         <v>1.6</v>
       </c>
       <c r="I408" s="35" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="409" ht="39.7" customHeight="1">
@@ -32181,11 +32181,11 @@
       </c>
       <c r="C417" s="9" t="inlineStr">
         <is>
-          <t>3.52 m2 x 3.00</t>
+          <t>3.52 m2 x 2.80</t>
         </is>
       </c>
       <c r="D417" s="8" t="n">
-        <v>10.56</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="E417" s="25" t="n">
         <v>6</v>

</xml_diff>

<commit_message>
Balance termico: el vestidor tiene 1,70 de muro exterior
Del lado largo de 4,87, hay 1,70 que dan al exterior y 3,17 que dan a
locales vecinos. Se parte el muro en los dos tramos.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -25114,7 +25114,7 @@
       <c r="A105" s="9" t="n"/>
       <c r="B105" s="34" t="inlineStr">
         <is>
-          <t>AISLADAS (    )</t>
+          <t>AISLADAS ()</t>
         </is>
       </c>
       <c r="C105" s="9">
@@ -25133,8 +25133,12 @@
         <v/>
       </c>
       <c r="G105" s="2" t="n"/>
-      <c r="H105" s="35" t="n"/>
-      <c r="I105" s="35" t="n"/>
+      <c r="H105" s="35" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="I105" s="35" t="n">
+        <v>2.8</v>
+      </c>
     </row>
     <row r="106" ht="62" customHeight="1">
       <c r="A106" s="9" t="n"/>
@@ -25166,7 +25170,7 @@
       <c r="A107" s="9" t="n"/>
       <c r="B107" s="34" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES (resto del lado largo)</t>
         </is>
       </c>
       <c r="C107" s="9">
@@ -25186,7 +25190,7 @@
       </c>
       <c r="G107" s="2" t="n"/>
       <c r="H107" s="35" t="n">
-        <v>4.87</v>
+        <v>3.17</v>
       </c>
       <c r="I107" s="35" t="n">
         <v>2.8</v>

</xml_diff>

<commit_message>
Unificar las medidas de local entre iluminacion y balance termico
Las medidas relevadas para el balance reemplazan a las de la planilla
original en cuatro locales: living 8,66 x 4,06, hall 3,52 x 2,15, bano
suite 3,38 x 1,72 y play room 4,13 x 4,08. Los trece locales siguen
verificando iluminacion y ventilacion.

Las carpinterias de 3,00 de alto quedan como estan: el cielorraso
suspendido va a 2,80 pero sube a la losa antes de la abertura, por la
garganta de luz. No hay conflicto con la Planilla 3 ni con las areas de
ventana del balance.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -2915,10 +2915,10 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>8.4</v>
+        <v>8.66</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>4</v>
+        <v>4.06</v>
       </c>
       <c r="D8" s="8">
         <f>B8*C8</f>
@@ -2959,7 +2959,7 @@
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>3.5</v>
+        <v>3.52</v>
       </c>
       <c r="C9" s="8" t="n">
         <v>2.15</v>
@@ -3051,10 +3051,10 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>3.3</v>
+        <v>3.38</v>
       </c>
       <c r="C11" s="8" t="n">
-        <v>1.7</v>
+        <v>1.72</v>
       </c>
       <c r="D11" s="8">
         <f>B11*C11</f>
@@ -3269,10 +3269,10 @@
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>4</v>
+        <v>4.13</v>
       </c>
       <c r="C16" s="8" t="n">
-        <v>4.1</v>
+        <v>4.08</v>
       </c>
       <c r="D16" s="8">
         <f>B16*C16</f>

</xml_diff>

<commit_message>
Balance termico: los muros se computan a 3,00 en todos los locales
El cielorraso suspendido de yeso va a 2,80 en varios locales, pero el
muro llega a la losa y el espacio sobre el cielorraso queda dentro de la
envolvente, asi que la pared pierde calor en toda su altura. Se deja sin
efecto la altura reducida del commit anterior.

Total 28.001 kcal/h, 95 elementos y 3 toalleros.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -6720,7 +6720,7 @@
     <row r="54" ht="39.7" customHeight="1">
       <c r="A54" s="23" t="inlineStr">
         <is>
-          <t>Altura de local: 3,00 m en general. En los locales con cielorraso suspendido de yeso (vestidor, suite, bano suite, bano visitas, los dos dormitorios de PA y el bano de PA) la altura libre es 2,80 m, dato del autor del proyecto.</t>
+          <t>Altura de local 3,00 m en todos. Varios tienen cielorraso suspendido de yeso a 2,80, pero el muro llega a la losa y el espacio sobre el cielorraso esta dentro de la envolvente, asi que la pared pierde calor en los 3,00.</t>
         </is>
       </c>
       <c r="B54" s="2" t="n"/>
@@ -24999,7 +24999,7 @@
     <row r="100" ht="39.7" customHeight="1">
       <c r="A100" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  08 - Vestidor   (PB)   -   altura 2.80 m</t>
+          <t>LOCAL  08 - Vestidor   (PB)   -   altura 3.00 m</t>
         </is>
       </c>
       <c r="B100" s="2" t="n"/>
@@ -25137,7 +25137,7 @@
         <v>1.7</v>
       </c>
       <c r="I105" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="106" ht="62" customHeight="1">
@@ -25193,7 +25193,7 @@
         <v>3.17</v>
       </c>
       <c r="I107" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="108" ht="62" customHeight="1">
@@ -25223,7 +25223,7 @@
         <v>3.38</v>
       </c>
       <c r="I108" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="109" ht="62" customHeight="1">
@@ -25253,7 +25253,7 @@
         <v>1.66</v>
       </c>
       <c r="I109" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="110" ht="62" customHeight="1">
@@ -25283,7 +25283,7 @@
         <v>1.49</v>
       </c>
       <c r="I110" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="111" ht="62" customHeight="1">
@@ -25313,7 +25313,7 @@
         <v>1.09</v>
       </c>
       <c r="I111" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="112" ht="62" customHeight="1">
@@ -25343,7 +25343,7 @@
         <v>0.57</v>
       </c>
       <c r="I112" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="113" ht="39.7" customHeight="1">
@@ -25537,11 +25537,11 @@
       </c>
       <c r="C121" s="9" t="inlineStr">
         <is>
-          <t>7.23 m2 x 2.80</t>
+          <t>7.23 m2 x 3.00</t>
         </is>
       </c>
       <c r="D121" s="8" t="n">
-        <v>20.24</v>
+        <v>21.69</v>
       </c>
       <c r="E121" s="25" t="n">
         <v>6</v>
@@ -26456,7 +26456,7 @@
     <row r="165" ht="39.7" customHeight="1">
       <c r="A165" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  09 - Dormitorio suite   (PB)   -   altura 2.80 m</t>
+          <t>LOCAL  09 - Dormitorio suite   (PB)   -   altura 3.00 m</t>
         </is>
       </c>
       <c r="B165" s="2" t="n"/>
@@ -26628,7 +26628,7 @@
         <v>3.5</v>
       </c>
       <c r="I171" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="172" ht="62" customHeight="1">
@@ -26658,7 +26658,7 @@
         <v>3.5</v>
       </c>
       <c r="I172" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="173" ht="62" customHeight="1">
@@ -26688,7 +26688,7 @@
         <v>3.5</v>
       </c>
       <c r="I173" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="174" ht="62" customHeight="1">
@@ -26718,7 +26718,7 @@
         <v>3.5</v>
       </c>
       <c r="I174" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="175" ht="62" customHeight="1">
@@ -26984,11 +26984,11 @@
       </c>
       <c r="C186" s="9" t="inlineStr">
         <is>
-          <t>12.25 m2 x 2.80</t>
+          <t>12.25 m2 x 3.00</t>
         </is>
       </c>
       <c r="D186" s="8" t="n">
-        <v>34.3</v>
+        <v>36.75</v>
       </c>
       <c r="E186" s="25" t="n">
         <v>12</v>
@@ -27207,7 +27207,7 @@
     <row r="199" ht="39.7" customHeight="1">
       <c r="A199" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  10 - Bano suite   (PB)   -   altura 2.80 m</t>
+          <t>LOCAL  10 - Bano suite   (PB)   -   altura 3.00 m</t>
         </is>
       </c>
       <c r="B199" s="2" t="n"/>
@@ -27349,7 +27349,7 @@
         <v>3.38</v>
       </c>
       <c r="I204" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="205" ht="62" customHeight="1">
@@ -27405,7 +27405,7 @@
         <v>1.72</v>
       </c>
       <c r="I206" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="207" ht="62" customHeight="1">
@@ -27435,7 +27435,7 @@
         <v>3.38</v>
       </c>
       <c r="I207" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="208" ht="62" customHeight="1">
@@ -27465,7 +27465,7 @@
         <v>1.72</v>
       </c>
       <c r="I208" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="209" ht="39.7" customHeight="1">
@@ -27659,11 +27659,11 @@
       </c>
       <c r="C217" s="9" t="inlineStr">
         <is>
-          <t>5.81 m2 x 2.80</t>
+          <t>5.81 m2 x 3.00</t>
         </is>
       </c>
       <c r="D217" s="8" t="n">
-        <v>16.27</v>
+        <v>17.43</v>
       </c>
       <c r="E217" s="25" t="n">
         <v>6</v>
@@ -27928,7 +27928,7 @@
     <row r="232" ht="39.7" customHeight="1">
       <c r="A232" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  11 - Bano visitas   (PB)   -   altura 2.80 m</t>
+          <t>LOCAL  11 - Bano visitas   (PB)   -   altura 3.00 m</t>
         </is>
       </c>
       <c r="B232" s="2" t="n"/>
@@ -28066,7 +28066,7 @@
         <v>1.3</v>
       </c>
       <c r="I237" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="238" ht="62" customHeight="1">
@@ -28122,7 +28122,7 @@
         <v>2.4</v>
       </c>
       <c r="I239" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="240" ht="62" customHeight="1">
@@ -28152,7 +28152,7 @@
         <v>2.4</v>
       </c>
       <c r="I240" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="241" ht="62" customHeight="1">
@@ -28182,7 +28182,7 @@
         <v>1.3</v>
       </c>
       <c r="I241" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="242" ht="39.7" customHeight="1">
@@ -28376,11 +28376,11 @@
       </c>
       <c r="C250" s="9" t="inlineStr">
         <is>
-          <t>3.12 m2 x 2.80</t>
+          <t>3.12 m2 x 3.00</t>
         </is>
       </c>
       <c r="D250" s="8" t="n">
-        <v>8.74</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="E250" s="25" t="n">
         <v>6</v>
@@ -28645,7 +28645,7 @@
     <row r="265" ht="39.7" customHeight="1">
       <c r="A265" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  13 - Dormitorio Norte   (PA)   -   altura 2.80 m</t>
+          <t>LOCAL  13 - Dormitorio Norte   (PA)   -   altura 3.00 m</t>
         </is>
       </c>
       <c r="B265" s="2" t="n"/>
@@ -28817,7 +28817,7 @@
         <v>4.25</v>
       </c>
       <c r="I271" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="272" ht="62" customHeight="1">
@@ -28847,7 +28847,7 @@
         <v>4</v>
       </c>
       <c r="I272" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="273" ht="62" customHeight="1">
@@ -28877,7 +28877,7 @@
         <v>4.25</v>
       </c>
       <c r="I273" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="274" ht="62" customHeight="1">
@@ -28907,7 +28907,7 @@
         <v>4</v>
       </c>
       <c r="I274" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="275" ht="62" customHeight="1">
@@ -29173,11 +29173,11 @@
       </c>
       <c r="C286" s="9" t="inlineStr">
         <is>
-          <t>17.00 m2 x 2.80</t>
+          <t>17.00 m2 x 3.00</t>
         </is>
       </c>
       <c r="D286" s="8" t="n">
-        <v>47.6</v>
+        <v>51</v>
       </c>
       <c r="E286" s="25" t="n">
         <v>12</v>
@@ -30124,7 +30124,7 @@
     <row r="332" ht="39.7" customHeight="1">
       <c r="A332" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  15 - Dormitorio Sur   (PA)   -   altura 2.80 m</t>
+          <t>LOCAL  15 - Dormitorio Sur   (PA)   -   altura 3.00 m</t>
         </is>
       </c>
       <c r="B332" s="2" t="n"/>
@@ -30296,7 +30296,7 @@
         <v>4.05</v>
       </c>
       <c r="I338" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="339" ht="62" customHeight="1">
@@ -30326,7 +30326,7 @@
         <v>3.5</v>
       </c>
       <c r="I339" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="340" ht="62" customHeight="1">
@@ -30356,7 +30356,7 @@
         <v>4.05</v>
       </c>
       <c r="I340" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="341" ht="62" customHeight="1">
@@ -30386,7 +30386,7 @@
         <v>3.5</v>
       </c>
       <c r="I341" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="342" ht="39.7" customHeight="1">
@@ -30603,11 +30603,11 @@
       </c>
       <c r="C351" s="9" t="inlineStr">
         <is>
-          <t>14.17 m2 x 2.80</t>
+          <t>14.17 m2 x 3.00</t>
         </is>
       </c>
       <c r="D351" s="8" t="n">
-        <v>39.68</v>
+        <v>42.51</v>
       </c>
       <c r="E351" s="25" t="n">
         <v>9</v>
@@ -30849,7 +30849,7 @@
     <row r="365" ht="39.7" customHeight="1">
       <c r="A365" s="5" t="inlineStr">
         <is>
-          <t>LOCAL  17 - Bano   (PA)   -   altura 2.80 m</t>
+          <t>LOCAL  17 - Bano   (PA)   -   altura 3.00 m</t>
         </is>
       </c>
       <c r="B365" s="2" t="n"/>
@@ -30991,7 +30991,7 @@
         <v>2.2</v>
       </c>
       <c r="I370" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="371" ht="62" customHeight="1">
@@ -31021,7 +31021,7 @@
         <v>1.6</v>
       </c>
       <c r="I371" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="372" ht="62" customHeight="1">
@@ -31051,7 +31051,7 @@
         <v>2.2</v>
       </c>
       <c r="I372" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="373" ht="62" customHeight="1">
@@ -31081,7 +31081,7 @@
         <v>1.6</v>
       </c>
       <c r="I373" s="35" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="374" ht="39.7" customHeight="1">
@@ -31298,11 +31298,11 @@
       </c>
       <c r="C383" s="9" t="inlineStr">
         <is>
-          <t>3.52 m2 x 2.80</t>
+          <t>3.52 m2 x 3.00</t>
         </is>
       </c>
       <c r="D383" s="8" t="n">
-        <v>9.859999999999999</v>
+        <v>10.56</v>
       </c>
       <c r="E383" s="25" t="n">
         <v>9</v>

</xml_diff>

<commit_message>
Planilla 3: orientar las aberturas con el plano de fachadas
El plano de fachadas asigna directamente cada abertura a su vista, asi
que reemplaza a lo que se venia deduciendo de la posicion de los muros.
Y lo contradice: de las trece aberturas dibujadas, solo PV04 y VA05
estaban bien orientadas.

Quedan trece orientadas por el plano, dos deducidas (PV02 va con PF03 y
PV04 (2) con PV04, por estar en el mismo pano) y cinco en un bloque
aparte, a confirmar: PF01 y su gemela del patio interno, VA01 (2), VA04 y
VA04 (2), que no figuran en las cuatro vistas.

La marca amarilla de la Planilla 3 queda sin efecto con este cambio: hay
que revisar la hoja entera.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -31,7 +31,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Iluminacion y ventilacion'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Planilla 3 higrotermica'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla 3 higrotermica'!$A$1:$M$37</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla 3 higrotermica'!$A$1:$M$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Planilla vigas'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Planilla vigas'!$A$1:$X$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Planilla losas'!$1:$3</definedName>
@@ -298,7 +298,6 @@
     <xf numFmtId="167" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -306,6 +305,7 @@
     <xf numFmtId="167" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -8365,7 +8365,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M89"/>
+  <dimension ref="A1:M92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21.6" customWidth="1" min="1" max="1"/>
@@ -8533,7 +8533,7 @@
     <row r="6" ht="39.7" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Plano: Fachada Noreste (borde derecho del plano)</t>
+          <t>Plano: Fachada Noreste</t>
         </is>
       </c>
       <c r="B6" s="4" t="n"/>
@@ -8552,21 +8552,21 @@
     <row r="7" ht="70" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>PV02</t>
+          <t>PA02</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
         <v>3</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>2.48</v>
+        <v>0.75</v>
       </c>
       <c r="D7" s="9">
         <f>IF(COUNT(B7,C7)&lt;2,"",B7*C7)</f>
         <v/>
       </c>
       <c r="E7" s="19">
-        <f>SUM(D7:D12)</f>
+        <f>SUM(D7:D13)</f>
         <v/>
       </c>
       <c r="F7" s="20">
@@ -8605,53 +8605,53 @@
       </c>
     </row>
     <row r="8" ht="70" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>PF03</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C8" s="9" t="n">
-        <v>2.88</v>
-      </c>
-      <c r="D8" s="9">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>VA02</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D8" s="8">
         <f>IF(COUNT(B8,C8)&lt;2,"",B8*C8)</f>
         <v/>
       </c>
-      <c r="E8" s="21" t="n"/>
-      <c r="F8" s="20">
+      <c r="E8" s="22" t="n"/>
+      <c r="F8" s="23">
         <f>IF(OR(D8="",$E$7=""),"",D8/$E$7)</f>
         <v/>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="8">
         <f>IF(A8="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H8" s="10" t="inlineStr">
+      <c r="H8" s="21" t="inlineStr">
         <is>
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I8" s="10" t="inlineStr">
+      <c r="I8" s="21" t="inlineStr">
         <is>
           <t>Sin Proteccion</t>
         </is>
       </c>
-      <c r="J8" s="9" t="n">
+      <c r="J8" s="8" t="n">
         <v>2.8</v>
       </c>
-      <c r="K8" s="10" t="inlineStr">
+      <c r="K8" s="21" t="inlineStr">
         <is>
           <t>Noreste</t>
         </is>
       </c>
-      <c r="L8" s="9">
+      <c r="L8" s="8">
         <f>IF(I8="","",IFERROR(VLOOKUP(I8,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
-      <c r="M8" s="10">
+      <c r="M8" s="21">
         <f>IF(OR(D8="",J8=""),"",IF(J8&lt;=G8,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
@@ -8659,20 +8659,20 @@
     <row r="9" ht="70" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>VA04</t>
+          <t>PV03</t>
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>2.52</v>
+        <v>3</v>
       </c>
       <c r="C9" s="9" t="n">
-        <v>2</v>
+        <v>1.76</v>
       </c>
       <c r="D9" s="9">
         <f>IF(COUNT(B9,C9)&lt;2,"",B9*C9)</f>
         <v/>
       </c>
-      <c r="E9" s="21" t="n"/>
+      <c r="E9" s="24" t="n"/>
       <c r="F9" s="20">
         <f>IF(OR(D9="",$E$7=""),"",D9/$E$7)</f>
         <v/>
@@ -8709,66 +8709,74 @@
       </c>
     </row>
     <row r="10" ht="70" customHeight="1">
-      <c r="A10" s="22" t="inlineStr">
-        <is>
-          <t>PF01 (2)</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="C10" s="8" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="D10" s="8">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>VA03</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D10" s="9">
         <f>IF(COUNT(B10,C10)&lt;2,"",B10*C10)</f>
         <v/>
       </c>
-      <c r="E10" s="23" t="n"/>
-      <c r="F10" s="24">
+      <c r="E10" s="24" t="n"/>
+      <c r="F10" s="20">
         <f>IF(OR(D10="",$E$7=""),"",D10/$E$7)</f>
         <v/>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="9">
         <f>IF(A10="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H10" s="22" t="inlineStr">
+      <c r="H10" s="10" t="inlineStr">
         <is>
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I10" s="22" t="inlineStr">
+      <c r="I10" s="10" t="inlineStr">
         <is>
           <t>Sin Proteccion</t>
         </is>
       </c>
-      <c r="J10" s="8" t="n">
+      <c r="J10" s="9" t="n">
         <v>2.8</v>
       </c>
-      <c r="K10" s="22" t="inlineStr">
+      <c r="K10" s="10" t="inlineStr">
         <is>
           <t>Noreste</t>
         </is>
       </c>
-      <c r="L10" s="8">
+      <c r="L10" s="9">
         <f>IF(I10="","",IFERROR(VLOOKUP(I10,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
-      <c r="M10" s="22">
+      <c r="M10" s="10">
         <f>IF(OR(D10="",J10=""),"",IF(J10&lt;=G10,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="70" customHeight="1">
-      <c r="A11" s="10" t="n"/>
-      <c r="B11" s="9" t="n"/>
-      <c r="C11" s="9" t="n"/>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>PF05</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>0.75</v>
+      </c>
       <c r="D11" s="9">
         <f>IF(COUNT(B11,C11)&lt;2,"",B11*C11)</f>
         <v/>
       </c>
-      <c r="E11" s="21" t="n"/>
+      <c r="E11" s="24" t="n"/>
       <c r="F11" s="20">
         <f>IF(OR(D11="",$E$7=""),"",D11/$E$7)</f>
         <v/>
@@ -8777,10 +8785,24 @@
         <f>IF(A11="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H11" s="10" t="n"/>
-      <c r="I11" s="10" t="n"/>
-      <c r="J11" s="9" t="n"/>
-      <c r="K11" s="10" t="n"/>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K11" s="10" t="inlineStr">
+        <is>
+          <t>Noreste</t>
+        </is>
+      </c>
       <c r="L11" s="9">
         <f>IF(I11="","",IFERROR(VLOOKUP(I11,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
@@ -8791,395 +8813,373 @@
       </c>
     </row>
     <row r="12" ht="70" customHeight="1">
-      <c r="A12" s="14" t="n"/>
-      <c r="B12" s="13" t="n"/>
-      <c r="C12" s="13" t="n"/>
-      <c r="D12" s="13">
+      <c r="A12" s="10" t="n"/>
+      <c r="B12" s="9" t="n"/>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="9">
         <f>IF(COUNT(B12,C12)&lt;2,"",B12*C12)</f>
         <v/>
       </c>
-      <c r="E12" s="25" t="n"/>
-      <c r="F12" s="26">
+      <c r="E12" s="24" t="n"/>
+      <c r="F12" s="20">
         <f>IF(OR(D12="",$E$7=""),"",D12/$E$7)</f>
         <v/>
       </c>
-      <c r="G12" s="13">
+      <c r="G12" s="9">
         <f>IF(A12="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H12" s="14" t="n"/>
-      <c r="I12" s="14" t="n"/>
-      <c r="J12" s="13" t="n"/>
-      <c r="K12" s="14" t="n"/>
-      <c r="L12" s="13">
+      <c r="H12" s="10" t="n"/>
+      <c r="I12" s="10" t="n"/>
+      <c r="J12" s="9" t="n"/>
+      <c r="K12" s="10" t="n"/>
+      <c r="L12" s="9">
         <f>IF(I12="","",IFERROR(VLOOKUP(I12,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
-      <c r="M12" s="14">
+      <c r="M12" s="10">
         <f>IF(OR(D12="",J12=""),"",IF(J12&lt;=G12,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="13" ht="39.7" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Plano: Fachada Sudoeste (borde izquierdo)</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="4" t="n"/>
-      <c r="E13" s="4" t="n"/>
-      <c r="F13" s="4" t="n"/>
-      <c r="G13" s="4" t="n"/>
-      <c r="H13" s="4" t="n"/>
-      <c r="I13" s="4" t="n"/>
-      <c r="J13" s="4" t="n"/>
-      <c r="K13" s="4" t="n"/>
-      <c r="L13" s="4" t="n"/>
-      <c r="M13" s="4" t="n"/>
-    </row>
-    <row r="14" ht="70" customHeight="1">
-      <c r="A14" s="22" t="inlineStr">
-        <is>
-          <t>PF01</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="n">
+    <row r="13" ht="70" customHeight="1">
+      <c r="A13" s="14" t="n"/>
+      <c r="B13" s="13" t="n"/>
+      <c r="C13" s="13" t="n"/>
+      <c r="D13" s="13">
+        <f>IF(COUNT(B13,C13)&lt;2,"",B13*C13)</f>
+        <v/>
+      </c>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="26">
+        <f>IF(OR(D13="",$E$7=""),"",D13/$E$7)</f>
+        <v/>
+      </c>
+      <c r="G13" s="13">
+        <f>IF(A13="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H13" s="14" t="n"/>
+      <c r="I13" s="14" t="n"/>
+      <c r="J13" s="13" t="n"/>
+      <c r="K13" s="14" t="n"/>
+      <c r="L13" s="13">
+        <f>IF(I13="","",IFERROR(VLOOKUP(I13,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M13" s="14">
+        <f>IF(OR(D13="",J13=""),"",IF(J13&lt;=G13,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="39.7" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Plano: Fachada Sudoeste</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+      <c r="D14" s="4" t="n"/>
+      <c r="E14" s="4" t="n"/>
+      <c r="F14" s="4" t="n"/>
+      <c r="G14" s="4" t="n"/>
+      <c r="H14" s="4" t="n"/>
+      <c r="I14" s="4" t="n"/>
+      <c r="J14" s="4" t="n"/>
+      <c r="K14" s="4" t="n"/>
+      <c r="L14" s="4" t="n"/>
+      <c r="M14" s="4" t="n"/>
+    </row>
+    <row r="15" ht="70" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>PA01</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="C14" s="8" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="D14" s="8">
-        <f>IF(COUNT(B14,C14)&lt;2,"",B14*C14)</f>
-        <v/>
-      </c>
-      <c r="E14" s="27">
-        <f>SUM(D14:D17)</f>
-        <v/>
-      </c>
-      <c r="F14" s="24">
-        <f>IF(OR(D14="",$E$14=""),"",D14/$E$14)</f>
-        <v/>
-      </c>
-      <c r="G14" s="8">
-        <f>IF(A14="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H14" s="22" t="inlineStr">
+      <c r="C15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="9">
+        <f>IF(COUNT(B15,C15)&lt;2,"",B15*C15)</f>
+        <v/>
+      </c>
+      <c r="E15" s="19">
+        <f>SUM(D15:D19)</f>
+        <v/>
+      </c>
+      <c r="F15" s="20">
+        <f>IF(OR(D15="",$E$15=""),"",D15/$E$15)</f>
+        <v/>
+      </c>
+      <c r="G15" s="9">
+        <f>IF(A15="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
         <is>
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I14" s="22" t="inlineStr">
+      <c r="I15" s="10" t="inlineStr">
         <is>
           <t>Sin Proteccion</t>
         </is>
       </c>
-      <c r="J14" s="8" t="n">
+      <c r="J15" s="9" t="n">
         <v>2.8</v>
       </c>
-      <c r="K14" s="22" t="inlineStr">
+      <c r="K15" s="10" t="inlineStr">
         <is>
           <t>Sudoeste</t>
         </is>
       </c>
-      <c r="L14" s="8">
-        <f>IF(I14="","",IFERROR(VLOOKUP(I14,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M14" s="22">
-        <f>IF(OR(D14="",J14=""),"",IF(J14&lt;=G14,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="70" customHeight="1">
-      <c r="A15" s="22" t="inlineStr">
-        <is>
-          <t>VA02</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="n">
-        <v>2.15</v>
-      </c>
-      <c r="C15" s="8" t="n">
+      <c r="L15" s="9">
+        <f>IF(I15="","",IFERROR(VLOOKUP(I15,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M15" s="10">
+        <f>IF(OR(D15="",J15=""),"",IF(J15&lt;=G15,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="70" customHeight="1">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>PF04</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C16" s="8" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="D16" s="8">
+        <f>IF(COUNT(B16,C16)&lt;2,"",B16*C16)</f>
+        <v/>
+      </c>
+      <c r="E16" s="22" t="n"/>
+      <c r="F16" s="23">
+        <f>IF(OR(D16="",$E$15=""),"",D16/$E$15)</f>
+        <v/>
+      </c>
+      <c r="G16" s="8">
+        <f>IF(A16="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H16" s="21" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I16" s="21" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K16" s="21" t="inlineStr">
+        <is>
+          <t>Sudoeste</t>
+        </is>
+      </c>
+      <c r="L16" s="8">
+        <f>IF(I16="","",IFERROR(VLOOKUP(I16,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M16" s="21">
+        <f>IF(OR(D16="",J16=""),"",IF(J16&lt;=G16,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="70" customHeight="1">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>VA01</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" s="8" t="n">
         <v>0.75</v>
       </c>
-      <c r="D15" s="8">
-        <f>IF(COUNT(B15,C15)&lt;2,"",B15*C15)</f>
-        <v/>
-      </c>
-      <c r="E15" s="23" t="n"/>
-      <c r="F15" s="24">
-        <f>IF(OR(D15="",$E$14=""),"",D15/$E$14)</f>
-        <v/>
-      </c>
-      <c r="G15" s="8">
-        <f>IF(A15="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H15" s="22" t="inlineStr">
+      <c r="D17" s="8">
+        <f>IF(COUNT(B17,C17)&lt;2,"",B17*C17)</f>
+        <v/>
+      </c>
+      <c r="E17" s="22" t="n"/>
+      <c r="F17" s="23">
+        <f>IF(OR(D17="",$E$15=""),"",D17/$E$15)</f>
+        <v/>
+      </c>
+      <c r="G17" s="8">
+        <f>IF(A17="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H17" s="21" t="inlineStr">
         <is>
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I15" s="22" t="inlineStr">
+      <c r="I17" s="21" t="inlineStr">
         <is>
           <t>Sin Proteccion</t>
         </is>
       </c>
-      <c r="J15" s="8" t="n">
+      <c r="J17" s="8" t="n">
         <v>2.8</v>
       </c>
-      <c r="K15" s="22" t="inlineStr">
+      <c r="K17" s="21" t="inlineStr">
         <is>
           <t>Sudoeste</t>
         </is>
       </c>
-      <c r="L15" s="8">
-        <f>IF(I15="","",IFERROR(VLOOKUP(I15,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M15" s="22">
-        <f>IF(OR(D15="",J15=""),"",IF(J15&lt;=G15,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="70" customHeight="1">
-      <c r="A16" s="10" t="n"/>
-      <c r="B16" s="9" t="n"/>
-      <c r="C16" s="9" t="n"/>
-      <c r="D16" s="9">
-        <f>IF(COUNT(B16,C16)&lt;2,"",B16*C16)</f>
-        <v/>
-      </c>
-      <c r="E16" s="21" t="n"/>
-      <c r="F16" s="20">
-        <f>IF(OR(D16="",$E$14=""),"",D16/$E$14)</f>
-        <v/>
-      </c>
-      <c r="G16" s="9">
-        <f>IF(A16="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H16" s="10" t="n"/>
-      <c r="I16" s="10" t="n"/>
-      <c r="J16" s="9" t="n"/>
-      <c r="K16" s="10" t="n"/>
-      <c r="L16" s="9">
-        <f>IF(I16="","",IFERROR(VLOOKUP(I16,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M16" s="10">
-        <f>IF(OR(D16="",J16=""),"",IF(J16&lt;=G16,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="70" customHeight="1">
-      <c r="A17" s="14" t="n"/>
-      <c r="B17" s="13" t="n"/>
-      <c r="C17" s="13" t="n"/>
-      <c r="D17" s="13">
-        <f>IF(COUNT(B17,C17)&lt;2,"",B17*C17)</f>
-        <v/>
-      </c>
-      <c r="E17" s="25" t="n"/>
-      <c r="F17" s="26">
-        <f>IF(OR(D17="",$E$14=""),"",D17/$E$14)</f>
-        <v/>
-      </c>
-      <c r="G17" s="13">
-        <f>IF(A17="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H17" s="14" t="n"/>
-      <c r="I17" s="14" t="n"/>
-      <c r="J17" s="13" t="n"/>
-      <c r="K17" s="14" t="n"/>
-      <c r="L17" s="13">
+      <c r="L17" s="8">
         <f>IF(I17="","",IFERROR(VLOOKUP(I17,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
-      <c r="M17" s="14">
+      <c r="M17" s="21">
         <f>IF(OR(D17="",J17=""),"",IF(J17&lt;=G17,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="18" ht="39.7" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Plano: Fachada Sudeste (borde inferior)</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="n"/>
-      <c r="C18" s="4" t="n"/>
-      <c r="D18" s="4" t="n"/>
-      <c r="E18" s="4" t="n"/>
-      <c r="F18" s="4" t="n"/>
-      <c r="G18" s="4" t="n"/>
-      <c r="H18" s="4" t="n"/>
-      <c r="I18" s="4" t="n"/>
-      <c r="J18" s="4" t="n"/>
-      <c r="K18" s="4" t="n"/>
-      <c r="L18" s="4" t="n"/>
-      <c r="M18" s="4" t="n"/>
+    <row r="18" ht="70" customHeight="1">
+      <c r="A18" s="10" t="n"/>
+      <c r="B18" s="9" t="n"/>
+      <c r="C18" s="9" t="n"/>
+      <c r="D18" s="9">
+        <f>IF(COUNT(B18,C18)&lt;2,"",B18*C18)</f>
+        <v/>
+      </c>
+      <c r="E18" s="24" t="n"/>
+      <c r="F18" s="20">
+        <f>IF(OR(D18="",$E$15=""),"",D18/$E$15)</f>
+        <v/>
+      </c>
+      <c r="G18" s="9">
+        <f>IF(A18="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H18" s="10" t="n"/>
+      <c r="I18" s="10" t="n"/>
+      <c r="J18" s="9" t="n"/>
+      <c r="K18" s="10" t="n"/>
+      <c r="L18" s="9">
+        <f>IF(I18="","",IFERROR(VLOOKUP(I18,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M18" s="10">
+        <f>IF(OR(D18="",J18=""),"",IF(J18&lt;=G18,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
     </row>
     <row r="19" ht="70" customHeight="1">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>PA01</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="n">
+      <c r="A19" s="14" t="n"/>
+      <c r="B19" s="13" t="n"/>
+      <c r="C19" s="13" t="n"/>
+      <c r="D19" s="13">
+        <f>IF(COUNT(B19,C19)&lt;2,"",B19*C19)</f>
+        <v/>
+      </c>
+      <c r="E19" s="25" t="n"/>
+      <c r="F19" s="26">
+        <f>IF(OR(D19="",$E$15=""),"",D19/$E$15)</f>
+        <v/>
+      </c>
+      <c r="G19" s="13">
+        <f>IF(A19="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H19" s="14" t="n"/>
+      <c r="I19" s="14" t="n"/>
+      <c r="J19" s="13" t="n"/>
+      <c r="K19" s="14" t="n"/>
+      <c r="L19" s="13">
+        <f>IF(I19="","",IFERROR(VLOOKUP(I19,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M19" s="14">
+        <f>IF(OR(D19="",J19=""),"",IF(J19&lt;=G19,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="39.7" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Plano: Fachada Sudeste</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n"/>
+      <c r="C20" s="4" t="n"/>
+      <c r="D20" s="4" t="n"/>
+      <c r="E20" s="4" t="n"/>
+      <c r="F20" s="4" t="n"/>
+      <c r="G20" s="4" t="n"/>
+      <c r="H20" s="4" t="n"/>
+      <c r="I20" s="4" t="n"/>
+      <c r="J20" s="4" t="n"/>
+      <c r="K20" s="4" t="n"/>
+      <c r="L20" s="4" t="n"/>
+      <c r="M20" s="4" t="n"/>
+    </row>
+    <row r="21" ht="70" customHeight="1">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>PF02</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="C19" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="9">
-        <f>IF(COUNT(B19,C19)&lt;2,"",B19*C19)</f>
-        <v/>
-      </c>
-      <c r="E19" s="19">
-        <f>SUM(D19:D26)</f>
-        <v/>
-      </c>
-      <c r="F19" s="20">
-        <f>IF(OR(D19="",$E$19=""),"",D19/$E$19)</f>
-        <v/>
-      </c>
-      <c r="G19" s="9">
-        <f>IF(A19="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H19" s="10" t="inlineStr">
+      <c r="C21" s="8" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D21" s="8">
+        <f>IF(COUNT(B21,C21)&lt;2,"",B21*C21)</f>
+        <v/>
+      </c>
+      <c r="E21" s="27">
+        <f>SUM(D21:D26)</f>
+        <v/>
+      </c>
+      <c r="F21" s="23">
+        <f>IF(OR(D21="",$E$21=""),"",D21/$E$21)</f>
+        <v/>
+      </c>
+      <c r="G21" s="8">
+        <f>IF(A21="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H21" s="21" t="inlineStr">
         <is>
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I19" s="10" t="inlineStr">
+      <c r="I21" s="21" t="inlineStr">
         <is>
           <t>Sin Proteccion</t>
         </is>
       </c>
-      <c r="J19" s="9" t="n">
+      <c r="J21" s="8" t="n">
         <v>2.8</v>
       </c>
-      <c r="K19" s="10" t="inlineStr">
+      <c r="K21" s="21" t="inlineStr">
         <is>
           <t>Sudeste</t>
         </is>
       </c>
-      <c r="L19" s="9">
-        <f>IF(I19="","",IFERROR(VLOOKUP(I19,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M19" s="10">
-        <f>IF(OR(D19="",J19=""),"",IF(J19&lt;=G19,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="70" customHeight="1">
-      <c r="A20" s="22" t="inlineStr">
-        <is>
-          <t>PV01</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="C20" s="8" t="n">
-        <v>7.7</v>
-      </c>
-      <c r="D20" s="8">
-        <f>IF(COUNT(B20,C20)&lt;2,"",B20*C20)</f>
-        <v/>
-      </c>
-      <c r="E20" s="23" t="n"/>
-      <c r="F20" s="24">
-        <f>IF(OR(D20="",$E$19=""),"",D20/$E$19)</f>
-        <v/>
-      </c>
-      <c r="G20" s="8">
-        <f>IF(A20="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H20" s="22" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I20" s="22" t="inlineStr">
-        <is>
-          <t>Sin Proteccion</t>
-        </is>
-      </c>
-      <c r="J20" s="8" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K20" s="22" t="inlineStr">
-        <is>
-          <t>Sudeste</t>
-        </is>
-      </c>
-      <c r="L20" s="8">
-        <f>IF(I20="","",IFERROR(VLOOKUP(I20,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M20" s="22">
-        <f>IF(OR(D20="",J20=""),"",IF(J20&lt;=G20,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="70" customHeight="1">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>VA01 (2)</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C21" s="9" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D21" s="9">
-        <f>IF(COUNT(B21,C21)&lt;2,"",B21*C21)</f>
-        <v/>
-      </c>
-      <c r="E21" s="21" t="n"/>
-      <c r="F21" s="20">
-        <f>IF(OR(D21="",$E$19=""),"",D21/$E$19)</f>
-        <v/>
-      </c>
-      <c r="G21" s="9">
-        <f>IF(A21="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H21" s="10" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I21" s="10" t="inlineStr">
-        <is>
-          <t>Sin Proteccion</t>
-        </is>
-      </c>
-      <c r="J21" s="9" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K21" s="10" t="inlineStr">
-        <is>
-          <t>Sudeste</t>
-        </is>
-      </c>
-      <c r="L21" s="9">
+      <c r="L21" s="8">
         <f>IF(I21="","",IFERROR(VLOOKUP(I21,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
-      <c r="M21" s="10">
+      <c r="M21" s="21">
         <f>IF(OR(D21="",J21=""),"",IF(J21&lt;=G21,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
@@ -9187,22 +9187,22 @@
     <row r="22" ht="70" customHeight="1">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>VA05</t>
+          <t>PV04</t>
         </is>
       </c>
       <c r="B22" s="9" t="n">
-        <v>2.52</v>
+        <v>3</v>
       </c>
       <c r="C22" s="9" t="n">
-        <v>1.4</v>
+        <v>2.06</v>
       </c>
       <c r="D22" s="9">
         <f>IF(COUNT(B22,C22)&lt;2,"",B22*C22)</f>
         <v/>
       </c>
-      <c r="E22" s="21" t="n"/>
+      <c r="E22" s="24" t="n"/>
       <c r="F22" s="20">
-        <f>IF(OR(D22="",$E$19=""),"",D22/$E$19)</f>
+        <f>IF(OR(D22="",$E$21=""),"",D22/$E$21)</f>
         <v/>
       </c>
       <c r="G22" s="9">
@@ -9239,22 +9239,22 @@
     <row r="23" ht="70" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>PV04</t>
+          <t>PV04 (2)</t>
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>3</v>
+        <v>2.95</v>
       </c>
       <c r="C23" s="9" t="n">
-        <v>2.06</v>
+        <v>1.5</v>
       </c>
       <c r="D23" s="9">
         <f>IF(COUNT(B23,C23)&lt;2,"",B23*C23)</f>
         <v/>
       </c>
-      <c r="E23" s="21" t="n"/>
+      <c r="E23" s="24" t="n"/>
       <c r="F23" s="20">
-        <f>IF(OR(D23="",$E$19=""),"",D23/$E$19)</f>
+        <f>IF(OR(D23="",$E$21=""),"",D23/$E$21)</f>
         <v/>
       </c>
       <c r="G23" s="9">
@@ -9291,22 +9291,22 @@
     <row r="24" ht="70" customHeight="1">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>PV04 (2)</t>
+          <t>VA05</t>
         </is>
       </c>
       <c r="B24" s="9" t="n">
-        <v>2.95</v>
+        <v>2.52</v>
       </c>
       <c r="C24" s="9" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="D24" s="9">
         <f>IF(COUNT(B24,C24)&lt;2,"",B24*C24)</f>
         <v/>
       </c>
-      <c r="E24" s="21" t="n"/>
+      <c r="E24" s="24" t="n"/>
       <c r="F24" s="20">
-        <f>IF(OR(D24="",$E$19=""),"",D24/$E$19)</f>
+        <f>IF(OR(D24="",$E$21=""),"",D24/$E$21)</f>
         <v/>
       </c>
       <c r="G24" s="9">
@@ -9348,9 +9348,9 @@
         <f>IF(COUNT(B25,C25)&lt;2,"",B25*C25)</f>
         <v/>
       </c>
-      <c r="E25" s="21" t="n"/>
+      <c r="E25" s="24" t="n"/>
       <c r="F25" s="20">
-        <f>IF(OR(D25="",$E$19=""),"",D25/$E$19)</f>
+        <f>IF(OR(D25="",$E$21=""),"",D25/$E$21)</f>
         <v/>
       </c>
       <c r="G25" s="9">
@@ -9380,7 +9380,7 @@
       </c>
       <c r="E26" s="25" t="n"/>
       <c r="F26" s="26">
-        <f>IF(OR(D26="",$E$19=""),"",D26/$E$19)</f>
+        <f>IF(OR(D26="",$E$21=""),"",D26/$E$21)</f>
         <v/>
       </c>
       <c r="G26" s="13">
@@ -9403,7 +9403,7 @@
     <row r="27" ht="39.7" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Plano: Fachada Noroeste (borde superior)</t>
+          <t>Plano: Fachada Noroeste</t>
         </is>
       </c>
       <c r="B27" s="4" t="n"/>
@@ -9420,78 +9420,78 @@
       <c r="M27" s="4" t="n"/>
     </row>
     <row r="28" ht="70" customHeight="1">
-      <c r="A28" s="22" t="inlineStr">
-        <is>
-          <t>PF02</t>
-        </is>
-      </c>
-      <c r="B28" s="8" t="n">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>PF03</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="C28" s="8" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="D28" s="8">
+      <c r="C28" s="9" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="D28" s="9">
         <f>IF(COUNT(B28,C28)&lt;2,"",B28*C28)</f>
         <v/>
       </c>
-      <c r="E28" s="27">
-        <f>SUM(D28:D37)</f>
-        <v/>
-      </c>
-      <c r="F28" s="24">
+      <c r="E28" s="19">
+        <f>SUM(D28:D32)</f>
+        <v/>
+      </c>
+      <c r="F28" s="20">
         <f>IF(OR(D28="",$E$28=""),"",D28/$E$28)</f>
         <v/>
       </c>
-      <c r="G28" s="8">
+      <c r="G28" s="9">
         <f>IF(A28="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H28" s="22" t="inlineStr">
+      <c r="H28" s="10" t="inlineStr">
         <is>
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I28" s="22" t="inlineStr">
+      <c r="I28" s="10" t="inlineStr">
         <is>
           <t>Sin Proteccion</t>
         </is>
       </c>
-      <c r="J28" s="8" t="n">
+      <c r="J28" s="9" t="n">
         <v>2.8</v>
       </c>
-      <c r="K28" s="22" t="inlineStr">
+      <c r="K28" s="10" t="inlineStr">
         <is>
           <t>Noroeste</t>
         </is>
       </c>
-      <c r="L28" s="8">
+      <c r="L28" s="9">
         <f>IF(I28="","",IFERROR(VLOOKUP(I28,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
-      <c r="M28" s="22">
+      <c r="M28" s="10">
         <f>IF(OR(D28="",J28=""),"",IF(J28&lt;=G28,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
     <row r="29" ht="70" customHeight="1">
-      <c r="A29" s="22" t="inlineStr">
-        <is>
-          <t>VA04 (2)</t>
+      <c r="A29" s="21" t="inlineStr">
+        <is>
+          <t>PV01</t>
         </is>
       </c>
       <c r="B29" s="8" t="n">
-        <v>2.52</v>
+        <v>3</v>
       </c>
       <c r="C29" s="8" t="n">
-        <v>2</v>
+        <v>7.7</v>
       </c>
       <c r="D29" s="8">
         <f>IF(COUNT(B29,C29)&lt;2,"",B29*C29)</f>
         <v/>
       </c>
-      <c r="E29" s="23" t="n"/>
-      <c r="F29" s="24">
+      <c r="E29" s="22" t="n"/>
+      <c r="F29" s="23">
         <f>IF(OR(D29="",$E$28=""),"",D29/$E$28)</f>
         <v/>
       </c>
@@ -9499,12 +9499,12 @@
         <f>IF(A29="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H29" s="22" t="inlineStr">
+      <c r="H29" s="21" t="inlineStr">
         <is>
           <t>DVH 6+9+3+3 (aluminio linea A30)</t>
         </is>
       </c>
-      <c r="I29" s="22" t="inlineStr">
+      <c r="I29" s="21" t="inlineStr">
         <is>
           <t>Sin Proteccion</t>
         </is>
@@ -9512,7 +9512,7 @@
       <c r="J29" s="8" t="n">
         <v>2.8</v>
       </c>
-      <c r="K29" s="22" t="inlineStr">
+      <c r="K29" s="21" t="inlineStr">
         <is>
           <t>Noroeste</t>
         </is>
@@ -9521,7 +9521,7 @@
         <f>IF(I29="","",IFERROR(VLOOKUP(I29,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
-      <c r="M29" s="22">
+      <c r="M29" s="21">
         <f>IF(OR(D29="",J29=""),"",IF(J29&lt;=G29,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
@@ -9529,20 +9529,20 @@
     <row r="30" ht="70" customHeight="1">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>PV03</t>
+          <t>PV02</t>
         </is>
       </c>
       <c r="B30" s="9" t="n">
         <v>3</v>
       </c>
       <c r="C30" s="9" t="n">
-        <v>1.76</v>
+        <v>2.48</v>
       </c>
       <c r="D30" s="9">
         <f>IF(COUNT(B30,C30)&lt;2,"",B30*C30)</f>
         <v/>
       </c>
-      <c r="E30" s="21" t="n"/>
+      <c r="E30" s="24" t="n"/>
       <c r="F30" s="20">
         <f>IF(OR(D30="",$E$28=""),"",D30/$E$28)</f>
         <v/>
@@ -9579,285 +9579,221 @@
       </c>
     </row>
     <row r="31" ht="70" customHeight="1">
-      <c r="A31" s="22" t="inlineStr">
-        <is>
-          <t>VA01</t>
-        </is>
-      </c>
-      <c r="B31" s="8" t="n">
+      <c r="A31" s="10" t="n"/>
+      <c r="B31" s="9" t="n"/>
+      <c r="C31" s="9" t="n"/>
+      <c r="D31" s="9">
+        <f>IF(COUNT(B31,C31)&lt;2,"",B31*C31)</f>
+        <v/>
+      </c>
+      <c r="E31" s="24" t="n"/>
+      <c r="F31" s="20">
+        <f>IF(OR(D31="",$E$28=""),"",D31/$E$28)</f>
+        <v/>
+      </c>
+      <c r="G31" s="9">
+        <f>IF(A31="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H31" s="10" t="n"/>
+      <c r="I31" s="10" t="n"/>
+      <c r="J31" s="9" t="n"/>
+      <c r="K31" s="10" t="n"/>
+      <c r="L31" s="9">
+        <f>IF(I31="","",IFERROR(VLOOKUP(I31,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M31" s="10">
+        <f>IF(OR(D31="",J31=""),"",IF(J31&lt;=G31,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="70" customHeight="1">
+      <c r="A32" s="14" t="n"/>
+      <c r="B32" s="13" t="n"/>
+      <c r="C32" s="13" t="n"/>
+      <c r="D32" s="13">
+        <f>IF(COUNT(B32,C32)&lt;2,"",B32*C32)</f>
+        <v/>
+      </c>
+      <c r="E32" s="25" t="n"/>
+      <c r="F32" s="26">
+        <f>IF(OR(D32="",$E$28=""),"",D32/$E$28)</f>
+        <v/>
+      </c>
+      <c r="G32" s="13">
+        <f>IF(A32="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H32" s="14" t="n"/>
+      <c r="I32" s="14" t="n"/>
+      <c r="J32" s="13" t="n"/>
+      <c r="K32" s="14" t="n"/>
+      <c r="L32" s="13">
+        <f>IF(I32="","",IFERROR(VLOOKUP(I32,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M32" s="14">
+        <f>IF(OR(D32="",J32=""),"",IF(J32&lt;=G32,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="39.7" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Plano: Orientacion a confirmar</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="n"/>
+      <c r="C33" s="4" t="n"/>
+      <c r="D33" s="4" t="n"/>
+      <c r="E33" s="4" t="n"/>
+      <c r="F33" s="4" t="n"/>
+      <c r="G33" s="4" t="n"/>
+      <c r="H33" s="4" t="n"/>
+      <c r="I33" s="4" t="n"/>
+      <c r="J33" s="4" t="n"/>
+      <c r="K33" s="4" t="n"/>
+      <c r="L33" s="4" t="n"/>
+      <c r="M33" s="4" t="n"/>
+    </row>
+    <row r="34" ht="70" customHeight="1">
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>PF01</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="C31" s="8" t="n">
+      <c r="C34" s="8" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="D34" s="8">
+        <f>IF(COUNT(B34,C34)&lt;2,"",B34*C34)</f>
+        <v/>
+      </c>
+      <c r="E34" s="27">
+        <f>SUM(D34:D40)</f>
+        <v/>
+      </c>
+      <c r="F34" s="23">
+        <f>IF(OR(D34="",$E$34=""),"",D34/$E$34)</f>
+        <v/>
+      </c>
+      <c r="G34" s="8">
+        <f>IF(A34="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H34" s="21" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I34" s="21" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J34" s="8" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K34" s="21" t="n"/>
+      <c r="L34" s="8">
+        <f>IF(I34="","",IFERROR(VLOOKUP(I34,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M34" s="21">
+        <f>IF(OR(D34="",J34=""),"",IF(J34&lt;=G34,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="70" customHeight="1">
+      <c r="A35" s="21" t="inlineStr">
+        <is>
+          <t>PF01 (2)</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C35" s="8" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="D35" s="8">
+        <f>IF(COUNT(B35,C35)&lt;2,"",B35*C35)</f>
+        <v/>
+      </c>
+      <c r="E35" s="22" t="n"/>
+      <c r="F35" s="23">
+        <f>IF(OR(D35="",$E$34=""),"",D35/$E$34)</f>
+        <v/>
+      </c>
+      <c r="G35" s="8">
+        <f>IF(A35="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H35" s="21" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I35" s="21" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J35" s="8" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K35" s="21" t="n"/>
+      <c r="L35" s="8">
+        <f>IF(I35="","",IFERROR(VLOOKUP(I35,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M35" s="21">
+        <f>IF(OR(D35="",J35=""),"",IF(J35&lt;=G35,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="70" customHeight="1">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>VA01 (2)</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C36" s="9" t="n">
         <v>0.75</v>
       </c>
-      <c r="D31" s="8">
-        <f>IF(COUNT(B31,C31)&lt;2,"",B31*C31)</f>
-        <v/>
-      </c>
-      <c r="E31" s="23" t="n"/>
-      <c r="F31" s="24">
-        <f>IF(OR(D31="",$E$28=""),"",D31/$E$28)</f>
-        <v/>
-      </c>
-      <c r="G31" s="8">
-        <f>IF(A31="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H31" s="22" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I31" s="22" t="inlineStr">
-        <is>
-          <t>Sin Proteccion</t>
-        </is>
-      </c>
-      <c r="J31" s="8" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K31" s="22" t="inlineStr">
-        <is>
-          <t>Noroeste</t>
-        </is>
-      </c>
-      <c r="L31" s="8">
-        <f>IF(I31="","",IFERROR(VLOOKUP(I31,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M31" s="22">
-        <f>IF(OR(D31="",J31=""),"",IF(J31&lt;=G31,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="70" customHeight="1">
-      <c r="A32" s="22" t="inlineStr">
-        <is>
-          <t>PF04</t>
-        </is>
-      </c>
-      <c r="B32" s="8" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="C32" s="8" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="D32" s="8">
-        <f>IF(COUNT(B32,C32)&lt;2,"",B32*C32)</f>
-        <v/>
-      </c>
-      <c r="E32" s="23" t="n"/>
-      <c r="F32" s="24">
-        <f>IF(OR(D32="",$E$28=""),"",D32/$E$28)</f>
-        <v/>
-      </c>
-      <c r="G32" s="8">
-        <f>IF(A32="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H32" s="22" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I32" s="22" t="inlineStr">
-        <is>
-          <t>Sin Proteccion</t>
-        </is>
-      </c>
-      <c r="J32" s="8" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K32" s="22" t="inlineStr">
-        <is>
-          <t>Noroeste</t>
-        </is>
-      </c>
-      <c r="L32" s="8">
-        <f>IF(I32="","",IFERROR(VLOOKUP(I32,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M32" s="22">
-        <f>IF(OR(D32="",J32=""),"",IF(J32&lt;=G32,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" ht="70" customHeight="1">
-      <c r="A33" s="10" t="inlineStr">
-        <is>
-          <t>PA02</t>
-        </is>
-      </c>
-      <c r="B33" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C33" s="9" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D33" s="9">
-        <f>IF(COUNT(B33,C33)&lt;2,"",B33*C33)</f>
-        <v/>
-      </c>
-      <c r="E33" s="21" t="n"/>
-      <c r="F33" s="20">
-        <f>IF(OR(D33="",$E$28=""),"",D33/$E$28)</f>
-        <v/>
-      </c>
-      <c r="G33" s="9">
-        <f>IF(A33="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H33" s="10" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I33" s="10" t="inlineStr">
-        <is>
-          <t>Sin Proteccion</t>
-        </is>
-      </c>
-      <c r="J33" s="9" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K33" s="10" t="inlineStr">
-        <is>
-          <t>Noroeste</t>
-        </is>
-      </c>
-      <c r="L33" s="9">
-        <f>IF(I33="","",IFERROR(VLOOKUP(I33,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M33" s="10">
-        <f>IF(OR(D33="",J33=""),"",IF(J33&lt;=G33,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" ht="70" customHeight="1">
-      <c r="A34" s="10" t="inlineStr">
-        <is>
-          <t>VA03</t>
-        </is>
-      </c>
-      <c r="B34" s="9" t="n">
-        <v>2.52</v>
-      </c>
-      <c r="C34" s="9" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D34" s="9">
-        <f>IF(COUNT(B34,C34)&lt;2,"",B34*C34)</f>
-        <v/>
-      </c>
-      <c r="E34" s="21" t="n"/>
-      <c r="F34" s="20">
-        <f>IF(OR(D34="",$E$28=""),"",D34/$E$28)</f>
-        <v/>
-      </c>
-      <c r="G34" s="9">
-        <f>IF(A34="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H34" s="10" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I34" s="10" t="inlineStr">
-        <is>
-          <t>Sin Proteccion</t>
-        </is>
-      </c>
-      <c r="J34" s="9" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K34" s="10" t="inlineStr">
-        <is>
-          <t>Noroeste</t>
-        </is>
-      </c>
-      <c r="L34" s="9">
-        <f>IF(I34="","",IFERROR(VLOOKUP(I34,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M34" s="10">
-        <f>IF(OR(D34="",J34=""),"",IF(J34&lt;=G34,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" ht="70" customHeight="1">
-      <c r="A35" s="10" t="inlineStr">
-        <is>
-          <t>PF05</t>
-        </is>
-      </c>
-      <c r="B35" s="9" t="n">
-        <v>2.52</v>
-      </c>
-      <c r="C35" s="9" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D35" s="9">
-        <f>IF(COUNT(B35,C35)&lt;2,"",B35*C35)</f>
-        <v/>
-      </c>
-      <c r="E35" s="21" t="n"/>
-      <c r="F35" s="20">
-        <f>IF(OR(D35="",$E$28=""),"",D35/$E$28)</f>
-        <v/>
-      </c>
-      <c r="G35" s="9">
-        <f>IF(A35="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H35" s="10" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I35" s="10" t="inlineStr">
-        <is>
-          <t>Sin Proteccion</t>
-        </is>
-      </c>
-      <c r="J35" s="9" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K35" s="10" t="inlineStr">
-        <is>
-          <t>Noroeste</t>
-        </is>
-      </c>
-      <c r="L35" s="9">
-        <f>IF(I35="","",IFERROR(VLOOKUP(I35,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M35" s="10">
-        <f>IF(OR(D35="",J35=""),"",IF(J35&lt;=G35,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="70" customHeight="1">
-      <c r="A36" s="10" t="n"/>
-      <c r="B36" s="9" t="n"/>
-      <c r="C36" s="9" t="n"/>
       <c r="D36" s="9">
         <f>IF(COUNT(B36,C36)&lt;2,"",B36*C36)</f>
         <v/>
       </c>
-      <c r="E36" s="21" t="n"/>
+      <c r="E36" s="24" t="n"/>
       <c r="F36" s="20">
-        <f>IF(OR(D36="",$E$28=""),"",D36/$E$28)</f>
+        <f>IF(OR(D36="",$E$34=""),"",D36/$E$34)</f>
         <v/>
       </c>
       <c r="G36" s="9">
         <f>IF(A36="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H36" s="10" t="n"/>
-      <c r="I36" s="10" t="n"/>
-      <c r="J36" s="9" t="n"/>
+      <c r="H36" s="10" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I36" s="10" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J36" s="9" t="n">
+        <v>2.8</v>
+      </c>
       <c r="K36" s="10" t="n"/>
       <c r="L36" s="9">
         <f>IF(I36="","",IFERROR(VLOOKUP(I36,Datos_higro!$A$21:$B$28,2,0),""))</f>
@@ -9869,96 +9805,165 @@
       </c>
     </row>
     <row r="37" ht="70" customHeight="1">
-      <c r="A37" s="14" t="n"/>
-      <c r="B37" s="13" t="n"/>
-      <c r="C37" s="13" t="n"/>
-      <c r="D37" s="13">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>VA04</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="C37" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" s="9">
         <f>IF(COUNT(B37,C37)&lt;2,"",B37*C37)</f>
         <v/>
       </c>
-      <c r="E37" s="25" t="n"/>
-      <c r="F37" s="26">
-        <f>IF(OR(D37="",$E$28=""),"",D37/$E$28)</f>
-        <v/>
-      </c>
-      <c r="G37" s="13">
+      <c r="E37" s="24" t="n"/>
+      <c r="F37" s="20">
+        <f>IF(OR(D37="",$E$34=""),"",D37/$E$34)</f>
+        <v/>
+      </c>
+      <c r="G37" s="9">
         <f>IF(A37="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H37" s="14" t="n"/>
-      <c r="I37" s="14" t="n"/>
-      <c r="J37" s="13" t="n"/>
-      <c r="K37" s="14" t="n"/>
-      <c r="L37" s="13">
+      <c r="H37" s="10" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I37" s="10" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J37" s="9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K37" s="10" t="n"/>
+      <c r="L37" s="9">
         <f>IF(I37="","",IFERROR(VLOOKUP(I37,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
-      <c r="M37" s="14">
+      <c r="M37" s="10">
         <f>IF(OR(D37="",J37=""),"",IF(J37&lt;=G37,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="16" t="inlineStr">
+    <row r="38" ht="70" customHeight="1">
+      <c r="A38" s="21" t="inlineStr">
+        <is>
+          <t>VA04 (2)</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="C38" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" s="8">
+        <f>IF(COUNT(B38,C38)&lt;2,"",B38*C38)</f>
+        <v/>
+      </c>
+      <c r="E38" s="22" t="n"/>
+      <c r="F38" s="23">
+        <f>IF(OR(D38="",$E$34=""),"",D38/$E$34)</f>
+        <v/>
+      </c>
+      <c r="G38" s="8">
+        <f>IF(A38="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H38" s="21" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I38" s="21" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J38" s="8" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K38" s="21" t="n"/>
+      <c r="L38" s="8">
+        <f>IF(I38="","",IFERROR(VLOOKUP(I38,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M38" s="21">
+        <f>IF(OR(D38="",J38=""),"",IF(J38&lt;=G38,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" ht="70" customHeight="1">
+      <c r="A39" s="10" t="n"/>
+      <c r="B39" s="9" t="n"/>
+      <c r="C39" s="9" t="n"/>
+      <c r="D39" s="9">
+        <f>IF(COUNT(B39,C39)&lt;2,"",B39*C39)</f>
+        <v/>
+      </c>
+      <c r="E39" s="24" t="n"/>
+      <c r="F39" s="20">
+        <f>IF(OR(D39="",$E$34=""),"",D39/$E$34)</f>
+        <v/>
+      </c>
+      <c r="G39" s="9">
+        <f>IF(A39="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H39" s="10" t="n"/>
+      <c r="I39" s="10" t="n"/>
+      <c r="J39" s="9" t="n"/>
+      <c r="K39" s="10" t="n"/>
+      <c r="L39" s="9">
+        <f>IF(I39="","",IFERROR(VLOOKUP(I39,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M39" s="10">
+        <f>IF(OR(D39="",J39=""),"",IF(J39&lt;=G39,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="70" customHeight="1">
+      <c r="A40" s="14" t="n"/>
+      <c r="B40" s="13" t="n"/>
+      <c r="C40" s="13" t="n"/>
+      <c r="D40" s="13">
+        <f>IF(COUNT(B40,C40)&lt;2,"",B40*C40)</f>
+        <v/>
+      </c>
+      <c r="E40" s="25" t="n"/>
+      <c r="F40" s="26">
+        <f>IF(OR(D40="",$E$34=""),"",D40/$E$34)</f>
+        <v/>
+      </c>
+      <c r="G40" s="13">
+        <f>IF(A40="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H40" s="14" t="n"/>
+      <c r="I40" s="14" t="n"/>
+      <c r="J40" s="13" t="n"/>
+      <c r="K40" s="14" t="n"/>
+      <c r="L40" s="13">
+        <f>IF(I40="","",IFERROR(VLOOKUP(I40,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M40" s="14">
+        <f>IF(OR(D40="",J40=""),"",IF(J40&lt;=G40,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="16" t="inlineStr">
         <is>
           <t>En amarillo, las ocho aberturas que cambiaron de fachada al orientar los muros. Cambia la orientacion, no las medidas.</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="n"/>
-      <c r="C38" s="2" t="n"/>
-      <c r="D38" s="2" t="n"/>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="2" t="n"/>
-      <c r="G38" s="2" t="n"/>
-      <c r="H38" s="2" t="n"/>
-      <c r="I38" s="2" t="n"/>
-      <c r="J38" s="2" t="n"/>
-      <c r="K38" s="2" t="n"/>
-      <c r="L38" s="2" t="n"/>
-      <c r="M38" s="2" t="n"/>
-    </row>
-    <row r="39" ht="39.7" customHeight="1">
-      <c r="A39" s="28" t="inlineStr">
-        <is>
-          <t>COMO SE COMPLETA</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="n"/>
-      <c r="C39" s="2" t="n"/>
-      <c r="D39" s="2" t="n"/>
-      <c r="E39" s="2" t="n"/>
-      <c r="F39" s="2" t="n"/>
-      <c r="G39" s="2" t="n"/>
-      <c r="H39" s="2" t="n"/>
-      <c r="I39" s="2" t="n"/>
-      <c r="J39" s="2" t="n"/>
-      <c r="K39" s="2" t="n"/>
-      <c r="L39" s="2" t="n"/>
-      <c r="M39" s="2" t="n"/>
-    </row>
-    <row r="40" ht="39.7" customHeight="1">
-      <c r="A40" s="29" t="inlineStr">
-        <is>
-          <t>Descripcion, altura y ancho del vano: de la planilla de carpinterias.</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="n"/>
-      <c r="C40" s="2" t="n"/>
-      <c r="D40" s="2" t="n"/>
-      <c r="E40" s="2" t="n"/>
-      <c r="F40" s="2" t="n"/>
-      <c r="G40" s="2" t="n"/>
-      <c r="H40" s="2" t="n"/>
-      <c r="I40" s="2" t="n"/>
-      <c r="J40" s="2" t="n"/>
-      <c r="K40" s="2" t="n"/>
-      <c r="L40" s="2" t="n"/>
-      <c r="M40" s="2" t="n"/>
-    </row>
-    <row r="41" ht="39.7" customHeight="1">
-      <c r="A41" s="29" t="inlineStr">
-        <is>
-          <t>Area del vano, area total por plano y porcentaje: se calculan solos.</t>
         </is>
       </c>
       <c r="B41" s="2" t="n"/>
@@ -9975,9 +9980,9 @@
       <c r="M41" s="2" t="n"/>
     </row>
     <row r="42" ht="39.7" customHeight="1">
-      <c r="A42" s="29" t="inlineStr">
-        <is>
-          <t>Tipo de vidrio y tipo de proteccion: desplegables; sus valores estan en la hoja Datos_higro.</t>
+      <c r="A42" s="28" t="inlineStr">
+        <is>
+          <t>COMO SE COMPLETA</t>
         </is>
       </c>
       <c r="B42" s="2" t="n"/>
@@ -9996,7 +10001,7 @@
     <row r="43" ht="39.7" customHeight="1">
       <c r="A43" s="29" t="inlineStr">
         <is>
-          <t>Transmitancia del cerramiento: cargarla segun el vidrio y el marco adoptados.</t>
+          <t>Descripcion, altura y ancho del vano: de la planilla de carpinterias.</t>
         </is>
       </c>
       <c r="B43" s="2" t="n"/>
@@ -10015,7 +10020,7 @@
     <row r="44" ht="39.7" customHeight="1">
       <c r="A44" s="29" t="inlineStr">
         <is>
-          <t>PROTECCION: la obra tiene cortinas blackout INTERIORES, y los panos fijos PF no tienen nada.</t>
+          <t>Area del vano, area total por plano y porcentaje: se calculan solos.</t>
         </is>
       </c>
       <c r="B44" s="2" t="n"/>
@@ -10034,7 +10039,7 @@
     <row r="45" ht="39.7" customHeight="1">
       <c r="A45" s="29" t="inlineStr">
         <is>
-          <t>Una cortina interior NO computa como proteccion solar: la radiacion ya atraveso el vidrio</t>
+          <t>Tipo de vidrio y tipo de proteccion: desplegables; sus valores estan en la hoja Datos_higro.</t>
         </is>
       </c>
       <c r="B45" s="2" t="n"/>
@@ -10053,7 +10058,7 @@
     <row r="46" ht="39.7" customHeight="1">
       <c r="A46" s="29" t="inlineStr">
         <is>
-          <t>cuando llega a la cortina. La ordenanza acredita protecciones exteriores (aleros, parasoles,</t>
+          <t>Transmitancia del cerramiento: cargarla segun el vidrio y el marco adoptados.</t>
         </is>
       </c>
       <c r="B46" s="2" t="n"/>
@@ -10072,7 +10077,7 @@
     <row r="47" ht="39.7" customHeight="1">
       <c r="A47" s="29" t="inlineStr">
         <is>
-          <t>cortinas de enrollar exteriores, toldos). Por eso las veinte aberturas van Sin Proteccion.</t>
+          <t>PROTECCION: la obra tiene cortinas blackout INTERIORES, y los panos fijos PF no tienen nada.</t>
         </is>
       </c>
       <c r="B47" s="2" t="n"/>
@@ -10088,8 +10093,12 @@
       <c r="L47" s="2" t="n"/>
       <c r="M47" s="2" t="n"/>
     </row>
-    <row r="48">
-      <c r="A48" s="29" t="inlineStr"/>
+    <row r="48" ht="39.7" customHeight="1">
+      <c r="A48" s="29" t="inlineStr">
+        <is>
+          <t>Una cortina interior NO computa como proteccion solar: la radiacion ya atraveso el vidrio</t>
+        </is>
+      </c>
       <c r="B48" s="2" t="n"/>
       <c r="C48" s="2" t="n"/>
       <c r="D48" s="2" t="n"/>
@@ -10106,7 +10115,7 @@
     <row r="49" ht="39.7" customHeight="1">
       <c r="A49" s="29" t="inlineStr">
         <is>
-          <t>CONSECUENCIA: el factor de exposicion solar da 0,88 esta muy por encima del maximo de 0,30 que la ordenanza admite para</t>
+          <t>cuando llega a la cortina. La ordenanza acredita protecciones exteriores (aleros, parasoles,</t>
         </is>
       </c>
       <c r="B49" s="2" t="n"/>
@@ -10125,7 +10134,7 @@
     <row r="50" ht="39.7" customHeight="1">
       <c r="A50" s="29" t="inlineStr">
         <is>
-          <t>el cuadrante Este/Oeste, donde caen las cuatro fachadas de esta casa por estar girada 45</t>
+          <t>cortinas de enrollar exteriores, toldos). Por eso las veinte aberturas van Sin Proteccion.</t>
         </is>
       </c>
       <c r="B50" s="2" t="n"/>
@@ -10141,12 +10150,8 @@
       <c r="L50" s="2" t="n"/>
       <c r="M50" s="2" t="n"/>
     </row>
-    <row r="51" ht="39.7" customHeight="1">
-      <c r="A51" s="29" t="inlineStr">
-        <is>
-          <t>grados. La verificacion de la planilla no lo controla, igual que la de la catedra, pero si lo</t>
-        </is>
-      </c>
+    <row r="51">
+      <c r="A51" s="29" t="inlineStr"/>
       <c r="B51" s="2" t="n"/>
       <c r="C51" s="2" t="n"/>
       <c r="D51" s="2" t="n"/>
@@ -10163,7 +10168,7 @@
     <row r="52" ht="39.7" customHeight="1">
       <c r="A52" s="29" t="inlineStr">
         <is>
-          <t>presentas en el municipio esas cinco aberturas no pasarian el factor de exposicion solar.</t>
+          <t>CONSECUENCIA: el factor de exposicion solar da 0,88 esta muy por encima del maximo de 0,30 que la ordenanza admite para</t>
         </is>
       </c>
       <c r="B52" s="2" t="n"/>
@@ -10182,7 +10187,7 @@
     <row r="53" ht="39.7" customHeight="1">
       <c r="A53" s="29" t="inlineStr">
         <is>
-          <t>Hay dos salidas posibles: (a) si la abertura ocupa menos del 20% del lado expuesto del local,</t>
+          <t>el cuadrante Este/Oeste, donde caen las cuatro fachadas de esta casa por estar girada 45</t>
         </is>
       </c>
       <c r="B53" s="2" t="n"/>
@@ -10201,7 +10206,7 @@
     <row r="54" ht="39.7" customHeight="1">
       <c r="A54" s="29" t="inlineStr">
         <is>
-          <t>no se verifica el FES; (b) cambiar el vidrio por uno de control solar, que baja el FES sin</t>
+          <t>grados. La verificacion de la planilla no lo controla, igual que la de la catedra, pero si lo</t>
         </is>
       </c>
       <c r="B54" s="2" t="n"/>
@@ -10220,7 +10225,7 @@
     <row r="55" ht="39.7" customHeight="1">
       <c r="A55" s="29" t="inlineStr">
         <is>
-          <t>tocar la obra. Agregar una proteccion exterior seria la tercera, pero implica obra.</t>
+          <t>presentas en el municipio esas cinco aberturas no pasarian el factor de exposicion solar.</t>
         </is>
       </c>
       <c r="B55" s="2" t="n"/>
@@ -10236,8 +10241,12 @@
       <c r="L55" s="2" t="n"/>
       <c r="M55" s="2" t="n"/>
     </row>
-    <row r="56">
-      <c r="A56" s="29" t="inlineStr"/>
+    <row r="56" ht="39.7" customHeight="1">
+      <c r="A56" s="29" t="inlineStr">
+        <is>
+          <t>Hay dos salidas posibles: (a) si la abertura ocupa menos del 20% del lado expuesto del local,</t>
+        </is>
+      </c>
       <c r="B56" s="2" t="n"/>
       <c r="C56" s="2" t="n"/>
       <c r="D56" s="2" t="n"/>
@@ -10254,7 +10263,7 @@
     <row r="57" ht="39.7" customHeight="1">
       <c r="A57" s="29" t="inlineStr">
         <is>
-          <t>Orientacion: ya cargada. Factor de exposicion solar: se completa SOLO al elegir el tipo de</t>
+          <t>no se verifica el FES; (b) cambiar el vidrio por uno de control solar, que baja el FES sin</t>
         </is>
       </c>
       <c r="B57" s="2" t="n"/>
@@ -10273,7 +10282,7 @@
     <row r="58" ht="39.7" customHeight="1">
       <c r="A58" s="29" t="inlineStr">
         <is>
-          <t>proteccion, con los valores de la tabla de Datos_higro (Sin Proteccion 0,88; Parasol</t>
+          <t>tocar la obra. Agregar una proteccion exterior seria la tercera, pero implica obra.</t>
         </is>
       </c>
       <c r="B58" s="2" t="n"/>
@@ -10289,12 +10298,8 @@
       <c r="L58" s="2" t="n"/>
       <c r="M58" s="2" t="n"/>
     </row>
-    <row r="59" ht="39.7" customHeight="1">
-      <c r="A59" s="29" t="inlineStr">
-        <is>
-          <t>horizontal fijo 1:2 0,35), que son los mismos de la planilla de la catedra.</t>
-        </is>
-      </c>
+    <row r="59">
+      <c r="A59" s="29" t="inlineStr"/>
       <c r="B59" s="2" t="n"/>
       <c r="C59" s="2" t="n"/>
       <c r="D59" s="2" t="n"/>
@@ -10311,7 +10316,7 @@
     <row r="60" ht="39.7" customHeight="1">
       <c r="A60" s="29" t="inlineStr">
         <is>
-          <t>En Datos_higro esta ademas el FES maximo admitido por cuadrante segun la ordenanza, como</t>
+          <t>Orientacion: ya cargada. Factor de exposicion solar: se completa SOLO al elegir el tipo de</t>
         </is>
       </c>
       <c r="B60" s="2" t="n"/>
@@ -10330,7 +10335,7 @@
     <row r="61" ht="39.7" customHeight="1">
       <c r="A61" s="29" t="inlineStr">
         <is>
-          <t>referencia: la verificacion no lo controla, igual que en la planilla de la catedra.</t>
+          <t>proteccion, con los valores de la tabla de Datos_higro (Sin Proteccion 0,88; Parasol</t>
         </is>
       </c>
       <c r="B61" s="2" t="n"/>
@@ -10346,8 +10351,12 @@
       <c r="L61" s="2" t="n"/>
       <c r="M61" s="2" t="n"/>
     </row>
-    <row r="62">
-      <c r="A62" s="29" t="inlineStr"/>
+    <row r="62" ht="39.7" customHeight="1">
+      <c r="A62" s="29" t="inlineStr">
+        <is>
+          <t>horizontal fijo 1:2 0,35), que son los mismos de la planilla de la catedra.</t>
+        </is>
+      </c>
       <c r="B62" s="2" t="n"/>
       <c r="C62" s="2" t="n"/>
       <c r="D62" s="2" t="n"/>
@@ -10364,7 +10373,7 @@
     <row r="63" ht="39.7" customHeight="1">
       <c r="A63" s="29" t="inlineStr">
         <is>
-          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
+          <t>En Datos_higro esta ademas el FES maximo admitido por cuadrante segun la ordenanza, como</t>
         </is>
       </c>
       <c r="B63" s="2" t="n"/>
@@ -10383,7 +10392,7 @@
     <row r="64" ht="39.7" customHeight="1">
       <c r="A64" s="29" t="inlineStr">
         <is>
-          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
+          <t>referencia: la verificacion no lo controla, igual que en la planilla de la catedra.</t>
         </is>
       </c>
       <c r="B64" s="2" t="n"/>
@@ -10417,7 +10426,7 @@
     <row r="66" ht="39.7" customHeight="1">
       <c r="A66" s="29" t="inlineStr">
         <is>
-          <t>ALTURAS: medidas sobre el dibujo de las vistas de la planilla de carpinterias, con la escala</t>
+          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
         </is>
       </c>
       <c r="B66" s="2" t="n"/>
@@ -10436,7 +10445,7 @@
     <row r="67" ht="39.7" customHeight="1">
       <c r="A67" s="29" t="inlineStr">
         <is>
-          <t>verificada contra los anchos acotados (error menor a 2 cm). La mayoria de las aberturas son de</t>
+          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
         </is>
       </c>
       <c r="B67" s="2" t="n"/>
@@ -10452,12 +10461,8 @@
       <c r="L67" s="2" t="n"/>
       <c r="M67" s="2" t="n"/>
     </row>
-    <row r="68" ht="39.7" customHeight="1">
-      <c r="A68" s="29" t="inlineStr">
-        <is>
-          <t>piso a cielorraso, 3,00 m. VERIFICARLAS contra el plano antes de presentar.</t>
-        </is>
-      </c>
+    <row r="68">
+      <c r="A68" s="29" t="inlineStr"/>
       <c r="B68" s="2" t="n"/>
       <c r="C68" s="2" t="n"/>
       <c r="D68" s="2" t="n"/>
@@ -10474,7 +10479,7 @@
     <row r="69" ht="39.7" customHeight="1">
       <c r="A69" s="29" t="inlineStr">
         <is>
-          <t>PF04 es la unica con antepecho: arranca a 1,09 y mide 0,60 de alto. El resto llega al piso.</t>
+          <t>ALTURAS: medidas sobre el dibujo de las vistas de la planilla de carpinterias, con la escala</t>
         </is>
       </c>
       <c r="B69" s="2" t="n"/>
@@ -10493,7 +10498,7 @@
     <row r="70" ht="39.7" customHeight="1">
       <c r="A70" s="29" t="inlineStr">
         <is>
-          <t>Las alturas de PV01 (3,00), PF04 (0,60) y PV04 (2) (2,95) las aporto el autor del proyecto.</t>
+          <t>verificada contra los anchos acotados (error menor a 2 cm). La mayoria de las aberturas son de</t>
         </is>
       </c>
       <c r="B70" s="2" t="n"/>
@@ -10509,8 +10514,12 @@
       <c r="L70" s="2" t="n"/>
       <c r="M70" s="2" t="n"/>
     </row>
-    <row r="71">
-      <c r="A71" s="29" t="inlineStr"/>
+    <row r="71" ht="39.7" customHeight="1">
+      <c r="A71" s="29" t="inlineStr">
+        <is>
+          <t>piso a cielorraso, 3,00 m. VERIFICARLAS contra el plano antes de presentar.</t>
+        </is>
+      </c>
       <c r="B71" s="2" t="n"/>
       <c r="C71" s="2" t="n"/>
       <c r="D71" s="2" t="n"/>
@@ -10527,7 +10536,7 @@
     <row r="72" ht="39.7" customHeight="1">
       <c r="A72" s="29" t="inlineStr">
         <is>
-          <t>ORIENTACION: el simbolo de norte del plano (circulo con aguja, en el patio interno) apunta a</t>
+          <t>PF04 es la unica con antepecho: arranca a 1,09 y mide 0,60 de alto. El resto llega al piso.</t>
         </is>
       </c>
       <c r="B72" s="2" t="n"/>
@@ -10546,7 +10555,7 @@
     <row r="73" ht="39.7" customHeight="1">
       <c r="A73" s="29" t="inlineStr">
         <is>
-          <t>45 grados hacia arriba y a la derecha de la hoja. Entonces las cuatro fachadas NO son N-S-E-O</t>
+          <t>Las alturas de PV01 (3,00), PF04 (0,60) y PV04 (2) (2,95) las aporto el autor del proyecto.</t>
         </is>
       </c>
       <c r="B73" s="2" t="n"/>
@@ -10562,12 +10571,8 @@
       <c r="L73" s="2" t="n"/>
       <c r="M73" s="2" t="n"/>
     </row>
-    <row r="74" ht="39.7" customHeight="1">
-      <c r="A74" s="29" t="inlineStr">
-        <is>
-          <t>sino: arriba = Noroeste, derecha = Noreste, abajo = Sudeste, izquierda = Sudoeste.</t>
-        </is>
-      </c>
+    <row r="74">
+      <c r="A74" s="29" t="inlineStr"/>
       <c r="B74" s="2" t="n"/>
       <c r="C74" s="2" t="n"/>
       <c r="D74" s="2" t="n"/>
@@ -10584,7 +10589,7 @@
     <row r="75" ht="39.7" customHeight="1">
       <c r="A75" s="29" t="inlineStr">
         <is>
-          <t>Cada abertura se asigno a la fachada por su posicion en planta. Las del patio interno se</t>
+          <t>ORIENTACION: el simbolo de norte del plano (circulo con aguja, en el patio interno) apunta a</t>
         </is>
       </c>
       <c r="B75" s="2" t="n"/>
@@ -10603,7 +10608,7 @@
     <row r="76" ht="39.7" customHeight="1">
       <c r="A76" s="29" t="inlineStr">
         <is>
-          <t>orientan por la pared en la que estan: miran hacia adentro del patio.</t>
+          <t>45 grados hacia arriba y a la derecha de la hoja. Entonces las cuatro fachadas NO son N-S-E-O</t>
         </is>
       </c>
       <c r="B76" s="2" t="n"/>
@@ -10622,7 +10627,7 @@
     <row r="77" ht="39.7" customHeight="1">
       <c r="A77" s="29" t="inlineStr">
         <is>
-          <t>Los rotulos Dormitorio Norte y Dormitorio Sur del plano no coinciden con el norte real;</t>
+          <t>sino: arriba = Noroeste, derecha = Noreste, abajo = Sudeste, izquierda = Sudoeste.</t>
         </is>
       </c>
       <c r="B77" s="2" t="n"/>
@@ -10641,7 +10646,7 @@
     <row r="78" ht="39.7" customHeight="1">
       <c r="A78" s="29" t="inlineStr">
         <is>
-          <t>parecen ser nombres de uso, no orientaciones.</t>
+          <t>Cada abertura se asigno a la fachada por su posicion en planta. Las del patio interno se</t>
         </is>
       </c>
       <c r="B78" s="2" t="n"/>
@@ -10657,8 +10662,12 @@
       <c r="L78" s="2" t="n"/>
       <c r="M78" s="2" t="n"/>
     </row>
-    <row r="79">
-      <c r="A79" s="29" t="inlineStr"/>
+    <row r="79" ht="39.7" customHeight="1">
+      <c r="A79" s="29" t="inlineStr">
+        <is>
+          <t>orientan por la pared en la que estan: miran hacia adentro del patio.</t>
+        </is>
+      </c>
       <c r="B79" s="2" t="n"/>
       <c r="C79" s="2" t="n"/>
       <c r="D79" s="2" t="n"/>
@@ -10675,7 +10684,7 @@
     <row r="80" ht="39.7" customHeight="1">
       <c r="A80" s="29" t="inlineStr">
         <is>
-          <t>CANTIDADES: la planilla de carpinterias trae la cantidad de cada abertura. Tres van dos veces:</t>
+          <t>Los rotulos Dormitorio Norte y Dormitorio Sur del plano no coinciden con el norte real;</t>
         </is>
       </c>
       <c r="B80" s="2" t="n"/>
@@ -10694,7 +10703,7 @@
     <row r="81" ht="39.7" customHeight="1">
       <c r="A81" s="29" t="inlineStr">
         <is>
-          <t>VA01 (01 Cocina y 09 Suite), VA04 (13 Dormitorio Norte y 14 Play Room) y PF01 (03 Lavadero y</t>
+          <t>parecen ser nombres de uso, no orientaciones.</t>
         </is>
       </c>
       <c r="B81" s="2" t="n"/>
@@ -10710,12 +10719,8 @@
       <c r="L81" s="2" t="n"/>
       <c r="M81" s="2" t="n"/>
     </row>
-    <row r="82" ht="39.7" customHeight="1">
-      <c r="A82" s="29" t="inlineStr">
-        <is>
-          <t>07 Hall de ingreso, a los dos lados del patio interno). Por eso la planilla tiene 20 filas y</t>
-        </is>
-      </c>
+    <row r="82">
+      <c r="A82" s="29" t="inlineStr"/>
       <c r="B82" s="2" t="n"/>
       <c r="C82" s="2" t="n"/>
       <c r="D82" s="2" t="n"/>
@@ -10732,7 +10737,7 @@
     <row r="83" ht="39.7" customHeight="1">
       <c r="A83" s="29" t="inlineStr">
         <is>
-          <t>no 17. Las demas aberturas son de una sola unidad.</t>
+          <t>CANTIDADES: la planilla de carpinterias trae la cantidad de cada abertura. Tres van dos veces:</t>
         </is>
       </c>
       <c r="B83" s="2" t="n"/>
@@ -10748,8 +10753,12 @@
       <c r="L83" s="2" t="n"/>
       <c r="M83" s="2" t="n"/>
     </row>
-    <row r="84">
-      <c r="A84" s="29" t="inlineStr"/>
+    <row r="84" ht="39.7" customHeight="1">
+      <c r="A84" s="29" t="inlineStr">
+        <is>
+          <t>VA01 (01 Cocina y 09 Suite), VA04 (13 Dormitorio Norte y 14 Play Room) y PF01 (03 Lavadero y</t>
+        </is>
+      </c>
       <c r="B84" s="2" t="n"/>
       <c r="C84" s="2" t="n"/>
       <c r="D84" s="2" t="n"/>
@@ -10766,7 +10775,7 @@
     <row r="85" ht="39.7" customHeight="1">
       <c r="A85" s="29" t="inlineStr">
         <is>
-          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
+          <t>07 Hall de ingreso, a los dos lados del patio interno). Por eso la planilla tiene 20 filas y</t>
         </is>
       </c>
       <c r="B85" s="2" t="n"/>
@@ -10782,8 +10791,12 @@
       <c r="L85" s="2" t="n"/>
       <c r="M85" s="2" t="n"/>
     </row>
-    <row r="86">
-      <c r="A86" s="29" t="inlineStr"/>
+    <row r="86" ht="39.7" customHeight="1">
+      <c r="A86" s="29" t="inlineStr">
+        <is>
+          <t>no 17. Las demas aberturas son de una sola unidad.</t>
+        </is>
+      </c>
       <c r="B86" s="2" t="n"/>
       <c r="C86" s="2" t="n"/>
       <c r="D86" s="2" t="n"/>
@@ -10797,12 +10810,8 @@
       <c r="L86" s="2" t="n"/>
       <c r="M86" s="2" t="n"/>
     </row>
-    <row r="87" ht="39.7" customHeight="1">
-      <c r="A87" s="29" t="inlineStr">
-        <is>
-          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
-        </is>
-      </c>
+    <row r="87">
+      <c r="A87" s="29" t="inlineStr"/>
       <c r="B87" s="2" t="n"/>
       <c r="C87" s="2" t="n"/>
       <c r="D87" s="2" t="n"/>
@@ -10819,7 +10828,7 @@
     <row r="88" ht="39.7" customHeight="1">
       <c r="A88" s="29" t="inlineStr">
         <is>
-          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
+          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
         </is>
       </c>
       <c r="B88" s="2" t="n"/>
@@ -10835,12 +10844,8 @@
       <c r="L88" s="2" t="n"/>
       <c r="M88" s="2" t="n"/>
     </row>
-    <row r="89" ht="39.7" customHeight="1">
-      <c r="A89" s="29" t="inlineStr">
-        <is>
-          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
-        </is>
-      </c>
+    <row r="89">
+      <c r="A89" s="29" t="inlineStr"/>
       <c r="B89" s="2" t="n"/>
       <c r="C89" s="2" t="n"/>
       <c r="D89" s="2" t="n"/>
@@ -10854,24 +10859,83 @@
       <c r="L89" s="2" t="n"/>
       <c r="M89" s="2" t="n"/>
     </row>
+    <row r="90" ht="39.7" customHeight="1">
+      <c r="A90" s="29" t="inlineStr">
+        <is>
+          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="n"/>
+      <c r="C90" s="2" t="n"/>
+      <c r="D90" s="2" t="n"/>
+      <c r="E90" s="2" t="n"/>
+      <c r="F90" s="2" t="n"/>
+      <c r="G90" s="2" t="n"/>
+      <c r="H90" s="2" t="n"/>
+      <c r="I90" s="2" t="n"/>
+      <c r="J90" s="2" t="n"/>
+      <c r="K90" s="2" t="n"/>
+      <c r="L90" s="2" t="n"/>
+      <c r="M90" s="2" t="n"/>
+    </row>
+    <row r="91" ht="39.7" customHeight="1">
+      <c r="A91" s="29" t="inlineStr">
+        <is>
+          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="n"/>
+      <c r="C91" s="2" t="n"/>
+      <c r="D91" s="2" t="n"/>
+      <c r="E91" s="2" t="n"/>
+      <c r="F91" s="2" t="n"/>
+      <c r="G91" s="2" t="n"/>
+      <c r="H91" s="2" t="n"/>
+      <c r="I91" s="2" t="n"/>
+      <c r="J91" s="2" t="n"/>
+      <c r="K91" s="2" t="n"/>
+      <c r="L91" s="2" t="n"/>
+      <c r="M91" s="2" t="n"/>
+    </row>
+    <row r="92" ht="39.7" customHeight="1">
+      <c r="A92" s="29" t="inlineStr">
+        <is>
+          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="n"/>
+      <c r="C92" s="2" t="n"/>
+      <c r="D92" s="2" t="n"/>
+      <c r="E92" s="2" t="n"/>
+      <c r="F92" s="2" t="n"/>
+      <c r="G92" s="2" t="n"/>
+      <c r="H92" s="2" t="n"/>
+      <c r="I92" s="2" t="n"/>
+      <c r="J92" s="2" t="n"/>
+      <c r="K92" s="2" t="n"/>
+      <c r="L92" s="2" t="n"/>
+      <c r="M92" s="2" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="16">
     <mergeCell ref="A1:A3"/>
-    <mergeCell ref="A13:M13"/>
-    <mergeCell ref="E14:E17"/>
+    <mergeCell ref="A14:M14"/>
+    <mergeCell ref="E34:E40"/>
     <mergeCell ref="A27:M27"/>
+    <mergeCell ref="E15:E19"/>
     <mergeCell ref="A6:M6"/>
+    <mergeCell ref="E21:E26"/>
     <mergeCell ref="B3:L3"/>
     <mergeCell ref="B2:L2"/>
     <mergeCell ref="A4:M4"/>
-    <mergeCell ref="E7:E12"/>
-    <mergeCell ref="A18:M18"/>
-    <mergeCell ref="E28:E37"/>
-    <mergeCell ref="E19:E26"/>
+    <mergeCell ref="E7:E13"/>
+    <mergeCell ref="E28:E32"/>
+    <mergeCell ref="A20:M20"/>
+    <mergeCell ref="A33:M33"/>
     <mergeCell ref="M1:M3"/>
     <mergeCell ref="B1:L1"/>
   </mergeCells>
-  <conditionalFormatting sqref="M6:M37">
+  <conditionalFormatting sqref="M6:M40">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"CUMPLE"</formula>
     </cfRule>
@@ -10880,13 +10944,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="H6:H37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Datos_higro!$A$10:$A$17</formula1>
     </dataValidation>
-    <dataValidation sqref="I6:I37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I6:I40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Datos_higro!$A$21:$A$28</formula1>
     </dataValidation>
-    <dataValidation sqref="K6:K37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K6:K40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Norte,Sur,Este,Oeste,Noreste,Noroeste,Sudeste,Sudoeste,Horizontal"</formula1>
     </dataValidation>
   </dataValidations>
@@ -11950,7 +12014,7 @@
       </c>
     </row>
     <row r="5" ht="70" customHeight="1">
-      <c r="A5" s="21" t="n"/>
+      <c r="A5" s="24" t="n"/>
       <c r="B5" s="18" t="inlineStr">
         <is>
           <t>VI 01b</t>
@@ -12067,7 +12131,7 @@
       </c>
     </row>
     <row r="6" ht="70" customHeight="1">
-      <c r="A6" s="21" t="n"/>
+      <c r="A6" s="24" t="n"/>
       <c r="B6" s="18" t="inlineStr">
         <is>
           <t>VI 02</t>
@@ -12184,7 +12248,7 @@
       </c>
     </row>
     <row r="7" ht="70" customHeight="1">
-      <c r="A7" s="21" t="n"/>
+      <c r="A7" s="24" t="n"/>
       <c r="B7" s="18" t="inlineStr">
         <is>
           <t>VI 03c</t>
@@ -12297,7 +12361,7 @@
       </c>
     </row>
     <row r="8" ht="70" customHeight="1">
-      <c r="A8" s="21" t="n"/>
+      <c r="A8" s="24" t="n"/>
       <c r="B8" s="18" t="inlineStr">
         <is>
           <t>VI 04a</t>
@@ -12418,7 +12482,7 @@
       </c>
     </row>
     <row r="9" ht="70" customHeight="1">
-      <c r="A9" s="21" t="n"/>
+      <c r="A9" s="24" t="n"/>
       <c r="B9" s="18" t="inlineStr">
         <is>
           <t>VI 04b</t>
@@ -12531,7 +12595,7 @@
       </c>
     </row>
     <row r="10" ht="70" customHeight="1">
-      <c r="A10" s="21" t="n"/>
+      <c r="A10" s="24" t="n"/>
       <c r="B10" s="18" t="inlineStr">
         <is>
           <t>VI 06</t>
@@ -12652,7 +12716,7 @@
       </c>
     </row>
     <row r="11" ht="70" customHeight="1">
-      <c r="A11" s="21" t="n"/>
+      <c r="A11" s="24" t="n"/>
       <c r="B11" s="18" t="inlineStr">
         <is>
           <t>VI 07a</t>
@@ -12769,7 +12833,7 @@
       </c>
     </row>
     <row r="12" ht="70" customHeight="1">
-      <c r="A12" s="21" t="n"/>
+      <c r="A12" s="24" t="n"/>
       <c r="B12" s="18" t="inlineStr">
         <is>
           <t>VI 07b</t>
@@ -12886,7 +12950,7 @@
       </c>
     </row>
     <row r="13" ht="70" customHeight="1">
-      <c r="A13" s="21" t="n"/>
+      <c r="A13" s="24" t="n"/>
       <c r="B13" s="18" t="inlineStr">
         <is>
           <t>VI 07c</t>
@@ -13007,7 +13071,7 @@
       </c>
     </row>
     <row r="14" ht="70" customHeight="1">
-      <c r="A14" s="21" t="n"/>
+      <c r="A14" s="24" t="n"/>
       <c r="B14" s="18" t="inlineStr">
         <is>
           <t>VI 08a</t>
@@ -13120,7 +13184,7 @@
       </c>
     </row>
     <row r="15" ht="70" customHeight="1">
-      <c r="A15" s="21" t="n"/>
+      <c r="A15" s="24" t="n"/>
       <c r="B15" s="18" t="inlineStr">
         <is>
           <t>VI 08b</t>
@@ -13237,7 +13301,7 @@
       </c>
     </row>
     <row r="16" ht="70" customHeight="1">
-      <c r="A16" s="21" t="n"/>
+      <c r="A16" s="24" t="n"/>
       <c r="B16" s="18" t="inlineStr">
         <is>
           <t>VI 09</t>
@@ -13358,7 +13422,7 @@
       </c>
     </row>
     <row r="17" ht="70" customHeight="1">
-      <c r="A17" s="21" t="n"/>
+      <c r="A17" s="24" t="n"/>
       <c r="B17" s="18" t="inlineStr">
         <is>
           <t>VI 10a</t>
@@ -13471,7 +13535,7 @@
       </c>
     </row>
     <row r="18" ht="70" customHeight="1">
-      <c r="A18" s="21" t="n"/>
+      <c r="A18" s="24" t="n"/>
       <c r="B18" s="18" t="inlineStr">
         <is>
           <t>VI 10b</t>
@@ -13584,7 +13648,7 @@
       </c>
     </row>
     <row r="19" ht="70" customHeight="1">
-      <c r="A19" s="21" t="n"/>
+      <c r="A19" s="24" t="n"/>
       <c r="B19" s="18" t="inlineStr">
         <is>
           <t>VI 10c</t>
@@ -13697,7 +13761,7 @@
       </c>
     </row>
     <row r="20" ht="70" customHeight="1">
-      <c r="A20" s="21" t="n"/>
+      <c r="A20" s="24" t="n"/>
       <c r="B20" s="18" t="inlineStr">
         <is>
           <t>VI 11a</t>
@@ -13814,7 +13878,7 @@
       </c>
     </row>
     <row r="21" ht="70" customHeight="1">
-      <c r="A21" s="21" t="n"/>
+      <c r="A21" s="24" t="n"/>
       <c r="B21" s="18" t="inlineStr">
         <is>
           <t>VI 11b</t>
@@ -13931,7 +13995,7 @@
       </c>
     </row>
     <row r="22" ht="70" customHeight="1">
-      <c r="A22" s="21" t="n"/>
+      <c r="A22" s="24" t="n"/>
       <c r="B22" s="18" t="inlineStr">
         <is>
           <t>VI 11c</t>
@@ -14048,7 +14112,7 @@
       </c>
     </row>
     <row r="23" ht="70" customHeight="1">
-      <c r="A23" s="21" t="n"/>
+      <c r="A23" s="24" t="n"/>
       <c r="B23" s="18" t="inlineStr">
         <is>
           <t>VCH 03a</t>
@@ -14165,7 +14229,7 @@
       </c>
     </row>
     <row r="24" ht="70" customHeight="1">
-      <c r="A24" s="21" t="n"/>
+      <c r="A24" s="24" t="n"/>
       <c r="B24" s="18" t="inlineStr">
         <is>
           <t>VCH 03b</t>
@@ -14516,7 +14580,7 @@
       </c>
     </row>
     <row r="27" ht="70" customHeight="1">
-      <c r="A27" s="21" t="n"/>
+      <c r="A27" s="24" t="n"/>
       <c r="B27" s="18" t="inlineStr">
         <is>
           <t>VI 13a</t>
@@ -14629,7 +14693,7 @@
       </c>
     </row>
     <row r="28" ht="70" customHeight="1">
-      <c r="A28" s="21" t="n"/>
+      <c r="A28" s="24" t="n"/>
       <c r="B28" s="18" t="inlineStr">
         <is>
           <t>VI 13b</t>
@@ -14742,7 +14806,7 @@
       </c>
     </row>
     <row r="29" ht="70" customHeight="1">
-      <c r="A29" s="21" t="n"/>
+      <c r="A29" s="24" t="n"/>
       <c r="B29" s="18" t="inlineStr">
         <is>
           <t>VI 14</t>
@@ -14855,7 +14919,7 @@
       </c>
     </row>
     <row r="30" ht="70" customHeight="1">
-      <c r="A30" s="21" t="n"/>
+      <c r="A30" s="24" t="n"/>
       <c r="B30" s="18" t="inlineStr">
         <is>
           <t>VI 15a</t>
@@ -14972,7 +15036,7 @@
       </c>
     </row>
     <row r="31" ht="70" customHeight="1">
-      <c r="A31" s="21" t="n"/>
+      <c r="A31" s="24" t="n"/>
       <c r="B31" s="18" t="inlineStr">
         <is>
           <t>VI 15b</t>
@@ -15089,7 +15153,7 @@
       </c>
     </row>
     <row r="32" ht="70" customHeight="1">
-      <c r="A32" s="21" t="n"/>
+      <c r="A32" s="24" t="n"/>
       <c r="B32" s="18" t="inlineStr">
         <is>
           <t>VI 16a</t>
@@ -15202,7 +15266,7 @@
       </c>
     </row>
     <row r="33" ht="70" customHeight="1">
-      <c r="A33" s="21" t="n"/>
+      <c r="A33" s="24" t="n"/>
       <c r="B33" s="18" t="inlineStr">
         <is>
           <t>VI 16b</t>
@@ -15761,7 +15825,7 @@
       </c>
     </row>
     <row r="5" ht="70" customHeight="1">
-      <c r="A5" s="21" t="n"/>
+      <c r="A5" s="24" t="n"/>
       <c r="B5" s="18" t="inlineStr">
         <is>
           <t>L02</t>
@@ -15833,7 +15897,7 @@
       </c>
     </row>
     <row r="6" ht="70" customHeight="1">
-      <c r="A6" s="21" t="n"/>
+      <c r="A6" s="24" t="n"/>
       <c r="B6" s="18" t="inlineStr">
         <is>
           <t>L03</t>
@@ -15901,7 +15965,7 @@
       </c>
     </row>
     <row r="7" ht="70" customHeight="1">
-      <c r="A7" s="21" t="n"/>
+      <c r="A7" s="24" t="n"/>
       <c r="B7" s="18" t="inlineStr">
         <is>
           <t>L04</t>
@@ -15969,7 +16033,7 @@
       </c>
     </row>
     <row r="8" ht="70" customHeight="1">
-      <c r="A8" s="21" t="n"/>
+      <c r="A8" s="24" t="n"/>
       <c r="B8" s="18" t="inlineStr">
         <is>
           <t>L05</t>
@@ -16037,7 +16101,7 @@
       </c>
     </row>
     <row r="9" ht="70" customHeight="1">
-      <c r="A9" s="21" t="n"/>
+      <c r="A9" s="24" t="n"/>
       <c r="B9" s="18" t="inlineStr">
         <is>
           <t>L06</t>
@@ -16105,7 +16169,7 @@
       </c>
     </row>
     <row r="10" ht="70" customHeight="1">
-      <c r="A10" s="21" t="n"/>
+      <c r="A10" s="24" t="n"/>
       <c r="B10" s="18" t="inlineStr">
         <is>
           <t>L07 (x)</t>
@@ -16179,7 +16243,7 @@
       </c>
     </row>
     <row r="11" ht="70" customHeight="1">
-      <c r="A11" s="21" t="n"/>
+      <c r="A11" s="24" t="n"/>
       <c r="B11" s="18" t="inlineStr">
         <is>
           <t>L07 (y)</t>
@@ -16397,7 +16461,7 @@
       </c>
     </row>
     <row r="14" ht="70" customHeight="1">
-      <c r="A14" s="21" t="n"/>
+      <c r="A14" s="24" t="n"/>
       <c r="B14" s="18" t="inlineStr">
         <is>
           <t>L10 (x)</t>
@@ -16827,7 +16891,7 @@
       </c>
     </row>
     <row r="5" ht="70" customHeight="1">
-      <c r="A5" s="21" t="n"/>
+      <c r="A5" s="24" t="n"/>
       <c r="B5" s="18" t="inlineStr">
         <is>
           <t>C7</t>
@@ -16892,7 +16956,7 @@
       </c>
     </row>
     <row r="6" ht="70" customHeight="1">
-      <c r="A6" s="21" t="n"/>
+      <c r="A6" s="24" t="n"/>
       <c r="B6" s="18" t="inlineStr">
         <is>
           <t>C8</t>
@@ -17091,7 +17155,7 @@
       </c>
     </row>
     <row r="9" ht="70" customHeight="1">
-      <c r="A9" s="21" t="n"/>
+      <c r="A9" s="24" t="n"/>
       <c r="B9" s="18" t="inlineStr">
         <is>
           <t>C2</t>
@@ -17156,7 +17220,7 @@
       </c>
     </row>
     <row r="10" ht="70" customHeight="1">
-      <c r="A10" s="21" t="n"/>
+      <c r="A10" s="24" t="n"/>
       <c r="B10" s="18" t="inlineStr">
         <is>
           <t>C3</t>
@@ -17221,7 +17285,7 @@
       </c>
     </row>
     <row r="11" ht="70" customHeight="1">
-      <c r="A11" s="21" t="n"/>
+      <c r="A11" s="24" t="n"/>
       <c r="B11" s="18" t="inlineStr">
         <is>
           <t>C4</t>
@@ -17286,7 +17350,7 @@
       </c>
     </row>
     <row r="12" ht="70" customHeight="1">
-      <c r="A12" s="21" t="n"/>
+      <c r="A12" s="24" t="n"/>
       <c r="B12" s="18" t="inlineStr">
         <is>
           <t>C5</t>
@@ -17351,7 +17415,7 @@
       </c>
     </row>
     <row r="13" ht="70" customHeight="1">
-      <c r="A13" s="21" t="n"/>
+      <c r="A13" s="24" t="n"/>
       <c r="B13" s="18" t="inlineStr">
         <is>
           <t>C6</t>
@@ -17416,7 +17480,7 @@
       </c>
     </row>
     <row r="14" ht="70" customHeight="1">
-      <c r="A14" s="21" t="n"/>
+      <c r="A14" s="24" t="n"/>
       <c r="B14" s="18" t="inlineStr">
         <is>
           <t>C7</t>
@@ -17481,7 +17545,7 @@
       </c>
     </row>
     <row r="15" ht="70" customHeight="1">
-      <c r="A15" s="21" t="n"/>
+      <c r="A15" s="24" t="n"/>
       <c r="B15" s="18" t="inlineStr">
         <is>
           <t>C8</t>
@@ -21864,7 +21928,7 @@
       </c>
     </row>
     <row r="5" ht="70" customHeight="1">
-      <c r="A5" s="21" t="n"/>
+      <c r="A5" s="24" t="n"/>
       <c r="B5" s="18" t="inlineStr">
         <is>
           <t>T2</t>
@@ -21925,7 +21989,7 @@
       </c>
     </row>
     <row r="6" ht="70" customHeight="1">
-      <c r="A6" s="21" t="n"/>
+      <c r="A6" s="24" t="n"/>
       <c r="B6" s="18" t="inlineStr">
         <is>
           <t>T3</t>
@@ -21986,7 +22050,7 @@
       </c>
     </row>
     <row r="7" ht="70" customHeight="1">
-      <c r="A7" s="21" t="n"/>
+      <c r="A7" s="24" t="n"/>
       <c r="B7" s="18" t="inlineStr">
         <is>
           <t>T4</t>
@@ -22047,7 +22111,7 @@
       </c>
     </row>
     <row r="8" ht="70" customHeight="1">
-      <c r="A8" s="21" t="n"/>
+      <c r="A8" s="24" t="n"/>
       <c r="B8" s="18" t="inlineStr">
         <is>
           <t>T5</t>
@@ -22108,7 +22172,7 @@
       </c>
     </row>
     <row r="9" ht="70" customHeight="1">
-      <c r="A9" s="21" t="n"/>
+      <c r="A9" s="24" t="n"/>
       <c r="B9" s="18" t="inlineStr">
         <is>
           <t>T6</t>
@@ -22169,7 +22233,7 @@
       </c>
     </row>
     <row r="10" ht="70" customHeight="1">
-      <c r="A10" s="21" t="n"/>
+      <c r="A10" s="24" t="n"/>
       <c r="B10" s="18" t="inlineStr">
         <is>
           <t>T7</t>
@@ -22356,7 +22420,7 @@
       </c>
     </row>
     <row r="13" ht="70" customHeight="1">
-      <c r="A13" s="21" t="n"/>
+      <c r="A13" s="24" t="n"/>
       <c r="B13" s="18" t="inlineStr">
         <is>
           <t>T10</t>
@@ -22417,7 +22481,7 @@
       </c>
     </row>
     <row r="14" ht="70" customHeight="1">
-      <c r="A14" s="21" t="n"/>
+      <c r="A14" s="24" t="n"/>
       <c r="B14" s="18" t="inlineStr">
         <is>
           <t>T11</t>
@@ -22478,7 +22542,7 @@
       </c>
     </row>
     <row r="15" ht="70" customHeight="1">
-      <c r="A15" s="21" t="n"/>
+      <c r="A15" s="24" t="n"/>
       <c r="B15" s="18" t="inlineStr">
         <is>
           <t>T12</t>

</xml_diff>

<commit_message>
Planilla 3: renombrar las unidades repetidas y orientar las dos PF01
Las carpinterias con cantidad 2 pasan a llamarse "a" y "b" en vez de
"X" y "X (2)", que se leia como si fueran dos modelos distintos: PF01 a
y PF01 b son las dos unidades de la misma carpinteria. Idem VA01, VA04 y
PV04.

PF01 a, la del lavadero, mira al Noroeste; PF01 b, la del hall, al
Sudoeste.

Quedan tres sin orientar: VA01 b de la suite y las dos VA04, del
dormitorio norte y del play room.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -8898,7 +8898,7 @@
         <v/>
       </c>
       <c r="E15" s="19">
-        <f>SUM(D15:D19)</f>
+        <f>SUM(D15:D20)</f>
         <v/>
       </c>
       <c r="F15" s="20">
@@ -8939,14 +8939,14 @@
     <row r="16" ht="70" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>PF04</t>
+          <t>PF01 b</t>
         </is>
       </c>
       <c r="B16" s="9" t="n">
-        <v>0.6</v>
+        <v>3</v>
       </c>
       <c r="C16" s="9" t="n">
-        <v>2.7</v>
+        <v>3.55</v>
       </c>
       <c r="D16" s="9">
         <f>IF(COUNT(B16,C16)&lt;2,"",B16*C16)</f>
@@ -8991,14 +8991,14 @@
     <row r="17" ht="70" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>VA01</t>
+          <t>PF04</t>
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>3</v>
+        <v>0.6</v>
       </c>
       <c r="C17" s="9" t="n">
-        <v>0.75</v>
+        <v>2.7</v>
       </c>
       <c r="D17" s="9">
         <f>IF(COUNT(B17,C17)&lt;2,"",B17*C17)</f>
@@ -9041,9 +9041,17 @@
       </c>
     </row>
     <row r="18" ht="70" customHeight="1">
-      <c r="A18" s="10" t="n"/>
-      <c r="B18" s="9" t="n"/>
-      <c r="C18" s="9" t="n"/>
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>VA01 a</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>0.75</v>
+      </c>
       <c r="D18" s="9">
         <f>IF(COUNT(B18,C18)&lt;2,"",B18*C18)</f>
         <v/>
@@ -9057,10 +9065,24 @@
         <f>IF(A18="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H18" s="10" t="n"/>
-      <c r="I18" s="10" t="n"/>
-      <c r="J18" s="9" t="n"/>
-      <c r="K18" s="10" t="n"/>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I18" s="10" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J18" s="9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K18" s="10" t="inlineStr">
+        <is>
+          <t>Sudoeste</t>
+        </is>
+      </c>
       <c r="L18" s="9">
         <f>IF(I18="","",IFERROR(VLOOKUP(I18,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
@@ -9071,128 +9093,106 @@
       </c>
     </row>
     <row r="19" ht="70" customHeight="1">
-      <c r="A19" s="14" t="n"/>
-      <c r="B19" s="13" t="n"/>
-      <c r="C19" s="13" t="n"/>
-      <c r="D19" s="13">
+      <c r="A19" s="10" t="n"/>
+      <c r="B19" s="9" t="n"/>
+      <c r="C19" s="9" t="n"/>
+      <c r="D19" s="9">
         <f>IF(COUNT(B19,C19)&lt;2,"",B19*C19)</f>
         <v/>
       </c>
-      <c r="E19" s="22" t="n"/>
-      <c r="F19" s="23">
+      <c r="E19" s="21" t="n"/>
+      <c r="F19" s="20">
         <f>IF(OR(D19="",$E$15=""),"",D19/$E$15)</f>
         <v/>
       </c>
-      <c r="G19" s="13">
+      <c r="G19" s="9">
         <f>IF(A19="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H19" s="14" t="n"/>
-      <c r="I19" s="14" t="n"/>
-      <c r="J19" s="13" t="n"/>
-      <c r="K19" s="14" t="n"/>
-      <c r="L19" s="13">
+      <c r="H19" s="10" t="n"/>
+      <c r="I19" s="10" t="n"/>
+      <c r="J19" s="9" t="n"/>
+      <c r="K19" s="10" t="n"/>
+      <c r="L19" s="9">
         <f>IF(I19="","",IFERROR(VLOOKUP(I19,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
-      <c r="M19" s="14">
+      <c r="M19" s="10">
         <f>IF(OR(D19="",J19=""),"",IF(J19&lt;=G19,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="20" ht="39.7" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="20" ht="70" customHeight="1">
+      <c r="A20" s="14" t="n"/>
+      <c r="B20" s="13" t="n"/>
+      <c r="C20" s="13" t="n"/>
+      <c r="D20" s="13">
+        <f>IF(COUNT(B20,C20)&lt;2,"",B20*C20)</f>
+        <v/>
+      </c>
+      <c r="E20" s="22" t="n"/>
+      <c r="F20" s="23">
+        <f>IF(OR(D20="",$E$15=""),"",D20/$E$15)</f>
+        <v/>
+      </c>
+      <c r="G20" s="13">
+        <f>IF(A20="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H20" s="14" t="n"/>
+      <c r="I20" s="14" t="n"/>
+      <c r="J20" s="13" t="n"/>
+      <c r="K20" s="14" t="n"/>
+      <c r="L20" s="13">
+        <f>IF(I20="","",IFERROR(VLOOKUP(I20,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M20" s="14">
+        <f>IF(OR(D20="",J20=""),"",IF(J20&lt;=G20,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="39.7" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Plano: Fachada Sudeste</t>
         </is>
       </c>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="4" t="n"/>
-      <c r="G20" s="4" t="n"/>
-      <c r="H20" s="4" t="n"/>
-      <c r="I20" s="4" t="n"/>
-      <c r="J20" s="4" t="n"/>
-      <c r="K20" s="4" t="n"/>
-      <c r="L20" s="4" t="n"/>
-      <c r="M20" s="4" t="n"/>
-    </row>
-    <row r="21" ht="70" customHeight="1">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>PF02</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C21" s="9" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="D21" s="9">
-        <f>IF(COUNT(B21,C21)&lt;2,"",B21*C21)</f>
-        <v/>
-      </c>
-      <c r="E21" s="19">
-        <f>SUM(D21:D26)</f>
-        <v/>
-      </c>
-      <c r="F21" s="20">
-        <f>IF(OR(D21="",$E$21=""),"",D21/$E$21)</f>
-        <v/>
-      </c>
-      <c r="G21" s="9">
-        <f>IF(A21="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H21" s="10" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I21" s="10" t="inlineStr">
-        <is>
-          <t>Sin Proteccion</t>
-        </is>
-      </c>
-      <c r="J21" s="9" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K21" s="10" t="inlineStr">
-        <is>
-          <t>Sudeste</t>
-        </is>
-      </c>
-      <c r="L21" s="9">
-        <f>IF(I21="","",IFERROR(VLOOKUP(I21,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M21" s="10">
-        <f>IF(OR(D21="",J21=""),"",IF(J21&lt;=G21,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
+      <c r="B21" s="4" t="n"/>
+      <c r="C21" s="4" t="n"/>
+      <c r="D21" s="4" t="n"/>
+      <c r="E21" s="4" t="n"/>
+      <c r="F21" s="4" t="n"/>
+      <c r="G21" s="4" t="n"/>
+      <c r="H21" s="4" t="n"/>
+      <c r="I21" s="4" t="n"/>
+      <c r="J21" s="4" t="n"/>
+      <c r="K21" s="4" t="n"/>
+      <c r="L21" s="4" t="n"/>
+      <c r="M21" s="4" t="n"/>
     </row>
     <row r="22" ht="70" customHeight="1">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>PV04</t>
+          <t>PF02</t>
         </is>
       </c>
       <c r="B22" s="9" t="n">
         <v>3</v>
       </c>
       <c r="C22" s="9" t="n">
-        <v>2.06</v>
+        <v>3.75</v>
       </c>
       <c r="D22" s="9">
         <f>IF(COUNT(B22,C22)&lt;2,"",B22*C22)</f>
         <v/>
       </c>
-      <c r="E22" s="21" t="n"/>
+      <c r="E22" s="19">
+        <f>SUM(D22:D27)</f>
+        <v/>
+      </c>
       <c r="F22" s="20">
-        <f>IF(OR(D22="",$E$21=""),"",D22/$E$21)</f>
+        <f>IF(OR(D22="",$E$22=""),"",D22/$E$22)</f>
         <v/>
       </c>
       <c r="G22" s="9">
@@ -9229,14 +9229,14 @@
     <row r="23" ht="70" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>PV04 (2)</t>
+          <t>PV04 a</t>
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>2.95</v>
+        <v>3</v>
       </c>
       <c r="C23" s="9" t="n">
-        <v>1.5</v>
+        <v>2.06</v>
       </c>
       <c r="D23" s="9">
         <f>IF(COUNT(B23,C23)&lt;2,"",B23*C23)</f>
@@ -9244,7 +9244,7 @@
       </c>
       <c r="E23" s="21" t="n"/>
       <c r="F23" s="20">
-        <f>IF(OR(D23="",$E$21=""),"",D23/$E$21)</f>
+        <f>IF(OR(D23="",$E$22=""),"",D23/$E$22)</f>
         <v/>
       </c>
       <c r="G23" s="9">
@@ -9281,14 +9281,14 @@
     <row r="24" ht="70" customHeight="1">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>VA05</t>
+          <t>PV04 b</t>
         </is>
       </c>
       <c r="B24" s="9" t="n">
-        <v>2.52</v>
+        <v>2.95</v>
       </c>
       <c r="C24" s="9" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="D24" s="9">
         <f>IF(COUNT(B24,C24)&lt;2,"",B24*C24)</f>
@@ -9296,7 +9296,7 @@
       </c>
       <c r="E24" s="21" t="n"/>
       <c r="F24" s="20">
-        <f>IF(OR(D24="",$E$21=""),"",D24/$E$21)</f>
+        <f>IF(OR(D24="",$E$22=""),"",D24/$E$22)</f>
         <v/>
       </c>
       <c r="G24" s="9">
@@ -9331,26 +9331,48 @@
       </c>
     </row>
     <row r="25" ht="70" customHeight="1">
-      <c r="A25" s="10" t="n"/>
-      <c r="B25" s="9" t="n"/>
-      <c r="C25" s="9" t="n"/>
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>VA05</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="C25" s="9" t="n">
+        <v>1.4</v>
+      </c>
       <c r="D25" s="9">
         <f>IF(COUNT(B25,C25)&lt;2,"",B25*C25)</f>
         <v/>
       </c>
       <c r="E25" s="21" t="n"/>
       <c r="F25" s="20">
-        <f>IF(OR(D25="",$E$21=""),"",D25/$E$21)</f>
+        <f>IF(OR(D25="",$E$22=""),"",D25/$E$22)</f>
         <v/>
       </c>
       <c r="G25" s="9">
         <f>IF(A25="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H25" s="10" t="n"/>
-      <c r="I25" s="10" t="n"/>
-      <c r="J25" s="9" t="n"/>
-      <c r="K25" s="10" t="n"/>
+      <c r="H25" s="10" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I25" s="10" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J25" s="9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K25" s="10" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
       <c r="L25" s="9">
         <f>IF(I25="","",IFERROR(VLOOKUP(I25,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
@@ -9361,128 +9383,106 @@
       </c>
     </row>
     <row r="26" ht="70" customHeight="1">
-      <c r="A26" s="14" t="n"/>
-      <c r="B26" s="13" t="n"/>
-      <c r="C26" s="13" t="n"/>
-      <c r="D26" s="13">
+      <c r="A26" s="10" t="n"/>
+      <c r="B26" s="9" t="n"/>
+      <c r="C26" s="9" t="n"/>
+      <c r="D26" s="9">
         <f>IF(COUNT(B26,C26)&lt;2,"",B26*C26)</f>
         <v/>
       </c>
-      <c r="E26" s="22" t="n"/>
-      <c r="F26" s="23">
-        <f>IF(OR(D26="",$E$21=""),"",D26/$E$21)</f>
-        <v/>
-      </c>
-      <c r="G26" s="13">
+      <c r="E26" s="21" t="n"/>
+      <c r="F26" s="20">
+        <f>IF(OR(D26="",$E$22=""),"",D26/$E$22)</f>
+        <v/>
+      </c>
+      <c r="G26" s="9">
         <f>IF(A26="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H26" s="14" t="n"/>
-      <c r="I26" s="14" t="n"/>
-      <c r="J26" s="13" t="n"/>
-      <c r="K26" s="14" t="n"/>
-      <c r="L26" s="13">
+      <c r="H26" s="10" t="n"/>
+      <c r="I26" s="10" t="n"/>
+      <c r="J26" s="9" t="n"/>
+      <c r="K26" s="10" t="n"/>
+      <c r="L26" s="9">
         <f>IF(I26="","",IFERROR(VLOOKUP(I26,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
-      <c r="M26" s="14">
+      <c r="M26" s="10">
         <f>IF(OR(D26="",J26=""),"",IF(J26&lt;=G26,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="27" ht="39.7" customHeight="1">
-      <c r="A27" s="5" t="inlineStr">
+    <row r="27" ht="70" customHeight="1">
+      <c r="A27" s="14" t="n"/>
+      <c r="B27" s="13" t="n"/>
+      <c r="C27" s="13" t="n"/>
+      <c r="D27" s="13">
+        <f>IF(COUNT(B27,C27)&lt;2,"",B27*C27)</f>
+        <v/>
+      </c>
+      <c r="E27" s="22" t="n"/>
+      <c r="F27" s="23">
+        <f>IF(OR(D27="",$E$22=""),"",D27/$E$22)</f>
+        <v/>
+      </c>
+      <c r="G27" s="13">
+        <f>IF(A27="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H27" s="14" t="n"/>
+      <c r="I27" s="14" t="n"/>
+      <c r="J27" s="13" t="n"/>
+      <c r="K27" s="14" t="n"/>
+      <c r="L27" s="13">
+        <f>IF(I27="","",IFERROR(VLOOKUP(I27,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M27" s="14">
+        <f>IF(OR(D27="",J27=""),"",IF(J27&lt;=G27,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="39.7" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>Plano: Fachada Noroeste</t>
         </is>
       </c>
-      <c r="B27" s="4" t="n"/>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="4" t="n"/>
-      <c r="G27" s="4" t="n"/>
-      <c r="H27" s="4" t="n"/>
-      <c r="I27" s="4" t="n"/>
-      <c r="J27" s="4" t="n"/>
-      <c r="K27" s="4" t="n"/>
-      <c r="L27" s="4" t="n"/>
-      <c r="M27" s="4" t="n"/>
-    </row>
-    <row r="28" ht="70" customHeight="1">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>PF03</t>
-        </is>
-      </c>
-      <c r="B28" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C28" s="9" t="n">
-        <v>2.88</v>
-      </c>
-      <c r="D28" s="9">
-        <f>IF(COUNT(B28,C28)&lt;2,"",B28*C28)</f>
-        <v/>
-      </c>
-      <c r="E28" s="19">
-        <f>SUM(D28:D32)</f>
-        <v/>
-      </c>
-      <c r="F28" s="20">
-        <f>IF(OR(D28="",$E$28=""),"",D28/$E$28)</f>
-        <v/>
-      </c>
-      <c r="G28" s="9">
-        <f>IF(A28="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H28" s="10" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I28" s="10" t="inlineStr">
-        <is>
-          <t>Sin Proteccion</t>
-        </is>
-      </c>
-      <c r="J28" s="9" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K28" s="10" t="inlineStr">
-        <is>
-          <t>Noroeste</t>
-        </is>
-      </c>
-      <c r="L28" s="9">
-        <f>IF(I28="","",IFERROR(VLOOKUP(I28,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M28" s="10">
-        <f>IF(OR(D28="",J28=""),"",IF(J28&lt;=G28,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
+      <c r="B28" s="4" t="n"/>
+      <c r="C28" s="4" t="n"/>
+      <c r="D28" s="4" t="n"/>
+      <c r="E28" s="4" t="n"/>
+      <c r="F28" s="4" t="n"/>
+      <c r="G28" s="4" t="n"/>
+      <c r="H28" s="4" t="n"/>
+      <c r="I28" s="4" t="n"/>
+      <c r="J28" s="4" t="n"/>
+      <c r="K28" s="4" t="n"/>
+      <c r="L28" s="4" t="n"/>
+      <c r="M28" s="4" t="n"/>
     </row>
     <row r="29" ht="70" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>PV01</t>
+          <t>PF03</t>
         </is>
       </c>
       <c r="B29" s="9" t="n">
         <v>3</v>
       </c>
       <c r="C29" s="9" t="n">
-        <v>7.7</v>
+        <v>2.88</v>
       </c>
       <c r="D29" s="9">
         <f>IF(COUNT(B29,C29)&lt;2,"",B29*C29)</f>
         <v/>
       </c>
-      <c r="E29" s="21" t="n"/>
+      <c r="E29" s="19">
+        <f>SUM(D29:D34)</f>
+        <v/>
+      </c>
       <c r="F29" s="20">
-        <f>IF(OR(D29="",$E$28=""),"",D29/$E$28)</f>
+        <f>IF(OR(D29="",$E$29=""),"",D29/$E$29)</f>
         <v/>
       </c>
       <c r="G29" s="9">
@@ -9519,14 +9519,14 @@
     <row r="30" ht="70" customHeight="1">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>PV02</t>
+          <t>PF01 a</t>
         </is>
       </c>
       <c r="B30" s="9" t="n">
         <v>3</v>
       </c>
       <c r="C30" s="9" t="n">
-        <v>2.48</v>
+        <v>3.55</v>
       </c>
       <c r="D30" s="9">
         <f>IF(COUNT(B30,C30)&lt;2,"",B30*C30)</f>
@@ -9534,7 +9534,7 @@
       </c>
       <c r="E30" s="21" t="n"/>
       <c r="F30" s="20">
-        <f>IF(OR(D30="",$E$28=""),"",D30/$E$28)</f>
+        <f>IF(OR(D30="",$E$29=""),"",D30/$E$29)</f>
         <v/>
       </c>
       <c r="G30" s="9">
@@ -9569,26 +9569,48 @@
       </c>
     </row>
     <row r="31" ht="70" customHeight="1">
-      <c r="A31" s="10" t="n"/>
-      <c r="B31" s="9" t="n"/>
-      <c r="C31" s="9" t="n"/>
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>PV01</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C31" s="9" t="n">
+        <v>7.7</v>
+      </c>
       <c r="D31" s="9">
         <f>IF(COUNT(B31,C31)&lt;2,"",B31*C31)</f>
         <v/>
       </c>
       <c r="E31" s="21" t="n"/>
       <c r="F31" s="20">
-        <f>IF(OR(D31="",$E$28=""),"",D31/$E$28)</f>
+        <f>IF(OR(D31="",$E$29=""),"",D31/$E$29)</f>
         <v/>
       </c>
       <c r="G31" s="9">
         <f>IF(A31="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H31" s="10" t="n"/>
-      <c r="I31" s="10" t="n"/>
-      <c r="J31" s="9" t="n"/>
-      <c r="K31" s="10" t="n"/>
+      <c r="H31" s="10" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I31" s="10" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J31" s="9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K31" s="10" t="inlineStr">
+        <is>
+          <t>Noroeste</t>
+        </is>
+      </c>
       <c r="L31" s="9">
         <f>IF(I31="","",IFERROR(VLOOKUP(I31,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
@@ -9599,157 +9621,140 @@
       </c>
     </row>
     <row r="32" ht="70" customHeight="1">
-      <c r="A32" s="14" t="n"/>
-      <c r="B32" s="13" t="n"/>
-      <c r="C32" s="13" t="n"/>
-      <c r="D32" s="13">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>PV02</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C32" s="9" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="D32" s="9">
         <f>IF(COUNT(B32,C32)&lt;2,"",B32*C32)</f>
         <v/>
       </c>
-      <c r="E32" s="22" t="n"/>
-      <c r="F32" s="23">
-        <f>IF(OR(D32="",$E$28=""),"",D32/$E$28)</f>
-        <v/>
-      </c>
-      <c r="G32" s="13">
+      <c r="E32" s="21" t="n"/>
+      <c r="F32" s="20">
+        <f>IF(OR(D32="",$E$29=""),"",D32/$E$29)</f>
+        <v/>
+      </c>
+      <c r="G32" s="9">
         <f>IF(A32="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H32" s="14" t="n"/>
-      <c r="I32" s="14" t="n"/>
-      <c r="J32" s="13" t="n"/>
-      <c r="K32" s="14" t="n"/>
-      <c r="L32" s="13">
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I32" s="10" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J32" s="9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K32" s="10" t="inlineStr">
+        <is>
+          <t>Noroeste</t>
+        </is>
+      </c>
+      <c r="L32" s="9">
         <f>IF(I32="","",IFERROR(VLOOKUP(I32,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
-      <c r="M32" s="14">
+      <c r="M32" s="10">
         <f>IF(OR(D32="",J32=""),"",IF(J32&lt;=G32,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="33" ht="39.7" customHeight="1">
-      <c r="A33" s="5" t="inlineStr">
+    <row r="33" ht="70" customHeight="1">
+      <c r="A33" s="10" t="n"/>
+      <c r="B33" s="9" t="n"/>
+      <c r="C33" s="9" t="n"/>
+      <c r="D33" s="9">
+        <f>IF(COUNT(B33,C33)&lt;2,"",B33*C33)</f>
+        <v/>
+      </c>
+      <c r="E33" s="21" t="n"/>
+      <c r="F33" s="20">
+        <f>IF(OR(D33="",$E$29=""),"",D33/$E$29)</f>
+        <v/>
+      </c>
+      <c r="G33" s="9">
+        <f>IF(A33="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H33" s="10" t="n"/>
+      <c r="I33" s="10" t="n"/>
+      <c r="J33" s="9" t="n"/>
+      <c r="K33" s="10" t="n"/>
+      <c r="L33" s="9">
+        <f>IF(I33="","",IFERROR(VLOOKUP(I33,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M33" s="10">
+        <f>IF(OR(D33="",J33=""),"",IF(J33&lt;=G33,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="70" customHeight="1">
+      <c r="A34" s="14" t="n"/>
+      <c r="B34" s="13" t="n"/>
+      <c r="C34" s="13" t="n"/>
+      <c r="D34" s="13">
+        <f>IF(COUNT(B34,C34)&lt;2,"",B34*C34)</f>
+        <v/>
+      </c>
+      <c r="E34" s="22" t="n"/>
+      <c r="F34" s="23">
+        <f>IF(OR(D34="",$E$29=""),"",D34/$E$29)</f>
+        <v/>
+      </c>
+      <c r="G34" s="13">
+        <f>IF(A34="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H34" s="14" t="n"/>
+      <c r="I34" s="14" t="n"/>
+      <c r="J34" s="13" t="n"/>
+      <c r="K34" s="14" t="n"/>
+      <c r="L34" s="13">
+        <f>IF(I34="","",IFERROR(VLOOKUP(I34,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M34" s="14">
+        <f>IF(OR(D34="",J34=""),"",IF(J34&lt;=G34,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="39.7" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>Plano: Orientacion a confirmar</t>
         </is>
       </c>
-      <c r="B33" s="4" t="n"/>
-      <c r="C33" s="4" t="n"/>
-      <c r="D33" s="4" t="n"/>
-      <c r="E33" s="4" t="n"/>
-      <c r="F33" s="4" t="n"/>
-      <c r="G33" s="4" t="n"/>
-      <c r="H33" s="4" t="n"/>
-      <c r="I33" s="4" t="n"/>
-      <c r="J33" s="4" t="n"/>
-      <c r="K33" s="4" t="n"/>
-      <c r="L33" s="4" t="n"/>
-      <c r="M33" s="4" t="n"/>
-    </row>
-    <row r="34" ht="70" customHeight="1">
-      <c r="A34" s="10" t="inlineStr">
-        <is>
-          <t>PF01</t>
-        </is>
-      </c>
-      <c r="B34" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C34" s="9" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="D34" s="9">
-        <f>IF(COUNT(B34,C34)&lt;2,"",B34*C34)</f>
-        <v/>
-      </c>
-      <c r="E34" s="19">
-        <f>SUM(D34:D40)</f>
-        <v/>
-      </c>
-      <c r="F34" s="20">
-        <f>IF(OR(D34="",$E$34=""),"",D34/$E$34)</f>
-        <v/>
-      </c>
-      <c r="G34" s="9">
-        <f>IF(A34="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H34" s="10" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I34" s="10" t="inlineStr">
-        <is>
-          <t>Sin Proteccion</t>
-        </is>
-      </c>
-      <c r="J34" s="9" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K34" s="10" t="n"/>
-      <c r="L34" s="9">
-        <f>IF(I34="","",IFERROR(VLOOKUP(I34,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M34" s="10">
-        <f>IF(OR(D34="",J34=""),"",IF(J34&lt;=G34,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" ht="70" customHeight="1">
-      <c r="A35" s="10" t="inlineStr">
-        <is>
-          <t>PF01 (2)</t>
-        </is>
-      </c>
-      <c r="B35" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C35" s="9" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="D35" s="9">
-        <f>IF(COUNT(B35,C35)&lt;2,"",B35*C35)</f>
-        <v/>
-      </c>
-      <c r="E35" s="21" t="n"/>
-      <c r="F35" s="20">
-        <f>IF(OR(D35="",$E$34=""),"",D35/$E$34)</f>
-        <v/>
-      </c>
-      <c r="G35" s="9">
-        <f>IF(A35="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H35" s="10" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I35" s="10" t="inlineStr">
-        <is>
-          <t>Sin Proteccion</t>
-        </is>
-      </c>
-      <c r="J35" s="9" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K35" s="10" t="n"/>
-      <c r="L35" s="9">
-        <f>IF(I35="","",IFERROR(VLOOKUP(I35,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M35" s="10">
-        <f>IF(OR(D35="",J35=""),"",IF(J35&lt;=G35,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
+      <c r="B35" s="4" t="n"/>
+      <c r="C35" s="4" t="n"/>
+      <c r="D35" s="4" t="n"/>
+      <c r="E35" s="4" t="n"/>
+      <c r="F35" s="4" t="n"/>
+      <c r="G35" s="4" t="n"/>
+      <c r="H35" s="4" t="n"/>
+      <c r="I35" s="4" t="n"/>
+      <c r="J35" s="4" t="n"/>
+      <c r="K35" s="4" t="n"/>
+      <c r="L35" s="4" t="n"/>
+      <c r="M35" s="4" t="n"/>
     </row>
     <row r="36" ht="70" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>VA01 (2)</t>
+          <t>VA01 b</t>
         </is>
       </c>
       <c r="B36" s="9" t="n">
@@ -9762,9 +9767,12 @@
         <f>IF(COUNT(B36,C36)&lt;2,"",B36*C36)</f>
         <v/>
       </c>
-      <c r="E36" s="21" t="n"/>
+      <c r="E36" s="19">
+        <f>SUM(D36:D40)</f>
+        <v/>
+      </c>
       <c r="F36" s="20">
-        <f>IF(OR(D36="",$E$34=""),"",D36/$E$34)</f>
+        <f>IF(OR(D36="",$E$36=""),"",D36/$E$36)</f>
         <v/>
       </c>
       <c r="G36" s="9">
@@ -9797,7 +9805,7 @@
     <row r="37" ht="70" customHeight="1">
       <c r="A37" s="10" t="inlineStr">
         <is>
-          <t>VA04</t>
+          <t>VA04 a</t>
         </is>
       </c>
       <c r="B37" s="9" t="n">
@@ -9812,7 +9820,7 @@
       </c>
       <c r="E37" s="21" t="n"/>
       <c r="F37" s="20">
-        <f>IF(OR(D37="",$E$34=""),"",D37/$E$34)</f>
+        <f>IF(OR(D37="",$E$36=""),"",D37/$E$36)</f>
         <v/>
       </c>
       <c r="G37" s="9">
@@ -9845,7 +9853,7 @@
     <row r="38" ht="70" customHeight="1">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>VA04 (2)</t>
+          <t>VA04 b</t>
         </is>
       </c>
       <c r="B38" s="9" t="n">
@@ -9860,7 +9868,7 @@
       </c>
       <c r="E38" s="21" t="n"/>
       <c r="F38" s="20">
-        <f>IF(OR(D38="",$E$34=""),"",D38/$E$34)</f>
+        <f>IF(OR(D38="",$E$36=""),"",D38/$E$36)</f>
         <v/>
       </c>
       <c r="G38" s="9">
@@ -9900,7 +9908,7 @@
       </c>
       <c r="E39" s="21" t="n"/>
       <c r="F39" s="20">
-        <f>IF(OR(D39="",$E$34=""),"",D39/$E$34)</f>
+        <f>IF(OR(D39="",$E$36=""),"",D39/$E$36)</f>
         <v/>
       </c>
       <c r="G39" s="9">
@@ -9930,7 +9938,7 @@
       </c>
       <c r="E40" s="22" t="n"/>
       <c r="F40" s="23">
-        <f>IF(OR(D40="",$E$34=""),"",D40/$E$34)</f>
+        <f>IF(OR(D40="",$E$36=""),"",D40/$E$36)</f>
         <v/>
       </c>
       <c r="G40" s="13">
@@ -10910,20 +10918,20 @@
   <mergeCells count="16">
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="A14:M14"/>
-    <mergeCell ref="E34:E40"/>
-    <mergeCell ref="A27:M27"/>
-    <mergeCell ref="E15:E19"/>
     <mergeCell ref="A6:M6"/>
-    <mergeCell ref="E21:E26"/>
+    <mergeCell ref="E15:E20"/>
     <mergeCell ref="B3:L3"/>
     <mergeCell ref="B2:L2"/>
     <mergeCell ref="A4:M4"/>
     <mergeCell ref="E7:E13"/>
-    <mergeCell ref="E28:E32"/>
-    <mergeCell ref="A20:M20"/>
-    <mergeCell ref="A33:M33"/>
+    <mergeCell ref="A21:M21"/>
+    <mergeCell ref="E29:E34"/>
+    <mergeCell ref="A35:M35"/>
+    <mergeCell ref="E36:E40"/>
+    <mergeCell ref="E22:E27"/>
     <mergeCell ref="M1:M3"/>
     <mergeCell ref="B1:L1"/>
+    <mergeCell ref="A28:M28"/>
   </mergeCells>
   <conditionalFormatting sqref="M6:M40">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">

</xml_diff>

<commit_message>
Planilla 3: mostrar las unidades repetidas con su designacion real
Las dos unidades de PF01, VA01, VA04 y PV04 se muestran las dos con el
mismo nombre, como en la planilla de carpinterias. La fachada y la
ubicacion ya las distinguen. El sufijo a y b se mantiene solo adentro
del generador, para que cada fila conserve su altura: las dos PV04 miden
distinto, 3,00 y 2,95.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -8939,7 +8939,7 @@
     <row r="16" ht="70" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>PF01 b</t>
+          <t>PF01</t>
         </is>
       </c>
       <c r="B16" s="9" t="n">
@@ -9043,7 +9043,7 @@
     <row r="18" ht="70" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>VA01 a</t>
+          <t>VA01</t>
         </is>
       </c>
       <c r="B18" s="9" t="n">
@@ -9229,7 +9229,7 @@
     <row r="23" ht="70" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>PV04 a</t>
+          <t>PV04</t>
         </is>
       </c>
       <c r="B23" s="9" t="n">
@@ -9281,7 +9281,7 @@
     <row r="24" ht="70" customHeight="1">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>PV04 b</t>
+          <t>PV04</t>
         </is>
       </c>
       <c r="B24" s="9" t="n">
@@ -9519,7 +9519,7 @@
     <row r="30" ht="70" customHeight="1">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>PF01 a</t>
+          <t>PF01</t>
         </is>
       </c>
       <c r="B30" s="9" t="n">
@@ -9754,7 +9754,7 @@
     <row r="36" ht="70" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>VA01 b</t>
+          <t>VA01</t>
         </is>
       </c>
       <c r="B36" s="9" t="n">
@@ -9805,7 +9805,7 @@
     <row r="37" ht="70" customHeight="1">
       <c r="A37" s="10" t="inlineStr">
         <is>
-          <t>VA04 a</t>
+          <t>VA04</t>
         </is>
       </c>
       <c r="B37" s="9" t="n">
@@ -9853,7 +9853,7 @@
     <row r="38" ht="70" customHeight="1">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>VA04 b</t>
+          <t>VA04</t>
         </is>
       </c>
       <c r="B38" s="9" t="n">

</xml_diff>

<commit_message>
Planilla 3: las dos VA04 van a la fachada Noroeste
Dato del autor del proyecto. En el PDF de fachadas estan dibujadas pero
sin rotulo de texto, por eso no aparecian en la extraccion.

Queda una sola sin orientar: la VA01 de la suite.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -9478,7 +9478,7 @@
         <v/>
       </c>
       <c r="E29" s="19">
-        <f>SUM(D29:D34)</f>
+        <f>SUM(D29:D36)</f>
         <v/>
       </c>
       <c r="F29" s="20">
@@ -9673,9 +9673,17 @@
       </c>
     </row>
     <row r="33" ht="70" customHeight="1">
-      <c r="A33" s="10" t="n"/>
-      <c r="B33" s="9" t="n"/>
-      <c r="C33" s="9" t="n"/>
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>VA04</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="C33" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="D33" s="9">
         <f>IF(COUNT(B33,C33)&lt;2,"",B33*C33)</f>
         <v/>
@@ -9689,10 +9697,24 @@
         <f>IF(A33="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H33" s="10" t="n"/>
-      <c r="I33" s="10" t="n"/>
-      <c r="J33" s="9" t="n"/>
-      <c r="K33" s="10" t="n"/>
+      <c r="H33" s="10" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I33" s="10" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J33" s="9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K33" s="10" t="inlineStr">
+        <is>
+          <t>Noroeste</t>
+        </is>
+      </c>
       <c r="L33" s="9">
         <f>IF(I33="","",IFERROR(VLOOKUP(I33,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
@@ -9703,172 +9725,158 @@
       </c>
     </row>
     <row r="34" ht="70" customHeight="1">
-      <c r="A34" s="14" t="n"/>
-      <c r="B34" s="13" t="n"/>
-      <c r="C34" s="13" t="n"/>
-      <c r="D34" s="13">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>VA04</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="C34" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" s="9">
         <f>IF(COUNT(B34,C34)&lt;2,"",B34*C34)</f>
         <v/>
       </c>
-      <c r="E34" s="22" t="n"/>
-      <c r="F34" s="23">
+      <c r="E34" s="21" t="n"/>
+      <c r="F34" s="20">
         <f>IF(OR(D34="",$E$29=""),"",D34/$E$29)</f>
         <v/>
       </c>
-      <c r="G34" s="13">
+      <c r="G34" s="9">
         <f>IF(A34="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H34" s="14" t="n"/>
-      <c r="I34" s="14" t="n"/>
-      <c r="J34" s="13" t="n"/>
-      <c r="K34" s="14" t="n"/>
-      <c r="L34" s="13">
+      <c r="H34" s="10" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I34" s="10" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J34" s="9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K34" s="10" t="inlineStr">
+        <is>
+          <t>Noroeste</t>
+        </is>
+      </c>
+      <c r="L34" s="9">
         <f>IF(I34="","",IFERROR(VLOOKUP(I34,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
-      <c r="M34" s="14">
+      <c r="M34" s="10">
         <f>IF(OR(D34="",J34=""),"",IF(J34&lt;=G34,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="35" ht="39.7" customHeight="1">
-      <c r="A35" s="5" t="inlineStr">
+    <row r="35" ht="70" customHeight="1">
+      <c r="A35" s="10" t="n"/>
+      <c r="B35" s="9" t="n"/>
+      <c r="C35" s="9" t="n"/>
+      <c r="D35" s="9">
+        <f>IF(COUNT(B35,C35)&lt;2,"",B35*C35)</f>
+        <v/>
+      </c>
+      <c r="E35" s="21" t="n"/>
+      <c r="F35" s="20">
+        <f>IF(OR(D35="",$E$29=""),"",D35/$E$29)</f>
+        <v/>
+      </c>
+      <c r="G35" s="9">
+        <f>IF(A35="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H35" s="10" t="n"/>
+      <c r="I35" s="10" t="n"/>
+      <c r="J35" s="9" t="n"/>
+      <c r="K35" s="10" t="n"/>
+      <c r="L35" s="9">
+        <f>IF(I35="","",IFERROR(VLOOKUP(I35,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M35" s="10">
+        <f>IF(OR(D35="",J35=""),"",IF(J35&lt;=G35,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="70" customHeight="1">
+      <c r="A36" s="14" t="n"/>
+      <c r="B36" s="13" t="n"/>
+      <c r="C36" s="13" t="n"/>
+      <c r="D36" s="13">
+        <f>IF(COUNT(B36,C36)&lt;2,"",B36*C36)</f>
+        <v/>
+      </c>
+      <c r="E36" s="22" t="n"/>
+      <c r="F36" s="23">
+        <f>IF(OR(D36="",$E$29=""),"",D36/$E$29)</f>
+        <v/>
+      </c>
+      <c r="G36" s="13">
+        <f>IF(A36="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H36" s="14" t="n"/>
+      <c r="I36" s="14" t="n"/>
+      <c r="J36" s="13" t="n"/>
+      <c r="K36" s="14" t="n"/>
+      <c r="L36" s="13">
+        <f>IF(I36="","",IFERROR(VLOOKUP(I36,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M36" s="14">
+        <f>IF(OR(D36="",J36=""),"",IF(J36&lt;=G36,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="39.7" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>Plano: Orientacion a confirmar</t>
         </is>
       </c>
-      <c r="B35" s="4" t="n"/>
-      <c r="C35" s="4" t="n"/>
-      <c r="D35" s="4" t="n"/>
-      <c r="E35" s="4" t="n"/>
-      <c r="F35" s="4" t="n"/>
-      <c r="G35" s="4" t="n"/>
-      <c r="H35" s="4" t="n"/>
-      <c r="I35" s="4" t="n"/>
-      <c r="J35" s="4" t="n"/>
-      <c r="K35" s="4" t="n"/>
-      <c r="L35" s="4" t="n"/>
-      <c r="M35" s="4" t="n"/>
-    </row>
-    <row r="36" ht="70" customHeight="1">
-      <c r="A36" s="10" t="inlineStr">
-        <is>
-          <t>VA01</t>
-        </is>
-      </c>
-      <c r="B36" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C36" s="9" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D36" s="9">
-        <f>IF(COUNT(B36,C36)&lt;2,"",B36*C36)</f>
-        <v/>
-      </c>
-      <c r="E36" s="19">
-        <f>SUM(D36:D40)</f>
-        <v/>
-      </c>
-      <c r="F36" s="20">
-        <f>IF(OR(D36="",$E$36=""),"",D36/$E$36)</f>
-        <v/>
-      </c>
-      <c r="G36" s="9">
-        <f>IF(A36="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H36" s="10" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I36" s="10" t="inlineStr">
-        <is>
-          <t>Sin Proteccion</t>
-        </is>
-      </c>
-      <c r="J36" s="9" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K36" s="10" t="n"/>
-      <c r="L36" s="9">
-        <f>IF(I36="","",IFERROR(VLOOKUP(I36,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M36" s="10">
-        <f>IF(OR(D36="",J36=""),"",IF(J36&lt;=G36,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" ht="70" customHeight="1">
-      <c r="A37" s="10" t="inlineStr">
-        <is>
-          <t>VA04</t>
-        </is>
-      </c>
-      <c r="B37" s="9" t="n">
-        <v>2.52</v>
-      </c>
-      <c r="C37" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D37" s="9">
-        <f>IF(COUNT(B37,C37)&lt;2,"",B37*C37)</f>
-        <v/>
-      </c>
-      <c r="E37" s="21" t="n"/>
-      <c r="F37" s="20">
-        <f>IF(OR(D37="",$E$36=""),"",D37/$E$36)</f>
-        <v/>
-      </c>
-      <c r="G37" s="9">
-        <f>IF(A37="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H37" s="10" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I37" s="10" t="inlineStr">
-        <is>
-          <t>Sin Proteccion</t>
-        </is>
-      </c>
-      <c r="J37" s="9" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K37" s="10" t="n"/>
-      <c r="L37" s="9">
-        <f>IF(I37="","",IFERROR(VLOOKUP(I37,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M37" s="10">
-        <f>IF(OR(D37="",J37=""),"",IF(J37&lt;=G37,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
+      <c r="B37" s="4" t="n"/>
+      <c r="C37" s="4" t="n"/>
+      <c r="D37" s="4" t="n"/>
+      <c r="E37" s="4" t="n"/>
+      <c r="F37" s="4" t="n"/>
+      <c r="G37" s="4" t="n"/>
+      <c r="H37" s="4" t="n"/>
+      <c r="I37" s="4" t="n"/>
+      <c r="J37" s="4" t="n"/>
+      <c r="K37" s="4" t="n"/>
+      <c r="L37" s="4" t="n"/>
+      <c r="M37" s="4" t="n"/>
     </row>
     <row r="38" ht="70" customHeight="1">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>VA04</t>
+          <t>VA01</t>
         </is>
       </c>
       <c r="B38" s="9" t="n">
-        <v>2.52</v>
+        <v>3</v>
       </c>
       <c r="C38" s="9" t="n">
-        <v>2</v>
+        <v>0.75</v>
       </c>
       <c r="D38" s="9">
         <f>IF(COUNT(B38,C38)&lt;2,"",B38*C38)</f>
         <v/>
       </c>
-      <c r="E38" s="21" t="n"/>
+      <c r="E38" s="19">
+        <f>SUM(D38:D40)</f>
+        <v/>
+      </c>
       <c r="F38" s="20">
-        <f>IF(OR(D38="",$E$36=""),"",D38/$E$36)</f>
+        <f>IF(OR(D38="",$E$38=""),"",D38/$E$38)</f>
         <v/>
       </c>
       <c r="G38" s="9">
@@ -9908,7 +9916,7 @@
       </c>
       <c r="E39" s="21" t="n"/>
       <c r="F39" s="20">
-        <f>IF(OR(D39="",$E$36=""),"",D39/$E$36)</f>
+        <f>IF(OR(D39="",$E$38=""),"",D39/$E$38)</f>
         <v/>
       </c>
       <c r="G39" s="9">
@@ -9938,7 +9946,7 @@
       </c>
       <c r="E40" s="22" t="n"/>
       <c r="F40" s="23">
-        <f>IF(OR(D40="",$E$36=""),"",D40/$E$36)</f>
+        <f>IF(OR(D40="",$E$38=""),"",D40/$E$38)</f>
         <v/>
       </c>
       <c r="G40" s="13">
@@ -10918,6 +10926,7 @@
   <mergeCells count="16">
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="A14:M14"/>
+    <mergeCell ref="A37:M37"/>
     <mergeCell ref="A6:M6"/>
     <mergeCell ref="E15:E20"/>
     <mergeCell ref="B3:L3"/>
@@ -10925,9 +10934,8 @@
     <mergeCell ref="A4:M4"/>
     <mergeCell ref="E7:E13"/>
     <mergeCell ref="A21:M21"/>
-    <mergeCell ref="E29:E34"/>
-    <mergeCell ref="A35:M35"/>
-    <mergeCell ref="E36:E40"/>
+    <mergeCell ref="E29:E36"/>
+    <mergeCell ref="E38:E40"/>
     <mergeCell ref="E22:E27"/>
     <mergeCell ref="M1:M3"/>
     <mergeCell ref="B1:L1"/>

</xml_diff>

<commit_message>
Planilla 3: la VA01 de la suite va al Sudoeste
Con esto las veinte aberturas quedan orientadas y desaparece el bloque de
orientacion a confirmar. Las dos unidades de VA01, la de la cocina y la
de la suite, dan a la misma fachada.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -31,7 +31,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Iluminacion y ventilacion'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Planilla 3 higrotermica'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla 3 higrotermica'!$A$1:$M$40</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla 3 higrotermica'!$A$1:$M$37</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Planilla vigas'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Planilla vigas'!$A$1:$X$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Planilla losas'!$1:$3</definedName>
@@ -8355,7 +8355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M92"/>
+  <dimension ref="A1:M89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21.6" customWidth="1" min="1" max="1"/>
@@ -8898,7 +8898,7 @@
         <v/>
       </c>
       <c r="E15" s="19">
-        <f>SUM(D15:D20)</f>
+        <f>SUM(D15:D21)</f>
         <v/>
       </c>
       <c r="F15" s="20">
@@ -9093,9 +9093,17 @@
       </c>
     </row>
     <row r="19" ht="70" customHeight="1">
-      <c r="A19" s="10" t="n"/>
-      <c r="B19" s="9" t="n"/>
-      <c r="C19" s="9" t="n"/>
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>VA01</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" s="9" t="n">
+        <v>0.75</v>
+      </c>
       <c r="D19" s="9">
         <f>IF(COUNT(B19,C19)&lt;2,"",B19*C19)</f>
         <v/>
@@ -9109,10 +9117,24 @@
         <f>IF(A19="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H19" s="10" t="n"/>
-      <c r="I19" s="10" t="n"/>
-      <c r="J19" s="9" t="n"/>
-      <c r="K19" s="10" t="n"/>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J19" s="9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K19" s="10" t="inlineStr">
+        <is>
+          <t>Sudoeste</t>
+        </is>
+      </c>
       <c r="L19" s="9">
         <f>IF(I19="","",IFERROR(VLOOKUP(I19,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
@@ -9123,128 +9145,106 @@
       </c>
     </row>
     <row r="20" ht="70" customHeight="1">
-      <c r="A20" s="14" t="n"/>
-      <c r="B20" s="13" t="n"/>
-      <c r="C20" s="13" t="n"/>
-      <c r="D20" s="13">
+      <c r="A20" s="10" t="n"/>
+      <c r="B20" s="9" t="n"/>
+      <c r="C20" s="9" t="n"/>
+      <c r="D20" s="9">
         <f>IF(COUNT(B20,C20)&lt;2,"",B20*C20)</f>
         <v/>
       </c>
-      <c r="E20" s="22" t="n"/>
-      <c r="F20" s="23">
+      <c r="E20" s="21" t="n"/>
+      <c r="F20" s="20">
         <f>IF(OR(D20="",$E$15=""),"",D20/$E$15)</f>
         <v/>
       </c>
-      <c r="G20" s="13">
+      <c r="G20" s="9">
         <f>IF(A20="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H20" s="14" t="n"/>
-      <c r="I20" s="14" t="n"/>
-      <c r="J20" s="13" t="n"/>
-      <c r="K20" s="14" t="n"/>
-      <c r="L20" s="13">
+      <c r="H20" s="10" t="n"/>
+      <c r="I20" s="10" t="n"/>
+      <c r="J20" s="9" t="n"/>
+      <c r="K20" s="10" t="n"/>
+      <c r="L20" s="9">
         <f>IF(I20="","",IFERROR(VLOOKUP(I20,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
-      <c r="M20" s="14">
+      <c r="M20" s="10">
         <f>IF(OR(D20="",J20=""),"",IF(J20&lt;=G20,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="21" ht="39.7" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
+    <row r="21" ht="70" customHeight="1">
+      <c r="A21" s="14" t="n"/>
+      <c r="B21" s="13" t="n"/>
+      <c r="C21" s="13" t="n"/>
+      <c r="D21" s="13">
+        <f>IF(COUNT(B21,C21)&lt;2,"",B21*C21)</f>
+        <v/>
+      </c>
+      <c r="E21" s="22" t="n"/>
+      <c r="F21" s="23">
+        <f>IF(OR(D21="",$E$15=""),"",D21/$E$15)</f>
+        <v/>
+      </c>
+      <c r="G21" s="13">
+        <f>IF(A21="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H21" s="14" t="n"/>
+      <c r="I21" s="14" t="n"/>
+      <c r="J21" s="13" t="n"/>
+      <c r="K21" s="14" t="n"/>
+      <c r="L21" s="13">
+        <f>IF(I21="","",IFERROR(VLOOKUP(I21,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M21" s="14">
+        <f>IF(OR(D21="",J21=""),"",IF(J21&lt;=G21,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="39.7" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Plano: Fachada Sudeste</t>
         </is>
       </c>
-      <c r="B21" s="4" t="n"/>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="4" t="n"/>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="4" t="n"/>
-      <c r="G21" s="4" t="n"/>
-      <c r="H21" s="4" t="n"/>
-      <c r="I21" s="4" t="n"/>
-      <c r="J21" s="4" t="n"/>
-      <c r="K21" s="4" t="n"/>
-      <c r="L21" s="4" t="n"/>
-      <c r="M21" s="4" t="n"/>
-    </row>
-    <row r="22" ht="70" customHeight="1">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>PF02</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C22" s="9" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="D22" s="9">
-        <f>IF(COUNT(B22,C22)&lt;2,"",B22*C22)</f>
-        <v/>
-      </c>
-      <c r="E22" s="19">
-        <f>SUM(D22:D27)</f>
-        <v/>
-      </c>
-      <c r="F22" s="20">
-        <f>IF(OR(D22="",$E$22=""),"",D22/$E$22)</f>
-        <v/>
-      </c>
-      <c r="G22" s="9">
-        <f>IF(A22="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H22" s="10" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I22" s="10" t="inlineStr">
-        <is>
-          <t>Sin Proteccion</t>
-        </is>
-      </c>
-      <c r="J22" s="9" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K22" s="10" t="inlineStr">
-        <is>
-          <t>Sudeste</t>
-        </is>
-      </c>
-      <c r="L22" s="9">
-        <f>IF(I22="","",IFERROR(VLOOKUP(I22,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M22" s="10">
-        <f>IF(OR(D22="",J22=""),"",IF(J22&lt;=G22,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
+      <c r="B22" s="4" t="n"/>
+      <c r="C22" s="4" t="n"/>
+      <c r="D22" s="4" t="n"/>
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="n"/>
+      <c r="I22" s="4" t="n"/>
+      <c r="J22" s="4" t="n"/>
+      <c r="K22" s="4" t="n"/>
+      <c r="L22" s="4" t="n"/>
+      <c r="M22" s="4" t="n"/>
     </row>
     <row r="23" ht="70" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>PV04</t>
+          <t>PF02</t>
         </is>
       </c>
       <c r="B23" s="9" t="n">
         <v>3</v>
       </c>
       <c r="C23" s="9" t="n">
-        <v>2.06</v>
+        <v>3.75</v>
       </c>
       <c r="D23" s="9">
         <f>IF(COUNT(B23,C23)&lt;2,"",B23*C23)</f>
         <v/>
       </c>
-      <c r="E23" s="21" t="n"/>
+      <c r="E23" s="19">
+        <f>SUM(D23:D28)</f>
+        <v/>
+      </c>
       <c r="F23" s="20">
-        <f>IF(OR(D23="",$E$22=""),"",D23/$E$22)</f>
+        <f>IF(OR(D23="",$E$23=""),"",D23/$E$23)</f>
         <v/>
       </c>
       <c r="G23" s="9">
@@ -9285,10 +9285,10 @@
         </is>
       </c>
       <c r="B24" s="9" t="n">
-        <v>2.95</v>
+        <v>3</v>
       </c>
       <c r="C24" s="9" t="n">
-        <v>1.5</v>
+        <v>2.06</v>
       </c>
       <c r="D24" s="9">
         <f>IF(COUNT(B24,C24)&lt;2,"",B24*C24)</f>
@@ -9296,7 +9296,7 @@
       </c>
       <c r="E24" s="21" t="n"/>
       <c r="F24" s="20">
-        <f>IF(OR(D24="",$E$22=""),"",D24/$E$22)</f>
+        <f>IF(OR(D24="",$E$23=""),"",D24/$E$23)</f>
         <v/>
       </c>
       <c r="G24" s="9">
@@ -9333,14 +9333,14 @@
     <row r="25" ht="70" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>VA05</t>
+          <t>PV04</t>
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>2.52</v>
+        <v>2.95</v>
       </c>
       <c r="C25" s="9" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="D25" s="9">
         <f>IF(COUNT(B25,C25)&lt;2,"",B25*C25)</f>
@@ -9348,7 +9348,7 @@
       </c>
       <c r="E25" s="21" t="n"/>
       <c r="F25" s="20">
-        <f>IF(OR(D25="",$E$22=""),"",D25/$E$22)</f>
+        <f>IF(OR(D25="",$E$23=""),"",D25/$E$23)</f>
         <v/>
       </c>
       <c r="G25" s="9">
@@ -9383,26 +9383,48 @@
       </c>
     </row>
     <row r="26" ht="70" customHeight="1">
-      <c r="A26" s="10" t="n"/>
-      <c r="B26" s="9" t="n"/>
-      <c r="C26" s="9" t="n"/>
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>VA05</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="C26" s="9" t="n">
+        <v>1.4</v>
+      </c>
       <c r="D26" s="9">
         <f>IF(COUNT(B26,C26)&lt;2,"",B26*C26)</f>
         <v/>
       </c>
       <c r="E26" s="21" t="n"/>
       <c r="F26" s="20">
-        <f>IF(OR(D26="",$E$22=""),"",D26/$E$22)</f>
+        <f>IF(OR(D26="",$E$23=""),"",D26/$E$23)</f>
         <v/>
       </c>
       <c r="G26" s="9">
         <f>IF(A26="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H26" s="10" t="n"/>
-      <c r="I26" s="10" t="n"/>
-      <c r="J26" s="9" t="n"/>
-      <c r="K26" s="10" t="n"/>
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I26" s="10" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J26" s="9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K26" s="10" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
       <c r="L26" s="9">
         <f>IF(I26="","",IFERROR(VLOOKUP(I26,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
@@ -9413,128 +9435,106 @@
       </c>
     </row>
     <row r="27" ht="70" customHeight="1">
-      <c r="A27" s="14" t="n"/>
-      <c r="B27" s="13" t="n"/>
-      <c r="C27" s="13" t="n"/>
-      <c r="D27" s="13">
+      <c r="A27" s="10" t="n"/>
+      <c r="B27" s="9" t="n"/>
+      <c r="C27" s="9" t="n"/>
+      <c r="D27" s="9">
         <f>IF(COUNT(B27,C27)&lt;2,"",B27*C27)</f>
         <v/>
       </c>
-      <c r="E27" s="22" t="n"/>
-      <c r="F27" s="23">
-        <f>IF(OR(D27="",$E$22=""),"",D27/$E$22)</f>
-        <v/>
-      </c>
-      <c r="G27" s="13">
+      <c r="E27" s="21" t="n"/>
+      <c r="F27" s="20">
+        <f>IF(OR(D27="",$E$23=""),"",D27/$E$23)</f>
+        <v/>
+      </c>
+      <c r="G27" s="9">
         <f>IF(A27="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H27" s="14" t="n"/>
-      <c r="I27" s="14" t="n"/>
-      <c r="J27" s="13" t="n"/>
-      <c r="K27" s="14" t="n"/>
-      <c r="L27" s="13">
+      <c r="H27" s="10" t="n"/>
+      <c r="I27" s="10" t="n"/>
+      <c r="J27" s="9" t="n"/>
+      <c r="K27" s="10" t="n"/>
+      <c r="L27" s="9">
         <f>IF(I27="","",IFERROR(VLOOKUP(I27,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
-      <c r="M27" s="14">
+      <c r="M27" s="10">
         <f>IF(OR(D27="",J27=""),"",IF(J27&lt;=G27,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="28" ht="39.7" customHeight="1">
-      <c r="A28" s="5" t="inlineStr">
+    <row r="28" ht="70" customHeight="1">
+      <c r="A28" s="14" t="n"/>
+      <c r="B28" s="13" t="n"/>
+      <c r="C28" s="13" t="n"/>
+      <c r="D28" s="13">
+        <f>IF(COUNT(B28,C28)&lt;2,"",B28*C28)</f>
+        <v/>
+      </c>
+      <c r="E28" s="22" t="n"/>
+      <c r="F28" s="23">
+        <f>IF(OR(D28="",$E$23=""),"",D28/$E$23)</f>
+        <v/>
+      </c>
+      <c r="G28" s="13">
+        <f>IF(A28="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H28" s="14" t="n"/>
+      <c r="I28" s="14" t="n"/>
+      <c r="J28" s="13" t="n"/>
+      <c r="K28" s="14" t="n"/>
+      <c r="L28" s="13">
+        <f>IF(I28="","",IFERROR(VLOOKUP(I28,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M28" s="14">
+        <f>IF(OR(D28="",J28=""),"",IF(J28&lt;=G28,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="39.7" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>Plano: Fachada Noroeste</t>
         </is>
       </c>
-      <c r="B28" s="4" t="n"/>
-      <c r="C28" s="4" t="n"/>
-      <c r="D28" s="4" t="n"/>
-      <c r="E28" s="4" t="n"/>
-      <c r="F28" s="4" t="n"/>
-      <c r="G28" s="4" t="n"/>
-      <c r="H28" s="4" t="n"/>
-      <c r="I28" s="4" t="n"/>
-      <c r="J28" s="4" t="n"/>
-      <c r="K28" s="4" t="n"/>
-      <c r="L28" s="4" t="n"/>
-      <c r="M28" s="4" t="n"/>
-    </row>
-    <row r="29" ht="70" customHeight="1">
-      <c r="A29" s="10" t="inlineStr">
-        <is>
-          <t>PF03</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C29" s="9" t="n">
-        <v>2.88</v>
-      </c>
-      <c r="D29" s="9">
-        <f>IF(COUNT(B29,C29)&lt;2,"",B29*C29)</f>
-        <v/>
-      </c>
-      <c r="E29" s="19">
-        <f>SUM(D29:D36)</f>
-        <v/>
-      </c>
-      <c r="F29" s="20">
-        <f>IF(OR(D29="",$E$29=""),"",D29/$E$29)</f>
-        <v/>
-      </c>
-      <c r="G29" s="9">
-        <f>IF(A29="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H29" s="10" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I29" s="10" t="inlineStr">
-        <is>
-          <t>Sin Proteccion</t>
-        </is>
-      </c>
-      <c r="J29" s="9" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K29" s="10" t="inlineStr">
-        <is>
-          <t>Noroeste</t>
-        </is>
-      </c>
-      <c r="L29" s="9">
-        <f>IF(I29="","",IFERROR(VLOOKUP(I29,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M29" s="10">
-        <f>IF(OR(D29="",J29=""),"",IF(J29&lt;=G29,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
+      <c r="B29" s="4" t="n"/>
+      <c r="C29" s="4" t="n"/>
+      <c r="D29" s="4" t="n"/>
+      <c r="E29" s="4" t="n"/>
+      <c r="F29" s="4" t="n"/>
+      <c r="G29" s="4" t="n"/>
+      <c r="H29" s="4" t="n"/>
+      <c r="I29" s="4" t="n"/>
+      <c r="J29" s="4" t="n"/>
+      <c r="K29" s="4" t="n"/>
+      <c r="L29" s="4" t="n"/>
+      <c r="M29" s="4" t="n"/>
     </row>
     <row r="30" ht="70" customHeight="1">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>PF01</t>
+          <t>PF03</t>
         </is>
       </c>
       <c r="B30" s="9" t="n">
         <v>3</v>
       </c>
       <c r="C30" s="9" t="n">
-        <v>3.55</v>
+        <v>2.88</v>
       </c>
       <c r="D30" s="9">
         <f>IF(COUNT(B30,C30)&lt;2,"",B30*C30)</f>
         <v/>
       </c>
-      <c r="E30" s="21" t="n"/>
+      <c r="E30" s="19">
+        <f>SUM(D30:D37)</f>
+        <v/>
+      </c>
       <c r="F30" s="20">
-        <f>IF(OR(D30="",$E$29=""),"",D30/$E$29)</f>
+        <f>IF(OR(D30="",$E$30=""),"",D30/$E$30)</f>
         <v/>
       </c>
       <c r="G30" s="9">
@@ -9571,14 +9571,14 @@
     <row r="31" ht="70" customHeight="1">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>PV01</t>
+          <t>PF01</t>
         </is>
       </c>
       <c r="B31" s="9" t="n">
         <v>3</v>
       </c>
       <c r="C31" s="9" t="n">
-        <v>7.7</v>
+        <v>3.55</v>
       </c>
       <c r="D31" s="9">
         <f>IF(COUNT(B31,C31)&lt;2,"",B31*C31)</f>
@@ -9586,7 +9586,7 @@
       </c>
       <c r="E31" s="21" t="n"/>
       <c r="F31" s="20">
-        <f>IF(OR(D31="",$E$29=""),"",D31/$E$29)</f>
+        <f>IF(OR(D31="",$E$30=""),"",D31/$E$30)</f>
         <v/>
       </c>
       <c r="G31" s="9">
@@ -9623,14 +9623,14 @@
     <row r="32" ht="70" customHeight="1">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>PV02</t>
+          <t>PV01</t>
         </is>
       </c>
       <c r="B32" s="9" t="n">
         <v>3</v>
       </c>
       <c r="C32" s="9" t="n">
-        <v>2.48</v>
+        <v>7.7</v>
       </c>
       <c r="D32" s="9">
         <f>IF(COUNT(B32,C32)&lt;2,"",B32*C32)</f>
@@ -9638,7 +9638,7 @@
       </c>
       <c r="E32" s="21" t="n"/>
       <c r="F32" s="20">
-        <f>IF(OR(D32="",$E$29=""),"",D32/$E$29)</f>
+        <f>IF(OR(D32="",$E$30=""),"",D32/$E$30)</f>
         <v/>
       </c>
       <c r="G32" s="9">
@@ -9675,14 +9675,14 @@
     <row r="33" ht="70" customHeight="1">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>VA04</t>
+          <t>PV02</t>
         </is>
       </c>
       <c r="B33" s="9" t="n">
-        <v>2.52</v>
+        <v>3</v>
       </c>
       <c r="C33" s="9" t="n">
-        <v>2</v>
+        <v>2.48</v>
       </c>
       <c r="D33" s="9">
         <f>IF(COUNT(B33,C33)&lt;2,"",B33*C33)</f>
@@ -9690,7 +9690,7 @@
       </c>
       <c r="E33" s="21" t="n"/>
       <c r="F33" s="20">
-        <f>IF(OR(D33="",$E$29=""),"",D33/$E$29)</f>
+        <f>IF(OR(D33="",$E$30=""),"",D33/$E$30)</f>
         <v/>
       </c>
       <c r="G33" s="9">
@@ -9742,7 +9742,7 @@
       </c>
       <c r="E34" s="21" t="n"/>
       <c r="F34" s="20">
-        <f>IF(OR(D34="",$E$29=""),"",D34/$E$29)</f>
+        <f>IF(OR(D34="",$E$30=""),"",D34/$E$30)</f>
         <v/>
       </c>
       <c r="G34" s="9">
@@ -9777,26 +9777,48 @@
       </c>
     </row>
     <row r="35" ht="70" customHeight="1">
-      <c r="A35" s="10" t="n"/>
-      <c r="B35" s="9" t="n"/>
-      <c r="C35" s="9" t="n"/>
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>VA04</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="C35" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="D35" s="9">
         <f>IF(COUNT(B35,C35)&lt;2,"",B35*C35)</f>
         <v/>
       </c>
       <c r="E35" s="21" t="n"/>
       <c r="F35" s="20">
-        <f>IF(OR(D35="",$E$29=""),"",D35/$E$29)</f>
+        <f>IF(OR(D35="",$E$30=""),"",D35/$E$30)</f>
         <v/>
       </c>
       <c r="G35" s="9">
         <f>IF(A35="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H35" s="10" t="n"/>
-      <c r="I35" s="10" t="n"/>
-      <c r="J35" s="9" t="n"/>
-      <c r="K35" s="10" t="n"/>
+      <c r="H35" s="10" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I35" s="10" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J35" s="9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K35" s="10" t="inlineStr">
+        <is>
+          <t>Noroeste</t>
+        </is>
+      </c>
       <c r="L35" s="9">
         <f>IF(I35="","",IFERROR(VLOOKUP(I35,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
@@ -9807,169 +9829,126 @@
       </c>
     </row>
     <row r="36" ht="70" customHeight="1">
-      <c r="A36" s="14" t="n"/>
-      <c r="B36" s="13" t="n"/>
-      <c r="C36" s="13" t="n"/>
-      <c r="D36" s="13">
+      <c r="A36" s="10" t="n"/>
+      <c r="B36" s="9" t="n"/>
+      <c r="C36" s="9" t="n"/>
+      <c r="D36" s="9">
         <f>IF(COUNT(B36,C36)&lt;2,"",B36*C36)</f>
         <v/>
       </c>
-      <c r="E36" s="22" t="n"/>
-      <c r="F36" s="23">
-        <f>IF(OR(D36="",$E$29=""),"",D36/$E$29)</f>
-        <v/>
-      </c>
-      <c r="G36" s="13">
+      <c r="E36" s="21" t="n"/>
+      <c r="F36" s="20">
+        <f>IF(OR(D36="",$E$30=""),"",D36/$E$30)</f>
+        <v/>
+      </c>
+      <c r="G36" s="9">
         <f>IF(A36="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H36" s="14" t="n"/>
-      <c r="I36" s="14" t="n"/>
-      <c r="J36" s="13" t="n"/>
-      <c r="K36" s="14" t="n"/>
-      <c r="L36" s="13">
+      <c r="H36" s="10" t="n"/>
+      <c r="I36" s="10" t="n"/>
+      <c r="J36" s="9" t="n"/>
+      <c r="K36" s="10" t="n"/>
+      <c r="L36" s="9">
         <f>IF(I36="","",IFERROR(VLOOKUP(I36,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
-      <c r="M36" s="14">
+      <c r="M36" s="10">
         <f>IF(OR(D36="",J36=""),"",IF(J36&lt;=G36,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="37" ht="39.7" customHeight="1">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>Plano: Orientacion a confirmar</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="n"/>
-      <c r="C37" s="4" t="n"/>
-      <c r="D37" s="4" t="n"/>
-      <c r="E37" s="4" t="n"/>
-      <c r="F37" s="4" t="n"/>
-      <c r="G37" s="4" t="n"/>
-      <c r="H37" s="4" t="n"/>
-      <c r="I37" s="4" t="n"/>
-      <c r="J37" s="4" t="n"/>
-      <c r="K37" s="4" t="n"/>
-      <c r="L37" s="4" t="n"/>
-      <c r="M37" s="4" t="n"/>
-    </row>
-    <row r="38" ht="70" customHeight="1">
-      <c r="A38" s="10" t="inlineStr">
-        <is>
-          <t>VA01</t>
-        </is>
-      </c>
-      <c r="B38" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C38" s="9" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D38" s="9">
-        <f>IF(COUNT(B38,C38)&lt;2,"",B38*C38)</f>
-        <v/>
-      </c>
-      <c r="E38" s="19">
-        <f>SUM(D38:D40)</f>
-        <v/>
-      </c>
-      <c r="F38" s="20">
-        <f>IF(OR(D38="",$E$38=""),"",D38/$E$38)</f>
-        <v/>
-      </c>
-      <c r="G38" s="9">
-        <f>IF(A38="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H38" s="10" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I38" s="10" t="inlineStr">
-        <is>
-          <t>Sin Proteccion</t>
-        </is>
-      </c>
-      <c r="J38" s="9" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K38" s="10" t="n"/>
-      <c r="L38" s="9">
-        <f>IF(I38="","",IFERROR(VLOOKUP(I38,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M38" s="10">
-        <f>IF(OR(D38="",J38=""),"",IF(J38&lt;=G38,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39" ht="70" customHeight="1">
-      <c r="A39" s="10" t="n"/>
-      <c r="B39" s="9" t="n"/>
-      <c r="C39" s="9" t="n"/>
-      <c r="D39" s="9">
-        <f>IF(COUNT(B39,C39)&lt;2,"",B39*C39)</f>
-        <v/>
-      </c>
-      <c r="E39" s="21" t="n"/>
-      <c r="F39" s="20">
-        <f>IF(OR(D39="",$E$38=""),"",D39/$E$38)</f>
-        <v/>
-      </c>
-      <c r="G39" s="9">
-        <f>IF(A39="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H39" s="10" t="n"/>
-      <c r="I39" s="10" t="n"/>
-      <c r="J39" s="9" t="n"/>
-      <c r="K39" s="10" t="n"/>
-      <c r="L39" s="9">
-        <f>IF(I39="","",IFERROR(VLOOKUP(I39,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M39" s="10">
-        <f>IF(OR(D39="",J39=""),"",IF(J39&lt;=G39,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" ht="70" customHeight="1">
-      <c r="A40" s="14" t="n"/>
-      <c r="B40" s="13" t="n"/>
-      <c r="C40" s="13" t="n"/>
-      <c r="D40" s="13">
-        <f>IF(COUNT(B40,C40)&lt;2,"",B40*C40)</f>
-        <v/>
-      </c>
-      <c r="E40" s="22" t="n"/>
-      <c r="F40" s="23">
-        <f>IF(OR(D40="",$E$38=""),"",D40/$E$38)</f>
-        <v/>
-      </c>
-      <c r="G40" s="13">
-        <f>IF(A40="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H40" s="14" t="n"/>
-      <c r="I40" s="14" t="n"/>
-      <c r="J40" s="13" t="n"/>
-      <c r="K40" s="14" t="n"/>
-      <c r="L40" s="13">
-        <f>IF(I40="","",IFERROR(VLOOKUP(I40,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M40" s="14">
-        <f>IF(OR(D40="",J40=""),"",IF(J40&lt;=G40,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="16" t="inlineStr">
+    <row r="37" ht="70" customHeight="1">
+      <c r="A37" s="14" t="n"/>
+      <c r="B37" s="13" t="n"/>
+      <c r="C37" s="13" t="n"/>
+      <c r="D37" s="13">
+        <f>IF(COUNT(B37,C37)&lt;2,"",B37*C37)</f>
+        <v/>
+      </c>
+      <c r="E37" s="22" t="n"/>
+      <c r="F37" s="23">
+        <f>IF(OR(D37="",$E$30=""),"",D37/$E$30)</f>
+        <v/>
+      </c>
+      <c r="G37" s="13">
+        <f>IF(A37="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H37" s="14" t="n"/>
+      <c r="I37" s="14" t="n"/>
+      <c r="J37" s="13" t="n"/>
+      <c r="K37" s="14" t="n"/>
+      <c r="L37" s="13">
+        <f>IF(I37="","",IFERROR(VLOOKUP(I37,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M37" s="14">
+        <f>IF(OR(D37="",J37=""),"",IF(J37&lt;=G37,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
         <is>
           <t>HOJA REHECHA: las orientaciones se tomaron del plano de fachadas y cambiaron casi todas. Hay que reemplazar la planilla entera, no alcanza con retocar celdas.</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+      <c r="G38" s="2" t="n"/>
+      <c r="H38" s="2" t="n"/>
+      <c r="I38" s="2" t="n"/>
+      <c r="J38" s="2" t="n"/>
+      <c r="K38" s="2" t="n"/>
+      <c r="L38" s="2" t="n"/>
+      <c r="M38" s="2" t="n"/>
+    </row>
+    <row r="39" ht="39.7" customHeight="1">
+      <c r="A39" s="24" t="inlineStr">
+        <is>
+          <t>COMO SE COMPLETA</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="n"/>
+      <c r="H39" s="2" t="n"/>
+      <c r="I39" s="2" t="n"/>
+      <c r="J39" s="2" t="n"/>
+      <c r="K39" s="2" t="n"/>
+      <c r="L39" s="2" t="n"/>
+      <c r="M39" s="2" t="n"/>
+    </row>
+    <row r="40" ht="39.7" customHeight="1">
+      <c r="A40" s="25" t="inlineStr">
+        <is>
+          <t>Descripcion, altura y ancho del vano: de la planilla de carpinterias.</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2" t="n"/>
+      <c r="H40" s="2" t="n"/>
+      <c r="I40" s="2" t="n"/>
+      <c r="J40" s="2" t="n"/>
+      <c r="K40" s="2" t="n"/>
+      <c r="L40" s="2" t="n"/>
+      <c r="M40" s="2" t="n"/>
+    </row>
+    <row r="41" ht="39.7" customHeight="1">
+      <c r="A41" s="25" t="inlineStr">
+        <is>
+          <t>Area del vano, area total por plano y porcentaje: se calculan solos.</t>
         </is>
       </c>
       <c r="B41" s="2" t="n"/>
@@ -9986,9 +9965,9 @@
       <c r="M41" s="2" t="n"/>
     </row>
     <row r="42" ht="39.7" customHeight="1">
-      <c r="A42" s="24" t="inlineStr">
-        <is>
-          <t>COMO SE COMPLETA</t>
+      <c r="A42" s="25" t="inlineStr">
+        <is>
+          <t>Tipo de vidrio y tipo de proteccion: desplegables; sus valores estan en la hoja Datos_higro.</t>
         </is>
       </c>
       <c r="B42" s="2" t="n"/>
@@ -10007,7 +9986,7 @@
     <row r="43" ht="39.7" customHeight="1">
       <c r="A43" s="25" t="inlineStr">
         <is>
-          <t>Descripcion, altura y ancho del vano: de la planilla de carpinterias.</t>
+          <t>Transmitancia del cerramiento: cargarla segun el vidrio y el marco adoptados.</t>
         </is>
       </c>
       <c r="B43" s="2" t="n"/>
@@ -10026,7 +10005,7 @@
     <row r="44" ht="39.7" customHeight="1">
       <c r="A44" s="25" t="inlineStr">
         <is>
-          <t>Area del vano, area total por plano y porcentaje: se calculan solos.</t>
+          <t>PROTECCION: la obra tiene cortinas blackout INTERIORES, y los panos fijos PF no tienen nada.</t>
         </is>
       </c>
       <c r="B44" s="2" t="n"/>
@@ -10045,7 +10024,7 @@
     <row r="45" ht="39.7" customHeight="1">
       <c r="A45" s="25" t="inlineStr">
         <is>
-          <t>Tipo de vidrio y tipo de proteccion: desplegables; sus valores estan en la hoja Datos_higro.</t>
+          <t>Una cortina interior NO computa como proteccion solar: la radiacion ya atraveso el vidrio</t>
         </is>
       </c>
       <c r="B45" s="2" t="n"/>
@@ -10064,7 +10043,7 @@
     <row r="46" ht="39.7" customHeight="1">
       <c r="A46" s="25" t="inlineStr">
         <is>
-          <t>Transmitancia del cerramiento: cargarla segun el vidrio y el marco adoptados.</t>
+          <t>cuando llega a la cortina. La ordenanza acredita protecciones exteriores (aleros, parasoles,</t>
         </is>
       </c>
       <c r="B46" s="2" t="n"/>
@@ -10083,7 +10062,7 @@
     <row r="47" ht="39.7" customHeight="1">
       <c r="A47" s="25" t="inlineStr">
         <is>
-          <t>PROTECCION: la obra tiene cortinas blackout INTERIORES, y los panos fijos PF no tienen nada.</t>
+          <t>cortinas de enrollar exteriores, toldos). Por eso las veinte aberturas van Sin Proteccion.</t>
         </is>
       </c>
       <c r="B47" s="2" t="n"/>
@@ -10099,12 +10078,8 @@
       <c r="L47" s="2" t="n"/>
       <c r="M47" s="2" t="n"/>
     </row>
-    <row r="48" ht="39.7" customHeight="1">
-      <c r="A48" s="25" t="inlineStr">
-        <is>
-          <t>Una cortina interior NO computa como proteccion solar: la radiacion ya atraveso el vidrio</t>
-        </is>
-      </c>
+    <row r="48">
+      <c r="A48" s="25" t="inlineStr"/>
       <c r="B48" s="2" t="n"/>
       <c r="C48" s="2" t="n"/>
       <c r="D48" s="2" t="n"/>
@@ -10121,7 +10096,7 @@
     <row r="49" ht="39.7" customHeight="1">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>cuando llega a la cortina. La ordenanza acredita protecciones exteriores (aleros, parasoles,</t>
+          <t>CONSECUENCIA: el factor de exposicion solar da 0,88 esta muy por encima del maximo de 0,30 que la ordenanza admite para</t>
         </is>
       </c>
       <c r="B49" s="2" t="n"/>
@@ -10140,7 +10115,7 @@
     <row r="50" ht="39.7" customHeight="1">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>cortinas de enrollar exteriores, toldos). Por eso las veinte aberturas van Sin Proteccion.</t>
+          <t>el cuadrante Este/Oeste, donde caen las cuatro fachadas de esta casa por estar girada 45</t>
         </is>
       </c>
       <c r="B50" s="2" t="n"/>
@@ -10156,8 +10131,12 @@
       <c r="L50" s="2" t="n"/>
       <c r="M50" s="2" t="n"/>
     </row>
-    <row r="51">
-      <c r="A51" s="25" t="inlineStr"/>
+    <row r="51" ht="39.7" customHeight="1">
+      <c r="A51" s="25" t="inlineStr">
+        <is>
+          <t>grados. La verificacion de la planilla no lo controla, igual que la de la catedra, pero si lo</t>
+        </is>
+      </c>
       <c r="B51" s="2" t="n"/>
       <c r="C51" s="2" t="n"/>
       <c r="D51" s="2" t="n"/>
@@ -10174,7 +10153,7 @@
     <row r="52" ht="39.7" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>CONSECUENCIA: el factor de exposicion solar da 0,88 esta muy por encima del maximo de 0,30 que la ordenanza admite para</t>
+          <t>presentas en el municipio esas cinco aberturas no pasarian el factor de exposicion solar.</t>
         </is>
       </c>
       <c r="B52" s="2" t="n"/>
@@ -10193,7 +10172,7 @@
     <row r="53" ht="39.7" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>el cuadrante Este/Oeste, donde caen las cuatro fachadas de esta casa por estar girada 45</t>
+          <t>Hay dos salidas posibles: (a) si la abertura ocupa menos del 20% del lado expuesto del local,</t>
         </is>
       </c>
       <c r="B53" s="2" t="n"/>
@@ -10212,7 +10191,7 @@
     <row r="54" ht="39.7" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>grados. La verificacion de la planilla no lo controla, igual que la de la catedra, pero si lo</t>
+          <t>no se verifica el FES; (b) cambiar el vidrio por uno de control solar, que baja el FES sin</t>
         </is>
       </c>
       <c r="B54" s="2" t="n"/>
@@ -10231,7 +10210,7 @@
     <row r="55" ht="39.7" customHeight="1">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>presentas en el municipio esas cinco aberturas no pasarian el factor de exposicion solar.</t>
+          <t>tocar la obra. Agregar una proteccion exterior seria la tercera, pero implica obra.</t>
         </is>
       </c>
       <c r="B55" s="2" t="n"/>
@@ -10247,12 +10226,8 @@
       <c r="L55" s="2" t="n"/>
       <c r="M55" s="2" t="n"/>
     </row>
-    <row r="56" ht="39.7" customHeight="1">
-      <c r="A56" s="25" t="inlineStr">
-        <is>
-          <t>Hay dos salidas posibles: (a) si la abertura ocupa menos del 20% del lado expuesto del local,</t>
-        </is>
-      </c>
+    <row r="56">
+      <c r="A56" s="25" t="inlineStr"/>
       <c r="B56" s="2" t="n"/>
       <c r="C56" s="2" t="n"/>
       <c r="D56" s="2" t="n"/>
@@ -10269,7 +10244,7 @@
     <row r="57" ht="39.7" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>no se verifica el FES; (b) cambiar el vidrio por uno de control solar, que baja el FES sin</t>
+          <t>Orientacion: ya cargada. Factor de exposicion solar: se completa SOLO al elegir el tipo de</t>
         </is>
       </c>
       <c r="B57" s="2" t="n"/>
@@ -10288,7 +10263,7 @@
     <row r="58" ht="39.7" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>tocar la obra. Agregar una proteccion exterior seria la tercera, pero implica obra.</t>
+          <t>proteccion, con los valores de la tabla de Datos_higro (Sin Proteccion 0,88; Parasol</t>
         </is>
       </c>
       <c r="B58" s="2" t="n"/>
@@ -10304,8 +10279,12 @@
       <c r="L58" s="2" t="n"/>
       <c r="M58" s="2" t="n"/>
     </row>
-    <row r="59">
-      <c r="A59" s="25" t="inlineStr"/>
+    <row r="59" ht="39.7" customHeight="1">
+      <c r="A59" s="25" t="inlineStr">
+        <is>
+          <t>horizontal fijo 1:2 0,35), que son los mismos de la planilla de la catedra.</t>
+        </is>
+      </c>
       <c r="B59" s="2" t="n"/>
       <c r="C59" s="2" t="n"/>
       <c r="D59" s="2" t="n"/>
@@ -10322,7 +10301,7 @@
     <row r="60" ht="39.7" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>Orientacion: ya cargada. Factor de exposicion solar: se completa SOLO al elegir el tipo de</t>
+          <t>En Datos_higro esta ademas el FES maximo admitido por cuadrante segun la ordenanza, como</t>
         </is>
       </c>
       <c r="B60" s="2" t="n"/>
@@ -10341,7 +10320,7 @@
     <row r="61" ht="39.7" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>proteccion, con los valores de la tabla de Datos_higro (Sin Proteccion 0,88; Parasol</t>
+          <t>referencia: la verificacion no lo controla, igual que en la planilla de la catedra.</t>
         </is>
       </c>
       <c r="B61" s="2" t="n"/>
@@ -10357,12 +10336,8 @@
       <c r="L61" s="2" t="n"/>
       <c r="M61" s="2" t="n"/>
     </row>
-    <row r="62" ht="39.7" customHeight="1">
-      <c r="A62" s="25" t="inlineStr">
-        <is>
-          <t>horizontal fijo 1:2 0,35), que son los mismos de la planilla de la catedra.</t>
-        </is>
-      </c>
+    <row r="62">
+      <c r="A62" s="25" t="inlineStr"/>
       <c r="B62" s="2" t="n"/>
       <c r="C62" s="2" t="n"/>
       <c r="D62" s="2" t="n"/>
@@ -10379,7 +10354,7 @@
     <row r="63" ht="39.7" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>En Datos_higro esta ademas el FES maximo admitido por cuadrante segun la ordenanza, como</t>
+          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
         </is>
       </c>
       <c r="B63" s="2" t="n"/>
@@ -10398,7 +10373,7 @@
     <row r="64" ht="39.7" customHeight="1">
       <c r="A64" s="25" t="inlineStr">
         <is>
-          <t>referencia: la verificacion no lo controla, igual que en la planilla de la catedra.</t>
+          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
         </is>
       </c>
       <c r="B64" s="2" t="n"/>
@@ -10432,7 +10407,7 @@
     <row r="66" ht="39.7" customHeight="1">
       <c r="A66" s="25" t="inlineStr">
         <is>
-          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
+          <t>ALTURAS: medidas sobre el dibujo de las vistas de la planilla de carpinterias, con la escala</t>
         </is>
       </c>
       <c r="B66" s="2" t="n"/>
@@ -10451,7 +10426,7 @@
     <row r="67" ht="39.7" customHeight="1">
       <c r="A67" s="25" t="inlineStr">
         <is>
-          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
+          <t>verificada contra los anchos acotados (error menor a 2 cm). La mayoria de las aberturas son de</t>
         </is>
       </c>
       <c r="B67" s="2" t="n"/>
@@ -10467,8 +10442,12 @@
       <c r="L67" s="2" t="n"/>
       <c r="M67" s="2" t="n"/>
     </row>
-    <row r="68">
-      <c r="A68" s="25" t="inlineStr"/>
+    <row r="68" ht="39.7" customHeight="1">
+      <c r="A68" s="25" t="inlineStr">
+        <is>
+          <t>piso a cielorraso, 3,00 m. VERIFICARLAS contra el plano antes de presentar.</t>
+        </is>
+      </c>
       <c r="B68" s="2" t="n"/>
       <c r="C68" s="2" t="n"/>
       <c r="D68" s="2" t="n"/>
@@ -10485,7 +10464,7 @@
     <row r="69" ht="39.7" customHeight="1">
       <c r="A69" s="25" t="inlineStr">
         <is>
-          <t>ALTURAS: medidas sobre el dibujo de las vistas de la planilla de carpinterias, con la escala</t>
+          <t>PF04 es la unica con antepecho: arranca a 1,09 y mide 0,60 de alto. El resto llega al piso.</t>
         </is>
       </c>
       <c r="B69" s="2" t="n"/>
@@ -10504,7 +10483,7 @@
     <row r="70" ht="39.7" customHeight="1">
       <c r="A70" s="25" t="inlineStr">
         <is>
-          <t>verificada contra los anchos acotados (error menor a 2 cm). La mayoria de las aberturas son de</t>
+          <t>Las alturas de PV01 (3,00), PF04 (0,60) y PV04 (2) (2,95) las aporto el autor del proyecto.</t>
         </is>
       </c>
       <c r="B70" s="2" t="n"/>
@@ -10520,12 +10499,8 @@
       <c r="L70" s="2" t="n"/>
       <c r="M70" s="2" t="n"/>
     </row>
-    <row r="71" ht="39.7" customHeight="1">
-      <c r="A71" s="25" t="inlineStr">
-        <is>
-          <t>piso a cielorraso, 3,00 m. VERIFICARLAS contra el plano antes de presentar.</t>
-        </is>
-      </c>
+    <row r="71">
+      <c r="A71" s="25" t="inlineStr"/>
       <c r="B71" s="2" t="n"/>
       <c r="C71" s="2" t="n"/>
       <c r="D71" s="2" t="n"/>
@@ -10542,7 +10517,7 @@
     <row r="72" ht="39.7" customHeight="1">
       <c r="A72" s="25" t="inlineStr">
         <is>
-          <t>PF04 es la unica con antepecho: arranca a 1,09 y mide 0,60 de alto. El resto llega al piso.</t>
+          <t>ORIENTACION: el simbolo de norte del plano (circulo con aguja, en el patio interno) apunta a</t>
         </is>
       </c>
       <c r="B72" s="2" t="n"/>
@@ -10561,7 +10536,7 @@
     <row r="73" ht="39.7" customHeight="1">
       <c r="A73" s="25" t="inlineStr">
         <is>
-          <t>Las alturas de PV01 (3,00), PF04 (0,60) y PV04 (2) (2,95) las aporto el autor del proyecto.</t>
+          <t>45 grados hacia arriba y a la derecha de la hoja. Entonces las cuatro fachadas NO son N-S-E-O</t>
         </is>
       </c>
       <c r="B73" s="2" t="n"/>
@@ -10577,8 +10552,12 @@
       <c r="L73" s="2" t="n"/>
       <c r="M73" s="2" t="n"/>
     </row>
-    <row r="74">
-      <c r="A74" s="25" t="inlineStr"/>
+    <row r="74" ht="39.7" customHeight="1">
+      <c r="A74" s="25" t="inlineStr">
+        <is>
+          <t>sino: arriba = Noroeste, derecha = Noreste, abajo = Sudeste, izquierda = Sudoeste.</t>
+        </is>
+      </c>
       <c r="B74" s="2" t="n"/>
       <c r="C74" s="2" t="n"/>
       <c r="D74" s="2" t="n"/>
@@ -10595,7 +10574,7 @@
     <row r="75" ht="39.7" customHeight="1">
       <c r="A75" s="25" t="inlineStr">
         <is>
-          <t>ORIENTACION: el simbolo de norte del plano (circulo con aguja, en el patio interno) apunta a</t>
+          <t>Cada abertura se asigno a la fachada por su posicion en planta. Las del patio interno se</t>
         </is>
       </c>
       <c r="B75" s="2" t="n"/>
@@ -10614,7 +10593,7 @@
     <row r="76" ht="39.7" customHeight="1">
       <c r="A76" s="25" t="inlineStr">
         <is>
-          <t>45 grados hacia arriba y a la derecha de la hoja. Entonces las cuatro fachadas NO son N-S-E-O</t>
+          <t>orientan por la pared en la que estan: miran hacia adentro del patio.</t>
         </is>
       </c>
       <c r="B76" s="2" t="n"/>
@@ -10633,7 +10612,7 @@
     <row r="77" ht="39.7" customHeight="1">
       <c r="A77" s="25" t="inlineStr">
         <is>
-          <t>sino: arriba = Noroeste, derecha = Noreste, abajo = Sudeste, izquierda = Sudoeste.</t>
+          <t>Los rotulos Dormitorio Norte y Dormitorio Sur del plano no coinciden con el norte real;</t>
         </is>
       </c>
       <c r="B77" s="2" t="n"/>
@@ -10652,7 +10631,7 @@
     <row r="78" ht="39.7" customHeight="1">
       <c r="A78" s="25" t="inlineStr">
         <is>
-          <t>Cada abertura se asigno a la fachada por su posicion en planta. Las del patio interno se</t>
+          <t>parecen ser nombres de uso, no orientaciones.</t>
         </is>
       </c>
       <c r="B78" s="2" t="n"/>
@@ -10668,12 +10647,8 @@
       <c r="L78" s="2" t="n"/>
       <c r="M78" s="2" t="n"/>
     </row>
-    <row r="79" ht="39.7" customHeight="1">
-      <c r="A79" s="25" t="inlineStr">
-        <is>
-          <t>orientan por la pared en la que estan: miran hacia adentro del patio.</t>
-        </is>
-      </c>
+    <row r="79">
+      <c r="A79" s="25" t="inlineStr"/>
       <c r="B79" s="2" t="n"/>
       <c r="C79" s="2" t="n"/>
       <c r="D79" s="2" t="n"/>
@@ -10690,7 +10665,7 @@
     <row r="80" ht="39.7" customHeight="1">
       <c r="A80" s="25" t="inlineStr">
         <is>
-          <t>Los rotulos Dormitorio Norte y Dormitorio Sur del plano no coinciden con el norte real;</t>
+          <t>CANTIDADES: la planilla de carpinterias trae la cantidad de cada abertura. Tres van dos veces:</t>
         </is>
       </c>
       <c r="B80" s="2" t="n"/>
@@ -10709,7 +10684,7 @@
     <row r="81" ht="39.7" customHeight="1">
       <c r="A81" s="25" t="inlineStr">
         <is>
-          <t>parecen ser nombres de uso, no orientaciones.</t>
+          <t>VA01 (01 Cocina y 09 Suite), VA04 (13 Dormitorio Norte y 14 Play Room) y PF01 (03 Lavadero y</t>
         </is>
       </c>
       <c r="B81" s="2" t="n"/>
@@ -10725,8 +10700,12 @@
       <c r="L81" s="2" t="n"/>
       <c r="M81" s="2" t="n"/>
     </row>
-    <row r="82">
-      <c r="A82" s="25" t="inlineStr"/>
+    <row r="82" ht="39.7" customHeight="1">
+      <c r="A82" s="25" t="inlineStr">
+        <is>
+          <t>07 Hall de ingreso, a los dos lados del patio interno). Por eso la planilla tiene 20 filas y</t>
+        </is>
+      </c>
       <c r="B82" s="2" t="n"/>
       <c r="C82" s="2" t="n"/>
       <c r="D82" s="2" t="n"/>
@@ -10743,7 +10722,7 @@
     <row r="83" ht="39.7" customHeight="1">
       <c r="A83" s="25" t="inlineStr">
         <is>
-          <t>CANTIDADES: la planilla de carpinterias trae la cantidad de cada abertura. Tres van dos veces:</t>
+          <t>no 17. Las demas aberturas son de una sola unidad.</t>
         </is>
       </c>
       <c r="B83" s="2" t="n"/>
@@ -10759,12 +10738,8 @@
       <c r="L83" s="2" t="n"/>
       <c r="M83" s="2" t="n"/>
     </row>
-    <row r="84" ht="39.7" customHeight="1">
-      <c r="A84" s="25" t="inlineStr">
-        <is>
-          <t>VA01 (01 Cocina y 09 Suite), VA04 (13 Dormitorio Norte y 14 Play Room) y PF01 (03 Lavadero y</t>
-        </is>
-      </c>
+    <row r="84">
+      <c r="A84" s="25" t="inlineStr"/>
       <c r="B84" s="2" t="n"/>
       <c r="C84" s="2" t="n"/>
       <c r="D84" s="2" t="n"/>
@@ -10781,7 +10756,7 @@
     <row r="85" ht="39.7" customHeight="1">
       <c r="A85" s="25" t="inlineStr">
         <is>
-          <t>07 Hall de ingreso, a los dos lados del patio interno). Por eso la planilla tiene 20 filas y</t>
+          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
         </is>
       </c>
       <c r="B85" s="2" t="n"/>
@@ -10797,12 +10772,8 @@
       <c r="L85" s="2" t="n"/>
       <c r="M85" s="2" t="n"/>
     </row>
-    <row r="86" ht="39.7" customHeight="1">
-      <c r="A86" s="25" t="inlineStr">
-        <is>
-          <t>no 17. Las demas aberturas son de una sola unidad.</t>
-        </is>
-      </c>
+    <row r="86">
+      <c r="A86" s="25" t="inlineStr"/>
       <c r="B86" s="2" t="n"/>
       <c r="C86" s="2" t="n"/>
       <c r="D86" s="2" t="n"/>
@@ -10816,8 +10787,12 @@
       <c r="L86" s="2" t="n"/>
       <c r="M86" s="2" t="n"/>
     </row>
-    <row r="87">
-      <c r="A87" s="25" t="inlineStr"/>
+    <row r="87" ht="39.7" customHeight="1">
+      <c r="A87" s="25" t="inlineStr">
+        <is>
+          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
+        </is>
+      </c>
       <c r="B87" s="2" t="n"/>
       <c r="C87" s="2" t="n"/>
       <c r="D87" s="2" t="n"/>
@@ -10834,7 +10809,7 @@
     <row r="88" ht="39.7" customHeight="1">
       <c r="A88" s="25" t="inlineStr">
         <is>
-          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
+          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
         </is>
       </c>
       <c r="B88" s="2" t="n"/>
@@ -10850,8 +10825,12 @@
       <c r="L88" s="2" t="n"/>
       <c r="M88" s="2" t="n"/>
     </row>
-    <row r="89">
-      <c r="A89" s="25" t="inlineStr"/>
+    <row r="89" ht="39.7" customHeight="1">
+      <c r="A89" s="25" t="inlineStr">
+        <is>
+          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
+        </is>
+      </c>
       <c r="B89" s="2" t="n"/>
       <c r="C89" s="2" t="n"/>
       <c r="D89" s="2" t="n"/>
@@ -10865,83 +10844,24 @@
       <c r="L89" s="2" t="n"/>
       <c r="M89" s="2" t="n"/>
     </row>
-    <row r="90" ht="39.7" customHeight="1">
-      <c r="A90" s="25" t="inlineStr">
-        <is>
-          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
-        </is>
-      </c>
-      <c r="B90" s="2" t="n"/>
-      <c r="C90" s="2" t="n"/>
-      <c r="D90" s="2" t="n"/>
-      <c r="E90" s="2" t="n"/>
-      <c r="F90" s="2" t="n"/>
-      <c r="G90" s="2" t="n"/>
-      <c r="H90" s="2" t="n"/>
-      <c r="I90" s="2" t="n"/>
-      <c r="J90" s="2" t="n"/>
-      <c r="K90" s="2" t="n"/>
-      <c r="L90" s="2" t="n"/>
-      <c r="M90" s="2" t="n"/>
-    </row>
-    <row r="91" ht="39.7" customHeight="1">
-      <c r="A91" s="25" t="inlineStr">
-        <is>
-          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
-        </is>
-      </c>
-      <c r="B91" s="2" t="n"/>
-      <c r="C91" s="2" t="n"/>
-      <c r="D91" s="2" t="n"/>
-      <c r="E91" s="2" t="n"/>
-      <c r="F91" s="2" t="n"/>
-      <c r="G91" s="2" t="n"/>
-      <c r="H91" s="2" t="n"/>
-      <c r="I91" s="2" t="n"/>
-      <c r="J91" s="2" t="n"/>
-      <c r="K91" s="2" t="n"/>
-      <c r="L91" s="2" t="n"/>
-      <c r="M91" s="2" t="n"/>
-    </row>
-    <row r="92" ht="39.7" customHeight="1">
-      <c r="A92" s="25" t="inlineStr">
-        <is>
-          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
-        </is>
-      </c>
-      <c r="B92" s="2" t="n"/>
-      <c r="C92" s="2" t="n"/>
-      <c r="D92" s="2" t="n"/>
-      <c r="E92" s="2" t="n"/>
-      <c r="F92" s="2" t="n"/>
-      <c r="G92" s="2" t="n"/>
-      <c r="H92" s="2" t="n"/>
-      <c r="I92" s="2" t="n"/>
-      <c r="J92" s="2" t="n"/>
-      <c r="K92" s="2" t="n"/>
-      <c r="L92" s="2" t="n"/>
-      <c r="M92" s="2" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="14">
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="A14:M14"/>
-    <mergeCell ref="A37:M37"/>
     <mergeCell ref="A6:M6"/>
-    <mergeCell ref="E15:E20"/>
+    <mergeCell ref="A22:M22"/>
     <mergeCell ref="B3:L3"/>
     <mergeCell ref="B2:L2"/>
     <mergeCell ref="A4:M4"/>
     <mergeCell ref="E7:E13"/>
-    <mergeCell ref="A21:M21"/>
-    <mergeCell ref="E29:E36"/>
-    <mergeCell ref="E38:E40"/>
-    <mergeCell ref="E22:E27"/>
+    <mergeCell ref="E30:E37"/>
+    <mergeCell ref="A29:M29"/>
+    <mergeCell ref="E23:E28"/>
     <mergeCell ref="M1:M3"/>
     <mergeCell ref="B1:L1"/>
-    <mergeCell ref="A28:M28"/>
+    <mergeCell ref="E15:E21"/>
   </mergeCells>
-  <conditionalFormatting sqref="M6:M40">
+  <conditionalFormatting sqref="M6:M37">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"CUMPLE"</formula>
     </cfRule>
@@ -10950,13 +10870,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="H6:H40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Datos_higro!$A$10:$A$17</formula1>
     </dataValidation>
-    <dataValidation sqref="I6:I40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I6:I37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Datos_higro!$A$21:$A$28</formula1>
     </dataValidation>
-    <dataValidation sqref="K6:K40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K6:K37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Norte,Sur,Este,Oeste,Noreste,Noroeste,Sudeste,Sudoeste,Horizontal"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Balance termico: rehacer los rotulos de orientacion con el plano de fachadas
Cada muro exterior hereda la fachada de la abertura que lleva, que es un
dato del plano y no una deduccion. Doce de los veintiun muros quedan
orientados.

Los otros nueve quedan sin rotulo, por dos motivos distintos que se
anotan en la columna: son muros ciegos, o la abertura entra en mas de un
muro del mismo local y no se puede saber en cual esta. Preferible
dejarlo en blanco antes que poner una orientacion inventada.

No cambia ningun numero: con FO = 1 la orientacion no entra en el
calculo. El total sigue en 27.961 kcal/h.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -23066,7 +23066,7 @@
       <c r="A11" s="10" t="n"/>
       <c r="B11" s="36" t="inlineStr">
         <is>
-          <t>AISLADAS (NE)</t>
+          <t>AISLADAS (NO)</t>
         </is>
       </c>
       <c r="C11" s="10">
@@ -23096,7 +23096,7 @@
       <c r="A12" s="10" t="n"/>
       <c r="B12" s="36" t="inlineStr">
         <is>
-          <t>AISLADAS (NO)</t>
+          <t>AISLADAS (SO)</t>
         </is>
       </c>
       <c r="C12" s="10">
@@ -23791,7 +23791,7 @@
       <c r="A44" s="10" t="n"/>
       <c r="B44" s="36" t="inlineStr">
         <is>
-          <t>AISLADAS (NO)</t>
+          <t>AISLADAS (SE)</t>
         </is>
       </c>
       <c r="C44" s="10">
@@ -23877,7 +23877,7 @@
       <c r="A47" s="10" t="n"/>
       <c r="B47" s="36" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES (galeria, con la PV01)</t>
         </is>
       </c>
       <c r="C47" s="10">
@@ -24519,7 +24519,7 @@
       <c r="A77" s="10" t="n"/>
       <c r="B77" s="36" t="inlineStr">
         <is>
-          <t>AISLADAS (SE)</t>
+          <t>AISLADAS (SO)</t>
         </is>
       </c>
       <c r="C77" s="10">
@@ -24539,7 +24539,7 @@
       </c>
       <c r="G77" s="2" t="n"/>
       <c r="H77" s="37" t="n">
-        <v>2.15</v>
+        <v>3.52</v>
       </c>
       <c r="I77" s="37" t="n">
         <v>3</v>
@@ -24549,7 +24549,7 @@
       <c r="A78" s="10" t="n"/>
       <c r="B78" s="36" t="inlineStr">
         <is>
-          <t>AISLADAS (NE)</t>
+          <t>AISLADAS ()</t>
         </is>
       </c>
       <c r="C78" s="10">
@@ -24569,7 +24569,7 @@
       </c>
       <c r="G78" s="2" t="n"/>
       <c r="H78" s="37" t="n">
-        <v>3.52</v>
+        <v>2.15</v>
       </c>
       <c r="I78" s="37" t="n">
         <v>3</v>
@@ -25139,7 +25139,7 @@
       <c r="A105" s="10" t="n"/>
       <c r="B105" s="36" t="inlineStr">
         <is>
-          <t>AISLADAS (NE)</t>
+          <t>AISLADAS ()</t>
         </is>
       </c>
       <c r="C105" s="10">
@@ -25950,7 +25950,7 @@
       <c r="A141" s="10" t="n"/>
       <c r="B141" s="36" t="inlineStr">
         <is>
-          <t>AISLADAS (NO)</t>
+          <t>AISLADAS ()</t>
         </is>
       </c>
       <c r="C141" s="10">
@@ -25980,7 +25980,7 @@
       <c r="A142" s="10" t="n"/>
       <c r="B142" s="36" t="inlineStr">
         <is>
-          <t>AISLADAS (SO)</t>
+          <t>AISLADAS ()</t>
         </is>
       </c>
       <c r="C142" s="10">
@@ -26604,7 +26604,7 @@
       <c r="A170" s="10" t="n"/>
       <c r="B170" s="36" t="inlineStr">
         <is>
-          <t>AISLADAS (SO)</t>
+          <t>AISLADAS (NE)</t>
         </is>
       </c>
       <c r="C170" s="10">
@@ -26634,7 +26634,7 @@
       <c r="A171" s="10" t="n"/>
       <c r="B171" s="36" t="inlineStr">
         <is>
-          <t>AISLADAS (NE)</t>
+          <t>AISLADAS (SO)</t>
         </is>
       </c>
       <c r="C171" s="10">
@@ -26664,7 +26664,7 @@
       <c r="A172" s="10" t="n"/>
       <c r="B172" s="36" t="inlineStr">
         <is>
-          <t>AISLADAS (SE)</t>
+          <t>AISLADAS ()</t>
         </is>
       </c>
       <c r="C172" s="10">
@@ -27325,7 +27325,7 @@
       <c r="A203" s="10" t="n"/>
       <c r="B203" s="36" t="inlineStr">
         <is>
-          <t>AISLADAS (SO)</t>
+          <t>AISLADAS (NE)</t>
         </is>
       </c>
       <c r="C203" s="10">
@@ -28042,7 +28042,7 @@
       <c r="A236" s="10" t="n"/>
       <c r="B236" s="36" t="inlineStr">
         <is>
-          <t>AISLADAS (SO)</t>
+          <t>AISLADAS ()</t>
         </is>
       </c>
       <c r="C236" s="10">
@@ -28853,7 +28853,7 @@
       <c r="A272" s="10" t="n"/>
       <c r="B272" s="36" t="inlineStr">
         <is>
-          <t>AISLADAS (NE)</t>
+          <t>AISLADAS ()</t>
         </is>
       </c>
       <c r="C272" s="10">
@@ -28883,7 +28883,7 @@
       <c r="A273" s="10" t="n"/>
       <c r="B273" s="36" t="inlineStr">
         <is>
-          <t>INTERIORES (izquierda)</t>
+          <t>INTERIORES (    )</t>
         </is>
       </c>
       <c r="C273" s="10">
@@ -30302,7 +30302,7 @@
       <c r="A338" s="10" t="n"/>
       <c r="B338" s="36" t="inlineStr">
         <is>
-          <t>AISLADAS (NE)</t>
+          <t>AISLADAS ()</t>
         </is>
       </c>
       <c r="C338" s="10">
@@ -30967,7 +30967,7 @@
       <c r="A369" s="10" t="n"/>
       <c r="B369" s="36" t="inlineStr">
         <is>
-          <t>AISLADAS (SE)</t>
+          <t>AISLADAS ()</t>
         </is>
       </c>
       <c r="C369" s="10">
@@ -30997,7 +30997,7 @@
       <c r="A370" s="10" t="n"/>
       <c r="B370" s="36" t="inlineStr">
         <is>
-          <t>AISLADAS (SO)</t>
+          <t>AISLADAS ()</t>
         </is>
       </c>
       <c r="C370" s="10">

</xml_diff>

<commit_message>
Sacar la segunda PV04: no existe
El bloque rotulado PV04 1,50 al final de la fila de las PV en la planilla
de carpinterias no es una abertura: solo tiene el rotulo y la cota, sin
tipo de abertura, ubicacion, cantidad ni forma de abrir. La PV04 real
esta en el bloque anterior, con ficha completa, ubicacion 15 Dormitorio
Sur y cantidad 1.

Se aclara ademas que "corrediza (2 hojas)" es la forma de abrir y no la
cantidad de aberturas.

La Planilla 3 pasa de 20 a 19 aberturas y de 117,99 a 113,56 m2. En el
balance el dormitorio sur baja de 2.712 a 2.428 kcal/h y de 10 a 9
elementos; el total pasa a 27.677 kcal/h.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -31,7 +31,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Iluminacion y ventilacion'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Planilla 3 higrotermica'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla 3 higrotermica'!$A$1:$M$37</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla 3 higrotermica'!$A$1:$M$36</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Planilla vigas'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Planilla vigas'!$A$1:$X$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Planilla losas'!$1:$3</definedName>
@@ -42,7 +42,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="5">'Vigas de fundacion'!$A$1:$X$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Pilotes y cabezales'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Tabiques'!$1:$3</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="8">'Balance termico'!$A$1:$F$396</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="8">'Balance termico'!$A$1:$F$395</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -8355,7 +8355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M89"/>
+  <dimension ref="A1:M91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21.6" customWidth="1" min="1" max="1"/>
@@ -9240,7 +9240,7 @@
         <v/>
       </c>
       <c r="E23" s="19">
-        <f>SUM(D23:D28)</f>
+        <f>SUM(D23:D27)</f>
         <v/>
       </c>
       <c r="F23" s="20">
@@ -9333,14 +9333,14 @@
     <row r="25" ht="70" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>PV04</t>
+          <t>VA05</t>
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>2.95</v>
+        <v>2.52</v>
       </c>
       <c r="C25" s="9" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="D25" s="9">
         <f>IF(COUNT(B25,C25)&lt;2,"",B25*C25)</f>
@@ -9383,17 +9383,9 @@
       </c>
     </row>
     <row r="26" ht="70" customHeight="1">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>VA05</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="n">
-        <v>2.52</v>
-      </c>
-      <c r="C26" s="9" t="n">
-        <v>1.4</v>
-      </c>
+      <c r="A26" s="10" t="n"/>
+      <c r="B26" s="9" t="n"/>
+      <c r="C26" s="9" t="n"/>
       <c r="D26" s="9">
         <f>IF(COUNT(B26,C26)&lt;2,"",B26*C26)</f>
         <v/>
@@ -9407,24 +9399,10 @@
         <f>IF(A26="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H26" s="10" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I26" s="10" t="inlineStr">
-        <is>
-          <t>Sin Proteccion</t>
-        </is>
-      </c>
-      <c r="J26" s="9" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K26" s="10" t="inlineStr">
-        <is>
-          <t>Sudeste</t>
-        </is>
-      </c>
+      <c r="H26" s="10" t="n"/>
+      <c r="I26" s="10" t="n"/>
+      <c r="J26" s="9" t="n"/>
+      <c r="K26" s="10" t="n"/>
       <c r="L26" s="9">
         <f>IF(I26="","",IFERROR(VLOOKUP(I26,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
@@ -9435,106 +9413,128 @@
       </c>
     </row>
     <row r="27" ht="70" customHeight="1">
-      <c r="A27" s="10" t="n"/>
-      <c r="B27" s="9" t="n"/>
-      <c r="C27" s="9" t="n"/>
-      <c r="D27" s="9">
+      <c r="A27" s="14" t="n"/>
+      <c r="B27" s="13" t="n"/>
+      <c r="C27" s="13" t="n"/>
+      <c r="D27" s="13">
         <f>IF(COUNT(B27,C27)&lt;2,"",B27*C27)</f>
         <v/>
       </c>
-      <c r="E27" s="21" t="n"/>
-      <c r="F27" s="20">
+      <c r="E27" s="22" t="n"/>
+      <c r="F27" s="23">
         <f>IF(OR(D27="",$E$23=""),"",D27/$E$23)</f>
         <v/>
       </c>
-      <c r="G27" s="9">
+      <c r="G27" s="13">
         <f>IF(A27="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H27" s="10" t="n"/>
-      <c r="I27" s="10" t="n"/>
-      <c r="J27" s="9" t="n"/>
-      <c r="K27" s="10" t="n"/>
-      <c r="L27" s="9">
+      <c r="H27" s="14" t="n"/>
+      <c r="I27" s="14" t="n"/>
+      <c r="J27" s="13" t="n"/>
+      <c r="K27" s="14" t="n"/>
+      <c r="L27" s="13">
         <f>IF(I27="","",IFERROR(VLOOKUP(I27,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
-      <c r="M27" s="10">
+      <c r="M27" s="14">
         <f>IF(OR(D27="",J27=""),"",IF(J27&lt;=G27,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="28" ht="70" customHeight="1">
-      <c r="A28" s="14" t="n"/>
-      <c r="B28" s="13" t="n"/>
-      <c r="C28" s="13" t="n"/>
-      <c r="D28" s="13">
-        <f>IF(COUNT(B28,C28)&lt;2,"",B28*C28)</f>
-        <v/>
-      </c>
-      <c r="E28" s="22" t="n"/>
-      <c r="F28" s="23">
-        <f>IF(OR(D28="",$E$23=""),"",D28/$E$23)</f>
-        <v/>
-      </c>
-      <c r="G28" s="13">
-        <f>IF(A28="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H28" s="14" t="n"/>
-      <c r="I28" s="14" t="n"/>
-      <c r="J28" s="13" t="n"/>
-      <c r="K28" s="14" t="n"/>
-      <c r="L28" s="13">
-        <f>IF(I28="","",IFERROR(VLOOKUP(I28,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M28" s="14">
-        <f>IF(OR(D28="",J28=""),"",IF(J28&lt;=G28,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="39.7" customHeight="1">
-      <c r="A29" s="5" t="inlineStr">
+    <row r="28" ht="39.7" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>Plano: Fachada Noroeste</t>
         </is>
       </c>
-      <c r="B29" s="4" t="n"/>
-      <c r="C29" s="4" t="n"/>
-      <c r="D29" s="4" t="n"/>
-      <c r="E29" s="4" t="n"/>
-      <c r="F29" s="4" t="n"/>
-      <c r="G29" s="4" t="n"/>
-      <c r="H29" s="4" t="n"/>
-      <c r="I29" s="4" t="n"/>
-      <c r="J29" s="4" t="n"/>
-      <c r="K29" s="4" t="n"/>
-      <c r="L29" s="4" t="n"/>
-      <c r="M29" s="4" t="n"/>
+      <c r="B28" s="4" t="n"/>
+      <c r="C28" s="4" t="n"/>
+      <c r="D28" s="4" t="n"/>
+      <c r="E28" s="4" t="n"/>
+      <c r="F28" s="4" t="n"/>
+      <c r="G28" s="4" t="n"/>
+      <c r="H28" s="4" t="n"/>
+      <c r="I28" s="4" t="n"/>
+      <c r="J28" s="4" t="n"/>
+      <c r="K28" s="4" t="n"/>
+      <c r="L28" s="4" t="n"/>
+      <c r="M28" s="4" t="n"/>
+    </row>
+    <row r="29" ht="70" customHeight="1">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>PF03</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C29" s="9" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="D29" s="9">
+        <f>IF(COUNT(B29,C29)&lt;2,"",B29*C29)</f>
+        <v/>
+      </c>
+      <c r="E29" s="19">
+        <f>SUM(D29:D36)</f>
+        <v/>
+      </c>
+      <c r="F29" s="20">
+        <f>IF(OR(D29="",$E$29=""),"",D29/$E$29)</f>
+        <v/>
+      </c>
+      <c r="G29" s="9">
+        <f>IF(A29="","",Datos_higro!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H29" s="10" t="inlineStr">
+        <is>
+          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
+        </is>
+      </c>
+      <c r="I29" s="10" t="inlineStr">
+        <is>
+          <t>Sin Proteccion</t>
+        </is>
+      </c>
+      <c r="J29" s="9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K29" s="10" t="inlineStr">
+        <is>
+          <t>Noroeste</t>
+        </is>
+      </c>
+      <c r="L29" s="9">
+        <f>IF(I29="","",IFERROR(VLOOKUP(I29,Datos_higro!$A$21:$B$28,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="M29" s="10">
+        <f>IF(OR(D29="",J29=""),"",IF(J29&lt;=G29,"CUMPLE","NO CUMPLE"))</f>
+        <v/>
+      </c>
     </row>
     <row r="30" ht="70" customHeight="1">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>PF03</t>
+          <t>PF01</t>
         </is>
       </c>
       <c r="B30" s="9" t="n">
         <v>3</v>
       </c>
       <c r="C30" s="9" t="n">
-        <v>2.88</v>
+        <v>3.55</v>
       </c>
       <c r="D30" s="9">
         <f>IF(COUNT(B30,C30)&lt;2,"",B30*C30)</f>
         <v/>
       </c>
-      <c r="E30" s="19">
-        <f>SUM(D30:D37)</f>
-        <v/>
-      </c>
+      <c r="E30" s="21" t="n"/>
       <c r="F30" s="20">
-        <f>IF(OR(D30="",$E$30=""),"",D30/$E$30)</f>
+        <f>IF(OR(D30="",$E$29=""),"",D30/$E$29)</f>
         <v/>
       </c>
       <c r="G30" s="9">
@@ -9571,14 +9571,14 @@
     <row r="31" ht="70" customHeight="1">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>PF01</t>
+          <t>PV01</t>
         </is>
       </c>
       <c r="B31" s="9" t="n">
         <v>3</v>
       </c>
       <c r="C31" s="9" t="n">
-        <v>3.55</v>
+        <v>7.7</v>
       </c>
       <c r="D31" s="9">
         <f>IF(COUNT(B31,C31)&lt;2,"",B31*C31)</f>
@@ -9586,7 +9586,7 @@
       </c>
       <c r="E31" s="21" t="n"/>
       <c r="F31" s="20">
-        <f>IF(OR(D31="",$E$30=""),"",D31/$E$30)</f>
+        <f>IF(OR(D31="",$E$29=""),"",D31/$E$29)</f>
         <v/>
       </c>
       <c r="G31" s="9">
@@ -9623,14 +9623,14 @@
     <row r="32" ht="70" customHeight="1">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>PV01</t>
+          <t>PV02</t>
         </is>
       </c>
       <c r="B32" s="9" t="n">
         <v>3</v>
       </c>
       <c r="C32" s="9" t="n">
-        <v>7.7</v>
+        <v>2.48</v>
       </c>
       <c r="D32" s="9">
         <f>IF(COUNT(B32,C32)&lt;2,"",B32*C32)</f>
@@ -9638,7 +9638,7 @@
       </c>
       <c r="E32" s="21" t="n"/>
       <c r="F32" s="20">
-        <f>IF(OR(D32="",$E$30=""),"",D32/$E$30)</f>
+        <f>IF(OR(D32="",$E$29=""),"",D32/$E$29)</f>
         <v/>
       </c>
       <c r="G32" s="9">
@@ -9675,14 +9675,14 @@
     <row r="33" ht="70" customHeight="1">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>PV02</t>
+          <t>VA04</t>
         </is>
       </c>
       <c r="B33" s="9" t="n">
-        <v>3</v>
+        <v>2.52</v>
       </c>
       <c r="C33" s="9" t="n">
-        <v>2.48</v>
+        <v>2</v>
       </c>
       <c r="D33" s="9">
         <f>IF(COUNT(B33,C33)&lt;2,"",B33*C33)</f>
@@ -9690,7 +9690,7 @@
       </c>
       <c r="E33" s="21" t="n"/>
       <c r="F33" s="20">
-        <f>IF(OR(D33="",$E$30=""),"",D33/$E$30)</f>
+        <f>IF(OR(D33="",$E$29=""),"",D33/$E$29)</f>
         <v/>
       </c>
       <c r="G33" s="9">
@@ -9742,7 +9742,7 @@
       </c>
       <c r="E34" s="21" t="n"/>
       <c r="F34" s="20">
-        <f>IF(OR(D34="",$E$30=""),"",D34/$E$30)</f>
+        <f>IF(OR(D34="",$E$29=""),"",D34/$E$29)</f>
         <v/>
       </c>
       <c r="G34" s="9">
@@ -9777,48 +9777,26 @@
       </c>
     </row>
     <row r="35" ht="70" customHeight="1">
-      <c r="A35" s="10" t="inlineStr">
-        <is>
-          <t>VA04</t>
-        </is>
-      </c>
-      <c r="B35" s="9" t="n">
-        <v>2.52</v>
-      </c>
-      <c r="C35" s="9" t="n">
-        <v>2</v>
-      </c>
+      <c r="A35" s="10" t="n"/>
+      <c r="B35" s="9" t="n"/>
+      <c r="C35" s="9" t="n"/>
       <c r="D35" s="9">
         <f>IF(COUNT(B35,C35)&lt;2,"",B35*C35)</f>
         <v/>
       </c>
       <c r="E35" s="21" t="n"/>
       <c r="F35" s="20">
-        <f>IF(OR(D35="",$E$30=""),"",D35/$E$30)</f>
+        <f>IF(OR(D35="",$E$29=""),"",D35/$E$29)</f>
         <v/>
       </c>
       <c r="G35" s="9">
         <f>IF(A35="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H35" s="10" t="inlineStr">
-        <is>
-          <t>DVH 6+9+3+3 (aluminio linea A30)</t>
-        </is>
-      </c>
-      <c r="I35" s="10" t="inlineStr">
-        <is>
-          <t>Sin Proteccion</t>
-        </is>
-      </c>
-      <c r="J35" s="9" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K35" s="10" t="inlineStr">
-        <is>
-          <t>Noroeste</t>
-        </is>
-      </c>
+      <c r="H35" s="10" t="n"/>
+      <c r="I35" s="10" t="n"/>
+      <c r="J35" s="9" t="n"/>
+      <c r="K35" s="10" t="n"/>
       <c r="L35" s="9">
         <f>IF(I35="","",IFERROR(VLOOKUP(I35,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
@@ -9829,69 +9807,58 @@
       </c>
     </row>
     <row r="36" ht="70" customHeight="1">
-      <c r="A36" s="10" t="n"/>
-      <c r="B36" s="9" t="n"/>
-      <c r="C36" s="9" t="n"/>
-      <c r="D36" s="9">
+      <c r="A36" s="14" t="n"/>
+      <c r="B36" s="13" t="n"/>
+      <c r="C36" s="13" t="n"/>
+      <c r="D36" s="13">
         <f>IF(COUNT(B36,C36)&lt;2,"",B36*C36)</f>
         <v/>
       </c>
-      <c r="E36" s="21" t="n"/>
-      <c r="F36" s="20">
-        <f>IF(OR(D36="",$E$30=""),"",D36/$E$30)</f>
-        <v/>
-      </c>
-      <c r="G36" s="9">
+      <c r="E36" s="22" t="n"/>
+      <c r="F36" s="23">
+        <f>IF(OR(D36="",$E$29=""),"",D36/$E$29)</f>
+        <v/>
+      </c>
+      <c r="G36" s="13">
         <f>IF(A36="","",Datos_higro!$B$4)</f>
         <v/>
       </c>
-      <c r="H36" s="10" t="n"/>
-      <c r="I36" s="10" t="n"/>
-      <c r="J36" s="9" t="n"/>
-      <c r="K36" s="10" t="n"/>
-      <c r="L36" s="9">
+      <c r="H36" s="14" t="n"/>
+      <c r="I36" s="14" t="n"/>
+      <c r="J36" s="13" t="n"/>
+      <c r="K36" s="14" t="n"/>
+      <c r="L36" s="13">
         <f>IF(I36="","",IFERROR(VLOOKUP(I36,Datos_higro!$A$21:$B$28,2,0),""))</f>
         <v/>
       </c>
-      <c r="M36" s="10">
+      <c r="M36" s="14">
         <f>IF(OR(D36="",J36=""),"",IF(J36&lt;=G36,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
     </row>
-    <row r="37" ht="70" customHeight="1">
-      <c r="A37" s="14" t="n"/>
-      <c r="B37" s="13" t="n"/>
-      <c r="C37" s="13" t="n"/>
-      <c r="D37" s="13">
-        <f>IF(COUNT(B37,C37)&lt;2,"",B37*C37)</f>
-        <v/>
-      </c>
-      <c r="E37" s="22" t="n"/>
-      <c r="F37" s="23">
-        <f>IF(OR(D37="",$E$30=""),"",D37/$E$30)</f>
-        <v/>
-      </c>
-      <c r="G37" s="13">
-        <f>IF(A37="","",Datos_higro!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H37" s="14" t="n"/>
-      <c r="I37" s="14" t="n"/>
-      <c r="J37" s="13" t="n"/>
-      <c r="K37" s="14" t="n"/>
-      <c r="L37" s="13">
-        <f>IF(I37="","",IFERROR(VLOOKUP(I37,Datos_higro!$A$21:$B$28,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="M37" s="14">
-        <f>IF(OR(D37="",J37=""),"",IF(J37&lt;=G37,"CUMPLE","NO CUMPLE"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="16" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
         <is>
           <t>HOJA REHECHA: las orientaciones se tomaron del plano de fachadas y cambiaron casi todas. Hay que reemplazar la planilla entera, no alcanza con retocar celdas.</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="n"/>
+      <c r="H37" s="2" t="n"/>
+      <c r="I37" s="2" t="n"/>
+      <c r="J37" s="2" t="n"/>
+      <c r="K37" s="2" t="n"/>
+      <c r="L37" s="2" t="n"/>
+      <c r="M37" s="2" t="n"/>
+    </row>
+    <row r="38" ht="39.7" customHeight="1">
+      <c r="A38" s="24" t="inlineStr">
+        <is>
+          <t>COMO SE COMPLETA</t>
         </is>
       </c>
       <c r="B38" s="2" t="n"/>
@@ -9908,9 +9875,9 @@
       <c r="M38" s="2" t="n"/>
     </row>
     <row r="39" ht="39.7" customHeight="1">
-      <c r="A39" s="24" t="inlineStr">
-        <is>
-          <t>COMO SE COMPLETA</t>
+      <c r="A39" s="25" t="inlineStr">
+        <is>
+          <t>Descripcion, altura y ancho del vano: de la planilla de carpinterias.</t>
         </is>
       </c>
       <c r="B39" s="2" t="n"/>
@@ -9929,7 +9896,7 @@
     <row r="40" ht="39.7" customHeight="1">
       <c r="A40" s="25" t="inlineStr">
         <is>
-          <t>Descripcion, altura y ancho del vano: de la planilla de carpinterias.</t>
+          <t>Area del vano, area total por plano y porcentaje: se calculan solos.</t>
         </is>
       </c>
       <c r="B40" s="2" t="n"/>
@@ -9948,7 +9915,7 @@
     <row r="41" ht="39.7" customHeight="1">
       <c r="A41" s="25" t="inlineStr">
         <is>
-          <t>Area del vano, area total por plano y porcentaje: se calculan solos.</t>
+          <t>Tipo de vidrio y tipo de proteccion: desplegables; sus valores estan en la hoja Datos_higro.</t>
         </is>
       </c>
       <c r="B41" s="2" t="n"/>
@@ -9967,7 +9934,7 @@
     <row r="42" ht="39.7" customHeight="1">
       <c r="A42" s="25" t="inlineStr">
         <is>
-          <t>Tipo de vidrio y tipo de proteccion: desplegables; sus valores estan en la hoja Datos_higro.</t>
+          <t>Transmitancia del cerramiento: cargarla segun el vidrio y el marco adoptados.</t>
         </is>
       </c>
       <c r="B42" s="2" t="n"/>
@@ -9986,7 +9953,7 @@
     <row r="43" ht="39.7" customHeight="1">
       <c r="A43" s="25" t="inlineStr">
         <is>
-          <t>Transmitancia del cerramiento: cargarla segun el vidrio y el marco adoptados.</t>
+          <t>PROTECCION: la obra tiene cortinas blackout INTERIORES, y los panos fijos PF no tienen nada.</t>
         </is>
       </c>
       <c r="B43" s="2" t="n"/>
@@ -10005,7 +9972,7 @@
     <row r="44" ht="39.7" customHeight="1">
       <c r="A44" s="25" t="inlineStr">
         <is>
-          <t>PROTECCION: la obra tiene cortinas blackout INTERIORES, y los panos fijos PF no tienen nada.</t>
+          <t>Una cortina interior NO computa como proteccion solar: la radiacion ya atraveso el vidrio</t>
         </is>
       </c>
       <c r="B44" s="2" t="n"/>
@@ -10024,7 +9991,7 @@
     <row r="45" ht="39.7" customHeight="1">
       <c r="A45" s="25" t="inlineStr">
         <is>
-          <t>Una cortina interior NO computa como proteccion solar: la radiacion ya atraveso el vidrio</t>
+          <t>cuando llega a la cortina. La ordenanza acredita protecciones exteriores (aleros, parasoles,</t>
         </is>
       </c>
       <c r="B45" s="2" t="n"/>
@@ -10043,7 +10010,7 @@
     <row r="46" ht="39.7" customHeight="1">
       <c r="A46" s="25" t="inlineStr">
         <is>
-          <t>cuando llega a la cortina. La ordenanza acredita protecciones exteriores (aleros, parasoles,</t>
+          <t>cortinas de enrollar exteriores, toldos). Por eso las veinte aberturas van Sin Proteccion.</t>
         </is>
       </c>
       <c r="B46" s="2" t="n"/>
@@ -10059,12 +10026,8 @@
       <c r="L46" s="2" t="n"/>
       <c r="M46" s="2" t="n"/>
     </row>
-    <row r="47" ht="39.7" customHeight="1">
-      <c r="A47" s="25" t="inlineStr">
-        <is>
-          <t>cortinas de enrollar exteriores, toldos). Por eso las veinte aberturas van Sin Proteccion.</t>
-        </is>
-      </c>
+    <row r="47">
+      <c r="A47" s="25" t="inlineStr"/>
       <c r="B47" s="2" t="n"/>
       <c r="C47" s="2" t="n"/>
       <c r="D47" s="2" t="n"/>
@@ -10078,8 +10041,12 @@
       <c r="L47" s="2" t="n"/>
       <c r="M47" s="2" t="n"/>
     </row>
-    <row r="48">
-      <c r="A48" s="25" t="inlineStr"/>
+    <row r="48" ht="39.7" customHeight="1">
+      <c r="A48" s="25" t="inlineStr">
+        <is>
+          <t>CONSECUENCIA: el factor de exposicion solar da 0,88 esta muy por encima del maximo de 0,30 que la ordenanza admite para</t>
+        </is>
+      </c>
       <c r="B48" s="2" t="n"/>
       <c r="C48" s="2" t="n"/>
       <c r="D48" s="2" t="n"/>
@@ -10096,7 +10063,7 @@
     <row r="49" ht="39.7" customHeight="1">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>CONSECUENCIA: el factor de exposicion solar da 0,88 esta muy por encima del maximo de 0,30 que la ordenanza admite para</t>
+          <t>el cuadrante Este/Oeste, donde caen las cuatro fachadas de esta casa por estar girada 45</t>
         </is>
       </c>
       <c r="B49" s="2" t="n"/>
@@ -10115,7 +10082,7 @@
     <row r="50" ht="39.7" customHeight="1">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>el cuadrante Este/Oeste, donde caen las cuatro fachadas de esta casa por estar girada 45</t>
+          <t>grados. La verificacion de la planilla no lo controla, igual que la de la catedra, pero si lo</t>
         </is>
       </c>
       <c r="B50" s="2" t="n"/>
@@ -10134,7 +10101,7 @@
     <row r="51" ht="39.7" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>grados. La verificacion de la planilla no lo controla, igual que la de la catedra, pero si lo</t>
+          <t>presentas en el municipio esas cinco aberturas no pasarian el factor de exposicion solar.</t>
         </is>
       </c>
       <c r="B51" s="2" t="n"/>
@@ -10153,7 +10120,7 @@
     <row r="52" ht="39.7" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>presentas en el municipio esas cinco aberturas no pasarian el factor de exposicion solar.</t>
+          <t>Hay dos salidas posibles: (a) si la abertura ocupa menos del 20% del lado expuesto del local,</t>
         </is>
       </c>
       <c r="B52" s="2" t="n"/>
@@ -10172,7 +10139,7 @@
     <row r="53" ht="39.7" customHeight="1">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>Hay dos salidas posibles: (a) si la abertura ocupa menos del 20% del lado expuesto del local,</t>
+          <t>no se verifica el FES; (b) cambiar el vidrio por uno de control solar, que baja el FES sin</t>
         </is>
       </c>
       <c r="B53" s="2" t="n"/>
@@ -10191,7 +10158,7 @@
     <row r="54" ht="39.7" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>no se verifica el FES; (b) cambiar el vidrio por uno de control solar, que baja el FES sin</t>
+          <t>tocar la obra. Agregar una proteccion exterior seria la tercera, pero implica obra.</t>
         </is>
       </c>
       <c r="B54" s="2" t="n"/>
@@ -10207,12 +10174,8 @@
       <c r="L54" s="2" t="n"/>
       <c r="M54" s="2" t="n"/>
     </row>
-    <row r="55" ht="39.7" customHeight="1">
-      <c r="A55" s="25" t="inlineStr">
-        <is>
-          <t>tocar la obra. Agregar una proteccion exterior seria la tercera, pero implica obra.</t>
-        </is>
-      </c>
+    <row r="55">
+      <c r="A55" s="25" t="inlineStr"/>
       <c r="B55" s="2" t="n"/>
       <c r="C55" s="2" t="n"/>
       <c r="D55" s="2" t="n"/>
@@ -10226,8 +10189,12 @@
       <c r="L55" s="2" t="n"/>
       <c r="M55" s="2" t="n"/>
     </row>
-    <row r="56">
-      <c r="A56" s="25" t="inlineStr"/>
+    <row r="56" ht="39.7" customHeight="1">
+      <c r="A56" s="25" t="inlineStr">
+        <is>
+          <t>Orientacion: ya cargada. Factor de exposicion solar: se completa SOLO al elegir el tipo de</t>
+        </is>
+      </c>
       <c r="B56" s="2" t="n"/>
       <c r="C56" s="2" t="n"/>
       <c r="D56" s="2" t="n"/>
@@ -10244,7 +10211,7 @@
     <row r="57" ht="39.7" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>Orientacion: ya cargada. Factor de exposicion solar: se completa SOLO al elegir el tipo de</t>
+          <t>proteccion, con los valores de la tabla de Datos_higro (Sin Proteccion 0,88; Parasol</t>
         </is>
       </c>
       <c r="B57" s="2" t="n"/>
@@ -10263,7 +10230,7 @@
     <row r="58" ht="39.7" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>proteccion, con los valores de la tabla de Datos_higro (Sin Proteccion 0,88; Parasol</t>
+          <t>horizontal fijo 1:2 0,35), que son los mismos de la planilla de la catedra.</t>
         </is>
       </c>
       <c r="B58" s="2" t="n"/>
@@ -10282,7 +10249,7 @@
     <row r="59" ht="39.7" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>horizontal fijo 1:2 0,35), que son los mismos de la planilla de la catedra.</t>
+          <t>En Datos_higro esta ademas el FES maximo admitido por cuadrante segun la ordenanza, como</t>
         </is>
       </c>
       <c r="B59" s="2" t="n"/>
@@ -10301,7 +10268,7 @@
     <row r="60" ht="39.7" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>En Datos_higro esta ademas el FES maximo admitido por cuadrante segun la ordenanza, como</t>
+          <t>referencia: la verificacion no lo controla, igual que en la planilla de la catedra.</t>
         </is>
       </c>
       <c r="B60" s="2" t="n"/>
@@ -10317,12 +10284,8 @@
       <c r="L60" s="2" t="n"/>
       <c r="M60" s="2" t="n"/>
     </row>
-    <row r="61" ht="39.7" customHeight="1">
-      <c r="A61" s="25" t="inlineStr">
-        <is>
-          <t>referencia: la verificacion no lo controla, igual que en la planilla de la catedra.</t>
-        </is>
-      </c>
+    <row r="61">
+      <c r="A61" s="25" t="inlineStr"/>
       <c r="B61" s="2" t="n"/>
       <c r="C61" s="2" t="n"/>
       <c r="D61" s="2" t="n"/>
@@ -10336,8 +10299,12 @@
       <c r="L61" s="2" t="n"/>
       <c r="M61" s="2" t="n"/>
     </row>
-    <row r="62">
-      <c r="A62" s="25" t="inlineStr"/>
+    <row r="62" ht="39.7" customHeight="1">
+      <c r="A62" s="25" t="inlineStr">
+        <is>
+          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
+        </is>
+      </c>
       <c r="B62" s="2" t="n"/>
       <c r="C62" s="2" t="n"/>
       <c r="D62" s="2" t="n"/>
@@ -10354,7 +10321,7 @@
     <row r="63" ht="39.7" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>CARGADO de la planilla de carpinterias: designacion, ubicacion, ancho y tipo de vidrio</t>
+          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
         </is>
       </c>
       <c r="B63" s="2" t="n"/>
@@ -10370,12 +10337,8 @@
       <c r="L63" s="2" t="n"/>
       <c r="M63" s="2" t="n"/>
     </row>
-    <row r="64" ht="39.7" customHeight="1">
-      <c r="A64" s="25" t="inlineStr">
-        <is>
-          <t>(DVH 6+9+3+3, carpinteria de aluminio linea A30 pintado negro, igual en todas las aberturas).</t>
-        </is>
-      </c>
+    <row r="64">
+      <c r="A64" s="25" t="inlineStr"/>
       <c r="B64" s="2" t="n"/>
       <c r="C64" s="2" t="n"/>
       <c r="D64" s="2" t="n"/>
@@ -10389,8 +10352,12 @@
       <c r="L64" s="2" t="n"/>
       <c r="M64" s="2" t="n"/>
     </row>
-    <row r="65">
-      <c r="A65" s="25" t="inlineStr"/>
+    <row r="65" ht="39.7" customHeight="1">
+      <c r="A65" s="25" t="inlineStr">
+        <is>
+          <t>ALTURAS: medidas sobre el dibujo de las vistas de la planilla de carpinterias, con la escala</t>
+        </is>
+      </c>
       <c r="B65" s="2" t="n"/>
       <c r="C65" s="2" t="n"/>
       <c r="D65" s="2" t="n"/>
@@ -10407,7 +10374,7 @@
     <row r="66" ht="39.7" customHeight="1">
       <c r="A66" s="25" t="inlineStr">
         <is>
-          <t>ALTURAS: medidas sobre el dibujo de las vistas de la planilla de carpinterias, con la escala</t>
+          <t>verificada contra los anchos acotados (error menor a 2 cm). La mayoria de las aberturas son de</t>
         </is>
       </c>
       <c r="B66" s="2" t="n"/>
@@ -10426,7 +10393,7 @@
     <row r="67" ht="39.7" customHeight="1">
       <c r="A67" s="25" t="inlineStr">
         <is>
-          <t>verificada contra los anchos acotados (error menor a 2 cm). La mayoria de las aberturas son de</t>
+          <t>piso a cielorraso, 3,00 m. VERIFICARLAS contra el plano antes de presentar.</t>
         </is>
       </c>
       <c r="B67" s="2" t="n"/>
@@ -10445,7 +10412,7 @@
     <row r="68" ht="39.7" customHeight="1">
       <c r="A68" s="25" t="inlineStr">
         <is>
-          <t>piso a cielorraso, 3,00 m. VERIFICARLAS contra el plano antes de presentar.</t>
+          <t>PF04 es la unica con antepecho: arranca a 1,09 y mide 0,60 de alto. El resto llega al piso.</t>
         </is>
       </c>
       <c r="B68" s="2" t="n"/>
@@ -10464,7 +10431,7 @@
     <row r="69" ht="39.7" customHeight="1">
       <c r="A69" s="25" t="inlineStr">
         <is>
-          <t>PF04 es la unica con antepecho: arranca a 1,09 y mide 0,60 de alto. El resto llega al piso.</t>
+          <t>Las alturas de PV01 (3,00) y PF04 (0,60) las aporto el autor del proyecto.</t>
         </is>
       </c>
       <c r="B69" s="2" t="n"/>
@@ -10483,7 +10450,7 @@
     <row r="70" ht="39.7" customHeight="1">
       <c r="A70" s="25" t="inlineStr">
         <is>
-          <t>Las alturas de PV01 (3,00), PF04 (0,60) y PV04 (2) (2,95) las aporto el autor del proyecto.</t>
+          <t>El bloque suelto rotulado PV04 1,50 de la planilla de carpinterias no es una abertura:</t>
         </is>
       </c>
       <c r="B70" s="2" t="n"/>
@@ -10499,8 +10466,12 @@
       <c r="L70" s="2" t="n"/>
       <c r="M70" s="2" t="n"/>
     </row>
-    <row r="71">
-      <c r="A71" s="25" t="inlineStr"/>
+    <row r="71" ht="39.7" customHeight="1">
+      <c r="A71" s="25" t="inlineStr">
+        <is>
+          <t>no tiene ficha, ni ubicacion ni cantidad. PV04 es una sola, de 2,06, cantidad 1.</t>
+        </is>
+      </c>
       <c r="B71" s="2" t="n"/>
       <c r="C71" s="2" t="n"/>
       <c r="D71" s="2" t="n"/>
@@ -10517,7 +10488,7 @@
     <row r="72" ht="39.7" customHeight="1">
       <c r="A72" s="25" t="inlineStr">
         <is>
-          <t>ORIENTACION: el simbolo de norte del plano (circulo con aguja, en el patio interno) apunta a</t>
+          <t>"2 hojas" es la forma de abrir, no la cantidad de aberturas.</t>
         </is>
       </c>
       <c r="B72" s="2" t="n"/>
@@ -10533,12 +10504,8 @@
       <c r="L72" s="2" t="n"/>
       <c r="M72" s="2" t="n"/>
     </row>
-    <row r="73" ht="39.7" customHeight="1">
-      <c r="A73" s="25" t="inlineStr">
-        <is>
-          <t>45 grados hacia arriba y a la derecha de la hoja. Entonces las cuatro fachadas NO son N-S-E-O</t>
-        </is>
-      </c>
+    <row r="73">
+      <c r="A73" s="25" t="inlineStr"/>
       <c r="B73" s="2" t="n"/>
       <c r="C73" s="2" t="n"/>
       <c r="D73" s="2" t="n"/>
@@ -10555,7 +10522,7 @@
     <row r="74" ht="39.7" customHeight="1">
       <c r="A74" s="25" t="inlineStr">
         <is>
-          <t>sino: arriba = Noroeste, derecha = Noreste, abajo = Sudeste, izquierda = Sudoeste.</t>
+          <t>ORIENTACION: el simbolo de norte del plano (circulo con aguja, en el patio interno) apunta a</t>
         </is>
       </c>
       <c r="B74" s="2" t="n"/>
@@ -10574,7 +10541,7 @@
     <row r="75" ht="39.7" customHeight="1">
       <c r="A75" s="25" t="inlineStr">
         <is>
-          <t>Cada abertura se asigno a la fachada por su posicion en planta. Las del patio interno se</t>
+          <t>45 grados hacia arriba y a la derecha de la hoja. Entonces las cuatro fachadas NO son N-S-E-O</t>
         </is>
       </c>
       <c r="B75" s="2" t="n"/>
@@ -10593,7 +10560,7 @@
     <row r="76" ht="39.7" customHeight="1">
       <c r="A76" s="25" t="inlineStr">
         <is>
-          <t>orientan por la pared en la que estan: miran hacia adentro del patio.</t>
+          <t>sino: arriba = Noroeste, derecha = Noreste, abajo = Sudeste, izquierda = Sudoeste.</t>
         </is>
       </c>
       <c r="B76" s="2" t="n"/>
@@ -10612,7 +10579,7 @@
     <row r="77" ht="39.7" customHeight="1">
       <c r="A77" s="25" t="inlineStr">
         <is>
-          <t>Los rotulos Dormitorio Norte y Dormitorio Sur del plano no coinciden con el norte real;</t>
+          <t>Cada abertura se asigno a la fachada por su posicion en planta. Las del patio interno se</t>
         </is>
       </c>
       <c r="B77" s="2" t="n"/>
@@ -10631,7 +10598,7 @@
     <row r="78" ht="39.7" customHeight="1">
       <c r="A78" s="25" t="inlineStr">
         <is>
-          <t>parecen ser nombres de uso, no orientaciones.</t>
+          <t>orientan por la pared en la que estan: miran hacia adentro del patio.</t>
         </is>
       </c>
       <c r="B78" s="2" t="n"/>
@@ -10647,8 +10614,12 @@
       <c r="L78" s="2" t="n"/>
       <c r="M78" s="2" t="n"/>
     </row>
-    <row r="79">
-      <c r="A79" s="25" t="inlineStr"/>
+    <row r="79" ht="39.7" customHeight="1">
+      <c r="A79" s="25" t="inlineStr">
+        <is>
+          <t>Los rotulos Dormitorio Norte y Dormitorio Sur del plano no coinciden con el norte real;</t>
+        </is>
+      </c>
       <c r="B79" s="2" t="n"/>
       <c r="C79" s="2" t="n"/>
       <c r="D79" s="2" t="n"/>
@@ -10665,7 +10636,7 @@
     <row r="80" ht="39.7" customHeight="1">
       <c r="A80" s="25" t="inlineStr">
         <is>
-          <t>CANTIDADES: la planilla de carpinterias trae la cantidad de cada abertura. Tres van dos veces:</t>
+          <t>parecen ser nombres de uso, no orientaciones.</t>
         </is>
       </c>
       <c r="B80" s="2" t="n"/>
@@ -10681,12 +10652,8 @@
       <c r="L80" s="2" t="n"/>
       <c r="M80" s="2" t="n"/>
     </row>
-    <row r="81" ht="39.7" customHeight="1">
-      <c r="A81" s="25" t="inlineStr">
-        <is>
-          <t>VA01 (01 Cocina y 09 Suite), VA04 (13 Dormitorio Norte y 14 Play Room) y PF01 (03 Lavadero y</t>
-        </is>
-      </c>
+    <row r="81">
+      <c r="A81" s="25" t="inlineStr"/>
       <c r="B81" s="2" t="n"/>
       <c r="C81" s="2" t="n"/>
       <c r="D81" s="2" t="n"/>
@@ -10703,7 +10670,7 @@
     <row r="82" ht="39.7" customHeight="1">
       <c r="A82" s="25" t="inlineStr">
         <is>
-          <t>07 Hall de ingreso, a los dos lados del patio interno). Por eso la planilla tiene 20 filas y</t>
+          <t>CANTIDADES: la planilla de carpinterias trae la cantidad de cada abertura. Tres van dos veces:</t>
         </is>
       </c>
       <c r="B82" s="2" t="n"/>
@@ -10722,7 +10689,7 @@
     <row r="83" ht="39.7" customHeight="1">
       <c r="A83" s="25" t="inlineStr">
         <is>
-          <t>no 17. Las demas aberturas son de una sola unidad.</t>
+          <t>VA01 (01 Cocina y 09 Suite), VA04 (13 Dormitorio Norte y 14 Play Room) y PF01 (03 Lavadero y</t>
         </is>
       </c>
       <c r="B83" s="2" t="n"/>
@@ -10738,8 +10705,12 @@
       <c r="L83" s="2" t="n"/>
       <c r="M83" s="2" t="n"/>
     </row>
-    <row r="84">
-      <c r="A84" s="25" t="inlineStr"/>
+    <row r="84" ht="39.7" customHeight="1">
+      <c r="A84" s="25" t="inlineStr">
+        <is>
+          <t>07 Hall de ingreso, a los dos lados del patio interno). Por eso la planilla tiene 20 filas y</t>
+        </is>
+      </c>
       <c r="B84" s="2" t="n"/>
       <c r="C84" s="2" t="n"/>
       <c r="D84" s="2" t="n"/>
@@ -10756,7 +10727,7 @@
     <row r="85" ht="39.7" customHeight="1">
       <c r="A85" s="25" t="inlineStr">
         <is>
-          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
+          <t>no 17. Las demas aberturas son de una sola unidad.</t>
         </is>
       </c>
       <c r="B85" s="2" t="n"/>
@@ -10790,7 +10761,7 @@
     <row r="87" ht="39.7" customHeight="1">
       <c r="A87" s="25" t="inlineStr">
         <is>
-          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
+          <t>Las puertas interiores de madera PM01 a PM08 no se cargan: no son cerramientos exteriores.</t>
         </is>
       </c>
       <c r="B87" s="2" t="n"/>
@@ -10806,12 +10777,8 @@
       <c r="L87" s="2" t="n"/>
       <c r="M87" s="2" t="n"/>
     </row>
-    <row r="88" ht="39.7" customHeight="1">
-      <c r="A88" s="25" t="inlineStr">
-        <is>
-          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
-        </is>
-      </c>
+    <row r="88">
+      <c r="A88" s="25" t="inlineStr"/>
       <c r="B88" s="2" t="n"/>
       <c r="C88" s="2" t="n"/>
       <c r="D88" s="2" t="n"/>
@@ -10828,7 +10795,7 @@
     <row r="89" ht="39.7" customHeight="1">
       <c r="A89" s="25" t="inlineStr">
         <is>
-          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
+          <t>DATO DE CONTRASTE: la planilla de iluminacion y ventilacion da la superficie vidriada</t>
         </is>
       </c>
       <c r="B89" s="2" t="n"/>
@@ -10844,8 +10811,47 @@
       <c r="L89" s="2" t="n"/>
       <c r="M89" s="2" t="n"/>
     </row>
+    <row r="90" ht="39.7" customHeight="1">
+      <c r="A90" s="25" t="inlineStr">
+        <is>
+          <t>proyectada de cada local. La suma da 97,4 m2, que es el orden de magnitud que deberia</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="n"/>
+      <c r="C90" s="2" t="n"/>
+      <c r="D90" s="2" t="n"/>
+      <c r="E90" s="2" t="n"/>
+      <c r="F90" s="2" t="n"/>
+      <c r="G90" s="2" t="n"/>
+      <c r="H90" s="2" t="n"/>
+      <c r="I90" s="2" t="n"/>
+      <c r="J90" s="2" t="n"/>
+      <c r="K90" s="2" t="n"/>
+      <c r="L90" s="2" t="n"/>
+      <c r="M90" s="2" t="n"/>
+    </row>
+    <row r="91" ht="39.7" customHeight="1">
+      <c r="A91" s="25" t="inlineStr">
+        <is>
+          <t>dar el total de vanos de los cuatro planos. Sirve para controlar que no falte ninguno.</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="n"/>
+      <c r="C91" s="2" t="n"/>
+      <c r="D91" s="2" t="n"/>
+      <c r="E91" s="2" t="n"/>
+      <c r="F91" s="2" t="n"/>
+      <c r="G91" s="2" t="n"/>
+      <c r="H91" s="2" t="n"/>
+      <c r="I91" s="2" t="n"/>
+      <c r="J91" s="2" t="n"/>
+      <c r="K91" s="2" t="n"/>
+      <c r="L91" s="2" t="n"/>
+      <c r="M91" s="2" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A28:M28"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="A14:M14"/>
     <mergeCell ref="A6:M6"/>
@@ -10854,14 +10860,13 @@
     <mergeCell ref="B2:L2"/>
     <mergeCell ref="A4:M4"/>
     <mergeCell ref="E7:E13"/>
-    <mergeCell ref="E30:E37"/>
-    <mergeCell ref="A29:M29"/>
-    <mergeCell ref="E23:E28"/>
+    <mergeCell ref="E29:E36"/>
+    <mergeCell ref="E23:E27"/>
     <mergeCell ref="M1:M3"/>
     <mergeCell ref="B1:L1"/>
     <mergeCell ref="E15:E21"/>
   </mergeCells>
-  <conditionalFormatting sqref="M6:M37">
+  <conditionalFormatting sqref="M6:M36">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"CUMPLE"</formula>
     </cfRule>
@@ -10870,13 +10875,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="H6:H37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Datos_higro!$A$10:$A$17</formula1>
     </dataValidation>
-    <dataValidation sqref="I6:I37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I6:I36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Datos_higro!$A$21:$A$28</formula1>
     </dataValidation>
-    <dataValidation sqref="K6:K37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K6:K36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Norte,Sur,Este,Oeste,Noreste,Noroeste,Sudeste,Sudoeste,Horizontal"</formula1>
     </dataValidation>
   </dataValidations>
@@ -22806,7 +22811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I393"/>
+  <dimension ref="A1:I392"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.1" customWidth="1" min="1" max="1"/>
@@ -30219,60 +30224,60 @@
         <v>3</v>
       </c>
     </row>
-    <row r="335" ht="62" customHeight="1">
-      <c r="A335" s="10" t="n"/>
-      <c r="B335" s="36" t="inlineStr">
-        <is>
-          <t>PV04 (2)</t>
-        </is>
-      </c>
-      <c r="C335" s="10">
-        <f>IF(COUNT(H335,I335)&lt;2,"",TEXT(H335,"0.00")&amp;" x "&amp;TEXT(I335,"0.00"))</f>
-        <v/>
-      </c>
-      <c r="D335" s="9">
-        <f>IF(COUNT(H335,I335)&lt;2,"",ROUND(H335*I335,2))</f>
-        <v/>
-      </c>
-      <c r="E335" s="27" t="n">
-        <v>60</v>
-      </c>
-      <c r="F335" s="30">
-        <f>IF(D335="","",ROUND(D335*E335,1))</f>
-        <v/>
-      </c>
+    <row r="335" ht="39.7" customHeight="1">
+      <c r="A335" s="18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B335" s="35" t="inlineStr">
+        <is>
+          <t>PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C335" s="10" t="n"/>
+      <c r="D335" s="10" t="n"/>
+      <c r="E335" s="10" t="n"/>
+      <c r="F335" s="10" t="n"/>
       <c r="G335" s="2" t="n"/>
-      <c r="H335" s="37" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="I335" s="37" t="n">
-        <v>2.95</v>
-      </c>
-    </row>
-    <row r="336" ht="39.7" customHeight="1">
-      <c r="A336" s="18" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B336" s="35" t="inlineStr">
-        <is>
-          <t>PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C336" s="10" t="n"/>
-      <c r="D336" s="10" t="n"/>
-      <c r="E336" s="10" t="n"/>
-      <c r="F336" s="10" t="n"/>
+      <c r="H335" s="2" t="n"/>
+      <c r="I335" s="2" t="n"/>
+    </row>
+    <row r="336" ht="62" customHeight="1">
+      <c r="A336" s="10" t="n"/>
+      <c r="B336" s="36" t="inlineStr">
+        <is>
+          <t>AISLADAS (SE)</t>
+        </is>
+      </c>
+      <c r="C336" s="10">
+        <f>IF(COUNT(H336,I336)&lt;2,"",TEXT(H336,"0.00")&amp;" x "&amp;TEXT(I336,"0.00"))</f>
+        <v/>
+      </c>
+      <c r="D336" s="9">
+        <f>IF(COUNT(H336,I336)&lt;2,"",ROUND(H336*I336,2))</f>
+        <v/>
+      </c>
+      <c r="E336" s="27" t="n">
+        <v>20</v>
+      </c>
+      <c r="F336" s="30">
+        <f>IF(D336="","",ROUND(D336*E336,1))</f>
+        <v/>
+      </c>
       <c r="G336" s="2" t="n"/>
-      <c r="H336" s="2" t="n"/>
-      <c r="I336" s="2" t="n"/>
+      <c r="H336" s="37" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="I336" s="37" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="337" ht="62" customHeight="1">
       <c r="A337" s="10" t="n"/>
       <c r="B337" s="36" t="inlineStr">
         <is>
-          <t>AISLADAS (SE)</t>
+          <t>AISLADAS ()</t>
         </is>
       </c>
       <c r="C337" s="10">
@@ -30292,7 +30297,7 @@
       </c>
       <c r="G337" s="2" t="n"/>
       <c r="H337" s="37" t="n">
-        <v>4.05</v>
+        <v>3.5</v>
       </c>
       <c r="I337" s="37" t="n">
         <v>3</v>
@@ -30302,7 +30307,7 @@
       <c r="A338" s="10" t="n"/>
       <c r="B338" s="36" t="inlineStr">
         <is>
-          <t>AISLADAS ()</t>
+          <t>INTERIORES (    )</t>
         </is>
       </c>
       <c r="C338" s="10">
@@ -30314,7 +30319,7 @@
         <v/>
       </c>
       <c r="E338" s="27" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F338" s="30">
         <f>IF(D338="","",ROUND(D338*E338,1))</f>
@@ -30322,7 +30327,7 @@
       </c>
       <c r="G338" s="2" t="n"/>
       <c r="H338" s="37" t="n">
-        <v>3.5</v>
+        <v>4.05</v>
       </c>
       <c r="I338" s="37" t="n">
         <v>3</v>
@@ -30352,75 +30357,71 @@
       </c>
       <c r="G339" s="2" t="n"/>
       <c r="H339" s="37" t="n">
-        <v>4.05</v>
+        <v>3.5</v>
       </c>
       <c r="I339" s="37" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="340" ht="62" customHeight="1">
-      <c r="A340" s="10" t="n"/>
-      <c r="B340" s="36" t="inlineStr">
-        <is>
-          <t>INTERIORES (    )</t>
-        </is>
-      </c>
-      <c r="C340" s="10">
-        <f>IF(COUNT(H340,I340)&lt;2,"",TEXT(H340,"0.00")&amp;" x "&amp;TEXT(I340,"0.00"))</f>
-        <v/>
-      </c>
-      <c r="D340" s="9">
-        <f>IF(COUNT(H340,I340)&lt;2,"",ROUND(H340*I340,2))</f>
-        <v/>
-      </c>
-      <c r="E340" s="27" t="n">
-        <v>25</v>
-      </c>
-      <c r="F340" s="30">
-        <f>IF(D340="","",ROUND(D340*E340,1))</f>
-        <v/>
-      </c>
+    <row r="340" ht="39.7" customHeight="1">
+      <c r="A340" s="18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B340" s="35" t="inlineStr">
+        <is>
+          <t>TECHOS O CIELORRASOS</t>
+        </is>
+      </c>
+      <c r="C340" s="10" t="n"/>
+      <c r="D340" s="10" t="n"/>
+      <c r="E340" s="10" t="n"/>
+      <c r="F340" s="10" t="n"/>
       <c r="G340" s="2" t="n"/>
-      <c r="H340" s="37" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="I340" s="37" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="341" ht="39.7" customHeight="1">
-      <c r="A341" s="18" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B341" s="35" t="inlineStr">
-        <is>
-          <t>TECHOS O CIELORRASOS</t>
-        </is>
-      </c>
-      <c r="C341" s="10" t="n"/>
-      <c r="D341" s="10" t="n"/>
-      <c r="E341" s="10" t="n"/>
-      <c r="F341" s="10" t="n"/>
+      <c r="H340" s="2" t="n"/>
+      <c r="I340" s="2" t="n"/>
+    </row>
+    <row r="341" ht="62" customHeight="1">
+      <c r="A341" s="10" t="n"/>
+      <c r="B341" s="36" t="inlineStr">
+        <is>
+          <t>TECHO NO AISLADO</t>
+        </is>
+      </c>
+      <c r="C341" s="10" t="inlineStr"/>
+      <c r="D341" s="9">
+        <f>IF(COUNT(H341,I341)&lt;2,"",ROUND(H341*I341,2))</f>
+        <v/>
+      </c>
+      <c r="E341" s="27" t="n">
+        <v>30</v>
+      </c>
+      <c r="F341" s="30">
+        <f>IF(D341="","",ROUND(D341*E341,1))</f>
+        <v/>
+      </c>
       <c r="G341" s="2" t="n"/>
-      <c r="H341" s="2" t="n"/>
-      <c r="I341" s="2" t="n"/>
-    </row>
-    <row r="342" ht="62" customHeight="1">
+      <c r="H341" s="37" t="n"/>
+      <c r="I341" s="37" t="n"/>
+    </row>
+    <row r="342" ht="39.7" customHeight="1">
       <c r="A342" s="10" t="n"/>
       <c r="B342" s="36" t="inlineStr">
         <is>
-          <t>TECHO NO AISLADO</t>
-        </is>
-      </c>
-      <c r="C342" s="10" t="inlineStr"/>
-      <c r="D342" s="9">
-        <f>IF(COUNT(H342,I342)&lt;2,"",ROUND(H342*I342,2))</f>
-        <v/>
+          <t>TECHO AISLADO</t>
+        </is>
+      </c>
+      <c r="C342" s="10" t="inlineStr">
+        <is>
+          <t>por croquis</t>
+        </is>
+      </c>
+      <c r="D342" s="9" t="n">
+        <v>14.17</v>
       </c>
       <c r="E342" s="27" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F342" s="30">
         <f>IF(D342="","",ROUND(D342*E342,1))</f>
@@ -30430,23 +30431,20 @@
       <c r="H342" s="37" t="n"/>
       <c r="I342" s="37" t="n"/>
     </row>
-    <row r="343" ht="39.7" customHeight="1">
+    <row r="343" ht="62" customHeight="1">
       <c r="A343" s="10" t="n"/>
       <c r="B343" s="36" t="inlineStr">
         <is>
-          <t>TECHO AISLADO</t>
-        </is>
-      </c>
-      <c r="C343" s="10" t="inlineStr">
-        <is>
-          <t>por croquis</t>
-        </is>
-      </c>
-      <c r="D343" s="9" t="n">
-        <v>14.17</v>
+          <t>TECHO ENTREPISO</t>
+        </is>
+      </c>
+      <c r="C343" s="10" t="inlineStr"/>
+      <c r="D343" s="9">
+        <f>IF(COUNT(H343,I343)&lt;2,"",ROUND(H343*I343,2))</f>
+        <v/>
       </c>
       <c r="E343" s="27" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F343" s="30">
         <f>IF(D343="","",ROUND(D343*E343,1))</f>
@@ -30456,62 +30454,65 @@
       <c r="H343" s="37" t="n"/>
       <c r="I343" s="37" t="n"/>
     </row>
-    <row r="344" ht="62" customHeight="1">
-      <c r="A344" s="10" t="n"/>
-      <c r="B344" s="36" t="inlineStr">
-        <is>
-          <t>TECHO ENTREPISO</t>
-        </is>
-      </c>
-      <c r="C344" s="10" t="inlineStr"/>
-      <c r="D344" s="9">
-        <f>IF(COUNT(H344,I344)&lt;2,"",ROUND(H344*I344,2))</f>
-        <v/>
-      </c>
-      <c r="E344" s="27" t="n">
-        <v>15</v>
-      </c>
-      <c r="F344" s="30">
-        <f>IF(D344="","",ROUND(D344*E344,1))</f>
-        <v/>
-      </c>
+    <row r="344" ht="39.7" customHeight="1">
+      <c r="A344" s="18" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B344" s="35" t="inlineStr">
+        <is>
+          <t>PISO</t>
+        </is>
+      </c>
+      <c r="C344" s="10" t="n"/>
+      <c r="D344" s="10" t="n"/>
+      <c r="E344" s="10" t="n"/>
+      <c r="F344" s="10" t="n"/>
       <c r="G344" s="2" t="n"/>
-      <c r="H344" s="37" t="n"/>
-      <c r="I344" s="37" t="n"/>
-    </row>
-    <row r="345" ht="39.7" customHeight="1">
-      <c r="A345" s="18" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B345" s="35" t="inlineStr">
-        <is>
-          <t>PISO</t>
-        </is>
-      </c>
-      <c r="C345" s="10" t="n"/>
-      <c r="D345" s="10" t="n"/>
-      <c r="E345" s="10" t="n"/>
-      <c r="F345" s="10" t="n"/>
+      <c r="H344" s="2" t="n"/>
+      <c r="I344" s="2" t="n"/>
+    </row>
+    <row r="345" ht="62" customHeight="1">
+      <c r="A345" s="10" t="n"/>
+      <c r="B345" s="36" t="inlineStr">
+        <is>
+          <t>SOBRE TIERRA</t>
+        </is>
+      </c>
+      <c r="C345" s="10" t="inlineStr"/>
+      <c r="D345" s="9">
+        <f>IF(COUNT(H345,I345)&lt;2,"",ROUND(H345*I345,2))</f>
+        <v/>
+      </c>
+      <c r="E345" s="27" t="n">
+        <v>10</v>
+      </c>
+      <c r="F345" s="30">
+        <f>IF(D345="","",ROUND(D345*E345,1))</f>
+        <v/>
+      </c>
       <c r="G345" s="2" t="n"/>
-      <c r="H345" s="2" t="n"/>
-      <c r="I345" s="2" t="n"/>
-    </row>
-    <row r="346" ht="62" customHeight="1">
+      <c r="H345" s="37" t="n"/>
+      <c r="I345" s="37" t="n"/>
+    </row>
+    <row r="346" ht="39.7" customHeight="1">
       <c r="A346" s="10" t="n"/>
       <c r="B346" s="36" t="inlineStr">
         <is>
-          <t>SOBRE TIERRA</t>
-        </is>
-      </c>
-      <c r="C346" s="10" t="inlineStr"/>
-      <c r="D346" s="9">
-        <f>IF(COUNT(H346,I346)&lt;2,"",ROUND(H346*I346,2))</f>
-        <v/>
+          <t>SOBRE LOCAL OCUPADO</t>
+        </is>
+      </c>
+      <c r="C346" s="10" t="inlineStr">
+        <is>
+          <t>por croquis</t>
+        </is>
+      </c>
+      <c r="D346" s="9" t="n">
+        <v>14.17</v>
       </c>
       <c r="E346" s="27" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F346" s="30">
         <f>IF(D346="","",ROUND(D346*E346,1))</f>
@@ -30522,68 +30523,68 @@
       <c r="I346" s="37" t="n"/>
     </row>
     <row r="347" ht="39.7" customHeight="1">
-      <c r="A347" s="10" t="n"/>
-      <c r="B347" s="36" t="inlineStr">
-        <is>
-          <t>SOBRE LOCAL OCUPADO</t>
-        </is>
-      </c>
-      <c r="C347" s="10" t="inlineStr">
-        <is>
-          <t>por croquis</t>
-        </is>
-      </c>
-      <c r="D347" s="9" t="n">
-        <v>14.17</v>
-      </c>
-      <c r="E347" s="27" t="n">
-        <v>15</v>
-      </c>
-      <c r="F347" s="30">
-        <f>IF(D347="","",ROUND(D347*E347,1))</f>
-        <v/>
-      </c>
+      <c r="A347" s="18" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B347" s="35" t="inlineStr">
+        <is>
+          <t>INFILTRACION</t>
+        </is>
+      </c>
+      <c r="C347" s="10" t="n"/>
+      <c r="D347" s="18" t="inlineStr">
+        <is>
+          <t>VOLUMEN (m3)</t>
+        </is>
+      </c>
+      <c r="E347" s="10" t="n"/>
+      <c r="F347" s="10" t="n"/>
       <c r="G347" s="2" t="n"/>
-      <c r="H347" s="37" t="n"/>
-      <c r="I347" s="37" t="n"/>
-    </row>
-    <row r="348" ht="39.7" customHeight="1">
-      <c r="A348" s="18" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B348" s="35" t="inlineStr">
-        <is>
-          <t>INFILTRACION</t>
-        </is>
-      </c>
-      <c r="C348" s="10" t="n"/>
-      <c r="D348" s="18" t="inlineStr">
-        <is>
-          <t>VOLUMEN (m3)</t>
-        </is>
-      </c>
-      <c r="E348" s="10" t="n"/>
-      <c r="F348" s="10" t="n"/>
+      <c r="H347" s="2" t="n"/>
+      <c r="I347" s="2" t="n"/>
+    </row>
+    <row r="348" ht="62" customHeight="1">
+      <c r="A348" s="10" t="n"/>
+      <c r="B348" s="36" t="inlineStr">
+        <is>
+          <t>UNA PARED EXTERIOR</t>
+        </is>
+      </c>
+      <c r="C348" s="10" t="inlineStr"/>
+      <c r="D348" s="9">
+        <f>IF(COUNT(H348,I348)&lt;2,"",ROUND(H348*I348,2))</f>
+        <v/>
+      </c>
+      <c r="E348" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="F348" s="30">
+        <f>IF(D348="","",ROUND(D348*E348,1))</f>
+        <v/>
+      </c>
       <c r="G348" s="2" t="n"/>
-      <c r="H348" s="2" t="n"/>
-      <c r="I348" s="2" t="n"/>
-    </row>
-    <row r="349" ht="62" customHeight="1">
+      <c r="H348" s="37" t="n"/>
+      <c r="I348" s="37" t="n"/>
+    </row>
+    <row r="349" ht="39.7" customHeight="1">
       <c r="A349" s="10" t="n"/>
       <c r="B349" s="36" t="inlineStr">
         <is>
-          <t>UNA PARED EXTERIOR</t>
-        </is>
-      </c>
-      <c r="C349" s="10" t="inlineStr"/>
-      <c r="D349" s="9">
-        <f>IF(COUNT(H349,I349)&lt;2,"",ROUND(H349*I349,2))</f>
-        <v/>
+          <t>DOS PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C349" s="10" t="inlineStr">
+        <is>
+          <t>14.17 m2 x 3.00</t>
+        </is>
+      </c>
+      <c r="D349" s="9" t="n">
+        <v>42.51</v>
       </c>
       <c r="E349" s="27" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F349" s="30">
         <f>IF(D349="","",ROUND(D349*E349,1))</f>
@@ -30593,23 +30594,20 @@
       <c r="H349" s="37" t="n"/>
       <c r="I349" s="37" t="n"/>
     </row>
-    <row r="350" ht="39.7" customHeight="1">
+    <row r="350" ht="62" customHeight="1">
       <c r="A350" s="10" t="n"/>
       <c r="B350" s="36" t="inlineStr">
         <is>
-          <t>DOS PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C350" s="10" t="inlineStr">
-        <is>
-          <t>14.17 m2 x 3.00</t>
-        </is>
-      </c>
-      <c r="D350" s="9" t="n">
-        <v>42.51</v>
+          <t>TRES O MAS PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C350" s="10" t="inlineStr"/>
+      <c r="D350" s="9">
+        <f>IF(COUNT(H350,I350)&lt;2,"",ROUND(H350*I350,2))</f>
+        <v/>
       </c>
       <c r="E350" s="27" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F350" s="30">
         <f>IF(D350="","",ROUND(D350*E350,1))</f>
@@ -30619,129 +30617,124 @@
       <c r="H350" s="37" t="n"/>
       <c r="I350" s="37" t="n"/>
     </row>
-    <row r="351" ht="62" customHeight="1">
-      <c r="A351" s="10" t="n"/>
-      <c r="B351" s="36" t="inlineStr">
-        <is>
-          <t>TRES O MAS PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C351" s="10" t="inlineStr"/>
-      <c r="D351" s="9">
-        <f>IF(COUNT(H351,I351)&lt;2,"",ROUND(H351*I351,2))</f>
-        <v/>
-      </c>
-      <c r="E351" s="27" t="n">
-        <v>12</v>
-      </c>
-      <c r="F351" s="30">
-        <f>IF(D351="","",ROUND(D351*E351,1))</f>
+    <row r="351" ht="70" customHeight="1">
+      <c r="A351" s="18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B351" s="35" t="inlineStr">
+        <is>
+          <t>SUBTOTAL</t>
+        </is>
+      </c>
+      <c r="C351" s="10" t="n"/>
+      <c r="D351" s="10" t="n"/>
+      <c r="E351" s="10" t="n"/>
+      <c r="F351" s="38">
+        <f>IF(F334="",0,F334)+IF(F336="",0,F336)+IF(F337="",0,F337)+IF(F338="",0,F338)+IF(F339="",0,F339)+IF(F341="",0,F341)+IF(F342="",0,F342)+IF(F343="",0,F343)+IF(F345="",0,F345)+IF(F346="",0,F346)+IF(F348="",0,F348)+IF(F349="",0,F349)+IF(F350="",0,F350)</f>
         <v/>
       </c>
       <c r="G351" s="2" t="n"/>
-      <c r="H351" s="37" t="n"/>
-      <c r="I351" s="37" t="n"/>
-    </row>
-    <row r="352" ht="70" customHeight="1">
+      <c r="H351" s="2" t="n"/>
+      <c r="I351" s="2" t="n"/>
+    </row>
+    <row r="352" ht="47" customHeight="1">
       <c r="A352" s="18" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B352" s="35" t="inlineStr">
         <is>
-          <t>SUBTOTAL</t>
-        </is>
-      </c>
-      <c r="C352" s="10" t="n"/>
-      <c r="D352" s="10" t="n"/>
-      <c r="E352" s="10" t="n"/>
+          <t>PERDIDA TOTAL</t>
+        </is>
+      </c>
+      <c r="C352" s="10">
+        <f>TEXT(F351,"0.00")&amp;"  X  "&amp;Datos_balance!$B$4&amp;" (FI)  X  "&amp;Datos_balance!$B$5&amp;" (FO)  X  "&amp;Datos_balance!$B$6&amp;" (FZ)"</f>
+        <v/>
+      </c>
+      <c r="D352" s="2" t="n"/>
+      <c r="E352" s="2" t="n"/>
       <c r="F352" s="38">
-        <f>IF(F334="",0,F334)+IF(F335="",0,F335)+IF(F337="",0,F337)+IF(F338="",0,F338)+IF(F339="",0,F339)+IF(F340="",0,F340)+IF(F342="",0,F342)+IF(F343="",0,F343)+IF(F344="",0,F344)+IF(F346="",0,F346)+IF(F347="",0,F347)+IF(F349="",0,F349)+IF(F350="",0,F350)+IF(F351="",0,F351)</f>
+        <f>ROUND(F351*Datos_balance!$B$4*Datos_balance!$B$5*Datos_balance!$B$6,1)</f>
         <v/>
       </c>
       <c r="G352" s="2" t="n"/>
       <c r="H352" s="2" t="n"/>
       <c r="I352" s="2" t="n"/>
     </row>
-    <row r="353" ht="47" customHeight="1">
-      <c r="A353" s="18" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B353" s="35" t="inlineStr">
-        <is>
-          <t>PERDIDA TOTAL</t>
-        </is>
-      </c>
-      <c r="C353" s="10">
-        <f>TEXT(F352,"0.00")&amp;"  X  "&amp;Datos_balance!$B$4&amp;" (FI)  X  "&amp;Datos_balance!$B$5&amp;" (FO)  X  "&amp;Datos_balance!$B$6&amp;" (FZ)"</f>
-        <v/>
-      </c>
+    <row r="353" ht="39.7" customHeight="1">
+      <c r="A353" s="10" t="n"/>
+      <c r="B353" s="11" t="inlineStr">
+        <is>
+          <t>Carga de locales sin emisor</t>
+        </is>
+      </c>
+      <c r="C353" s="10" t="n"/>
       <c r="D353" s="2" t="n"/>
       <c r="E353" s="2" t="n"/>
-      <c r="F353" s="38">
-        <f>ROUND(F352*Datos_balance!$B$4*Datos_balance!$B$5*Datos_balance!$B$6,1)</f>
-        <v/>
-      </c>
+      <c r="F353" s="30" t="n"/>
       <c r="G353" s="2" t="n"/>
       <c r="H353" s="2" t="n"/>
       <c r="I353" s="2" t="n"/>
     </row>
     <row r="354" ht="39.7" customHeight="1">
       <c r="A354" s="10" t="n"/>
-      <c r="B354" s="11" t="inlineStr">
-        <is>
-          <t>Carga de locales sin emisor</t>
+      <c r="B354" s="35" t="inlineStr">
+        <is>
+          <t>CARGA TOTAL A CUBRIR</t>
         </is>
       </c>
       <c r="C354" s="10" t="n"/>
       <c r="D354" s="2" t="n"/>
       <c r="E354" s="2" t="n"/>
-      <c r="F354" s="30" t="n"/>
+      <c r="F354" s="38">
+        <f>F352+IF(F353="",0,F353)</f>
+        <v/>
+      </c>
       <c r="G354" s="2" t="n"/>
       <c r="H354" s="2" t="n"/>
       <c r="I354" s="2" t="n"/>
     </row>
-    <row r="355" ht="39.7" customHeight="1">
-      <c r="A355" s="10" t="n"/>
-      <c r="B355" s="35" t="inlineStr">
-        <is>
-          <t>CARGA TOTAL A CUBRIR</t>
-        </is>
-      </c>
-      <c r="C355" s="10" t="n"/>
+    <row r="355">
+      <c r="A355" s="2" t="n"/>
+      <c r="B355" s="2" t="n"/>
+      <c r="C355" s="2" t="n"/>
       <c r="D355" s="2" t="n"/>
       <c r="E355" s="2" t="n"/>
-      <c r="F355" s="38">
-        <f>F353+IF(F354="",0,F354)</f>
-        <v/>
-      </c>
+      <c r="F355" s="2" t="n"/>
       <c r="G355" s="2" t="n"/>
       <c r="H355" s="2" t="n"/>
       <c r="I355" s="2" t="n"/>
     </row>
-    <row r="356">
-      <c r="A356" s="2" t="n"/>
-      <c r="B356" s="2" t="n"/>
-      <c r="C356" s="2" t="n"/>
+    <row r="356" ht="62" customHeight="1">
+      <c r="A356" s="10" t="n"/>
+      <c r="B356" s="11" t="inlineStr">
+        <is>
+          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
+        </is>
+      </c>
+      <c r="C356" s="10">
+        <f>TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2,"0")&amp;" - "&amp;TEXT(Datos_balance!$B$11,"0")&amp;" = "&amp;TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2-Datos_balance!$B$11,"0")&amp;" C"</f>
+        <v/>
+      </c>
       <c r="D356" s="2" t="n"/>
       <c r="E356" s="2" t="n"/>
-      <c r="F356" s="2" t="n"/>
+      <c r="F356" s="10" t="n"/>
       <c r="G356" s="2" t="n"/>
       <c r="H356" s="2" t="n"/>
       <c r="I356" s="2" t="n"/>
     </row>
-    <row r="357" ht="62" customHeight="1">
+    <row r="357" ht="39.7" customHeight="1">
       <c r="A357" s="10" t="n"/>
       <c r="B357" s="11" t="inlineStr">
         <is>
-          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
-        </is>
-      </c>
-      <c r="C357" s="10">
-        <f>TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2,"0")&amp;" - "&amp;TEXT(Datos_balance!$B$11,"0")&amp;" = "&amp;TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2-Datos_balance!$B$11,"0")&amp;" C"</f>
+          <t>Kcal/h por elemento</t>
+        </is>
+      </c>
+      <c r="C357" s="9">
+        <f>ROUND(Datos_balance!$B$14*Datos_balance!$B$15,2)</f>
         <v/>
       </c>
       <c r="D357" s="2" t="n"/>
@@ -30755,11 +30748,11 @@
       <c r="A358" s="10" t="n"/>
       <c r="B358" s="11" t="inlineStr">
         <is>
-          <t>Kcal/h por elemento</t>
-        </is>
-      </c>
-      <c r="C358" s="9">
-        <f>ROUND(Datos_balance!$B$14*Datos_balance!$B$15,2)</f>
+          <t>Elementos necesarios</t>
+        </is>
+      </c>
+      <c r="C358" s="27">
+        <f>ROUNDUP(F354/(Datos_balance!$B$14*Datos_balance!$B$15),0)</f>
         <v/>
       </c>
       <c r="D358" s="2" t="n"/>
@@ -30773,11 +30766,11 @@
       <c r="A359" s="10" t="n"/>
       <c r="B359" s="11" t="inlineStr">
         <is>
-          <t>Elementos necesarios</t>
+          <t>Ancho del radiador (cm)</t>
         </is>
       </c>
       <c r="C359" s="27">
-        <f>ROUNDUP(F355/(Datos_balance!$B$14*Datos_balance!$B$15),0)</f>
+        <f>ROUNDUP(F354/(Datos_balance!$B$14*Datos_balance!$B$15),0)*Datos_balance!$B$16</f>
         <v/>
       </c>
       <c r="D359" s="2" t="n"/>
@@ -30788,37 +30781,30 @@
       <c r="I359" s="2" t="n"/>
     </row>
     <row r="360" ht="39.7" customHeight="1">
-      <c r="A360" s="10" t="n"/>
-      <c r="B360" s="11" t="inlineStr">
-        <is>
-          <t>Ancho del radiador (cm)</t>
-        </is>
-      </c>
-      <c r="C360" s="27">
-        <f>ROUNDUP(F355/(Datos_balance!$B$14*Datos_balance!$B$15),0)*Datos_balance!$B$16</f>
-        <v/>
-      </c>
-      <c r="D360" s="2" t="n"/>
-      <c r="E360" s="2" t="n"/>
-      <c r="F360" s="10" t="n"/>
+      <c r="A360" s="14" t="n"/>
+      <c r="B360" s="15" t="inlineStr">
+        <is>
+          <t>Radiador adoptado</t>
+        </is>
+      </c>
+      <c r="C360" s="14">
+        <f>Datos_balance!$B$13</f>
+        <v/>
+      </c>
+      <c r="D360" s="22" t="n"/>
+      <c r="E360" s="22" t="n"/>
+      <c r="F360" s="14" t="n"/>
       <c r="G360" s="2" t="n"/>
       <c r="H360" s="2" t="n"/>
       <c r="I360" s="2" t="n"/>
     </row>
-    <row r="361" ht="39.7" customHeight="1">
-      <c r="A361" s="14" t="n"/>
-      <c r="B361" s="15" t="inlineStr">
-        <is>
-          <t>Radiador adoptado</t>
-        </is>
-      </c>
-      <c r="C361" s="14">
-        <f>Datos_balance!$B$13</f>
-        <v/>
-      </c>
-      <c r="D361" s="22" t="n"/>
-      <c r="E361" s="22" t="n"/>
-      <c r="F361" s="14" t="n"/>
+    <row r="361">
+      <c r="A361" s="2" t="n"/>
+      <c r="B361" s="2" t="n"/>
+      <c r="C361" s="2" t="n"/>
+      <c r="D361" s="2" t="n"/>
+      <c r="E361" s="2" t="n"/>
+      <c r="F361" s="2" t="n"/>
       <c r="G361" s="2" t="n"/>
       <c r="H361" s="2" t="n"/>
       <c r="I361" s="2" t="n"/>
@@ -30834,8 +30820,12 @@
       <c r="H362" s="2" t="n"/>
       <c r="I362" s="2" t="n"/>
     </row>
-    <row r="363">
-      <c r="A363" s="2" t="n"/>
+    <row r="363" ht="39.7" customHeight="1">
+      <c r="A363" s="5" t="inlineStr">
+        <is>
+          <t>LOCAL  17 - Bano   (PA)   -   altura 3.00 m</t>
+        </is>
+      </c>
       <c r="B363" s="2" t="n"/>
       <c r="C363" s="2" t="n"/>
       <c r="D363" s="2" t="n"/>
@@ -30846,122 +30836,137 @@
       <c r="I363" s="2" t="n"/>
     </row>
     <row r="364" ht="39.7" customHeight="1">
-      <c r="A364" s="5" t="inlineStr">
-        <is>
-          <t>LOCAL  17 - Bano   (PA)   -   altura 3.00 m</t>
-        </is>
-      </c>
-      <c r="B364" s="2" t="n"/>
-      <c r="C364" s="2" t="n"/>
-      <c r="D364" s="2" t="n"/>
-      <c r="E364" s="2" t="n"/>
-      <c r="F364" s="2" t="n"/>
+      <c r="A364" s="3" t="inlineStr">
+        <is>
+          <t>Nro</t>
+        </is>
+      </c>
+      <c r="B364" s="3" t="inlineStr">
+        <is>
+          <t>DESCRIPCION</t>
+        </is>
+      </c>
+      <c r="C364" s="3" t="inlineStr">
+        <is>
+          <t>DIMENSIONES (m)</t>
+        </is>
+      </c>
+      <c r="D364" s="3" t="inlineStr">
+        <is>
+          <t>AREA (m2)</t>
+        </is>
+      </c>
+      <c r="E364" s="3" t="inlineStr">
+        <is>
+          <t>FACTOR</t>
+        </is>
+      </c>
+      <c r="F364" s="3" t="inlineStr">
+        <is>
+          <t>PERDIDA CALOR (Kcal/h)</t>
+        </is>
+      </c>
       <c r="G364" s="2" t="n"/>
       <c r="H364" s="2" t="n"/>
       <c r="I364" s="2" t="n"/>
     </row>
     <row r="365" ht="39.7" customHeight="1">
-      <c r="A365" s="3" t="inlineStr">
-        <is>
-          <t>Nro</t>
-        </is>
-      </c>
-      <c r="B365" s="3" t="inlineStr">
-        <is>
-          <t>DESCRIPCION</t>
-        </is>
-      </c>
-      <c r="C365" s="3" t="inlineStr">
-        <is>
-          <t>DIMENSIONES (m)</t>
-        </is>
-      </c>
-      <c r="D365" s="3" t="inlineStr">
-        <is>
-          <t>AREA (m2)</t>
-        </is>
-      </c>
-      <c r="E365" s="3" t="inlineStr">
-        <is>
-          <t>FACTOR</t>
-        </is>
-      </c>
-      <c r="F365" s="3" t="inlineStr">
-        <is>
-          <t>PERDIDA CALOR (Kcal/h)</t>
-        </is>
-      </c>
+      <c r="A365" s="18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B365" s="35" t="inlineStr">
+        <is>
+          <t>VENTANA</t>
+        </is>
+      </c>
+      <c r="C365" s="10" t="n"/>
+      <c r="D365" s="10" t="n"/>
+      <c r="E365" s="10" t="n"/>
+      <c r="F365" s="10" t="n"/>
       <c r="G365" s="2" t="n"/>
       <c r="H365" s="2" t="n"/>
       <c r="I365" s="2" t="n"/>
     </row>
-    <row r="366" ht="39.7" customHeight="1">
-      <c r="A366" s="18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B366" s="35" t="inlineStr">
-        <is>
-          <t>VENTANA</t>
-        </is>
-      </c>
-      <c r="C366" s="10" t="n"/>
-      <c r="D366" s="10" t="n"/>
-      <c r="E366" s="10" t="n"/>
-      <c r="F366" s="10" t="n"/>
+    <row r="366" ht="62" customHeight="1">
+      <c r="A366" s="10" t="n"/>
+      <c r="B366" s="36" t="inlineStr">
+        <is>
+          <t>VA03</t>
+        </is>
+      </c>
+      <c r="C366" s="10">
+        <f>IF(COUNT(H366,I366)&lt;2,"",TEXT(H366,"0.00")&amp;" x "&amp;TEXT(I366,"0.00"))</f>
+        <v/>
+      </c>
+      <c r="D366" s="9">
+        <f>IF(COUNT(H366,I366)&lt;2,"",ROUND(H366*I366,2))</f>
+        <v/>
+      </c>
+      <c r="E366" s="27" t="n">
+        <v>60</v>
+      </c>
+      <c r="F366" s="30">
+        <f>IF(D366="","",ROUND(D366*E366,1))</f>
+        <v/>
+      </c>
       <c r="G366" s="2" t="n"/>
-      <c r="H366" s="2" t="n"/>
-      <c r="I366" s="2" t="n"/>
-    </row>
-    <row r="367" ht="62" customHeight="1">
-      <c r="A367" s="10" t="n"/>
-      <c r="B367" s="36" t="inlineStr">
-        <is>
-          <t>VA03</t>
-        </is>
-      </c>
-      <c r="C367" s="10">
-        <f>IF(COUNT(H367,I367)&lt;2,"",TEXT(H367,"0.00")&amp;" x "&amp;TEXT(I367,"0.00"))</f>
-        <v/>
-      </c>
-      <c r="D367" s="9">
-        <f>IF(COUNT(H367,I367)&lt;2,"",ROUND(H367*I367,2))</f>
-        <v/>
-      </c>
-      <c r="E367" s="27" t="n">
-        <v>60</v>
-      </c>
-      <c r="F367" s="30">
-        <f>IF(D367="","",ROUND(D367*E367,1))</f>
-        <v/>
-      </c>
+      <c r="H366" s="37" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I366" s="37" t="n">
+        <v>2.52</v>
+      </c>
+    </row>
+    <row r="367" ht="39.7" customHeight="1">
+      <c r="A367" s="18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B367" s="35" t="inlineStr">
+        <is>
+          <t>PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C367" s="10" t="n"/>
+      <c r="D367" s="10" t="n"/>
+      <c r="E367" s="10" t="n"/>
+      <c r="F367" s="10" t="n"/>
       <c r="G367" s="2" t="n"/>
-      <c r="H367" s="37" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="I367" s="37" t="n">
-        <v>2.52</v>
-      </c>
-    </row>
-    <row r="368" ht="39.7" customHeight="1">
-      <c r="A368" s="18" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B368" s="35" t="inlineStr">
-        <is>
-          <t>PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C368" s="10" t="n"/>
-      <c r="D368" s="10" t="n"/>
-      <c r="E368" s="10" t="n"/>
-      <c r="F368" s="10" t="n"/>
+      <c r="H367" s="2" t="n"/>
+      <c r="I367" s="2" t="n"/>
+    </row>
+    <row r="368" ht="62" customHeight="1">
+      <c r="A368" s="10" t="n"/>
+      <c r="B368" s="36" t="inlineStr">
+        <is>
+          <t>AISLADAS ()</t>
+        </is>
+      </c>
+      <c r="C368" s="10">
+        <f>IF(COUNT(H368,I368)&lt;2,"",TEXT(H368,"0.00")&amp;" x "&amp;TEXT(I368,"0.00"))</f>
+        <v/>
+      </c>
+      <c r="D368" s="9">
+        <f>IF(COUNT(H368,I368)&lt;2,"",ROUND(H368*I368,2))</f>
+        <v/>
+      </c>
+      <c r="E368" s="27" t="n">
+        <v>20</v>
+      </c>
+      <c r="F368" s="30">
+        <f>IF(D368="","",ROUND(D368*E368,1))</f>
+        <v/>
+      </c>
       <c r="G368" s="2" t="n"/>
-      <c r="H368" s="2" t="n"/>
-      <c r="I368" s="2" t="n"/>
+      <c r="H368" s="37" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="I368" s="37" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="369" ht="62" customHeight="1">
       <c r="A369" s="10" t="n"/>
@@ -30987,7 +30992,7 @@
       </c>
       <c r="G369" s="2" t="n"/>
       <c r="H369" s="37" t="n">
-        <v>2.2</v>
+        <v>1.6</v>
       </c>
       <c r="I369" s="37" t="n">
         <v>3</v>
@@ -30997,7 +31002,7 @@
       <c r="A370" s="10" t="n"/>
       <c r="B370" s="36" t="inlineStr">
         <is>
-          <t>AISLADAS ()</t>
+          <t>INTERIORES (    )</t>
         </is>
       </c>
       <c r="C370" s="10">
@@ -31009,7 +31014,7 @@
         <v/>
       </c>
       <c r="E370" s="27" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F370" s="30">
         <f>IF(D370="","",ROUND(D370*E370,1))</f>
@@ -31017,7 +31022,7 @@
       </c>
       <c r="G370" s="2" t="n"/>
       <c r="H370" s="37" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="I370" s="37" t="n">
         <v>3</v>
@@ -31047,75 +31052,71 @@
       </c>
       <c r="G371" s="2" t="n"/>
       <c r="H371" s="37" t="n">
-        <v>2.2</v>
+        <v>1.6</v>
       </c>
       <c r="I371" s="37" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="372" ht="62" customHeight="1">
-      <c r="A372" s="10" t="n"/>
-      <c r="B372" s="36" t="inlineStr">
-        <is>
-          <t>INTERIORES (    )</t>
-        </is>
-      </c>
-      <c r="C372" s="10">
-        <f>IF(COUNT(H372,I372)&lt;2,"",TEXT(H372,"0.00")&amp;" x "&amp;TEXT(I372,"0.00"))</f>
-        <v/>
-      </c>
-      <c r="D372" s="9">
-        <f>IF(COUNT(H372,I372)&lt;2,"",ROUND(H372*I372,2))</f>
-        <v/>
-      </c>
-      <c r="E372" s="27" t="n">
-        <v>25</v>
-      </c>
-      <c r="F372" s="30">
-        <f>IF(D372="","",ROUND(D372*E372,1))</f>
-        <v/>
-      </c>
+    <row r="372" ht="39.7" customHeight="1">
+      <c r="A372" s="18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B372" s="35" t="inlineStr">
+        <is>
+          <t>TECHOS O CIELORRASOS</t>
+        </is>
+      </c>
+      <c r="C372" s="10" t="n"/>
+      <c r="D372" s="10" t="n"/>
+      <c r="E372" s="10" t="n"/>
+      <c r="F372" s="10" t="n"/>
       <c r="G372" s="2" t="n"/>
-      <c r="H372" s="37" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="I372" s="37" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="373" ht="39.7" customHeight="1">
-      <c r="A373" s="18" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B373" s="35" t="inlineStr">
-        <is>
-          <t>TECHOS O CIELORRASOS</t>
-        </is>
-      </c>
-      <c r="C373" s="10" t="n"/>
-      <c r="D373" s="10" t="n"/>
-      <c r="E373" s="10" t="n"/>
-      <c r="F373" s="10" t="n"/>
+      <c r="H372" s="2" t="n"/>
+      <c r="I372" s="2" t="n"/>
+    </row>
+    <row r="373" ht="62" customHeight="1">
+      <c r="A373" s="10" t="n"/>
+      <c r="B373" s="36" t="inlineStr">
+        <is>
+          <t>TECHO NO AISLADO</t>
+        </is>
+      </c>
+      <c r="C373" s="10" t="inlineStr"/>
+      <c r="D373" s="9">
+        <f>IF(COUNT(H373,I373)&lt;2,"",ROUND(H373*I373,2))</f>
+        <v/>
+      </c>
+      <c r="E373" s="27" t="n">
+        <v>30</v>
+      </c>
+      <c r="F373" s="30">
+        <f>IF(D373="","",ROUND(D373*E373,1))</f>
+        <v/>
+      </c>
       <c r="G373" s="2" t="n"/>
-      <c r="H373" s="2" t="n"/>
-      <c r="I373" s="2" t="n"/>
-    </row>
-    <row r="374" ht="62" customHeight="1">
+      <c r="H373" s="37" t="n"/>
+      <c r="I373" s="37" t="n"/>
+    </row>
+    <row r="374" ht="39.7" customHeight="1">
       <c r="A374" s="10" t="n"/>
       <c r="B374" s="36" t="inlineStr">
         <is>
-          <t>TECHO NO AISLADO</t>
-        </is>
-      </c>
-      <c r="C374" s="10" t="inlineStr"/>
-      <c r="D374" s="9">
-        <f>IF(COUNT(H374,I374)&lt;2,"",ROUND(H374*I374,2))</f>
-        <v/>
+          <t>TECHO AISLADO</t>
+        </is>
+      </c>
+      <c r="C374" s="10" t="inlineStr">
+        <is>
+          <t>por croquis</t>
+        </is>
+      </c>
+      <c r="D374" s="9" t="n">
+        <v>3.52</v>
       </c>
       <c r="E374" s="27" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F374" s="30">
         <f>IF(D374="","",ROUND(D374*E374,1))</f>
@@ -31125,23 +31126,20 @@
       <c r="H374" s="37" t="n"/>
       <c r="I374" s="37" t="n"/>
     </row>
-    <row r="375" ht="39.7" customHeight="1">
+    <row r="375" ht="62" customHeight="1">
       <c r="A375" s="10" t="n"/>
       <c r="B375" s="36" t="inlineStr">
         <is>
-          <t>TECHO AISLADO</t>
-        </is>
-      </c>
-      <c r="C375" s="10" t="inlineStr">
-        <is>
-          <t>por croquis</t>
-        </is>
-      </c>
-      <c r="D375" s="9" t="n">
-        <v>3.52</v>
+          <t>TECHO ENTREPISO</t>
+        </is>
+      </c>
+      <c r="C375" s="10" t="inlineStr"/>
+      <c r="D375" s="9">
+        <f>IF(COUNT(H375,I375)&lt;2,"",ROUND(H375*I375,2))</f>
+        <v/>
       </c>
       <c r="E375" s="27" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F375" s="30">
         <f>IF(D375="","",ROUND(D375*E375,1))</f>
@@ -31151,62 +31149,65 @@
       <c r="H375" s="37" t="n"/>
       <c r="I375" s="37" t="n"/>
     </row>
-    <row r="376" ht="62" customHeight="1">
-      <c r="A376" s="10" t="n"/>
-      <c r="B376" s="36" t="inlineStr">
-        <is>
-          <t>TECHO ENTREPISO</t>
-        </is>
-      </c>
-      <c r="C376" s="10" t="inlineStr"/>
-      <c r="D376" s="9">
-        <f>IF(COUNT(H376,I376)&lt;2,"",ROUND(H376*I376,2))</f>
-        <v/>
-      </c>
-      <c r="E376" s="27" t="n">
-        <v>15</v>
-      </c>
-      <c r="F376" s="30">
-        <f>IF(D376="","",ROUND(D376*E376,1))</f>
-        <v/>
-      </c>
+    <row r="376" ht="39.7" customHeight="1">
+      <c r="A376" s="18" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B376" s="35" t="inlineStr">
+        <is>
+          <t>PISO</t>
+        </is>
+      </c>
+      <c r="C376" s="10" t="n"/>
+      <c r="D376" s="10" t="n"/>
+      <c r="E376" s="10" t="n"/>
+      <c r="F376" s="10" t="n"/>
       <c r="G376" s="2" t="n"/>
-      <c r="H376" s="37" t="n"/>
-      <c r="I376" s="37" t="n"/>
-    </row>
-    <row r="377" ht="39.7" customHeight="1">
-      <c r="A377" s="18" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B377" s="35" t="inlineStr">
-        <is>
-          <t>PISO</t>
-        </is>
-      </c>
-      <c r="C377" s="10" t="n"/>
-      <c r="D377" s="10" t="n"/>
-      <c r="E377" s="10" t="n"/>
-      <c r="F377" s="10" t="n"/>
+      <c r="H376" s="2" t="n"/>
+      <c r="I376" s="2" t="n"/>
+    </row>
+    <row r="377" ht="62" customHeight="1">
+      <c r="A377" s="10" t="n"/>
+      <c r="B377" s="36" t="inlineStr">
+        <is>
+          <t>SOBRE TIERRA</t>
+        </is>
+      </c>
+      <c r="C377" s="10" t="inlineStr"/>
+      <c r="D377" s="9">
+        <f>IF(COUNT(H377,I377)&lt;2,"",ROUND(H377*I377,2))</f>
+        <v/>
+      </c>
+      <c r="E377" s="27" t="n">
+        <v>10</v>
+      </c>
+      <c r="F377" s="30">
+        <f>IF(D377="","",ROUND(D377*E377,1))</f>
+        <v/>
+      </c>
       <c r="G377" s="2" t="n"/>
-      <c r="H377" s="2" t="n"/>
-      <c r="I377" s="2" t="n"/>
-    </row>
-    <row r="378" ht="62" customHeight="1">
+      <c r="H377" s="37" t="n"/>
+      <c r="I377" s="37" t="n"/>
+    </row>
+    <row r="378" ht="39.7" customHeight="1">
       <c r="A378" s="10" t="n"/>
       <c r="B378" s="36" t="inlineStr">
         <is>
-          <t>SOBRE TIERRA</t>
-        </is>
-      </c>
-      <c r="C378" s="10" t="inlineStr"/>
-      <c r="D378" s="9">
-        <f>IF(COUNT(H378,I378)&lt;2,"",ROUND(H378*I378,2))</f>
-        <v/>
+          <t>SOBRE LOCAL OCUPADO</t>
+        </is>
+      </c>
+      <c r="C378" s="10" t="inlineStr">
+        <is>
+          <t>por croquis</t>
+        </is>
+      </c>
+      <c r="D378" s="9" t="n">
+        <v>3.52</v>
       </c>
       <c r="E378" s="27" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F378" s="30">
         <f>IF(D378="","",ROUND(D378*E378,1))</f>
@@ -31217,68 +31218,68 @@
       <c r="I378" s="37" t="n"/>
     </row>
     <row r="379" ht="39.7" customHeight="1">
-      <c r="A379" s="10" t="n"/>
-      <c r="B379" s="36" t="inlineStr">
-        <is>
-          <t>SOBRE LOCAL OCUPADO</t>
-        </is>
-      </c>
-      <c r="C379" s="10" t="inlineStr">
-        <is>
-          <t>por croquis</t>
-        </is>
-      </c>
-      <c r="D379" s="9" t="n">
-        <v>3.52</v>
-      </c>
-      <c r="E379" s="27" t="n">
-        <v>15</v>
-      </c>
-      <c r="F379" s="30">
-        <f>IF(D379="","",ROUND(D379*E379,1))</f>
-        <v/>
-      </c>
+      <c r="A379" s="18" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B379" s="35" t="inlineStr">
+        <is>
+          <t>INFILTRACION</t>
+        </is>
+      </c>
+      <c r="C379" s="10" t="n"/>
+      <c r="D379" s="18" t="inlineStr">
+        <is>
+          <t>VOLUMEN (m3)</t>
+        </is>
+      </c>
+      <c r="E379" s="10" t="n"/>
+      <c r="F379" s="10" t="n"/>
       <c r="G379" s="2" t="n"/>
-      <c r="H379" s="37" t="n"/>
-      <c r="I379" s="37" t="n"/>
-    </row>
-    <row r="380" ht="39.7" customHeight="1">
-      <c r="A380" s="18" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B380" s="35" t="inlineStr">
-        <is>
-          <t>INFILTRACION</t>
-        </is>
-      </c>
-      <c r="C380" s="10" t="n"/>
-      <c r="D380" s="18" t="inlineStr">
-        <is>
-          <t>VOLUMEN (m3)</t>
-        </is>
-      </c>
-      <c r="E380" s="10" t="n"/>
-      <c r="F380" s="10" t="n"/>
+      <c r="H379" s="2" t="n"/>
+      <c r="I379" s="2" t="n"/>
+    </row>
+    <row r="380" ht="62" customHeight="1">
+      <c r="A380" s="10" t="n"/>
+      <c r="B380" s="36" t="inlineStr">
+        <is>
+          <t>UNA PARED EXTERIOR</t>
+        </is>
+      </c>
+      <c r="C380" s="10" t="inlineStr"/>
+      <c r="D380" s="9">
+        <f>IF(COUNT(H380,I380)&lt;2,"",ROUND(H380*I380,2))</f>
+        <v/>
+      </c>
+      <c r="E380" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="F380" s="30">
+        <f>IF(D380="","",ROUND(D380*E380,1))</f>
+        <v/>
+      </c>
       <c r="G380" s="2" t="n"/>
-      <c r="H380" s="2" t="n"/>
-      <c r="I380" s="2" t="n"/>
-    </row>
-    <row r="381" ht="62" customHeight="1">
+      <c r="H380" s="37" t="n"/>
+      <c r="I380" s="37" t="n"/>
+    </row>
+    <row r="381" ht="39.7" customHeight="1">
       <c r="A381" s="10" t="n"/>
       <c r="B381" s="36" t="inlineStr">
         <is>
-          <t>UNA PARED EXTERIOR</t>
-        </is>
-      </c>
-      <c r="C381" s="10" t="inlineStr"/>
-      <c r="D381" s="9">
-        <f>IF(COUNT(H381,I381)&lt;2,"",ROUND(H381*I381,2))</f>
-        <v/>
+          <t>DOS PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C381" s="10" t="inlineStr">
+        <is>
+          <t>3.52 m2 x 3.00</t>
+        </is>
+      </c>
+      <c r="D381" s="9" t="n">
+        <v>10.56</v>
       </c>
       <c r="E381" s="27" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F381" s="30">
         <f>IF(D381="","",ROUND(D381*E381,1))</f>
@@ -31288,23 +31289,20 @@
       <c r="H381" s="37" t="n"/>
       <c r="I381" s="37" t="n"/>
     </row>
-    <row r="382" ht="39.7" customHeight="1">
+    <row r="382" ht="62" customHeight="1">
       <c r="A382" s="10" t="n"/>
       <c r="B382" s="36" t="inlineStr">
         <is>
-          <t>DOS PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C382" s="10" t="inlineStr">
-        <is>
-          <t>3.52 m2 x 3.00</t>
-        </is>
-      </c>
-      <c r="D382" s="9" t="n">
-        <v>10.56</v>
+          <t>TRES O MAS PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C382" s="10" t="inlineStr"/>
+      <c r="D382" s="9">
+        <f>IF(COUNT(H382,I382)&lt;2,"",ROUND(H382*I382,2))</f>
+        <v/>
       </c>
       <c r="E382" s="27" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F382" s="30">
         <f>IF(D382="","",ROUND(D382*E382,1))</f>
@@ -31314,129 +31312,124 @@
       <c r="H382" s="37" t="n"/>
       <c r="I382" s="37" t="n"/>
     </row>
-    <row r="383" ht="62" customHeight="1">
-      <c r="A383" s="10" t="n"/>
-      <c r="B383" s="36" t="inlineStr">
-        <is>
-          <t>TRES O MAS PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C383" s="10" t="inlineStr"/>
-      <c r="D383" s="9">
-        <f>IF(COUNT(H383,I383)&lt;2,"",ROUND(H383*I383,2))</f>
-        <v/>
-      </c>
-      <c r="E383" s="27" t="n">
-        <v>12</v>
-      </c>
-      <c r="F383" s="30">
-        <f>IF(D383="","",ROUND(D383*E383,1))</f>
+    <row r="383" ht="70" customHeight="1">
+      <c r="A383" s="18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B383" s="35" t="inlineStr">
+        <is>
+          <t>SUBTOTAL</t>
+        </is>
+      </c>
+      <c r="C383" s="10" t="n"/>
+      <c r="D383" s="10" t="n"/>
+      <c r="E383" s="10" t="n"/>
+      <c r="F383" s="38">
+        <f>IF(F366="",0,F366)+IF(F368="",0,F368)+IF(F369="",0,F369)+IF(F370="",0,F370)+IF(F371="",0,F371)+IF(F373="",0,F373)+IF(F374="",0,F374)+IF(F375="",0,F375)+IF(F377="",0,F377)+IF(F378="",0,F378)+IF(F380="",0,F380)+IF(F381="",0,F381)+IF(F382="",0,F382)</f>
         <v/>
       </c>
       <c r="G383" s="2" t="n"/>
-      <c r="H383" s="37" t="n"/>
-      <c r="I383" s="37" t="n"/>
-    </row>
-    <row r="384" ht="70" customHeight="1">
+      <c r="H383" s="2" t="n"/>
+      <c r="I383" s="2" t="n"/>
+    </row>
+    <row r="384" ht="47" customHeight="1">
       <c r="A384" s="18" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B384" s="35" t="inlineStr">
         <is>
-          <t>SUBTOTAL</t>
-        </is>
-      </c>
-      <c r="C384" s="10" t="n"/>
-      <c r="D384" s="10" t="n"/>
-      <c r="E384" s="10" t="n"/>
+          <t>PERDIDA TOTAL</t>
+        </is>
+      </c>
+      <c r="C384" s="10">
+        <f>TEXT(F383,"0.00")&amp;"  X  "&amp;Datos_balance!$B$4&amp;" (FI)  X  "&amp;Datos_balance!$B$5&amp;" (FO)  X  "&amp;Datos_balance!$B$6&amp;" (FZ)"</f>
+        <v/>
+      </c>
+      <c r="D384" s="2" t="n"/>
+      <c r="E384" s="2" t="n"/>
       <c r="F384" s="38">
-        <f>IF(F367="",0,F367)+IF(F369="",0,F369)+IF(F370="",0,F370)+IF(F371="",0,F371)+IF(F372="",0,F372)+IF(F374="",0,F374)+IF(F375="",0,F375)+IF(F376="",0,F376)+IF(F378="",0,F378)+IF(F379="",0,F379)+IF(F381="",0,F381)+IF(F382="",0,F382)+IF(F383="",0,F383)</f>
+        <f>ROUND(F383*Datos_balance!$B$4*Datos_balance!$B$5*Datos_balance!$B$6,1)</f>
         <v/>
       </c>
       <c r="G384" s="2" t="n"/>
       <c r="H384" s="2" t="n"/>
       <c r="I384" s="2" t="n"/>
     </row>
-    <row r="385" ht="47" customHeight="1">
-      <c r="A385" s="18" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B385" s="35" t="inlineStr">
-        <is>
-          <t>PERDIDA TOTAL</t>
-        </is>
-      </c>
-      <c r="C385" s="10">
-        <f>TEXT(F384,"0.00")&amp;"  X  "&amp;Datos_balance!$B$4&amp;" (FI)  X  "&amp;Datos_balance!$B$5&amp;" (FO)  X  "&amp;Datos_balance!$B$6&amp;" (FZ)"</f>
-        <v/>
-      </c>
+    <row r="385" ht="39.7" customHeight="1">
+      <c r="A385" s="10" t="n"/>
+      <c r="B385" s="11" t="inlineStr">
+        <is>
+          <t>Carga de locales sin emisor</t>
+        </is>
+      </c>
+      <c r="C385" s="10" t="n"/>
       <c r="D385" s="2" t="n"/>
       <c r="E385" s="2" t="n"/>
-      <c r="F385" s="38">
-        <f>ROUND(F384*Datos_balance!$B$4*Datos_balance!$B$5*Datos_balance!$B$6,1)</f>
-        <v/>
-      </c>
+      <c r="F385" s="30" t="n"/>
       <c r="G385" s="2" t="n"/>
       <c r="H385" s="2" t="n"/>
       <c r="I385" s="2" t="n"/>
     </row>
     <row r="386" ht="39.7" customHeight="1">
       <c r="A386" s="10" t="n"/>
-      <c r="B386" s="11" t="inlineStr">
-        <is>
-          <t>Carga de locales sin emisor</t>
+      <c r="B386" s="35" t="inlineStr">
+        <is>
+          <t>CARGA TOTAL A CUBRIR</t>
         </is>
       </c>
       <c r="C386" s="10" t="n"/>
       <c r="D386" s="2" t="n"/>
       <c r="E386" s="2" t="n"/>
-      <c r="F386" s="30" t="n"/>
+      <c r="F386" s="38">
+        <f>F384+IF(F385="",0,F385)</f>
+        <v/>
+      </c>
       <c r="G386" s="2" t="n"/>
       <c r="H386" s="2" t="n"/>
       <c r="I386" s="2" t="n"/>
     </row>
-    <row r="387" ht="39.7" customHeight="1">
-      <c r="A387" s="10" t="n"/>
-      <c r="B387" s="35" t="inlineStr">
-        <is>
-          <t>CARGA TOTAL A CUBRIR</t>
-        </is>
-      </c>
-      <c r="C387" s="10" t="n"/>
+    <row r="387">
+      <c r="A387" s="2" t="n"/>
+      <c r="B387" s="2" t="n"/>
+      <c r="C387" s="2" t="n"/>
       <c r="D387" s="2" t="n"/>
       <c r="E387" s="2" t="n"/>
-      <c r="F387" s="38">
-        <f>F385+IF(F386="",0,F386)</f>
-        <v/>
-      </c>
+      <c r="F387" s="2" t="n"/>
       <c r="G387" s="2" t="n"/>
       <c r="H387" s="2" t="n"/>
       <c r="I387" s="2" t="n"/>
     </row>
-    <row r="388">
-      <c r="A388" s="2" t="n"/>
-      <c r="B388" s="2" t="n"/>
-      <c r="C388" s="2" t="n"/>
+    <row r="388" ht="62" customHeight="1">
+      <c r="A388" s="10" t="n"/>
+      <c r="B388" s="11" t="inlineStr">
+        <is>
+          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
+        </is>
+      </c>
+      <c r="C388" s="10">
+        <f>TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2,"0")&amp;" - "&amp;TEXT(Datos_balance!$B$11,"0")&amp;" = "&amp;TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2-Datos_balance!$B$11,"0")&amp;" C"</f>
+        <v/>
+      </c>
       <c r="D388" s="2" t="n"/>
       <c r="E388" s="2" t="n"/>
-      <c r="F388" s="2" t="n"/>
+      <c r="F388" s="10" t="n"/>
       <c r="G388" s="2" t="n"/>
       <c r="H388" s="2" t="n"/>
       <c r="I388" s="2" t="n"/>
     </row>
-    <row r="389" ht="62" customHeight="1">
+    <row r="389" ht="39.7" customHeight="1">
       <c r="A389" s="10" t="n"/>
       <c r="B389" s="11" t="inlineStr">
         <is>
-          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
-        </is>
-      </c>
-      <c r="C389" s="10">
-        <f>TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2,"0")&amp;" - "&amp;TEXT(Datos_balance!$B$11,"0")&amp;" = "&amp;TEXT((Datos_balance!$B$9+Datos_balance!$B$10)/2-Datos_balance!$B$11,"0")&amp;" C"</f>
+          <t>Kcal/h del toallero Scala/Domino 80</t>
+        </is>
+      </c>
+      <c r="C389" s="27">
+        <f>ROUND(Datos_balance!$B$18*Datos_balance!$B$15,0)</f>
         <v/>
       </c>
       <c r="D389" s="2" t="n"/>
@@ -31450,11 +31443,11 @@
       <c r="A390" s="10" t="n"/>
       <c r="B390" s="11" t="inlineStr">
         <is>
-          <t>Kcal/h del toallero Scala/Domino 80</t>
+          <t>Kcal/h del toallero Scala/Domino 150</t>
         </is>
       </c>
       <c r="C390" s="27">
-        <f>ROUND(Datos_balance!$B$18*Datos_balance!$B$15,0)</f>
+        <f>ROUND(Datos_balance!$B$19*Datos_balance!$B$15,0)</f>
         <v/>
       </c>
       <c r="D390" s="2" t="n"/>
@@ -31464,15 +31457,15 @@
       <c r="H390" s="2" t="n"/>
       <c r="I390" s="2" t="n"/>
     </row>
-    <row r="391" ht="39.7" customHeight="1">
+    <row r="391" ht="47" customHeight="1">
       <c r="A391" s="10" t="n"/>
       <c r="B391" s="11" t="inlineStr">
         <is>
-          <t>Kcal/h del toallero Scala/Domino 150</t>
+          <t>Toalleros necesarios</t>
         </is>
       </c>
       <c r="C391" s="27">
-        <f>ROUND(Datos_balance!$B$19*Datos_balance!$B$15,0)</f>
+        <f>IF(F386&lt;=Datos_balance!$B$18*Datos_balance!$B$15,1,ROUNDUP(F386/(Datos_balance!$B$19*Datos_balance!$B$15),0))</f>
         <v/>
       </c>
       <c r="D391" s="2" t="n"/>
@@ -31483,40 +31476,22 @@
       <c r="I391" s="2" t="n"/>
     </row>
     <row r="392" ht="47" customHeight="1">
-      <c r="A392" s="10" t="n"/>
-      <c r="B392" s="11" t="inlineStr">
-        <is>
-          <t>Toalleros necesarios</t>
-        </is>
-      </c>
-      <c r="C392" s="27">
-        <f>IF(F387&lt;=Datos_balance!$B$18*Datos_balance!$B$15,1,ROUNDUP(F387/(Datos_balance!$B$19*Datos_balance!$B$15),0))</f>
-        <v/>
-      </c>
-      <c r="D392" s="2" t="n"/>
-      <c r="E392" s="2" t="n"/>
-      <c r="F392" s="10" t="n"/>
+      <c r="A392" s="14" t="n"/>
+      <c r="B392" s="15" t="inlineStr">
+        <is>
+          <t>Toallero adoptado</t>
+        </is>
+      </c>
+      <c r="C392" s="14">
+        <f>IF(F386&lt;=Datos_balance!$B$18*Datos_balance!$B$15,"Peisa Scala / Domino 80  (500 x 800 mm)","Peisa Scala / Domino 150  (500 x 1500 mm)")</f>
+        <v/>
+      </c>
+      <c r="D392" s="22" t="n"/>
+      <c r="E392" s="22" t="n"/>
+      <c r="F392" s="14" t="n"/>
       <c r="G392" s="2" t="n"/>
       <c r="H392" s="2" t="n"/>
       <c r="I392" s="2" t="n"/>
-    </row>
-    <row r="393" ht="47" customHeight="1">
-      <c r="A393" s="14" t="n"/>
-      <c r="B393" s="15" t="inlineStr">
-        <is>
-          <t>Toallero adoptado</t>
-        </is>
-      </c>
-      <c r="C393" s="14">
-        <f>IF(F387&lt;=Datos_balance!$B$18*Datos_balance!$B$15,"Peisa Scala / Domino 80  (500 x 800 mm)","Peisa Scala / Domino 150  (500 x 1500 mm)")</f>
-        <v/>
-      </c>
-      <c r="D393" s="22" t="n"/>
-      <c r="E393" s="22" t="n"/>
-      <c r="F393" s="14" t="n"/>
-      <c r="G393" s="2" t="n"/>
-      <c r="H393" s="2" t="n"/>
-      <c r="I393" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="101">
@@ -31537,7 +31512,6 @@
     <mergeCell ref="A72:F72"/>
     <mergeCell ref="A38:F38"/>
     <mergeCell ref="C292:E292"/>
-    <mergeCell ref="C355:E355"/>
     <mergeCell ref="C293:E293"/>
     <mergeCell ref="C220:E220"/>
     <mergeCell ref="C391:E391"/>
@@ -31551,6 +31525,7 @@
     <mergeCell ref="C133:E133"/>
     <mergeCell ref="C127:E127"/>
     <mergeCell ref="C320:E320"/>
+    <mergeCell ref="C356:E356"/>
     <mergeCell ref="C130:E130"/>
     <mergeCell ref="C295:E295"/>
     <mergeCell ref="C61:E61"/>
@@ -31559,6 +31534,7 @@
     <mergeCell ref="C224:E224"/>
     <mergeCell ref="C32:E32"/>
     <mergeCell ref="C125:E125"/>
+    <mergeCell ref="C352:E352"/>
     <mergeCell ref="C161:E161"/>
     <mergeCell ref="C131:E131"/>
     <mergeCell ref="C258:E258"/>
@@ -31590,24 +31566,22 @@
     <mergeCell ref="C254:E254"/>
     <mergeCell ref="C354:E354"/>
     <mergeCell ref="C62:E62"/>
-    <mergeCell ref="C387:E387"/>
     <mergeCell ref="C191:E191"/>
     <mergeCell ref="C225:E225"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="C353:E353"/>
-    <mergeCell ref="C393:E393"/>
     <mergeCell ref="C227:E227"/>
+    <mergeCell ref="A363:F363"/>
     <mergeCell ref="C93:E93"/>
     <mergeCell ref="C226:E226"/>
     <mergeCell ref="A264:F264"/>
-    <mergeCell ref="A364:F364"/>
     <mergeCell ref="C291:E291"/>
+    <mergeCell ref="C388:E388"/>
     <mergeCell ref="C188:E188"/>
     <mergeCell ref="C222:E222"/>
     <mergeCell ref="C27:E27"/>
     <mergeCell ref="C132:E132"/>
     <mergeCell ref="A298:F298"/>
-    <mergeCell ref="C361:E361"/>
     <mergeCell ref="C253:E253"/>
     <mergeCell ref="C327:E327"/>
     <mergeCell ref="C358:E358"/>
@@ -31620,6 +31594,7 @@
     <mergeCell ref="C386:E386"/>
     <mergeCell ref="C97:E97"/>
     <mergeCell ref="C29:E29"/>
+    <mergeCell ref="C384:E384"/>
     <mergeCell ref="C65:E65"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Croquis de mejor calidad: imagen a 1000 px y nombre de cuerpo fijo
- la imagen se recorta, se reduce a 1000 px y recien ahi se escribe el nombre,
  con un cuerpo proporcional a la salida, para que se lea igual en todos
- margen de encuadre a 9%, que dejaba demasiado aire

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -2360,7 +2360,7 @@
       <row>37</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4381500" cy="4886325"/>
+    <ext cx="4381500" cy="5000625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -2385,7 +2385,7 @@
       <row>84</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4381500" cy="4886325"/>
+    <ext cx="4381500" cy="5000625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -2410,7 +2410,7 @@
       <row>125</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4381500" cy="4886325"/>
+    <ext cx="4381500" cy="5000625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -2435,7 +2435,7 @@
       <row>174</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4381500" cy="4886325"/>
+    <ext cx="4381500" cy="5000625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -2460,7 +2460,7 @@
       <row>215</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4381500" cy="4219575"/>
+    <ext cx="4381500" cy="4171950"/>
     <pic>
       <nvPicPr>
         <cNvPr id="5" name="Image 5" descr="Picture"/>
@@ -2485,7 +2485,7 @@
       <row>261</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4381500" cy="4886325"/>
+    <ext cx="4381500" cy="5000625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="6" name="Image 6" descr="Picture"/>
@@ -2510,7 +2510,7 @@
       <row>307</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4381500" cy="4886325"/>
+    <ext cx="4381500" cy="5000625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="7" name="Image 7" descr="Picture"/>
@@ -2535,7 +2535,7 @@
       <row>353</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4381500" cy="4886325"/>
+    <ext cx="4381500" cy="5000625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="8" name="Image 8" descr="Picture"/>
@@ -2560,7 +2560,7 @@
       <row>400</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4381500" cy="4219575"/>
+    <ext cx="4381500" cy="4171950"/>
     <pic>
       <nvPicPr>
         <cNvPr id="9" name="Image 9" descr="Picture"/>
@@ -2585,7 +2585,7 @@
       <row>445</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4381500" cy="4219575"/>
+    <ext cx="4381500" cy="4171950"/>
     <pic>
       <nvPicPr>
         <cNvPr id="10" name="Image 10" descr="Picture"/>
@@ -2610,7 +2610,7 @@
       <row>489</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4381500" cy="4219575"/>
+    <ext cx="4381500" cy="4171950"/>
     <pic>
       <nvPicPr>
         <cNvPr id="11" name="Image 11" descr="Picture"/>
@@ -2635,7 +2635,7 @@
       <row>533</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4381500" cy="4219575"/>
+    <ext cx="4381500" cy="4171950"/>
     <pic>
       <nvPicPr>
         <cNvPr id="12" name="Image 12" descr="Picture"/>

</xml_diff>

<commit_message>
El rotulo del croquis nombra el local, para no confundirlo con el bloque siguiente
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -344,7 +344,7 @@
     <xf numFmtId="165" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -23945,7 +23945,7 @@
       <c r="A37" s="2" t="n"/>
       <c r="B37" s="39" t="inlineStr">
         <is>
-          <t>Ubicacion del local en planta</t>
+          <t>Ubicacion en planta de 01 - Cocina / comedor</t>
         </is>
       </c>
       <c r="C37" s="2" t="n"/>
@@ -24850,7 +24850,7 @@
       <c r="A84" s="2" t="n"/>
       <c r="B84" s="39" t="inlineStr">
         <is>
-          <t>Ubicacion del local en planta</t>
+          <t>Ubicacion en planta de 06 - Living / comedor</t>
         </is>
       </c>
       <c r="C84" s="2" t="n"/>
@@ -25621,7 +25621,7 @@
       <c r="A125" s="2" t="n"/>
       <c r="B125" s="39" t="inlineStr">
         <is>
-          <t>Ubicacion del local en planta</t>
+          <t>Ubicacion en planta de 07 - Hall / ingreso</t>
         </is>
       </c>
       <c r="C125" s="2" t="n"/>
@@ -26575,7 +26575,7 @@
       <c r="A174" s="2" t="n"/>
       <c r="B174" s="39" t="inlineStr">
         <is>
-          <t>Ubicacion del local en planta</t>
+          <t>Ubicacion en planta de 08 - Vestidor</t>
         </is>
       </c>
       <c r="C174" s="2" t="n"/>
@@ -27346,7 +27346,7 @@
       <c r="A215" s="2" t="n"/>
       <c r="B215" s="39" t="inlineStr">
         <is>
-          <t>Ubicacion del local en planta</t>
+          <t>Ubicacion en planta de Escalera</t>
         </is>
       </c>
       <c r="C215" s="2" t="n"/>
@@ -28233,7 +28233,7 @@
       <c r="A261" s="2" t="n"/>
       <c r="B261" s="39" t="inlineStr">
         <is>
-          <t>Ubicacion del local en planta</t>
+          <t>Ubicacion en planta de 09 - Dormitorio suite</t>
         </is>
       </c>
       <c r="C261" s="2" t="n"/>
@@ -29101,7 +29101,7 @@
       <c r="A307" s="2" t="n"/>
       <c r="B307" s="39" t="inlineStr">
         <is>
-          <t>Ubicacion del local en planta</t>
+          <t>Ubicacion en planta de 10 - Bano suite</t>
         </is>
       </c>
       <c r="C307" s="2" t="n"/>
@@ -29965,7 +29965,7 @@
       <c r="A353" s="2" t="n"/>
       <c r="B353" s="39" t="inlineStr">
         <is>
-          <t>Ubicacion del local en planta</t>
+          <t>Ubicacion en planta de 11 - Bano visitas</t>
         </is>
       </c>
       <c r="C353" s="2" t="n"/>
@@ -30863,7 +30863,7 @@
       <c r="A400" s="2" t="n"/>
       <c r="B400" s="39" t="inlineStr">
         <is>
-          <t>Ubicacion del local en planta</t>
+          <t>Ubicacion en planta de 13 - Dormitorio Norte</t>
         </is>
       </c>
       <c r="C400" s="2" t="n"/>
@@ -31727,7 +31727,7 @@
       <c r="A445" s="2" t="n"/>
       <c r="B445" s="39" t="inlineStr">
         <is>
-          <t>Ubicacion del local en planta</t>
+          <t>Ubicacion en planta de 14 - Play room</t>
         </is>
       </c>
       <c r="C445" s="2" t="n"/>
@@ -32558,7 +32558,7 @@
       <c r="A489" s="2" t="n"/>
       <c r="B489" s="39" t="inlineStr">
         <is>
-          <t>Ubicacion del local en planta</t>
+          <t>Ubicacion en planta de 15 - Dormitorio Sur</t>
         </is>
       </c>
       <c r="C489" s="2" t="n"/>
@@ -33389,7 +33389,7 @@
       <c r="A533" s="2" t="n"/>
       <c r="B533" s="39" t="inlineStr">
         <is>
-          <t>Ubicacion del local en planta</t>
+          <t>Ubicacion en planta de 17 - Bano</t>
         </is>
       </c>
       <c r="C533" s="2" t="n"/>

</xml_diff>

<commit_message>
Formato: titulos de 1 cm, interiores en puntos, fila en blanco entre bloques
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura.xlsx
+++ b/planillas/planillas_estructura.xlsx
@@ -23134,16 +23134,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="39.7" customHeight="1">
-      <c r="A1" s="18" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>FORMULARIO DE BALANCE TERMICO PARA CALEFACCION</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
+      <c r="B1" s="10" t="n"/>
+      <c r="C1" s="10" t="n"/>
+      <c r="D1" s="10" t="n"/>
+      <c r="E1" s="10" t="n"/>
+      <c r="F1" s="10" t="n"/>
       <c r="G1" s="2" t="n"/>
       <c r="H1" s="3" t="inlineStr">
         <is>
@@ -23668,7 +23668,7 @@
       <c r="C22" s="10" t="n"/>
       <c r="D22" s="18" t="inlineStr">
         <is>
-          <t>VOLUMEN (m3)</t>
+          <t>VOL. (m3)</t>
         </is>
       </c>
       <c r="E22" s="10" t="n"/>
@@ -24566,7 +24566,7 @@
       <c r="C69" s="10" t="n"/>
       <c r="D69" s="18" t="inlineStr">
         <is>
-          <t>VOLUMEN (m3)</t>
+          <t>VOL. (m3)</t>
         </is>
       </c>
       <c r="E69" s="10" t="n"/>
@@ -25445,7 +25445,7 @@
       <c r="C115" s="10" t="n"/>
       <c r="D115" s="18" t="inlineStr">
         <is>
-          <t>VOLUMEN (m3)</t>
+          <t>VOL. (m3)</t>
         </is>
       </c>
       <c r="E115" s="10" t="n"/>
@@ -26298,7 +26298,7 @@
       <c r="C159" s="10" t="n"/>
       <c r="D159" s="18" t="inlineStr">
         <is>
-          <t>VOLUMEN (m3)</t>
+          <t>VOL. (m3)</t>
         </is>
       </c>
       <c r="E159" s="10" t="n"/>
@@ -27140,7 +27140,7 @@
       <c r="C204" s="10" t="n"/>
       <c r="D204" s="18" t="inlineStr">
         <is>
-          <t>VOLUMEN (m3)</t>
+          <t>VOL. (m3)</t>
         </is>
       </c>
       <c r="E204" s="10" t="n"/>
@@ -27956,7 +27956,7 @@
       <c r="C246" s="10" t="n"/>
       <c r="D246" s="18" t="inlineStr">
         <is>
-          <t>VOLUMEN (m3)</t>
+          <t>VOL. (m3)</t>
         </is>
       </c>
       <c r="E246" s="10" t="n"/>
@@ -28824,7 +28824,7 @@
       <c r="C292" s="10" t="n"/>
       <c r="D292" s="18" t="inlineStr">
         <is>
-          <t>VOLUMEN (m3)</t>
+          <t>VOL. (m3)</t>
         </is>
       </c>
       <c r="E292" s="10" t="n"/>
@@ -29688,7 +29688,7 @@
       <c r="C338" s="10" t="n"/>
       <c r="D338" s="18" t="inlineStr">
         <is>
-          <t>VOLUMEN (m3)</t>
+          <t>VOL. (m3)</t>
         </is>
       </c>
       <c r="E338" s="10" t="n"/>
@@ -30586,7 +30586,7 @@
       <c r="C385" s="10" t="n"/>
       <c r="D385" s="18" t="inlineStr">
         <is>
-          <t>VOLUMEN (m3)</t>
+          <t>VOL. (m3)</t>
         </is>
       </c>
       <c r="E385" s="10" t="n"/>
@@ -31413,7 +31413,7 @@
       <c r="C429" s="10" t="n"/>
       <c r="D429" s="18" t="inlineStr">
         <is>
-          <t>VOLUMEN (m3)</t>
+          <t>VOL. (m3)</t>
         </is>
       </c>
       <c r="E429" s="10" t="n"/>
@@ -32251,7 +32251,7 @@
       <c r="C473" s="10" t="n"/>
       <c r="D473" s="18" t="inlineStr">
         <is>
-          <t>VOLUMEN (m3)</t>
+          <t>VOL. (m3)</t>
         </is>
       </c>
       <c r="E473" s="10" t="n"/>
@@ -33082,7 +33082,7 @@
       <c r="C517" s="10" t="n"/>
       <c r="D517" s="18" t="inlineStr">
         <is>
-          <t>VOLUMEN (m3)</t>
+          <t>VOL. (m3)</t>
         </is>
       </c>
       <c r="E517" s="10" t="n"/>

</xml_diff>